<commit_message>
Admin: Display campaign cutting dates in Detail view and optimize summary loading
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFE3E068-177F-3E43-8885-65E80AA55D04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CBE88A1-8BAA-FF47-855B-D64B4D1DB489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2440" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
+    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
   <sheets>
     <sheet name="pagado_pendiente" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="56">
   <si>
     <t>Asesor</t>
   </si>
@@ -90,9 +90,6 @@
   </si>
   <si>
     <t>GABRIELA CASTAÐEDA SALAZAR</t>
-  </si>
-  <si>
-    <t>CLAUDIA VALERIA HERNANDEZ MACIAS</t>
   </si>
   <si>
     <t>JULIANA RIASCOS VALENCIA</t>
@@ -373,7 +370,163 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="24">
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <border>
         <top style="thin">
@@ -881,7 +1034,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46081</v>
+        <v>46091</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -895,28 +1048,28 @@
       <c r="D2" s="9"/>
       <c r="E2" s="8"/>
       <c r="F2" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I2" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="J2" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="K2" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="L2" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="M2" s="12" t="s">
         <v>47</v>
-      </c>
-      <c r="J2" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="K2" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="L2" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="M2" s="12" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
@@ -930,227 +1083,227 @@
         <v>2</v>
       </c>
       <c r="D3" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>54</v>
-      </c>
       <c r="J3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
-        <v>90355</v>
+        <v>87538</v>
       </c>
       <c r="B4" s="2">
         <v>2043</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="D4" s="11">
-        <v>43949</v>
+        <v>43731</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F4" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G4" s="4">
-        <v>65475.85</v>
+        <v>0</v>
       </c>
       <c r="H4" s="4">
-        <v>78223.64</v>
+        <v>67732.53</v>
       </c>
       <c r="I4" s="4">
-        <v>143699.49</v>
+        <v>67732.53</v>
       </c>
       <c r="J4" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" s="4">
-        <v>73149.789999999994</v>
+        <v>327363.81</v>
       </c>
       <c r="L4" s="4">
-        <v>32434.68</v>
+        <v>279799.13</v>
       </c>
       <c r="M4" s="4">
-        <v>105584.47</v>
+        <v>607162.93999999994</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
-        <v>87538</v>
+        <v>110453</v>
       </c>
       <c r="B5" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D5" s="11">
-        <v>43731</v>
+        <v>45600</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F5" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5" s="4">
-        <v>7105.46</v>
+        <v>1840.93</v>
       </c>
       <c r="H5" s="4">
-        <v>115600.42</v>
+        <v>53733.89</v>
       </c>
       <c r="I5" s="4">
-        <v>122705.88</v>
+        <v>55574.82</v>
       </c>
       <c r="J5" s="3">
         <v>1</v>
       </c>
       <c r="K5" s="4">
-        <v>24219.9</v>
+        <v>1770.92</v>
       </c>
       <c r="L5" s="4">
-        <v>290298.78000000003</v>
+        <v>191490.39</v>
       </c>
       <c r="M5" s="4">
-        <v>314518.68</v>
+        <v>193261.31</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>47116</v>
+        <v>115047</v>
       </c>
       <c r="B6" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="D6" s="11">
-        <v>44616</v>
+        <v>45944</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F6" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G6" s="4">
-        <v>3031.24</v>
+        <v>0</v>
       </c>
       <c r="H6" s="4">
-        <v>80954.98</v>
+        <v>17733.23</v>
       </c>
       <c r="I6" s="4">
-        <v>83986.22</v>
+        <v>17733.23</v>
       </c>
       <c r="J6" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" s="4">
-        <v>0</v>
+        <v>24502.57</v>
       </c>
       <c r="L6" s="4">
-        <v>30944.62</v>
+        <v>34641.980000000003</v>
       </c>
       <c r="M6" s="4">
-        <v>30944.62</v>
+        <v>59144.55</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>110453</v>
+        <v>104718</v>
       </c>
       <c r="B7" s="2">
-        <v>2856</v>
+        <v>2692</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D7" s="11">
-        <v>45600</v>
+        <v>45264</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F7" s="3">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G7" s="4">
-        <v>20571.09</v>
+        <v>0</v>
       </c>
       <c r="H7" s="4">
-        <v>36575.69</v>
+        <v>12271.64</v>
       </c>
       <c r="I7" s="4">
-        <v>57146.78</v>
+        <v>12271.64</v>
       </c>
       <c r="J7" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" s="4">
-        <v>1770.92</v>
+        <v>0</v>
       </c>
       <c r="L7" s="4">
-        <v>190572.16</v>
+        <v>101498.18</v>
       </c>
       <c r="M7" s="4">
-        <v>192343.08</v>
+        <v>101498.18</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>116876</v>
+        <v>94205</v>
       </c>
       <c r="B8" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="D8" s="11">
-        <v>46006</v>
+        <v>44116</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F8" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G8" s="4">
-        <v>3287.41</v>
+        <v>0</v>
       </c>
       <c r="H8" s="4">
-        <v>49917.93</v>
+        <v>10135.31</v>
       </c>
       <c r="I8" s="4">
-        <v>53205.34</v>
+        <v>10135.31</v>
       </c>
       <c r="J8" s="3">
         <v>0</v>
@@ -1159,10 +1312,10 @@
         <v>0</v>
       </c>
       <c r="L8" s="4">
-        <v>22059.07</v>
+        <v>0</v>
       </c>
       <c r="M8" s="4">
-        <v>22059.07</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -1173,25 +1326,25 @@
         <v>2043</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D9" s="11">
         <v>43371</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F9" s="3">
         <v>1</v>
       </c>
       <c r="G9" s="4">
-        <v>24126.87</v>
+        <v>2550.13</v>
       </c>
       <c r="H9" s="4">
-        <v>22146.95</v>
+        <v>4599.88</v>
       </c>
       <c r="I9" s="4">
-        <v>46273.82</v>
+        <v>7150.01</v>
       </c>
       <c r="J9" s="3">
         <v>0</v>
@@ -1200,39 +1353,39 @@
         <v>0</v>
       </c>
       <c r="L9" s="4">
-        <v>76193.69</v>
+        <v>104245.15</v>
       </c>
       <c r="M9" s="4">
-        <v>76193.69</v>
+        <v>104245.15</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>108404</v>
+        <v>114157</v>
       </c>
       <c r="B10" s="2">
         <v>2692</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D10" s="11">
-        <v>45467</v>
+        <v>45904</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F10" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" s="4">
-        <v>1664.46</v>
+        <v>0</v>
       </c>
       <c r="H10" s="4">
-        <v>42912.38</v>
+        <v>5489.13</v>
       </c>
       <c r="I10" s="4">
-        <v>44576.84</v>
+        <v>5489.13</v>
       </c>
       <c r="J10" s="3">
         <v>0</v>
@@ -1241,39 +1394,39 @@
         <v>0</v>
       </c>
       <c r="L10" s="4">
-        <v>48840.36</v>
+        <v>57999.18</v>
       </c>
       <c r="M10" s="4">
-        <v>48840.36</v>
+        <v>57999.18</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>104718</v>
+        <v>111056</v>
       </c>
       <c r="B11" s="2">
         <v>2692</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D11" s="11">
-        <v>45264</v>
+        <v>45639</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F11" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G11" s="4">
-        <v>8808.02</v>
+        <v>0</v>
       </c>
       <c r="H11" s="4">
-        <v>31919.65</v>
+        <v>5403.95</v>
       </c>
       <c r="I11" s="4">
-        <v>40727.67</v>
+        <v>5403.95</v>
       </c>
       <c r="J11" s="3">
         <v>0</v>
@@ -1282,68 +1435,68 @@
         <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>108479.01</v>
+        <v>61189.599999999999</v>
       </c>
       <c r="M11" s="4">
-        <v>108479.01</v>
+        <v>61189.599999999999</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>104750</v>
+        <v>116883</v>
       </c>
       <c r="B12" s="2">
-        <v>2692</v>
+        <v>2856</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="D12" s="11">
-        <v>45236</v>
+        <v>46007</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F12" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12" s="4">
-        <v>13090.79</v>
+        <v>5187.54</v>
       </c>
       <c r="H12" s="4">
-        <v>15670.39</v>
+        <v>0</v>
       </c>
       <c r="I12" s="4">
-        <v>28761.18</v>
+        <v>5187.54</v>
       </c>
       <c r="J12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" s="4">
-        <v>0</v>
+        <v>1820.53</v>
       </c>
       <c r="L12" s="4">
-        <v>37181.47</v>
+        <v>45347.65</v>
       </c>
       <c r="M12" s="4">
-        <v>37181.47</v>
+        <v>47168.18</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>107488</v>
+        <v>80925</v>
       </c>
       <c r="B13" s="2">
         <v>2043</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="D13" s="11">
-        <v>45440</v>
+        <v>43439</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F13" s="3">
         <v>0</v>
@@ -1352,10 +1505,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="4">
-        <v>27019.22</v>
+        <v>5119.8</v>
       </c>
       <c r="I13" s="4">
-        <v>27019.22</v>
+        <v>5119.8</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1364,39 +1517,39 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>128333.66</v>
+        <v>10061.92</v>
       </c>
       <c r="M13" s="4">
-        <v>128333.66</v>
+        <v>10061.92</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>113450</v>
+        <v>117440</v>
       </c>
       <c r="B14" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="D14" s="11">
-        <v>45852</v>
+        <v>46059</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F14" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G14" s="4">
-        <v>0</v>
+        <v>3011.72</v>
       </c>
       <c r="H14" s="4">
-        <v>24276.99</v>
+        <v>1975.99</v>
       </c>
       <c r="I14" s="4">
-        <v>24276.99</v>
+        <v>4987.71</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1405,27 +1558,27 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>9978.11</v>
+        <v>0</v>
       </c>
       <c r="M14" s="4">
-        <v>9978.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>115047</v>
+        <v>107488</v>
       </c>
       <c r="B15" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="D15" s="11">
-        <v>45944</v>
+        <v>45440</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F15" s="3">
         <v>0</v>
@@ -1434,10 +1587,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>20161.64</v>
+        <v>4851.87</v>
       </c>
       <c r="I15" s="4">
-        <v>20161.64</v>
+        <v>4851.87</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1446,39 +1599,39 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>42989.9</v>
+        <v>159802.49</v>
       </c>
       <c r="M15" s="4">
-        <v>42989.9</v>
+        <v>159802.49</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>115404</v>
+        <v>113076</v>
       </c>
       <c r="B16" s="2">
         <v>2043</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D16" s="11">
-        <v>45986</v>
+        <v>45806</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F16" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" s="4">
-        <v>1981.57</v>
+        <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>15334.37</v>
+        <v>4524.1099999999997</v>
       </c>
       <c r="I16" s="4">
-        <v>17315.939999999999</v>
+        <v>4524.1099999999997</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1487,27 +1640,27 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>45330.52</v>
+        <v>13572.34</v>
       </c>
       <c r="M16" s="4">
-        <v>45330.52</v>
+        <v>13572.34</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>81618</v>
+        <v>108405</v>
       </c>
       <c r="B17" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D17" s="11">
-        <v>43447</v>
+        <v>45471</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F17" s="3">
         <v>0</v>
@@ -1516,10 +1669,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>14949.86</v>
+        <v>4475.29</v>
       </c>
       <c r="I17" s="4">
-        <v>14949.86</v>
+        <v>4475.29</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1528,27 +1681,27 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>14949.86</v>
+        <v>37991</v>
       </c>
       <c r="M17" s="4">
-        <v>14949.86</v>
+        <v>37991</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>110575</v>
+        <v>104343</v>
       </c>
       <c r="B18" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D18" s="11">
-        <v>45583</v>
+        <v>45201</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F18" s="3">
         <v>0</v>
@@ -1557,10 +1710,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>14277.28</v>
+        <v>4424.0600000000004</v>
       </c>
       <c r="I18" s="4">
-        <v>14277.28</v>
+        <v>4424.0600000000004</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1569,27 +1722,27 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>114218.2</v>
+        <v>43343.73</v>
       </c>
       <c r="M18" s="4">
-        <v>114218.2</v>
+        <v>43343.73</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>105696</v>
+        <v>104750</v>
       </c>
       <c r="B19" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D19" s="11">
-        <v>45279</v>
+        <v>45236</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F19" s="3">
         <v>0</v>
@@ -1598,39 +1751,39 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>12844.22</v>
+        <v>4419.92</v>
       </c>
       <c r="I19" s="4">
-        <v>12844.22</v>
+        <v>4419.92</v>
       </c>
       <c r="J19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19" s="4">
-        <v>0</v>
+        <v>2072.5100000000002</v>
       </c>
       <c r="L19" s="4">
-        <v>31290.400000000001</v>
+        <v>66328.12</v>
       </c>
       <c r="M19" s="4">
-        <v>31290.400000000001</v>
+        <v>68400.63</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>111056</v>
+        <v>108404</v>
       </c>
       <c r="B20" s="2">
         <v>2692</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D20" s="11">
-        <v>45639</v>
+        <v>45467</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F20" s="3">
         <v>0</v>
@@ -1639,10 +1792,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>11995.43</v>
+        <v>4237.95</v>
       </c>
       <c r="I20" s="4">
-        <v>11995.43</v>
+        <v>4237.95</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1651,27 +1804,27 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>66593.55</v>
+        <v>44602.41</v>
       </c>
       <c r="M20" s="4">
-        <v>66593.55</v>
+        <v>44602.41</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>114431</v>
+        <v>88234</v>
       </c>
       <c r="B21" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="D21" s="11">
-        <v>45930</v>
+        <v>43794</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F21" s="3">
         <v>0</v>
@@ -1680,10 +1833,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>9754.2000000000007</v>
+        <v>4210.32</v>
       </c>
       <c r="I21" s="4">
-        <v>9754.2000000000007</v>
+        <v>4210.32</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1692,27 +1845,27 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>53809.919999999998</v>
+        <v>19836.599999999999</v>
       </c>
       <c r="M21" s="4">
-        <v>53809.919999999998</v>
+        <v>19836.599999999999</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>102825</v>
+        <v>116060</v>
       </c>
       <c r="B22" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="D22" s="11">
-        <v>45117</v>
+        <v>46010</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F22" s="3">
         <v>0</v>
@@ -1721,10 +1874,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>9729.5300000000007</v>
+        <v>3165</v>
       </c>
       <c r="I22" s="4">
-        <v>9729.5300000000007</v>
+        <v>3165</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1733,27 +1886,27 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>24959.51</v>
+        <v>44057.32</v>
       </c>
       <c r="M22" s="4">
-        <v>24959.51</v>
+        <v>44057.32</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>80925</v>
+        <v>47116</v>
       </c>
       <c r="B23" s="2">
         <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D23" s="11">
-        <v>43439</v>
+        <v>44616</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F23" s="3">
         <v>0</v>
@@ -1762,10 +1915,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>9411.2000000000007</v>
+        <v>3133.99</v>
       </c>
       <c r="I23" s="4">
-        <v>9411.2000000000007</v>
+        <v>3133.99</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1774,39 +1927,39 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>5119.8</v>
+        <v>91983.31</v>
       </c>
       <c r="M23" s="4">
-        <v>5119.8</v>
+        <v>91983.31</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>108405</v>
+        <v>106018</v>
       </c>
       <c r="B24" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="D24" s="11">
-        <v>45471</v>
+        <v>45344</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F24" s="3">
         <v>0</v>
       </c>
       <c r="G24" s="4">
-        <v>-6.98</v>
+        <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>9017.2000000000007</v>
+        <v>3075.71</v>
       </c>
       <c r="I24" s="4">
-        <v>9010.2199999999993</v>
+        <v>3075.71</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1815,27 +1968,27 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>13898.44</v>
+        <v>25066.53</v>
       </c>
       <c r="M24" s="4">
-        <v>13898.44</v>
+        <v>25066.53</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>110105</v>
+        <v>65046</v>
       </c>
       <c r="B25" s="2">
         <v>2043</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="D25" s="11">
-        <v>45560</v>
+        <v>44763</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F25" s="3">
         <v>0</v>
@@ -1844,10 +1997,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>8858.33</v>
+        <v>2759.08</v>
       </c>
       <c r="I25" s="4">
-        <v>8858.33</v>
+        <v>2759.08</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -1856,27 +2009,27 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>11320.23</v>
+        <v>20012.810000000001</v>
       </c>
       <c r="M25" s="4">
-        <v>11320.23</v>
+        <v>20012.810000000001</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>101640</v>
+        <v>114100</v>
       </c>
       <c r="B26" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D26" s="11">
-        <v>45104</v>
+        <v>45863</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F26" s="3">
         <v>0</v>
@@ -1885,10 +2038,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>8735.75</v>
+        <v>2391.88</v>
       </c>
       <c r="I26" s="4">
-        <v>8735.75</v>
+        <v>2391.88</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -1897,27 +2050,27 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>0</v>
+        <v>55439.85</v>
       </c>
       <c r="M26" s="4">
-        <v>0</v>
+        <v>55439.85</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>100677</v>
+        <v>101640</v>
       </c>
       <c r="B27" s="2">
         <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="D27" s="11">
-        <v>44999</v>
+        <v>45104</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F27" s="3">
         <v>0</v>
@@ -1926,51 +2079,51 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>8446.18</v>
+        <v>2316.9899999999998</v>
       </c>
       <c r="I27" s="4">
-        <v>8446.18</v>
+        <v>2316.9899999999998</v>
       </c>
       <c r="J27" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" s="4">
-        <v>24232.54</v>
+        <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>23672.25</v>
+        <v>5546.81</v>
       </c>
       <c r="M27" s="4">
-        <v>47904.79</v>
+        <v>5546.81</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>116060</v>
+        <v>116876</v>
       </c>
       <c r="B28" s="2">
         <v>2856</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D28" s="11">
-        <v>46010</v>
+        <v>46006</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F28" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G28" s="4">
-        <v>1816.78</v>
+        <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>6612.15</v>
+        <v>2005.37</v>
       </c>
       <c r="I28" s="4">
-        <v>8428.93</v>
+        <v>2005.37</v>
       </c>
       <c r="J28" s="3">
         <v>0</v>
@@ -1979,39 +2132,39 @@
         <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>42738.89</v>
+        <v>20053.7</v>
       </c>
       <c r="M28" s="4">
-        <v>42738.89</v>
+        <v>20053.7</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>94156</v>
+        <v>102825</v>
       </c>
       <c r="B29" s="2">
         <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="D29" s="11">
-        <v>44159</v>
+        <v>45117</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F29" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G29" s="4">
-        <v>2310.19</v>
+        <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>4435.79</v>
+        <v>1742.75</v>
       </c>
       <c r="I29" s="4">
-        <v>6745.98</v>
+        <v>1742.75</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2020,27 +2173,27 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>0</v>
+        <v>23216.76</v>
       </c>
       <c r="M29" s="4">
-        <v>0</v>
+        <v>23216.76</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>112522</v>
+        <v>105696</v>
       </c>
       <c r="B30" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="D30" s="11">
-        <v>45776</v>
+        <v>45279</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F30" s="3">
         <v>0</v>
@@ -2049,10 +2202,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>6667.5</v>
+        <v>1719.39</v>
       </c>
       <c r="I30" s="4">
-        <v>6667.5</v>
+        <v>1719.39</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2061,27 +2214,27 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>8371.91</v>
+        <v>38126.730000000003</v>
       </c>
       <c r="M30" s="4">
-        <v>8371.91</v>
+        <v>38126.730000000003</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>114157</v>
+        <v>100677</v>
       </c>
       <c r="B31" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D31" s="11">
-        <v>45904</v>
+        <v>44999</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F31" s="3">
         <v>0</v>
@@ -2090,39 +2243,39 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>6490.94</v>
+        <v>1693.49</v>
       </c>
       <c r="I31" s="4">
-        <v>6490.94</v>
+        <v>1693.49</v>
       </c>
       <c r="J31" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K31" s="4">
-        <v>0</v>
+        <v>24232.54</v>
       </c>
       <c r="L31" s="4">
-        <v>61000.91</v>
+        <v>36490.53</v>
       </c>
       <c r="M31" s="4">
-        <v>61000.91</v>
+        <v>60723.07</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>95148</v>
+        <v>109007</v>
       </c>
       <c r="B32" s="2">
         <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D32" s="11">
-        <v>44916</v>
+        <v>45525</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F32" s="3">
         <v>0</v>
@@ -2131,10 +2284,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>6222.75</v>
+        <v>853.76</v>
       </c>
       <c r="I32" s="4">
-        <v>6222.75</v>
+        <v>853.76</v>
       </c>
       <c r="J32" s="3">
         <v>0</v>
@@ -2143,27 +2296,27 @@
         <v>0</v>
       </c>
       <c r="L32" s="4">
-        <v>0</v>
+        <v>1331.18</v>
       </c>
       <c r="M32" s="4">
-        <v>0</v>
+        <v>1331.18</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>109007</v>
+        <v>115404</v>
       </c>
       <c r="B33" s="2">
         <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="D33" s="11">
-        <v>45525</v>
+        <v>45986</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F33" s="3">
         <v>0</v>
@@ -2172,10 +2325,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>6150.74</v>
+        <v>653.92999999999995</v>
       </c>
       <c r="I33" s="4">
-        <v>6150.74</v>
+        <v>653.92999999999995</v>
       </c>
       <c r="J33" s="3">
         <v>0</v>
@@ -2184,27 +2337,27 @@
         <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>0</v>
+        <v>45330.52</v>
       </c>
       <c r="M33" s="4">
-        <v>0</v>
+        <v>45330.52</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>106018</v>
+        <v>116795</v>
       </c>
       <c r="B34" s="2">
         <v>2043</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D34" s="11">
-        <v>45344</v>
+        <v>46000</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F34" s="3">
         <v>0</v>
@@ -2213,10 +2366,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>5769.79</v>
+        <v>0</v>
       </c>
       <c r="I34" s="4">
-        <v>5769.79</v>
+        <v>0</v>
       </c>
       <c r="J34" s="3">
         <v>0</v>
@@ -2225,27 +2378,27 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>22590.41</v>
+        <v>4746.34</v>
       </c>
       <c r="M34" s="4">
-        <v>22590.41</v>
+        <v>4746.34</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>90177</v>
+        <v>114431</v>
       </c>
       <c r="B35" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D35" s="11">
-        <v>43949</v>
+        <v>45930</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F35" s="3">
         <v>0</v>
@@ -2254,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="4">
-        <v>5160.08</v>
+        <v>0</v>
       </c>
       <c r="I35" s="4">
-        <v>5160.08</v>
+        <v>0</v>
       </c>
       <c r="J35" s="3">
         <v>0</v>
@@ -2266,27 +2419,27 @@
         <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>10320.16</v>
+        <v>61795.28</v>
       </c>
       <c r="M35" s="4">
-        <v>10320.16</v>
+        <v>61795.28</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>114100</v>
+        <v>112522</v>
       </c>
       <c r="B36" s="2">
         <v>2856</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="D36" s="11">
-        <v>45863</v>
+        <v>45776</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F36" s="3">
         <v>0</v>
@@ -2295,10 +2448,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="4">
-        <v>4506.41</v>
+        <v>0</v>
       </c>
       <c r="I36" s="4">
-        <v>4506.41</v>
+        <v>0</v>
       </c>
       <c r="J36" s="3">
         <v>0</v>
@@ -2307,27 +2460,27 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>38370.230000000003</v>
+        <v>8371.91</v>
       </c>
       <c r="M36" s="4">
-        <v>38370.230000000003</v>
+        <v>8371.91</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>108658</v>
+        <v>110575</v>
       </c>
       <c r="B37" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D37" s="11">
-        <v>45497</v>
+        <v>45583</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F37" s="3">
         <v>0</v>
@@ -2336,10 +2489,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="4">
-        <v>4403.49</v>
+        <v>0</v>
       </c>
       <c r="I37" s="4">
-        <v>4403.49</v>
+        <v>0</v>
       </c>
       <c r="J37" s="3">
         <v>0</v>
@@ -2348,27 +2501,27 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>0</v>
+        <v>114218.2</v>
       </c>
       <c r="M37" s="4">
-        <v>0</v>
+        <v>114218.2</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>113076</v>
+        <v>110105</v>
       </c>
       <c r="B38" s="2">
         <v>2043</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D38" s="11">
-        <v>45806</v>
+        <v>45560</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F38" s="3">
         <v>0</v>
@@ -2377,10 +2530,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="4">
-        <v>4337.79</v>
+        <v>0</v>
       </c>
       <c r="I38" s="4">
-        <v>4337.79</v>
+        <v>0</v>
       </c>
       <c r="J38" s="3">
         <v>0</v>
@@ -2389,27 +2542,27 @@
         <v>0</v>
       </c>
       <c r="L38" s="4">
-        <v>18096.46</v>
+        <v>16578.8</v>
       </c>
       <c r="M38" s="4">
-        <v>18096.46</v>
+        <v>16578.8</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>88234</v>
+        <v>109998</v>
       </c>
       <c r="B39" s="2">
         <v>2043</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="D39" s="11">
-        <v>43794</v>
+        <v>45596</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F39" s="3">
         <v>0</v>
@@ -2418,10 +2571,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="4">
-        <v>4210.32</v>
+        <v>0</v>
       </c>
       <c r="I39" s="4">
-        <v>4210.32</v>
+        <v>0</v>
       </c>
       <c r="J39" s="3">
         <v>0</v>
@@ -2430,68 +2583,68 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>24046.91</v>
+        <v>7370.69</v>
       </c>
       <c r="M39" s="4">
-        <v>24046.91</v>
+        <v>7370.69</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>116883</v>
+        <v>108658</v>
       </c>
       <c r="B40" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="D40" s="11">
-        <v>46007</v>
+        <v>45497</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G40" s="4">
-        <v>2572.19</v>
+        <v>0</v>
       </c>
       <c r="H40" s="4">
-        <v>1438.55</v>
+        <v>0</v>
       </c>
       <c r="I40" s="4">
-        <v>4010.74</v>
+        <v>0</v>
       </c>
       <c r="J40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K40" s="4">
-        <v>5187.54</v>
+        <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>21463.65</v>
+        <v>1558.85</v>
       </c>
       <c r="M40" s="4">
-        <v>26651.19</v>
+        <v>1558.85</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>116795</v>
+        <v>95148</v>
       </c>
       <c r="B41" s="2">
         <v>2043</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="D41" s="11">
-        <v>46000</v>
+        <v>44916</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F41" s="3">
         <v>0</v>
@@ -2500,10 +2653,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="4">
-        <v>3164.3</v>
+        <v>0</v>
       </c>
       <c r="I41" s="4">
-        <v>3164.3</v>
+        <v>0</v>
       </c>
       <c r="J41" s="3">
         <v>0</v>
@@ -2512,27 +2665,27 @@
         <v>0</v>
       </c>
       <c r="L41" s="4">
-        <v>0</v>
+        <v>3858.2</v>
       </c>
       <c r="M41" s="4">
-        <v>0</v>
+        <v>3858.2</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>104343</v>
+        <v>94156</v>
       </c>
       <c r="B42" s="2">
         <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="D42" s="11">
-        <v>45201</v>
+        <v>44159</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F42" s="3">
         <v>0</v>
@@ -2541,10 +2694,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="4">
-        <v>3017.9</v>
+        <v>0</v>
       </c>
       <c r="I42" s="4">
-        <v>3017.9</v>
+        <v>0</v>
       </c>
       <c r="J42" s="3">
         <v>0</v>
@@ -2553,27 +2706,27 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>44819.11</v>
+        <v>7582.41</v>
       </c>
       <c r="M42" s="4">
-        <v>44819.11</v>
+        <v>7582.41</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>109998</v>
+        <v>90355</v>
       </c>
       <c r="B43" s="2">
         <v>2043</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D43" s="11">
-        <v>45596</v>
+        <v>43949</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F43" s="3">
         <v>0</v>
@@ -2582,39 +2735,39 @@
         <v>0</v>
       </c>
       <c r="H43" s="4">
-        <v>2844.92</v>
+        <v>0</v>
       </c>
       <c r="I43" s="4">
-        <v>2844.92</v>
+        <v>0</v>
       </c>
       <c r="J43" s="3">
         <v>1</v>
       </c>
       <c r="K43" s="4">
-        <v>28702.080000000002</v>
+        <v>73149.789999999994</v>
       </c>
       <c r="L43" s="4">
-        <v>4525.75</v>
+        <v>45845.07</v>
       </c>
       <c r="M43" s="4">
-        <v>33227.83</v>
+        <v>118994.86</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>63441</v>
+        <v>90177</v>
       </c>
       <c r="B44" s="2">
-        <v>2511</v>
+        <v>2043</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D44" s="11">
-        <v>44733</v>
+        <v>43949</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F44" s="3">
         <v>0</v>
@@ -2623,10 +2776,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="4">
-        <v>1827.5</v>
+        <v>0</v>
       </c>
       <c r="I44" s="4">
-        <v>1827.5</v>
+        <v>0</v>
       </c>
       <c r="J44" s="3">
         <v>0</v>
@@ -2635,27 +2788,27 @@
         <v>0</v>
       </c>
       <c r="L44" s="4">
-        <v>10965.01</v>
+        <v>10320.16</v>
       </c>
       <c r="M44" s="4">
-        <v>10965.01</v>
+        <v>10320.16</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
-        <v>65046</v>
+        <v>81618</v>
       </c>
       <c r="B45" s="2">
         <v>2043</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="D45" s="11">
-        <v>44763</v>
+        <v>43447</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F45" s="3">
         <v>0</v>
@@ -2664,10 +2817,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="4">
-        <v>1729.15</v>
+        <v>0</v>
       </c>
       <c r="I45" s="4">
-        <v>1729.15</v>
+        <v>0</v>
       </c>
       <c r="J45" s="3">
         <v>0</v>
@@ -2676,27 +2829,27 @@
         <v>0</v>
       </c>
       <c r="L45" s="4">
-        <v>22771.9</v>
+        <v>14949.86</v>
       </c>
       <c r="M45" s="4">
-        <v>22771.9</v>
+        <v>14949.86</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
-        <v>111960</v>
+        <v>63441</v>
       </c>
       <c r="B46" s="2">
-        <v>2856</v>
+        <v>2511</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="D46" s="11">
-        <v>45707</v>
+        <v>44733</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F46" s="3">
         <v>0</v>
@@ -2705,10 +2858,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="4">
-        <v>1719.21</v>
+        <v>0</v>
       </c>
       <c r="I46" s="4">
-        <v>1719.21</v>
+        <v>0</v>
       </c>
       <c r="J46" s="3">
         <v>0</v>
@@ -2717,27 +2870,27 @@
         <v>0</v>
       </c>
       <c r="L46" s="4">
-        <v>0</v>
+        <v>10965.01</v>
       </c>
       <c r="M46" s="4">
-        <v>0</v>
+        <v>10965.01</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
-        <v>117440</v>
+        <v>113450</v>
       </c>
       <c r="B47" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>56</v>
+        <v>21</v>
       </c>
       <c r="D47" s="11">
-        <v>46059</v>
+        <v>45852</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F47" s="3">
         <v>0</v>
@@ -2746,116 +2899,122 @@
         <v>0</v>
       </c>
       <c r="H47" s="4">
-        <v>0</v>
+        <v>-16394.27</v>
       </c>
       <c r="I47" s="4">
-        <v>0</v>
+        <v>-16394.27</v>
       </c>
       <c r="J47" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K47" s="4">
-        <v>2445.87</v>
+        <v>0</v>
       </c>
       <c r="L47" s="4">
-        <v>0</v>
+        <v>8694.17</v>
       </c>
       <c r="M47" s="4">
-        <v>2445.87</v>
+        <v>8694.17</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A48" s="2">
-        <v>94205</v>
-      </c>
-      <c r="B48" s="2">
-        <v>2043</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D48" s="11">
-        <v>44116</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F48" s="3">
-        <v>0</v>
-      </c>
-      <c r="G48" s="4">
-        <v>0</v>
-      </c>
-      <c r="H48" s="4">
-        <v>0</v>
-      </c>
-      <c r="I48" s="4">
-        <v>0</v>
-      </c>
-      <c r="J48" s="3">
-        <v>0</v>
-      </c>
-      <c r="K48" s="4">
-        <v>0</v>
-      </c>
-      <c r="L48" s="4">
-        <v>10135.31</v>
-      </c>
-      <c r="M48" s="4">
-        <v>10135.31</v>
-      </c>
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="11"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4"/>
+      <c r="I48" s="4"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="4"/>
+      <c r="L48" s="4"/>
+      <c r="M48" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="A4:B4">
-    <cfRule type="expression" dxfId="11" priority="3" stopIfTrue="1">
+  <conditionalFormatting sqref="A48:B48">
+    <cfRule type="expression" dxfId="22" priority="13" stopIfTrue="1">
+      <formula>$S48=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="21" priority="14" stopIfTrue="1">
+      <formula>$S47=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C48:H48 K48:L48">
+    <cfRule type="expression" dxfId="19" priority="18" stopIfTrue="1">
+      <formula>$S48=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="18" priority="19" stopIfTrue="1">
+      <formula>$S47=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I48 M48">
+    <cfRule type="expression" dxfId="16" priority="20" stopIfTrue="1">
+      <formula>$S48=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="21" stopIfTrue="1">
+      <formula>$S47=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J48">
+    <cfRule type="expression" dxfId="13" priority="16" stopIfTrue="1">
+      <formula>$S48=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="12" priority="17" stopIfTrue="1">
+      <formula>$S47=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:A47 J5:J47">
+    <cfRule type="expression" dxfId="11" priority="4" stopIfTrue="1">
+      <formula>$S5=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="5" stopIfTrue="1">
+      <formula>$S4=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K5:L47 C5:H47">
+    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
+      <formula>$S5=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="8" priority="7" stopIfTrue="1">
+      <formula>$S4=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I5:I47 M5:M47">
+    <cfRule type="expression" dxfId="7" priority="8" stopIfTrue="1">
+      <formula>$S5=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="9" stopIfTrue="1">
+      <formula>$S4=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J4 A4">
+    <cfRule type="expression" dxfId="5" priority="10" stopIfTrue="1">
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:B48">
-    <cfRule type="expression" dxfId="10" priority="1" stopIfTrue="1">
-      <formula>$S5=1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="9" priority="2" stopIfTrue="1">
-      <formula>$S4=1</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="C4:H4 K4:L4">
-    <cfRule type="expression" dxfId="8" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="11" stopIfTrue="1">
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C5:H48 K5:L48">
-    <cfRule type="expression" dxfId="7" priority="6" stopIfTrue="1">
-      <formula>$S5=1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="7" stopIfTrue="1">
-      <formula>$S4=1</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="I4 M4">
-    <cfRule type="expression" dxfId="5" priority="12" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="12" stopIfTrue="1">
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I48 M5:M48">
-    <cfRule type="expression" dxfId="4" priority="8" stopIfTrue="1">
-      <formula>$S5=1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="9" stopIfTrue="1">
-      <formula>$S4=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J4">
-    <cfRule type="expression" dxfId="2" priority="10" stopIfTrue="1">
+  <conditionalFormatting sqref="B4">
+    <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J5:J48">
-    <cfRule type="expression" dxfId="1" priority="4" stopIfTrue="1">
+  <conditionalFormatting sqref="B5:B47">
+    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Fix: Clear cache on snapshot and use Mexico City timezone for all logs/captures
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CBE88A1-8BAA-FF47-855B-D64B4D1DB489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D80DA906-8419-1443-8080-CF3338D341FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="57">
   <si>
     <t>Asesor</t>
   </si>
@@ -204,6 +204,9 @@
   </si>
   <si>
     <t>MONSERRAT VELASCO SANTOS</t>
+  </si>
+  <si>
+    <t>5</t>
   </si>
 </sst>
 </file>
@@ -370,7 +373,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="25">
     <dxf>
       <border>
         <top style="thin">
@@ -529,6 +532,22 @@
     </dxf>
     <dxf>
       <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
         <top style="thin">
           <color indexed="64"/>
         </top>
@@ -542,7 +561,7 @@
         <right style="hair">
           <color indexed="64"/>
         </right>
-        <top style="hair">
+        <top style="thin">
           <color indexed="64"/>
         </top>
         <bottom style="hair">
@@ -552,13 +571,13 @@
     </dxf>
     <dxf>
       <border>
-        <left style="thin">
+        <left style="hair">
           <color indexed="64"/>
         </left>
-        <right style="hair">
+        <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="thin">
+        <top style="hair">
           <color indexed="64"/>
         </top>
         <bottom style="hair">
@@ -581,22 +600,6 @@
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
         <top style="thin">
           <color indexed="64"/>
         </top>
@@ -626,6 +629,13 @@
         <bottom style="hair">
           <color indexed="64"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
       </border>
     </dxf>
     <dxf>
@@ -1034,7 +1044,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1130,28 +1140,28 @@
         <v>54</v>
       </c>
       <c r="F4" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G4" s="4">
-        <v>0</v>
+        <v>327363.81</v>
       </c>
       <c r="H4" s="4">
         <v>67732.53</v>
       </c>
       <c r="I4" s="4">
-        <v>67732.53</v>
+        <v>395096.34</v>
       </c>
       <c r="J4" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K4" s="4">
-        <v>327363.81</v>
+        <v>0</v>
       </c>
       <c r="L4" s="4">
         <v>279799.13</v>
       </c>
       <c r="M4" s="4">
-        <v>607162.93999999994</v>
+        <v>279799.13</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1218,10 +1228,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="4">
-        <v>17733.23</v>
+        <v>19759.79</v>
       </c>
       <c r="I6" s="4">
-        <v>17733.23</v>
+        <v>19759.79</v>
       </c>
       <c r="J6" s="3">
         <v>1</v>
@@ -1320,57 +1330,57 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>80122</v>
+        <v>104750</v>
       </c>
       <c r="B9" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="D9" s="11">
-        <v>43371</v>
+        <v>45236</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F9" s="3">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>0</v>
+      </c>
+      <c r="H9" s="4">
+        <v>9657.42</v>
+      </c>
+      <c r="I9" s="4">
+        <v>9657.42</v>
+      </c>
+      <c r="J9" s="3">
         <v>1</v>
       </c>
-      <c r="G9" s="4">
-        <v>2550.13</v>
-      </c>
-      <c r="H9" s="4">
-        <v>4599.88</v>
-      </c>
-      <c r="I9" s="4">
-        <v>7150.01</v>
-      </c>
-      <c r="J9" s="3">
-        <v>0</v>
-      </c>
       <c r="K9" s="4">
-        <v>0</v>
+        <v>2072.5100000000002</v>
       </c>
       <c r="L9" s="4">
-        <v>104245.15</v>
+        <v>59042.879999999997</v>
       </c>
       <c r="M9" s="4">
-        <v>104245.15</v>
+        <v>61115.39</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>114157</v>
+        <v>108405</v>
       </c>
       <c r="B10" s="2">
         <v>2692</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="D10" s="11">
-        <v>45904</v>
+        <v>45471</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>54</v>
@@ -1382,10 +1392,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="4">
-        <v>5489.13</v>
+        <v>7485.18</v>
       </c>
       <c r="I10" s="4">
-        <v>5489.13</v>
+        <v>7485.18</v>
       </c>
       <c r="J10" s="3">
         <v>0</v>
@@ -1394,39 +1404,39 @@
         <v>0</v>
       </c>
       <c r="L10" s="4">
-        <v>57999.18</v>
+        <v>34981.11</v>
       </c>
       <c r="M10" s="4">
-        <v>57999.18</v>
+        <v>34981.11</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>111056</v>
+        <v>80122</v>
       </c>
       <c r="B11" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="D11" s="11">
-        <v>45639</v>
+        <v>43371</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F11" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" s="4">
-        <v>0</v>
+        <v>2550.13</v>
       </c>
       <c r="H11" s="4">
-        <v>5403.95</v>
+        <v>4599.88</v>
       </c>
       <c r="I11" s="4">
-        <v>5403.95</v>
+        <v>7150.01</v>
       </c>
       <c r="J11" s="3">
         <v>0</v>
@@ -1435,65 +1445,65 @@
         <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>61189.599999999999</v>
+        <v>104245.15</v>
       </c>
       <c r="M11" s="4">
-        <v>61189.599999999999</v>
+        <v>104245.15</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>116883</v>
+        <v>107488</v>
       </c>
       <c r="B12" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D12" s="11">
-        <v>46007</v>
+        <v>45440</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F12" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" s="4">
-        <v>5187.54</v>
+        <v>0</v>
       </c>
       <c r="H12" s="4">
-        <v>0</v>
+        <v>6570.73</v>
       </c>
       <c r="I12" s="4">
-        <v>5187.54</v>
+        <v>6570.73</v>
       </c>
       <c r="J12" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" s="4">
-        <v>1820.53</v>
+        <v>0</v>
       </c>
       <c r="L12" s="4">
-        <v>45347.65</v>
+        <v>158083.63</v>
       </c>
       <c r="M12" s="4">
-        <v>47168.18</v>
+        <v>158083.63</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>80925</v>
+        <v>108404</v>
       </c>
       <c r="B13" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="D13" s="11">
-        <v>43439</v>
+        <v>45467</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>54</v>
@@ -1505,10 +1515,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="4">
-        <v>5119.8</v>
+        <v>5851.31</v>
       </c>
       <c r="I13" s="4">
-        <v>5119.8</v>
+        <v>5851.31</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1517,39 +1527,39 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>10061.92</v>
+        <v>42989.04</v>
       </c>
       <c r="M13" s="4">
-        <v>10061.92</v>
+        <v>42989.04</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>117440</v>
+        <v>114157</v>
       </c>
       <c r="B14" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="D14" s="11">
-        <v>46059</v>
+        <v>45904</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F14" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G14" s="4">
-        <v>3011.72</v>
+        <v>0</v>
       </c>
       <c r="H14" s="4">
-        <v>1975.99</v>
+        <v>5489.13</v>
       </c>
       <c r="I14" s="4">
-        <v>4987.71</v>
+        <v>5489.13</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1558,24 +1568,24 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>0</v>
+        <v>57999.18</v>
       </c>
       <c r="M14" s="4">
-        <v>0</v>
+        <v>57999.18</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>107488</v>
+        <v>111056</v>
       </c>
       <c r="B15" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="D15" s="11">
-        <v>45440</v>
+        <v>45639</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>54</v>
@@ -1587,10 +1597,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>4851.87</v>
+        <v>5403.95</v>
       </c>
       <c r="I15" s="4">
-        <v>4851.87</v>
+        <v>5403.95</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1599,65 +1609,65 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>159802.49</v>
+        <v>61189.599999999999</v>
       </c>
       <c r="M15" s="4">
-        <v>159802.49</v>
+        <v>61189.599999999999</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>113076</v>
+        <v>116883</v>
       </c>
       <c r="B16" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D16" s="11">
-        <v>45806</v>
+        <v>46007</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F16" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="4">
-        <v>0</v>
+        <v>5187.54</v>
       </c>
       <c r="H16" s="4">
-        <v>4524.1099999999997</v>
+        <v>0</v>
       </c>
       <c r="I16" s="4">
-        <v>4524.1099999999997</v>
+        <v>5187.54</v>
       </c>
       <c r="J16" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" s="4">
-        <v>0</v>
+        <v>1820.53</v>
       </c>
       <c r="L16" s="4">
-        <v>13572.34</v>
+        <v>45347.65</v>
       </c>
       <c r="M16" s="4">
-        <v>13572.34</v>
+        <v>47168.18</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>108405</v>
+        <v>80925</v>
       </c>
       <c r="B17" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D17" s="11">
-        <v>45471</v>
+        <v>43439</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>54</v>
@@ -1669,10 +1679,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>4475.29</v>
+        <v>5119.8</v>
       </c>
       <c r="I17" s="4">
-        <v>4475.29</v>
+        <v>5119.8</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1681,65 +1691,65 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>37991</v>
+        <v>10061.92</v>
       </c>
       <c r="M17" s="4">
-        <v>37991</v>
+        <v>10061.92</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>104343</v>
+        <v>117440</v>
       </c>
       <c r="B18" s="2">
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="D18" s="11">
-        <v>45201</v>
+        <v>46059</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F18" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G18" s="4">
-        <v>0</v>
+        <v>3011.72</v>
       </c>
       <c r="H18" s="4">
-        <v>4424.0600000000004</v>
+        <v>1975.99</v>
       </c>
       <c r="I18" s="4">
-        <v>4424.0600000000004</v>
+        <v>4987.71</v>
       </c>
       <c r="J18" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" s="4">
-        <v>0</v>
+        <v>4931.22</v>
       </c>
       <c r="L18" s="4">
-        <v>43343.73</v>
+        <v>0</v>
       </c>
       <c r="M18" s="4">
-        <v>43343.73</v>
+        <v>4931.22</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>104750</v>
+        <v>113076</v>
       </c>
       <c r="B19" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="D19" s="11">
-        <v>45236</v>
+        <v>45806</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>54</v>
@@ -1751,36 +1761,36 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>4419.92</v>
+        <v>4524.1099999999997</v>
       </c>
       <c r="I19" s="4">
-        <v>4419.92</v>
+        <v>4524.1099999999997</v>
       </c>
       <c r="J19" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K19" s="4">
-        <v>2072.5100000000002</v>
+        <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>66328.12</v>
+        <v>13572.34</v>
       </c>
       <c r="M19" s="4">
-        <v>68400.63</v>
+        <v>13572.34</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>108404</v>
+        <v>104343</v>
       </c>
       <c r="B20" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D20" s="11">
-        <v>45467</v>
+        <v>45201</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>54</v>
@@ -1792,10 +1802,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>4237.95</v>
+        <v>4424.0600000000004</v>
       </c>
       <c r="I20" s="4">
-        <v>4237.95</v>
+        <v>4424.0600000000004</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1804,10 +1814,10 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>44602.41</v>
+        <v>43343.73</v>
       </c>
       <c r="M20" s="4">
-        <v>44602.41</v>
+        <v>43343.73</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
@@ -1853,16 +1863,16 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>116060</v>
+        <v>100677</v>
       </c>
       <c r="B22" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D22" s="11">
-        <v>46010</v>
+        <v>44999</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>54</v>
@@ -1874,36 +1884,36 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>3165</v>
+        <v>3921.11</v>
       </c>
       <c r="I22" s="4">
-        <v>3165</v>
+        <v>3921.11</v>
       </c>
       <c r="J22" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22" s="4">
-        <v>0</v>
+        <v>24232.54</v>
       </c>
       <c r="L22" s="4">
-        <v>44057.32</v>
+        <v>34262.92</v>
       </c>
       <c r="M22" s="4">
-        <v>44057.32</v>
+        <v>58495.46</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>47116</v>
+        <v>116060</v>
       </c>
       <c r="B23" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="D23" s="11">
-        <v>44616</v>
+        <v>46010</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>54</v>
@@ -1915,10 +1925,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>3133.99</v>
+        <v>3165</v>
       </c>
       <c r="I23" s="4">
-        <v>3133.99</v>
+        <v>3165</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1927,24 +1937,24 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>91983.31</v>
+        <v>44057.32</v>
       </c>
       <c r="M23" s="4">
-        <v>91983.31</v>
+        <v>44057.32</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>106018</v>
+        <v>47116</v>
       </c>
       <c r="B24" s="2">
         <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="D24" s="11">
-        <v>45344</v>
+        <v>44616</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>54</v>
@@ -1956,10 +1966,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>3075.71</v>
+        <v>3133.99</v>
       </c>
       <c r="I24" s="4">
-        <v>3075.71</v>
+        <v>3133.99</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1968,24 +1978,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>25066.53</v>
+        <v>91983.31</v>
       </c>
       <c r="M24" s="4">
-        <v>25066.53</v>
+        <v>91983.31</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>65046</v>
+        <v>106018</v>
       </c>
       <c r="B25" s="2">
         <v>2043</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D25" s="11">
-        <v>44763</v>
+        <v>45344</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>54</v>
@@ -1997,10 +2007,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>2759.08</v>
+        <v>3075.71</v>
       </c>
       <c r="I25" s="4">
-        <v>2759.08</v>
+        <v>3075.71</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -2009,24 +2019,24 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>20012.810000000001</v>
+        <v>25066.53</v>
       </c>
       <c r="M25" s="4">
-        <v>20012.810000000001</v>
+        <v>25066.53</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>114100</v>
+        <v>65046</v>
       </c>
       <c r="B26" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D26" s="11">
-        <v>45863</v>
+        <v>44763</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>54</v>
@@ -2038,10 +2048,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>2391.88</v>
+        <v>2759.08</v>
       </c>
       <c r="I26" s="4">
-        <v>2391.88</v>
+        <v>2759.08</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2050,24 +2060,24 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>55439.85</v>
+        <v>20012.810000000001</v>
       </c>
       <c r="M26" s="4">
-        <v>55439.85</v>
+        <v>20012.810000000001</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>101640</v>
+        <v>114100</v>
       </c>
       <c r="B27" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D27" s="11">
-        <v>45104</v>
+        <v>45863</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>54</v>
@@ -2079,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>2316.9899999999998</v>
+        <v>2391.88</v>
       </c>
       <c r="I27" s="4">
-        <v>2316.9899999999998</v>
+        <v>2391.88</v>
       </c>
       <c r="J27" s="3">
         <v>0</v>
@@ -2091,24 +2101,24 @@
         <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>5546.81</v>
+        <v>55439.85</v>
       </c>
       <c r="M27" s="4">
-        <v>5546.81</v>
+        <v>55439.85</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>116876</v>
+        <v>101640</v>
       </c>
       <c r="B28" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="D28" s="11">
-        <v>46006</v>
+        <v>45104</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>54</v>
@@ -2120,10 +2130,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>2005.37</v>
+        <v>2316.9899999999998</v>
       </c>
       <c r="I28" s="4">
-        <v>2005.37</v>
+        <v>2316.9899999999998</v>
       </c>
       <c r="J28" s="3">
         <v>0</v>
@@ -2132,24 +2142,24 @@
         <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>20053.7</v>
+        <v>5546.81</v>
       </c>
       <c r="M28" s="4">
-        <v>20053.7</v>
+        <v>5546.81</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>102825</v>
+        <v>116876</v>
       </c>
       <c r="B29" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="D29" s="11">
-        <v>45117</v>
+        <v>46006</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>54</v>
@@ -2161,10 +2171,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>1742.75</v>
+        <v>2005.37</v>
       </c>
       <c r="I29" s="4">
-        <v>1742.75</v>
+        <v>2005.37</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2173,24 +2183,24 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>23216.76</v>
+        <v>20053.7</v>
       </c>
       <c r="M29" s="4">
-        <v>23216.76</v>
+        <v>20053.7</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>105696</v>
+        <v>102825</v>
       </c>
       <c r="B30" s="2">
         <v>2043</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="D30" s="11">
-        <v>45279</v>
+        <v>45117</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>54</v>
@@ -2202,10 +2212,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>1719.39</v>
+        <v>1742.75</v>
       </c>
       <c r="I30" s="4">
-        <v>1719.39</v>
+        <v>1742.75</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2214,24 +2224,24 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>38126.730000000003</v>
+        <v>23216.76</v>
       </c>
       <c r="M30" s="4">
-        <v>38126.730000000003</v>
+        <v>23216.76</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>100677</v>
+        <v>105696</v>
       </c>
       <c r="B31" s="2">
         <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D31" s="11">
-        <v>44999</v>
+        <v>45279</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>54</v>
@@ -2243,22 +2253,22 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>1693.49</v>
+        <v>1719.39</v>
       </c>
       <c r="I31" s="4">
-        <v>1693.49</v>
+        <v>1719.39</v>
       </c>
       <c r="J31" s="3">
         <v>1</v>
       </c>
       <c r="K31" s="4">
-        <v>24232.54</v>
+        <v>30470.73</v>
       </c>
       <c r="L31" s="4">
-        <v>36490.53</v>
+        <v>38126.730000000003</v>
       </c>
       <c r="M31" s="4">
-        <v>60723.07</v>
+        <v>68597.460000000006</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
@@ -2357,7 +2367,7 @@
         <v>46000</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F34" s="3">
         <v>0</v>
@@ -2935,10 +2945,10 @@
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="A48:B48">
-    <cfRule type="expression" dxfId="22" priority="13" stopIfTrue="1">
+    <cfRule type="expression" dxfId="23" priority="13" stopIfTrue="1">
       <formula>$S48=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="14" stopIfTrue="1">
+    <cfRule type="expression" dxfId="22" priority="14" stopIfTrue="1">
       <formula>$S47=1</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2946,24 +2956,20 @@
     <cfRule type="expression" dxfId="19" priority="18" stopIfTrue="1">
       <formula>$S48=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="19" stopIfTrue="1">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C48:M48">
+    <cfRule type="expression" dxfId="18" priority="29" stopIfTrue="1">
       <formula>$S47=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I48 M48">
-    <cfRule type="expression" dxfId="16" priority="20" stopIfTrue="1">
+    <cfRule type="expression" dxfId="15" priority="20" stopIfTrue="1">
       <formula>$S48=1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="15" priority="21" stopIfTrue="1">
-      <formula>$S47=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J48">
-    <cfRule type="expression" dxfId="13" priority="16" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="16" stopIfTrue="1">
       <formula>$S48=1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="12" priority="17" stopIfTrue="1">
-      <formula>$S47=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:A47 J5:J47">

</xml_diff>

<commit_message>
data: update Estatus de Pólizas report - 2026-03-18
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C46E9DEE-6E2B-EA40-B063-7B0E0514123A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C1A5D7-8881-0246-8740-3CDE2C798D32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="58">
   <si>
     <t>Asesor</t>
   </si>
@@ -207,6 +207,9 @@
   </si>
   <si>
     <t>5</t>
+  </si>
+  <si>
+    <t>4</t>
   </si>
 </sst>
 </file>
@@ -1044,7 +1047,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46093</v>
+        <v>46097</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1146,22 +1149,22 @@
         <v>327363.81</v>
       </c>
       <c r="H4" s="4">
-        <v>67732.53</v>
+        <v>70292.42</v>
       </c>
       <c r="I4" s="4">
-        <v>395096.34</v>
+        <v>397656.23</v>
       </c>
       <c r="J4" s="5">
         <v>1</v>
       </c>
       <c r="K4" s="4">
-        <v>20861.689999999999</v>
+        <v>63872.52</v>
       </c>
       <c r="L4" s="4">
-        <v>300660.82</v>
+        <v>343671.65</v>
       </c>
       <c r="M4" s="4">
-        <v>321522.51</v>
+        <v>407544.17</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1207,57 +1210,57 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>115047</v>
+        <v>104718</v>
       </c>
       <c r="B6" s="2">
-        <v>2856</v>
+        <v>2692</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D6" s="11">
-        <v>45944</v>
+        <v>45264</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F6" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="4">
-        <v>0</v>
+        <v>13028.98</v>
       </c>
       <c r="H6" s="4">
-        <v>19759.79</v>
+        <v>12271.64</v>
       </c>
       <c r="I6" s="4">
-        <v>19759.79</v>
+        <v>25300.62</v>
       </c>
       <c r="J6" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" s="4">
-        <v>24502.57</v>
+        <v>0</v>
       </c>
       <c r="L6" s="4">
-        <v>34641.980000000003</v>
+        <v>114527.16</v>
       </c>
       <c r="M6" s="4">
-        <v>59144.55</v>
+        <v>114527.16</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>104718</v>
+        <v>115047</v>
       </c>
       <c r="B7" s="2">
-        <v>2692</v>
+        <v>2856</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D7" s="11">
-        <v>45264</v>
+        <v>45944</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>54</v>
@@ -1269,77 +1272,77 @@
         <v>0</v>
       </c>
       <c r="H7" s="4">
-        <v>12271.64</v>
+        <v>19759.79</v>
       </c>
       <c r="I7" s="4">
-        <v>12271.64</v>
+        <v>19759.79</v>
       </c>
       <c r="J7" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7" s="4">
-        <v>0</v>
+        <v>24502.57</v>
       </c>
       <c r="L7" s="4">
-        <v>101498.18</v>
+        <v>34641.980000000003</v>
       </c>
       <c r="M7" s="4">
-        <v>101498.18</v>
+        <v>59144.55</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>104750</v>
+        <v>80122</v>
       </c>
       <c r="B8" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D8" s="11">
-        <v>45236</v>
+        <v>43371</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="4">
-        <v>0</v>
+        <v>2550.13</v>
       </c>
       <c r="H8" s="4">
-        <v>11995.77</v>
+        <v>10621.13</v>
       </c>
       <c r="I8" s="4">
-        <v>11995.77</v>
+        <v>13171.26</v>
       </c>
       <c r="J8" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" s="4">
-        <v>2072.5100000000002</v>
+        <v>0</v>
       </c>
       <c r="L8" s="4">
-        <v>59042.879999999997</v>
+        <v>98223.89</v>
       </c>
       <c r="M8" s="4">
-        <v>61115.39</v>
+        <v>98223.89</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>94205</v>
+        <v>107488</v>
       </c>
       <c r="B9" s="2">
         <v>2043</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="D9" s="11">
-        <v>44116</v>
+        <v>45440</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>54</v>
@@ -1351,10 +1354,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="4">
-        <v>10135.31</v>
+        <v>12622.15</v>
       </c>
       <c r="I9" s="4">
-        <v>10135.31</v>
+        <v>12622.15</v>
       </c>
       <c r="J9" s="3">
         <v>0</v>
@@ -1363,24 +1366,24 @@
         <v>0</v>
       </c>
       <c r="L9" s="4">
-        <v>0</v>
+        <v>152032.18</v>
       </c>
       <c r="M9" s="4">
-        <v>0</v>
+        <v>152032.18</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>108405</v>
+        <v>104750</v>
       </c>
       <c r="B10" s="2">
         <v>2692</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="D10" s="11">
-        <v>45471</v>
+        <v>45236</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>54</v>
@@ -1392,51 +1395,51 @@
         <v>0</v>
       </c>
       <c r="H10" s="4">
-        <v>7485.18</v>
+        <v>11995.77</v>
       </c>
       <c r="I10" s="4">
-        <v>7485.18</v>
+        <v>11995.77</v>
       </c>
       <c r="J10" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" s="4">
-        <v>0</v>
+        <v>2072.5100000000002</v>
       </c>
       <c r="L10" s="4">
-        <v>34981.11</v>
+        <v>59042.879999999997</v>
       </c>
       <c r="M10" s="4">
-        <v>34981.11</v>
+        <v>61115.39</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>80122</v>
+        <v>116883</v>
       </c>
       <c r="B11" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="D11" s="11">
-        <v>43371</v>
+        <v>46007</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F11" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11" s="4">
-        <v>2550.13</v>
+        <v>7008.07</v>
       </c>
       <c r="H11" s="4">
-        <v>4599.88</v>
+        <v>4010.74</v>
       </c>
       <c r="I11" s="4">
-        <v>7150.01</v>
+        <v>11018.81</v>
       </c>
       <c r="J11" s="3">
         <v>0</v>
@@ -1445,39 +1448,39 @@
         <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>104245.15</v>
+        <v>41489.449999999997</v>
       </c>
       <c r="M11" s="4">
-        <v>104245.15</v>
+        <v>41489.449999999997</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>116883</v>
+        <v>94205</v>
       </c>
       <c r="B12" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="D12" s="11">
-        <v>46007</v>
+        <v>44116</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F12" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G12" s="4">
-        <v>7008.07</v>
+        <v>0</v>
       </c>
       <c r="H12" s="4">
-        <v>0</v>
+        <v>10135.31</v>
       </c>
       <c r="I12" s="4">
-        <v>7008.07</v>
+        <v>10135.31</v>
       </c>
       <c r="J12" s="3">
         <v>0</v>
@@ -1486,39 +1489,39 @@
         <v>0</v>
       </c>
       <c r="L12" s="4">
-        <v>45347.65</v>
+        <v>0</v>
       </c>
       <c r="M12" s="4">
-        <v>45347.65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>107488</v>
+        <v>117440</v>
       </c>
       <c r="B13" s="2">
         <v>2043</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="D13" s="11">
-        <v>45440</v>
+        <v>46059</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F13" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G13" s="4">
-        <v>0</v>
+        <v>5692.2</v>
       </c>
       <c r="H13" s="4">
-        <v>6570.73</v>
+        <v>4226.8900000000003</v>
       </c>
       <c r="I13" s="4">
-        <v>6570.73</v>
+        <v>9919.09</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1527,24 +1530,24 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>158083.63</v>
+        <v>0</v>
       </c>
       <c r="M13" s="4">
-        <v>158083.63</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>108404</v>
+        <v>108405</v>
       </c>
       <c r="B14" s="2">
         <v>2692</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="D14" s="11">
-        <v>45467</v>
+        <v>45471</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>54</v>
@@ -1556,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="4">
-        <v>5851.31</v>
+        <v>7485.18</v>
       </c>
       <c r="I14" s="4">
-        <v>5851.31</v>
+        <v>7485.18</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1568,10 +1571,10 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>42989.04</v>
+        <v>34981.11</v>
       </c>
       <c r="M14" s="4">
-        <v>42989.04</v>
+        <v>34981.11</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
@@ -1597,10 +1600,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>5489.13</v>
+        <v>7114.26</v>
       </c>
       <c r="I15" s="4">
-        <v>5489.13</v>
+        <v>7114.26</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1609,24 +1612,24 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>57999.18</v>
+        <v>56374.05</v>
       </c>
       <c r="M15" s="4">
-        <v>57999.18</v>
+        <v>56374.05</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>111056</v>
+        <v>108404</v>
       </c>
       <c r="B16" s="2">
         <v>2692</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D16" s="11">
-        <v>45639</v>
+        <v>45467</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>54</v>
@@ -1638,10 +1641,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>5403.95</v>
+        <v>5851.31</v>
       </c>
       <c r="I16" s="4">
-        <v>5403.95</v>
+        <v>5851.31</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1650,24 +1653,24 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>61189.599999999999</v>
+        <v>42989.04</v>
       </c>
       <c r="M16" s="4">
-        <v>61189.599999999999</v>
+        <v>42989.04</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>80925</v>
+        <v>111056</v>
       </c>
       <c r="B17" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="D17" s="11">
-        <v>43439</v>
+        <v>45639</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>54</v>
@@ -1679,10 +1682,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>5119.8</v>
+        <v>5403.95</v>
       </c>
       <c r="I17" s="4">
-        <v>5119.8</v>
+        <v>5403.95</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1691,65 +1694,65 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>10061.92</v>
+        <v>61189.599999999999</v>
       </c>
       <c r="M17" s="4">
-        <v>10061.92</v>
+        <v>61189.599999999999</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>117440</v>
+        <v>90177</v>
       </c>
       <c r="B18" s="2">
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="D18" s="11">
-        <v>46059</v>
+        <v>43949</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F18" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G18" s="4">
-        <v>3011.72</v>
+        <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>1975.99</v>
+        <v>5160.08</v>
       </c>
       <c r="I18" s="4">
-        <v>4987.71</v>
+        <v>5160.08</v>
       </c>
       <c r="J18" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" s="4">
-        <v>4931.22</v>
+        <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>0</v>
+        <v>5160.08</v>
       </c>
       <c r="M18" s="4">
-        <v>4931.22</v>
+        <v>5160.08</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>113076</v>
+        <v>80925</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="D19" s="11">
-        <v>45806</v>
+        <v>43439</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>54</v>
@@ -1761,10 +1764,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>4524.1099999999997</v>
+        <v>5119.8</v>
       </c>
       <c r="I19" s="4">
-        <v>4524.1099999999997</v>
+        <v>5119.8</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1773,24 +1776,24 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>13572.34</v>
+        <v>10061.92</v>
       </c>
       <c r="M19" s="4">
-        <v>13572.34</v>
+        <v>10061.92</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>104343</v>
+        <v>113076</v>
       </c>
       <c r="B20" s="2">
         <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D20" s="11">
-        <v>45201</v>
+        <v>45806</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>54</v>
@@ -1802,10 +1805,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>4424.0600000000004</v>
+        <v>4524.1099999999997</v>
       </c>
       <c r="I20" s="4">
-        <v>4424.0600000000004</v>
+        <v>4524.1099999999997</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1814,24 +1817,24 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>43343.73</v>
+        <v>13572.34</v>
       </c>
       <c r="M20" s="4">
-        <v>43343.73</v>
+        <v>13572.34</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>88234</v>
+        <v>104343</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D21" s="11">
-        <v>43794</v>
+        <v>45201</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>54</v>
@@ -1843,10 +1846,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>4210.32</v>
+        <v>4424.0600000000004</v>
       </c>
       <c r="I21" s="4">
-        <v>4210.32</v>
+        <v>4424.0600000000004</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1855,24 +1858,24 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>19836.599999999999</v>
+        <v>43343.73</v>
       </c>
       <c r="M21" s="4">
-        <v>19836.599999999999</v>
+        <v>43343.73</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>100677</v>
+        <v>88234</v>
       </c>
       <c r="B22" s="2">
         <v>2043</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="D22" s="11">
-        <v>44999</v>
+        <v>43794</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>54</v>
@@ -1884,36 +1887,36 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>3921.11</v>
+        <v>4210.32</v>
       </c>
       <c r="I22" s="4">
-        <v>3921.11</v>
+        <v>4210.32</v>
       </c>
       <c r="J22" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K22" s="4">
-        <v>24232.54</v>
+        <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>34262.92</v>
+        <v>19836.599999999999</v>
       </c>
       <c r="M22" s="4">
-        <v>58495.46</v>
+        <v>19836.599999999999</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>114100</v>
+        <v>100677</v>
       </c>
       <c r="B23" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D23" s="11">
-        <v>45863</v>
+        <v>44999</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>54</v>
@@ -1925,36 +1928,36 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>3336.41</v>
+        <v>3921.11</v>
       </c>
       <c r="I23" s="4">
-        <v>3336.41</v>
+        <v>3921.11</v>
       </c>
       <c r="J23" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" s="4">
-        <v>0</v>
+        <v>24232.54</v>
       </c>
       <c r="L23" s="4">
-        <v>55439.85</v>
+        <v>34262.92</v>
       </c>
       <c r="M23" s="4">
-        <v>55439.85</v>
+        <v>58495.46</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>116060</v>
+        <v>114100</v>
       </c>
       <c r="B24" s="2">
         <v>2856</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="D24" s="11">
-        <v>46010</v>
+        <v>45863</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>54</v>
@@ -1966,10 +1969,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>3165</v>
+        <v>3336.41</v>
       </c>
       <c r="I24" s="4">
-        <v>3165</v>
+        <v>3336.41</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1978,24 +1981,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>44057.32</v>
+        <v>55439.85</v>
       </c>
       <c r="M24" s="4">
-        <v>44057.32</v>
+        <v>55439.85</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>47116</v>
+        <v>116060</v>
       </c>
       <c r="B25" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="D25" s="11">
-        <v>44616</v>
+        <v>46010</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>54</v>
@@ -2007,10 +2010,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>3133.99</v>
+        <v>3165</v>
       </c>
       <c r="I25" s="4">
-        <v>3133.99</v>
+        <v>3165</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -2019,24 +2022,24 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>91983.31</v>
+        <v>44057.32</v>
       </c>
       <c r="M25" s="4">
-        <v>91983.31</v>
+        <v>44057.32</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>106018</v>
+        <v>47116</v>
       </c>
       <c r="B26" s="2">
         <v>2043</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="D26" s="11">
-        <v>45344</v>
+        <v>44616</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>54</v>
@@ -2048,10 +2051,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>3075.71</v>
+        <v>3133.99</v>
       </c>
       <c r="I26" s="4">
-        <v>3075.71</v>
+        <v>3133.99</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2060,24 +2063,24 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>25066.53</v>
+        <v>91983.31</v>
       </c>
       <c r="M26" s="4">
-        <v>25066.53</v>
+        <v>91983.31</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>65046</v>
+        <v>106018</v>
       </c>
       <c r="B27" s="2">
         <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D27" s="11">
-        <v>44763</v>
+        <v>45344</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>54</v>
@@ -2089,36 +2092,36 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>2759.08</v>
+        <v>3075.71</v>
       </c>
       <c r="I27" s="4">
-        <v>2759.08</v>
+        <v>3075.71</v>
       </c>
       <c r="J27" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" s="4">
-        <v>0</v>
+        <v>2842.67</v>
       </c>
       <c r="L27" s="4">
-        <v>20012.810000000001</v>
+        <v>25066.53</v>
       </c>
       <c r="M27" s="4">
-        <v>20012.810000000001</v>
+        <v>27909.200000000001</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>101640</v>
+        <v>65046</v>
       </c>
       <c r="B28" s="2">
         <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="D28" s="11">
-        <v>45104</v>
+        <v>44763</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>54</v>
@@ -2130,10 +2133,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>2316.9899999999998</v>
+        <v>2759.08</v>
       </c>
       <c r="I28" s="4">
-        <v>2316.9899999999998</v>
+        <v>2759.08</v>
       </c>
       <c r="J28" s="3">
         <v>0</v>
@@ -2142,24 +2145,24 @@
         <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>5546.81</v>
+        <v>20012.810000000001</v>
       </c>
       <c r="M28" s="4">
-        <v>5546.81</v>
+        <v>20012.810000000001</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>116876</v>
+        <v>101640</v>
       </c>
       <c r="B29" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="D29" s="11">
-        <v>46006</v>
+        <v>45104</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>54</v>
@@ -2171,10 +2174,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>2005.37</v>
+        <v>2316.9899999999998</v>
       </c>
       <c r="I29" s="4">
-        <v>2005.37</v>
+        <v>2316.9899999999998</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2183,24 +2186,24 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>20053.7</v>
+        <v>5546.81</v>
       </c>
       <c r="M29" s="4">
-        <v>20053.7</v>
+        <v>5546.81</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>102825</v>
+        <v>116876</v>
       </c>
       <c r="B30" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="D30" s="11">
-        <v>45117</v>
+        <v>46006</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>54</v>
@@ -2212,10 +2215,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>1742.75</v>
+        <v>2005.37</v>
       </c>
       <c r="I30" s="4">
-        <v>1742.75</v>
+        <v>2005.37</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2224,24 +2227,24 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>23216.76</v>
+        <v>20053.7</v>
       </c>
       <c r="M30" s="4">
-        <v>23216.76</v>
+        <v>20053.7</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>105696</v>
+        <v>102825</v>
       </c>
       <c r="B31" s="2">
         <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="D31" s="11">
-        <v>45279</v>
+        <v>45117</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>54</v>
@@ -2253,36 +2256,36 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>1719.39</v>
+        <v>1742.75</v>
       </c>
       <c r="I31" s="4">
-        <v>1719.39</v>
+        <v>1742.75</v>
       </c>
       <c r="J31" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K31" s="4">
-        <v>30470.73</v>
+        <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>38126.730000000003</v>
+        <v>23216.76</v>
       </c>
       <c r="M31" s="4">
-        <v>68597.460000000006</v>
+        <v>23216.76</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>109007</v>
+        <v>105696</v>
       </c>
       <c r="B32" s="2">
         <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="D32" s="11">
-        <v>45525</v>
+        <v>45279</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>54</v>
@@ -2294,36 +2297,36 @@
         <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>853.76</v>
+        <v>1719.39</v>
       </c>
       <c r="I32" s="4">
-        <v>853.76</v>
+        <v>1719.39</v>
       </c>
       <c r="J32" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K32" s="4">
-        <v>0</v>
+        <v>30470.73</v>
       </c>
       <c r="L32" s="4">
-        <v>1331.18</v>
+        <v>38126.730000000003</v>
       </c>
       <c r="M32" s="4">
-        <v>1331.18</v>
+        <v>68597.460000000006</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>115404</v>
+        <v>109007</v>
       </c>
       <c r="B33" s="2">
         <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="D33" s="11">
-        <v>45986</v>
+        <v>45525</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>54</v>
@@ -2335,10 +2338,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>653.92999999999995</v>
+        <v>853.76</v>
       </c>
       <c r="I33" s="4">
-        <v>653.92999999999995</v>
+        <v>853.76</v>
       </c>
       <c r="J33" s="3">
         <v>0</v>
@@ -2347,27 +2350,27 @@
         <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>45330.52</v>
+        <v>1331.18</v>
       </c>
       <c r="M33" s="4">
-        <v>45330.52</v>
+        <v>1331.18</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>116795</v>
+        <v>115404</v>
       </c>
       <c r="B34" s="2">
         <v>2043</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D34" s="11">
-        <v>46000</v>
+        <v>45986</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F34" s="3">
         <v>0</v>
@@ -2376,10 +2379,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>0</v>
+        <v>653.92999999999995</v>
       </c>
       <c r="I34" s="4">
-        <v>0</v>
+        <v>653.92999999999995</v>
       </c>
       <c r="J34" s="3">
         <v>0</v>
@@ -2388,27 +2391,27 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>4746.34</v>
+        <v>45330.52</v>
       </c>
       <c r="M34" s="4">
-        <v>4746.34</v>
+        <v>45330.52</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>114431</v>
+        <v>116795</v>
       </c>
       <c r="B35" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D35" s="11">
-        <v>45930</v>
+        <v>46000</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F35" s="3">
         <v>0</v>
@@ -2429,24 +2432,24 @@
         <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>61795.28</v>
+        <v>4746.34</v>
       </c>
       <c r="M35" s="4">
-        <v>61795.28</v>
+        <v>4746.34</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>112522</v>
+        <v>114431</v>
       </c>
       <c r="B36" s="2">
-        <v>2856</v>
+        <v>2692</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D36" s="11">
-        <v>45776</v>
+        <v>45930</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>54</v>
@@ -2470,24 +2473,24 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>8371.91</v>
+        <v>61795.28</v>
       </c>
       <c r="M36" s="4">
-        <v>8371.91</v>
+        <v>61795.28</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>110575</v>
+        <v>112522</v>
       </c>
       <c r="B37" s="2">
-        <v>2692</v>
+        <v>2856</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D37" s="11">
-        <v>45583</v>
+        <v>45776</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>54</v>
@@ -2511,24 +2514,24 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>114218.2</v>
+        <v>8371.91</v>
       </c>
       <c r="M37" s="4">
-        <v>114218.2</v>
+        <v>8371.91</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>110105</v>
+        <v>110575</v>
       </c>
       <c r="B38" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D38" s="11">
-        <v>45560</v>
+        <v>45583</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>54</v>
@@ -2552,24 +2555,24 @@
         <v>0</v>
       </c>
       <c r="L38" s="4">
-        <v>16578.8</v>
+        <v>114218.2</v>
       </c>
       <c r="M38" s="4">
-        <v>16578.8</v>
+        <v>114218.2</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>109998</v>
+        <v>110105</v>
       </c>
       <c r="B39" s="2">
         <v>2043</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D39" s="11">
-        <v>45596</v>
+        <v>45560</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>54</v>
@@ -2593,24 +2596,24 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>7370.69</v>
+        <v>16578.8</v>
       </c>
       <c r="M39" s="4">
-        <v>7370.69</v>
+        <v>16578.8</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>108658</v>
+        <v>109998</v>
       </c>
       <c r="B40" s="2">
         <v>2043</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D40" s="11">
-        <v>45497</v>
+        <v>45596</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>54</v>
@@ -2634,24 +2637,24 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>1558.85</v>
+        <v>2844.94</v>
       </c>
       <c r="M40" s="4">
-        <v>1558.85</v>
+        <v>2844.94</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>95148</v>
+        <v>108658</v>
       </c>
       <c r="B41" s="2">
         <v>2043</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D41" s="11">
-        <v>44916</v>
+        <v>45497</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>54</v>
@@ -2675,24 +2678,24 @@
         <v>0</v>
       </c>
       <c r="L41" s="4">
-        <v>3858.2</v>
+        <v>1558.85</v>
       </c>
       <c r="M41" s="4">
-        <v>3858.2</v>
+        <v>1558.85</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>94156</v>
+        <v>95148</v>
       </c>
       <c r="B42" s="2">
         <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D42" s="11">
-        <v>44159</v>
+        <v>44916</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>54</v>
@@ -2716,24 +2719,24 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>7582.41</v>
+        <v>3858.2</v>
       </c>
       <c r="M42" s="4">
-        <v>7582.41</v>
+        <v>3858.2</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>90355</v>
+        <v>94156</v>
       </c>
       <c r="B43" s="2">
         <v>2043</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D43" s="11">
-        <v>43949</v>
+        <v>44159</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>54</v>
@@ -2751,27 +2754,27 @@
         <v>0</v>
       </c>
       <c r="J43" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K43" s="4">
-        <v>73149.789999999994</v>
+        <v>0</v>
       </c>
       <c r="L43" s="4">
-        <v>45845.07</v>
+        <v>7582.41</v>
       </c>
       <c r="M43" s="4">
-        <v>118994.86</v>
+        <v>7582.41</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>90177</v>
+        <v>90355</v>
       </c>
       <c r="B44" s="2">
         <v>2043</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D44" s="11">
         <v>43949</v>
@@ -2792,16 +2795,16 @@
         <v>0</v>
       </c>
       <c r="J44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K44" s="4">
-        <v>0</v>
+        <v>73149.789999999994</v>
       </c>
       <c r="L44" s="4">
-        <v>10320.16</v>
+        <v>45845.07</v>
       </c>
       <c r="M44" s="4">
-        <v>10320.16</v>
+        <v>118994.86</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
@@ -2818,7 +2821,7 @@
         <v>43447</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F45" s="3">
         <v>0</v>
@@ -2958,7 +2961,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48:M48">
-    <cfRule type="expression" dxfId="18" priority="41" stopIfTrue="1">
+    <cfRule type="expression" dxfId="18" priority="53" stopIfTrue="1">
       <formula>$S47=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
fix: activity tracking on admin login and db path check, refresh snapshot
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C1A5D7-8881-0246-8740-3CDE2C798D32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5A7A9D8-525C-0B45-9C5F-BDD0920C6CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="59">
   <si>
     <t>Asesor</t>
   </si>
@@ -210,6 +210,9 @@
   </si>
   <si>
     <t>4</t>
+  </si>
+  <si>
+    <t>KAREN MUÐOZ GARCIA</t>
   </si>
 </sst>
 </file>
@@ -1047,7 +1050,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46097</v>
+        <v>46100</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1143,28 +1146,28 @@
         <v>54</v>
       </c>
       <c r="F4" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4" s="4">
-        <v>327363.81</v>
+        <v>391236.33</v>
       </c>
       <c r="H4" s="4">
         <v>70292.42</v>
       </c>
       <c r="I4" s="4">
-        <v>397656.23</v>
+        <v>461528.75</v>
       </c>
       <c r="J4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" s="4">
-        <v>63872.52</v>
+        <v>0</v>
       </c>
       <c r="L4" s="4">
         <v>343671.65</v>
       </c>
       <c r="M4" s="4">
-        <v>407544.17</v>
+        <v>343671.65</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1190,10 +1193,10 @@
         <v>1840.93</v>
       </c>
       <c r="H5" s="4">
-        <v>59500.38</v>
+        <v>76322.12</v>
       </c>
       <c r="I5" s="4">
-        <v>61341.31</v>
+        <v>78163.05</v>
       </c>
       <c r="J5" s="3">
         <v>1</v>
@@ -1202,24 +1205,24 @@
         <v>1770.92</v>
       </c>
       <c r="L5" s="4">
-        <v>185723.9</v>
+        <v>181909.6</v>
       </c>
       <c r="M5" s="4">
-        <v>187494.82</v>
+        <v>183680.52</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>104718</v>
+        <v>115047</v>
       </c>
       <c r="B6" s="2">
-        <v>2692</v>
+        <v>2856</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D6" s="11">
-        <v>45264</v>
+        <v>45944</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>54</v>
@@ -1228,13 +1231,13 @@
         <v>1</v>
       </c>
       <c r="G6" s="4">
-        <v>13028.98</v>
+        <v>1488.25</v>
       </c>
       <c r="H6" s="4">
-        <v>12271.64</v>
+        <v>42774.11</v>
       </c>
       <c r="I6" s="4">
-        <v>25300.62</v>
+        <v>44262.36</v>
       </c>
       <c r="J6" s="3">
         <v>0</v>
@@ -1243,80 +1246,80 @@
         <v>0</v>
       </c>
       <c r="L6" s="4">
-        <v>114527.16</v>
+        <v>34641.980000000003</v>
       </c>
       <c r="M6" s="4">
-        <v>114527.16</v>
+        <v>34641.980000000003</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>115047</v>
+        <v>104750</v>
       </c>
       <c r="B7" s="2">
-        <v>2856</v>
+        <v>2692</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D7" s="11">
-        <v>45944</v>
+        <v>45236</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F7" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" s="4">
-        <v>0</v>
+        <v>-3520.38</v>
       </c>
       <c r="H7" s="4">
-        <v>19759.79</v>
+        <v>39264.269999999997</v>
       </c>
       <c r="I7" s="4">
-        <v>19759.79</v>
+        <v>35743.89</v>
       </c>
       <c r="J7" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" s="4">
-        <v>24502.57</v>
+        <v>37848.660000000003</v>
       </c>
       <c r="L7" s="4">
-        <v>34641.980000000003</v>
+        <v>61941.82</v>
       </c>
       <c r="M7" s="4">
-        <v>59144.55</v>
+        <v>99790.48</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>80122</v>
+        <v>107488</v>
       </c>
       <c r="B8" s="2">
         <v>2043</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="D8" s="11">
-        <v>43371</v>
+        <v>45440</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F8" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" s="4">
-        <v>2550.13</v>
+        <v>0</v>
       </c>
       <c r="H8" s="4">
-        <v>10621.13</v>
+        <v>32610.63</v>
       </c>
       <c r="I8" s="4">
-        <v>13171.26</v>
+        <v>32610.63</v>
       </c>
       <c r="J8" s="3">
         <v>0</v>
@@ -1325,39 +1328,39 @@
         <v>0</v>
       </c>
       <c r="L8" s="4">
-        <v>98223.89</v>
+        <v>132043.74</v>
       </c>
       <c r="M8" s="4">
-        <v>98223.89</v>
+        <v>132043.74</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>107488</v>
+        <v>104718</v>
       </c>
       <c r="B9" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="D9" s="11">
-        <v>45440</v>
+        <v>45264</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F9" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="4">
-        <v>0</v>
+        <v>13028.98</v>
       </c>
       <c r="H9" s="4">
-        <v>12622.15</v>
+        <v>18442.25</v>
       </c>
       <c r="I9" s="4">
-        <v>12622.15</v>
+        <v>31471.23</v>
       </c>
       <c r="J9" s="3">
         <v>0</v>
@@ -1366,80 +1369,80 @@
         <v>0</v>
       </c>
       <c r="L9" s="4">
-        <v>152032.18</v>
+        <v>108356.53</v>
       </c>
       <c r="M9" s="4">
-        <v>152032.18</v>
+        <v>108356.53</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>104750</v>
+        <v>80122</v>
       </c>
       <c r="B10" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="D10" s="11">
-        <v>45236</v>
+        <v>43371</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F10" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="4">
-        <v>0</v>
+        <v>2550.13</v>
       </c>
       <c r="H10" s="4">
-        <v>11995.77</v>
+        <v>12339.99</v>
       </c>
       <c r="I10" s="4">
-        <v>11995.77</v>
+        <v>14890.12</v>
       </c>
       <c r="J10" s="3">
         <v>1</v>
       </c>
       <c r="K10" s="4">
-        <v>2072.5100000000002</v>
+        <v>97248.01</v>
       </c>
       <c r="L10" s="4">
-        <v>59042.879999999997</v>
+        <v>96505.02</v>
       </c>
       <c r="M10" s="4">
-        <v>61115.39</v>
+        <v>193753.03</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>116883</v>
+        <v>90355</v>
       </c>
       <c r="B11" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="D11" s="11">
-        <v>46007</v>
+        <v>43949</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F11" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G11" s="4">
-        <v>7008.07</v>
+        <v>0</v>
       </c>
       <c r="H11" s="4">
-        <v>4010.74</v>
+        <v>13410.43</v>
       </c>
       <c r="I11" s="4">
-        <v>11018.81</v>
+        <v>13410.43</v>
       </c>
       <c r="J11" s="3">
         <v>0</v>
@@ -1448,24 +1451,24 @@
         <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>41489.449999999997</v>
+        <v>32434.68</v>
       </c>
       <c r="M11" s="4">
-        <v>41489.449999999997</v>
+        <v>32434.68</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>94205</v>
+        <v>114157</v>
       </c>
       <c r="B12" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="D12" s="11">
-        <v>44116</v>
+        <v>45904</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>54</v>
@@ -1477,51 +1480,51 @@
         <v>0</v>
       </c>
       <c r="H12" s="4">
-        <v>10135.31</v>
+        <v>13292.63</v>
       </c>
       <c r="I12" s="4">
-        <v>10135.31</v>
+        <v>13292.63</v>
       </c>
       <c r="J12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" s="4">
-        <v>0</v>
+        <v>1684.95</v>
       </c>
       <c r="L12" s="4">
-        <v>0</v>
+        <v>68730.09</v>
       </c>
       <c r="M12" s="4">
-        <v>0</v>
+        <v>70415.039999999994</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>117440</v>
+        <v>116883</v>
       </c>
       <c r="B13" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="D13" s="11">
-        <v>46059</v>
+        <v>46007</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F13" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G13" s="4">
-        <v>5692.2</v>
+        <v>7008.07</v>
       </c>
       <c r="H13" s="4">
-        <v>4226.8900000000003</v>
+        <v>4010.74</v>
       </c>
       <c r="I13" s="4">
-        <v>9919.09</v>
+        <v>11018.81</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1530,24 +1533,24 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>0</v>
+        <v>41489.449999999997</v>
       </c>
       <c r="M13" s="4">
-        <v>0</v>
+        <v>41489.449999999997</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>108405</v>
+        <v>94205</v>
       </c>
       <c r="B14" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="D14" s="11">
-        <v>45471</v>
+        <v>44116</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>54</v>
@@ -1559,10 +1562,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="4">
-        <v>7485.18</v>
+        <v>10135.31</v>
       </c>
       <c r="I14" s="4">
-        <v>7485.18</v>
+        <v>10135.31</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1571,39 +1574,39 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>34981.11</v>
+        <v>0</v>
       </c>
       <c r="M14" s="4">
-        <v>34981.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>114157</v>
+        <v>117440</v>
       </c>
       <c r="B15" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="D15" s="11">
-        <v>45904</v>
+        <v>46059</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F15" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G15" s="4">
-        <v>0</v>
+        <v>5692.2</v>
       </c>
       <c r="H15" s="4">
-        <v>7114.26</v>
+        <v>4226.8900000000003</v>
       </c>
       <c r="I15" s="4">
-        <v>7114.26</v>
+        <v>9919.09</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1612,39 +1615,39 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>56374.05</v>
+        <v>0</v>
       </c>
       <c r="M15" s="4">
-        <v>56374.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>108404</v>
+        <v>106018</v>
       </c>
       <c r="B16" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D16" s="11">
-        <v>45467</v>
+        <v>45344</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F16" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="4">
-        <v>0</v>
+        <v>580.95000000000005</v>
       </c>
       <c r="H16" s="4">
-        <v>5851.31</v>
+        <v>8612.6200000000008</v>
       </c>
       <c r="I16" s="4">
-        <v>5851.31</v>
+        <v>9193.57</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1653,24 +1656,24 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>42989.04</v>
+        <v>22590.41</v>
       </c>
       <c r="M16" s="4">
-        <v>42989.04</v>
+        <v>22590.41</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>111056</v>
+        <v>110105</v>
       </c>
       <c r="B17" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="D17" s="11">
-        <v>45639</v>
+        <v>45560</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>54</v>
@@ -1682,10 +1685,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>5403.95</v>
+        <v>8858.33</v>
       </c>
       <c r="I17" s="4">
-        <v>5403.95</v>
+        <v>8858.33</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1694,24 +1697,24 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>61189.599999999999</v>
+        <v>7719.98</v>
       </c>
       <c r="M17" s="4">
-        <v>61189.599999999999</v>
+        <v>7719.98</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>90177</v>
+        <v>114100</v>
       </c>
       <c r="B18" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="D18" s="11">
-        <v>43949</v>
+        <v>45863</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>54</v>
@@ -1723,10 +1726,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>5160.08</v>
+        <v>8427.17</v>
       </c>
       <c r="I18" s="4">
-        <v>5160.08</v>
+        <v>8427.17</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1735,24 +1738,24 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>5160.08</v>
+        <v>53325.32</v>
       </c>
       <c r="M18" s="4">
-        <v>5160.08</v>
+        <v>53325.32</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>80925</v>
+        <v>108405</v>
       </c>
       <c r="B19" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D19" s="11">
-        <v>43439</v>
+        <v>45471</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>54</v>
@@ -1764,10 +1767,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>5119.8</v>
+        <v>7485.18</v>
       </c>
       <c r="I19" s="4">
-        <v>5119.8</v>
+        <v>7485.18</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1776,24 +1779,24 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>10061.92</v>
+        <v>34981.11</v>
       </c>
       <c r="M19" s="4">
-        <v>10061.92</v>
+        <v>34981.11</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>113076</v>
+        <v>100677</v>
       </c>
       <c r="B20" s="2">
         <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D20" s="11">
-        <v>45806</v>
+        <v>44999</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>54</v>
@@ -1805,10 +1808,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>4524.1099999999997</v>
+        <v>6339.76</v>
       </c>
       <c r="I20" s="4">
-        <v>4524.1099999999997</v>
+        <v>6339.76</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1817,24 +1820,24 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>13572.34</v>
+        <v>19751.150000000001</v>
       </c>
       <c r="M20" s="4">
-        <v>13572.34</v>
+        <v>19751.150000000001</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>104343</v>
+        <v>105696</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D21" s="11">
-        <v>45201</v>
+        <v>45279</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>54</v>
@@ -1846,36 +1849,36 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>4424.0600000000004</v>
+        <v>6285.09</v>
       </c>
       <c r="I21" s="4">
-        <v>4424.0600000000004</v>
+        <v>6285.09</v>
       </c>
       <c r="J21" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21" s="4">
-        <v>0</v>
+        <v>31875.97</v>
       </c>
       <c r="L21" s="4">
-        <v>43343.73</v>
+        <v>30430.65</v>
       </c>
       <c r="M21" s="4">
-        <v>43343.73</v>
+        <v>62306.62</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>88234</v>
+        <v>108404</v>
       </c>
       <c r="B22" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D22" s="11">
-        <v>43794</v>
+        <v>45467</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>54</v>
@@ -1887,10 +1890,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>4210.32</v>
+        <v>5851.31</v>
       </c>
       <c r="I22" s="4">
-        <v>4210.32</v>
+        <v>5851.31</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1899,24 +1902,24 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>19836.599999999999</v>
+        <v>42989.04</v>
       </c>
       <c r="M22" s="4">
-        <v>19836.599999999999</v>
+        <v>42989.04</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>100677</v>
+        <v>111056</v>
       </c>
       <c r="B23" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="D23" s="11">
-        <v>44999</v>
+        <v>45639</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>54</v>
@@ -1928,36 +1931,36 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>3921.11</v>
+        <v>5403.95</v>
       </c>
       <c r="I23" s="4">
-        <v>3921.11</v>
+        <v>5403.95</v>
       </c>
       <c r="J23" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23" s="4">
-        <v>24232.54</v>
+        <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>34262.92</v>
+        <v>61189.599999999999</v>
       </c>
       <c r="M23" s="4">
-        <v>58495.46</v>
+        <v>61189.599999999999</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>114100</v>
+        <v>90177</v>
       </c>
       <c r="B24" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="D24" s="11">
-        <v>45863</v>
+        <v>43949</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>54</v>
@@ -1969,10 +1972,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>3336.41</v>
+        <v>5160.08</v>
       </c>
       <c r="I24" s="4">
-        <v>3336.41</v>
+        <v>5160.08</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1981,24 +1984,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>55439.85</v>
+        <v>5160.08</v>
       </c>
       <c r="M24" s="4">
-        <v>55439.85</v>
+        <v>5160.08</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>116060</v>
+        <v>80925</v>
       </c>
       <c r="B25" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="D25" s="11">
-        <v>46010</v>
+        <v>43439</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>54</v>
@@ -2010,10 +2013,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>3165</v>
+        <v>5119.8</v>
       </c>
       <c r="I25" s="4">
-        <v>3165</v>
+        <v>5119.8</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -2022,24 +2025,24 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>44057.32</v>
+        <v>10061.92</v>
       </c>
       <c r="M25" s="4">
-        <v>44057.32</v>
+        <v>10061.92</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>47116</v>
+        <v>116060</v>
       </c>
       <c r="B26" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="D26" s="11">
-        <v>44616</v>
+        <v>46010</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>54</v>
@@ -2051,10 +2054,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>3133.99</v>
+        <v>4927.55</v>
       </c>
       <c r="I26" s="4">
-        <v>3133.99</v>
+        <v>4927.55</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2063,24 +2066,24 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>91983.31</v>
+        <v>42294.77</v>
       </c>
       <c r="M26" s="4">
-        <v>91983.31</v>
+        <v>42294.77</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>106018</v>
+        <v>113076</v>
       </c>
       <c r="B27" s="2">
         <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="D27" s="11">
-        <v>45344</v>
+        <v>45806</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>54</v>
@@ -2092,36 +2095,36 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>3075.71</v>
+        <v>4524.1099999999997</v>
       </c>
       <c r="I27" s="4">
-        <v>3075.71</v>
+        <v>4524.1099999999997</v>
       </c>
       <c r="J27" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" s="4">
-        <v>2842.67</v>
+        <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>25066.53</v>
+        <v>13572.34</v>
       </c>
       <c r="M27" s="4">
-        <v>27909.200000000001</v>
+        <v>13572.34</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>65046</v>
+        <v>104343</v>
       </c>
       <c r="B28" s="2">
         <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D28" s="11">
-        <v>44763</v>
+        <v>45201</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>54</v>
@@ -2133,10 +2136,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>2759.08</v>
+        <v>4424.0600000000004</v>
       </c>
       <c r="I28" s="4">
-        <v>2759.08</v>
+        <v>4424.0600000000004</v>
       </c>
       <c r="J28" s="3">
         <v>0</v>
@@ -2145,24 +2148,24 @@
         <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>20012.810000000001</v>
+        <v>43343.73</v>
       </c>
       <c r="M28" s="4">
-        <v>20012.810000000001</v>
+        <v>43343.73</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>101640</v>
+        <v>88234</v>
       </c>
       <c r="B29" s="2">
         <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D29" s="11">
-        <v>45104</v>
+        <v>43794</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>54</v>
@@ -2174,10 +2177,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>2316.9899999999998</v>
+        <v>4210.32</v>
       </c>
       <c r="I29" s="4">
-        <v>2316.9899999999998</v>
+        <v>4210.32</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2186,24 +2189,24 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>5546.81</v>
+        <v>19836.599999999999</v>
       </c>
       <c r="M29" s="4">
-        <v>5546.81</v>
+        <v>19836.599999999999</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>116876</v>
+        <v>95148</v>
       </c>
       <c r="B30" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D30" s="11">
-        <v>46006</v>
+        <v>44916</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>54</v>
@@ -2215,10 +2218,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>2005.37</v>
+        <v>3858.24</v>
       </c>
       <c r="I30" s="4">
-        <v>2005.37</v>
+        <v>3858.24</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2227,24 +2230,24 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>20053.7</v>
+        <v>0</v>
       </c>
       <c r="M30" s="4">
-        <v>20053.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>102825</v>
+        <v>47116</v>
       </c>
       <c r="B31" s="2">
         <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="D31" s="11">
-        <v>45117</v>
+        <v>44616</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>54</v>
@@ -2256,10 +2259,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>1742.75</v>
+        <v>3133.99</v>
       </c>
       <c r="I31" s="4">
-        <v>1742.75</v>
+        <v>3133.99</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -2268,24 +2271,24 @@
         <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>23216.76</v>
+        <v>87333.01</v>
       </c>
       <c r="M31" s="4">
-        <v>23216.76</v>
+        <v>87333.01</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>105696</v>
+        <v>109998</v>
       </c>
       <c r="B32" s="2">
         <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="D32" s="11">
-        <v>45279</v>
+        <v>45596</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>54</v>
@@ -2297,36 +2300,36 @@
         <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>1719.39</v>
+        <v>2844.92</v>
       </c>
       <c r="I32" s="4">
-        <v>1719.39</v>
+        <v>2844.92</v>
       </c>
       <c r="J32" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32" s="4">
-        <v>30470.73</v>
+        <v>0</v>
       </c>
       <c r="L32" s="4">
-        <v>38126.730000000003</v>
+        <v>0</v>
       </c>
       <c r="M32" s="4">
-        <v>68597.460000000006</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>109007</v>
+        <v>65046</v>
       </c>
       <c r="B33" s="2">
         <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="D33" s="11">
-        <v>45525</v>
+        <v>44763</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>54</v>
@@ -2338,36 +2341,36 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>853.76</v>
+        <v>2759.08</v>
       </c>
       <c r="I33" s="4">
-        <v>853.76</v>
+        <v>2759.08</v>
       </c>
       <c r="J33" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K33" s="4">
-        <v>0</v>
+        <v>25197.91</v>
       </c>
       <c r="L33" s="4">
-        <v>1331.18</v>
+        <v>20012.810000000001</v>
       </c>
       <c r="M33" s="4">
-        <v>1331.18</v>
+        <v>45210.720000000001</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>115404</v>
+        <v>81044</v>
       </c>
       <c r="B34" s="2">
-        <v>2043</v>
+        <v>2511</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="D34" s="11">
-        <v>45986</v>
+        <v>44872</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>54</v>
@@ -2379,10 +2382,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>653.92999999999995</v>
+        <v>2385.52</v>
       </c>
       <c r="I34" s="4">
-        <v>653.92999999999995</v>
+        <v>2385.52</v>
       </c>
       <c r="J34" s="3">
         <v>0</v>
@@ -2391,27 +2394,27 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>45330.52</v>
+        <v>0</v>
       </c>
       <c r="M34" s="4">
-        <v>45330.52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>116795</v>
+        <v>101640</v>
       </c>
       <c r="B35" s="2">
         <v>2043</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="D35" s="11">
-        <v>46000</v>
+        <v>45104</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F35" s="3">
         <v>0</v>
@@ -2420,10 +2423,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="4">
-        <v>0</v>
+        <v>2316.9899999999998</v>
       </c>
       <c r="I35" s="4">
-        <v>0</v>
+        <v>2316.9899999999998</v>
       </c>
       <c r="J35" s="3">
         <v>0</v>
@@ -2432,24 +2435,24 @@
         <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>4746.34</v>
+        <v>5546.81</v>
       </c>
       <c r="M35" s="4">
-        <v>4746.34</v>
+        <v>5546.81</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>114431</v>
+        <v>109007</v>
       </c>
       <c r="B36" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D36" s="11">
-        <v>45930</v>
+        <v>45525</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>54</v>
@@ -2461,10 +2464,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="4">
-        <v>0</v>
+        <v>2205.21</v>
       </c>
       <c r="I36" s="4">
-        <v>0</v>
+        <v>2205.21</v>
       </c>
       <c r="J36" s="3">
         <v>0</v>
@@ -2473,24 +2476,24 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>61795.28</v>
+        <v>0</v>
       </c>
       <c r="M36" s="4">
-        <v>61795.28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>112522</v>
+        <v>116876</v>
       </c>
       <c r="B37" s="2">
         <v>2856</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D37" s="11">
-        <v>45776</v>
+        <v>46006</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>54</v>
@@ -2502,10 +2505,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="4">
-        <v>0</v>
+        <v>2005.37</v>
       </c>
       <c r="I37" s="4">
-        <v>0</v>
+        <v>2005.37</v>
       </c>
       <c r="J37" s="3">
         <v>0</v>
@@ -2514,24 +2517,24 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>8371.91</v>
+        <v>20053.7</v>
       </c>
       <c r="M37" s="4">
-        <v>8371.91</v>
+        <v>20053.7</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>110575</v>
+        <v>102825</v>
       </c>
       <c r="B38" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="D38" s="11">
-        <v>45583</v>
+        <v>45117</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>54</v>
@@ -2543,10 +2546,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="4">
-        <v>0</v>
+        <v>1742.75</v>
       </c>
       <c r="I38" s="4">
-        <v>0</v>
+        <v>1742.75</v>
       </c>
       <c r="J38" s="3">
         <v>0</v>
@@ -2555,24 +2558,24 @@
         <v>0</v>
       </c>
       <c r="L38" s="4">
-        <v>114218.2</v>
+        <v>23216.76</v>
       </c>
       <c r="M38" s="4">
-        <v>114218.2</v>
+        <v>23216.76</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>110105</v>
+        <v>114431</v>
       </c>
       <c r="B39" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D39" s="11">
-        <v>45560</v>
+        <v>45930</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>54</v>
@@ -2584,10 +2587,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="4">
-        <v>0</v>
+        <v>1676.4</v>
       </c>
       <c r="I39" s="4">
-        <v>0</v>
+        <v>1676.4</v>
       </c>
       <c r="J39" s="3">
         <v>0</v>
@@ -2596,24 +2599,24 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>16578.8</v>
+        <v>41884.31</v>
       </c>
       <c r="M39" s="4">
-        <v>16578.8</v>
+        <v>41884.31</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>109998</v>
+        <v>115404</v>
       </c>
       <c r="B40" s="2">
         <v>2043</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D40" s="11">
-        <v>45596</v>
+        <v>45986</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>54</v>
@@ -2625,10 +2628,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="4">
-        <v>0</v>
+        <v>653.92999999999995</v>
       </c>
       <c r="I40" s="4">
-        <v>0</v>
+        <v>653.92999999999995</v>
       </c>
       <c r="J40" s="3">
         <v>0</v>
@@ -2637,27 +2640,27 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>2844.94</v>
+        <v>45330.52</v>
       </c>
       <c r="M40" s="4">
-        <v>2844.94</v>
+        <v>45330.52</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>108658</v>
+        <v>116795</v>
       </c>
       <c r="B41" s="2">
         <v>2043</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="D41" s="11">
-        <v>45497</v>
+        <v>46000</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F41" s="3">
         <v>0</v>
@@ -2678,24 +2681,24 @@
         <v>0</v>
       </c>
       <c r="L41" s="4">
-        <v>1558.85</v>
+        <v>4746.34</v>
       </c>
       <c r="M41" s="4">
-        <v>1558.85</v>
+        <v>4746.34</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>95148</v>
+        <v>112522</v>
       </c>
       <c r="B42" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D42" s="11">
-        <v>44916</v>
+        <v>45776</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>54</v>
@@ -2719,24 +2722,24 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>3858.2</v>
+        <v>8371.91</v>
       </c>
       <c r="M42" s="4">
-        <v>3858.2</v>
+        <v>8371.91</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>94156</v>
+        <v>110575</v>
       </c>
       <c r="B43" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="D43" s="11">
-        <v>44159</v>
+        <v>45583</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>54</v>
@@ -2760,24 +2763,24 @@
         <v>0</v>
       </c>
       <c r="L43" s="4">
-        <v>7582.41</v>
+        <v>114218.2</v>
       </c>
       <c r="M43" s="4">
-        <v>7582.41</v>
+        <v>114218.2</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>90355</v>
+        <v>108658</v>
       </c>
       <c r="B44" s="2">
         <v>2043</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D44" s="11">
-        <v>43949</v>
+        <v>45497</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>54</v>
@@ -2795,33 +2798,33 @@
         <v>0</v>
       </c>
       <c r="J44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K44" s="4">
-        <v>73149.789999999994</v>
+        <v>0</v>
       </c>
       <c r="L44" s="4">
-        <v>45845.07</v>
+        <v>1558.85</v>
       </c>
       <c r="M44" s="4">
-        <v>118994.86</v>
+        <v>1558.85</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
-        <v>81618</v>
+        <v>94156</v>
       </c>
       <c r="B45" s="2">
         <v>2043</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D45" s="11">
-        <v>43447</v>
+        <v>44159</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F45" s="3">
         <v>0</v>
@@ -2836,33 +2839,33 @@
         <v>0</v>
       </c>
       <c r="J45" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K45" s="4">
-        <v>0</v>
+        <v>2285.38</v>
       </c>
       <c r="L45" s="4">
-        <v>14949.86</v>
+        <v>5124.38</v>
       </c>
       <c r="M45" s="4">
-        <v>14949.86</v>
+        <v>7409.76</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
-        <v>63441</v>
+        <v>81618</v>
       </c>
       <c r="B46" s="2">
-        <v>2511</v>
+        <v>2043</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D46" s="11">
-        <v>44733</v>
+        <v>43447</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F46" s="3">
         <v>0</v>
@@ -2883,99 +2886,97 @@
         <v>0</v>
       </c>
       <c r="L46" s="4">
-        <v>10965.01</v>
+        <v>14949.86</v>
       </c>
       <c r="M46" s="4">
-        <v>10965.01</v>
+        <v>14949.86</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
+        <v>63441</v>
+      </c>
+      <c r="B47" s="2">
+        <v>2511</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D47" s="11">
+        <v>44733</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F47" s="3">
+        <v>0</v>
+      </c>
+      <c r="G47" s="4">
+        <v>0</v>
+      </c>
+      <c r="H47" s="4">
+        <v>0</v>
+      </c>
+      <c r="I47" s="4">
+        <v>0</v>
+      </c>
+      <c r="J47" s="3">
+        <v>0</v>
+      </c>
+      <c r="K47" s="4">
+        <v>0</v>
+      </c>
+      <c r="L47" s="4">
+        <v>10965.01</v>
+      </c>
+      <c r="M47" s="4">
+        <v>10965.01</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A48" s="2">
         <v>113450</v>
       </c>
-      <c r="B47" s="2">
+      <c r="B48" s="2">
         <v>2692</v>
       </c>
-      <c r="C47" s="2" t="s">
+      <c r="C48" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D47" s="11">
+      <c r="D48" s="11">
         <v>45852</v>
       </c>
-      <c r="E47" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F47" s="3">
-        <v>0</v>
-      </c>
-      <c r="G47" s="4">
-        <v>0</v>
-      </c>
-      <c r="H47" s="4">
+      <c r="E48" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F48" s="3">
+        <v>0</v>
+      </c>
+      <c r="G48" s="4">
+        <v>0</v>
+      </c>
+      <c r="H48" s="4">
         <v>-16394.27</v>
       </c>
-      <c r="I47" s="4">
+      <c r="I48" s="4">
         <v>-16394.27</v>
       </c>
-      <c r="J47" s="3">
-        <v>0</v>
-      </c>
-      <c r="K47" s="4">
-        <v>0</v>
-      </c>
-      <c r="L47" s="4">
+      <c r="J48" s="3">
+        <v>0</v>
+      </c>
+      <c r="K48" s="4">
+        <v>0</v>
+      </c>
+      <c r="L48" s="4">
         <v>8694.17</v>
       </c>
-      <c r="M47" s="4">
+      <c r="M48" s="4">
         <v>8694.17</v>
       </c>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="2"/>
-      <c r="F48" s="3"/>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-      <c r="I48" s="4"/>
-      <c r="J48" s="3"/>
-      <c r="K48" s="4"/>
-      <c r="L48" s="4"/>
-      <c r="M48" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="A48:B48">
-    <cfRule type="expression" dxfId="23" priority="13" stopIfTrue="1">
-      <formula>$S48=1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="22" priority="14" stopIfTrue="1">
-      <formula>$S47=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C48:H48 K48:L48">
-    <cfRule type="expression" dxfId="19" priority="18" stopIfTrue="1">
-      <formula>$S48=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C48:M48">
-    <cfRule type="expression" dxfId="18" priority="53" stopIfTrue="1">
-      <formula>$S47=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I48 M48">
-    <cfRule type="expression" dxfId="15" priority="20" stopIfTrue="1">
-      <formula>$S48=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J48">
-    <cfRule type="expression" dxfId="12" priority="16" stopIfTrue="1">
-      <formula>$S48=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A47 J5:J47">
+  <conditionalFormatting sqref="A5:A48 J5:J48">
     <cfRule type="expression" dxfId="11" priority="4" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
@@ -2983,7 +2984,7 @@
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:L47 C5:H47">
+  <conditionalFormatting sqref="K5:L48 C5:H48">
     <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
@@ -2991,7 +2992,7 @@
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I47 M5:M47">
+  <conditionalFormatting sqref="I5:I48 M5:M48">
     <cfRule type="expression" dxfId="7" priority="8" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
@@ -3019,7 +3020,7 @@
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B47">
+  <conditionalFormatting sqref="B5:B48">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>

</xml_diff>

<commit_message>
Update Pagado y Emitido report to March 20
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5A7A9D8-525C-0B45-9C5F-BDD0920C6CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8BC990B-68F0-F843-BC60-3ABB0181AC48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -379,7 +379,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="25">
+  <dxfs count="24">
     <dxf>
       <border>
         <top style="thin">
@@ -538,6 +538,13 @@
     </dxf>
     <dxf>
       <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -545,6 +552,22 @@
           <color indexed="64"/>
         </right>
         <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
           <color indexed="64"/>
         </top>
         <bottom style="hair">
@@ -561,13 +584,13 @@
     </dxf>
     <dxf>
       <border>
-        <left style="thin">
+        <left style="hair">
           <color indexed="64"/>
         </left>
-        <right style="hair">
+        <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="thin">
+        <top style="hair">
           <color indexed="64"/>
         </top>
         <bottom style="hair">
@@ -583,7 +606,7 @@
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="hair">
+        <top style="thin">
           <color indexed="64"/>
         </top>
         <bottom style="hair">
@@ -603,45 +626,15 @@
         <left style="hair">
           <color indexed="64"/>
         </left>
-        <right style="thin">
+        <right style="hair">
           <color indexed="64"/>
         </right>
-        <top style="thin">
+        <top style="hair">
           <color indexed="64"/>
         </top>
         <bottom style="hair">
           <color indexed="64"/>
         </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
       </border>
     </dxf>
     <dxf>
@@ -1050,7 +1043,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1152,10 +1145,10 @@
         <v>391236.33</v>
       </c>
       <c r="H4" s="4">
-        <v>70292.42</v>
+        <v>73270.22</v>
       </c>
       <c r="I4" s="4">
-        <v>461528.75</v>
+        <v>464506.55</v>
       </c>
       <c r="J4" s="5">
         <v>0</v>
@@ -1164,65 +1157,65 @@
         <v>0</v>
       </c>
       <c r="L4" s="4">
-        <v>343671.65</v>
+        <v>340693.85</v>
       </c>
       <c r="M4" s="4">
-        <v>343671.65</v>
+        <v>340693.85</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
-        <v>110453</v>
+        <v>80122</v>
       </c>
       <c r="B5" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="D5" s="11">
-        <v>45600</v>
+        <v>43371</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F5" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" s="4">
-        <v>1840.93</v>
+        <v>99798.14</v>
       </c>
       <c r="H5" s="4">
-        <v>76322.12</v>
+        <v>12339.99</v>
       </c>
       <c r="I5" s="4">
-        <v>78163.05</v>
+        <v>112138.13</v>
       </c>
       <c r="J5" s="3">
         <v>1</v>
       </c>
       <c r="K5" s="4">
-        <v>1770.92</v>
+        <v>6346.39</v>
       </c>
       <c r="L5" s="4">
-        <v>181909.6</v>
+        <v>115544.18</v>
       </c>
       <c r="M5" s="4">
-        <v>183680.52</v>
+        <v>121890.57</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>115047</v>
+        <v>110453</v>
       </c>
       <c r="B6" s="2">
         <v>2856</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6" s="11">
-        <v>45944</v>
+        <v>45600</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>54</v>
@@ -1231,25 +1224,25 @@
         <v>1</v>
       </c>
       <c r="G6" s="4">
-        <v>1488.25</v>
+        <v>1840.93</v>
       </c>
       <c r="H6" s="4">
-        <v>42774.11</v>
+        <v>76322.12</v>
       </c>
       <c r="I6" s="4">
-        <v>44262.36</v>
+        <v>78163.05</v>
       </c>
       <c r="J6" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" s="4">
-        <v>0</v>
+        <v>1770.92</v>
       </c>
       <c r="L6" s="4">
-        <v>34641.980000000003</v>
+        <v>181909.6</v>
       </c>
       <c r="M6" s="4">
-        <v>34641.980000000003</v>
+        <v>183680.52</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -1269,57 +1262,57 @@
         <v>54</v>
       </c>
       <c r="F7" s="3">
+        <v>2</v>
+      </c>
+      <c r="G7" s="4">
+        <v>32255.77</v>
+      </c>
+      <c r="H7" s="4">
+        <v>41016.79</v>
+      </c>
+      <c r="I7" s="4">
+        <v>73272.56</v>
+      </c>
+      <c r="J7" s="3">
         <v>1</v>
       </c>
-      <c r="G7" s="4">
-        <v>-3520.38</v>
-      </c>
-      <c r="H7" s="4">
-        <v>39264.269999999997</v>
-      </c>
-      <c r="I7" s="4">
-        <v>35743.89</v>
-      </c>
-      <c r="J7" s="3">
-        <v>2</v>
-      </c>
       <c r="K7" s="4">
-        <v>37848.660000000003</v>
+        <v>2072.5100000000002</v>
       </c>
       <c r="L7" s="4">
-        <v>61941.82</v>
+        <v>60303.09</v>
       </c>
       <c r="M7" s="4">
-        <v>99790.48</v>
+        <v>62375.6</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>107488</v>
+        <v>115047</v>
       </c>
       <c r="B8" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="D8" s="11">
-        <v>45440</v>
+        <v>45944</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="4">
-        <v>0</v>
+        <v>1488.25</v>
       </c>
       <c r="H8" s="4">
-        <v>32610.63</v>
+        <v>44493.67</v>
       </c>
       <c r="I8" s="4">
-        <v>32610.63</v>
+        <v>45981.919999999998</v>
       </c>
       <c r="J8" s="3">
         <v>0</v>
@@ -1328,24 +1321,24 @@
         <v>0</v>
       </c>
       <c r="L8" s="4">
-        <v>132043.74</v>
+        <v>32922.42</v>
       </c>
       <c r="M8" s="4">
-        <v>132043.74</v>
+        <v>32922.42</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>104718</v>
+        <v>105696</v>
       </c>
       <c r="B9" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="D9" s="11">
-        <v>45264</v>
+        <v>45279</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>54</v>
@@ -1354,13 +1347,13 @@
         <v>1</v>
       </c>
       <c r="G9" s="4">
-        <v>13028.98</v>
+        <v>31875.97</v>
       </c>
       <c r="H9" s="4">
-        <v>18442.25</v>
+        <v>9320.44</v>
       </c>
       <c r="I9" s="4">
-        <v>31471.23</v>
+        <v>41196.410000000003</v>
       </c>
       <c r="J9" s="3">
         <v>0</v>
@@ -1369,80 +1362,80 @@
         <v>0</v>
       </c>
       <c r="L9" s="4">
-        <v>108356.53</v>
+        <v>27850.23</v>
       </c>
       <c r="M9" s="4">
-        <v>108356.53</v>
+        <v>27850.23</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>80122</v>
+        <v>107488</v>
       </c>
       <c r="B10" s="2">
         <v>2043</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="D10" s="11">
-        <v>43371</v>
+        <v>45440</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F10" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" s="4">
-        <v>2550.13</v>
+        <v>0</v>
       </c>
       <c r="H10" s="4">
-        <v>12339.99</v>
+        <v>38679.050000000003</v>
       </c>
       <c r="I10" s="4">
-        <v>14890.12</v>
+        <v>38679.050000000003</v>
       </c>
       <c r="J10" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" s="4">
-        <v>97248.01</v>
+        <v>0</v>
       </c>
       <c r="L10" s="4">
-        <v>96505.02</v>
+        <v>125975.29</v>
       </c>
       <c r="M10" s="4">
-        <v>193753.03</v>
+        <v>125975.29</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>90355</v>
+        <v>104718</v>
       </c>
       <c r="B11" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="D11" s="11">
-        <v>43949</v>
+        <v>45264</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F11" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" s="4">
-        <v>0</v>
+        <v>13028.98</v>
       </c>
       <c r="H11" s="4">
-        <v>13410.43</v>
+        <v>18442.25</v>
       </c>
       <c r="I11" s="4">
-        <v>13410.43</v>
+        <v>31471.23</v>
       </c>
       <c r="J11" s="3">
         <v>0</v>
@@ -1451,10 +1444,10 @@
         <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>32434.68</v>
+        <v>108356.53</v>
       </c>
       <c r="M11" s="4">
-        <v>32434.68</v>
+        <v>108356.53</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
@@ -1474,57 +1467,57 @@
         <v>54</v>
       </c>
       <c r="F12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" s="4">
-        <v>0</v>
+        <v>1684.95</v>
       </c>
       <c r="H12" s="4">
         <v>13292.63</v>
       </c>
       <c r="I12" s="4">
-        <v>13292.63</v>
+        <v>14977.58</v>
       </c>
       <c r="J12" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" s="4">
-        <v>1684.95</v>
+        <v>0</v>
       </c>
       <c r="L12" s="4">
         <v>68730.09</v>
       </c>
       <c r="M12" s="4">
-        <v>70415.039999999994</v>
+        <v>68730.09</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>116883</v>
+        <v>90355</v>
       </c>
       <c r="B13" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="D13" s="11">
-        <v>46007</v>
+        <v>43949</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F13" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G13" s="4">
-        <v>7008.07</v>
+        <v>0</v>
       </c>
       <c r="H13" s="4">
-        <v>4010.74</v>
+        <v>13410.43</v>
       </c>
       <c r="I13" s="4">
-        <v>11018.81</v>
+        <v>13410.43</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1533,39 +1526,39 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>41489.449999999997</v>
+        <v>32434.68</v>
       </c>
       <c r="M13" s="4">
-        <v>41489.449999999997</v>
+        <v>32434.68</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>94205</v>
+        <v>116883</v>
       </c>
       <c r="B14" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="D14" s="11">
-        <v>44116</v>
+        <v>46007</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F14" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G14" s="4">
-        <v>0</v>
+        <v>7008.07</v>
       </c>
       <c r="H14" s="4">
-        <v>10135.31</v>
+        <v>4010.74</v>
       </c>
       <c r="I14" s="4">
-        <v>10135.31</v>
+        <v>11018.81</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1574,39 +1567,39 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>0</v>
+        <v>41489.449999999997</v>
       </c>
       <c r="M14" s="4">
-        <v>0</v>
+        <v>41489.449999999997</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>117440</v>
+        <v>94205</v>
       </c>
       <c r="B15" s="2">
         <v>2043</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="D15" s="11">
-        <v>46059</v>
+        <v>44116</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F15" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G15" s="4">
-        <v>5692.2</v>
+        <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>4226.8900000000003</v>
+        <v>10135.31</v>
       </c>
       <c r="I15" s="4">
-        <v>9919.09</v>
+        <v>10135.31</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1623,31 +1616,31 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>106018</v>
+        <v>117440</v>
       </c>
       <c r="B16" s="2">
         <v>2043</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="D16" s="11">
-        <v>45344</v>
+        <v>46059</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F16" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G16" s="4">
-        <v>580.95000000000005</v>
+        <v>5692.2</v>
       </c>
       <c r="H16" s="4">
-        <v>8612.6200000000008</v>
+        <v>4226.8900000000003</v>
       </c>
       <c r="I16" s="4">
-        <v>9193.57</v>
+        <v>9919.09</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1656,39 +1649,39 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>22590.41</v>
+        <v>0</v>
       </c>
       <c r="M16" s="4">
-        <v>22590.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>110105</v>
+        <v>106018</v>
       </c>
       <c r="B17" s="2">
         <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="D17" s="11">
-        <v>45560</v>
+        <v>45344</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F17" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" s="4">
-        <v>0</v>
+        <v>580.95000000000005</v>
       </c>
       <c r="H17" s="4">
-        <v>8858.33</v>
+        <v>8612.6200000000008</v>
       </c>
       <c r="I17" s="4">
-        <v>8858.33</v>
+        <v>9193.57</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1697,24 +1690,24 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>7719.98</v>
+        <v>22590.41</v>
       </c>
       <c r="M17" s="4">
-        <v>7719.98</v>
+        <v>22590.41</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>114100</v>
+        <v>110105</v>
       </c>
       <c r="B18" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="D18" s="11">
-        <v>45863</v>
+        <v>45560</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>54</v>
@@ -1726,10 +1719,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>8427.17</v>
+        <v>8858.33</v>
       </c>
       <c r="I18" s="4">
-        <v>8427.17</v>
+        <v>8858.33</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1738,24 +1731,24 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>53325.32</v>
+        <v>7719.98</v>
       </c>
       <c r="M18" s="4">
-        <v>53325.32</v>
+        <v>7719.98</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>108405</v>
+        <v>114100</v>
       </c>
       <c r="B19" s="2">
-        <v>2692</v>
+        <v>2856</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="D19" s="11">
-        <v>45471</v>
+        <v>45863</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>54</v>
@@ -1767,10 +1760,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>7485.18</v>
+        <v>8427.17</v>
       </c>
       <c r="I19" s="4">
-        <v>7485.18</v>
+        <v>8427.17</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1779,24 +1772,24 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>34981.11</v>
+        <v>53325.32</v>
       </c>
       <c r="M19" s="4">
-        <v>34981.11</v>
+        <v>53325.32</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>100677</v>
+        <v>108405</v>
       </c>
       <c r="B20" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="D20" s="11">
-        <v>44999</v>
+        <v>45471</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>54</v>
@@ -1808,10 +1801,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>6339.76</v>
+        <v>7485.18</v>
       </c>
       <c r="I20" s="4">
-        <v>6339.76</v>
+        <v>7485.18</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1820,24 +1813,24 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>19751.150000000001</v>
+        <v>34981.11</v>
       </c>
       <c r="M20" s="4">
-        <v>19751.150000000001</v>
+        <v>34981.11</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>105696</v>
+        <v>100677</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D21" s="11">
-        <v>45279</v>
+        <v>44999</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>54</v>
@@ -1849,22 +1842,22 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>6285.09</v>
+        <v>6339.76</v>
       </c>
       <c r="I21" s="4">
-        <v>6285.09</v>
+        <v>6339.76</v>
       </c>
       <c r="J21" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21" s="4">
-        <v>31875.97</v>
+        <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>30430.65</v>
+        <v>19751.150000000001</v>
       </c>
       <c r="M21" s="4">
-        <v>62306.62</v>
+        <v>19751.150000000001</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
@@ -2566,16 +2559,16 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>114431</v>
+        <v>112522</v>
       </c>
       <c r="B39" s="2">
-        <v>2692</v>
+        <v>2856</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D39" s="11">
-        <v>45930</v>
+        <v>45776</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>54</v>
@@ -2587,10 +2580,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="4">
-        <v>1676.4</v>
+        <v>1737.52</v>
       </c>
       <c r="I39" s="4">
-        <v>1676.4</v>
+        <v>1737.52</v>
       </c>
       <c r="J39" s="3">
         <v>0</v>
@@ -2599,24 +2592,24 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>41884.31</v>
+        <v>6634.38</v>
       </c>
       <c r="M39" s="4">
-        <v>41884.31</v>
+        <v>6634.38</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>115404</v>
+        <v>114431</v>
       </c>
       <c r="B40" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D40" s="11">
-        <v>45986</v>
+        <v>45930</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>54</v>
@@ -2628,10 +2621,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="4">
-        <v>653.92999999999995</v>
+        <v>1676.4</v>
       </c>
       <c r="I40" s="4">
-        <v>653.92999999999995</v>
+        <v>1676.4</v>
       </c>
       <c r="J40" s="3">
         <v>0</v>
@@ -2640,10 +2633,10 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>45330.52</v>
+        <v>41884.31</v>
       </c>
       <c r="M40" s="4">
-        <v>45330.52</v>
+        <v>41884.31</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
@@ -2669,10 +2662,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="4">
-        <v>0</v>
+        <v>1582.15</v>
       </c>
       <c r="I41" s="4">
-        <v>0</v>
+        <v>1582.15</v>
       </c>
       <c r="J41" s="3">
         <v>0</v>
@@ -2681,24 +2674,24 @@
         <v>0</v>
       </c>
       <c r="L41" s="4">
-        <v>4746.34</v>
+        <v>0</v>
       </c>
       <c r="M41" s="4">
-        <v>4746.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>112522</v>
+        <v>115404</v>
       </c>
       <c r="B42" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D42" s="11">
-        <v>45776</v>
+        <v>45986</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>54</v>
@@ -2710,10 +2703,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="4">
-        <v>0</v>
+        <v>653.92999999999995</v>
       </c>
       <c r="I42" s="4">
-        <v>0</v>
+        <v>653.92999999999995</v>
       </c>
       <c r="J42" s="3">
         <v>0</v>
@@ -2722,10 +2715,10 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>8371.91</v>
+        <v>45330.52</v>
       </c>
       <c r="M42" s="4">
-        <v>8371.91</v>
+        <v>45330.52</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
@@ -2956,10 +2949,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="4">
-        <v>-16394.27</v>
+        <v>-14615.07</v>
       </c>
       <c r="I48" s="4">
-        <v>-16394.27</v>
+        <v>-14615.07</v>
       </c>
       <c r="J48" s="3">
         <v>0</v>
@@ -2968,10 +2961,10 @@
         <v>0</v>
       </c>
       <c r="L48" s="4">
-        <v>8694.17</v>
+        <v>6914.97</v>
       </c>
       <c r="M48" s="4">
-        <v>8694.17</v>
+        <v>6914.97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Pagado y Emitido report to March 23
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8BC990B-68F0-F843-BC60-3ABB0181AC48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431F0A88-C0AB-5B44-8891-72523CC7883B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -1043,7 +1043,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46101</v>
+        <v>46104</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1145,22 +1145,22 @@
         <v>391236.33</v>
       </c>
       <c r="H4" s="4">
-        <v>73270.22</v>
+        <v>76262.23</v>
       </c>
       <c r="I4" s="4">
-        <v>464506.55</v>
+        <v>467498.56</v>
       </c>
       <c r="J4" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" s="4">
-        <v>0</v>
+        <v>93758.720000000001</v>
       </c>
       <c r="L4" s="4">
-        <v>340693.85</v>
+        <v>337701.84</v>
       </c>
       <c r="M4" s="4">
-        <v>340693.85</v>
+        <v>431460.56</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1432,10 +1432,10 @@
         <v>13028.98</v>
       </c>
       <c r="H11" s="4">
-        <v>18442.25</v>
+        <v>20161.810000000001</v>
       </c>
       <c r="I11" s="4">
-        <v>31471.23</v>
+        <v>33190.79</v>
       </c>
       <c r="J11" s="3">
         <v>0</v>
@@ -1444,10 +1444,10 @@
         <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>108356.53</v>
+        <v>106636.97</v>
       </c>
       <c r="M11" s="4">
-        <v>108356.53</v>
+        <v>106636.97</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
@@ -1643,16 +1643,16 @@
         <v>9919.09</v>
       </c>
       <c r="J16" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" s="4">
-        <v>0</v>
+        <v>2967.98</v>
       </c>
       <c r="L16" s="4">
         <v>0</v>
       </c>
       <c r="M16" s="4">
-        <v>0</v>
+        <v>2967.98</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
@@ -1780,16 +1780,16 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>108405</v>
+        <v>100677</v>
       </c>
       <c r="B20" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="D20" s="11">
-        <v>45471</v>
+        <v>44999</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>54</v>
@@ -1801,10 +1801,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>7485.18</v>
+        <v>8062.37</v>
       </c>
       <c r="I20" s="4">
-        <v>7485.18</v>
+        <v>8062.37</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1813,24 +1813,24 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>34981.11</v>
+        <v>18028.54</v>
       </c>
       <c r="M20" s="4">
-        <v>34981.11</v>
+        <v>18028.54</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>100677</v>
+        <v>108405</v>
       </c>
       <c r="B21" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="D21" s="11">
-        <v>44999</v>
+        <v>45471</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>54</v>
@@ -1842,10 +1842,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>6339.76</v>
+        <v>7485.18</v>
       </c>
       <c r="I21" s="4">
-        <v>6339.76</v>
+        <v>7485.18</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1854,10 +1854,10 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>19751.150000000001</v>
+        <v>34981.11</v>
       </c>
       <c r="M21" s="4">
-        <v>19751.150000000001</v>
+        <v>34981.11</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
@@ -2272,16 +2272,16 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>109998</v>
+        <v>109007</v>
       </c>
       <c r="B32" s="2">
         <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D32" s="11">
-        <v>45596</v>
+        <v>45525</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>54</v>
@@ -2293,10 +2293,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>2844.92</v>
+        <v>3058.98</v>
       </c>
       <c r="I32" s="4">
-        <v>2844.92</v>
+        <v>3058.98</v>
       </c>
       <c r="J32" s="3">
         <v>0</v>
@@ -2313,16 +2313,16 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>65046</v>
+        <v>109998</v>
       </c>
       <c r="B33" s="2">
         <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="D33" s="11">
-        <v>44763</v>
+        <v>45596</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>54</v>
@@ -2334,36 +2334,36 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>2759.08</v>
+        <v>2844.92</v>
       </c>
       <c r="I33" s="4">
-        <v>2759.08</v>
+        <v>2844.92</v>
       </c>
       <c r="J33" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33" s="4">
-        <v>25197.91</v>
+        <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>20012.810000000001</v>
+        <v>0</v>
       </c>
       <c r="M33" s="4">
-        <v>45210.720000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>81044</v>
+        <v>65046</v>
       </c>
       <c r="B34" s="2">
-        <v>2511</v>
+        <v>2043</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="D34" s="11">
-        <v>44872</v>
+        <v>44763</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>54</v>
@@ -2375,36 +2375,36 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>2385.52</v>
+        <v>2759.08</v>
       </c>
       <c r="I34" s="4">
-        <v>2385.52</v>
+        <v>2759.08</v>
       </c>
       <c r="J34" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K34" s="4">
-        <v>0</v>
+        <v>25197.91</v>
       </c>
       <c r="L34" s="4">
-        <v>0</v>
+        <v>20012.810000000001</v>
       </c>
       <c r="M34" s="4">
-        <v>0</v>
+        <v>45210.720000000001</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>101640</v>
+        <v>81044</v>
       </c>
       <c r="B35" s="2">
-        <v>2043</v>
+        <v>2511</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="D35" s="11">
-        <v>45104</v>
+        <v>44872</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>54</v>
@@ -2416,10 +2416,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="4">
-        <v>2316.9899999999998</v>
+        <v>2385.52</v>
       </c>
       <c r="I35" s="4">
-        <v>2316.9899999999998</v>
+        <v>2385.52</v>
       </c>
       <c r="J35" s="3">
         <v>0</v>
@@ -2428,24 +2428,24 @@
         <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>5546.81</v>
+        <v>0</v>
       </c>
       <c r="M35" s="4">
-        <v>5546.81</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>109007</v>
+        <v>101640</v>
       </c>
       <c r="B36" s="2">
         <v>2043</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="D36" s="11">
-        <v>45525</v>
+        <v>45104</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>54</v>
@@ -2457,10 +2457,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="4">
-        <v>2205.21</v>
+        <v>2316.9899999999998</v>
       </c>
       <c r="I36" s="4">
-        <v>2205.21</v>
+        <v>2316.9899999999998</v>
       </c>
       <c r="J36" s="3">
         <v>0</v>
@@ -2469,10 +2469,10 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>0</v>
+        <v>5546.81</v>
       </c>
       <c r="M36" s="4">
-        <v>0</v>
+        <v>5546.81</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
fix: allow negative values in calculations and update March 27 reports
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431F0A88-C0AB-5B44-8891-72523CC7883B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A27D4F6B-40CC-8143-9D7D-7DE4422CCAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -223,7 +223,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="#,##0.0_ ;\-#,##0.0\ "/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1026,7 +1026,7 @@
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
   <dimension ref="A1:M48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="15.1640625" customWidth="1"/>
     <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
@@ -1041,16 +1041,16 @@
     <col min="11" max="14" width="11.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="24">
       <c r="A1" s="7">
-        <v>46104</v>
+        <v>46105</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13">
       <c r="A2" s="8"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1081,7 +1081,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1122,7 +1122,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13">
       <c r="A4" s="2">
         <v>87538</v>
       </c>
@@ -1145,10 +1145,10 @@
         <v>391236.33</v>
       </c>
       <c r="H4" s="4">
-        <v>76262.23</v>
+        <v>83391.67</v>
       </c>
       <c r="I4" s="4">
-        <v>467498.56</v>
+        <v>474628</v>
       </c>
       <c r="J4" s="5">
         <v>1</v>
@@ -1157,13 +1157,13 @@
         <v>93758.720000000001</v>
       </c>
       <c r="L4" s="4">
-        <v>337701.84</v>
+        <v>330572.40000000002</v>
       </c>
       <c r="M4" s="4">
-        <v>431460.56</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+        <v>424331.12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" s="2">
         <v>80122</v>
       </c>
@@ -1204,7 +1204,7 @@
         <v>121890.57</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13">
       <c r="A6" s="2">
         <v>110453</v>
       </c>
@@ -1227,10 +1227,10 @@
         <v>1840.93</v>
       </c>
       <c r="H6" s="4">
-        <v>76322.12</v>
+        <v>79031.03</v>
       </c>
       <c r="I6" s="4">
-        <v>78163.05</v>
+        <v>80871.960000000006</v>
       </c>
       <c r="J6" s="3">
         <v>1</v>
@@ -1239,13 +1239,13 @@
         <v>1770.92</v>
       </c>
       <c r="L6" s="4">
-        <v>181909.6</v>
+        <v>173783.01</v>
       </c>
       <c r="M6" s="4">
-        <v>183680.52</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+        <v>175553.93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7" s="2">
         <v>104750</v>
       </c>
@@ -1286,7 +1286,7 @@
         <v>62375.6</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13">
       <c r="A8" s="2">
         <v>115047</v>
       </c>
@@ -1327,7 +1327,7 @@
         <v>32922.42</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13">
       <c r="A9" s="2">
         <v>105696</v>
       </c>
@@ -1368,7 +1368,7 @@
         <v>27850.23</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13">
       <c r="A10" s="2">
         <v>107488</v>
       </c>
@@ -1409,7 +1409,7 @@
         <v>125975.29</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13">
       <c r="A11" s="2">
         <v>104718</v>
       </c>
@@ -1432,10 +1432,10 @@
         <v>13028.98</v>
       </c>
       <c r="H11" s="4">
-        <v>20161.810000000001</v>
+        <v>22607.66</v>
       </c>
       <c r="I11" s="4">
-        <v>33190.79</v>
+        <v>35636.639999999999</v>
       </c>
       <c r="J11" s="3">
         <v>0</v>
@@ -1444,13 +1444,13 @@
         <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>106636.97</v>
+        <v>104191.1</v>
       </c>
       <c r="M11" s="4">
-        <v>106636.97</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+        <v>104191.1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
       <c r="A12" s="2">
         <v>114157</v>
       </c>
@@ -1491,7 +1491,7 @@
         <v>68730.09</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13">
       <c r="A13" s="2">
         <v>90355</v>
       </c>
@@ -1532,7 +1532,7 @@
         <v>32434.68</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13">
       <c r="A14" s="2">
         <v>116883</v>
       </c>
@@ -1573,18 +1573,18 @@
         <v>41489.449999999997</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13">
       <c r="A15" s="2">
-        <v>94205</v>
+        <v>80925</v>
       </c>
       <c r="B15" s="2">
         <v>2043</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D15" s="11">
-        <v>44116</v>
+        <v>43439</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>54</v>
@@ -1596,10 +1596,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>10135.31</v>
+        <v>10230.700000000001</v>
       </c>
       <c r="I15" s="4">
-        <v>10135.31</v>
+        <v>10230.700000000001</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1614,264 +1614,264 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13">
       <c r="A16" s="2">
-        <v>117440</v>
+        <v>94205</v>
       </c>
       <c r="B16" s="2">
         <v>2043</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="D16" s="11">
-        <v>46059</v>
+        <v>44116</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F16" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G16" s="4">
-        <v>5692.2</v>
+        <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>4226.8900000000003</v>
+        <v>10135.31</v>
       </c>
       <c r="I16" s="4">
-        <v>9919.09</v>
+        <v>10135.31</v>
       </c>
       <c r="J16" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K16" s="4">
-        <v>2967.98</v>
+        <v>0</v>
       </c>
       <c r="L16" s="4">
         <v>0</v>
       </c>
       <c r="M16" s="4">
-        <v>2967.98</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
       <c r="A17" s="2">
-        <v>106018</v>
+        <v>117440</v>
       </c>
       <c r="B17" s="2">
         <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="D17" s="11">
-        <v>45344</v>
+        <v>46059</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F17" s="3">
+        <v>3</v>
+      </c>
+      <c r="G17" s="4">
+        <v>5692.2</v>
+      </c>
+      <c r="H17" s="4">
+        <v>4226.8900000000003</v>
+      </c>
+      <c r="I17" s="4">
+        <v>9919.09</v>
+      </c>
+      <c r="J17" s="3">
         <v>1</v>
       </c>
-      <c r="G17" s="4">
-        <v>580.95000000000005</v>
-      </c>
-      <c r="H17" s="4">
-        <v>8612.6200000000008</v>
-      </c>
-      <c r="I17" s="4">
-        <v>9193.57</v>
-      </c>
-      <c r="J17" s="3">
-        <v>0</v>
-      </c>
       <c r="K17" s="4">
-        <v>0</v>
+        <v>2967.98</v>
       </c>
       <c r="L17" s="4">
-        <v>22590.41</v>
+        <v>0</v>
       </c>
       <c r="M17" s="4">
-        <v>22590.41</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+        <v>2967.98</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
       <c r="A18" s="2">
-        <v>110105</v>
+        <v>106018</v>
       </c>
       <c r="B18" s="2">
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="11">
+        <v>45344</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F18" s="3">
+        <v>1</v>
+      </c>
+      <c r="G18" s="4">
+        <v>580.95000000000005</v>
+      </c>
+      <c r="H18" s="4">
+        <v>8612.6200000000008</v>
+      </c>
+      <c r="I18" s="4">
+        <v>9193.57</v>
+      </c>
+      <c r="J18" s="3">
+        <v>0</v>
+      </c>
+      <c r="K18" s="4">
+        <v>0</v>
+      </c>
+      <c r="L18" s="4">
+        <v>22590.41</v>
+      </c>
+      <c r="M18" s="4">
+        <v>22590.41</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
+      <c r="A19" s="2">
+        <v>110105</v>
+      </c>
+      <c r="B19" s="2">
+        <v>2043</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D18" s="11">
+      <c r="D19" s="11">
         <v>45560</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F18" s="3">
-        <v>0</v>
-      </c>
-      <c r="G18" s="4">
-        <v>0</v>
-      </c>
-      <c r="H18" s="4">
+      <c r="E19" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F19" s="3">
+        <v>0</v>
+      </c>
+      <c r="G19" s="4">
+        <v>0</v>
+      </c>
+      <c r="H19" s="4">
         <v>8858.33</v>
       </c>
-      <c r="I18" s="4">
+      <c r="I19" s="4">
         <v>8858.33</v>
       </c>
-      <c r="J18" s="3">
-        <v>0</v>
-      </c>
-      <c r="K18" s="4">
-        <v>0</v>
-      </c>
-      <c r="L18" s="4">
+      <c r="J19" s="3">
+        <v>0</v>
+      </c>
+      <c r="K19" s="4">
+        <v>0</v>
+      </c>
+      <c r="L19" s="4">
         <v>7719.98</v>
       </c>
-      <c r="M18" s="4">
+      <c r="M19" s="4">
         <v>7719.98</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A19" s="2">
+    <row r="20" spans="1:13">
+      <c r="A20" s="2">
         <v>114100</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B20" s="2">
         <v>2856</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D20" s="11">
         <v>45863</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F19" s="3">
-        <v>0</v>
-      </c>
-      <c r="G19" s="4">
-        <v>0</v>
-      </c>
-      <c r="H19" s="4">
+      <c r="E20" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F20" s="3">
+        <v>0</v>
+      </c>
+      <c r="G20" s="4">
+        <v>0</v>
+      </c>
+      <c r="H20" s="4">
         <v>8427.17</v>
       </c>
-      <c r="I19" s="4">
+      <c r="I20" s="4">
         <v>8427.17</v>
       </c>
-      <c r="J19" s="3">
-        <v>0</v>
-      </c>
-      <c r="K19" s="4">
-        <v>0</v>
-      </c>
-      <c r="L19" s="4">
+      <c r="J20" s="3">
+        <v>0</v>
+      </c>
+      <c r="K20" s="4">
+        <v>0</v>
+      </c>
+      <c r="L20" s="4">
         <v>53325.32</v>
       </c>
-      <c r="M19" s="4">
+      <c r="M20" s="4">
         <v>53325.32</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A20" s="2">
+    <row r="21" spans="1:13">
+      <c r="A21" s="2">
         <v>100677</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B21" s="2">
         <v>2043</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D20" s="11">
+      <c r="D21" s="11">
         <v>44999</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F20" s="3">
-        <v>0</v>
-      </c>
-      <c r="G20" s="4">
-        <v>0</v>
-      </c>
-      <c r="H20" s="4">
+      <c r="E21" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F21" s="3">
+        <v>0</v>
+      </c>
+      <c r="G21" s="4">
+        <v>0</v>
+      </c>
+      <c r="H21" s="4">
         <v>8062.37</v>
       </c>
-      <c r="I20" s="4">
+      <c r="I21" s="4">
         <v>8062.37</v>
       </c>
-      <c r="J20" s="3">
-        <v>0</v>
-      </c>
-      <c r="K20" s="4">
-        <v>0</v>
-      </c>
-      <c r="L20" s="4">
+      <c r="J21" s="3">
+        <v>0</v>
+      </c>
+      <c r="K21" s="4">
+        <v>0</v>
+      </c>
+      <c r="L21" s="4">
         <v>18028.54</v>
       </c>
-      <c r="M20" s="4">
+      <c r="M21" s="4">
         <v>18028.54</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A21" s="2">
+    <row r="22" spans="1:13">
+      <c r="A22" s="2">
         <v>108405</v>
-      </c>
-      <c r="B21" s="2">
-        <v>2692</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D21" s="11">
-        <v>45471</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F21" s="3">
-        <v>0</v>
-      </c>
-      <c r="G21" s="4">
-        <v>0</v>
-      </c>
-      <c r="H21" s="4">
-        <v>7485.18</v>
-      </c>
-      <c r="I21" s="4">
-        <v>7485.18</v>
-      </c>
-      <c r="J21" s="3">
-        <v>0</v>
-      </c>
-      <c r="K21" s="4">
-        <v>0</v>
-      </c>
-      <c r="L21" s="4">
-        <v>34981.11</v>
-      </c>
-      <c r="M21" s="4">
-        <v>34981.11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A22" s="2">
-        <v>108404</v>
       </c>
       <c r="B22" s="2">
         <v>2692</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="D22" s="11">
-        <v>45467</v>
+        <v>45471</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>54</v>
@@ -1883,10 +1883,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>5851.31</v>
+        <v>7485.18</v>
       </c>
       <c r="I22" s="4">
-        <v>5851.31</v>
+        <v>7485.18</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1895,106 +1895,106 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>42989.04</v>
+        <v>34981.11</v>
       </c>
       <c r="M22" s="4">
-        <v>42989.04</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+        <v>34981.11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13">
       <c r="A23" s="2">
-        <v>111056</v>
+        <v>108404</v>
       </c>
       <c r="B23" s="2">
         <v>2692</v>
       </c>
       <c r="C23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" s="11">
+        <v>45467</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F23" s="3">
+        <v>0</v>
+      </c>
+      <c r="G23" s="4">
+        <v>0</v>
+      </c>
+      <c r="H23" s="4">
+        <v>5851.31</v>
+      </c>
+      <c r="I23" s="4">
+        <v>5851.31</v>
+      </c>
+      <c r="J23" s="3">
+        <v>0</v>
+      </c>
+      <c r="K23" s="4">
+        <v>0</v>
+      </c>
+      <c r="L23" s="4">
+        <v>42989.04</v>
+      </c>
+      <c r="M23" s="4">
+        <v>42989.04</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13">
+      <c r="A24" s="2">
+        <v>111056</v>
+      </c>
+      <c r="B24" s="2">
+        <v>2692</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D24" s="11">
         <v>45639</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F23" s="3">
-        <v>0</v>
-      </c>
-      <c r="G23" s="4">
-        <v>0</v>
-      </c>
-      <c r="H23" s="4">
+      <c r="E24" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F24" s="3">
+        <v>0</v>
+      </c>
+      <c r="G24" s="4">
+        <v>0</v>
+      </c>
+      <c r="H24" s="4">
         <v>5403.95</v>
       </c>
-      <c r="I23" s="4">
+      <c r="I24" s="4">
         <v>5403.95</v>
       </c>
-      <c r="J23" s="3">
-        <v>0</v>
-      </c>
-      <c r="K23" s="4">
-        <v>0</v>
-      </c>
-      <c r="L23" s="4">
+      <c r="J24" s="3">
+        <v>0</v>
+      </c>
+      <c r="K24" s="4">
+        <v>0</v>
+      </c>
+      <c r="L24" s="4">
         <v>61189.599999999999</v>
       </c>
-      <c r="M23" s="4">
+      <c r="M24" s="4">
         <v>61189.599999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A24" s="2">
-        <v>90177</v>
-      </c>
-      <c r="B24" s="2">
-        <v>2043</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D24" s="11">
-        <v>43949</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F24" s="3">
-        <v>0</v>
-      </c>
-      <c r="G24" s="4">
-        <v>0</v>
-      </c>
-      <c r="H24" s="4">
-        <v>5160.08</v>
-      </c>
-      <c r="I24" s="4">
-        <v>5160.08</v>
-      </c>
-      <c r="J24" s="3">
-        <v>0</v>
-      </c>
-      <c r="K24" s="4">
-        <v>0</v>
-      </c>
-      <c r="L24" s="4">
-        <v>5160.08</v>
-      </c>
-      <c r="M24" s="4">
-        <v>5160.08</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:13">
       <c r="A25" s="2">
-        <v>80925</v>
+        <v>47116</v>
       </c>
       <c r="B25" s="2">
         <v>2043</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D25" s="11">
-        <v>43439</v>
+        <v>44616</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>54</v>
@@ -2006,10 +2006,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>5119.8</v>
+        <v>5188.62</v>
       </c>
       <c r="I25" s="4">
-        <v>5119.8</v>
+        <v>5188.62</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -2018,106 +2018,106 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>10061.92</v>
+        <v>85626.41</v>
       </c>
       <c r="M25" s="4">
-        <v>10061.92</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+        <v>85626.41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13">
       <c r="A26" s="2">
+        <v>90177</v>
+      </c>
+      <c r="B26" s="2">
+        <v>2043</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D26" s="11">
+        <v>43949</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F26" s="3">
+        <v>0</v>
+      </c>
+      <c r="G26" s="4">
+        <v>0</v>
+      </c>
+      <c r="H26" s="4">
+        <v>5160.08</v>
+      </c>
+      <c r="I26" s="4">
+        <v>5160.08</v>
+      </c>
+      <c r="J26" s="3">
+        <v>0</v>
+      </c>
+      <c r="K26" s="4">
+        <v>0</v>
+      </c>
+      <c r="L26" s="4">
+        <v>5160.08</v>
+      </c>
+      <c r="M26" s="4">
+        <v>5160.08</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13">
+      <c r="A27" s="2">
         <v>116060</v>
       </c>
-      <c r="B26" s="2">
+      <c r="B27" s="2">
         <v>2856</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C27" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D26" s="11">
+      <c r="D27" s="11">
         <v>46010</v>
       </c>
-      <c r="E26" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F26" s="3">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
+      <c r="E27" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F27" s="3">
+        <v>0</v>
+      </c>
+      <c r="G27" s="4">
+        <v>0</v>
+      </c>
+      <c r="H27" s="4">
         <v>4927.55</v>
       </c>
-      <c r="I26" s="4">
+      <c r="I27" s="4">
         <v>4927.55</v>
       </c>
-      <c r="J26" s="3">
-        <v>0</v>
-      </c>
-      <c r="K26" s="4">
-        <v>0</v>
-      </c>
-      <c r="L26" s="4">
+      <c r="J27" s="3">
+        <v>0</v>
+      </c>
+      <c r="K27" s="4">
+        <v>0</v>
+      </c>
+      <c r="L27" s="4">
         <v>42294.77</v>
       </c>
-      <c r="M26" s="4">
+      <c r="M27" s="4">
         <v>42294.77</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A27" s="2">
-        <v>113076</v>
-      </c>
-      <c r="B27" s="2">
-        <v>2043</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D27" s="11">
-        <v>45806</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F27" s="3">
-        <v>0</v>
-      </c>
-      <c r="G27" s="4">
-        <v>0</v>
-      </c>
-      <c r="H27" s="4">
-        <v>4524.1099999999997</v>
-      </c>
-      <c r="I27" s="4">
-        <v>4524.1099999999997</v>
-      </c>
-      <c r="J27" s="3">
-        <v>0</v>
-      </c>
-      <c r="K27" s="4">
-        <v>0</v>
-      </c>
-      <c r="L27" s="4">
-        <v>13572.34</v>
-      </c>
-      <c r="M27" s="4">
-        <v>13572.34</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13">
       <c r="A28" s="2">
-        <v>104343</v>
+        <v>94156</v>
       </c>
       <c r="B28" s="2">
         <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="D28" s="11">
-        <v>45201</v>
+        <v>44159</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>54</v>
@@ -2129,36 +2129,36 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>4424.0600000000004</v>
+        <v>4602.76</v>
       </c>
       <c r="I28" s="4">
-        <v>4424.0600000000004</v>
+        <v>4602.76</v>
       </c>
       <c r="J28" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28" s="4">
-        <v>0</v>
+        <v>2285.38</v>
       </c>
       <c r="L28" s="4">
-        <v>43343.73</v>
+        <v>0</v>
       </c>
       <c r="M28" s="4">
-        <v>43343.73</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+        <v>2285.38</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
       <c r="A29" s="2">
-        <v>88234</v>
+        <v>113076</v>
       </c>
       <c r="B29" s="2">
         <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="D29" s="11">
-        <v>43794</v>
+        <v>45806</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>54</v>
@@ -2170,10 +2170,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>4210.32</v>
+        <v>4524.1099999999997</v>
       </c>
       <c r="I29" s="4">
-        <v>4210.32</v>
+        <v>4524.1099999999997</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2182,24 +2182,24 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>19836.599999999999</v>
+        <v>13572.34</v>
       </c>
       <c r="M29" s="4">
-        <v>19836.599999999999</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+        <v>13572.34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13">
       <c r="A30" s="2">
-        <v>95148</v>
+        <v>104343</v>
       </c>
       <c r="B30" s="2">
         <v>2043</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="D30" s="11">
-        <v>44916</v>
+        <v>45201</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>54</v>
@@ -2211,10 +2211,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>3858.24</v>
+        <v>4424.0600000000004</v>
       </c>
       <c r="I30" s="4">
-        <v>3858.24</v>
+        <v>4424.0600000000004</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2223,24 +2223,24 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>0</v>
+        <v>43343.73</v>
       </c>
       <c r="M30" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+        <v>43343.73</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13">
       <c r="A31" s="2">
-        <v>47116</v>
+        <v>88234</v>
       </c>
       <c r="B31" s="2">
         <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>44</v>
+        <v>11</v>
       </c>
       <c r="D31" s="11">
-        <v>44616</v>
+        <v>43794</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>54</v>
@@ -2252,10 +2252,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>3133.99</v>
+        <v>4210.32</v>
       </c>
       <c r="I31" s="4">
-        <v>3133.99</v>
+        <v>4210.32</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -2264,24 +2264,24 @@
         <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>87333.01</v>
+        <v>19836.599999999999</v>
       </c>
       <c r="M31" s="4">
-        <v>87333.01</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+        <v>19836.599999999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13">
       <c r="A32" s="2">
-        <v>109007</v>
+        <v>95148</v>
       </c>
       <c r="B32" s="2">
         <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D32" s="11">
-        <v>45525</v>
+        <v>44916</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>54</v>
@@ -2293,10 +2293,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>3058.98</v>
+        <v>3858.24</v>
       </c>
       <c r="I32" s="4">
-        <v>3058.98</v>
+        <v>3858.24</v>
       </c>
       <c r="J32" s="3">
         <v>0</v>
@@ -2311,18 +2311,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:13">
       <c r="A33" s="2">
-        <v>109998</v>
+        <v>109007</v>
       </c>
       <c r="B33" s="2">
         <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D33" s="11">
-        <v>45596</v>
+        <v>45525</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>54</v>
@@ -2334,10 +2334,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>2844.92</v>
+        <v>3058.98</v>
       </c>
       <c r="I33" s="4">
-        <v>2844.92</v>
+        <v>3058.98</v>
       </c>
       <c r="J33" s="3">
         <v>0</v>
@@ -2352,469 +2352,469 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:13">
       <c r="A34" s="2">
-        <v>65046</v>
+        <v>109998</v>
       </c>
       <c r="B34" s="2">
         <v>2043</v>
       </c>
       <c r="C34" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D34" s="11">
+        <v>45596</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F34" s="3">
+        <v>0</v>
+      </c>
+      <c r="G34" s="4">
+        <v>0</v>
+      </c>
+      <c r="H34" s="4">
+        <v>2844.92</v>
+      </c>
+      <c r="I34" s="4">
+        <v>2844.92</v>
+      </c>
+      <c r="J34" s="3">
+        <v>0</v>
+      </c>
+      <c r="K34" s="4">
+        <v>0</v>
+      </c>
+      <c r="L34" s="4">
+        <v>0</v>
+      </c>
+      <c r="M34" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13">
+      <c r="A35" s="2">
+        <v>65046</v>
+      </c>
+      <c r="B35" s="2">
+        <v>2043</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D34" s="11">
+      <c r="D35" s="11">
         <v>44763</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F34" s="3">
-        <v>0</v>
-      </c>
-      <c r="G34" s="4">
-        <v>0</v>
-      </c>
-      <c r="H34" s="4">
+      <c r="E35" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F35" s="3">
+        <v>0</v>
+      </c>
+      <c r="G35" s="4">
+        <v>0</v>
+      </c>
+      <c r="H35" s="4">
         <v>2759.08</v>
       </c>
-      <c r="I34" s="4">
+      <c r="I35" s="4">
         <v>2759.08</v>
       </c>
-      <c r="J34" s="3">
+      <c r="J35" s="3">
         <v>1</v>
       </c>
-      <c r="K34" s="4">
+      <c r="K35" s="4">
         <v>25197.91</v>
       </c>
-      <c r="L34" s="4">
+      <c r="L35" s="4">
         <v>20012.810000000001</v>
       </c>
-      <c r="M34" s="4">
+      <c r="M35" s="4">
         <v>45210.720000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A35" s="2">
+    <row r="36" spans="1:13">
+      <c r="A36" s="2">
         <v>81044</v>
       </c>
-      <c r="B35" s="2">
+      <c r="B36" s="2">
         <v>2511</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D35" s="11">
+      <c r="D36" s="11">
         <v>44872</v>
       </c>
-      <c r="E35" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F35" s="3">
-        <v>0</v>
-      </c>
-      <c r="G35" s="4">
-        <v>0</v>
-      </c>
-      <c r="H35" s="4">
+      <c r="E36" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F36" s="3">
+        <v>0</v>
+      </c>
+      <c r="G36" s="4">
+        <v>0</v>
+      </c>
+      <c r="H36" s="4">
         <v>2385.52</v>
       </c>
-      <c r="I35" s="4">
+      <c r="I36" s="4">
         <v>2385.52</v>
       </c>
-      <c r="J35" s="3">
-        <v>0</v>
-      </c>
-      <c r="K35" s="4">
-        <v>0</v>
-      </c>
-      <c r="L35" s="4">
-        <v>0</v>
-      </c>
-      <c r="M35" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A36" s="2">
+      <c r="J36" s="3">
+        <v>0</v>
+      </c>
+      <c r="K36" s="4">
+        <v>0</v>
+      </c>
+      <c r="L36" s="4">
+        <v>0</v>
+      </c>
+      <c r="M36" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13">
+      <c r="A37" s="2">
         <v>101640</v>
       </c>
-      <c r="B36" s="2">
+      <c r="B37" s="2">
         <v>2043</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C37" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D36" s="11">
+      <c r="D37" s="11">
         <v>45104</v>
       </c>
-      <c r="E36" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F36" s="3">
-        <v>0</v>
-      </c>
-      <c r="G36" s="4">
-        <v>0</v>
-      </c>
-      <c r="H36" s="4">
+      <c r="E37" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F37" s="3">
+        <v>0</v>
+      </c>
+      <c r="G37" s="4">
+        <v>0</v>
+      </c>
+      <c r="H37" s="4">
         <v>2316.9899999999998</v>
       </c>
-      <c r="I36" s="4">
+      <c r="I37" s="4">
         <v>2316.9899999999998</v>
       </c>
-      <c r="J36" s="3">
-        <v>0</v>
-      </c>
-      <c r="K36" s="4">
-        <v>0</v>
-      </c>
-      <c r="L36" s="4">
+      <c r="J37" s="3">
+        <v>0</v>
+      </c>
+      <c r="K37" s="4">
+        <v>0</v>
+      </c>
+      <c r="L37" s="4">
         <v>5546.81</v>
       </c>
-      <c r="M36" s="4">
+      <c r="M37" s="4">
         <v>5546.81</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A37" s="2">
+    <row r="38" spans="1:13">
+      <c r="A38" s="2">
         <v>116876</v>
       </c>
-      <c r="B37" s="2">
+      <c r="B38" s="2">
         <v>2856</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C38" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D37" s="11">
+      <c r="D38" s="11">
         <v>46006</v>
       </c>
-      <c r="E37" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F37" s="3">
-        <v>0</v>
-      </c>
-      <c r="G37" s="4">
-        <v>0</v>
-      </c>
-      <c r="H37" s="4">
+      <c r="E38" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F38" s="3">
+        <v>0</v>
+      </c>
+      <c r="G38" s="4">
+        <v>0</v>
+      </c>
+      <c r="H38" s="4">
         <v>2005.37</v>
       </c>
-      <c r="I37" s="4">
+      <c r="I38" s="4">
         <v>2005.37</v>
       </c>
-      <c r="J37" s="3">
-        <v>0</v>
-      </c>
-      <c r="K37" s="4">
-        <v>0</v>
-      </c>
-      <c r="L37" s="4">
+      <c r="J38" s="3">
+        <v>0</v>
+      </c>
+      <c r="K38" s="4">
+        <v>0</v>
+      </c>
+      <c r="L38" s="4">
         <v>20053.7</v>
       </c>
-      <c r="M37" s="4">
+      <c r="M38" s="4">
         <v>20053.7</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A38" s="2">
+    <row r="39" spans="1:13">
+      <c r="A39" s="2">
         <v>102825</v>
       </c>
-      <c r="B38" s="2">
+      <c r="B39" s="2">
         <v>2043</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="C39" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D38" s="11">
+      <c r="D39" s="11">
         <v>45117</v>
       </c>
-      <c r="E38" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F38" s="3">
-        <v>0</v>
-      </c>
-      <c r="G38" s="4">
-        <v>0</v>
-      </c>
-      <c r="H38" s="4">
+      <c r="E39" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F39" s="3">
+        <v>0</v>
+      </c>
+      <c r="G39" s="4">
+        <v>0</v>
+      </c>
+      <c r="H39" s="4">
         <v>1742.75</v>
       </c>
-      <c r="I38" s="4">
+      <c r="I39" s="4">
         <v>1742.75</v>
       </c>
-      <c r="J38" s="3">
-        <v>0</v>
-      </c>
-      <c r="K38" s="4">
-        <v>0</v>
-      </c>
-      <c r="L38" s="4">
+      <c r="J39" s="3">
+        <v>0</v>
+      </c>
+      <c r="K39" s="4">
+        <v>0</v>
+      </c>
+      <c r="L39" s="4">
         <v>23216.76</v>
       </c>
-      <c r="M38" s="4">
+      <c r="M39" s="4">
         <v>23216.76</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A39" s="2">
+    <row r="40" spans="1:13">
+      <c r="A40" s="2">
         <v>112522</v>
       </c>
-      <c r="B39" s="2">
+      <c r="B40" s="2">
         <v>2856</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="C40" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D39" s="11">
+      <c r="D40" s="11">
         <v>45776</v>
       </c>
-      <c r="E39" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F39" s="3">
-        <v>0</v>
-      </c>
-      <c r="G39" s="4">
-        <v>0</v>
-      </c>
-      <c r="H39" s="4">
+      <c r="E40" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F40" s="3">
+        <v>0</v>
+      </c>
+      <c r="G40" s="4">
+        <v>0</v>
+      </c>
+      <c r="H40" s="4">
         <v>1737.52</v>
       </c>
-      <c r="I39" s="4">
+      <c r="I40" s="4">
         <v>1737.52</v>
       </c>
-      <c r="J39" s="3">
-        <v>0</v>
-      </c>
-      <c r="K39" s="4">
-        <v>0</v>
-      </c>
-      <c r="L39" s="4">
+      <c r="J40" s="3">
+        <v>0</v>
+      </c>
+      <c r="K40" s="4">
+        <v>0</v>
+      </c>
+      <c r="L40" s="4">
         <v>6634.38</v>
       </c>
-      <c r="M39" s="4">
+      <c r="M40" s="4">
         <v>6634.38</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A40" s="2">
+    <row r="41" spans="1:13">
+      <c r="A41" s="2">
         <v>114431</v>
       </c>
-      <c r="B40" s="2">
+      <c r="B41" s="2">
         <v>2692</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="C41" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D40" s="11">
+      <c r="D41" s="11">
         <v>45930</v>
       </c>
-      <c r="E40" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F40" s="3">
-        <v>0</v>
-      </c>
-      <c r="G40" s="4">
-        <v>0</v>
-      </c>
-      <c r="H40" s="4">
+      <c r="E41" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F41" s="3">
+        <v>0</v>
+      </c>
+      <c r="G41" s="4">
+        <v>0</v>
+      </c>
+      <c r="H41" s="4">
         <v>1676.4</v>
       </c>
-      <c r="I40" s="4">
+      <c r="I41" s="4">
         <v>1676.4</v>
       </c>
-      <c r="J40" s="3">
-        <v>0</v>
-      </c>
-      <c r="K40" s="4">
-        <v>0</v>
-      </c>
-      <c r="L40" s="4">
+      <c r="J41" s="3">
+        <v>0</v>
+      </c>
+      <c r="K41" s="4">
+        <v>0</v>
+      </c>
+      <c r="L41" s="4">
         <v>41884.31</v>
       </c>
-      <c r="M40" s="4">
+      <c r="M41" s="4">
         <v>41884.31</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A41" s="2">
+    <row r="42" spans="1:13">
+      <c r="A42" s="2">
         <v>116795</v>
-      </c>
-      <c r="B41" s="2">
-        <v>2043</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D41" s="11">
-        <v>46000</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F41" s="3">
-        <v>0</v>
-      </c>
-      <c r="G41" s="4">
-        <v>0</v>
-      </c>
-      <c r="H41" s="4">
-        <v>1582.15</v>
-      </c>
-      <c r="I41" s="4">
-        <v>1582.15</v>
-      </c>
-      <c r="J41" s="3">
-        <v>0</v>
-      </c>
-      <c r="K41" s="4">
-        <v>0</v>
-      </c>
-      <c r="L41" s="4">
-        <v>0</v>
-      </c>
-      <c r="M41" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A42" s="2">
-        <v>115404</v>
       </c>
       <c r="B42" s="2">
         <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D42" s="11">
+        <v>46000</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F42" s="3">
+        <v>0</v>
+      </c>
+      <c r="G42" s="4">
+        <v>0</v>
+      </c>
+      <c r="H42" s="4">
+        <v>1582.15</v>
+      </c>
+      <c r="I42" s="4">
+        <v>1582.15</v>
+      </c>
+      <c r="J42" s="3">
+        <v>0</v>
+      </c>
+      <c r="K42" s="4">
+        <v>0</v>
+      </c>
+      <c r="L42" s="4">
+        <v>0</v>
+      </c>
+      <c r="M42" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13">
+      <c r="A43" s="2">
+        <v>115404</v>
+      </c>
+      <c r="B43" s="2">
+        <v>2043</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D42" s="11">
+      <c r="D43" s="11">
         <v>45986</v>
       </c>
-      <c r="E42" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F42" s="3">
-        <v>0</v>
-      </c>
-      <c r="G42" s="4">
-        <v>0</v>
-      </c>
-      <c r="H42" s="4">
+      <c r="E43" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F43" s="3">
+        <v>0</v>
+      </c>
+      <c r="G43" s="4">
+        <v>0</v>
+      </c>
+      <c r="H43" s="4">
         <v>653.92999999999995</v>
       </c>
-      <c r="I42" s="4">
+      <c r="I43" s="4">
         <v>653.92999999999995</v>
       </c>
-      <c r="J42" s="3">
-        <v>0</v>
-      </c>
-      <c r="K42" s="4">
-        <v>0</v>
-      </c>
-      <c r="L42" s="4">
+      <c r="J43" s="3">
+        <v>0</v>
+      </c>
+      <c r="K43" s="4">
+        <v>0</v>
+      </c>
+      <c r="L43" s="4">
         <v>45330.52</v>
       </c>
-      <c r="M42" s="4">
+      <c r="M43" s="4">
         <v>45330.52</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A43" s="2">
+    <row r="44" spans="1:13">
+      <c r="A44" s="2">
         <v>110575</v>
       </c>
-      <c r="B43" s="2">
+      <c r="B44" s="2">
         <v>2692</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="C44" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D43" s="11">
+      <c r="D44" s="11">
         <v>45583</v>
       </c>
-      <c r="E43" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F43" s="3">
-        <v>0</v>
-      </c>
-      <c r="G43" s="4">
-        <v>0</v>
-      </c>
-      <c r="H43" s="4">
-        <v>0</v>
-      </c>
-      <c r="I43" s="4">
-        <v>0</v>
-      </c>
-      <c r="J43" s="3">
-        <v>0</v>
-      </c>
-      <c r="K43" s="4">
-        <v>0</v>
-      </c>
-      <c r="L43" s="4">
+      <c r="E44" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F44" s="3">
+        <v>0</v>
+      </c>
+      <c r="G44" s="4">
+        <v>0</v>
+      </c>
+      <c r="H44" s="4">
+        <v>0</v>
+      </c>
+      <c r="I44" s="4">
+        <v>0</v>
+      </c>
+      <c r="J44" s="3">
+        <v>0</v>
+      </c>
+      <c r="K44" s="4">
+        <v>0</v>
+      </c>
+      <c r="L44" s="4">
         <v>114218.2</v>
       </c>
-      <c r="M43" s="4">
+      <c r="M44" s="4">
         <v>114218.2</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A44" s="2">
+    <row r="45" spans="1:13">
+      <c r="A45" s="2">
         <v>108658</v>
-      </c>
-      <c r="B44" s="2">
-        <v>2043</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D44" s="11">
-        <v>45497</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F44" s="3">
-        <v>0</v>
-      </c>
-      <c r="G44" s="4">
-        <v>0</v>
-      </c>
-      <c r="H44" s="4">
-        <v>0</v>
-      </c>
-      <c r="I44" s="4">
-        <v>0</v>
-      </c>
-      <c r="J44" s="3">
-        <v>0</v>
-      </c>
-      <c r="K44" s="4">
-        <v>0</v>
-      </c>
-      <c r="L44" s="4">
-        <v>1558.85</v>
-      </c>
-      <c r="M44" s="4">
-        <v>1558.85</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A45" s="2">
-        <v>94156</v>
       </c>
       <c r="B45" s="2">
         <v>2043</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D45" s="11">
-        <v>44159</v>
+        <v>45497</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>54</v>
@@ -2832,19 +2832,19 @@
         <v>0</v>
       </c>
       <c r="J45" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K45" s="4">
-        <v>2285.38</v>
+        <v>0</v>
       </c>
       <c r="L45" s="4">
-        <v>5124.38</v>
+        <v>1558.85</v>
       </c>
       <c r="M45" s="4">
-        <v>7409.76</v>
-      </c>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
+        <v>1558.85</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13">
       <c r="A46" s="2">
         <v>81618</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>14949.86</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:13">
       <c r="A47" s="2">
         <v>63441</v>
       </c>
@@ -2926,7 +2926,7 @@
         <v>10965.01</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:13">
       <c r="A48" s="2">
         <v>113450</v>
       </c>

</xml_diff>

<commit_message>
chore: update report data to March 26 and sync snapshot
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A27D4F6B-40CC-8143-9D7D-7DE4422CCAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96A724BE-EBED-0E4B-9867-B865E15DB370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -223,7 +223,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="#,##0.0_ ;\-#,##0.0\ "/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -379,163 +379,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="12">
     <dxf>
       <border>
         <top style="thin">
@@ -1026,7 +870,7 @@
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
   <dimension ref="A1:M48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.1640625" customWidth="1"/>
     <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
@@ -1041,16 +885,16 @@
     <col min="11" max="14" width="11.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="24">
+    <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46105</v>
+        <v>46107</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="8"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1081,7 +925,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1122,7 +966,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>87538</v>
       </c>
@@ -1145,25 +989,25 @@
         <v>391236.33</v>
       </c>
       <c r="H4" s="4">
-        <v>83391.67</v>
+        <v>92905.23</v>
       </c>
       <c r="I4" s="4">
-        <v>474628</v>
+        <v>484141.56</v>
       </c>
       <c r="J4" s="5">
         <v>1</v>
       </c>
       <c r="K4" s="4">
-        <v>93758.720000000001</v>
+        <v>71561.37</v>
       </c>
       <c r="L4" s="4">
-        <v>330572.40000000002</v>
+        <v>321058.83</v>
       </c>
       <c r="M4" s="4">
-        <v>424331.12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
+        <v>392620.2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>80122</v>
       </c>
@@ -1180,31 +1024,31 @@
         <v>54</v>
       </c>
       <c r="F5" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5" s="4">
-        <v>99798.14</v>
+        <v>106144.53</v>
       </c>
       <c r="H5" s="4">
         <v>12339.99</v>
       </c>
       <c r="I5" s="4">
-        <v>112138.13</v>
+        <v>118484.52</v>
       </c>
       <c r="J5" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" s="4">
-        <v>6346.39</v>
+        <v>0</v>
       </c>
       <c r="L5" s="4">
         <v>115544.18</v>
       </c>
       <c r="M5" s="4">
-        <v>121890.57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
+        <v>115544.18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>110453</v>
       </c>
@@ -1245,7 +1089,7 @@
         <v>175553.93</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>104750</v>
       </c>
@@ -1286,7 +1130,7 @@
         <v>62375.6</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>115047</v>
       </c>
@@ -1327,33 +1171,33 @@
         <v>32922.42</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>105696</v>
+        <v>107488</v>
       </c>
       <c r="B9" s="2">
         <v>2043</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D9" s="11">
-        <v>45279</v>
+        <v>45440</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F9" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" s="4">
-        <v>31875.97</v>
+        <v>0</v>
       </c>
       <c r="H9" s="4">
-        <v>9320.44</v>
+        <v>42987.72</v>
       </c>
       <c r="I9" s="4">
-        <v>41196.410000000003</v>
+        <v>42987.72</v>
       </c>
       <c r="J9" s="3">
         <v>0</v>
@@ -1362,39 +1206,39 @@
         <v>0</v>
       </c>
       <c r="L9" s="4">
-        <v>27850.23</v>
+        <v>125975.29</v>
       </c>
       <c r="M9" s="4">
-        <v>27850.23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
+        <v>125975.29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>107488</v>
+        <v>105696</v>
       </c>
       <c r="B10" s="2">
         <v>2043</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D10" s="11">
-        <v>45440</v>
+        <v>45279</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F10" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="4">
-        <v>0</v>
+        <v>31875.97</v>
       </c>
       <c r="H10" s="4">
-        <v>38679.050000000003</v>
+        <v>11041.22</v>
       </c>
       <c r="I10" s="4">
-        <v>38679.050000000003</v>
+        <v>42917.19</v>
       </c>
       <c r="J10" s="3">
         <v>0</v>
@@ -1403,13 +1247,13 @@
         <v>0</v>
       </c>
       <c r="L10" s="4">
-        <v>125975.29</v>
+        <v>26129.439999999999</v>
       </c>
       <c r="M10" s="4">
-        <v>125975.29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
+        <v>26129.439999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>104718</v>
       </c>
@@ -1450,18 +1294,18 @@
         <v>104191.1</v>
       </c>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>114157</v>
+        <v>65046</v>
       </c>
       <c r="B12" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D12" s="11">
-        <v>45904</v>
+        <v>44763</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>54</v>
@@ -1470,136 +1314,136 @@
         <v>1</v>
       </c>
       <c r="G12" s="4">
+        <v>1448.05</v>
+      </c>
+      <c r="H12" s="4">
+        <v>26508.94</v>
+      </c>
+      <c r="I12" s="4">
+        <v>27956.99</v>
+      </c>
+      <c r="J12" s="3">
+        <v>0</v>
+      </c>
+      <c r="K12" s="4">
+        <v>0</v>
+      </c>
+      <c r="L12" s="4">
+        <v>20012.810000000001</v>
+      </c>
+      <c r="M12" s="4">
+        <v>20012.810000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A13" s="2">
+        <v>114157</v>
+      </c>
+      <c r="B13" s="2">
+        <v>2692</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="11">
+        <v>45904</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F13" s="3">
+        <v>1</v>
+      </c>
+      <c r="G13" s="4">
         <v>1684.95</v>
       </c>
-      <c r="H12" s="4">
-        <v>13292.63</v>
-      </c>
-      <c r="I12" s="4">
-        <v>14977.58</v>
-      </c>
-      <c r="J12" s="3">
-        <v>0</v>
-      </c>
-      <c r="K12" s="4">
-        <v>0</v>
-      </c>
-      <c r="L12" s="4">
-        <v>68730.09</v>
-      </c>
-      <c r="M12" s="4">
-        <v>68730.09</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13">
-      <c r="A13" s="2">
+      <c r="H13" s="4">
+        <v>15671</v>
+      </c>
+      <c r="I13" s="4">
+        <v>17355.95</v>
+      </c>
+      <c r="J13" s="3">
+        <v>0</v>
+      </c>
+      <c r="K13" s="4">
+        <v>0</v>
+      </c>
+      <c r="L13" s="4">
+        <v>66351.72</v>
+      </c>
+      <c r="M13" s="4">
+        <v>66351.72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A14" s="2">
         <v>90355</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B14" s="2">
         <v>2043</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D13" s="11">
+      <c r="D14" s="11">
         <v>43949</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F13" s="3">
-        <v>0</v>
-      </c>
-      <c r="G13" s="4">
-        <v>0</v>
-      </c>
-      <c r="H13" s="4">
+      <c r="E14" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="3">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4">
+        <v>0</v>
+      </c>
+      <c r="H14" s="4">
         <v>13410.43</v>
       </c>
-      <c r="I13" s="4">
+      <c r="I14" s="4">
         <v>13410.43</v>
       </c>
-      <c r="J13" s="3">
-        <v>0</v>
-      </c>
-      <c r="K13" s="4">
-        <v>0</v>
-      </c>
-      <c r="L13" s="4">
+      <c r="J14" s="3">
+        <v>0</v>
+      </c>
+      <c r="K14" s="4">
+        <v>0</v>
+      </c>
+      <c r="L14" s="4">
         <v>32434.68</v>
       </c>
-      <c r="M13" s="4">
+      <c r="M14" s="4">
         <v>32434.68</v>
       </c>
     </row>
-    <row r="14" spans="1:13">
-      <c r="A14" s="2">
-        <v>116883</v>
-      </c>
-      <c r="B14" s="2">
-        <v>2856</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D14" s="11">
-        <v>46007</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F14" s="3">
-        <v>2</v>
-      </c>
-      <c r="G14" s="4">
-        <v>7008.07</v>
-      </c>
-      <c r="H14" s="4">
-        <v>4010.74</v>
-      </c>
-      <c r="I14" s="4">
-        <v>11018.81</v>
-      </c>
-      <c r="J14" s="3">
-        <v>0</v>
-      </c>
-      <c r="K14" s="4">
-        <v>0</v>
-      </c>
-      <c r="L14" s="4">
-        <v>41489.449999999997</v>
-      </c>
-      <c r="M14" s="4">
-        <v>41489.449999999997</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>80925</v>
+        <v>117440</v>
       </c>
       <c r="B15" s="2">
         <v>2043</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="D15" s="11">
-        <v>43439</v>
+        <v>46059</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F15" s="3">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G15" s="4">
-        <v>0</v>
+        <v>7435.48</v>
       </c>
       <c r="H15" s="4">
-        <v>10230.700000000001</v>
+        <v>5452</v>
       </c>
       <c r="I15" s="4">
-        <v>10230.700000000001</v>
+        <v>12887.48</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1614,115 +1458,115 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>94205</v>
+        <v>116883</v>
       </c>
       <c r="B16" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="D16" s="11">
-        <v>44116</v>
+        <v>46007</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F16" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G16" s="4">
-        <v>0</v>
+        <v>7008.07</v>
       </c>
       <c r="H16" s="4">
-        <v>10135.31</v>
+        <v>4010.74</v>
       </c>
       <c r="I16" s="4">
-        <v>10135.31</v>
+        <v>11018.81</v>
       </c>
       <c r="J16" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" s="4">
-        <v>0</v>
+        <v>1722.61</v>
       </c>
       <c r="L16" s="4">
-        <v>0</v>
+        <v>60438.19</v>
       </c>
       <c r="M16" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13">
+        <v>62160.800000000003</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>117440</v>
+        <v>80925</v>
       </c>
       <c r="B17" s="2">
         <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="D17" s="11">
-        <v>46059</v>
+        <v>43439</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F17" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G17" s="4">
-        <v>5692.2</v>
+        <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>4226.8900000000003</v>
+        <v>10230.700000000001</v>
       </c>
       <c r="I17" s="4">
-        <v>9919.09</v>
+        <v>10230.700000000001</v>
       </c>
       <c r="J17" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K17" s="4">
-        <v>2967.98</v>
+        <v>0</v>
       </c>
       <c r="L17" s="4">
         <v>0</v>
       </c>
       <c r="M17" s="4">
-        <v>2967.98</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>106018</v>
+        <v>94205</v>
       </c>
       <c r="B18" s="2">
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="D18" s="11">
-        <v>45344</v>
+        <v>44116</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F18" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" s="4">
-        <v>580.95000000000005</v>
+        <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>8612.6200000000008</v>
+        <v>10135.31</v>
       </c>
       <c r="I18" s="4">
-        <v>9193.57</v>
+        <v>10135.31</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1731,39 +1575,39 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>22590.41</v>
+        <v>0</v>
       </c>
       <c r="M18" s="4">
-        <v>22590.41</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>110105</v>
+        <v>106018</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="D19" s="11">
-        <v>45560</v>
+        <v>45344</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" s="4">
-        <v>0</v>
+        <v>580.95000000000005</v>
       </c>
       <c r="H19" s="4">
-        <v>8858.33</v>
+        <v>8612.6200000000008</v>
       </c>
       <c r="I19" s="4">
-        <v>8858.33</v>
+        <v>9193.57</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1772,24 +1616,24 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>7719.98</v>
+        <v>22590.41</v>
       </c>
       <c r="M19" s="4">
-        <v>7719.98</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13">
+        <v>22590.41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>114100</v>
+        <v>113076</v>
       </c>
       <c r="B20" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="D20" s="11">
-        <v>45863</v>
+        <v>45806</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>54</v>
@@ -1801,10 +1645,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>8427.17</v>
+        <v>8861.9</v>
       </c>
       <c r="I20" s="4">
-        <v>8427.17</v>
+        <v>8861.9</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1813,244 +1657,244 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>53325.32</v>
+        <v>13572.34</v>
       </c>
       <c r="M20" s="4">
-        <v>53325.32</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13">
+        <v>13572.34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>100677</v>
+        <v>110105</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="11">
+        <v>45560</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F21" s="3">
+        <v>0</v>
+      </c>
+      <c r="G21" s="4">
+        <v>0</v>
+      </c>
+      <c r="H21" s="4">
+        <v>8858.33</v>
+      </c>
+      <c r="I21" s="4">
+        <v>8858.33</v>
+      </c>
+      <c r="J21" s="3">
+        <v>0</v>
+      </c>
+      <c r="K21" s="4">
+        <v>0</v>
+      </c>
+      <c r="L21" s="4">
+        <v>7719.98</v>
+      </c>
+      <c r="M21" s="4">
+        <v>7719.98</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A22" s="2">
+        <v>114100</v>
+      </c>
+      <c r="B22" s="2">
+        <v>2856</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="11">
+        <v>45863</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F22" s="3">
+        <v>0</v>
+      </c>
+      <c r="G22" s="4">
+        <v>0</v>
+      </c>
+      <c r="H22" s="4">
+        <v>8427.17</v>
+      </c>
+      <c r="I22" s="4">
+        <v>8427.17</v>
+      </c>
+      <c r="J22" s="3">
+        <v>0</v>
+      </c>
+      <c r="K22" s="4">
+        <v>0</v>
+      </c>
+      <c r="L22" s="4">
+        <v>53325.32</v>
+      </c>
+      <c r="M22" s="4">
+        <v>53325.32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A23" s="2">
+        <v>100677</v>
+      </c>
+      <c r="B23" s="2">
+        <v>2043</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D23" s="11">
         <v>44999</v>
       </c>
-      <c r="E21" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F21" s="3">
-        <v>0</v>
-      </c>
-      <c r="G21" s="4">
-        <v>0</v>
-      </c>
-      <c r="H21" s="4">
+      <c r="E23" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F23" s="3">
+        <v>0</v>
+      </c>
+      <c r="G23" s="4">
+        <v>0</v>
+      </c>
+      <c r="H23" s="4">
         <v>8062.37</v>
       </c>
-      <c r="I21" s="4">
+      <c r="I23" s="4">
         <v>8062.37</v>
       </c>
-      <c r="J21" s="3">
-        <v>0</v>
-      </c>
-      <c r="K21" s="4">
-        <v>0</v>
-      </c>
-      <c r="L21" s="4">
+      <c r="J23" s="3">
+        <v>0</v>
+      </c>
+      <c r="K23" s="4">
+        <v>0</v>
+      </c>
+      <c r="L23" s="4">
         <v>18028.54</v>
       </c>
-      <c r="M21" s="4">
+      <c r="M23" s="4">
         <v>18028.54</v>
       </c>
     </row>
-    <row r="22" spans="1:13">
-      <c r="A22" s="2">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A24" s="2">
+        <v>109007</v>
+      </c>
+      <c r="B24" s="2">
+        <v>2043</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D24" s="11">
+        <v>45525</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F24" s="3">
+        <v>0</v>
+      </c>
+      <c r="G24" s="4">
+        <v>0</v>
+      </c>
+      <c r="H24" s="4">
+        <v>7858.27</v>
+      </c>
+      <c r="I24" s="4">
+        <v>7858.27</v>
+      </c>
+      <c r="J24" s="3">
+        <v>0</v>
+      </c>
+      <c r="K24" s="4">
+        <v>0</v>
+      </c>
+      <c r="L24" s="4">
+        <v>0</v>
+      </c>
+      <c r="M24" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A25" s="2">
         <v>108405</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B25" s="2">
         <v>2692</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C25" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D25" s="11">
         <v>45471</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F22" s="3">
-        <v>0</v>
-      </c>
-      <c r="G22" s="4">
-        <v>0</v>
-      </c>
-      <c r="H22" s="4">
+      <c r="E25" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F25" s="3">
+        <v>0</v>
+      </c>
+      <c r="G25" s="4">
+        <v>0</v>
+      </c>
+      <c r="H25" s="4">
         <v>7485.18</v>
       </c>
-      <c r="I22" s="4">
+      <c r="I25" s="4">
         <v>7485.18</v>
       </c>
-      <c r="J22" s="3">
-        <v>0</v>
-      </c>
-      <c r="K22" s="4">
-        <v>0</v>
-      </c>
-      <c r="L22" s="4">
+      <c r="J25" s="3">
+        <v>0</v>
+      </c>
+      <c r="K25" s="4">
+        <v>0</v>
+      </c>
+      <c r="L25" s="4">
         <v>34981.11</v>
       </c>
-      <c r="M22" s="4">
+      <c r="M25" s="4">
         <v>34981.11</v>
       </c>
     </row>
-    <row r="23" spans="1:13">
-      <c r="A23" s="2">
-        <v>108404</v>
-      </c>
-      <c r="B23" s="2">
-        <v>2692</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D23" s="11">
-        <v>45467</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F23" s="3">
-        <v>0</v>
-      </c>
-      <c r="G23" s="4">
-        <v>0</v>
-      </c>
-      <c r="H23" s="4">
-        <v>5851.31</v>
-      </c>
-      <c r="I23" s="4">
-        <v>5851.31</v>
-      </c>
-      <c r="J23" s="3">
-        <v>0</v>
-      </c>
-      <c r="K23" s="4">
-        <v>0</v>
-      </c>
-      <c r="L23" s="4">
-        <v>42989.04</v>
-      </c>
-      <c r="M23" s="4">
-        <v>42989.04</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13">
-      <c r="A24" s="2">
-        <v>111056</v>
-      </c>
-      <c r="B24" s="2">
-        <v>2692</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" s="11">
-        <v>45639</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F24" s="3">
-        <v>0</v>
-      </c>
-      <c r="G24" s="4">
-        <v>0</v>
-      </c>
-      <c r="H24" s="4">
-        <v>5403.95</v>
-      </c>
-      <c r="I24" s="4">
-        <v>5403.95</v>
-      </c>
-      <c r="J24" s="3">
-        <v>0</v>
-      </c>
-      <c r="K24" s="4">
-        <v>0</v>
-      </c>
-      <c r="L24" s="4">
-        <v>61189.599999999999</v>
-      </c>
-      <c r="M24" s="4">
-        <v>61189.599999999999</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13">
-      <c r="A25" s="2">
-        <v>47116</v>
-      </c>
-      <c r="B25" s="2">
-        <v>2043</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D25" s="11">
-        <v>44616</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F25" s="3">
-        <v>0</v>
-      </c>
-      <c r="G25" s="4">
-        <v>0</v>
-      </c>
-      <c r="H25" s="4">
-        <v>5188.62</v>
-      </c>
-      <c r="I25" s="4">
-        <v>5188.62</v>
-      </c>
-      <c r="J25" s="3">
-        <v>0</v>
-      </c>
-      <c r="K25" s="4">
-        <v>0</v>
-      </c>
-      <c r="L25" s="4">
-        <v>85626.41</v>
-      </c>
-      <c r="M25" s="4">
-        <v>85626.41</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>90177</v>
+        <v>94156</v>
       </c>
       <c r="B26" s="2">
         <v>2043</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D26" s="11">
-        <v>43949</v>
+        <v>44159</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F26" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G26" s="4">
-        <v>0</v>
+        <v>1421.55</v>
       </c>
       <c r="H26" s="4">
-        <v>5160.08</v>
+        <v>5466.12</v>
       </c>
       <c r="I26" s="4">
-        <v>5160.08</v>
+        <v>6887.67</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2059,13 +1903,13 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>5160.08</v>
+        <v>0</v>
       </c>
       <c r="M26" s="4">
-        <v>5160.08</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
         <v>116060</v>
       </c>
@@ -2088,10 +1932,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>4927.55</v>
+        <v>6744.33</v>
       </c>
       <c r="I27" s="4">
-        <v>4927.55</v>
+        <v>6744.33</v>
       </c>
       <c r="J27" s="3">
         <v>0</v>
@@ -2100,24 +1944,24 @@
         <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>42294.77</v>
+        <v>40477.99</v>
       </c>
       <c r="M27" s="4">
-        <v>42294.77</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13">
+        <v>40477.99</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>94156</v>
+        <v>108404</v>
       </c>
       <c r="B28" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="D28" s="11">
-        <v>44159</v>
+        <v>45467</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>54</v>
@@ -2129,36 +1973,36 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>4602.76</v>
+        <v>5851.31</v>
       </c>
       <c r="I28" s="4">
-        <v>4602.76</v>
+        <v>5851.31</v>
       </c>
       <c r="J28" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" s="4">
-        <v>2285.38</v>
+        <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>0</v>
+        <v>40999.71</v>
       </c>
       <c r="M28" s="4">
-        <v>2285.38</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13">
+        <v>40999.71</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>113076</v>
+        <v>47116</v>
       </c>
       <c r="B29" s="2">
         <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="D29" s="11">
-        <v>45806</v>
+        <v>44616</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>54</v>
@@ -2170,10 +2014,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>4524.1099999999997</v>
+        <v>5700.86</v>
       </c>
       <c r="I29" s="4">
-        <v>4524.1099999999997</v>
+        <v>5700.86</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2182,24 +2026,24 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>13572.34</v>
+        <v>69913.55</v>
       </c>
       <c r="M29" s="4">
-        <v>13572.34</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13">
+        <v>69913.55</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>104343</v>
+        <v>111056</v>
       </c>
       <c r="B30" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="D30" s="11">
-        <v>45201</v>
+        <v>45639</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>54</v>
@@ -2211,10 +2055,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>4424.0600000000004</v>
+        <v>5403.95</v>
       </c>
       <c r="I30" s="4">
-        <v>4424.0600000000004</v>
+        <v>5403.95</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2223,24 +2067,24 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>43343.73</v>
+        <v>61189.599999999999</v>
       </c>
       <c r="M30" s="4">
-        <v>43343.73</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13">
+        <v>61189.599999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>88234</v>
+        <v>90177</v>
       </c>
       <c r="B31" s="2">
         <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="D31" s="11">
-        <v>43794</v>
+        <v>43949</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>54</v>
@@ -2252,10 +2096,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>4210.32</v>
+        <v>5160.08</v>
       </c>
       <c r="I31" s="4">
-        <v>4210.32</v>
+        <v>5160.08</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -2264,24 +2108,24 @@
         <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>19836.599999999999</v>
+        <v>5160.08</v>
       </c>
       <c r="M31" s="4">
-        <v>19836.599999999999</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13">
+        <v>5160.08</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>95148</v>
+        <v>104343</v>
       </c>
       <c r="B32" s="2">
         <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="D32" s="11">
-        <v>44916</v>
+        <v>45201</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>54</v>
@@ -2293,10 +2137,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>3858.24</v>
+        <v>4424.0600000000004</v>
       </c>
       <c r="I32" s="4">
-        <v>3858.24</v>
+        <v>4424.0600000000004</v>
       </c>
       <c r="J32" s="3">
         <v>0</v>
@@ -2305,24 +2149,24 @@
         <v>0</v>
       </c>
       <c r="L32" s="4">
-        <v>0</v>
+        <v>40395.040000000001</v>
       </c>
       <c r="M32" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13">
+        <v>40395.040000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>109007</v>
+        <v>88234</v>
       </c>
       <c r="B33" s="2">
         <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="D33" s="11">
-        <v>45525</v>
+        <v>43794</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>54</v>
@@ -2334,10 +2178,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>3058.98</v>
+        <v>4210.32</v>
       </c>
       <c r="I33" s="4">
-        <v>3058.98</v>
+        <v>4210.32</v>
       </c>
       <c r="J33" s="3">
         <v>0</v>
@@ -2346,229 +2190,229 @@
         <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>0</v>
+        <v>19836.599999999999</v>
       </c>
       <c r="M33" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13">
+        <v>19836.599999999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>109998</v>
+        <v>95148</v>
       </c>
       <c r="B34" s="2">
         <v>2043</v>
       </c>
       <c r="C34" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D34" s="11">
+        <v>44916</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F34" s="3">
+        <v>0</v>
+      </c>
+      <c r="G34" s="4">
+        <v>0</v>
+      </c>
+      <c r="H34" s="4">
+        <v>3858.24</v>
+      </c>
+      <c r="I34" s="4">
+        <v>3858.24</v>
+      </c>
+      <c r="J34" s="3">
+        <v>0</v>
+      </c>
+      <c r="K34" s="4">
+        <v>0</v>
+      </c>
+      <c r="L34" s="4">
+        <v>0</v>
+      </c>
+      <c r="M34" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A35" s="2">
+        <v>114431</v>
+      </c>
+      <c r="B35" s="2">
+        <v>2692</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D35" s="11">
+        <v>45930</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F35" s="3">
+        <v>0</v>
+      </c>
+      <c r="G35" s="4">
+        <v>0</v>
+      </c>
+      <c r="H35" s="4">
+        <v>3405.55</v>
+      </c>
+      <c r="I35" s="4">
+        <v>3405.55</v>
+      </c>
+      <c r="J35" s="3">
+        <v>0</v>
+      </c>
+      <c r="K35" s="4">
+        <v>0</v>
+      </c>
+      <c r="L35" s="4">
+        <v>40155.160000000003</v>
+      </c>
+      <c r="M35" s="4">
+        <v>40155.160000000003</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A36" s="2">
+        <v>109998</v>
+      </c>
+      <c r="B36" s="2">
+        <v>2043</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D34" s="11">
+      <c r="D36" s="11">
         <v>45596</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F34" s="3">
-        <v>0</v>
-      </c>
-      <c r="G34" s="4">
-        <v>0</v>
-      </c>
-      <c r="H34" s="4">
+      <c r="E36" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F36" s="3">
+        <v>0</v>
+      </c>
+      <c r="G36" s="4">
+        <v>0</v>
+      </c>
+      <c r="H36" s="4">
         <v>2844.92</v>
       </c>
-      <c r="I34" s="4">
+      <c r="I36" s="4">
         <v>2844.92</v>
       </c>
-      <c r="J34" s="3">
-        <v>0</v>
-      </c>
-      <c r="K34" s="4">
-        <v>0</v>
-      </c>
-      <c r="L34" s="4">
-        <v>0</v>
-      </c>
-      <c r="M34" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:13">
-      <c r="A35" s="2">
-        <v>65046</v>
-      </c>
-      <c r="B35" s="2">
+      <c r="J36" s="3">
+        <v>0</v>
+      </c>
+      <c r="K36" s="4">
+        <v>0</v>
+      </c>
+      <c r="L36" s="4">
+        <v>0</v>
+      </c>
+      <c r="M36" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A37" s="2">
+        <v>81044</v>
+      </c>
+      <c r="B37" s="2">
+        <v>2511</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D37" s="11">
+        <v>44872</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F37" s="3">
+        <v>0</v>
+      </c>
+      <c r="G37" s="4">
+        <v>0</v>
+      </c>
+      <c r="H37" s="4">
+        <v>2385.52</v>
+      </c>
+      <c r="I37" s="4">
+        <v>2385.52</v>
+      </c>
+      <c r="J37" s="3">
+        <v>0</v>
+      </c>
+      <c r="K37" s="4">
+        <v>0</v>
+      </c>
+      <c r="L37" s="4">
+        <v>0</v>
+      </c>
+      <c r="M37" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A38" s="2">
+        <v>115404</v>
+      </c>
+      <c r="B38" s="2">
         <v>2043</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D35" s="11">
-        <v>44763</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F35" s="3">
-        <v>0</v>
-      </c>
-      <c r="G35" s="4">
-        <v>0</v>
-      </c>
-      <c r="H35" s="4">
-        <v>2759.08</v>
-      </c>
-      <c r="I35" s="4">
-        <v>2759.08</v>
-      </c>
-      <c r="J35" s="3">
-        <v>1</v>
-      </c>
-      <c r="K35" s="4">
-        <v>25197.91</v>
-      </c>
-      <c r="L35" s="4">
-        <v>20012.810000000001</v>
-      </c>
-      <c r="M35" s="4">
-        <v>45210.720000000001</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13">
-      <c r="A36" s="2">
-        <v>81044</v>
-      </c>
-      <c r="B36" s="2">
-        <v>2511</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D36" s="11">
-        <v>44872</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F36" s="3">
-        <v>0</v>
-      </c>
-      <c r="G36" s="4">
-        <v>0</v>
-      </c>
-      <c r="H36" s="4">
-        <v>2385.52</v>
-      </c>
-      <c r="I36" s="4">
-        <v>2385.52</v>
-      </c>
-      <c r="J36" s="3">
-        <v>0</v>
-      </c>
-      <c r="K36" s="4">
-        <v>0</v>
-      </c>
-      <c r="L36" s="4">
-        <v>0</v>
-      </c>
-      <c r="M36" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:13">
-      <c r="A37" s="2">
+      <c r="C38" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D38" s="11">
+        <v>45986</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F38" s="3">
+        <v>0</v>
+      </c>
+      <c r="G38" s="4">
+        <v>0</v>
+      </c>
+      <c r="H38" s="4">
+        <v>2379.42</v>
+      </c>
+      <c r="I38" s="4">
+        <v>2379.42</v>
+      </c>
+      <c r="J38" s="3">
+        <v>0</v>
+      </c>
+      <c r="K38" s="4">
+        <v>0</v>
+      </c>
+      <c r="L38" s="4">
+        <v>43605.03</v>
+      </c>
+      <c r="M38" s="4">
+        <v>43605.03</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A39" s="2">
         <v>101640</v>
-      </c>
-      <c r="B37" s="2">
-        <v>2043</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D37" s="11">
-        <v>45104</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F37" s="3">
-        <v>0</v>
-      </c>
-      <c r="G37" s="4">
-        <v>0</v>
-      </c>
-      <c r="H37" s="4">
-        <v>2316.9899999999998</v>
-      </c>
-      <c r="I37" s="4">
-        <v>2316.9899999999998</v>
-      </c>
-      <c r="J37" s="3">
-        <v>0</v>
-      </c>
-      <c r="K37" s="4">
-        <v>0</v>
-      </c>
-      <c r="L37" s="4">
-        <v>5546.81</v>
-      </c>
-      <c r="M37" s="4">
-        <v>5546.81</v>
-      </c>
-    </row>
-    <row r="38" spans="1:13">
-      <c r="A38" s="2">
-        <v>116876</v>
-      </c>
-      <c r="B38" s="2">
-        <v>2856</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D38" s="11">
-        <v>46006</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F38" s="3">
-        <v>0</v>
-      </c>
-      <c r="G38" s="4">
-        <v>0</v>
-      </c>
-      <c r="H38" s="4">
-        <v>2005.37</v>
-      </c>
-      <c r="I38" s="4">
-        <v>2005.37</v>
-      </c>
-      <c r="J38" s="3">
-        <v>0</v>
-      </c>
-      <c r="K38" s="4">
-        <v>0</v>
-      </c>
-      <c r="L38" s="4">
-        <v>20053.7</v>
-      </c>
-      <c r="M38" s="4">
-        <v>20053.7</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13">
-      <c r="A39" s="2">
-        <v>102825</v>
       </c>
       <c r="B39" s="2">
         <v>2043</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D39" s="11">
-        <v>45117</v>
+        <v>45104</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>54</v>
@@ -2580,10 +2424,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="4">
-        <v>1742.75</v>
+        <v>2316.9899999999998</v>
       </c>
       <c r="I39" s="4">
-        <v>1742.75</v>
+        <v>2316.9899999999998</v>
       </c>
       <c r="J39" s="3">
         <v>0</v>
@@ -2592,24 +2436,24 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>23216.76</v>
+        <v>5546.81</v>
       </c>
       <c r="M39" s="4">
-        <v>23216.76</v>
-      </c>
-    </row>
-    <row r="40" spans="1:13">
+        <v>5546.81</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>112522</v>
+        <v>116876</v>
       </c>
       <c r="B40" s="2">
         <v>2856</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D40" s="11">
-        <v>45776</v>
+        <v>46006</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>54</v>
@@ -2621,10 +2465,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="4">
-        <v>1737.52</v>
+        <v>2005.37</v>
       </c>
       <c r="I40" s="4">
-        <v>1737.52</v>
+        <v>2005.37</v>
       </c>
       <c r="J40" s="3">
         <v>0</v>
@@ -2633,24 +2477,24 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>6634.38</v>
+        <v>20053.7</v>
       </c>
       <c r="M40" s="4">
-        <v>6634.38</v>
-      </c>
-    </row>
-    <row r="41" spans="1:13">
+        <v>20053.7</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>114431</v>
+        <v>63441</v>
       </c>
       <c r="B41" s="2">
-        <v>2692</v>
+        <v>2511</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="D41" s="11">
-        <v>45930</v>
+        <v>44733</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>54</v>
@@ -2662,10 +2506,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="4">
-        <v>1676.4</v>
+        <v>1827.5</v>
       </c>
       <c r="I41" s="4">
-        <v>1676.4</v>
+        <v>1827.5</v>
       </c>
       <c r="J41" s="3">
         <v>0</v>
@@ -2674,259 +2518,259 @@
         <v>0</v>
       </c>
       <c r="L41" s="4">
-        <v>41884.31</v>
+        <v>9137.51</v>
       </c>
       <c r="M41" s="4">
-        <v>41884.31</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13">
+        <v>9137.51</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>116795</v>
+        <v>102825</v>
       </c>
       <c r="B42" s="2">
         <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D42" s="11">
+        <v>45117</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F42" s="3">
+        <v>0</v>
+      </c>
+      <c r="G42" s="4">
+        <v>0</v>
+      </c>
+      <c r="H42" s="4">
+        <v>1742.75</v>
+      </c>
+      <c r="I42" s="4">
+        <v>1742.75</v>
+      </c>
+      <c r="J42" s="3">
+        <v>0</v>
+      </c>
+      <c r="K42" s="4">
+        <v>0</v>
+      </c>
+      <c r="L42" s="4">
+        <v>23216.76</v>
+      </c>
+      <c r="M42" s="4">
+        <v>23216.76</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A43" s="2">
+        <v>112522</v>
+      </c>
+      <c r="B43" s="2">
+        <v>2856</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D43" s="11">
+        <v>45776</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F43" s="3">
+        <v>0</v>
+      </c>
+      <c r="G43" s="4">
+        <v>0</v>
+      </c>
+      <c r="H43" s="4">
+        <v>1737.52</v>
+      </c>
+      <c r="I43" s="4">
+        <v>1737.52</v>
+      </c>
+      <c r="J43" s="3">
+        <v>0</v>
+      </c>
+      <c r="K43" s="4">
+        <v>0</v>
+      </c>
+      <c r="L43" s="4">
+        <v>6634.38</v>
+      </c>
+      <c r="M43" s="4">
+        <v>6634.38</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A44" s="2">
+        <v>116795</v>
+      </c>
+      <c r="B44" s="2">
+        <v>2043</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D42" s="11">
+      <c r="D44" s="11">
         <v>46000</v>
       </c>
-      <c r="E42" s="2" t="s">
+      <c r="E44" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F42" s="3">
-        <v>0</v>
-      </c>
-      <c r="G42" s="4">
-        <v>0</v>
-      </c>
-      <c r="H42" s="4">
+      <c r="F44" s="3">
+        <v>0</v>
+      </c>
+      <c r="G44" s="4">
+        <v>0</v>
+      </c>
+      <c r="H44" s="4">
         <v>1582.15</v>
       </c>
-      <c r="I42" s="4">
+      <c r="I44" s="4">
         <v>1582.15</v>
       </c>
-      <c r="J42" s="3">
-        <v>0</v>
-      </c>
-      <c r="K42" s="4">
-        <v>0</v>
-      </c>
-      <c r="L42" s="4">
-        <v>0</v>
-      </c>
-      <c r="M42" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:13">
-      <c r="A43" s="2">
-        <v>115404</v>
-      </c>
-      <c r="B43" s="2">
-        <v>2043</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D43" s="11">
-        <v>45986</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F43" s="3">
-        <v>0</v>
-      </c>
-      <c r="G43" s="4">
-        <v>0</v>
-      </c>
-      <c r="H43" s="4">
-        <v>653.92999999999995</v>
-      </c>
-      <c r="I43" s="4">
-        <v>653.92999999999995</v>
-      </c>
-      <c r="J43" s="3">
-        <v>0</v>
-      </c>
-      <c r="K43" s="4">
-        <v>0</v>
-      </c>
-      <c r="L43" s="4">
-        <v>45330.52</v>
-      </c>
-      <c r="M43" s="4">
-        <v>45330.52</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13">
-      <c r="A44" s="2">
+      <c r="J44" s="3">
+        <v>0</v>
+      </c>
+      <c r="K44" s="4">
+        <v>0</v>
+      </c>
+      <c r="L44" s="4">
+        <v>0</v>
+      </c>
+      <c r="M44" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A45" s="2">
         <v>110575</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B45" s="2">
         <v>2692</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="C45" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D44" s="11">
+      <c r="D45" s="11">
         <v>45583</v>
       </c>
-      <c r="E44" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F44" s="3">
-        <v>0</v>
-      </c>
-      <c r="G44" s="4">
-        <v>0</v>
-      </c>
-      <c r="H44" s="4">
-        <v>0</v>
-      </c>
-      <c r="I44" s="4">
-        <v>0</v>
-      </c>
-      <c r="J44" s="3">
-        <v>0</v>
-      </c>
-      <c r="K44" s="4">
-        <v>0</v>
-      </c>
-      <c r="L44" s="4">
+      <c r="E45" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F45" s="3">
+        <v>0</v>
+      </c>
+      <c r="G45" s="4">
+        <v>0</v>
+      </c>
+      <c r="H45" s="4">
+        <v>0</v>
+      </c>
+      <c r="I45" s="4">
+        <v>0</v>
+      </c>
+      <c r="J45" s="3">
+        <v>0</v>
+      </c>
+      <c r="K45" s="4">
+        <v>0</v>
+      </c>
+      <c r="L45" s="4">
         <v>114218.2</v>
       </c>
-      <c r="M44" s="4">
+      <c r="M45" s="4">
         <v>114218.2</v>
       </c>
     </row>
-    <row r="45" spans="1:13">
-      <c r="A45" s="2">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A46" s="2">
         <v>108658</v>
-      </c>
-      <c r="B45" s="2">
-        <v>2043</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D45" s="11">
-        <v>45497</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F45" s="3">
-        <v>0</v>
-      </c>
-      <c r="G45" s="4">
-        <v>0</v>
-      </c>
-      <c r="H45" s="4">
-        <v>0</v>
-      </c>
-      <c r="I45" s="4">
-        <v>0</v>
-      </c>
-      <c r="J45" s="3">
-        <v>0</v>
-      </c>
-      <c r="K45" s="4">
-        <v>0</v>
-      </c>
-      <c r="L45" s="4">
-        <v>1558.85</v>
-      </c>
-      <c r="M45" s="4">
-        <v>1558.85</v>
-      </c>
-    </row>
-    <row r="46" spans="1:13">
-      <c r="A46" s="2">
-        <v>81618</v>
       </c>
       <c r="B46" s="2">
         <v>2043</v>
       </c>
       <c r="C46" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D46" s="11">
+        <v>45497</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F46" s="3">
+        <v>0</v>
+      </c>
+      <c r="G46" s="4">
+        <v>0</v>
+      </c>
+      <c r="H46" s="4">
+        <v>0</v>
+      </c>
+      <c r="I46" s="4">
+        <v>0</v>
+      </c>
+      <c r="J46" s="3">
+        <v>0</v>
+      </c>
+      <c r="K46" s="4">
+        <v>0</v>
+      </c>
+      <c r="L46" s="4">
+        <v>1558.85</v>
+      </c>
+      <c r="M46" s="4">
+        <v>1558.85</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A47" s="2">
+        <v>81618</v>
+      </c>
+      <c r="B47" s="2">
+        <v>2043</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D46" s="11">
+      <c r="D47" s="11">
         <v>43447</v>
       </c>
-      <c r="E46" s="2" t="s">
+      <c r="E47" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="F46" s="3">
-        <v>0</v>
-      </c>
-      <c r="G46" s="4">
-        <v>0</v>
-      </c>
-      <c r="H46" s="4">
-        <v>0</v>
-      </c>
-      <c r="I46" s="4">
-        <v>0</v>
-      </c>
-      <c r="J46" s="3">
-        <v>0</v>
-      </c>
-      <c r="K46" s="4">
-        <v>0</v>
-      </c>
-      <c r="L46" s="4">
+      <c r="F47" s="3">
+        <v>0</v>
+      </c>
+      <c r="G47" s="4">
+        <v>0</v>
+      </c>
+      <c r="H47" s="4">
+        <v>0</v>
+      </c>
+      <c r="I47" s="4">
+        <v>0</v>
+      </c>
+      <c r="J47" s="3">
+        <v>0</v>
+      </c>
+      <c r="K47" s="4">
+        <v>0</v>
+      </c>
+      <c r="L47" s="4">
         <v>14949.86</v>
       </c>
-      <c r="M46" s="4">
+      <c r="M47" s="4">
         <v>14949.86</v>
       </c>
     </row>
-    <row r="47" spans="1:13">
-      <c r="A47" s="2">
-        <v>63441</v>
-      </c>
-      <c r="B47" s="2">
-        <v>2511</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D47" s="11">
-        <v>44733</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F47" s="3">
-        <v>0</v>
-      </c>
-      <c r="G47" s="4">
-        <v>0</v>
-      </c>
-      <c r="H47" s="4">
-        <v>0</v>
-      </c>
-      <c r="I47" s="4">
-        <v>0</v>
-      </c>
-      <c r="J47" s="3">
-        <v>0</v>
-      </c>
-      <c r="K47" s="4">
-        <v>0</v>
-      </c>
-      <c r="L47" s="4">
-        <v>10965.01</v>
-      </c>
-      <c r="M47" s="4">
-        <v>10965.01</v>
-      </c>
-    </row>
-    <row r="48" spans="1:13">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
         <v>113450</v>
       </c>
@@ -2969,55 +2813,55 @@
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="A5:A48 J5:J48">
-    <cfRule type="expression" dxfId="11" priority="4" stopIfTrue="1">
+  <conditionalFormatting sqref="A4:B4">
+    <cfRule type="expression" dxfId="11" priority="3" stopIfTrue="1">
+      <formula>$S$34=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:B48">
+    <cfRule type="expression" dxfId="10" priority="1" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="2" stopIfTrue="1">
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:L48 C5:H48">
-    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
+  <conditionalFormatting sqref="C4:H4 K4:L4">
+    <cfRule type="expression" dxfId="8" priority="11" stopIfTrue="1">
+      <formula>$S$34=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C5:H48 K5:L48">
+    <cfRule type="expression" dxfId="7" priority="6" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="7" stopIfTrue="1">
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="I4 M4">
+    <cfRule type="expression" dxfId="5" priority="12" stopIfTrue="1">
+      <formula>$S$34=1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="I5:I48 M5:M48">
-    <cfRule type="expression" dxfId="7" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="8" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="9" stopIfTrue="1">
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J4 A4">
-    <cfRule type="expression" dxfId="5" priority="10" stopIfTrue="1">
+  <conditionalFormatting sqref="J4">
+    <cfRule type="expression" dxfId="2" priority="10" stopIfTrue="1">
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C4:H4 K4:L4">
-    <cfRule type="expression" dxfId="4" priority="11" stopIfTrue="1">
-      <formula>$S$34=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I4 M4">
-    <cfRule type="expression" dxfId="3" priority="12" stopIfTrue="1">
-      <formula>$S$34=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B4">
-    <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
-      <formula>$S$34=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B48">
-    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="J5:J48">
+    <cfRule type="expression" dxfId="1" priority="4" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="5" stopIfTrue="1">
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-06 16:29)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D02405D-655A-A949-901D-2977A4C6737A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F2CE7F3-B86D-E84B-B777-F0BC66D9F983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="61">
   <si>
     <t>Asesor</t>
   </si>
@@ -213,6 +213,12 @@
   </si>
   <si>
     <t>KAREN MUÐOZ GARCIA</t>
+  </si>
+  <si>
+    <t>MARIO IVAN ROMERO GONZALEZ</t>
+  </si>
+  <si>
+    <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
   </si>
 </sst>
 </file>
@@ -1025,7 +1031,7 @@
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.1640625" customWidth="1"/>
@@ -1043,7 +1049,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1142,25 +1148,25 @@
         <v>4</v>
       </c>
       <c r="G4" s="4">
-        <v>394049.77</v>
+        <v>406177.63</v>
       </c>
       <c r="H4" s="4">
-        <v>113778.78</v>
+        <v>116388.43</v>
       </c>
       <c r="I4" s="4">
-        <v>507828.55</v>
+        <v>522566.06</v>
       </c>
       <c r="J4" s="5">
         <v>1</v>
       </c>
       <c r="K4" s="4">
-        <v>71561.37</v>
+        <v>72105.62</v>
       </c>
       <c r="L4" s="4">
-        <v>331133.08</v>
+        <v>338756.64</v>
       </c>
       <c r="M4" s="4">
-        <v>402694.45</v>
+        <v>410862.26</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1180,28 +1186,28 @@
         <v>54</v>
       </c>
       <c r="F5" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5" s="4">
-        <v>106144.53</v>
+        <v>178153.93</v>
       </c>
       <c r="H5" s="4">
-        <v>12339.99</v>
+        <v>12433.86</v>
       </c>
       <c r="I5" s="4">
-        <v>118484.52</v>
+        <v>190587.79</v>
       </c>
       <c r="J5" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K5" s="4">
-        <v>151343.35</v>
+        <v>84465.85</v>
       </c>
       <c r="L5" s="4">
-        <v>115544.18</v>
+        <v>116422.94</v>
       </c>
       <c r="M5" s="4">
-        <v>266887.53000000003</v>
+        <v>200888.79</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -1224,25 +1230,25 @@
         <v>1</v>
       </c>
       <c r="G6" s="4">
-        <v>1840.93</v>
+        <v>1854.93</v>
       </c>
       <c r="H6" s="4">
-        <v>79031.03</v>
+        <v>81364.38</v>
       </c>
       <c r="I6" s="4">
-        <v>80871.960000000006</v>
+        <v>83219.31</v>
       </c>
       <c r="J6" s="3">
         <v>1</v>
       </c>
       <c r="K6" s="4">
-        <v>1770.92</v>
+        <v>1784.38</v>
       </c>
       <c r="L6" s="4">
-        <v>173783.01</v>
+        <v>173372.39</v>
       </c>
       <c r="M6" s="4">
-        <v>175553.93</v>
+        <v>175156.77</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -1265,25 +1271,25 @@
         <v>2</v>
       </c>
       <c r="G7" s="4">
-        <v>32255.77</v>
+        <v>32501.09</v>
       </c>
       <c r="H7" s="4">
-        <v>41016.79</v>
+        <v>44335.51</v>
       </c>
       <c r="I7" s="4">
-        <v>73272.56</v>
+        <v>76836.600000000006</v>
       </c>
       <c r="J7" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K7" s="4">
-        <v>13126.46</v>
+        <v>28039.64</v>
       </c>
       <c r="L7" s="4">
-        <v>60303.09</v>
+        <v>57754.95</v>
       </c>
       <c r="M7" s="4">
-        <v>73429.55</v>
+        <v>85794.59</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
@@ -1309,10 +1315,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="4">
-        <v>62637.38</v>
+        <v>66591.3</v>
       </c>
       <c r="I8" s="4">
-        <v>62637.38</v>
+        <v>66591.3</v>
       </c>
       <c r="J8" s="3">
         <v>0</v>
@@ -1321,24 +1327,24 @@
         <v>0</v>
       </c>
       <c r="L8" s="4">
-        <v>106325.63</v>
+        <v>107694.21</v>
       </c>
       <c r="M8" s="4">
-        <v>106325.63</v>
+        <v>107694.21</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>115047</v>
+        <v>47116</v>
       </c>
       <c r="B9" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="D9" s="11">
-        <v>45944</v>
+        <v>44616</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>54</v>
@@ -1347,39 +1353,39 @@
         <v>1</v>
       </c>
       <c r="G9" s="4">
-        <v>1488.25</v>
+        <v>2117.52</v>
       </c>
       <c r="H9" s="4">
-        <v>44493.67</v>
+        <v>63467.86</v>
       </c>
       <c r="I9" s="4">
-        <v>45981.919999999998</v>
+        <v>65585.38</v>
       </c>
       <c r="J9" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" s="4">
-        <v>0</v>
+        <v>37033.42</v>
       </c>
       <c r="L9" s="4">
-        <v>32922.42</v>
+        <v>39817.339999999997</v>
       </c>
       <c r="M9" s="4">
-        <v>32922.42</v>
+        <v>76850.759999999995</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>105696</v>
+        <v>115047</v>
       </c>
       <c r="B10" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="D10" s="11">
-        <v>45279</v>
+        <v>45944</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>54</v>
@@ -1388,39 +1394,39 @@
         <v>1</v>
       </c>
       <c r="G10" s="4">
-        <v>31875.97</v>
+        <v>1499.56</v>
       </c>
       <c r="H10" s="4">
-        <v>12844.22</v>
+        <v>51080.26</v>
       </c>
       <c r="I10" s="4">
-        <v>44720.19</v>
+        <v>52579.82</v>
       </c>
       <c r="J10" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" s="4">
-        <v>35845.9</v>
+        <v>0</v>
       </c>
       <c r="L10" s="4">
-        <v>24326.44</v>
+        <v>31356.09</v>
       </c>
       <c r="M10" s="4">
-        <v>60172.34</v>
+        <v>31356.09</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>104718</v>
+        <v>105696</v>
       </c>
       <c r="B11" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="D11" s="11">
-        <v>45264</v>
+        <v>45279</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>54</v>
@@ -1429,54 +1435,54 @@
         <v>1</v>
       </c>
       <c r="G11" s="4">
-        <v>13028.98</v>
+        <v>32118.39</v>
       </c>
       <c r="H11" s="4">
-        <v>26254.29</v>
+        <v>14674.37</v>
       </c>
       <c r="I11" s="4">
-        <v>39283.269999999997</v>
+        <v>46792.76</v>
       </c>
       <c r="J11" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" s="4">
-        <v>0</v>
+        <v>36118.519999999997</v>
       </c>
       <c r="L11" s="4">
-        <v>100544.46</v>
+        <v>22778.99</v>
       </c>
       <c r="M11" s="4">
-        <v>100544.46</v>
+        <v>58897.51</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>115404</v>
+        <v>104718</v>
       </c>
       <c r="B12" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="D12" s="11">
-        <v>45986</v>
+        <v>45264</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" s="4">
-        <v>0</v>
+        <v>13128.07</v>
       </c>
       <c r="H12" s="4">
-        <v>33906.019999999997</v>
+        <v>26453.98</v>
       </c>
       <c r="I12" s="4">
-        <v>33906.019999999997</v>
+        <v>39582.050000000003</v>
       </c>
       <c r="J12" s="3">
         <v>0</v>
@@ -1485,24 +1491,24 @@
         <v>0</v>
       </c>
       <c r="L12" s="4">
-        <v>12078.43</v>
+        <v>101309.13</v>
       </c>
       <c r="M12" s="4">
-        <v>12078.43</v>
+        <v>101309.13</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>108405</v>
+        <v>115404</v>
       </c>
       <c r="B13" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="D13" s="11">
-        <v>45471</v>
+        <v>45986</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>54</v>
@@ -1514,10 +1520,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="4">
-        <v>33043.18</v>
+        <v>34822.78</v>
       </c>
       <c r="I13" s="4">
-        <v>33043.18</v>
+        <v>34822.78</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1526,24 +1532,24 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>9423.15</v>
+        <v>12170.29</v>
       </c>
       <c r="M13" s="4">
-        <v>9423.15</v>
+        <v>12170.29</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>47116</v>
+        <v>108405</v>
       </c>
       <c r="B14" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D14" s="11">
-        <v>44616</v>
+        <v>45471</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>54</v>
@@ -1555,10 +1561,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="4">
-        <v>29823.37</v>
+        <v>33294.480000000003</v>
       </c>
       <c r="I14" s="4">
-        <v>29823.37</v>
+        <v>33294.480000000003</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1567,10 +1573,10 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>39186.83</v>
+        <v>9494.81</v>
       </c>
       <c r="M14" s="4">
-        <v>39186.83</v>
+        <v>9494.81</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
@@ -1593,13 +1599,13 @@
         <v>1</v>
       </c>
       <c r="G15" s="4">
-        <v>1448.05</v>
+        <v>1459.06</v>
       </c>
       <c r="H15" s="4">
-        <v>26508.94</v>
+        <v>29490.62</v>
       </c>
       <c r="I15" s="4">
-        <v>27956.99</v>
+        <v>30949.68</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1608,10 +1614,10 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>20012.810000000001</v>
+        <v>17384.95</v>
       </c>
       <c r="M15" s="4">
-        <v>20012.810000000001</v>
+        <v>17384.95</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
@@ -1634,13 +1640,13 @@
         <v>1</v>
       </c>
       <c r="G16" s="4">
-        <v>1684.95</v>
+        <v>1697.76</v>
       </c>
       <c r="H16" s="4">
-        <v>15671</v>
+        <v>15790.19</v>
       </c>
       <c r="I16" s="4">
-        <v>17355.95</v>
+        <v>17487.95</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1649,10 +1655,10 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>66351.72</v>
+        <v>66856.350000000006</v>
       </c>
       <c r="M16" s="4">
-        <v>66351.72</v>
+        <v>66856.350000000006</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
@@ -1678,10 +1684,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>16666.28</v>
+        <v>16793.03</v>
       </c>
       <c r="I17" s="4">
-        <v>16666.28</v>
+        <v>16793.03</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1690,39 +1696,39 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>29178.83</v>
+        <v>29400.74</v>
       </c>
       <c r="M17" s="4">
-        <v>29178.83</v>
+        <v>29400.74</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>117440</v>
+        <v>104343</v>
       </c>
       <c r="B18" s="2">
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="D18" s="11">
-        <v>46059</v>
+        <v>45201</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F18" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G18" s="4">
-        <v>7435.48</v>
+        <v>10300.870000000001</v>
       </c>
       <c r="H18" s="4">
-        <v>7897.86</v>
+        <v>5495.48</v>
       </c>
       <c r="I18" s="4">
-        <v>15333.34</v>
+        <v>15796.35</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1731,39 +1737,39 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>0</v>
+        <v>49965.37</v>
       </c>
       <c r="M18" s="4">
-        <v>0</v>
+        <v>49965.37</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>80925</v>
+        <v>117440</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="D19" s="11">
-        <v>43439</v>
+        <v>46059</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F19" s="3">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G19" s="4">
-        <v>0</v>
+        <v>7492.03</v>
       </c>
       <c r="H19" s="4">
-        <v>14531</v>
+        <v>7957.91</v>
       </c>
       <c r="I19" s="4">
-        <v>14531</v>
+        <v>15449.94</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1780,16 +1786,16 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>110575</v>
+        <v>80925</v>
       </c>
       <c r="B20" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="D20" s="11">
-        <v>45583</v>
+        <v>43439</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>54</v>
@@ -1801,10 +1807,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>14277.28</v>
+        <v>14641.5</v>
       </c>
       <c r="I20" s="4">
-        <v>14277.28</v>
+        <v>14641.5</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1813,39 +1819,39 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>99940.93</v>
+        <v>0</v>
       </c>
       <c r="M20" s="4">
-        <v>99940.93</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>116883</v>
+        <v>110575</v>
       </c>
       <c r="B21" s="2">
-        <v>2856</v>
+        <v>2692</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D21" s="11">
-        <v>46007</v>
+        <v>45583</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F21" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G21" s="4">
-        <v>8730.68</v>
+        <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>4010.74</v>
+        <v>14385.86</v>
       </c>
       <c r="I21" s="4">
-        <v>12741.42</v>
+        <v>14385.86</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1854,39 +1860,39 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>60438.19</v>
+        <v>100701.01</v>
       </c>
       <c r="M21" s="4">
-        <v>60438.19</v>
+        <v>100701.01</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>100677</v>
+        <v>116883</v>
       </c>
       <c r="B22" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="D22" s="11">
-        <v>44999</v>
+        <v>46007</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F22" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G22" s="4">
-        <v>0</v>
+        <v>8797.08</v>
       </c>
       <c r="H22" s="4">
-        <v>10864.83</v>
+        <v>4041.24</v>
       </c>
       <c r="I22" s="4">
-        <v>10864.83</v>
+        <v>12838.32</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1895,39 +1901,39 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>18028.54</v>
+        <v>60897.84</v>
       </c>
       <c r="M22" s="4">
-        <v>18028.54</v>
+        <v>60897.84</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>94205</v>
+        <v>106018</v>
       </c>
       <c r="B23" s="2">
         <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="D23" s="11">
-        <v>44116</v>
+        <v>45344</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F23" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" s="4">
-        <v>0</v>
+        <v>585.37</v>
       </c>
       <c r="H23" s="4">
-        <v>10135.31</v>
+        <v>11777.23</v>
       </c>
       <c r="I23" s="4">
-        <v>10135.31</v>
+        <v>12362.6</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1936,39 +1942,39 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>0</v>
+        <v>22762.21</v>
       </c>
       <c r="M23" s="4">
-        <v>0</v>
+        <v>22762.21</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>106018</v>
+        <v>100677</v>
       </c>
       <c r="B24" s="2">
         <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D24" s="11">
-        <v>45344</v>
+        <v>44999</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F24" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" s="4">
-        <v>580.95000000000005</v>
+        <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>8612.6200000000008</v>
+        <v>10947.46</v>
       </c>
       <c r="I24" s="4">
-        <v>9193.57</v>
+        <v>10947.46</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1977,24 +1983,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>22590.41</v>
+        <v>18165.66</v>
       </c>
       <c r="M24" s="4">
-        <v>22590.41</v>
+        <v>18165.66</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>113076</v>
+        <v>114100</v>
       </c>
       <c r="B25" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="D25" s="11">
-        <v>45806</v>
+        <v>45863</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>54</v>
@@ -2006,10 +2012,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>8861.9</v>
+        <v>10901.34</v>
       </c>
       <c r="I25" s="4">
-        <v>8861.9</v>
+        <v>10901.34</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -2018,24 +2024,24 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>13572.34</v>
+        <v>53730.879999999997</v>
       </c>
       <c r="M25" s="4">
-        <v>13572.34</v>
+        <v>53730.879999999997</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>110105</v>
+        <v>111056</v>
       </c>
       <c r="B26" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="D26" s="11">
-        <v>45560</v>
+        <v>45639</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>54</v>
@@ -2047,10 +2053,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>8858.33</v>
+        <v>10890.1</v>
       </c>
       <c r="I26" s="4">
-        <v>8858.33</v>
+        <v>10890.1</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2059,24 +2065,24 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>7719.98</v>
+        <v>56209.91</v>
       </c>
       <c r="M26" s="4">
-        <v>7719.98</v>
+        <v>56209.91</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>116060</v>
+        <v>94205</v>
       </c>
       <c r="B27" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="D27" s="11">
-        <v>46010</v>
+        <v>44116</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>54</v>
@@ -2088,10 +2094,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>8428.93</v>
+        <v>10212.4</v>
       </c>
       <c r="I27" s="4">
-        <v>8428.93</v>
+        <v>10212.4</v>
       </c>
       <c r="J27" s="3">
         <v>0</v>
@@ -2100,24 +2106,24 @@
         <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>39159.56</v>
+        <v>0</v>
       </c>
       <c r="M27" s="4">
-        <v>39159.56</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>114100</v>
+        <v>113076</v>
       </c>
       <c r="B28" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="D28" s="11">
-        <v>45863</v>
+        <v>45806</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>54</v>
@@ -2129,10 +2135,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>8427.17</v>
+        <v>8929.2999999999993</v>
       </c>
       <c r="I28" s="4">
-        <v>8427.17</v>
+        <v>8929.2999999999993</v>
       </c>
       <c r="J28" s="3">
         <v>0</v>
@@ -2141,24 +2147,24 @@
         <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>53325.32</v>
+        <v>13675.57</v>
       </c>
       <c r="M28" s="4">
-        <v>53325.32</v>
+        <v>13675.57</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>109007</v>
+        <v>110105</v>
       </c>
       <c r="B29" s="2">
         <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D29" s="11">
-        <v>45525</v>
+        <v>45560</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>54</v>
@@ -2170,10 +2176,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>7858.27</v>
+        <v>8925.7000000000007</v>
       </c>
       <c r="I29" s="4">
-        <v>7858.27</v>
+        <v>8925.7000000000007</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2182,39 +2188,39 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>0</v>
+        <v>7778.69</v>
       </c>
       <c r="M29" s="4">
-        <v>0</v>
+        <v>7778.69</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>94156</v>
+        <v>116060</v>
       </c>
       <c r="B30" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="D30" s="11">
-        <v>44159</v>
+        <v>46010</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F30" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G30" s="4">
-        <v>1421.55</v>
+        <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>5466.12</v>
+        <v>8493.0300000000007</v>
       </c>
       <c r="I30" s="4">
-        <v>6887.67</v>
+        <v>8493.0300000000007</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2223,24 +2229,24 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>0</v>
+        <v>39457.379999999997</v>
       </c>
       <c r="M30" s="4">
-        <v>0</v>
+        <v>39457.379999999997</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>101640</v>
+        <v>109007</v>
       </c>
       <c r="B31" s="2">
         <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="D31" s="11">
-        <v>45104</v>
+        <v>45525</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>54</v>
@@ -2252,10 +2258,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>6369.67</v>
+        <v>7918.02</v>
       </c>
       <c r="I31" s="4">
-        <v>6369.67</v>
+        <v>7918.02</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -2264,39 +2270,39 @@
         <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>2366.0500000000002</v>
+        <v>0</v>
       </c>
       <c r="M31" s="4">
-        <v>2366.0500000000002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>108404</v>
+        <v>94156</v>
       </c>
       <c r="B32" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D32" s="11">
-        <v>45467</v>
+        <v>44159</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F32" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="4">
-        <v>0</v>
+        <v>1432.36</v>
       </c>
       <c r="H32" s="4">
-        <v>5851.31</v>
+        <v>5507.69</v>
       </c>
       <c r="I32" s="4">
-        <v>5851.31</v>
+        <v>6940.05</v>
       </c>
       <c r="J32" s="3">
         <v>0</v>
@@ -2305,24 +2311,24 @@
         <v>0</v>
       </c>
       <c r="L32" s="4">
-        <v>40999.71</v>
+        <v>0</v>
       </c>
       <c r="M32" s="4">
-        <v>40999.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>111056</v>
+        <v>101640</v>
       </c>
       <c r="B33" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D33" s="11">
-        <v>45639</v>
+        <v>45104</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>54</v>
@@ -2334,10 +2340,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>5403.95</v>
+        <v>6418.11</v>
       </c>
       <c r="I33" s="4">
-        <v>5403.95</v>
+        <v>6418.11</v>
       </c>
       <c r="J33" s="3">
         <v>0</v>
@@ -2346,24 +2352,24 @@
         <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>61189.599999999999</v>
+        <v>2384.04</v>
       </c>
       <c r="M33" s="4">
-        <v>61189.599999999999</v>
+        <v>2384.04</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>90177</v>
+        <v>108404</v>
       </c>
       <c r="B34" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="D34" s="11">
-        <v>43949</v>
+        <v>45467</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>54</v>
@@ -2375,10 +2381,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>5160.08</v>
+        <v>5895.82</v>
       </c>
       <c r="I34" s="4">
-        <v>5160.08</v>
+        <v>5895.82</v>
       </c>
       <c r="J34" s="3">
         <v>0</v>
@@ -2387,24 +2393,24 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>5160.08</v>
+        <v>41311.519999999997</v>
       </c>
       <c r="M34" s="4">
-        <v>5160.08</v>
+        <v>41311.519999999997</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>104343</v>
+        <v>90177</v>
       </c>
       <c r="B35" s="2">
         <v>2043</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="D35" s="11">
-        <v>45201</v>
+        <v>43949</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>54</v>
@@ -2416,22 +2422,22 @@
         <v>0</v>
       </c>
       <c r="H35" s="4">
-        <v>4424.0600000000004</v>
+        <v>5199.32</v>
       </c>
       <c r="I35" s="4">
-        <v>4424.0600000000004</v>
+        <v>5199.32</v>
       </c>
       <c r="J35" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K35" s="4">
-        <v>10223.11</v>
+        <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>50618.15</v>
+        <v>5199.32</v>
       </c>
       <c r="M35" s="4">
-        <v>60841.26</v>
+        <v>5199.32</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
@@ -2457,10 +2463,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="4">
-        <v>4210.32</v>
+        <v>4242.34</v>
       </c>
       <c r="I36" s="4">
-        <v>4210.32</v>
+        <v>4242.34</v>
       </c>
       <c r="J36" s="3">
         <v>0</v>
@@ -2469,10 +2475,10 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>19836.599999999999</v>
+        <v>19987.46</v>
       </c>
       <c r="M36" s="4">
-        <v>19836.599999999999</v>
+        <v>19987.46</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
@@ -2486,7 +2492,7 @@
         <v>25</v>
       </c>
       <c r="D37" s="11">
-        <v>46006</v>
+        <v>46111</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>54</v>
@@ -2498,10 +2504,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="4">
-        <v>4010.74</v>
+        <v>4041.24</v>
       </c>
       <c r="I37" s="4">
-        <v>4010.74</v>
+        <v>4041.24</v>
       </c>
       <c r="J37" s="3">
         <v>0</v>
@@ -2510,10 +2516,10 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>18048.330000000002</v>
+        <v>18185.59</v>
       </c>
       <c r="M37" s="4">
-        <v>18048.330000000002</v>
+        <v>18185.59</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
@@ -2539,10 +2545,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="4">
-        <v>3858.24</v>
+        <v>3887.59</v>
       </c>
       <c r="I38" s="4">
-        <v>3858.24</v>
+        <v>3887.59</v>
       </c>
       <c r="J38" s="3">
         <v>0</v>
@@ -2559,16 +2565,16 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>114431</v>
+        <v>102825</v>
       </c>
       <c r="B39" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="D39" s="11">
-        <v>45930</v>
+        <v>45117</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>54</v>
@@ -2580,10 +2586,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="4">
-        <v>3405.55</v>
+        <v>3512.02</v>
       </c>
       <c r="I39" s="4">
-        <v>3405.55</v>
+        <v>3512.02</v>
       </c>
       <c r="J39" s="3">
         <v>0</v>
@@ -2592,24 +2598,24 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>40155.160000000003</v>
+        <v>21637.32</v>
       </c>
       <c r="M39" s="4">
-        <v>40155.160000000003</v>
+        <v>21637.32</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>109998</v>
+        <v>114431</v>
       </c>
       <c r="B40" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D40" s="11">
-        <v>45596</v>
+        <v>45930</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>54</v>
@@ -2621,10 +2627,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="4">
-        <v>2844.92</v>
+        <v>3431.45</v>
       </c>
       <c r="I40" s="4">
-        <v>2844.92</v>
+        <v>3431.45</v>
       </c>
       <c r="J40" s="3">
         <v>0</v>
@@ -2633,24 +2639,24 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>0</v>
+        <v>40460.550000000003</v>
       </c>
       <c r="M40" s="4">
-        <v>0</v>
+        <v>40460.550000000003</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>81044</v>
+        <v>109998</v>
       </c>
       <c r="B41" s="2">
-        <v>2511</v>
+        <v>2043</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="D41" s="11">
-        <v>44872</v>
+        <v>45596</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>54</v>
@@ -2662,10 +2668,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="4">
-        <v>2385.52</v>
+        <v>2866.56</v>
       </c>
       <c r="I41" s="4">
-        <v>2385.52</v>
+        <v>2866.56</v>
       </c>
       <c r="J41" s="3">
         <v>0</v>
@@ -2682,16 +2688,16 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>63441</v>
+        <v>81044</v>
       </c>
       <c r="B42" s="2">
         <v>2511</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="D42" s="11">
-        <v>44733</v>
+        <v>44872</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>54</v>
@@ -2703,10 +2709,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="4">
-        <v>1827.5</v>
+        <v>2403.66</v>
       </c>
       <c r="I42" s="4">
-        <v>1827.5</v>
+        <v>2403.66</v>
       </c>
       <c r="J42" s="3">
         <v>0</v>
@@ -2715,24 +2721,24 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>9137.51</v>
+        <v>0</v>
       </c>
       <c r="M42" s="4">
-        <v>9137.51</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>102825</v>
+        <v>63441</v>
       </c>
       <c r="B43" s="2">
-        <v>2043</v>
+        <v>2511</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="D43" s="11">
-        <v>45117</v>
+        <v>44733</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>54</v>
@@ -2744,10 +2750,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="4">
-        <v>1742.75</v>
+        <v>1841.4</v>
       </c>
       <c r="I43" s="4">
-        <v>1742.75</v>
+        <v>1841.4</v>
       </c>
       <c r="J43" s="3">
         <v>0</v>
@@ -2756,39 +2762,39 @@
         <v>0</v>
       </c>
       <c r="L43" s="4">
-        <v>23216.76</v>
+        <v>9207.01</v>
       </c>
       <c r="M43" s="4">
-        <v>23216.76</v>
+        <v>9207.01</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>112522</v>
+        <v>118069</v>
       </c>
       <c r="B44" s="2">
         <v>2856</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="D44" s="11">
-        <v>45776</v>
+        <v>46105</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G44" s="4">
-        <v>0</v>
+        <v>1778.41</v>
       </c>
       <c r="H44" s="4">
-        <v>1737.52</v>
+        <v>0</v>
       </c>
       <c r="I44" s="4">
-        <v>1737.52</v>
+        <v>1778.41</v>
       </c>
       <c r="J44" s="3">
         <v>0</v>
@@ -2797,27 +2803,27 @@
         <v>0</v>
       </c>
       <c r="L44" s="4">
-        <v>6634.38</v>
+        <v>19562.52</v>
       </c>
       <c r="M44" s="4">
-        <v>6634.38</v>
+        <v>19562.52</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
-        <v>116795</v>
+        <v>112522</v>
       </c>
       <c r="B45" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="D45" s="11">
-        <v>46000</v>
+        <v>45776</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F45" s="3">
         <v>0</v>
@@ -2826,10 +2832,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="4">
-        <v>1582.15</v>
+        <v>1750.74</v>
       </c>
       <c r="I45" s="4">
-        <v>1582.15</v>
+        <v>1750.74</v>
       </c>
       <c r="J45" s="3">
         <v>0</v>
@@ -2838,10 +2844,10 @@
         <v>0</v>
       </c>
       <c r="L45" s="4">
-        <v>0</v>
+        <v>6684.84</v>
       </c>
       <c r="M45" s="4">
-        <v>0</v>
+        <v>6684.84</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
@@ -2867,10 +2873,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="4">
-        <v>1558.79</v>
+        <v>1621.51</v>
       </c>
       <c r="I46" s="4">
-        <v>1558.79</v>
+        <v>1621.51</v>
       </c>
       <c r="J46" s="3">
         <v>0</v>
@@ -2887,19 +2893,19 @@
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
-        <v>81618</v>
+        <v>116795</v>
       </c>
       <c r="B47" s="2">
         <v>2043</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D47" s="11">
-        <v>43447</v>
+        <v>46000</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F47" s="3">
         <v>0</v>
@@ -2908,10 +2914,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="4">
-        <v>0</v>
+        <v>1594.18</v>
       </c>
       <c r="I47" s="4">
-        <v>0</v>
+        <v>1594.18</v>
       </c>
       <c r="J47" s="3">
         <v>0</v>
@@ -2920,56 +2926,138 @@
         <v>0</v>
       </c>
       <c r="L47" s="4">
-        <v>14949.86</v>
+        <v>0</v>
       </c>
       <c r="M47" s="4">
-        <v>14949.86</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
+        <v>112083</v>
+      </c>
+      <c r="B48" s="2">
+        <v>2043</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D48" s="11">
+        <v>45736</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F48" s="3">
+        <v>0</v>
+      </c>
+      <c r="G48" s="4">
+        <v>0</v>
+      </c>
+      <c r="H48" s="4">
+        <v>0</v>
+      </c>
+      <c r="I48" s="4">
+        <v>0</v>
+      </c>
+      <c r="J48" s="3">
+        <v>1</v>
+      </c>
+      <c r="K48" s="4">
+        <v>20482.43</v>
+      </c>
+      <c r="L48" s="4">
+        <v>0</v>
+      </c>
+      <c r="M48" s="4">
+        <v>20482.43</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A49" s="2">
+        <v>81618</v>
+      </c>
+      <c r="B49" s="2">
+        <v>2043</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D49" s="11">
+        <v>43447</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F49" s="3">
+        <v>0</v>
+      </c>
+      <c r="G49" s="4">
+        <v>0</v>
+      </c>
+      <c r="H49" s="4">
+        <v>0</v>
+      </c>
+      <c r="I49" s="4">
+        <v>0</v>
+      </c>
+      <c r="J49" s="3">
+        <v>0</v>
+      </c>
+      <c r="K49" s="4">
+        <v>0</v>
+      </c>
+      <c r="L49" s="4">
+        <v>15063.56</v>
+      </c>
+      <c r="M49" s="4">
+        <v>15063.56</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A50" s="2">
         <v>113450</v>
       </c>
-      <c r="B48" s="2">
+      <c r="B50" s="2">
         <v>2692</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="C50" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D48" s="11">
+      <c r="D50" s="11">
         <v>45852</v>
       </c>
-      <c r="E48" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F48" s="3">
-        <v>0</v>
-      </c>
-      <c r="G48" s="4">
-        <v>0</v>
-      </c>
-      <c r="H48" s="4">
-        <v>-14615.07</v>
-      </c>
-      <c r="I48" s="4">
-        <v>-14615.07</v>
-      </c>
-      <c r="J48" s="3">
-        <v>0</v>
-      </c>
-      <c r="K48" s="4">
-        <v>0</v>
-      </c>
-      <c r="L48" s="4">
-        <v>6914.97</v>
-      </c>
-      <c r="M48" s="4">
-        <v>6914.97</v>
+      <c r="E50" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F50" s="3">
+        <v>0</v>
+      </c>
+      <c r="G50" s="4">
+        <v>0</v>
+      </c>
+      <c r="H50" s="4">
+        <v>-14684.32</v>
+      </c>
+      <c r="I50" s="4">
+        <v>-14684.32</v>
+      </c>
+      <c r="J50" s="3">
+        <v>0</v>
+      </c>
+      <c r="K50" s="4">
+        <v>0</v>
+      </c>
+      <c r="L50" s="4">
+        <v>7135.16</v>
+      </c>
+      <c r="M50" s="4">
+        <v>7135.16</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="A5:A48 J5:J48">
+  <conditionalFormatting sqref="A5:A50 J5:J50">
     <cfRule type="expression" dxfId="11" priority="4" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
@@ -2977,7 +3065,7 @@
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:L48 C5:H48">
+  <conditionalFormatting sqref="K5:L50 C5:H50">
     <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
@@ -2985,7 +3073,7 @@
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I48 M5:M48">
+  <conditionalFormatting sqref="I5:I50 M5:M50">
     <cfRule type="expression" dxfId="7" priority="8" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
@@ -3013,7 +3101,7 @@
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B48">
+  <conditionalFormatting sqref="B5:B50">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-15 09:41)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F2CE7F3-B86D-E84B-B777-F0BC66D9F983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C8DA191-B0B7-594B-AF6A-0272F8CDAAD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="56">
   <si>
     <t>Asesor</t>
   </si>
@@ -98,9 +98,6 @@
     <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
   </si>
   <si>
-    <t>GERARDO DANIEL BARAJAS TORRES</t>
-  </si>
-  <si>
     <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
   </si>
   <si>
@@ -140,15 +137,9 @@
     <t>ISAI ANTONIO ROJAS MARTINEZ</t>
   </si>
   <si>
-    <t>ROCIO IVON RUIZ GARCIA</t>
-  </si>
-  <si>
     <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
   </si>
   <si>
-    <t>JOSE ALBERTO CORONADO ROSAS</t>
-  </si>
-  <si>
     <t>MARIA TERESA ASENCIO LOZANO</t>
   </si>
   <si>
@@ -206,13 +197,7 @@
     <t>MONSERRAT VELASCO SANTOS</t>
   </si>
   <si>
-    <t>5</t>
-  </si>
-  <si>
     <t>4</t>
-  </si>
-  <si>
-    <t>KAREN MUÐOZ GARCIA</t>
   </si>
   <si>
     <t>MARIO IVAN ROMERO GONZALEZ</t>
@@ -1049,7 +1034,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46112</v>
+        <v>46125</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1063,28 +1048,28 @@
       <c r="D2" s="9"/>
       <c r="E2" s="8"/>
       <c r="F2" s="12" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="J2" s="12" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="K2" s="12" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="L2" s="12" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="M2" s="12" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
@@ -1098,34 +1083,34 @@
         <v>2</v>
       </c>
       <c r="D3" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>53</v>
-      </c>
       <c r="J3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="M3" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
@@ -1142,31 +1127,31 @@
         <v>43731</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F4" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G4" s="4">
-        <v>406177.63</v>
+        <v>73656.399999999994</v>
       </c>
       <c r="H4" s="4">
-        <v>116388.43</v>
+        <v>36746.69</v>
       </c>
       <c r="I4" s="4">
-        <v>522566.06</v>
+        <v>110403.09</v>
       </c>
       <c r="J4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" s="4">
-        <v>72105.62</v>
+        <v>0</v>
       </c>
       <c r="L4" s="4">
-        <v>338756.64</v>
+        <v>344649.08</v>
       </c>
       <c r="M4" s="4">
-        <v>410862.26</v>
+        <v>344649.08</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1177,37 +1162,37 @@
         <v>2043</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D5" s="11">
         <v>43371</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F5" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G5" s="4">
-        <v>178153.93</v>
+        <v>29477.7</v>
       </c>
       <c r="H5" s="4">
-        <v>12433.86</v>
+        <v>62549.13</v>
       </c>
       <c r="I5" s="4">
-        <v>190587.79</v>
+        <v>92026.83</v>
       </c>
       <c r="J5" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5" s="4">
-        <v>84465.85</v>
+        <v>23801.34</v>
       </c>
       <c r="L5" s="4">
         <v>116422.94</v>
       </c>
       <c r="M5" s="4">
-        <v>200888.79</v>
+        <v>140224.28</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -1224,31 +1209,31 @@
         <v>45600</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F6" s="3">
         <v>1</v>
       </c>
       <c r="G6" s="4">
-        <v>1854.93</v>
+        <v>2244.4699999999998</v>
       </c>
       <c r="H6" s="4">
-        <v>81364.38</v>
+        <v>33777.410000000003</v>
       </c>
       <c r="I6" s="4">
-        <v>83219.31</v>
+        <v>36021.879999999997</v>
       </c>
       <c r="J6" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" s="4">
-        <v>1784.38</v>
+        <v>0</v>
       </c>
       <c r="L6" s="4">
-        <v>173372.39</v>
+        <v>145975.84</v>
       </c>
       <c r="M6" s="4">
-        <v>175156.77</v>
+        <v>145975.84</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -1265,48 +1250,48 @@
         <v>45236</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F7" s="3">
         <v>2</v>
       </c>
       <c r="G7" s="4">
-        <v>32501.09</v>
+        <v>1799.5</v>
       </c>
       <c r="H7" s="4">
-        <v>44335.51</v>
+        <v>31457.13</v>
       </c>
       <c r="I7" s="4">
-        <v>76836.600000000006</v>
+        <v>33256.629999999997</v>
       </c>
       <c r="J7" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K7" s="4">
-        <v>28039.64</v>
+        <v>2088.27</v>
       </c>
       <c r="L7" s="4">
-        <v>57754.95</v>
+        <v>56777.83</v>
       </c>
       <c r="M7" s="4">
-        <v>85794.59</v>
+        <v>58866.1</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>107488</v>
+        <v>114100</v>
       </c>
       <c r="B8" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D8" s="11">
-        <v>45440</v>
+        <v>45863</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F8" s="3">
         <v>0</v>
@@ -1315,92 +1300,92 @@
         <v>0</v>
       </c>
       <c r="H8" s="4">
-        <v>66591.3</v>
+        <v>21150.02</v>
       </c>
       <c r="I8" s="4">
-        <v>66591.3</v>
+        <v>21150.02</v>
       </c>
       <c r="J8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" s="4">
-        <v>0</v>
+        <v>20413.86</v>
       </c>
       <c r="L8" s="4">
-        <v>107694.21</v>
+        <v>38941.47</v>
       </c>
       <c r="M8" s="4">
-        <v>107694.21</v>
+        <v>59355.33</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>47116</v>
+        <v>110575</v>
       </c>
       <c r="B9" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="D9" s="11">
-        <v>44616</v>
+        <v>45583</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F9" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" s="4">
-        <v>2117.52</v>
+        <v>0</v>
       </c>
       <c r="H9" s="4">
-        <v>63467.86</v>
+        <v>14385.86</v>
       </c>
       <c r="I9" s="4">
-        <v>65585.38</v>
+        <v>14385.86</v>
       </c>
       <c r="J9" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" s="4">
-        <v>37033.42</v>
+        <v>0</v>
       </c>
       <c r="L9" s="4">
-        <v>39817.339999999997</v>
+        <v>86315.15</v>
       </c>
       <c r="M9" s="4">
-        <v>76850.759999999995</v>
+        <v>86315.15</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>115047</v>
+        <v>107488</v>
       </c>
       <c r="B10" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="D10" s="11">
-        <v>45944</v>
+        <v>45440</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F10" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" s="4">
-        <v>1499.56</v>
+        <v>0</v>
       </c>
       <c r="H10" s="4">
-        <v>51080.26</v>
+        <v>8873.25</v>
       </c>
       <c r="I10" s="4">
-        <v>52579.82</v>
+        <v>8873.25</v>
       </c>
       <c r="J10" s="3">
         <v>0</v>
@@ -1409,109 +1394,109 @@
         <v>0</v>
       </c>
       <c r="L10" s="4">
-        <v>31356.09</v>
+        <v>108547.73</v>
       </c>
       <c r="M10" s="4">
-        <v>31356.09</v>
+        <v>108547.73</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>105696</v>
+        <v>108404</v>
       </c>
       <c r="B11" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D11" s="11">
-        <v>45279</v>
+        <v>45467</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F11" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" s="4">
-        <v>32118.39</v>
+        <v>0</v>
       </c>
       <c r="H11" s="4">
-        <v>14674.37</v>
+        <v>7900.28</v>
       </c>
       <c r="I11" s="4">
-        <v>46792.76</v>
+        <v>7900.28</v>
       </c>
       <c r="J11" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" s="4">
-        <v>36118.519999999997</v>
+        <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>22778.99</v>
+        <v>22176.42</v>
       </c>
       <c r="M11" s="4">
-        <v>58897.51</v>
+        <v>22176.42</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>104718</v>
+        <v>47116</v>
       </c>
       <c r="B12" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>8</v>
+        <v>41</v>
       </c>
       <c r="D12" s="11">
-        <v>45264</v>
+        <v>44616</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F12" s="3">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4">
+        <v>7784.62</v>
+      </c>
+      <c r="I12" s="4">
+        <v>7784.62</v>
+      </c>
+      <c r="J12" s="3">
         <v>1</v>
       </c>
-      <c r="G12" s="4">
-        <v>13128.07</v>
-      </c>
-      <c r="H12" s="4">
-        <v>26453.98</v>
-      </c>
-      <c r="I12" s="4">
-        <v>39582.050000000003</v>
-      </c>
-      <c r="J12" s="3">
-        <v>0</v>
-      </c>
       <c r="K12" s="4">
-        <v>0</v>
+        <v>15689.6</v>
       </c>
       <c r="L12" s="4">
-        <v>101309.13</v>
+        <v>60082.48</v>
       </c>
       <c r="M12" s="4">
-        <v>101309.13</v>
+        <v>75772.08</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>115404</v>
+        <v>117440</v>
       </c>
       <c r="B13" s="2">
         <v>2043</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="D13" s="11">
-        <v>45986</v>
+        <v>46059</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F13" s="3">
         <v>0</v>
@@ -1520,10 +1505,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="4">
-        <v>34822.78</v>
+        <v>7530.24</v>
       </c>
       <c r="I13" s="4">
-        <v>34822.78</v>
+        <v>7530.24</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1532,10 +1517,10 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>12170.29</v>
+        <v>5455.03</v>
       </c>
       <c r="M13" s="4">
-        <v>12170.29</v>
+        <v>5455.03</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
@@ -1546,13 +1531,13 @@
         <v>2692</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D14" s="11">
         <v>45471</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F14" s="3">
         <v>0</v>
@@ -1561,10 +1546,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="4">
-        <v>33294.480000000003</v>
+        <v>5525.52</v>
       </c>
       <c r="I14" s="4">
-        <v>33294.480000000003</v>
+        <v>5525.52</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1573,39 +1558,39 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>9494.81</v>
+        <v>7002.07</v>
       </c>
       <c r="M14" s="4">
-        <v>9494.81</v>
+        <v>7002.07</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>65046</v>
+        <v>115047</v>
       </c>
       <c r="B15" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="D15" s="11">
-        <v>44763</v>
+        <v>45944</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F15" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" s="4">
-        <v>1459.06</v>
+        <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>29490.62</v>
+        <v>5025.2</v>
       </c>
       <c r="I15" s="4">
-        <v>30949.68</v>
+        <v>5025.2</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1614,39 +1599,39 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>17384.95</v>
+        <v>35787.599999999999</v>
       </c>
       <c r="M15" s="4">
-        <v>17384.95</v>
+        <v>35787.599999999999</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>114157</v>
+        <v>113450</v>
       </c>
       <c r="B16" s="2">
         <v>2692</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D16" s="11">
-        <v>45904</v>
+        <v>45852</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F16" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" s="4">
-        <v>1697.76</v>
+        <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>15790.19</v>
+        <v>4898.1400000000003</v>
       </c>
       <c r="I16" s="4">
-        <v>17487.95</v>
+        <v>4898.1400000000003</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1655,27 +1640,27 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>66856.350000000006</v>
+        <v>5799.55</v>
       </c>
       <c r="M16" s="4">
-        <v>66856.350000000006</v>
+        <v>5799.55</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>90355</v>
+        <v>101640</v>
       </c>
       <c r="B17" s="2">
         <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="D17" s="11">
-        <v>43949</v>
+        <v>45104</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F17" s="3">
         <v>0</v>
@@ -1684,10 +1669,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>16793.03</v>
+        <v>4718.59</v>
       </c>
       <c r="I17" s="4">
-        <v>16793.03</v>
+        <v>4718.59</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1696,39 +1681,39 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>29400.74</v>
+        <v>3204.95</v>
       </c>
       <c r="M17" s="4">
-        <v>29400.74</v>
+        <v>3204.95</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>104343</v>
+        <v>100677</v>
       </c>
       <c r="B18" s="2">
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D18" s="11">
-        <v>45201</v>
+        <v>44999</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F18" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" s="4">
-        <v>10300.870000000001</v>
+        <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>5495.48</v>
+        <v>4681.6099999999997</v>
       </c>
       <c r="I18" s="4">
-        <v>15796.35</v>
+        <v>4681.6099999999997</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1737,39 +1722,39 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>49965.37</v>
+        <v>34806.33</v>
       </c>
       <c r="M18" s="4">
-        <v>49965.37</v>
+        <v>34806.33</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>117440</v>
+        <v>113076</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="D19" s="11">
-        <v>46059</v>
+        <v>45806</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F19" s="3">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G19" s="4">
-        <v>7492.03</v>
+        <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>7957.91</v>
+        <v>4558.5200000000004</v>
       </c>
       <c r="I19" s="4">
-        <v>15449.94</v>
+        <v>4558.5200000000004</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1778,27 +1763,27 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>0</v>
+        <v>9117.0400000000009</v>
       </c>
       <c r="M19" s="4">
-        <v>0</v>
+        <v>9117.0400000000009</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>80925</v>
+        <v>88234</v>
       </c>
       <c r="B20" s="2">
         <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D20" s="11">
-        <v>43439</v>
+        <v>43794</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F20" s="3">
         <v>0</v>
@@ -1807,10 +1792,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>14641.5</v>
+        <v>4242.34</v>
       </c>
       <c r="I20" s="4">
-        <v>14641.5</v>
+        <v>4242.34</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1819,27 +1804,27 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>0</v>
+        <v>15745.12</v>
       </c>
       <c r="M20" s="4">
-        <v>0</v>
+        <v>15745.12</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>110575</v>
+        <v>109998</v>
       </c>
       <c r="B21" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D21" s="11">
-        <v>45583</v>
+        <v>45596</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F21" s="3">
         <v>0</v>
@@ -1848,10 +1833,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>14385.86</v>
+        <v>2958.1</v>
       </c>
       <c r="I21" s="4">
-        <v>14385.86</v>
+        <v>2958.1</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1860,39 +1845,39 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>100701.01</v>
+        <v>0</v>
       </c>
       <c r="M21" s="4">
-        <v>100701.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>116883</v>
+        <v>112083</v>
       </c>
       <c r="B22" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="D22" s="11">
-        <v>46007</v>
+        <v>45736</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F22" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G22" s="4">
-        <v>8797.08</v>
+        <v>1795.63</v>
       </c>
       <c r="H22" s="4">
-        <v>4041.24</v>
+        <v>0</v>
       </c>
       <c r="I22" s="4">
-        <v>12838.32</v>
+        <v>1795.63</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1901,39 +1886,39 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>60897.84</v>
+        <v>19751.93</v>
       </c>
       <c r="M22" s="4">
-        <v>60897.84</v>
+        <v>19751.93</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>106018</v>
+        <v>104343</v>
       </c>
       <c r="B23" s="2">
         <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="D23" s="11">
-        <v>45344</v>
+        <v>45201</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F23" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" s="4">
-        <v>585.37</v>
+        <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>11777.23</v>
+        <v>1756.01</v>
       </c>
       <c r="I23" s="4">
-        <v>12362.6</v>
+        <v>1756.01</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1942,27 +1927,27 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>22762.21</v>
+        <v>60525.61</v>
       </c>
       <c r="M23" s="4">
-        <v>22762.21</v>
+        <v>60525.61</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>100677</v>
+        <v>104718</v>
       </c>
       <c r="B24" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="D24" s="11">
-        <v>44999</v>
+        <v>45264</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F24" s="3">
         <v>0</v>
@@ -1971,10 +1956,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>10947.46</v>
+        <v>1731.32</v>
       </c>
       <c r="I24" s="4">
-        <v>10947.46</v>
+        <v>1731.32</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1983,27 +1968,27 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>18165.66</v>
+        <v>104908.85</v>
       </c>
       <c r="M24" s="4">
-        <v>18165.66</v>
+        <v>104908.85</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>114100</v>
+        <v>114157</v>
       </c>
       <c r="B25" s="2">
-        <v>2856</v>
+        <v>2692</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D25" s="11">
-        <v>45863</v>
+        <v>45904</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F25" s="3">
         <v>0</v>
@@ -2012,10 +1997,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>10901.34</v>
+        <v>1637.49</v>
       </c>
       <c r="I25" s="4">
-        <v>10901.34</v>
+        <v>1637.49</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -2024,27 +2009,27 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>53730.879999999997</v>
+        <v>65218.85</v>
       </c>
       <c r="M25" s="4">
-        <v>53730.879999999997</v>
+        <v>65218.85</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>111056</v>
+        <v>118069</v>
       </c>
       <c r="B26" s="2">
-        <v>2692</v>
+        <v>2856</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>7</v>
+        <v>54</v>
       </c>
       <c r="D26" s="11">
-        <v>45639</v>
+        <v>46105</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F26" s="3">
         <v>0</v>
@@ -2053,10 +2038,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>10890.1</v>
+        <v>0</v>
       </c>
       <c r="I26" s="4">
-        <v>10890.1</v>
+        <v>0</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2065,27 +2050,27 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>56209.91</v>
+        <v>19562.52</v>
       </c>
       <c r="M26" s="4">
-        <v>56209.91</v>
+        <v>19562.52</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>94205</v>
+        <v>116883</v>
       </c>
       <c r="B27" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D27" s="11">
-        <v>44116</v>
+        <v>46007</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F27" s="3">
         <v>0</v>
@@ -2094,39 +2079,39 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>10212.4</v>
+        <v>0</v>
       </c>
       <c r="I27" s="4">
-        <v>10212.4</v>
+        <v>0</v>
       </c>
       <c r="J27" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" s="4">
-        <v>0</v>
+        <v>2174.0100000000002</v>
       </c>
       <c r="L27" s="4">
-        <v>0</v>
+        <v>88699.520000000004</v>
       </c>
       <c r="M27" s="4">
-        <v>0</v>
+        <v>90873.53</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>113076</v>
+        <v>116876</v>
       </c>
       <c r="B28" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D28" s="11">
-        <v>45806</v>
+        <v>46111</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F28" s="3">
         <v>0</v>
@@ -2135,10 +2120,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>8929.2999999999993</v>
+        <v>0</v>
       </c>
       <c r="I28" s="4">
-        <v>8929.2999999999993</v>
+        <v>0</v>
       </c>
       <c r="J28" s="3">
         <v>0</v>
@@ -2147,27 +2132,27 @@
         <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>13675.57</v>
+        <v>18185.59</v>
       </c>
       <c r="M28" s="4">
-        <v>13675.57</v>
+        <v>18185.59</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>110105</v>
+        <v>116060</v>
       </c>
       <c r="B29" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="D29" s="11">
-        <v>45560</v>
+        <v>46010</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F29" s="3">
         <v>0</v>
@@ -2176,10 +2161,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>8925.7000000000007</v>
+        <v>0</v>
       </c>
       <c r="I29" s="4">
-        <v>8925.7000000000007</v>
+        <v>0</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2188,27 +2173,27 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>7778.69</v>
+        <v>62278.86</v>
       </c>
       <c r="M29" s="4">
-        <v>7778.69</v>
+        <v>62278.86</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>116060</v>
+        <v>115404</v>
       </c>
       <c r="B30" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D30" s="11">
-        <v>46010</v>
+        <v>45986</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F30" s="3">
         <v>0</v>
@@ -2217,10 +2202,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>8493.0300000000007</v>
+        <v>0</v>
       </c>
       <c r="I30" s="4">
-        <v>8493.0300000000007</v>
+        <v>0</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2229,27 +2214,27 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>39457.379999999997</v>
+        <v>12170.29</v>
       </c>
       <c r="M30" s="4">
-        <v>39457.379999999997</v>
+        <v>12170.29</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>109007</v>
+        <v>114431</v>
       </c>
       <c r="B31" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="D31" s="11">
-        <v>45525</v>
+        <v>45930</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F31" s="3">
         <v>0</v>
@@ -2258,10 +2243,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>7918.02</v>
+        <v>0</v>
       </c>
       <c r="I31" s="4">
-        <v>7918.02</v>
+        <v>0</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -2270,39 +2255,39 @@
         <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>0</v>
+        <v>21758.76</v>
       </c>
       <c r="M31" s="4">
-        <v>0</v>
+        <v>21758.76</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>94156</v>
+        <v>112522</v>
       </c>
       <c r="B32" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D32" s="11">
-        <v>44159</v>
+        <v>45776</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F32" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" s="4">
-        <v>1432.36</v>
+        <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>5507.69</v>
+        <v>0</v>
       </c>
       <c r="I32" s="4">
-        <v>6940.05</v>
+        <v>0</v>
       </c>
       <c r="J32" s="3">
         <v>0</v>
@@ -2311,27 +2296,27 @@
         <v>0</v>
       </c>
       <c r="L32" s="4">
-        <v>0</v>
+        <v>6684.84</v>
       </c>
       <c r="M32" s="4">
-        <v>0</v>
+        <v>6684.84</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>101640</v>
+        <v>111056</v>
       </c>
       <c r="B33" s="2">
-        <v>2043</v>
+        <v>2692</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D33" s="11">
-        <v>45104</v>
+        <v>45639</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F33" s="3">
         <v>0</v>
@@ -2340,39 +2325,39 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>6418.11</v>
+        <v>0</v>
       </c>
       <c r="I33" s="4">
-        <v>6418.11</v>
+        <v>0</v>
       </c>
       <c r="J33" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K33" s="4">
-        <v>0</v>
+        <v>61752.21</v>
       </c>
       <c r="L33" s="4">
-        <v>2384.04</v>
+        <v>56209.91</v>
       </c>
       <c r="M33" s="4">
-        <v>2384.04</v>
+        <v>117962.12</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>108404</v>
+        <v>110105</v>
       </c>
       <c r="B34" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D34" s="11">
-        <v>45467</v>
+        <v>45560</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F34" s="3">
         <v>0</v>
@@ -2381,10 +2366,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>5895.82</v>
+        <v>0</v>
       </c>
       <c r="I34" s="4">
-        <v>5895.82</v>
+        <v>0</v>
       </c>
       <c r="J34" s="3">
         <v>0</v>
@@ -2393,27 +2378,27 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>41311.519999999997</v>
+        <v>13077.25</v>
       </c>
       <c r="M34" s="4">
-        <v>41311.519999999997</v>
+        <v>13077.25</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>90177</v>
+        <v>109007</v>
       </c>
       <c r="B35" s="2">
         <v>2043</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D35" s="11">
-        <v>43949</v>
+        <v>45525</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F35" s="3">
         <v>0</v>
@@ -2422,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="4">
-        <v>5199.32</v>
+        <v>0</v>
       </c>
       <c r="I35" s="4">
-        <v>5199.32</v>
+        <v>0</v>
       </c>
       <c r="J35" s="3">
         <v>0</v>
@@ -2434,27 +2419,27 @@
         <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>5199.32</v>
+        <v>6177.09</v>
       </c>
       <c r="M35" s="4">
-        <v>5199.32</v>
+        <v>6177.09</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>88234</v>
+        <v>106018</v>
       </c>
       <c r="B36" s="2">
         <v>2043</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D36" s="11">
-        <v>43794</v>
+        <v>45344</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F36" s="3">
         <v>0</v>
@@ -2463,10 +2448,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="4">
-        <v>4242.34</v>
+        <v>0</v>
       </c>
       <c r="I36" s="4">
-        <v>4242.34</v>
+        <v>0</v>
       </c>
       <c r="J36" s="3">
         <v>0</v>
@@ -2475,27 +2460,27 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>19987.46</v>
+        <v>30708.15</v>
       </c>
       <c r="M36" s="4">
-        <v>19987.46</v>
+        <v>30708.15</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>116876</v>
+        <v>105696</v>
       </c>
       <c r="B37" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="D37" s="11">
-        <v>46111</v>
+        <v>45279</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F37" s="3">
         <v>0</v>
@@ -2504,39 +2489,39 @@
         <v>0</v>
       </c>
       <c r="H37" s="4">
-        <v>4041.24</v>
+        <v>0</v>
       </c>
       <c r="I37" s="4">
-        <v>4041.24</v>
+        <v>0</v>
       </c>
       <c r="J37" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K37" s="4">
-        <v>0</v>
+        <v>36118.519999999997</v>
       </c>
       <c r="L37" s="4">
-        <v>18185.59</v>
+        <v>31399.77</v>
       </c>
       <c r="M37" s="4">
-        <v>18185.59</v>
+        <v>67518.289999999994</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>95148</v>
+        <v>102825</v>
       </c>
       <c r="B38" s="2">
         <v>2043</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="D38" s="11">
-        <v>44916</v>
+        <v>45117</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F38" s="3">
         <v>0</v>
@@ -2545,39 +2530,39 @@
         <v>0</v>
       </c>
       <c r="H38" s="4">
-        <v>3887.59</v>
+        <v>0</v>
       </c>
       <c r="I38" s="4">
-        <v>3887.59</v>
+        <v>0</v>
       </c>
       <c r="J38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K38" s="4">
-        <v>0</v>
+        <v>30557.77</v>
       </c>
       <c r="L38" s="4">
-        <v>0</v>
+        <v>21637.32</v>
       </c>
       <c r="M38" s="4">
-        <v>0</v>
+        <v>52195.09</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>102825</v>
+        <v>95148</v>
       </c>
       <c r="B39" s="2">
         <v>2043</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="D39" s="11">
-        <v>45117</v>
+        <v>44916</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F39" s="3">
         <v>0</v>
@@ -2586,10 +2571,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="4">
-        <v>3512.02</v>
+        <v>0</v>
       </c>
       <c r="I39" s="4">
-        <v>3512.02</v>
+        <v>0</v>
       </c>
       <c r="J39" s="3">
         <v>0</v>
@@ -2598,27 +2583,27 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>21637.32</v>
+        <v>3887.54</v>
       </c>
       <c r="M39" s="4">
-        <v>21637.32</v>
+        <v>3887.54</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>114431</v>
+        <v>94156</v>
       </c>
       <c r="B40" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="D40" s="11">
-        <v>45930</v>
+        <v>44159</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F40" s="3">
         <v>0</v>
@@ -2627,10 +2612,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="4">
-        <v>3431.45</v>
+        <v>0</v>
       </c>
       <c r="I40" s="4">
-        <v>3431.45</v>
+        <v>0</v>
       </c>
       <c r="J40" s="3">
         <v>0</v>
@@ -2639,27 +2624,27 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>40460.550000000003</v>
+        <v>7466.11</v>
       </c>
       <c r="M40" s="4">
-        <v>40460.550000000003</v>
+        <v>7466.11</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>109998</v>
+        <v>90355</v>
       </c>
       <c r="B41" s="2">
         <v>2043</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D41" s="11">
-        <v>45596</v>
+        <v>43949</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F41" s="3">
         <v>0</v>
@@ -2668,39 +2653,39 @@
         <v>0</v>
       </c>
       <c r="H41" s="4">
-        <v>2866.56</v>
+        <v>0</v>
       </c>
       <c r="I41" s="4">
-        <v>2866.56</v>
+        <v>0</v>
       </c>
       <c r="J41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K41" s="4">
-        <v>0</v>
+        <v>6757.44</v>
       </c>
       <c r="L41" s="4">
-        <v>0</v>
+        <v>42913.120000000003</v>
       </c>
       <c r="M41" s="4">
-        <v>0</v>
+        <v>49670.559999999998</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>81044</v>
+        <v>90177</v>
       </c>
       <c r="B42" s="2">
-        <v>2511</v>
+        <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="D42" s="11">
-        <v>44872</v>
+        <v>43949</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F42" s="3">
         <v>0</v>
@@ -2709,10 +2694,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="4">
-        <v>2403.66</v>
+        <v>0</v>
       </c>
       <c r="I42" s="4">
-        <v>2403.66</v>
+        <v>0</v>
       </c>
       <c r="J42" s="3">
         <v>0</v>
@@ -2721,27 +2706,27 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>0</v>
+        <v>5199.32</v>
       </c>
       <c r="M42" s="4">
-        <v>0</v>
+        <v>5199.32</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>63441</v>
+        <v>81618</v>
       </c>
       <c r="B43" s="2">
-        <v>2511</v>
+        <v>2043</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D43" s="11">
-        <v>44733</v>
+        <v>43447</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F43" s="3">
         <v>0</v>
@@ -2750,10 +2735,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="4">
-        <v>1841.4</v>
+        <v>0</v>
       </c>
       <c r="I43" s="4">
-        <v>1841.4</v>
+        <v>0</v>
       </c>
       <c r="J43" s="3">
         <v>0</v>
@@ -2762,39 +2747,39 @@
         <v>0</v>
       </c>
       <c r="L43" s="4">
-        <v>9207.01</v>
+        <v>15063.56</v>
       </c>
       <c r="M43" s="4">
-        <v>9207.01</v>
+        <v>15063.56</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>118069</v>
+        <v>80925</v>
       </c>
       <c r="B44" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="D44" s="11">
-        <v>46105</v>
+        <v>43439</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G44" s="4">
-        <v>1778.41</v>
+        <v>0</v>
       </c>
       <c r="H44" s="4">
         <v>0</v>
       </c>
       <c r="I44" s="4">
-        <v>1778.41</v>
+        <v>0</v>
       </c>
       <c r="J44" s="3">
         <v>0</v>
@@ -2803,27 +2788,27 @@
         <v>0</v>
       </c>
       <c r="L44" s="4">
-        <v>19562.52</v>
+        <v>10138.450000000001</v>
       </c>
       <c r="M44" s="4">
-        <v>19562.52</v>
+        <v>10138.450000000001</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
-        <v>112522</v>
+        <v>65046</v>
       </c>
       <c r="B45" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="D45" s="11">
-        <v>45776</v>
+        <v>44763</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F45" s="3">
         <v>0</v>
@@ -2832,10 +2817,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="4">
-        <v>1750.74</v>
+        <v>0</v>
       </c>
       <c r="I45" s="4">
-        <v>1750.74</v>
+        <v>0</v>
       </c>
       <c r="J45" s="3">
         <v>0</v>
@@ -2844,27 +2829,27 @@
         <v>0</v>
       </c>
       <c r="L45" s="4">
-        <v>6684.84</v>
+        <v>17384.95</v>
       </c>
       <c r="M45" s="4">
-        <v>6684.84</v>
+        <v>17384.95</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
-        <v>108658</v>
+        <v>63441</v>
       </c>
       <c r="B46" s="2">
-        <v>2043</v>
+        <v>2511</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D46" s="11">
-        <v>45497</v>
+        <v>44733</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F46" s="3">
         <v>0</v>
@@ -2873,10 +2858,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="4">
-        <v>1621.51</v>
+        <v>0</v>
       </c>
       <c r="I46" s="4">
-        <v>1621.51</v>
+        <v>0</v>
       </c>
       <c r="J46" s="3">
         <v>0</v>
@@ -2885,179 +2870,107 @@
         <v>0</v>
       </c>
       <c r="L46" s="4">
-        <v>0</v>
+        <v>9207.01</v>
       </c>
       <c r="M46" s="4">
-        <v>0</v>
+        <v>9207.01</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A47" s="2">
-        <v>116795</v>
-      </c>
-      <c r="B47" s="2">
-        <v>2043</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D47" s="11">
-        <v>46000</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F47" s="3">
-        <v>0</v>
-      </c>
-      <c r="G47" s="4">
-        <v>0</v>
-      </c>
-      <c r="H47" s="4">
-        <v>1594.18</v>
-      </c>
-      <c r="I47" s="4">
-        <v>1594.18</v>
-      </c>
-      <c r="J47" s="3">
-        <v>0</v>
-      </c>
-      <c r="K47" s="4">
-        <v>0</v>
-      </c>
-      <c r="L47" s="4">
-        <v>0</v>
-      </c>
-      <c r="M47" s="4">
-        <v>0</v>
-      </c>
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="4"/>
+      <c r="H47" s="4"/>
+      <c r="I47" s="4"/>
+      <c r="J47" s="3"/>
+      <c r="K47" s="4"/>
+      <c r="L47" s="4"/>
+      <c r="M47" s="4"/>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A48" s="2">
-        <v>112083</v>
-      </c>
-      <c r="B48" s="2">
-        <v>2043</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D48" s="11">
-        <v>45736</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F48" s="3">
-        <v>0</v>
-      </c>
-      <c r="G48" s="4">
-        <v>0</v>
-      </c>
-      <c r="H48" s="4">
-        <v>0</v>
-      </c>
-      <c r="I48" s="4">
-        <v>0</v>
-      </c>
-      <c r="J48" s="3">
-        <v>1</v>
-      </c>
-      <c r="K48" s="4">
-        <v>20482.43</v>
-      </c>
-      <c r="L48" s="4">
-        <v>0</v>
-      </c>
-      <c r="M48" s="4">
-        <v>20482.43</v>
-      </c>
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="11"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4"/>
+      <c r="I48" s="4"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="4"/>
+      <c r="L48" s="4"/>
+      <c r="M48" s="4"/>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A49" s="2">
-        <v>81618</v>
-      </c>
-      <c r="B49" s="2">
-        <v>2043</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D49" s="11">
-        <v>43447</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F49" s="3">
-        <v>0</v>
-      </c>
-      <c r="G49" s="4">
-        <v>0</v>
-      </c>
-      <c r="H49" s="4">
-        <v>0</v>
-      </c>
-      <c r="I49" s="4">
-        <v>0</v>
-      </c>
-      <c r="J49" s="3">
-        <v>0</v>
-      </c>
-      <c r="K49" s="4">
-        <v>0</v>
-      </c>
-      <c r="L49" s="4">
-        <v>15063.56</v>
-      </c>
-      <c r="M49" s="4">
-        <v>15063.56</v>
-      </c>
+      <c r="A49" s="2"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="4"/>
+      <c r="H49" s="4"/>
+      <c r="I49" s="4"/>
+      <c r="J49" s="3"/>
+      <c r="K49" s="4"/>
+      <c r="L49" s="4"/>
+      <c r="M49" s="4"/>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A50" s="2">
-        <v>113450</v>
-      </c>
-      <c r="B50" s="2">
-        <v>2692</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D50" s="11">
-        <v>45852</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F50" s="3">
-        <v>0</v>
-      </c>
-      <c r="G50" s="4">
-        <v>0</v>
-      </c>
-      <c r="H50" s="4">
-        <v>-14684.32</v>
-      </c>
-      <c r="I50" s="4">
-        <v>-14684.32</v>
-      </c>
-      <c r="J50" s="3">
-        <v>0</v>
-      </c>
-      <c r="K50" s="4">
-        <v>0</v>
-      </c>
-      <c r="L50" s="4">
-        <v>7135.16</v>
-      </c>
-      <c r="M50" s="4">
-        <v>7135.16</v>
-      </c>
+      <c r="A50" s="2"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="2"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="2"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="4"/>
+      <c r="I50" s="4"/>
+      <c r="J50" s="3"/>
+      <c r="K50" s="4"/>
+      <c r="L50" s="4"/>
+      <c r="M50" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="A5:A50 J5:J50">
+  <conditionalFormatting sqref="A47:B50">
+    <cfRule type="expression" dxfId="22" priority="13" stopIfTrue="1">
+      <formula>$S47=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="21" priority="14" stopIfTrue="1">
+      <formula>$S46=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C47:H50 K47:L50">
+    <cfRule type="expression" dxfId="19" priority="18" stopIfTrue="1">
+      <formula>$S47=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="18" priority="19" stopIfTrue="1">
+      <formula>$S46=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I47:I50 M47:M50">
+    <cfRule type="expression" dxfId="16" priority="20" stopIfTrue="1">
+      <formula>$S47=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="21" stopIfTrue="1">
+      <formula>$S46=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J47:J50">
+    <cfRule type="expression" dxfId="13" priority="16" stopIfTrue="1">
+      <formula>$S47=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="12" priority="17" stopIfTrue="1">
+      <formula>$S46=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:A46 J5:J46">
     <cfRule type="expression" dxfId="11" priority="4" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
@@ -3065,7 +2978,7 @@
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:L50 C5:H50">
+  <conditionalFormatting sqref="K5:L46 C5:H46">
     <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
@@ -3073,7 +2986,7 @@
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I50 M5:M50">
+  <conditionalFormatting sqref="I5:I46 M5:M46">
     <cfRule type="expression" dxfId="7" priority="8" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
@@ -3101,7 +3014,7 @@
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B50">
+  <conditionalFormatting sqref="B5:B46">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-20 12:29)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C8DA191-B0B7-594B-AF6A-0272F8CDAAD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A3F9C26-CCB1-034D-BBE4-E4ECAC955DC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -370,7 +370,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="25">
     <dxf>
       <border>
         <top style="thin">
@@ -529,6 +529,22 @@
     </dxf>
     <dxf>
       <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
         <top style="thin">
           <color indexed="64"/>
         </top>
@@ -542,7 +558,7 @@
         <right style="hair">
           <color indexed="64"/>
         </right>
-        <top style="hair">
+        <top style="thin">
           <color indexed="64"/>
         </top>
         <bottom style="hair">
@@ -552,13 +568,13 @@
     </dxf>
     <dxf>
       <border>
-        <left style="thin">
+        <left style="hair">
           <color indexed="64"/>
         </left>
-        <right style="hair">
+        <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="thin">
+        <top style="hair">
           <color indexed="64"/>
         </top>
         <bottom style="hair">
@@ -581,22 +597,6 @@
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
         <top style="thin">
           <color indexed="64"/>
         </top>
@@ -626,6 +626,13 @@
         <bottom style="hair">
           <color indexed="64"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
       </border>
     </dxf>
     <dxf>
@@ -1034,7 +1041,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46125</v>
+        <v>46129</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1136,22 +1143,22 @@
         <v>73656.399999999994</v>
       </c>
       <c r="H4" s="4">
-        <v>36746.69</v>
+        <v>39747.14</v>
       </c>
       <c r="I4" s="4">
-        <v>110403.09</v>
+        <v>113403.54</v>
       </c>
       <c r="J4" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" s="4">
-        <v>0</v>
+        <v>28877.5</v>
       </c>
       <c r="L4" s="4">
-        <v>344649.08</v>
+        <v>341648.63</v>
       </c>
       <c r="M4" s="4">
-        <v>344649.08</v>
+        <v>370526.13</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1177,10 +1184,10 @@
         <v>29477.7</v>
       </c>
       <c r="H5" s="4">
-        <v>62549.13</v>
+        <v>71225.600000000006</v>
       </c>
       <c r="I5" s="4">
-        <v>92026.83</v>
+        <v>100703.3</v>
       </c>
       <c r="J5" s="3">
         <v>1</v>
@@ -1189,10 +1196,10 @@
         <v>23801.34</v>
       </c>
       <c r="L5" s="4">
-        <v>116422.94</v>
+        <v>112121.47</v>
       </c>
       <c r="M5" s="4">
-        <v>140224.28</v>
+        <v>135922.81</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -1218,10 +1225,10 @@
         <v>2244.4699999999998</v>
       </c>
       <c r="H6" s="4">
-        <v>33777.410000000003</v>
+        <v>39653.03</v>
       </c>
       <c r="I6" s="4">
-        <v>36021.879999999997</v>
+        <v>41897.5</v>
       </c>
       <c r="J6" s="3">
         <v>0</v>
@@ -1230,10 +1237,10 @@
         <v>0</v>
       </c>
       <c r="L6" s="4">
-        <v>145975.84</v>
+        <v>140438.91</v>
       </c>
       <c r="M6" s="4">
-        <v>145975.84</v>
+        <v>140438.91</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -1241,7 +1248,7 @@
         <v>104750</v>
       </c>
       <c r="B7" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>10</v>
@@ -1279,72 +1286,72 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>114100</v>
+        <v>90355</v>
       </c>
       <c r="B8" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="D8" s="11">
-        <v>45863</v>
+        <v>43949</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="4">
-        <v>0</v>
+        <v>5257.75</v>
       </c>
       <c r="H8" s="4">
-        <v>21150.02</v>
+        <v>18372.009999999998</v>
       </c>
       <c r="I8" s="4">
-        <v>21150.02</v>
+        <v>23629.759999999998</v>
       </c>
       <c r="J8" s="3">
         <v>1</v>
       </c>
       <c r="K8" s="4">
-        <v>20413.86</v>
+        <v>12557.28</v>
       </c>
       <c r="L8" s="4">
-        <v>38941.47</v>
+        <v>41958.02</v>
       </c>
       <c r="M8" s="4">
-        <v>59355.33</v>
+        <v>54515.3</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>110575</v>
+        <v>47116</v>
       </c>
       <c r="B9" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="D9" s="11">
-        <v>45583</v>
+        <v>44616</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F9" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="4">
-        <v>0</v>
+        <v>15755.23</v>
       </c>
       <c r="H9" s="4">
-        <v>14385.86</v>
+        <v>7784.62</v>
       </c>
       <c r="I9" s="4">
-        <v>14385.86</v>
+        <v>23539.85</v>
       </c>
       <c r="J9" s="3">
         <v>0</v>
@@ -1353,24 +1360,24 @@
         <v>0</v>
       </c>
       <c r="L9" s="4">
-        <v>86315.15</v>
+        <v>60148.11</v>
       </c>
       <c r="M9" s="4">
-        <v>86315.15</v>
+        <v>60148.11</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>107488</v>
+        <v>114100</v>
       </c>
       <c r="B10" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D10" s="11">
-        <v>45440</v>
+        <v>45863</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>51</v>
@@ -1382,36 +1389,36 @@
         <v>0</v>
       </c>
       <c r="H10" s="4">
-        <v>8873.25</v>
+        <v>23280.63</v>
       </c>
       <c r="I10" s="4">
-        <v>8873.25</v>
+        <v>23280.63</v>
       </c>
       <c r="J10" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" s="4">
-        <v>0</v>
+        <v>20413.86</v>
       </c>
       <c r="L10" s="4">
-        <v>108547.73</v>
+        <v>36810.86</v>
       </c>
       <c r="M10" s="4">
-        <v>108547.73</v>
+        <v>57224.72</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>108404</v>
+        <v>107488</v>
       </c>
       <c r="B11" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D11" s="11">
-        <v>45467</v>
+        <v>45440</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>51</v>
@@ -1423,10 +1430,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="4">
-        <v>7900.28</v>
+        <v>20787.77</v>
       </c>
       <c r="I11" s="4">
-        <v>7900.28</v>
+        <v>20787.77</v>
       </c>
       <c r="J11" s="3">
         <v>0</v>
@@ -1435,24 +1442,24 @@
         <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>22176.42</v>
+        <v>96633.21</v>
       </c>
       <c r="M11" s="4">
-        <v>22176.42</v>
+        <v>96633.21</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>47116</v>
+        <v>110575</v>
       </c>
       <c r="B12" s="2">
         <v>2043</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="D12" s="11">
-        <v>44616</v>
+        <v>45583</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>51</v>
@@ -1464,22 +1471,22 @@
         <v>0</v>
       </c>
       <c r="H12" s="4">
-        <v>7784.62</v>
+        <v>14385.86</v>
       </c>
       <c r="I12" s="4">
-        <v>7784.62</v>
+        <v>14385.86</v>
       </c>
       <c r="J12" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" s="4">
-        <v>15689.6</v>
+        <v>0</v>
       </c>
       <c r="L12" s="4">
-        <v>60082.48</v>
+        <v>86315.15</v>
       </c>
       <c r="M12" s="4">
-        <v>75772.08</v>
+        <v>86315.15</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
@@ -1505,10 +1512,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="4">
-        <v>7530.24</v>
+        <v>10520.76</v>
       </c>
       <c r="I13" s="4">
-        <v>7530.24</v>
+        <v>10520.76</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1517,24 +1524,24 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>5455.03</v>
+        <v>2464.4699999999998</v>
       </c>
       <c r="M13" s="4">
-        <v>5455.03</v>
+        <v>2464.4699999999998</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>108405</v>
+        <v>108404</v>
       </c>
       <c r="B14" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="D14" s="11">
-        <v>45471</v>
+        <v>45467</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>51</v>
@@ -1546,10 +1553,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="4">
-        <v>5525.52</v>
+        <v>7900.28</v>
       </c>
       <c r="I14" s="4">
-        <v>5525.52</v>
+        <v>7900.28</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1558,24 +1565,24 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>7002.07</v>
+        <v>33081.01</v>
       </c>
       <c r="M14" s="4">
-        <v>7002.07</v>
+        <v>33081.01</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>115047</v>
+        <v>108405</v>
       </c>
       <c r="B15" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>5</v>
+        <v>42</v>
       </c>
       <c r="D15" s="11">
-        <v>45944</v>
+        <v>45471</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>51</v>
@@ -1587,10 +1594,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>5025.2</v>
+        <v>7542.1</v>
       </c>
       <c r="I15" s="4">
-        <v>5025.2</v>
+        <v>7542.1</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1599,24 +1606,24 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>35787.599999999999</v>
+        <v>4985.49</v>
       </c>
       <c r="M15" s="4">
-        <v>35787.599999999999</v>
+        <v>4985.49</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>113450</v>
+        <v>110105</v>
       </c>
       <c r="B16" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D16" s="11">
-        <v>45852</v>
+        <v>45560</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>51</v>
@@ -1628,10 +1635,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>4898.1400000000003</v>
+        <v>7373.6</v>
       </c>
       <c r="I16" s="4">
-        <v>4898.1400000000003</v>
+        <v>7373.6</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1640,24 +1647,24 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>5799.55</v>
+        <v>5703.16</v>
       </c>
       <c r="M16" s="4">
-        <v>5799.55</v>
+        <v>5703.16</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>101640</v>
+        <v>113450</v>
       </c>
       <c r="B17" s="2">
         <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="D17" s="11">
-        <v>45104</v>
+        <v>45852</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>51</v>
@@ -1669,10 +1676,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>4718.59</v>
+        <v>6690.87</v>
       </c>
       <c r="I17" s="4">
-        <v>4718.59</v>
+        <v>6690.87</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1681,24 +1688,24 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>3204.95</v>
+        <v>4006.82</v>
       </c>
       <c r="M17" s="4">
-        <v>3204.95</v>
+        <v>4006.82</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>100677</v>
+        <v>109998</v>
       </c>
       <c r="B18" s="2">
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="D18" s="11">
-        <v>44999</v>
+        <v>45596</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>51</v>
@@ -1710,10 +1717,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>4681.6099999999997</v>
+        <v>5824.66</v>
       </c>
       <c r="I18" s="4">
-        <v>4681.6099999999997</v>
+        <v>5824.66</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1722,24 +1729,24 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>34806.33</v>
+        <v>0</v>
       </c>
       <c r="M18" s="4">
-        <v>34806.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>113076</v>
+        <v>104718</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="D19" s="11">
-        <v>45806</v>
+        <v>45264</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>51</v>
@@ -1751,10 +1758,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>4558.5200000000004</v>
+        <v>5284.89</v>
       </c>
       <c r="I19" s="4">
-        <v>4558.5200000000004</v>
+        <v>5284.89</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1763,24 +1770,24 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>9117.0400000000009</v>
+        <v>101355.28</v>
       </c>
       <c r="M19" s="4">
-        <v>9117.0400000000009</v>
+        <v>101355.28</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>88234</v>
+        <v>90177</v>
       </c>
       <c r="B20" s="2">
         <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="D20" s="11">
-        <v>43794</v>
+        <v>43949</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>51</v>
@@ -1792,10 +1799,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>4242.34</v>
+        <v>5199.32</v>
       </c>
       <c r="I20" s="4">
-        <v>4242.34</v>
+        <v>5199.32</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1804,24 +1811,24 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>15745.12</v>
+        <v>0</v>
       </c>
       <c r="M20" s="4">
-        <v>15745.12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>109998</v>
+        <v>104343</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="D21" s="11">
-        <v>45596</v>
+        <v>45201</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>51</v>
@@ -1833,10 +1840,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>2958.1</v>
+        <v>5175.96</v>
       </c>
       <c r="I21" s="4">
-        <v>2958.1</v>
+        <v>5175.96</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1845,39 +1852,39 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>0</v>
+        <v>57105.67</v>
       </c>
       <c r="M21" s="4">
-        <v>0</v>
+        <v>57105.67</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>112083</v>
+        <v>115047</v>
       </c>
       <c r="B22" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="D22" s="11">
-        <v>45736</v>
+        <v>45944</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F22" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" s="4">
-        <v>1795.63</v>
+        <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>0</v>
+        <v>5025.2</v>
       </c>
       <c r="I22" s="4">
-        <v>1795.63</v>
+        <v>5025.2</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1886,24 +1893,24 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>19751.93</v>
+        <v>35787.599999999999</v>
       </c>
       <c r="M22" s="4">
-        <v>19751.93</v>
+        <v>35787.599999999999</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>104343</v>
+        <v>101640</v>
       </c>
       <c r="B23" s="2">
         <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="D23" s="11">
-        <v>45201</v>
+        <v>45104</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>51</v>
@@ -1915,10 +1922,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>1756.01</v>
+        <v>4718.59</v>
       </c>
       <c r="I23" s="4">
-        <v>1756.01</v>
+        <v>4718.59</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1927,24 +1934,24 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>60525.61</v>
+        <v>3204.95</v>
       </c>
       <c r="M23" s="4">
-        <v>60525.61</v>
+        <v>3204.95</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>104718</v>
+        <v>100677</v>
       </c>
       <c r="B24" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D24" s="11">
-        <v>45264</v>
+        <v>44999</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>51</v>
@@ -1956,10 +1963,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>1731.32</v>
+        <v>4681.6099999999997</v>
       </c>
       <c r="I24" s="4">
-        <v>1731.32</v>
+        <v>4681.6099999999997</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1968,24 +1975,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>104908.85</v>
+        <v>34806.33</v>
       </c>
       <c r="M24" s="4">
-        <v>104908.85</v>
+        <v>34806.33</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>114157</v>
+        <v>113076</v>
       </c>
       <c r="B25" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="D25" s="11">
-        <v>45904</v>
+        <v>45806</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>51</v>
@@ -1997,10 +2004,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>1637.49</v>
+        <v>4558.5200000000004</v>
       </c>
       <c r="I25" s="4">
-        <v>1637.49</v>
+        <v>4558.5200000000004</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -2009,24 +2016,24 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>65218.85</v>
+        <v>9117.0400000000009</v>
       </c>
       <c r="M25" s="4">
-        <v>65218.85</v>
+        <v>9117.0400000000009</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>118069</v>
+        <v>88234</v>
       </c>
       <c r="B26" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="D26" s="11">
-        <v>46105</v>
+        <v>43794</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>51</v>
@@ -2038,10 +2045,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>0</v>
+        <v>4242.34</v>
       </c>
       <c r="I26" s="4">
-        <v>0</v>
+        <v>4242.34</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2050,24 +2057,24 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>19562.52</v>
+        <v>15745.12</v>
       </c>
       <c r="M26" s="4">
-        <v>19562.52</v>
+        <v>15745.12</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>116883</v>
+        <v>95148</v>
       </c>
       <c r="B27" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="D27" s="11">
-        <v>46007</v>
+        <v>44916</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>51</v>
@@ -2079,36 +2086,36 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>0</v>
+        <v>3887.59</v>
       </c>
       <c r="I27" s="4">
-        <v>0</v>
+        <v>3887.59</v>
       </c>
       <c r="J27" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" s="4">
-        <v>2174.0100000000002</v>
+        <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>88699.520000000004</v>
+        <v>0</v>
       </c>
       <c r="M27" s="4">
-        <v>90873.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>116876</v>
+        <v>105696</v>
       </c>
       <c r="B28" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="D28" s="11">
-        <v>46111</v>
+        <v>45279</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>51</v>
@@ -2120,51 +2127,51 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>0</v>
+        <v>2866.56</v>
       </c>
       <c r="I28" s="4">
-        <v>0</v>
+        <v>2866.56</v>
       </c>
       <c r="J28" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28" s="4">
-        <v>0</v>
+        <v>36118.519999999997</v>
       </c>
       <c r="L28" s="4">
-        <v>18185.59</v>
+        <v>25379.03</v>
       </c>
       <c r="M28" s="4">
-        <v>18185.59</v>
+        <v>61497.55</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>116060</v>
+        <v>112083</v>
       </c>
       <c r="B29" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="D29" s="11">
-        <v>46010</v>
+        <v>45736</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F29" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" s="4">
-        <v>0</v>
+        <v>1795.63</v>
       </c>
       <c r="H29" s="4">
         <v>0</v>
       </c>
       <c r="I29" s="4">
-        <v>0</v>
+        <v>1795.63</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2173,24 +2180,24 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>62278.86</v>
+        <v>19751.93</v>
       </c>
       <c r="M29" s="4">
-        <v>62278.86</v>
+        <v>19751.93</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>115404</v>
+        <v>116060</v>
       </c>
       <c r="B30" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D30" s="11">
-        <v>45986</v>
+        <v>46010</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>51</v>
@@ -2202,10 +2209,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>0</v>
+        <v>1775.95</v>
       </c>
       <c r="I30" s="4">
-        <v>0</v>
+        <v>1775.95</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2214,24 +2221,24 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>12170.29</v>
+        <v>60502.91</v>
       </c>
       <c r="M30" s="4">
-        <v>12170.29</v>
+        <v>60502.91</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>114431</v>
+        <v>114157</v>
       </c>
       <c r="B31" s="2">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="D31" s="11">
-        <v>45930</v>
+        <v>45904</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>51</v>
@@ -2243,10 +2250,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>0</v>
+        <v>1637.49</v>
       </c>
       <c r="I31" s="4">
-        <v>0</v>
+        <v>1637.49</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -2255,27 +2262,27 @@
         <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>21758.76</v>
+        <v>37956.89</v>
       </c>
       <c r="M31" s="4">
-        <v>21758.76</v>
+        <v>37956.89</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>112522</v>
+        <v>118069</v>
       </c>
       <c r="B32" s="2">
         <v>2856</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="D32" s="11">
-        <v>45776</v>
+        <v>46105</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F32" s="3">
         <v>0</v>
@@ -2296,24 +2303,24 @@
         <v>0</v>
       </c>
       <c r="L32" s="4">
-        <v>6684.84</v>
+        <v>19562.52</v>
       </c>
       <c r="M32" s="4">
-        <v>6684.84</v>
+        <v>19562.52</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>111056</v>
+        <v>116883</v>
       </c>
       <c r="B33" s="2">
-        <v>2692</v>
+        <v>2856</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="D33" s="11">
-        <v>45639</v>
+        <v>46126</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>51</v>
@@ -2334,27 +2341,27 @@
         <v>1</v>
       </c>
       <c r="K33" s="4">
-        <v>61752.21</v>
+        <v>2174.0100000000002</v>
       </c>
       <c r="L33" s="4">
-        <v>56209.91</v>
+        <v>88699.520000000004</v>
       </c>
       <c r="M33" s="4">
-        <v>117962.12</v>
+        <v>90873.53</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>110105</v>
+        <v>116876</v>
       </c>
       <c r="B34" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D34" s="11">
-        <v>45560</v>
+        <v>46111</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>51</v>
@@ -2378,24 +2385,24 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>13077.25</v>
+        <v>18185.59</v>
       </c>
       <c r="M34" s="4">
-        <v>13077.25</v>
+        <v>18185.59</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>109007</v>
+        <v>115404</v>
       </c>
       <c r="B35" s="2">
         <v>2043</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D35" s="11">
-        <v>45525</v>
+        <v>45986</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>51</v>
@@ -2419,24 +2426,24 @@
         <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>6177.09</v>
+        <v>12170.29</v>
       </c>
       <c r="M35" s="4">
-        <v>6177.09</v>
+        <v>12170.29</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>106018</v>
+        <v>114431</v>
       </c>
       <c r="B36" s="2">
         <v>2043</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="D36" s="11">
-        <v>45344</v>
+        <v>45930</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>51</v>
@@ -2460,24 +2467,24 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>30708.15</v>
+        <v>21758.76</v>
       </c>
       <c r="M36" s="4">
-        <v>30708.15</v>
+        <v>21758.76</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>105696</v>
+        <v>112522</v>
       </c>
       <c r="B37" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="D37" s="11">
-        <v>45279</v>
+        <v>45776</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>51</v>
@@ -2495,30 +2502,30 @@
         <v>0</v>
       </c>
       <c r="J37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K37" s="4">
-        <v>36118.519999999997</v>
+        <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>31399.77</v>
+        <v>6684.84</v>
       </c>
       <c r="M37" s="4">
-        <v>67518.289999999994</v>
+        <v>6684.84</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>102825</v>
+        <v>111056</v>
       </c>
       <c r="B38" s="2">
         <v>2043</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D38" s="11">
-        <v>45117</v>
+        <v>45639</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>51</v>
@@ -2539,27 +2546,27 @@
         <v>1</v>
       </c>
       <c r="K38" s="4">
-        <v>30557.77</v>
+        <v>61752.21</v>
       </c>
       <c r="L38" s="4">
-        <v>21637.32</v>
+        <v>56209.91</v>
       </c>
       <c r="M38" s="4">
-        <v>52195.09</v>
+        <v>117962.12</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>95148</v>
+        <v>109007</v>
       </c>
       <c r="B39" s="2">
         <v>2043</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D39" s="11">
-        <v>44916</v>
+        <v>45525</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>51</v>
@@ -2583,24 +2590,24 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>3887.54</v>
+        <v>6177.09</v>
       </c>
       <c r="M39" s="4">
-        <v>3887.54</v>
+        <v>6177.09</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>94156</v>
+        <v>106018</v>
       </c>
       <c r="B40" s="2">
         <v>2043</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="D40" s="11">
-        <v>44159</v>
+        <v>45344</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>51</v>
@@ -2624,24 +2631,24 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>7466.11</v>
+        <v>30708.15</v>
       </c>
       <c r="M40" s="4">
-        <v>7466.11</v>
+        <v>30708.15</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>90355</v>
+        <v>102825</v>
       </c>
       <c r="B41" s="2">
         <v>2043</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="D41" s="11">
-        <v>43949</v>
+        <v>45117</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>51</v>
@@ -2662,27 +2669,27 @@
         <v>1</v>
       </c>
       <c r="K41" s="4">
-        <v>6757.44</v>
+        <v>30557.77</v>
       </c>
       <c r="L41" s="4">
-        <v>42913.120000000003</v>
+        <v>21637.32</v>
       </c>
       <c r="M41" s="4">
-        <v>49670.559999999998</v>
+        <v>52195.09</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>90177</v>
+        <v>94156</v>
       </c>
       <c r="B42" s="2">
         <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D42" s="11">
-        <v>43949</v>
+        <v>44159</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>51</v>
@@ -2706,10 +2713,10 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>5199.32</v>
+        <v>7466.11</v>
       </c>
       <c r="M42" s="4">
-        <v>5199.32</v>
+        <v>7466.11</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
@@ -2939,10 +2946,10 @@
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="A47:B50">
-    <cfRule type="expression" dxfId="22" priority="13" stopIfTrue="1">
+    <cfRule type="expression" dxfId="23" priority="13" stopIfTrue="1">
       <formula>$S47=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="14" stopIfTrue="1">
+    <cfRule type="expression" dxfId="22" priority="14" stopIfTrue="1">
       <formula>$S46=1</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2950,24 +2957,20 @@
     <cfRule type="expression" dxfId="19" priority="18" stopIfTrue="1">
       <formula>$S47=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="19" stopIfTrue="1">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C47:M50">
+    <cfRule type="expression" dxfId="18" priority="29" stopIfTrue="1">
       <formula>$S46=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I47:I50 M47:M50">
-    <cfRule type="expression" dxfId="16" priority="20" stopIfTrue="1">
+    <cfRule type="expression" dxfId="15" priority="20" stopIfTrue="1">
       <formula>$S47=1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="15" priority="21" stopIfTrue="1">
-      <formula>$S46=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J47:J50">
-    <cfRule type="expression" dxfId="13" priority="16" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="16" stopIfTrue="1">
       <formula>$S47=1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="12" priority="17" stopIfTrue="1">
-      <formula>$S46=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:A46 J5:J46">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-22 11:07)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A3F9C26-CCB1-034D-BBE4-E4ECAC955DC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{829B533F-1791-F547-A53F-03F448DB58ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -370,163 +370,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="25">
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="13">
     <dxf>
       <border>
         <left style="thin">
@@ -1041,7 +885,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1137,28 +981,28 @@
         <v>51</v>
       </c>
       <c r="F4" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G4" s="4">
-        <v>73656.399999999994</v>
+        <v>126272.25</v>
       </c>
       <c r="H4" s="4">
-        <v>39747.14</v>
+        <v>41937.230000000003</v>
       </c>
       <c r="I4" s="4">
-        <v>113403.54</v>
+        <v>168209.48</v>
       </c>
       <c r="J4" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" s="4">
-        <v>28877.5</v>
+        <v>0</v>
       </c>
       <c r="L4" s="4">
-        <v>341648.63</v>
+        <v>339458.54</v>
       </c>
       <c r="M4" s="4">
-        <v>370526.13</v>
+        <v>339458.54</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1245,98 +1089,98 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>104750</v>
+        <v>105696</v>
       </c>
       <c r="B7" s="2">
         <v>2043</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D7" s="11">
-        <v>45236</v>
+        <v>45279</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F7" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7" s="4">
-        <v>1799.5</v>
+        <v>36118.519999999997</v>
       </c>
       <c r="H7" s="4">
-        <v>31457.13</v>
+        <v>2866.56</v>
       </c>
       <c r="I7" s="4">
-        <v>33256.629999999997</v>
+        <v>38985.08</v>
       </c>
       <c r="J7" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" s="4">
-        <v>2088.27</v>
+        <v>0</v>
       </c>
       <c r="L7" s="4">
-        <v>56777.83</v>
+        <v>25379.03</v>
       </c>
       <c r="M7" s="4">
-        <v>58866.1</v>
+        <v>25379.03</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>90355</v>
+        <v>104750</v>
       </c>
       <c r="B8" s="2">
         <v>2043</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="D8" s="11">
-        <v>43949</v>
+        <v>45236</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F8" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" s="4">
-        <v>5257.75</v>
+        <v>1799.5</v>
       </c>
       <c r="H8" s="4">
-        <v>18372.009999999998</v>
+        <v>31457.13</v>
       </c>
       <c r="I8" s="4">
-        <v>23629.759999999998</v>
+        <v>33256.629999999997</v>
       </c>
       <c r="J8" s="3">
         <v>1</v>
       </c>
       <c r="K8" s="4">
-        <v>12557.28</v>
+        <v>2088.27</v>
       </c>
       <c r="L8" s="4">
-        <v>41958.02</v>
+        <v>56777.83</v>
       </c>
       <c r="M8" s="4">
-        <v>54515.3</v>
+        <v>58866.1</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>47116</v>
+        <v>90355</v>
       </c>
       <c r="B9" s="2">
         <v>2043</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D9" s="11">
-        <v>44616</v>
+        <v>43949</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>51</v>
@@ -1345,80 +1189,80 @@
         <v>1</v>
       </c>
       <c r="G9" s="4">
-        <v>15755.23</v>
+        <v>5257.75</v>
       </c>
       <c r="H9" s="4">
-        <v>7784.62</v>
+        <v>18372.009999999998</v>
       </c>
       <c r="I9" s="4">
-        <v>23539.85</v>
+        <v>23629.759999999998</v>
       </c>
       <c r="J9" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" s="4">
-        <v>0</v>
+        <v>12557.28</v>
       </c>
       <c r="L9" s="4">
-        <v>60148.11</v>
+        <v>41958.02</v>
       </c>
       <c r="M9" s="4">
-        <v>60148.11</v>
+        <v>54515.3</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>114100</v>
+        <v>47116</v>
       </c>
       <c r="B10" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="D10" s="11">
-        <v>45863</v>
+        <v>44616</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F10" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="4">
-        <v>0</v>
+        <v>15755.23</v>
       </c>
       <c r="H10" s="4">
-        <v>23280.63</v>
+        <v>7784.62</v>
       </c>
       <c r="I10" s="4">
-        <v>23280.63</v>
+        <v>23539.85</v>
       </c>
       <c r="J10" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" s="4">
-        <v>20413.86</v>
+        <v>0</v>
       </c>
       <c r="L10" s="4">
-        <v>36810.86</v>
+        <v>60148.11</v>
       </c>
       <c r="M10" s="4">
-        <v>57224.72</v>
+        <v>60148.11</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>107488</v>
+        <v>114100</v>
       </c>
       <c r="B11" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D11" s="11">
-        <v>45440</v>
+        <v>45863</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>51</v>
@@ -1430,36 +1274,36 @@
         <v>0</v>
       </c>
       <c r="H11" s="4">
-        <v>20787.77</v>
+        <v>23280.63</v>
       </c>
       <c r="I11" s="4">
-        <v>20787.77</v>
+        <v>23280.63</v>
       </c>
       <c r="J11" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" s="4">
-        <v>0</v>
+        <v>20413.86</v>
       </c>
       <c r="L11" s="4">
-        <v>96633.21</v>
+        <v>36810.86</v>
       </c>
       <c r="M11" s="4">
-        <v>96633.21</v>
+        <v>57224.72</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>110575</v>
+        <v>107488</v>
       </c>
       <c r="B12" s="2">
         <v>2043</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="D12" s="11">
-        <v>45583</v>
+        <v>45440</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>51</v>
@@ -1471,10 +1315,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="4">
-        <v>14385.86</v>
+        <v>20787.77</v>
       </c>
       <c r="I12" s="4">
-        <v>14385.86</v>
+        <v>20787.77</v>
       </c>
       <c r="J12" s="3">
         <v>0</v>
@@ -1483,24 +1327,24 @@
         <v>0</v>
       </c>
       <c r="L12" s="4">
-        <v>86315.15</v>
+        <v>96633.21</v>
       </c>
       <c r="M12" s="4">
-        <v>86315.15</v>
+        <v>96633.21</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>117440</v>
+        <v>110575</v>
       </c>
       <c r="B13" s="2">
         <v>2043</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="D13" s="11">
-        <v>46059</v>
+        <v>45583</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>51</v>
@@ -1512,10 +1356,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="4">
-        <v>10520.76</v>
+        <v>14385.86</v>
       </c>
       <c r="I13" s="4">
-        <v>10520.76</v>
+        <v>14385.86</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1524,24 +1368,24 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>2464.4699999999998</v>
+        <v>86315.15</v>
       </c>
       <c r="M13" s="4">
-        <v>2464.4699999999998</v>
+        <v>86315.15</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>108404</v>
+        <v>117440</v>
       </c>
       <c r="B14" s="2">
         <v>2043</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="D14" s="11">
-        <v>45467</v>
+        <v>46059</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>51</v>
@@ -1553,10 +1397,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="4">
-        <v>7900.28</v>
+        <v>10520.76</v>
       </c>
       <c r="I14" s="4">
-        <v>7900.28</v>
+        <v>10520.76</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1565,24 +1409,24 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>33081.01</v>
+        <v>2464.4699999999998</v>
       </c>
       <c r="M14" s="4">
-        <v>33081.01</v>
+        <v>2464.4699999999998</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>108405</v>
+        <v>108404</v>
       </c>
       <c r="B15" s="2">
         <v>2043</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="D15" s="11">
-        <v>45471</v>
+        <v>45467</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>51</v>
@@ -1594,10 +1438,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>7542.1</v>
+        <v>7900.28</v>
       </c>
       <c r="I15" s="4">
-        <v>7542.1</v>
+        <v>7900.28</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1606,24 +1450,24 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>4985.49</v>
+        <v>33081.01</v>
       </c>
       <c r="M15" s="4">
-        <v>4985.49</v>
+        <v>33081.01</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>110105</v>
+        <v>108405</v>
       </c>
       <c r="B16" s="2">
         <v>2043</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D16" s="11">
-        <v>45560</v>
+        <v>45471</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>51</v>
@@ -1635,10 +1479,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>7373.6</v>
+        <v>7542.1</v>
       </c>
       <c r="I16" s="4">
-        <v>7373.6</v>
+        <v>7542.1</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1647,24 +1491,24 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>5703.16</v>
+        <v>4985.49</v>
       </c>
       <c r="M16" s="4">
-        <v>5703.16</v>
+        <v>4985.49</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>113450</v>
+        <v>110105</v>
       </c>
       <c r="B17" s="2">
         <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D17" s="11">
-        <v>45852</v>
+        <v>45560</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>51</v>
@@ -1676,10 +1520,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>6690.87</v>
+        <v>7373.6</v>
       </c>
       <c r="I17" s="4">
-        <v>6690.87</v>
+        <v>7373.6</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1688,24 +1532,24 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>4006.82</v>
+        <v>5703.16</v>
       </c>
       <c r="M17" s="4">
-        <v>4006.82</v>
+        <v>5703.16</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>109998</v>
+        <v>113450</v>
       </c>
       <c r="B18" s="2">
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="D18" s="11">
-        <v>45596</v>
+        <v>45852</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>51</v>
@@ -1717,10 +1561,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>5824.66</v>
+        <v>6690.87</v>
       </c>
       <c r="I18" s="4">
-        <v>5824.66</v>
+        <v>6690.87</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1729,24 +1573,24 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>0</v>
+        <v>4006.82</v>
       </c>
       <c r="M18" s="4">
-        <v>0</v>
+        <v>4006.82</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>104718</v>
+        <v>109998</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="D19" s="11">
-        <v>45264</v>
+        <v>45596</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>51</v>
@@ -1758,10 +1602,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>5284.89</v>
+        <v>5824.66</v>
       </c>
       <c r="I19" s="4">
-        <v>5284.89</v>
+        <v>5824.66</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1770,24 +1614,24 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>101355.28</v>
+        <v>0</v>
       </c>
       <c r="M19" s="4">
-        <v>101355.28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>90177</v>
+        <v>104718</v>
       </c>
       <c r="B20" s="2">
         <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="D20" s="11">
-        <v>43949</v>
+        <v>45264</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>51</v>
@@ -1799,10 +1643,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>5199.32</v>
+        <v>5284.89</v>
       </c>
       <c r="I20" s="4">
-        <v>5199.32</v>
+        <v>5284.89</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1811,24 +1655,24 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>0</v>
+        <v>101355.28</v>
       </c>
       <c r="M20" s="4">
-        <v>0</v>
+        <v>101355.28</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>104343</v>
+        <v>90177</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="D21" s="11">
-        <v>45201</v>
+        <v>43949</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>51</v>
@@ -1840,10 +1684,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>5175.96</v>
+        <v>5199.32</v>
       </c>
       <c r="I21" s="4">
-        <v>5175.96</v>
+        <v>5199.32</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1852,24 +1696,24 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>57105.67</v>
+        <v>0</v>
       </c>
       <c r="M21" s="4">
-        <v>57105.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>115047</v>
+        <v>104343</v>
       </c>
       <c r="B22" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="D22" s="11">
-        <v>45944</v>
+        <v>45201</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>51</v>
@@ -1881,36 +1725,36 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>5025.2</v>
+        <v>5175.96</v>
       </c>
       <c r="I22" s="4">
-        <v>5025.2</v>
+        <v>5175.96</v>
       </c>
       <c r="J22" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22" s="4">
-        <v>0</v>
+        <v>2473.56</v>
       </c>
       <c r="L22" s="4">
-        <v>35787.599999999999</v>
+        <v>57105.67</v>
       </c>
       <c r="M22" s="4">
-        <v>35787.599999999999</v>
+        <v>59579.23</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>101640</v>
+        <v>115047</v>
       </c>
       <c r="B23" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D23" s="11">
-        <v>45104</v>
+        <v>45944</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>51</v>
@@ -1922,10 +1766,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>4718.59</v>
+        <v>5025.2</v>
       </c>
       <c r="I23" s="4">
-        <v>4718.59</v>
+        <v>5025.2</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1934,24 +1778,24 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>3204.95</v>
+        <v>35787.599999999999</v>
       </c>
       <c r="M23" s="4">
-        <v>3204.95</v>
+        <v>35787.599999999999</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>100677</v>
+        <v>101640</v>
       </c>
       <c r="B24" s="2">
         <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D24" s="11">
-        <v>44999</v>
+        <v>45104</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>51</v>
@@ -1963,10 +1807,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>4681.6099999999997</v>
+        <v>4718.59</v>
       </c>
       <c r="I24" s="4">
-        <v>4681.6099999999997</v>
+        <v>4718.59</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1975,24 +1819,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>34806.33</v>
+        <v>3204.95</v>
       </c>
       <c r="M24" s="4">
-        <v>34806.33</v>
+        <v>3204.95</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>113076</v>
+        <v>100677</v>
       </c>
       <c r="B25" s="2">
         <v>2043</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="D25" s="11">
-        <v>45806</v>
+        <v>44999</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>51</v>
@@ -2004,10 +1848,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>4558.5200000000004</v>
+        <v>4681.6099999999997</v>
       </c>
       <c r="I25" s="4">
-        <v>4558.5200000000004</v>
+        <v>4681.6099999999997</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -2016,24 +1860,24 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>9117.0400000000009</v>
+        <v>34806.33</v>
       </c>
       <c r="M25" s="4">
-        <v>9117.0400000000009</v>
+        <v>34806.33</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>88234</v>
+        <v>113076</v>
       </c>
       <c r="B26" s="2">
         <v>2043</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="D26" s="11">
-        <v>43794</v>
+        <v>45806</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>51</v>
@@ -2045,10 +1889,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>4242.34</v>
+        <v>4558.5200000000004</v>
       </c>
       <c r="I26" s="4">
-        <v>4242.34</v>
+        <v>4558.5200000000004</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2057,24 +1901,24 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>15745.12</v>
+        <v>9117.0400000000009</v>
       </c>
       <c r="M26" s="4">
-        <v>15745.12</v>
+        <v>9117.0400000000009</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>95148</v>
+        <v>88234</v>
       </c>
       <c r="B27" s="2">
         <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="D27" s="11">
-        <v>44916</v>
+        <v>43794</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>51</v>
@@ -2086,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>3887.59</v>
+        <v>4242.34</v>
       </c>
       <c r="I27" s="4">
-        <v>3887.59</v>
+        <v>4242.34</v>
       </c>
       <c r="J27" s="3">
         <v>0</v>
@@ -2098,24 +1942,24 @@
         <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>0</v>
+        <v>15745.12</v>
       </c>
       <c r="M27" s="4">
-        <v>0</v>
+        <v>15745.12</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>105696</v>
+        <v>95148</v>
       </c>
       <c r="B28" s="2">
         <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="D28" s="11">
-        <v>45279</v>
+        <v>44916</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>51</v>
@@ -2127,51 +1971,51 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>2866.56</v>
+        <v>3887.59</v>
       </c>
       <c r="I28" s="4">
-        <v>2866.56</v>
+        <v>3887.59</v>
       </c>
       <c r="J28" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" s="4">
-        <v>36118.519999999997</v>
+        <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>25379.03</v>
+        <v>0</v>
       </c>
       <c r="M28" s="4">
-        <v>61497.55</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>112083</v>
+        <v>106018</v>
       </c>
       <c r="B29" s="2">
         <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="D29" s="11">
-        <v>45736</v>
+        <v>45344</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F29" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G29" s="4">
-        <v>1795.63</v>
+        <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>0</v>
+        <v>3669.62</v>
       </c>
       <c r="I29" s="4">
-        <v>1795.63</v>
+        <v>3669.62</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2180,24 +2024,24 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>19751.93</v>
+        <v>25348.91</v>
       </c>
       <c r="M29" s="4">
-        <v>19751.93</v>
+        <v>25348.91</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>116060</v>
+        <v>114157</v>
       </c>
       <c r="B30" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D30" s="11">
-        <v>46010</v>
+        <v>45904</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>51</v>
@@ -2209,10 +2053,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>1775.95</v>
+        <v>3335.25</v>
       </c>
       <c r="I30" s="4">
-        <v>1775.95</v>
+        <v>3335.25</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2221,24 +2065,24 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>60502.91</v>
+        <v>36259.129999999997</v>
       </c>
       <c r="M30" s="4">
-        <v>60502.91</v>
+        <v>36259.129999999997</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>114157</v>
+        <v>116883</v>
       </c>
       <c r="B31" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D31" s="11">
-        <v>45904</v>
+        <v>46126</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>51</v>
@@ -2250,51 +2094,51 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>1637.49</v>
+        <v>1834.37</v>
       </c>
       <c r="I31" s="4">
-        <v>1637.49</v>
+        <v>1834.37</v>
       </c>
       <c r="J31" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K31" s="4">
-        <v>0</v>
+        <v>2174.0100000000002</v>
       </c>
       <c r="L31" s="4">
-        <v>37956.89</v>
+        <v>86865.15</v>
       </c>
       <c r="M31" s="4">
-        <v>37956.89</v>
+        <v>89039.16</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>118069</v>
+        <v>112083</v>
       </c>
       <c r="B32" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D32" s="11">
-        <v>46105</v>
+        <v>45736</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F32" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="4">
-        <v>0</v>
+        <v>1795.63</v>
       </c>
       <c r="H32" s="4">
         <v>0</v>
       </c>
       <c r="I32" s="4">
-        <v>0</v>
+        <v>1795.63</v>
       </c>
       <c r="J32" s="3">
         <v>0</v>
@@ -2303,24 +2147,24 @@
         <v>0</v>
       </c>
       <c r="L32" s="4">
-        <v>19562.52</v>
+        <v>19751.93</v>
       </c>
       <c r="M32" s="4">
-        <v>19562.52</v>
+        <v>19751.93</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>116883</v>
+        <v>116060</v>
       </c>
       <c r="B33" s="2">
         <v>2856</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D33" s="11">
-        <v>46126</v>
+        <v>46010</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>51</v>
@@ -2332,36 +2176,36 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>0</v>
+        <v>1775.95</v>
       </c>
       <c r="I33" s="4">
-        <v>0</v>
+        <v>1775.95</v>
       </c>
       <c r="J33" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33" s="4">
-        <v>2174.0100000000002</v>
+        <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>88699.520000000004</v>
+        <v>60502.91</v>
       </c>
       <c r="M33" s="4">
-        <v>90873.53</v>
+        <v>60502.91</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>116876</v>
+        <v>112522</v>
       </c>
       <c r="B34" s="2">
         <v>2856</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D34" s="11">
-        <v>46111</v>
+        <v>45776</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>51</v>
@@ -2373,10 +2217,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>0</v>
+        <v>1750.74</v>
       </c>
       <c r="I34" s="4">
-        <v>0</v>
+        <v>1750.74</v>
       </c>
       <c r="J34" s="3">
         <v>0</v>
@@ -2385,24 +2229,24 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>18185.59</v>
+        <v>4934.1099999999997</v>
       </c>
       <c r="M34" s="4">
-        <v>18185.59</v>
+        <v>4934.1099999999997</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>115404</v>
+        <v>118069</v>
       </c>
       <c r="B35" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>22</v>
+        <v>54</v>
       </c>
       <c r="D35" s="11">
-        <v>45986</v>
+        <v>46105</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>51</v>
@@ -2426,24 +2270,24 @@
         <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>12170.29</v>
+        <v>19562.52</v>
       </c>
       <c r="M35" s="4">
-        <v>12170.29</v>
+        <v>19562.52</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>114431</v>
+        <v>116876</v>
       </c>
       <c r="B36" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D36" s="11">
-        <v>45930</v>
+        <v>46111</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>51</v>
@@ -2467,24 +2311,24 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>21758.76</v>
+        <v>18185.59</v>
       </c>
       <c r="M36" s="4">
-        <v>21758.76</v>
+        <v>18185.59</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>112522</v>
+        <v>115404</v>
       </c>
       <c r="B37" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="D37" s="11">
-        <v>45776</v>
+        <v>45986</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>51</v>
@@ -2508,24 +2352,24 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>6684.84</v>
+        <v>12170.29</v>
       </c>
       <c r="M37" s="4">
-        <v>6684.84</v>
+        <v>12170.29</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>111056</v>
+        <v>114431</v>
       </c>
       <c r="B38" s="2">
         <v>2043</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="D38" s="11">
-        <v>45639</v>
+        <v>45930</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>51</v>
@@ -2543,30 +2387,30 @@
         <v>0</v>
       </c>
       <c r="J38" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K38" s="4">
-        <v>61752.21</v>
+        <v>0</v>
       </c>
       <c r="L38" s="4">
-        <v>56209.91</v>
+        <v>21758.76</v>
       </c>
       <c r="M38" s="4">
-        <v>117962.12</v>
+        <v>21758.76</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>109007</v>
+        <v>111056</v>
       </c>
       <c r="B39" s="2">
         <v>2043</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="D39" s="11">
-        <v>45525</v>
+        <v>45639</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>51</v>
@@ -2584,30 +2428,30 @@
         <v>0</v>
       </c>
       <c r="J39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K39" s="4">
-        <v>0</v>
+        <v>61752.21</v>
       </c>
       <c r="L39" s="4">
-        <v>6177.09</v>
+        <v>56209.91</v>
       </c>
       <c r="M39" s="4">
-        <v>6177.09</v>
+        <v>117962.12</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>106018</v>
+        <v>109007</v>
       </c>
       <c r="B40" s="2">
         <v>2043</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="D40" s="11">
-        <v>45344</v>
+        <v>45525</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>51</v>
@@ -2631,10 +2475,10 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>30708.15</v>
+        <v>6177.09</v>
       </c>
       <c r="M40" s="4">
-        <v>30708.15</v>
+        <v>6177.09</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
@@ -2945,84 +2789,67 @@
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="A47:B50">
-    <cfRule type="expression" dxfId="23" priority="13" stopIfTrue="1">
-      <formula>$S47=1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="22" priority="14" stopIfTrue="1">
-      <formula>$S46=1</formula>
+  <conditionalFormatting sqref="A4:B4">
+    <cfRule type="expression" dxfId="12" priority="3" stopIfTrue="1">
+      <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C47:H50 K47:L50">
-    <cfRule type="expression" dxfId="19" priority="18" stopIfTrue="1">
-      <formula>$S47=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C47:M50">
-    <cfRule type="expression" dxfId="18" priority="29" stopIfTrue="1">
-      <formula>$S46=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I47:I50 M47:M50">
-    <cfRule type="expression" dxfId="15" priority="20" stopIfTrue="1">
-      <formula>$S47=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J47:J50">
-    <cfRule type="expression" dxfId="12" priority="16" stopIfTrue="1">
-      <formula>$S47=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A46 J5:J46">
-    <cfRule type="expression" dxfId="11" priority="4" stopIfTrue="1">
+  <conditionalFormatting sqref="A5:B50">
+    <cfRule type="expression" dxfId="11" priority="1" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="2" stopIfTrue="1">
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:L46 C5:H46">
-    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
-      <formula>$S5=1</formula>
+  <conditionalFormatting sqref="C4:H4 K4:L4">
+    <cfRule type="expression" dxfId="9" priority="11" stopIfTrue="1">
+      <formula>$S$34=1</formula>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C5:H46 K5:L46">
     <cfRule type="expression" dxfId="8" priority="7" stopIfTrue="1">
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 M5:M46">
-    <cfRule type="expression" dxfId="7" priority="8" stopIfTrue="1">
+  <conditionalFormatting sqref="C5:H50 K5:L50">
+    <cfRule type="expression" dxfId="7" priority="6" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="9" stopIfTrue="1">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C47:M50">
+    <cfRule type="expression" dxfId="6" priority="41" stopIfTrue="1">
+      <formula>$S46=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I4 M4">
+    <cfRule type="expression" dxfId="5" priority="12" stopIfTrue="1">
+      <formula>$S$34=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I5:I46 M5:M46">
+    <cfRule type="expression" dxfId="4" priority="9" stopIfTrue="1">
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J4 A4">
-    <cfRule type="expression" dxfId="5" priority="10" stopIfTrue="1">
+  <conditionalFormatting sqref="I5:I50 M5:M50">
+    <cfRule type="expression" dxfId="3" priority="8" stopIfTrue="1">
+      <formula>$S5=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J4">
+    <cfRule type="expression" dxfId="2" priority="10" stopIfTrue="1">
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C4:H4 K4:L4">
-    <cfRule type="expression" dxfId="4" priority="11" stopIfTrue="1">
-      <formula>$S$34=1</formula>
+  <conditionalFormatting sqref="J5:J46">
+    <cfRule type="expression" dxfId="1" priority="5" stopIfTrue="1">
+      <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4 M4">
-    <cfRule type="expression" dxfId="3" priority="12" stopIfTrue="1">
-      <formula>$S$34=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B4">
-    <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
-      <formula>$S$34=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B46">
-    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="J5:J50">
+    <cfRule type="expression" dxfId="0" priority="4" stopIfTrue="1">
       <formula>$S5=1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
-      <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-24 14:11)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{829B533F-1791-F547-A53F-03F448DB58ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C54DF9D-36C5-3043-AD0F-F0FCD8EA30AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="58">
   <si>
     <t>Asesor</t>
   </si>
@@ -204,6 +204,12 @@
   </si>
   <si>
     <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+  </si>
+  <si>
+    <t>GERARDO DANIEL BARAJAS TORRES</t>
+  </si>
+  <si>
+    <t>5</t>
   </si>
 </sst>
 </file>
@@ -370,7 +376,163 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="25">
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <border>
         <left style="thin">
@@ -885,7 +1047,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46132</v>
+        <v>46134</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -987,10 +1149,10 @@
         <v>126272.25</v>
       </c>
       <c r="H4" s="4">
-        <v>41937.230000000003</v>
+        <v>47077.95</v>
       </c>
       <c r="I4" s="4">
-        <v>168209.48</v>
+        <v>173350.2</v>
       </c>
       <c r="J4" s="5">
         <v>0</v>
@@ -999,10 +1161,10 @@
         <v>0</v>
       </c>
       <c r="L4" s="4">
-        <v>339458.54</v>
+        <v>334317.82</v>
       </c>
       <c r="M4" s="4">
-        <v>339458.54</v>
+        <v>334317.82</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1048,16 +1210,16 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>110453</v>
+        <v>105696</v>
       </c>
       <c r="B6" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D6" s="11">
-        <v>45600</v>
+        <v>45279</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>51</v>
@@ -1066,13 +1228,13 @@
         <v>1</v>
       </c>
       <c r="G6" s="4">
-        <v>2244.4699999999998</v>
+        <v>36118.519999999997</v>
       </c>
       <c r="H6" s="4">
-        <v>39653.03</v>
+        <v>7658.86</v>
       </c>
       <c r="I6" s="4">
-        <v>41897.5</v>
+        <v>43777.38</v>
       </c>
       <c r="J6" s="3">
         <v>0</v>
@@ -1081,24 +1243,24 @@
         <v>0</v>
       </c>
       <c r="L6" s="4">
-        <v>140438.91</v>
+        <v>21045.119999999999</v>
       </c>
       <c r="M6" s="4">
-        <v>140438.91</v>
+        <v>21045.119999999999</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>105696</v>
+        <v>110453</v>
       </c>
       <c r="B7" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="D7" s="11">
-        <v>45279</v>
+        <v>45600</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>51</v>
@@ -1107,13 +1269,13 @@
         <v>1</v>
       </c>
       <c r="G7" s="4">
-        <v>36118.519999999997</v>
+        <v>2244.4699999999998</v>
       </c>
       <c r="H7" s="4">
-        <v>2866.56</v>
+        <v>39653.03</v>
       </c>
       <c r="I7" s="4">
-        <v>38985.08</v>
+        <v>41897.5</v>
       </c>
       <c r="J7" s="3">
         <v>0</v>
@@ -1122,10 +1284,10 @@
         <v>0</v>
       </c>
       <c r="L7" s="4">
-        <v>25379.03</v>
+        <v>140438.91</v>
       </c>
       <c r="M7" s="4">
-        <v>25379.03</v>
+        <v>140438.91</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
@@ -1171,16 +1333,16 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>90355</v>
+        <v>47116</v>
       </c>
       <c r="B9" s="2">
         <v>2043</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D9" s="11">
-        <v>43949</v>
+        <v>44616</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>51</v>
@@ -1189,39 +1351,39 @@
         <v>1</v>
       </c>
       <c r="G9" s="4">
-        <v>5257.75</v>
+        <v>15755.23</v>
       </c>
       <c r="H9" s="4">
-        <v>18372.009999999998</v>
+        <v>13806.31</v>
       </c>
       <c r="I9" s="4">
-        <v>23629.759999999998</v>
+        <v>29561.54</v>
       </c>
       <c r="J9" s="3">
         <v>1</v>
       </c>
       <c r="K9" s="4">
-        <v>12557.28</v>
+        <v>1731.94</v>
       </c>
       <c r="L9" s="4">
-        <v>41958.02</v>
+        <v>74830.31</v>
       </c>
       <c r="M9" s="4">
-        <v>54515.3</v>
+        <v>76562.25</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>47116</v>
+        <v>90355</v>
       </c>
       <c r="B10" s="2">
         <v>2043</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D10" s="11">
-        <v>44616</v>
+        <v>43949</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>51</v>
@@ -1230,25 +1392,25 @@
         <v>1</v>
       </c>
       <c r="G10" s="4">
-        <v>15755.23</v>
+        <v>5257.75</v>
       </c>
       <c r="H10" s="4">
-        <v>7784.62</v>
+        <v>18372.009999999998</v>
       </c>
       <c r="I10" s="4">
-        <v>23539.85</v>
+        <v>23629.759999999998</v>
       </c>
       <c r="J10" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4">
-        <v>0</v>
+        <v>60855.23</v>
       </c>
       <c r="L10" s="4">
-        <v>60148.11</v>
+        <v>41958.02</v>
       </c>
       <c r="M10" s="4">
-        <v>60148.11</v>
+        <v>102813.25</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
@@ -1315,10 +1477,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="4">
-        <v>20787.77</v>
+        <v>23045.68</v>
       </c>
       <c r="I12" s="4">
-        <v>20787.77</v>
+        <v>23045.68</v>
       </c>
       <c r="J12" s="3">
         <v>0</v>
@@ -1327,10 +1489,10 @@
         <v>0</v>
       </c>
       <c r="L12" s="4">
-        <v>96633.21</v>
+        <v>94375.29</v>
       </c>
       <c r="M12" s="4">
-        <v>96633.21</v>
+        <v>94375.29</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
@@ -1417,16 +1579,16 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>108404</v>
+        <v>110105</v>
       </c>
       <c r="B15" s="2">
         <v>2043</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D15" s="11">
-        <v>45467</v>
+        <v>45560</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>51</v>
@@ -1438,10 +1600,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>7900.28</v>
+        <v>8925.7000000000007</v>
       </c>
       <c r="I15" s="4">
-        <v>7900.28</v>
+        <v>8925.7000000000007</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1450,24 +1612,24 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>33081.01</v>
+        <v>4151.0600000000004</v>
       </c>
       <c r="M15" s="4">
-        <v>33081.01</v>
+        <v>4151.0600000000004</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>108405</v>
+        <v>104718</v>
       </c>
       <c r="B16" s="2">
         <v>2043</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="D16" s="11">
-        <v>45471</v>
+        <v>45264</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>51</v>
@@ -1479,10 +1641,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>7542.1</v>
+        <v>8151.45</v>
       </c>
       <c r="I16" s="4">
-        <v>7542.1</v>
+        <v>8151.45</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1491,24 +1653,24 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>4985.49</v>
+        <v>98488.71</v>
       </c>
       <c r="M16" s="4">
-        <v>4985.49</v>
+        <v>98488.71</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>110105</v>
+        <v>108404</v>
       </c>
       <c r="B17" s="2">
         <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="D17" s="11">
-        <v>45560</v>
+        <v>45467</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>51</v>
@@ -1520,10 +1682,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>7373.6</v>
+        <v>7900.28</v>
       </c>
       <c r="I17" s="4">
-        <v>7373.6</v>
+        <v>7900.28</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1532,39 +1694,39 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>5703.16</v>
+        <v>33081.01</v>
       </c>
       <c r="M17" s="4">
-        <v>5703.16</v>
+        <v>33081.01</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>113450</v>
+        <v>104343</v>
       </c>
       <c r="B18" s="2">
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D18" s="11">
-        <v>45852</v>
+        <v>45201</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F18" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" s="4">
-        <v>0</v>
+        <v>1732.64</v>
       </c>
       <c r="H18" s="4">
-        <v>6690.87</v>
+        <v>5916.56</v>
       </c>
       <c r="I18" s="4">
-        <v>6690.87</v>
+        <v>7649.2</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1573,24 +1735,24 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>4006.82</v>
+        <v>57105.67</v>
       </c>
       <c r="M18" s="4">
-        <v>4006.82</v>
+        <v>57105.67</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>109998</v>
+        <v>108405</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="D19" s="11">
-        <v>45596</v>
+        <v>45471</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>51</v>
@@ -1602,10 +1764,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>5824.66</v>
+        <v>7542.1</v>
       </c>
       <c r="I19" s="4">
-        <v>5824.66</v>
+        <v>7542.1</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1614,24 +1776,24 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>0</v>
+        <v>4985.49</v>
       </c>
       <c r="M19" s="4">
-        <v>0</v>
+        <v>4985.49</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>104718</v>
+        <v>116060</v>
       </c>
       <c r="B20" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="D20" s="11">
-        <v>45264</v>
+        <v>46010</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>51</v>
@@ -1643,10 +1805,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>5284.89</v>
+        <v>6795.62</v>
       </c>
       <c r="I20" s="4">
-        <v>5284.89</v>
+        <v>6795.62</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1655,24 +1817,24 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>101355.28</v>
+        <v>55485.25</v>
       </c>
       <c r="M20" s="4">
-        <v>101355.28</v>
+        <v>55485.25</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>90177</v>
+        <v>113450</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="D21" s="11">
-        <v>43949</v>
+        <v>45852</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>51</v>
@@ -1684,10 +1846,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>5199.32</v>
+        <v>6690.87</v>
       </c>
       <c r="I21" s="4">
-        <v>5199.32</v>
+        <v>6690.87</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1696,24 +1858,24 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>0</v>
+        <v>4006.82</v>
       </c>
       <c r="M21" s="4">
-        <v>0</v>
+        <v>4006.82</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>104343</v>
+        <v>100677</v>
       </c>
       <c r="B22" s="2">
         <v>2043</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D22" s="11">
-        <v>45201</v>
+        <v>44999</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>51</v>
@@ -1725,36 +1887,36 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>5175.96</v>
+        <v>6417.32</v>
       </c>
       <c r="I22" s="4">
-        <v>5175.96</v>
+        <v>6417.32</v>
       </c>
       <c r="J22" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K22" s="4">
-        <v>2473.56</v>
+        <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>57105.67</v>
+        <v>33070.61</v>
       </c>
       <c r="M22" s="4">
-        <v>59579.23</v>
+        <v>33070.61</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>115047</v>
+        <v>106018</v>
       </c>
       <c r="B23" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D23" s="11">
-        <v>45944</v>
+        <v>45344</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>51</v>
@@ -1766,10 +1928,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>5025.2</v>
+        <v>6164.56</v>
       </c>
       <c r="I23" s="4">
-        <v>5025.2</v>
+        <v>6164.56</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1778,24 +1940,24 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>35787.599999999999</v>
+        <v>25348.91</v>
       </c>
       <c r="M23" s="4">
-        <v>35787.599999999999</v>
+        <v>25348.91</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>101640</v>
+        <v>109998</v>
       </c>
       <c r="B24" s="2">
         <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="D24" s="11">
-        <v>45104</v>
+        <v>45596</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>51</v>
@@ -1807,10 +1969,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>4718.59</v>
+        <v>5824.66</v>
       </c>
       <c r="I24" s="4">
-        <v>4718.59</v>
+        <v>5824.66</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1819,24 +1981,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>3204.95</v>
+        <v>0</v>
       </c>
       <c r="M24" s="4">
-        <v>3204.95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>100677</v>
+        <v>90177</v>
       </c>
       <c r="B25" s="2">
         <v>2043</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="D25" s="11">
-        <v>44999</v>
+        <v>43949</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>51</v>
@@ -1848,10 +2010,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>4681.6099999999997</v>
+        <v>5199.32</v>
       </c>
       <c r="I25" s="4">
-        <v>4681.6099999999997</v>
+        <v>5199.32</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -1860,24 +2022,24 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>34806.33</v>
+        <v>0</v>
       </c>
       <c r="M25" s="4">
-        <v>34806.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>113076</v>
+        <v>80925</v>
       </c>
       <c r="B26" s="2">
         <v>2043</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="D26" s="11">
-        <v>45806</v>
+        <v>43439</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>51</v>
@@ -1889,10 +2051,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>4558.5200000000004</v>
+        <v>5149.7700000000004</v>
       </c>
       <c r="I26" s="4">
-        <v>4558.5200000000004</v>
+        <v>5149.7700000000004</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -1901,24 +2063,24 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>9117.0400000000009</v>
+        <v>5647.54</v>
       </c>
       <c r="M26" s="4">
-        <v>9117.0400000000009</v>
+        <v>5647.54</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>88234</v>
+        <v>115047</v>
       </c>
       <c r="B27" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="D27" s="11">
-        <v>43794</v>
+        <v>45944</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>51</v>
@@ -1930,10 +2092,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>4242.34</v>
+        <v>5025.2</v>
       </c>
       <c r="I27" s="4">
-        <v>4242.34</v>
+        <v>5025.2</v>
       </c>
       <c r="J27" s="3">
         <v>0</v>
@@ -1942,24 +2104,24 @@
         <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>15745.12</v>
+        <v>35787.599999999999</v>
       </c>
       <c r="M27" s="4">
-        <v>15745.12</v>
+        <v>35787.599999999999</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>95148</v>
+        <v>109007</v>
       </c>
       <c r="B28" s="2">
         <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D28" s="11">
-        <v>44916</v>
+        <v>45525</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>51</v>
@@ -1971,10 +2133,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>3887.59</v>
+        <v>4835.79</v>
       </c>
       <c r="I28" s="4">
-        <v>3887.59</v>
+        <v>4835.79</v>
       </c>
       <c r="J28" s="3">
         <v>0</v>
@@ -1983,24 +2145,24 @@
         <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>0</v>
+        <v>1341.3</v>
       </c>
       <c r="M28" s="4">
-        <v>0</v>
+        <v>1341.3</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>106018</v>
+        <v>101640</v>
       </c>
       <c r="B29" s="2">
         <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D29" s="11">
-        <v>45344</v>
+        <v>45104</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>51</v>
@@ -2012,10 +2174,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>3669.62</v>
+        <v>4718.59</v>
       </c>
       <c r="I29" s="4">
-        <v>3669.62</v>
+        <v>4718.59</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2024,24 +2186,24 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>25348.91</v>
+        <v>3204.95</v>
       </c>
       <c r="M29" s="4">
-        <v>25348.91</v>
+        <v>3204.95</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>114157</v>
+        <v>113076</v>
       </c>
       <c r="B30" s="2">
         <v>2043</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="D30" s="11">
-        <v>45904</v>
+        <v>45806</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>51</v>
@@ -2053,10 +2215,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>3335.25</v>
+        <v>4558.5200000000004</v>
       </c>
       <c r="I30" s="4">
-        <v>3335.25</v>
+        <v>4558.5200000000004</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2065,24 +2227,24 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>36259.129999999997</v>
+        <v>9117.0400000000009</v>
       </c>
       <c r="M30" s="4">
-        <v>36259.129999999997</v>
+        <v>9117.0400000000009</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>116883</v>
+        <v>88234</v>
       </c>
       <c r="B31" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="D31" s="11">
-        <v>46126</v>
+        <v>43794</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>51</v>
@@ -2094,51 +2256,51 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>1834.37</v>
+        <v>4242.34</v>
       </c>
       <c r="I31" s="4">
-        <v>1834.37</v>
+        <v>4242.34</v>
       </c>
       <c r="J31" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K31" s="4">
-        <v>2174.0100000000002</v>
+        <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>86865.15</v>
+        <v>15745.12</v>
       </c>
       <c r="M31" s="4">
-        <v>89039.16</v>
+        <v>15745.12</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>112083</v>
+        <v>95148</v>
       </c>
       <c r="B32" s="2">
         <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="D32" s="11">
-        <v>45736</v>
+        <v>44916</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F32" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" s="4">
-        <v>1795.63</v>
+        <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>0</v>
+        <v>3887.59</v>
       </c>
       <c r="I32" s="4">
-        <v>1795.63</v>
+        <v>3887.59</v>
       </c>
       <c r="J32" s="3">
         <v>0</v>
@@ -2147,24 +2309,24 @@
         <v>0</v>
       </c>
       <c r="L32" s="4">
-        <v>19751.93</v>
+        <v>0</v>
       </c>
       <c r="M32" s="4">
-        <v>19751.93</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>116060</v>
+        <v>114157</v>
       </c>
       <c r="B33" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D33" s="11">
-        <v>46010</v>
+        <v>45904</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>51</v>
@@ -2176,10 +2338,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>1775.95</v>
+        <v>3335.25</v>
       </c>
       <c r="I33" s="4">
-        <v>1775.95</v>
+        <v>3335.25</v>
       </c>
       <c r="J33" s="3">
         <v>0</v>
@@ -2188,24 +2350,24 @@
         <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>60502.91</v>
+        <v>36259.129999999997</v>
       </c>
       <c r="M33" s="4">
-        <v>60502.91</v>
+        <v>36259.129999999997</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>112522</v>
+        <v>94156</v>
       </c>
       <c r="B34" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D34" s="11">
-        <v>45776</v>
+        <v>44159</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>51</v>
@@ -2217,10 +2379,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>1750.74</v>
+        <v>2302.81</v>
       </c>
       <c r="I34" s="4">
-        <v>1750.74</v>
+        <v>2302.81</v>
       </c>
       <c r="J34" s="3">
         <v>0</v>
@@ -2229,24 +2391,24 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>4934.1099999999997</v>
+        <v>5163.3500000000004</v>
       </c>
       <c r="M34" s="4">
-        <v>4934.1099999999997</v>
+        <v>5163.3500000000004</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>118069</v>
+        <v>116883</v>
       </c>
       <c r="B35" s="2">
         <v>2856</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="D35" s="11">
-        <v>46105</v>
+        <v>46126</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>51</v>
@@ -2258,51 +2420,51 @@
         <v>0</v>
       </c>
       <c r="H35" s="4">
-        <v>0</v>
+        <v>1834.37</v>
       </c>
       <c r="I35" s="4">
-        <v>0</v>
+        <v>1834.37</v>
       </c>
       <c r="J35" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K35" s="4">
-        <v>0</v>
+        <v>2174.0100000000002</v>
       </c>
       <c r="L35" s="4">
-        <v>19562.52</v>
+        <v>86865.15</v>
       </c>
       <c r="M35" s="4">
-        <v>19562.52</v>
+        <v>89039.16</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>116876</v>
+        <v>112083</v>
       </c>
       <c r="B36" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="D36" s="11">
-        <v>46111</v>
+        <v>45736</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F36" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G36" s="4">
-        <v>0</v>
+        <v>1795.63</v>
       </c>
       <c r="H36" s="4">
         <v>0</v>
       </c>
       <c r="I36" s="4">
-        <v>0</v>
+        <v>1795.63</v>
       </c>
       <c r="J36" s="3">
         <v>0</v>
@@ -2311,24 +2473,24 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>18185.59</v>
+        <v>19751.93</v>
       </c>
       <c r="M36" s="4">
-        <v>18185.59</v>
+        <v>19751.93</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>115404</v>
+        <v>112522</v>
       </c>
       <c r="B37" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D37" s="11">
-        <v>45986</v>
+        <v>45776</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>51</v>
@@ -2340,10 +2502,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="4">
-        <v>0</v>
+        <v>1750.74</v>
       </c>
       <c r="I37" s="4">
-        <v>0</v>
+        <v>1750.74</v>
       </c>
       <c r="J37" s="3">
         <v>0</v>
@@ -2352,27 +2514,27 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>12170.29</v>
+        <v>4934.1099999999997</v>
       </c>
       <c r="M37" s="4">
-        <v>12170.29</v>
+        <v>4934.1099999999997</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>114431</v>
+        <v>116795</v>
       </c>
       <c r="B38" s="2">
         <v>2043</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="D38" s="11">
-        <v>45930</v>
+        <v>46000</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F38" s="3">
         <v>0</v>
@@ -2381,10 +2543,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="4">
-        <v>0</v>
+        <v>1594.18</v>
       </c>
       <c r="I38" s="4">
-        <v>0</v>
+        <v>1594.18</v>
       </c>
       <c r="J38" s="3">
         <v>0</v>
@@ -2393,24 +2555,24 @@
         <v>0</v>
       </c>
       <c r="L38" s="4">
-        <v>21758.76</v>
+        <v>0</v>
       </c>
       <c r="M38" s="4">
-        <v>21758.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>111056</v>
+        <v>118069</v>
       </c>
       <c r="B39" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>7</v>
+        <v>54</v>
       </c>
       <c r="D39" s="11">
-        <v>45639</v>
+        <v>46105</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>51</v>
@@ -2428,30 +2590,30 @@
         <v>0</v>
       </c>
       <c r="J39" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K39" s="4">
-        <v>61752.21</v>
+        <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>56209.91</v>
+        <v>19562.52</v>
       </c>
       <c r="M39" s="4">
-        <v>117962.12</v>
+        <v>19562.52</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>109007</v>
+        <v>116876</v>
       </c>
       <c r="B40" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D40" s="11">
-        <v>45525</v>
+        <v>46111</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>51</v>
@@ -2475,24 +2637,24 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>6177.09</v>
+        <v>18185.59</v>
       </c>
       <c r="M40" s="4">
-        <v>6177.09</v>
+        <v>18185.59</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>102825</v>
+        <v>115404</v>
       </c>
       <c r="B41" s="2">
         <v>2043</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="D41" s="11">
-        <v>45117</v>
+        <v>45986</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>51</v>
@@ -2510,30 +2672,30 @@
         <v>0</v>
       </c>
       <c r="J41" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K41" s="4">
-        <v>30557.77</v>
+        <v>0</v>
       </c>
       <c r="L41" s="4">
-        <v>21637.32</v>
+        <v>12170.29</v>
       </c>
       <c r="M41" s="4">
-        <v>52195.09</v>
+        <v>12170.29</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>94156</v>
+        <v>114431</v>
       </c>
       <c r="B42" s="2">
         <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="D42" s="11">
-        <v>44159</v>
+        <v>45930</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>51</v>
@@ -2557,27 +2719,27 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>7466.11</v>
+        <v>21758.76</v>
       </c>
       <c r="M42" s="4">
-        <v>7466.11</v>
+        <v>21758.76</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>81618</v>
+        <v>111056</v>
       </c>
       <c r="B43" s="2">
         <v>2043</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="D43" s="11">
-        <v>43447</v>
+        <v>45639</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F43" s="3">
         <v>0</v>
@@ -2592,30 +2754,30 @@
         <v>0</v>
       </c>
       <c r="J43" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K43" s="4">
-        <v>0</v>
+        <v>61752.21</v>
       </c>
       <c r="L43" s="4">
-        <v>15063.56</v>
+        <v>56209.91</v>
       </c>
       <c r="M43" s="4">
-        <v>15063.56</v>
+        <v>117962.12</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>80925</v>
+        <v>102825</v>
       </c>
       <c r="B44" s="2">
         <v>2043</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="D44" s="11">
-        <v>43439</v>
+        <v>45117</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>51</v>
@@ -2633,33 +2795,33 @@
         <v>0</v>
       </c>
       <c r="J44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K44" s="4">
-        <v>0</v>
+        <v>30557.77</v>
       </c>
       <c r="L44" s="4">
-        <v>10138.450000000001</v>
+        <v>21637.32</v>
       </c>
       <c r="M44" s="4">
-        <v>10138.450000000001</v>
+        <v>52195.09</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
-        <v>65046</v>
+        <v>81618</v>
       </c>
       <c r="B45" s="2">
         <v>2043</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="D45" s="11">
-        <v>44763</v>
+        <v>43447</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F45" s="3">
         <v>0</v>
@@ -2680,67 +2842,93 @@
         <v>0</v>
       </c>
       <c r="L45" s="4">
-        <v>17384.95</v>
+        <v>15063.56</v>
       </c>
       <c r="M45" s="4">
-        <v>17384.95</v>
+        <v>15063.56</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
+        <v>65046</v>
+      </c>
+      <c r="B46" s="2">
+        <v>2043</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D46" s="11">
+        <v>44763</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F46" s="3">
+        <v>0</v>
+      </c>
+      <c r="G46" s="4">
+        <v>0</v>
+      </c>
+      <c r="H46" s="4">
+        <v>0</v>
+      </c>
+      <c r="I46" s="4">
+        <v>0</v>
+      </c>
+      <c r="J46" s="3">
+        <v>0</v>
+      </c>
+      <c r="K46" s="4">
+        <v>0</v>
+      </c>
+      <c r="L46" s="4">
+        <v>17384.95</v>
+      </c>
+      <c r="M46" s="4">
+        <v>17384.95</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A47" s="2">
         <v>63441</v>
       </c>
-      <c r="B46" s="2">
+      <c r="B47" s="2">
         <v>2511</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="C47" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D46" s="11">
+      <c r="D47" s="11">
         <v>44733</v>
       </c>
-      <c r="E46" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F46" s="3">
-        <v>0</v>
-      </c>
-      <c r="G46" s="4">
-        <v>0</v>
-      </c>
-      <c r="H46" s="4">
-        <v>0</v>
-      </c>
-      <c r="I46" s="4">
-        <v>0</v>
-      </c>
-      <c r="J46" s="3">
-        <v>0</v>
-      </c>
-      <c r="K46" s="4">
-        <v>0</v>
-      </c>
-      <c r="L46" s="4">
+      <c r="E47" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F47" s="3">
+        <v>0</v>
+      </c>
+      <c r="G47" s="4">
+        <v>0</v>
+      </c>
+      <c r="H47" s="4">
+        <v>0</v>
+      </c>
+      <c r="I47" s="4">
+        <v>0</v>
+      </c>
+      <c r="J47" s="3">
+        <v>0</v>
+      </c>
+      <c r="K47" s="4">
+        <v>0</v>
+      </c>
+      <c r="L47" s="4">
         <v>9207.01</v>
       </c>
-      <c r="M46" s="4">
+      <c r="M47" s="4">
         <v>9207.01</v>
       </c>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4"/>
-      <c r="I47" s="4"/>
-      <c r="J47" s="3"/>
-      <c r="K47" s="4"/>
-      <c r="L47" s="4"/>
-      <c r="M47" s="4"/>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
@@ -2789,67 +2977,84 @@
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="A4:B4">
-    <cfRule type="expression" dxfId="12" priority="3" stopIfTrue="1">
-      <formula>$S$34=1</formula>
+  <conditionalFormatting sqref="A48:B50">
+    <cfRule type="expression" dxfId="23" priority="13" stopIfTrue="1">
+      <formula>$S48=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="22" priority="14" stopIfTrue="1">
+      <formula>$S47=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:B50">
-    <cfRule type="expression" dxfId="11" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="C48:H50 K48:L50">
+    <cfRule type="expression" dxfId="19" priority="18" stopIfTrue="1">
+      <formula>$S48=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C48:M50">
+    <cfRule type="expression" dxfId="18" priority="53" stopIfTrue="1">
+      <formula>$S47=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I48:I50 M48:M50">
+    <cfRule type="expression" dxfId="15" priority="20" stopIfTrue="1">
+      <formula>$S48=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J48:J50">
+    <cfRule type="expression" dxfId="12" priority="16" stopIfTrue="1">
+      <formula>$S48=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:A47 J5:J47">
+    <cfRule type="expression" dxfId="11" priority="4" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="5" stopIfTrue="1">
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C4:H4 K4:L4">
-    <cfRule type="expression" dxfId="9" priority="11" stopIfTrue="1">
-      <formula>$S$34=1</formula>
+  <conditionalFormatting sqref="K5:L47 C5:H47">
+    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
+      <formula>$S5=1</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C5:H46 K5:L46">
     <cfRule type="expression" dxfId="8" priority="7" stopIfTrue="1">
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C5:H50 K5:L50">
-    <cfRule type="expression" dxfId="7" priority="6" stopIfTrue="1">
+  <conditionalFormatting sqref="I5:I47 M5:M47">
+    <cfRule type="expression" dxfId="7" priority="8" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
+    <cfRule type="expression" dxfId="6" priority="9" stopIfTrue="1">
+      <formula>$S4=1</formula>
+    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C47:M50">
-    <cfRule type="expression" dxfId="6" priority="41" stopIfTrue="1">
-      <formula>$S46=1</formula>
+  <conditionalFormatting sqref="J4 A4">
+    <cfRule type="expression" dxfId="5" priority="10" stopIfTrue="1">
+      <formula>$S$34=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:H4 K4:L4">
+    <cfRule type="expression" dxfId="4" priority="11" stopIfTrue="1">
+      <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I4 M4">
-    <cfRule type="expression" dxfId="5" priority="12" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="12" stopIfTrue="1">
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I46 M5:M46">
-    <cfRule type="expression" dxfId="4" priority="9" stopIfTrue="1">
-      <formula>$S4=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I50 M5:M50">
-    <cfRule type="expression" dxfId="3" priority="8" stopIfTrue="1">
-      <formula>$S5=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J4">
-    <cfRule type="expression" dxfId="2" priority="10" stopIfTrue="1">
+  <conditionalFormatting sqref="B4">
+    <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J5:J46">
-    <cfRule type="expression" dxfId="1" priority="5" stopIfTrue="1">
+  <conditionalFormatting sqref="B5:B47">
+    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+      <formula>$S5=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
       <formula>$S4=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J5:J50">
-    <cfRule type="expression" dxfId="0" priority="4" stopIfTrue="1">
-      <formula>$S5=1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-24 14:26)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C54DF9D-36C5-3043-AD0F-F0FCD8EA30AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13F65E2A-039B-BA42-9961-B3534D0CB267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -376,163 +376,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="25">
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="13">
     <dxf>
       <border>
         <left style="thin">
@@ -2977,84 +2821,67 @@
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="A48:B50">
-    <cfRule type="expression" dxfId="23" priority="13" stopIfTrue="1">
-      <formula>$S48=1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="22" priority="14" stopIfTrue="1">
-      <formula>$S47=1</formula>
+  <conditionalFormatting sqref="A4:B4">
+    <cfRule type="expression" dxfId="12" priority="3" stopIfTrue="1">
+      <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C48:H50 K48:L50">
-    <cfRule type="expression" dxfId="19" priority="18" stopIfTrue="1">
-      <formula>$S48=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C48:M50">
-    <cfRule type="expression" dxfId="18" priority="53" stopIfTrue="1">
-      <formula>$S47=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I48:I50 M48:M50">
-    <cfRule type="expression" dxfId="15" priority="20" stopIfTrue="1">
-      <formula>$S48=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J48:J50">
-    <cfRule type="expression" dxfId="12" priority="16" stopIfTrue="1">
-      <formula>$S48=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A47 J5:J47">
-    <cfRule type="expression" dxfId="11" priority="4" stopIfTrue="1">
+  <conditionalFormatting sqref="A5:B50">
+    <cfRule type="expression" dxfId="11" priority="1" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="2" stopIfTrue="1">
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:L47 C5:H47">
-    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
-      <formula>$S5=1</formula>
+  <conditionalFormatting sqref="C4:H4 K4:L4">
+    <cfRule type="expression" dxfId="9" priority="11" stopIfTrue="1">
+      <formula>$S$34=1</formula>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C5:H47 K5:L47">
     <cfRule type="expression" dxfId="8" priority="7" stopIfTrue="1">
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I47 M5:M47">
-    <cfRule type="expression" dxfId="7" priority="8" stopIfTrue="1">
+  <conditionalFormatting sqref="C5:H50 K5:L50">
+    <cfRule type="expression" dxfId="7" priority="6" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="9" stopIfTrue="1">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C48:M50">
+    <cfRule type="expression" dxfId="6" priority="53" stopIfTrue="1">
+      <formula>$S47=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I4 M4">
+    <cfRule type="expression" dxfId="5" priority="12" stopIfTrue="1">
+      <formula>$S$34=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I5:I47 M5:M47">
+    <cfRule type="expression" dxfId="4" priority="9" stopIfTrue="1">
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J4 A4">
-    <cfRule type="expression" dxfId="5" priority="10" stopIfTrue="1">
+  <conditionalFormatting sqref="I5:I50 M5:M50">
+    <cfRule type="expression" dxfId="3" priority="8" stopIfTrue="1">
+      <formula>$S5=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J4">
+    <cfRule type="expression" dxfId="2" priority="10" stopIfTrue="1">
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C4:H4 K4:L4">
-    <cfRule type="expression" dxfId="4" priority="11" stopIfTrue="1">
-      <formula>$S$34=1</formula>
+  <conditionalFormatting sqref="J5:J47">
+    <cfRule type="expression" dxfId="1" priority="5" stopIfTrue="1">
+      <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4 M4">
-    <cfRule type="expression" dxfId="3" priority="12" stopIfTrue="1">
-      <formula>$S$34=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B4">
-    <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
-      <formula>$S$34=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B47">
-    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="J5:J50">
+    <cfRule type="expression" dxfId="0" priority="4" stopIfTrue="1">
       <formula>$S5=1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
-      <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-27 17:52)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13F65E2A-039B-BA42-9961-B3534D0CB267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2D14EE6-3CD3-C74E-BDD7-8AAEB58CC3E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -376,7 +376,163 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="25">
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <border>
         <left style="thin">
@@ -891,7 +1047,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46134</v>
+        <v>46136</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -987,16 +1143,16 @@
         <v>51</v>
       </c>
       <c r="F4" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G4" s="4">
-        <v>126272.25</v>
+        <v>127823.03</v>
       </c>
       <c r="H4" s="4">
-        <v>47077.95</v>
+        <v>53266.86</v>
       </c>
       <c r="I4" s="4">
-        <v>173350.2</v>
+        <v>181089.89</v>
       </c>
       <c r="J4" s="5">
         <v>0</v>
@@ -1005,10 +1161,10 @@
         <v>0</v>
       </c>
       <c r="L4" s="4">
-        <v>334317.82</v>
+        <v>329260.12</v>
       </c>
       <c r="M4" s="4">
-        <v>334317.82</v>
+        <v>329260.12</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1028,57 +1184,57 @@
         <v>51</v>
       </c>
       <c r="F5" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5" s="4">
-        <v>29477.7</v>
+        <v>74426.78</v>
       </c>
       <c r="H5" s="4">
         <v>71225.600000000006</v>
       </c>
       <c r="I5" s="4">
-        <v>100703.3</v>
+        <v>145652.38</v>
       </c>
       <c r="J5" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" s="4">
-        <v>23801.34</v>
+        <v>54163.64</v>
       </c>
       <c r="L5" s="4">
-        <v>112121.47</v>
+        <v>157070.54999999999</v>
       </c>
       <c r="M5" s="4">
-        <v>135922.81</v>
+        <v>211234.19</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>105696</v>
+        <v>110453</v>
       </c>
       <c r="B6" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="D6" s="11">
-        <v>45279</v>
+        <v>45600</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F6" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G6" s="4">
-        <v>36118.519999999997</v>
+        <v>23526.36</v>
       </c>
       <c r="H6" s="4">
-        <v>7658.86</v>
+        <v>45171.7</v>
       </c>
       <c r="I6" s="4">
-        <v>43777.38</v>
+        <v>68698.06</v>
       </c>
       <c r="J6" s="3">
         <v>0</v>
@@ -1087,24 +1243,24 @@
         <v>0</v>
       </c>
       <c r="L6" s="4">
-        <v>21045.119999999999</v>
+        <v>138388.95000000001</v>
       </c>
       <c r="M6" s="4">
-        <v>21045.119999999999</v>
+        <v>138388.95000000001</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>110453</v>
+        <v>111056</v>
       </c>
       <c r="B7" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D7" s="11">
-        <v>45600</v>
+        <v>45639</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>51</v>
@@ -1113,13 +1269,13 @@
         <v>1</v>
       </c>
       <c r="G7" s="4">
-        <v>2244.4699999999998</v>
+        <v>3045.6</v>
       </c>
       <c r="H7" s="4">
-        <v>39653.03</v>
+        <v>58706.61</v>
       </c>
       <c r="I7" s="4">
-        <v>41897.5</v>
+        <v>61752.21</v>
       </c>
       <c r="J7" s="3">
         <v>0</v>
@@ -1128,51 +1284,51 @@
         <v>0</v>
       </c>
       <c r="L7" s="4">
-        <v>140438.91</v>
+        <v>56209.91</v>
       </c>
       <c r="M7" s="4">
-        <v>140438.91</v>
+        <v>56209.91</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>104750</v>
+        <v>105696</v>
       </c>
       <c r="B8" s="2">
         <v>2043</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D8" s="11">
-        <v>45236</v>
+        <v>45279</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F8" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G8" s="4">
-        <v>1799.5</v>
+        <v>36118.519999999997</v>
       </c>
       <c r="H8" s="4">
-        <v>31457.13</v>
+        <v>7658.86</v>
       </c>
       <c r="I8" s="4">
-        <v>33256.629999999997</v>
+        <v>43777.38</v>
       </c>
       <c r="J8" s="3">
         <v>1</v>
       </c>
       <c r="K8" s="4">
-        <v>2088.27</v>
+        <v>2051.19</v>
       </c>
       <c r="L8" s="4">
-        <v>56777.83</v>
+        <v>43608.26</v>
       </c>
       <c r="M8" s="4">
-        <v>58866.1</v>
+        <v>45659.45</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -1192,124 +1348,124 @@
         <v>51</v>
       </c>
       <c r="F9" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9" s="4">
-        <v>15755.23</v>
+        <v>17487.169999999998</v>
       </c>
       <c r="H9" s="4">
-        <v>13806.31</v>
+        <v>19976.490000000002</v>
       </c>
       <c r="I9" s="4">
-        <v>29561.54</v>
+        <v>37463.660000000003</v>
       </c>
       <c r="J9" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" s="4">
-        <v>1731.94</v>
+        <v>0</v>
       </c>
       <c r="L9" s="4">
         <v>74830.31</v>
       </c>
       <c r="M9" s="4">
-        <v>76562.25</v>
+        <v>74830.31</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>90355</v>
+        <v>104750</v>
       </c>
       <c r="B10" s="2">
         <v>2043</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="D10" s="11">
-        <v>43949</v>
+        <v>45236</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F10" s="3">
+        <v>2</v>
+      </c>
+      <c r="G10" s="4">
+        <v>1799.5</v>
+      </c>
+      <c r="H10" s="4">
+        <v>31457.13</v>
+      </c>
+      <c r="I10" s="4">
+        <v>33256.629999999997</v>
+      </c>
+      <c r="J10" s="3">
         <v>1</v>
       </c>
-      <c r="G10" s="4">
-        <v>5257.75</v>
-      </c>
-      <c r="H10" s="4">
-        <v>18372.009999999998</v>
-      </c>
-      <c r="I10" s="4">
-        <v>23629.759999999998</v>
-      </c>
-      <c r="J10" s="3">
-        <v>2</v>
-      </c>
       <c r="K10" s="4">
-        <v>60855.23</v>
+        <v>2088.27</v>
       </c>
       <c r="L10" s="4">
-        <v>41958.02</v>
+        <v>56777.83</v>
       </c>
       <c r="M10" s="4">
-        <v>102813.25</v>
+        <v>58866.1</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>114100</v>
+        <v>90355</v>
       </c>
       <c r="B11" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="D11" s="11">
-        <v>45863</v>
+        <v>43949</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F11" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" s="4">
-        <v>0</v>
+        <v>5257.75</v>
       </c>
       <c r="H11" s="4">
-        <v>23280.63</v>
+        <v>18372.009999999998</v>
       </c>
       <c r="I11" s="4">
-        <v>23280.63</v>
+        <v>23629.759999999998</v>
       </c>
       <c r="J11" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K11" s="4">
-        <v>20413.86</v>
+        <v>100899.82</v>
       </c>
       <c r="L11" s="4">
-        <v>36810.86</v>
+        <v>41958.02</v>
       </c>
       <c r="M11" s="4">
-        <v>57224.72</v>
+        <v>142857.84</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>107488</v>
+        <v>114100</v>
       </c>
       <c r="B12" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D12" s="11">
-        <v>45440</v>
+        <v>45863</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>51</v>
@@ -1321,36 +1477,36 @@
         <v>0</v>
       </c>
       <c r="H12" s="4">
-        <v>23045.68</v>
+        <v>23280.63</v>
       </c>
       <c r="I12" s="4">
-        <v>23045.68</v>
+        <v>23280.63</v>
       </c>
       <c r="J12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" s="4">
-        <v>0</v>
+        <v>20413.86</v>
       </c>
       <c r="L12" s="4">
-        <v>94375.29</v>
+        <v>36810.86</v>
       </c>
       <c r="M12" s="4">
-        <v>94375.29</v>
+        <v>57224.72</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>110575</v>
+        <v>107488</v>
       </c>
       <c r="B13" s="2">
         <v>2043</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="D13" s="11">
-        <v>45583</v>
+        <v>45440</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>51</v>
@@ -1362,10 +1518,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="4">
-        <v>14385.86</v>
+        <v>23045.68</v>
       </c>
       <c r="I13" s="4">
-        <v>14385.86</v>
+        <v>23045.68</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1374,24 +1530,24 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>86315.15</v>
+        <v>90033.83</v>
       </c>
       <c r="M13" s="4">
-        <v>86315.15</v>
+        <v>90033.83</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>117440</v>
+        <v>106018</v>
       </c>
       <c r="B14" s="2">
         <v>2043</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="D14" s="11">
-        <v>46059</v>
+        <v>45344</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>51</v>
@@ -1403,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="4">
-        <v>10520.76</v>
+        <v>17545.669999999998</v>
       </c>
       <c r="I14" s="4">
-        <v>10520.76</v>
+        <v>17545.669999999998</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1415,24 +1571,24 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>2464.4699999999998</v>
+        <v>13967.81</v>
       </c>
       <c r="M14" s="4">
-        <v>2464.4699999999998</v>
+        <v>13967.81</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>110105</v>
+        <v>110575</v>
       </c>
       <c r="B15" s="2">
         <v>2043</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D15" s="11">
-        <v>45560</v>
+        <v>45583</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>51</v>
@@ -1444,10 +1600,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>8925.7000000000007</v>
+        <v>14385.86</v>
       </c>
       <c r="I15" s="4">
-        <v>8925.7000000000007</v>
+        <v>14385.86</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1456,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>4151.0600000000004</v>
+        <v>86315.15</v>
       </c>
       <c r="M15" s="4">
-        <v>4151.0600000000004</v>
+        <v>86315.15</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
@@ -1485,10 +1641,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>8151.45</v>
+        <v>10615.91</v>
       </c>
       <c r="I16" s="4">
-        <v>8151.45</v>
+        <v>10615.91</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1497,24 +1653,24 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>98488.71</v>
+        <v>96024.24</v>
       </c>
       <c r="M16" s="4">
-        <v>98488.71</v>
+        <v>96024.24</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>108404</v>
+        <v>117440</v>
       </c>
       <c r="B17" s="2">
         <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="D17" s="11">
-        <v>45467</v>
+        <v>46059</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>51</v>
@@ -1526,51 +1682,51 @@
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>7900.28</v>
+        <v>10520.76</v>
       </c>
       <c r="I17" s="4">
-        <v>7900.28</v>
+        <v>10520.76</v>
       </c>
       <c r="J17" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17" s="4">
-        <v>0</v>
+        <v>5401.65</v>
       </c>
       <c r="L17" s="4">
-        <v>33081.01</v>
+        <v>61882.6</v>
       </c>
       <c r="M17" s="4">
-        <v>33081.01</v>
+        <v>67284.25</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>104343</v>
+        <v>113450</v>
       </c>
       <c r="B18" s="2">
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D18" s="11">
-        <v>45201</v>
+        <v>45852</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F18" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" s="4">
-        <v>1732.64</v>
+        <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>5916.56</v>
+        <v>10253.4</v>
       </c>
       <c r="I18" s="4">
-        <v>7649.2</v>
+        <v>10253.4</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1579,24 +1735,24 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>57105.67</v>
+        <v>4006.82</v>
       </c>
       <c r="M18" s="4">
-        <v>57105.67</v>
+        <v>4006.82</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>108405</v>
+        <v>110105</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D19" s="11">
-        <v>45471</v>
+        <v>45560</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>51</v>
@@ -1608,10 +1764,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>7542.1</v>
+        <v>8925.7000000000007</v>
       </c>
       <c r="I19" s="4">
-        <v>7542.1</v>
+        <v>8925.7000000000007</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1620,24 +1776,24 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>4985.49</v>
+        <v>4151.0600000000004</v>
       </c>
       <c r="M19" s="4">
-        <v>4985.49</v>
+        <v>4151.0600000000004</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>116060</v>
+        <v>108404</v>
       </c>
       <c r="B20" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D20" s="11">
-        <v>46010</v>
+        <v>45467</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>51</v>
@@ -1649,10 +1805,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>6795.62</v>
+        <v>7900.28</v>
       </c>
       <c r="I20" s="4">
-        <v>6795.62</v>
+        <v>7900.28</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1661,39 +1817,39 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>55485.25</v>
+        <v>33081.01</v>
       </c>
       <c r="M20" s="4">
-        <v>55485.25</v>
+        <v>33081.01</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>113450</v>
+        <v>104343</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D21" s="11">
-        <v>45852</v>
+        <v>45201</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F21" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21" s="4">
-        <v>0</v>
+        <v>1732.64</v>
       </c>
       <c r="H21" s="4">
-        <v>6690.87</v>
+        <v>5916.56</v>
       </c>
       <c r="I21" s="4">
-        <v>6690.87</v>
+        <v>7649.2</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1702,24 +1858,24 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>4006.82</v>
+        <v>57105.67</v>
       </c>
       <c r="M21" s="4">
-        <v>4006.82</v>
+        <v>57105.67</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>100677</v>
+        <v>108405</v>
       </c>
       <c r="B22" s="2">
         <v>2043</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="D22" s="11">
-        <v>44999</v>
+        <v>45471</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>51</v>
@@ -1731,10 +1887,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>6417.32</v>
+        <v>7542.1</v>
       </c>
       <c r="I22" s="4">
-        <v>6417.32</v>
+        <v>7542.1</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1743,24 +1899,24 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>33070.61</v>
+        <v>4985.49</v>
       </c>
       <c r="M22" s="4">
-        <v>33070.61</v>
+        <v>4985.49</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>106018</v>
+        <v>116060</v>
       </c>
       <c r="B23" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D23" s="11">
-        <v>45344</v>
+        <v>46010</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>51</v>
@@ -1772,10 +1928,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>6164.56</v>
+        <v>6795.62</v>
       </c>
       <c r="I23" s="4">
-        <v>6164.56</v>
+        <v>6795.62</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1784,24 +1940,24 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>25348.91</v>
+        <v>55485.25</v>
       </c>
       <c r="M23" s="4">
-        <v>25348.91</v>
+        <v>55485.25</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>109998</v>
+        <v>100677</v>
       </c>
       <c r="B24" s="2">
         <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D24" s="11">
-        <v>45596</v>
+        <v>44999</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>51</v>
@@ -1813,10 +1969,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>5824.66</v>
+        <v>6417.32</v>
       </c>
       <c r="I24" s="4">
-        <v>5824.66</v>
+        <v>6417.32</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1825,24 +1981,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>0</v>
+        <v>33070.61</v>
       </c>
       <c r="M24" s="4">
-        <v>0</v>
+        <v>33070.61</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>90177</v>
+        <v>109007</v>
       </c>
       <c r="B25" s="2">
         <v>2043</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D25" s="11">
-        <v>43949</v>
+        <v>45525</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>51</v>
@@ -1854,10 +2010,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>5199.32</v>
+        <v>6197.51</v>
       </c>
       <c r="I25" s="4">
-        <v>5199.32</v>
+        <v>6197.51</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -1874,16 +2030,16 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>80925</v>
+        <v>109998</v>
       </c>
       <c r="B26" s="2">
         <v>2043</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="D26" s="11">
-        <v>43439</v>
+        <v>45596</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>51</v>
@@ -1895,10 +2051,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>5149.7700000000004</v>
+        <v>5824.66</v>
       </c>
       <c r="I26" s="4">
-        <v>5149.7700000000004</v>
+        <v>5824.66</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -1907,24 +2063,24 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>5647.54</v>
+        <v>0</v>
       </c>
       <c r="M26" s="4">
-        <v>5647.54</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>115047</v>
+        <v>90177</v>
       </c>
       <c r="B27" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="D27" s="11">
-        <v>45944</v>
+        <v>43949</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>51</v>
@@ -1936,10 +2092,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>5025.2</v>
+        <v>5199.32</v>
       </c>
       <c r="I27" s="4">
-        <v>5025.2</v>
+        <v>5199.32</v>
       </c>
       <c r="J27" s="3">
         <v>0</v>
@@ -1948,24 +2104,24 @@
         <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>35787.599999999999</v>
+        <v>0</v>
       </c>
       <c r="M27" s="4">
-        <v>35787.599999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>109007</v>
+        <v>80925</v>
       </c>
       <c r="B28" s="2">
         <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D28" s="11">
-        <v>45525</v>
+        <v>43439</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>51</v>
@@ -1977,10 +2133,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>4835.79</v>
+        <v>5149.7700000000004</v>
       </c>
       <c r="I28" s="4">
-        <v>4835.79</v>
+        <v>5149.7700000000004</v>
       </c>
       <c r="J28" s="3">
         <v>0</v>
@@ -1989,24 +2145,24 @@
         <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>1341.3</v>
+        <v>0</v>
       </c>
       <c r="M28" s="4">
-        <v>1341.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>101640</v>
+        <v>115047</v>
       </c>
       <c r="B29" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D29" s="11">
-        <v>45104</v>
+        <v>45944</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>51</v>
@@ -2018,10 +2174,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>4718.59</v>
+        <v>5025.2</v>
       </c>
       <c r="I29" s="4">
-        <v>4718.59</v>
+        <v>5025.2</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2030,24 +2186,24 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>3204.95</v>
+        <v>35787.599999999999</v>
       </c>
       <c r="M29" s="4">
-        <v>3204.95</v>
+        <v>35787.599999999999</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>113076</v>
+        <v>101640</v>
       </c>
       <c r="B30" s="2">
         <v>2043</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="D30" s="11">
-        <v>45806</v>
+        <v>45104</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>51</v>
@@ -2059,10 +2215,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>4558.5200000000004</v>
+        <v>4718.59</v>
       </c>
       <c r="I30" s="4">
-        <v>4558.5200000000004</v>
+        <v>4718.59</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2071,24 +2227,24 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>9117.0400000000009</v>
+        <v>3204.95</v>
       </c>
       <c r="M30" s="4">
-        <v>9117.0400000000009</v>
+        <v>3204.95</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>88234</v>
+        <v>113076</v>
       </c>
       <c r="B31" s="2">
         <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="D31" s="11">
-        <v>43794</v>
+        <v>45806</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>51</v>
@@ -2100,10 +2256,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>4242.34</v>
+        <v>4558.5200000000004</v>
       </c>
       <c r="I31" s="4">
-        <v>4242.34</v>
+        <v>4558.5200000000004</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -2112,24 +2268,24 @@
         <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>15745.12</v>
+        <v>9117.0400000000009</v>
       </c>
       <c r="M31" s="4">
-        <v>15745.12</v>
+        <v>9117.0400000000009</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>95148</v>
+        <v>88234</v>
       </c>
       <c r="B32" s="2">
         <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="D32" s="11">
-        <v>44916</v>
+        <v>43794</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>51</v>
@@ -2141,36 +2297,36 @@
         <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>3887.59</v>
+        <v>4242.34</v>
       </c>
       <c r="I32" s="4">
-        <v>3887.59</v>
+        <v>4242.34</v>
       </c>
       <c r="J32" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K32" s="4">
-        <v>0</v>
+        <v>3454.14</v>
       </c>
       <c r="L32" s="4">
-        <v>0</v>
+        <v>15745.12</v>
       </c>
       <c r="M32" s="4">
-        <v>0</v>
+        <v>19199.259999999998</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>114157</v>
+        <v>95148</v>
       </c>
       <c r="B33" s="2">
         <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="D33" s="11">
-        <v>45904</v>
+        <v>44916</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>51</v>
@@ -2182,10 +2338,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>3335.25</v>
+        <v>3887.59</v>
       </c>
       <c r="I33" s="4">
-        <v>3335.25</v>
+        <v>3887.59</v>
       </c>
       <c r="J33" s="3">
         <v>0</v>
@@ -2194,24 +2350,24 @@
         <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>36259.129999999997</v>
+        <v>0</v>
       </c>
       <c r="M33" s="4">
-        <v>36259.129999999997</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>94156</v>
+        <v>114157</v>
       </c>
       <c r="B34" s="2">
         <v>2043</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="D34" s="11">
-        <v>44159</v>
+        <v>45904</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>51</v>
@@ -2223,10 +2379,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>2302.81</v>
+        <v>3335.25</v>
       </c>
       <c r="I34" s="4">
-        <v>2302.81</v>
+        <v>3335.25</v>
       </c>
       <c r="J34" s="3">
         <v>0</v>
@@ -2235,24 +2391,24 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>5163.3500000000004</v>
+        <v>36259.129999999997</v>
       </c>
       <c r="M34" s="4">
-        <v>5163.3500000000004</v>
+        <v>36259.129999999997</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>116883</v>
+        <v>94156</v>
       </c>
       <c r="B35" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="D35" s="11">
-        <v>46126</v>
+        <v>44159</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>51</v>
@@ -2264,92 +2420,92 @@
         <v>0</v>
       </c>
       <c r="H35" s="4">
-        <v>1834.37</v>
+        <v>2302.81</v>
       </c>
       <c r="I35" s="4">
-        <v>1834.37</v>
+        <v>2302.81</v>
       </c>
       <c r="J35" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K35" s="4">
-        <v>2174.0100000000002</v>
+        <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>86865.15</v>
+        <v>5163.3500000000004</v>
       </c>
       <c r="M35" s="4">
-        <v>89039.16</v>
+        <v>5163.3500000000004</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>112083</v>
+        <v>116883</v>
       </c>
       <c r="B36" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="D36" s="11">
-        <v>45736</v>
+        <v>46126</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F36" s="3">
+        <v>0</v>
+      </c>
+      <c r="G36" s="4">
+        <v>0</v>
+      </c>
+      <c r="H36" s="4">
+        <v>1834.37</v>
+      </c>
+      <c r="I36" s="4">
+        <v>1834.37</v>
+      </c>
+      <c r="J36" s="3">
         <v>1</v>
       </c>
-      <c r="G36" s="4">
-        <v>1795.63</v>
-      </c>
-      <c r="H36" s="4">
-        <v>0</v>
-      </c>
-      <c r="I36" s="4">
-        <v>1795.63</v>
-      </c>
-      <c r="J36" s="3">
-        <v>0</v>
-      </c>
       <c r="K36" s="4">
-        <v>0</v>
+        <v>2174.0100000000002</v>
       </c>
       <c r="L36" s="4">
-        <v>19751.93</v>
+        <v>86865.15</v>
       </c>
       <c r="M36" s="4">
-        <v>19751.93</v>
+        <v>89039.16</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>112522</v>
+        <v>112083</v>
       </c>
       <c r="B37" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="D37" s="11">
-        <v>45776</v>
+        <v>45736</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F37" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G37" s="4">
-        <v>0</v>
+        <v>1795.63</v>
       </c>
       <c r="H37" s="4">
-        <v>1750.74</v>
+        <v>0</v>
       </c>
       <c r="I37" s="4">
-        <v>1750.74</v>
+        <v>1795.63</v>
       </c>
       <c r="J37" s="3">
         <v>0</v>
@@ -2358,27 +2514,27 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>4934.1099999999997</v>
+        <v>19751.93</v>
       </c>
       <c r="M37" s="4">
-        <v>4934.1099999999997</v>
+        <v>19751.93</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>116795</v>
+        <v>112522</v>
       </c>
       <c r="B38" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="D38" s="11">
-        <v>46000</v>
+        <v>45776</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="F38" s="3">
         <v>0</v>
@@ -2387,10 +2543,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="4">
-        <v>1594.18</v>
+        <v>1750.74</v>
       </c>
       <c r="I38" s="4">
-        <v>1594.18</v>
+        <v>1750.74</v>
       </c>
       <c r="J38" s="3">
         <v>0</v>
@@ -2399,27 +2555,27 @@
         <v>0</v>
       </c>
       <c r="L38" s="4">
-        <v>0</v>
+        <v>4934.1099999999997</v>
       </c>
       <c r="M38" s="4">
-        <v>0</v>
+        <v>4934.1099999999997</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>118069</v>
+        <v>116795</v>
       </c>
       <c r="B39" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D39" s="11">
-        <v>46105</v>
+        <v>46000</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F39" s="3">
         <v>0</v>
@@ -2428,10 +2584,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="4">
-        <v>0</v>
+        <v>1594.18</v>
       </c>
       <c r="I39" s="4">
-        <v>0</v>
+        <v>1594.18</v>
       </c>
       <c r="J39" s="3">
         <v>0</v>
@@ -2440,24 +2596,24 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>19562.52</v>
+        <v>0</v>
       </c>
       <c r="M39" s="4">
-        <v>19562.52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>116876</v>
+        <v>118069</v>
       </c>
       <c r="B40" s="2">
         <v>2856</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="D40" s="11">
-        <v>46111</v>
+        <v>46105</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>51</v>
@@ -2481,24 +2637,24 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>18185.59</v>
+        <v>19562.52</v>
       </c>
       <c r="M40" s="4">
-        <v>18185.59</v>
+        <v>19562.52</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>115404</v>
+        <v>116876</v>
       </c>
       <c r="B41" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D41" s="11">
-        <v>45986</v>
+        <v>46111</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>51</v>
@@ -2522,24 +2678,24 @@
         <v>0</v>
       </c>
       <c r="L41" s="4">
-        <v>12170.29</v>
+        <v>18185.59</v>
       </c>
       <c r="M41" s="4">
-        <v>12170.29</v>
+        <v>18185.59</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>114431</v>
+        <v>115404</v>
       </c>
       <c r="B42" s="2">
         <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D42" s="11">
-        <v>45930</v>
+        <v>45986</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>51</v>
@@ -2563,24 +2719,24 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>21758.76</v>
+        <v>12170.29</v>
       </c>
       <c r="M42" s="4">
-        <v>21758.76</v>
+        <v>12170.29</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>111056</v>
+        <v>114431</v>
       </c>
       <c r="B43" s="2">
         <v>2043</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="D43" s="11">
-        <v>45639</v>
+        <v>45930</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>51</v>
@@ -2598,16 +2754,16 @@
         <v>0</v>
       </c>
       <c r="J43" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K43" s="4">
-        <v>61752.21</v>
+        <v>0</v>
       </c>
       <c r="L43" s="4">
-        <v>56209.91</v>
+        <v>21758.76</v>
       </c>
       <c r="M43" s="4">
-        <v>117962.12</v>
+        <v>21758.76</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
@@ -2821,67 +2977,84 @@
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="A4:B4">
-    <cfRule type="expression" dxfId="12" priority="3" stopIfTrue="1">
-      <formula>$S$34=1</formula>
+  <conditionalFormatting sqref="A48:B50">
+    <cfRule type="expression" dxfId="23" priority="13" stopIfTrue="1">
+      <formula>$S48=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="22" priority="14" stopIfTrue="1">
+      <formula>$S47=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:B50">
-    <cfRule type="expression" dxfId="11" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="C48:H50 K48:L50">
+    <cfRule type="expression" dxfId="19" priority="18" stopIfTrue="1">
+      <formula>$S48=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C48:M50">
+    <cfRule type="expression" dxfId="18" priority="65" stopIfTrue="1">
+      <formula>$S47=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I48:I50 M48:M50">
+    <cfRule type="expression" dxfId="15" priority="20" stopIfTrue="1">
+      <formula>$S48=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J48:J50">
+    <cfRule type="expression" dxfId="12" priority="16" stopIfTrue="1">
+      <formula>$S48=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:A47 J5:J47">
+    <cfRule type="expression" dxfId="11" priority="4" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="5" stopIfTrue="1">
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C4:H4 K4:L4">
-    <cfRule type="expression" dxfId="9" priority="11" stopIfTrue="1">
-      <formula>$S$34=1</formula>
+  <conditionalFormatting sqref="K5:L47 C5:H47">
+    <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
+      <formula>$S5=1</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C5:H47 K5:L47">
     <cfRule type="expression" dxfId="8" priority="7" stopIfTrue="1">
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C5:H50 K5:L50">
-    <cfRule type="expression" dxfId="7" priority="6" stopIfTrue="1">
+  <conditionalFormatting sqref="I5:I47 M5:M47">
+    <cfRule type="expression" dxfId="7" priority="8" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
+    <cfRule type="expression" dxfId="6" priority="9" stopIfTrue="1">
+      <formula>$S4=1</formula>
+    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C48:M50">
-    <cfRule type="expression" dxfId="6" priority="53" stopIfTrue="1">
-      <formula>$S47=1</formula>
+  <conditionalFormatting sqref="J4 A4">
+    <cfRule type="expression" dxfId="5" priority="10" stopIfTrue="1">
+      <formula>$S$34=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:H4 K4:L4">
+    <cfRule type="expression" dxfId="4" priority="11" stopIfTrue="1">
+      <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I4 M4">
-    <cfRule type="expression" dxfId="5" priority="12" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="12" stopIfTrue="1">
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I47 M5:M47">
-    <cfRule type="expression" dxfId="4" priority="9" stopIfTrue="1">
-      <formula>$S4=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I50 M5:M50">
-    <cfRule type="expression" dxfId="3" priority="8" stopIfTrue="1">
-      <formula>$S5=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J4">
-    <cfRule type="expression" dxfId="2" priority="10" stopIfTrue="1">
+  <conditionalFormatting sqref="B4">
+    <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J5:J47">
-    <cfRule type="expression" dxfId="1" priority="5" stopIfTrue="1">
+  <conditionalFormatting sqref="B5:B47">
+    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+      <formula>$S5=1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="2" stopIfTrue="1">
       <formula>$S4=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J5:J50">
-    <cfRule type="expression" dxfId="0" priority="4" stopIfTrue="1">
-      <formula>$S5=1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-29 09:22)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2D14EE6-3CD3-C74E-BDD7-8AAEB58CC3E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{643550F4-5D0B-9248-B272-5CAEA203B9D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -1047,7 +1047,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1149,22 +1149,22 @@
         <v>127823.03</v>
       </c>
       <c r="H4" s="4">
-        <v>53266.86</v>
+        <v>68335.240000000005</v>
       </c>
       <c r="I4" s="4">
-        <v>181089.89</v>
+        <v>196158.27</v>
       </c>
       <c r="J4" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" s="4">
-        <v>0</v>
+        <v>75822.33</v>
       </c>
       <c r="L4" s="4">
-        <v>329260.12</v>
+        <v>314191.74</v>
       </c>
       <c r="M4" s="4">
-        <v>329260.12</v>
+        <v>390014.07</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1184,28 +1184,28 @@
         <v>51</v>
       </c>
       <c r="F5" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5" s="4">
-        <v>74426.78</v>
+        <v>104789.08</v>
       </c>
       <c r="H5" s="4">
         <v>71225.600000000006</v>
       </c>
       <c r="I5" s="4">
-        <v>145652.38</v>
+        <v>176014.68</v>
       </c>
       <c r="J5" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5" s="4">
-        <v>54163.64</v>
+        <v>23801.34</v>
       </c>
       <c r="L5" s="4">
         <v>157070.54999999999</v>
       </c>
       <c r="M5" s="4">
-        <v>211234.19</v>
+        <v>180871.89</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -1313,22 +1313,22 @@
         <v>36118.519999999997</v>
       </c>
       <c r="H8" s="4">
-        <v>7658.86</v>
+        <v>11209.44</v>
       </c>
       <c r="I8" s="4">
-        <v>43777.38</v>
+        <v>47327.96</v>
       </c>
       <c r="J8" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" s="4">
-        <v>2051.19</v>
+        <v>9720.59</v>
       </c>
       <c r="L8" s="4">
-        <v>43608.26</v>
+        <v>63065.88</v>
       </c>
       <c r="M8" s="4">
-        <v>45659.45</v>
+        <v>72786.47</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -1374,16 +1374,16 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>104750</v>
+        <v>90355</v>
       </c>
       <c r="B10" s="2">
         <v>2043</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D10" s="11">
-        <v>45236</v>
+        <v>43949</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>51</v>
@@ -1392,80 +1392,80 @@
         <v>2</v>
       </c>
       <c r="G10" s="4">
-        <v>1799.5</v>
+        <v>17815.03</v>
       </c>
       <c r="H10" s="4">
-        <v>31457.13</v>
+        <v>18372.009999999998</v>
       </c>
       <c r="I10" s="4">
-        <v>33256.629999999997</v>
+        <v>36187.040000000001</v>
       </c>
       <c r="J10" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4">
-        <v>2088.27</v>
+        <v>88342.54</v>
       </c>
       <c r="L10" s="4">
-        <v>56777.83</v>
+        <v>41958.02</v>
       </c>
       <c r="M10" s="4">
-        <v>58866.1</v>
+        <v>130300.56</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>90355</v>
+        <v>104750</v>
       </c>
       <c r="B11" s="2">
         <v>2043</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="D11" s="11">
-        <v>43949</v>
+        <v>45236</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F11" s="3">
+        <v>2</v>
+      </c>
+      <c r="G11" s="4">
+        <v>1799.5</v>
+      </c>
+      <c r="H11" s="4">
+        <v>31457.13</v>
+      </c>
+      <c r="I11" s="4">
+        <v>33256.629999999997</v>
+      </c>
+      <c r="J11" s="3">
         <v>1</v>
       </c>
-      <c r="G11" s="4">
-        <v>5257.75</v>
-      </c>
-      <c r="H11" s="4">
-        <v>18372.009999999998</v>
-      </c>
-      <c r="I11" s="4">
-        <v>23629.759999999998</v>
-      </c>
-      <c r="J11" s="3">
-        <v>3</v>
-      </c>
       <c r="K11" s="4">
-        <v>100899.82</v>
+        <v>2088.27</v>
       </c>
       <c r="L11" s="4">
-        <v>41958.02</v>
+        <v>56777.83</v>
       </c>
       <c r="M11" s="4">
-        <v>142857.84</v>
+        <v>58866.1</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>114100</v>
+        <v>110575</v>
       </c>
       <c r="B12" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="D12" s="11">
-        <v>45863</v>
+        <v>45583</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>51</v>
@@ -1477,22 +1477,22 @@
         <v>0</v>
       </c>
       <c r="H12" s="4">
-        <v>23280.63</v>
+        <v>28771.72</v>
       </c>
       <c r="I12" s="4">
-        <v>23280.63</v>
+        <v>28771.72</v>
       </c>
       <c r="J12" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" s="4">
-        <v>20413.86</v>
+        <v>0</v>
       </c>
       <c r="L12" s="4">
-        <v>36810.86</v>
+        <v>71929.289999999994</v>
       </c>
       <c r="M12" s="4">
-        <v>57224.72</v>
+        <v>71929.289999999994</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
@@ -1518,10 +1518,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="4">
-        <v>23045.68</v>
+        <v>27387.119999999999</v>
       </c>
       <c r="I13" s="4">
-        <v>23045.68</v>
+        <v>27387.119999999999</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1538,16 +1538,16 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>106018</v>
+        <v>114100</v>
       </c>
       <c r="B14" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D14" s="11">
-        <v>45344</v>
+        <v>45863</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>51</v>
@@ -1559,36 +1559,36 @@
         <v>0</v>
       </c>
       <c r="H14" s="4">
-        <v>17545.669999999998</v>
+        <v>23280.63</v>
       </c>
       <c r="I14" s="4">
-        <v>17545.669999999998</v>
+        <v>23280.63</v>
       </c>
       <c r="J14" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" s="4">
-        <v>0</v>
+        <v>20413.86</v>
       </c>
       <c r="L14" s="4">
-        <v>13967.81</v>
+        <v>36810.86</v>
       </c>
       <c r="M14" s="4">
-        <v>13967.81</v>
+        <v>57224.72</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>110575</v>
+        <v>116060</v>
       </c>
       <c r="B15" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D15" s="11">
-        <v>45583</v>
+        <v>46010</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>51</v>
@@ -1600,10 +1600,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>14385.86</v>
+        <v>20308.48</v>
       </c>
       <c r="I15" s="4">
-        <v>14385.86</v>
+        <v>20308.48</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1612,24 +1612,24 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>86315.15</v>
+        <v>41972.38</v>
       </c>
       <c r="M15" s="4">
-        <v>86315.15</v>
+        <v>41972.38</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>104718</v>
+        <v>106018</v>
       </c>
       <c r="B16" s="2">
         <v>2043</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D16" s="11">
-        <v>45264</v>
+        <v>45344</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>51</v>
@@ -1641,10 +1641,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>10615.91</v>
+        <v>17545.669999999998</v>
       </c>
       <c r="I16" s="4">
-        <v>10615.91</v>
+        <v>17545.669999999998</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1653,24 +1653,24 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>96024.24</v>
+        <v>13967.81</v>
       </c>
       <c r="M16" s="4">
-        <v>96024.24</v>
+        <v>13967.81</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>117440</v>
+        <v>100677</v>
       </c>
       <c r="B17" s="2">
         <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="D17" s="11">
-        <v>46059</v>
+        <v>44999</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>51</v>
@@ -1682,36 +1682,36 @@
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>10520.76</v>
+        <v>12060.56</v>
       </c>
       <c r="I17" s="4">
-        <v>10520.76</v>
+        <v>12060.56</v>
       </c>
       <c r="J17" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K17" s="4">
-        <v>5401.65</v>
+        <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>61882.6</v>
+        <v>33070.61</v>
       </c>
       <c r="M17" s="4">
-        <v>67284.25</v>
+        <v>33070.61</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>113450</v>
+        <v>104718</v>
       </c>
       <c r="B18" s="2">
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D18" s="11">
-        <v>45852</v>
+        <v>45264</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>51</v>
@@ -1723,10 +1723,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>10253.4</v>
+        <v>10615.91</v>
       </c>
       <c r="I18" s="4">
-        <v>10253.4</v>
+        <v>10615.91</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1735,24 +1735,24 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>4006.82</v>
+        <v>96024.24</v>
       </c>
       <c r="M18" s="4">
-        <v>4006.82</v>
+        <v>96024.24</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>110105</v>
+        <v>117440</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="D19" s="11">
-        <v>45560</v>
+        <v>46059</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>51</v>
@@ -1764,36 +1764,36 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>8925.7000000000007</v>
+        <v>10520.76</v>
       </c>
       <c r="I19" s="4">
-        <v>8925.7000000000007</v>
+        <v>10520.76</v>
       </c>
       <c r="J19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19" s="4">
-        <v>0</v>
+        <v>5401.65</v>
       </c>
       <c r="L19" s="4">
-        <v>4151.0600000000004</v>
+        <v>61882.6</v>
       </c>
       <c r="M19" s="4">
-        <v>4151.0600000000004</v>
+        <v>67284.25</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>108404</v>
+        <v>113450</v>
       </c>
       <c r="B20" s="2">
         <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D20" s="11">
-        <v>45467</v>
+        <v>45852</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>51</v>
@@ -1805,10 +1805,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>7900.28</v>
+        <v>10253.4</v>
       </c>
       <c r="I20" s="4">
-        <v>7900.28</v>
+        <v>10253.4</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1817,39 +1817,39 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>33081.01</v>
+        <v>4006.82</v>
       </c>
       <c r="M20" s="4">
-        <v>33081.01</v>
+        <v>4006.82</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>104343</v>
+        <v>110105</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="D21" s="11">
-        <v>45201</v>
+        <v>45560</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F21" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" s="4">
-        <v>1732.64</v>
+        <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>5916.56</v>
+        <v>8925.7000000000007</v>
       </c>
       <c r="I21" s="4">
-        <v>7649.2</v>
+        <v>8925.7000000000007</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1858,24 +1858,24 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>57105.67</v>
+        <v>4151.0600000000004</v>
       </c>
       <c r="M21" s="4">
-        <v>57105.67</v>
+        <v>4151.0600000000004</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>108405</v>
+        <v>108404</v>
       </c>
       <c r="B22" s="2">
         <v>2043</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="D22" s="11">
-        <v>45471</v>
+        <v>45467</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>51</v>
@@ -1887,10 +1887,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>7542.1</v>
+        <v>7900.28</v>
       </c>
       <c r="I22" s="4">
-        <v>7542.1</v>
+        <v>7900.28</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1899,39 +1899,39 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>4985.49</v>
+        <v>33081.01</v>
       </c>
       <c r="M22" s="4">
-        <v>4985.49</v>
+        <v>33081.01</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>116060</v>
+        <v>104343</v>
       </c>
       <c r="B23" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D23" s="11">
-        <v>46010</v>
+        <v>45201</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F23" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" s="4">
-        <v>0</v>
+        <v>1732.64</v>
       </c>
       <c r="H23" s="4">
-        <v>6795.62</v>
+        <v>5916.56</v>
       </c>
       <c r="I23" s="4">
-        <v>6795.62</v>
+        <v>7649.2</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1940,24 +1940,24 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>55485.25</v>
+        <v>54134.55</v>
       </c>
       <c r="M23" s="4">
-        <v>55485.25</v>
+        <v>54134.55</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>100677</v>
+        <v>108405</v>
       </c>
       <c r="B24" s="2">
         <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="D24" s="11">
-        <v>44999</v>
+        <v>45471</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>51</v>
@@ -1969,10 +1969,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>6417.32</v>
+        <v>7542.1</v>
       </c>
       <c r="I24" s="4">
-        <v>6417.32</v>
+        <v>7542.1</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1981,10 +1981,10 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>33070.61</v>
+        <v>4985.49</v>
       </c>
       <c r="M24" s="4">
-        <v>33070.61</v>
+        <v>4985.49</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
@@ -2991,7 +2991,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48:M50">
-    <cfRule type="expression" dxfId="18" priority="65" stopIfTrue="1">
+    <cfRule type="expression" dxfId="18" priority="77" stopIfTrue="1">
       <formula>$S47=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-30 12:40)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{643550F4-5D0B-9248-B272-5CAEA203B9D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94D3DEA6-2740-9244-9919-1852E4BC4084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -1047,7 +1047,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1149,10 +1149,10 @@
         <v>127823.03</v>
       </c>
       <c r="H4" s="4">
-        <v>68335.240000000005</v>
+        <v>86433.33</v>
       </c>
       <c r="I4" s="4">
-        <v>196158.27</v>
+        <v>214256.36</v>
       </c>
       <c r="J4" s="5">
         <v>1</v>
@@ -1161,10 +1161,10 @@
         <v>75822.33</v>
       </c>
       <c r="L4" s="4">
-        <v>314191.74</v>
+        <v>299717.86</v>
       </c>
       <c r="M4" s="4">
-        <v>390014.07</v>
+        <v>375540.19</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1196,30 +1196,30 @@
         <v>176014.68</v>
       </c>
       <c r="J5" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" s="4">
-        <v>23801.34</v>
+        <v>88667.6</v>
       </c>
       <c r="L5" s="4">
         <v>157070.54999999999</v>
       </c>
       <c r="M5" s="4">
-        <v>180871.89</v>
+        <v>245738.15</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>110453</v>
+        <v>90355</v>
       </c>
       <c r="B6" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>4</v>
+        <v>35</v>
       </c>
       <c r="D6" s="11">
-        <v>45600</v>
+        <v>43949</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>51</v>
@@ -1228,54 +1228,54 @@
         <v>3</v>
       </c>
       <c r="G6" s="4">
-        <v>23526.36</v>
+        <v>66112.98</v>
       </c>
       <c r="H6" s="4">
-        <v>45171.7</v>
+        <v>18372.009999999998</v>
       </c>
       <c r="I6" s="4">
-        <v>68698.06</v>
+        <v>84484.99</v>
       </c>
       <c r="J6" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" s="4">
-        <v>0</v>
+        <v>40044.589999999997</v>
       </c>
       <c r="L6" s="4">
-        <v>138388.95000000001</v>
+        <v>41958.02</v>
       </c>
       <c r="M6" s="4">
-        <v>138388.95000000001</v>
+        <v>82002.61</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>111056</v>
+        <v>110453</v>
       </c>
       <c r="B7" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D7" s="11">
-        <v>45639</v>
+        <v>45600</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F7" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G7" s="4">
-        <v>3045.6</v>
+        <v>23526.36</v>
       </c>
       <c r="H7" s="4">
-        <v>58706.61</v>
+        <v>45171.7</v>
       </c>
       <c r="I7" s="4">
-        <v>61752.21</v>
+        <v>68698.06</v>
       </c>
       <c r="J7" s="3">
         <v>0</v>
@@ -1284,24 +1284,24 @@
         <v>0</v>
       </c>
       <c r="L7" s="4">
-        <v>56209.91</v>
+        <v>138388.95000000001</v>
       </c>
       <c r="M7" s="4">
-        <v>56209.91</v>
+        <v>138388.95000000001</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>105696</v>
+        <v>111056</v>
       </c>
       <c r="B8" s="2">
         <v>2043</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D8" s="11">
-        <v>45279</v>
+        <v>45639</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>51</v>
@@ -1310,39 +1310,39 @@
         <v>1</v>
       </c>
       <c r="G8" s="4">
-        <v>36118.519999999997</v>
+        <v>3045.6</v>
       </c>
       <c r="H8" s="4">
-        <v>11209.44</v>
+        <v>58706.61</v>
       </c>
       <c r="I8" s="4">
-        <v>47327.96</v>
+        <v>61752.21</v>
       </c>
       <c r="J8" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K8" s="4">
-        <v>9720.59</v>
+        <v>0</v>
       </c>
       <c r="L8" s="4">
-        <v>63065.88</v>
+        <v>56209.91</v>
       </c>
       <c r="M8" s="4">
-        <v>72786.47</v>
+        <v>56209.91</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>47116</v>
+        <v>105696</v>
       </c>
       <c r="B9" s="2">
         <v>2043</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="D9" s="11">
-        <v>44616</v>
+        <v>45279</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>51</v>
@@ -1351,39 +1351,39 @@
         <v>2</v>
       </c>
       <c r="G9" s="4">
-        <v>17487.169999999998</v>
+        <v>38169.71</v>
       </c>
       <c r="H9" s="4">
-        <v>19976.490000000002</v>
+        <v>11209.44</v>
       </c>
       <c r="I9" s="4">
-        <v>37463.660000000003</v>
+        <v>49379.15</v>
       </c>
       <c r="J9" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" s="4">
-        <v>0</v>
+        <v>7669.4</v>
       </c>
       <c r="L9" s="4">
-        <v>74830.31</v>
+        <v>63065.88</v>
       </c>
       <c r="M9" s="4">
-        <v>74830.31</v>
+        <v>70735.28</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>90355</v>
+        <v>47116</v>
       </c>
       <c r="B10" s="2">
         <v>2043</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D10" s="11">
-        <v>43949</v>
+        <v>44616</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>51</v>
@@ -1392,25 +1392,25 @@
         <v>2</v>
       </c>
       <c r="G10" s="4">
-        <v>17815.03</v>
+        <v>17487.169999999998</v>
       </c>
       <c r="H10" s="4">
-        <v>18372.009999999998</v>
+        <v>19976.490000000002</v>
       </c>
       <c r="I10" s="4">
-        <v>36187.040000000001</v>
+        <v>37463.660000000003</v>
       </c>
       <c r="J10" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K10" s="4">
-        <v>88342.54</v>
+        <v>0</v>
       </c>
       <c r="L10" s="4">
-        <v>41958.02</v>
+        <v>74830.31</v>
       </c>
       <c r="M10" s="4">
-        <v>130300.56</v>
+        <v>74830.31</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
@@ -1442,16 +1442,16 @@
         <v>33256.629999999997</v>
       </c>
       <c r="J11" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" s="4">
-        <v>2088.27</v>
+        <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>56777.83</v>
+        <v>31450.71</v>
       </c>
       <c r="M11" s="4">
-        <v>58866.1</v>
+        <v>31450.71</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
@@ -1620,31 +1620,31 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>106018</v>
+        <v>117440</v>
       </c>
       <c r="B16" s="2">
         <v>2043</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="D16" s="11">
-        <v>45344</v>
+        <v>46059</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F16" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="4">
-        <v>0</v>
+        <v>5401.65</v>
       </c>
       <c r="H16" s="4">
-        <v>17545.669999999998</v>
+        <v>12985.22</v>
       </c>
       <c r="I16" s="4">
-        <v>17545.669999999998</v>
+        <v>18386.87</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1653,24 +1653,24 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>13967.81</v>
+        <v>59418.13</v>
       </c>
       <c r="M16" s="4">
-        <v>13967.81</v>
+        <v>59418.13</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>100677</v>
+        <v>106018</v>
       </c>
       <c r="B17" s="2">
         <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D17" s="11">
-        <v>44999</v>
+        <v>45344</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>51</v>
@@ -1682,10 +1682,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>12060.56</v>
+        <v>17545.669999999998</v>
       </c>
       <c r="I17" s="4">
-        <v>12060.56</v>
+        <v>17545.669999999998</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1694,10 +1694,10 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>33070.61</v>
+        <v>13967.81</v>
       </c>
       <c r="M17" s="4">
-        <v>33070.61</v>
+        <v>13967.81</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
@@ -1723,10 +1723,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>10615.91</v>
+        <v>12348.02</v>
       </c>
       <c r="I18" s="4">
-        <v>10615.91</v>
+        <v>12348.02</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1735,24 +1735,24 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>96024.24</v>
+        <v>94292.13</v>
       </c>
       <c r="M18" s="4">
-        <v>96024.24</v>
+        <v>94292.13</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>117440</v>
+        <v>100677</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="D19" s="11">
-        <v>46059</v>
+        <v>44999</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>51</v>
@@ -1764,22 +1764,22 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>10520.76</v>
+        <v>12060.56</v>
       </c>
       <c r="I19" s="4">
-        <v>10520.76</v>
+        <v>12060.56</v>
       </c>
       <c r="J19" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K19" s="4">
-        <v>5401.65</v>
+        <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>61882.6</v>
+        <v>33070.61</v>
       </c>
       <c r="M19" s="4">
-        <v>67284.25</v>
+        <v>33070.61</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
@@ -1866,16 +1866,16 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>108404</v>
+        <v>101640</v>
       </c>
       <c r="B22" s="2">
         <v>2043</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D22" s="11">
-        <v>45467</v>
+        <v>45104</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>51</v>
@@ -1887,10 +1887,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>7900.28</v>
+        <v>8802.09</v>
       </c>
       <c r="I22" s="4">
-        <v>7900.28</v>
+        <v>8802.09</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1899,39 +1899,39 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>33081.01</v>
+        <v>0</v>
       </c>
       <c r="M22" s="4">
-        <v>33081.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>104343</v>
+        <v>108404</v>
       </c>
       <c r="B23" s="2">
         <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D23" s="11">
-        <v>45201</v>
+        <v>45467</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F23" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" s="4">
-        <v>1732.64</v>
+        <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>5916.56</v>
+        <v>7900.28</v>
       </c>
       <c r="I23" s="4">
-        <v>7649.2</v>
+        <v>7900.28</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1940,39 +1940,39 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>54134.55</v>
+        <v>33081.01</v>
       </c>
       <c r="M23" s="4">
-        <v>54134.55</v>
+        <v>33081.01</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>108405</v>
+        <v>104343</v>
       </c>
       <c r="B24" s="2">
         <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="D24" s="11">
-        <v>45471</v>
+        <v>45201</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F24" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" s="4">
-        <v>0</v>
+        <v>1732.64</v>
       </c>
       <c r="H24" s="4">
-        <v>7542.1</v>
+        <v>5916.56</v>
       </c>
       <c r="I24" s="4">
-        <v>7542.1</v>
+        <v>7649.2</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1981,24 +1981,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>4985.49</v>
+        <v>54134.55</v>
       </c>
       <c r="M24" s="4">
-        <v>4985.49</v>
+        <v>54134.55</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>109007</v>
+        <v>116883</v>
       </c>
       <c r="B25" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D25" s="11">
-        <v>45525</v>
+        <v>46126</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>51</v>
@@ -2010,36 +2010,36 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>6197.51</v>
+        <v>7611.32</v>
       </c>
       <c r="I25" s="4">
-        <v>6197.51</v>
+        <v>7611.32</v>
       </c>
       <c r="J25" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K25" s="4">
-        <v>0</v>
+        <v>2174.0100000000002</v>
       </c>
       <c r="L25" s="4">
-        <v>0</v>
+        <v>81241.899999999994</v>
       </c>
       <c r="M25" s="4">
-        <v>0</v>
+        <v>83415.91</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>109998</v>
+        <v>108405</v>
       </c>
       <c r="B26" s="2">
         <v>2043</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="D26" s="11">
-        <v>45596</v>
+        <v>45471</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>51</v>
@@ -2051,10 +2051,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>5824.66</v>
+        <v>7542.1</v>
       </c>
       <c r="I26" s="4">
-        <v>5824.66</v>
+        <v>7542.1</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2063,24 +2063,24 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>0</v>
+        <v>4985.49</v>
       </c>
       <c r="M26" s="4">
-        <v>0</v>
+        <v>4985.49</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>90177</v>
+        <v>109007</v>
       </c>
       <c r="B27" s="2">
         <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D27" s="11">
-        <v>43949</v>
+        <v>45525</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>51</v>
@@ -2092,10 +2092,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>5199.32</v>
+        <v>6197.51</v>
       </c>
       <c r="I27" s="4">
-        <v>5199.32</v>
+        <v>6197.51</v>
       </c>
       <c r="J27" s="3">
         <v>0</v>
@@ -2112,16 +2112,16 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>80925</v>
+        <v>109998</v>
       </c>
       <c r="B28" s="2">
         <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="D28" s="11">
-        <v>43439</v>
+        <v>45596</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>51</v>
@@ -2133,10 +2133,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>5149.7700000000004</v>
+        <v>5824.66</v>
       </c>
       <c r="I28" s="4">
-        <v>5149.7700000000004</v>
+        <v>5824.66</v>
       </c>
       <c r="J28" s="3">
         <v>0</v>
@@ -2153,16 +2153,16 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>115047</v>
+        <v>90177</v>
       </c>
       <c r="B29" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="D29" s="11">
-        <v>45944</v>
+        <v>43949</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>51</v>
@@ -2174,10 +2174,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>5025.2</v>
+        <v>5199.32</v>
       </c>
       <c r="I29" s="4">
-        <v>5025.2</v>
+        <v>5199.32</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2186,24 +2186,24 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>35787.599999999999</v>
+        <v>0</v>
       </c>
       <c r="M29" s="4">
-        <v>35787.599999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>101640</v>
+        <v>80925</v>
       </c>
       <c r="B30" s="2">
         <v>2043</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="D30" s="11">
-        <v>45104</v>
+        <v>43439</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>51</v>
@@ -2215,10 +2215,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>4718.59</v>
+        <v>5149.7700000000004</v>
       </c>
       <c r="I30" s="4">
-        <v>4718.59</v>
+        <v>5149.7700000000004</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2227,24 +2227,24 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>3204.95</v>
+        <v>0</v>
       </c>
       <c r="M30" s="4">
-        <v>3204.95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>113076</v>
+        <v>115047</v>
       </c>
       <c r="B31" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="D31" s="11">
-        <v>45806</v>
+        <v>45944</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>51</v>
@@ -2256,10 +2256,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>4558.5200000000004</v>
+        <v>5025.2</v>
       </c>
       <c r="I31" s="4">
-        <v>4558.5200000000004</v>
+        <v>5025.2</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -2268,24 +2268,24 @@
         <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>9117.0400000000009</v>
+        <v>35787.599999999999</v>
       </c>
       <c r="M31" s="4">
-        <v>9117.0400000000009</v>
+        <v>35787.599999999999</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>88234</v>
+        <v>113076</v>
       </c>
       <c r="B32" s="2">
         <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="D32" s="11">
-        <v>43794</v>
+        <v>45806</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>51</v>
@@ -2297,36 +2297,36 @@
         <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>4242.34</v>
+        <v>4558.5200000000004</v>
       </c>
       <c r="I32" s="4">
-        <v>4242.34</v>
+        <v>4558.5200000000004</v>
       </c>
       <c r="J32" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32" s="4">
-        <v>3454.14</v>
+        <v>0</v>
       </c>
       <c r="L32" s="4">
-        <v>15745.12</v>
+        <v>9117.0400000000009</v>
       </c>
       <c r="M32" s="4">
-        <v>19199.259999999998</v>
+        <v>9117.0400000000009</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>95148</v>
+        <v>88234</v>
       </c>
       <c r="B33" s="2">
         <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="D33" s="11">
-        <v>44916</v>
+        <v>43794</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>51</v>
@@ -2338,36 +2338,36 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>3887.59</v>
+        <v>4242.34</v>
       </c>
       <c r="I33" s="4">
-        <v>3887.59</v>
+        <v>4242.34</v>
       </c>
       <c r="J33" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K33" s="4">
-        <v>0</v>
+        <v>3454.14</v>
       </c>
       <c r="L33" s="4">
-        <v>0</v>
+        <v>15745.12</v>
       </c>
       <c r="M33" s="4">
-        <v>0</v>
+        <v>19199.259999999998</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>114157</v>
+        <v>95148</v>
       </c>
       <c r="B34" s="2">
         <v>2043</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="D34" s="11">
-        <v>45904</v>
+        <v>44916</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>51</v>
@@ -2379,10 +2379,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>3335.25</v>
+        <v>3887.59</v>
       </c>
       <c r="I34" s="4">
-        <v>3335.25</v>
+        <v>3887.59</v>
       </c>
       <c r="J34" s="3">
         <v>0</v>
@@ -2391,24 +2391,24 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>36259.129999999997</v>
+        <v>0</v>
       </c>
       <c r="M34" s="4">
-        <v>36259.129999999997</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>94156</v>
+        <v>114157</v>
       </c>
       <c r="B35" s="2">
         <v>2043</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="D35" s="11">
-        <v>44159</v>
+        <v>45904</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>51</v>
@@ -2420,10 +2420,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="4">
-        <v>2302.81</v>
+        <v>3335.25</v>
       </c>
       <c r="I35" s="4">
-        <v>2302.81</v>
+        <v>3335.25</v>
       </c>
       <c r="J35" s="3">
         <v>0</v>
@@ -2432,24 +2432,24 @@
         <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>5163.3500000000004</v>
+        <v>36259.129999999997</v>
       </c>
       <c r="M35" s="4">
-        <v>5163.3500000000004</v>
+        <v>36259.129999999997</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>116883</v>
+        <v>94156</v>
       </c>
       <c r="B36" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="D36" s="11">
-        <v>46126</v>
+        <v>44159</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>51</v>
@@ -2461,51 +2461,51 @@
         <v>0</v>
       </c>
       <c r="H36" s="4">
-        <v>1834.37</v>
+        <v>2302.81</v>
       </c>
       <c r="I36" s="4">
-        <v>1834.37</v>
+        <v>2302.81</v>
       </c>
       <c r="J36" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K36" s="4">
-        <v>2174.0100000000002</v>
+        <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>86865.15</v>
+        <v>5163.3500000000004</v>
       </c>
       <c r="M36" s="4">
-        <v>89039.16</v>
+        <v>5163.3500000000004</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>112083</v>
+        <v>116876</v>
       </c>
       <c r="B37" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="D37" s="11">
-        <v>45736</v>
+        <v>46111</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G37" s="4">
-        <v>1795.63</v>
+        <v>0</v>
       </c>
       <c r="H37" s="4">
-        <v>0</v>
+        <v>2020.62</v>
       </c>
       <c r="I37" s="4">
-        <v>1795.63</v>
+        <v>2020.62</v>
       </c>
       <c r="J37" s="3">
         <v>0</v>
@@ -2514,39 +2514,39 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>19751.93</v>
+        <v>16164.97</v>
       </c>
       <c r="M37" s="4">
-        <v>19751.93</v>
+        <v>16164.97</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>112522</v>
+        <v>112083</v>
       </c>
       <c r="B38" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="D38" s="11">
-        <v>45776</v>
+        <v>45736</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G38" s="4">
-        <v>0</v>
+        <v>1795.63</v>
       </c>
       <c r="H38" s="4">
-        <v>1750.74</v>
+        <v>0</v>
       </c>
       <c r="I38" s="4">
-        <v>1750.74</v>
+        <v>1795.63</v>
       </c>
       <c r="J38" s="3">
         <v>0</v>
@@ -2555,27 +2555,27 @@
         <v>0</v>
       </c>
       <c r="L38" s="4">
-        <v>4934.1099999999997</v>
+        <v>19751.93</v>
       </c>
       <c r="M38" s="4">
-        <v>4934.1099999999997</v>
+        <v>19751.93</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>116795</v>
+        <v>118069</v>
       </c>
       <c r="B39" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D39" s="11">
-        <v>46000</v>
+        <v>46105</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="F39" s="3">
         <v>0</v>
@@ -2584,10 +2584,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="4">
-        <v>1594.18</v>
+        <v>1778.41</v>
       </c>
       <c r="I39" s="4">
-        <v>1594.18</v>
+        <v>1778.41</v>
       </c>
       <c r="J39" s="3">
         <v>0</v>
@@ -2596,24 +2596,24 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>0</v>
+        <v>17784.11</v>
       </c>
       <c r="M39" s="4">
-        <v>0</v>
+        <v>17784.11</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>118069</v>
+        <v>112522</v>
       </c>
       <c r="B40" s="2">
         <v>2856</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="D40" s="11">
-        <v>46105</v>
+        <v>45776</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>51</v>
@@ -2625,10 +2625,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="4">
-        <v>0</v>
+        <v>1750.74</v>
       </c>
       <c r="I40" s="4">
-        <v>0</v>
+        <v>1750.74</v>
       </c>
       <c r="J40" s="3">
         <v>0</v>
@@ -2637,24 +2637,24 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>19562.52</v>
+        <v>4934.1099999999997</v>
       </c>
       <c r="M40" s="4">
-        <v>19562.52</v>
+        <v>4934.1099999999997</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>116876</v>
+        <v>115404</v>
       </c>
       <c r="B41" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D41" s="11">
-        <v>46111</v>
+        <v>45986</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>51</v>
@@ -2666,10 +2666,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="4">
-        <v>0</v>
+        <v>1738.61</v>
       </c>
       <c r="I41" s="4">
-        <v>0</v>
+        <v>1738.61</v>
       </c>
       <c r="J41" s="3">
         <v>0</v>
@@ -2678,27 +2678,27 @@
         <v>0</v>
       </c>
       <c r="L41" s="4">
-        <v>18185.59</v>
+        <v>10431.68</v>
       </c>
       <c r="M41" s="4">
-        <v>18185.59</v>
+        <v>10431.68</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>115404</v>
+        <v>116795</v>
       </c>
       <c r="B42" s="2">
         <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>22</v>
+        <v>56</v>
       </c>
       <c r="D42" s="11">
-        <v>45986</v>
+        <v>46000</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F42" s="3">
         <v>0</v>
@@ -2707,10 +2707,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="4">
-        <v>0</v>
+        <v>1594.18</v>
       </c>
       <c r="I42" s="4">
-        <v>0</v>
+        <v>1594.18</v>
       </c>
       <c r="J42" s="3">
         <v>0</v>
@@ -2719,10 +2719,10 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>12170.29</v>
+        <v>0</v>
       </c>
       <c r="M42" s="4">
-        <v>12170.29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
@@ -2991,7 +2991,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48:M50">
-    <cfRule type="expression" dxfId="18" priority="77" stopIfTrue="1">
+    <cfRule type="expression" dxfId="18" priority="89" stopIfTrue="1">
       <formula>$S47=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-05-04 14:32)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94D3DEA6-2740-9244-9919-1852E4BC4084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26620C4B-3B17-DA47-9A27-E950498A5E5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -1047,7 +1047,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1128,84 +1128,84 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
-        <v>87538</v>
+        <v>80122</v>
       </c>
       <c r="B4" s="2">
         <v>2043</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="D4" s="11">
-        <v>43731</v>
+        <v>43371</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F4" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G4" s="4">
-        <v>127823.03</v>
+        <v>234521.60000000001</v>
       </c>
       <c r="H4" s="4">
-        <v>86433.33</v>
+        <v>71225.600000000006</v>
       </c>
       <c r="I4" s="4">
-        <v>214256.36</v>
+        <v>305747.20000000001</v>
       </c>
       <c r="J4" s="5">
         <v>1</v>
       </c>
       <c r="K4" s="4">
-        <v>75822.33</v>
+        <v>23801.34</v>
       </c>
       <c r="L4" s="4">
-        <v>299717.86</v>
+        <v>157070.54999999999</v>
       </c>
       <c r="M4" s="4">
-        <v>375540.19</v>
+        <v>180871.89</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
-        <v>80122</v>
+        <v>87538</v>
       </c>
       <c r="B5" s="2">
         <v>2043</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="D5" s="11">
-        <v>43371</v>
+        <v>43731</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F5" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G5" s="4">
-        <v>104789.08</v>
+        <v>127823.03</v>
       </c>
       <c r="H5" s="4">
-        <v>71225.600000000006</v>
+        <v>86433.33</v>
       </c>
       <c r="I5" s="4">
-        <v>176014.68</v>
+        <v>214256.36</v>
       </c>
       <c r="J5" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5" s="4">
-        <v>88667.6</v>
+        <v>75822.33</v>
       </c>
       <c r="L5" s="4">
-        <v>157070.54999999999</v>
+        <v>299717.86</v>
       </c>
       <c r="M5" s="4">
-        <v>245738.15</v>
+        <v>375540.19</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -1225,28 +1225,28 @@
         <v>51</v>
       </c>
       <c r="F6" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G6" s="4">
-        <v>66112.98</v>
+        <v>71150.12</v>
       </c>
       <c r="H6" s="4">
-        <v>18372.009999999998</v>
+        <v>98607.02</v>
       </c>
       <c r="I6" s="4">
-        <v>84484.99</v>
+        <v>169757.14</v>
       </c>
       <c r="J6" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" s="4">
-        <v>40044.589999999997</v>
+        <v>0</v>
       </c>
       <c r="L6" s="4">
         <v>41958.02</v>
       </c>
       <c r="M6" s="4">
-        <v>82002.61</v>
+        <v>41958.02</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -1348,28 +1348,28 @@
         <v>51</v>
       </c>
       <c r="F9" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G9" s="4">
-        <v>38169.71</v>
+        <v>45839.11</v>
       </c>
       <c r="H9" s="4">
         <v>11209.44</v>
       </c>
       <c r="I9" s="4">
-        <v>49379.15</v>
+        <v>57048.55</v>
       </c>
       <c r="J9" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" s="4">
-        <v>7669.4</v>
+        <v>0</v>
       </c>
       <c r="L9" s="4">
         <v>63065.88</v>
       </c>
       <c r="M9" s="4">
-        <v>70735.28</v>
+        <v>63065.88</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
@@ -1415,16 +1415,16 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>104750</v>
+        <v>116883</v>
       </c>
       <c r="B11" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="D11" s="11">
-        <v>45236</v>
+        <v>46126</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>51</v>
@@ -1433,13 +1433,13 @@
         <v>2</v>
       </c>
       <c r="G11" s="4">
-        <v>1799.5</v>
+        <v>27295.61</v>
       </c>
       <c r="H11" s="4">
-        <v>31457.13</v>
+        <v>7611.32</v>
       </c>
       <c r="I11" s="4">
-        <v>33256.629999999997</v>
+        <v>34906.93</v>
       </c>
       <c r="J11" s="3">
         <v>0</v>
@@ -1448,39 +1448,39 @@
         <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>31450.71</v>
+        <v>81241.899999999994</v>
       </c>
       <c r="M11" s="4">
-        <v>31450.71</v>
+        <v>81241.899999999994</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>110575</v>
+        <v>104750</v>
       </c>
       <c r="B12" s="2">
         <v>2043</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D12" s="11">
-        <v>45583</v>
+        <v>45236</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F12" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G12" s="4">
-        <v>0</v>
+        <v>1799.5</v>
       </c>
       <c r="H12" s="4">
-        <v>28771.72</v>
+        <v>31457.13</v>
       </c>
       <c r="I12" s="4">
-        <v>28771.72</v>
+        <v>33256.629999999997</v>
       </c>
       <c r="J12" s="3">
         <v>0</v>
@@ -1489,24 +1489,24 @@
         <v>0</v>
       </c>
       <c r="L12" s="4">
-        <v>71929.289999999994</v>
+        <v>31450.71</v>
       </c>
       <c r="M12" s="4">
-        <v>71929.289999999994</v>
+        <v>31450.71</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>107488</v>
+        <v>114100</v>
       </c>
       <c r="B13" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D13" s="11">
-        <v>45440</v>
+        <v>45863</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>51</v>
@@ -1518,36 +1518,36 @@
         <v>0</v>
       </c>
       <c r="H13" s="4">
-        <v>27387.119999999999</v>
+        <v>32519.97</v>
       </c>
       <c r="I13" s="4">
-        <v>27387.119999999999</v>
+        <v>32519.97</v>
       </c>
       <c r="J13" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" s="4">
-        <v>0</v>
+        <v>20413.86</v>
       </c>
       <c r="L13" s="4">
-        <v>90033.83</v>
+        <v>27571.52</v>
       </c>
       <c r="M13" s="4">
-        <v>90033.83</v>
+        <v>47985.38</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>114100</v>
+        <v>110575</v>
       </c>
       <c r="B14" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="D14" s="11">
-        <v>45863</v>
+        <v>45583</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>51</v>
@@ -1559,36 +1559,36 @@
         <v>0</v>
       </c>
       <c r="H14" s="4">
-        <v>23280.63</v>
+        <v>28771.72</v>
       </c>
       <c r="I14" s="4">
-        <v>23280.63</v>
+        <v>28771.72</v>
       </c>
       <c r="J14" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14" s="4">
-        <v>20413.86</v>
+        <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>36810.86</v>
+        <v>71929.289999999994</v>
       </c>
       <c r="M14" s="4">
-        <v>57224.72</v>
+        <v>71929.289999999994</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>116060</v>
+        <v>107488</v>
       </c>
       <c r="B15" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D15" s="11">
-        <v>46010</v>
+        <v>45440</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>51</v>
@@ -1600,10 +1600,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>20308.48</v>
+        <v>27387.119999999999</v>
       </c>
       <c r="I15" s="4">
-        <v>20308.48</v>
+        <v>27387.119999999999</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1612,39 +1612,39 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>41972.38</v>
+        <v>90033.83</v>
       </c>
       <c r="M15" s="4">
-        <v>41972.38</v>
+        <v>90033.83</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>117440</v>
+        <v>116060</v>
       </c>
       <c r="B16" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="D16" s="11">
-        <v>46059</v>
+        <v>46010</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F16" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" s="4">
-        <v>5401.65</v>
+        <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>12985.22</v>
+        <v>20308.48</v>
       </c>
       <c r="I16" s="4">
-        <v>18386.87</v>
+        <v>20308.48</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1653,39 +1653,39 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>59418.13</v>
+        <v>41972.38</v>
       </c>
       <c r="M16" s="4">
-        <v>59418.13</v>
+        <v>41972.38</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>106018</v>
+        <v>117440</v>
       </c>
       <c r="B17" s="2">
         <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="D17" s="11">
-        <v>45344</v>
+        <v>46059</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F17" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" s="4">
-        <v>0</v>
+        <v>5401.65</v>
       </c>
       <c r="H17" s="4">
-        <v>17545.669999999998</v>
+        <v>12985.22</v>
       </c>
       <c r="I17" s="4">
-        <v>17545.669999999998</v>
+        <v>18386.87</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1694,24 +1694,24 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>13967.81</v>
+        <v>59418.13</v>
       </c>
       <c r="M17" s="4">
-        <v>13967.81</v>
+        <v>59418.13</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>104718</v>
+        <v>106018</v>
       </c>
       <c r="B18" s="2">
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D18" s="11">
-        <v>45264</v>
+        <v>45344</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>51</v>
@@ -1723,10 +1723,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>12348.02</v>
+        <v>17545.669999999998</v>
       </c>
       <c r="I18" s="4">
-        <v>12348.02</v>
+        <v>17545.669999999998</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1735,24 +1735,24 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>94292.13</v>
+        <v>13967.81</v>
       </c>
       <c r="M18" s="4">
-        <v>94292.13</v>
+        <v>13967.81</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>100677</v>
+        <v>104718</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="D19" s="11">
-        <v>44999</v>
+        <v>45264</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>51</v>
@@ -1764,10 +1764,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>12060.56</v>
+        <v>12348.02</v>
       </c>
       <c r="I19" s="4">
-        <v>12060.56</v>
+        <v>12348.02</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1776,24 +1776,24 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>33070.61</v>
+        <v>94292.13</v>
       </c>
       <c r="M19" s="4">
-        <v>33070.61</v>
+        <v>94292.13</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>113450</v>
+        <v>100677</v>
       </c>
       <c r="B20" s="2">
         <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D20" s="11">
-        <v>45852</v>
+        <v>44999</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>51</v>
@@ -1805,10 +1805,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>10253.4</v>
+        <v>12060.56</v>
       </c>
       <c r="I20" s="4">
-        <v>10253.4</v>
+        <v>12060.56</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1817,24 +1817,24 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>4006.82</v>
+        <v>33070.61</v>
       </c>
       <c r="M20" s="4">
-        <v>4006.82</v>
+        <v>33070.61</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>110105</v>
+        <v>113450</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D21" s="11">
-        <v>45560</v>
+        <v>45852</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>51</v>
@@ -1846,10 +1846,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>8925.7000000000007</v>
+        <v>10253.4</v>
       </c>
       <c r="I21" s="4">
-        <v>8925.7000000000007</v>
+        <v>10253.4</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1858,24 +1858,24 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>4151.0600000000004</v>
+        <v>4006.82</v>
       </c>
       <c r="M21" s="4">
-        <v>4151.0600000000004</v>
+        <v>4006.82</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>101640</v>
+        <v>108404</v>
       </c>
       <c r="B22" s="2">
         <v>2043</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D22" s="11">
-        <v>45104</v>
+        <v>45467</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>51</v>
@@ -1887,10 +1887,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>8802.09</v>
+        <v>9835.77</v>
       </c>
       <c r="I22" s="4">
-        <v>8802.09</v>
+        <v>9835.77</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1899,24 +1899,24 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>0</v>
+        <v>20240.93</v>
       </c>
       <c r="M22" s="4">
-        <v>0</v>
+        <v>20240.93</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>108404</v>
+        <v>113076</v>
       </c>
       <c r="B23" s="2">
         <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="D23" s="11">
-        <v>45467</v>
+        <v>45806</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>51</v>
@@ -1928,10 +1928,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>7900.28</v>
+        <v>9117.0400000000009</v>
       </c>
       <c r="I23" s="4">
-        <v>7900.28</v>
+        <v>9117.0400000000009</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1940,39 +1940,39 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>33081.01</v>
+        <v>4558.5200000000004</v>
       </c>
       <c r="M23" s="4">
-        <v>33081.01</v>
+        <v>4558.5200000000004</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>104343</v>
+        <v>110105</v>
       </c>
       <c r="B24" s="2">
         <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="D24" s="11">
-        <v>45201</v>
+        <v>45560</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F24" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" s="4">
-        <v>1732.64</v>
+        <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>5916.56</v>
+        <v>8925.7000000000007</v>
       </c>
       <c r="I24" s="4">
-        <v>7649.2</v>
+        <v>8925.7000000000007</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1981,24 +1981,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>54134.55</v>
+        <v>4151.0600000000004</v>
       </c>
       <c r="M24" s="4">
-        <v>54134.55</v>
+        <v>4151.0600000000004</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>116883</v>
+        <v>101640</v>
       </c>
       <c r="B25" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="D25" s="11">
-        <v>46126</v>
+        <v>45104</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>51</v>
@@ -2010,51 +2010,51 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>7611.32</v>
+        <v>8802.09</v>
       </c>
       <c r="I25" s="4">
-        <v>7611.32</v>
+        <v>8802.09</v>
       </c>
       <c r="J25" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K25" s="4">
-        <v>2174.0100000000002</v>
+        <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>81241.899999999994</v>
+        <v>0</v>
       </c>
       <c r="M25" s="4">
-        <v>83415.91</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>108405</v>
+        <v>104343</v>
       </c>
       <c r="B26" s="2">
         <v>2043</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="D26" s="11">
-        <v>45471</v>
+        <v>45201</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F26" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G26" s="4">
-        <v>0</v>
+        <v>1732.64</v>
       </c>
       <c r="H26" s="4">
-        <v>7542.1</v>
+        <v>6954.33</v>
       </c>
       <c r="I26" s="4">
-        <v>7542.1</v>
+        <v>8686.9699999999993</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2063,24 +2063,24 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>4985.49</v>
+        <v>53096.78</v>
       </c>
       <c r="M26" s="4">
-        <v>4985.49</v>
+        <v>53096.78</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>109007</v>
+        <v>102825</v>
       </c>
       <c r="B27" s="2">
         <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="D27" s="11">
-        <v>45525</v>
+        <v>45117</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>51</v>
@@ -2092,36 +2092,36 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>6197.51</v>
+        <v>8047.52</v>
       </c>
       <c r="I27" s="4">
-        <v>6197.51</v>
+        <v>8047.52</v>
       </c>
       <c r="J27" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" s="4">
-        <v>0</v>
+        <v>30557.77</v>
       </c>
       <c r="L27" s="4">
-        <v>0</v>
+        <v>13589.8</v>
       </c>
       <c r="M27" s="4">
-        <v>0</v>
+        <v>44147.57</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>109998</v>
+        <v>108405</v>
       </c>
       <c r="B28" s="2">
         <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="D28" s="11">
-        <v>45596</v>
+        <v>45471</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>51</v>
@@ -2133,10 +2133,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>5824.66</v>
+        <v>7542.1</v>
       </c>
       <c r="I28" s="4">
-        <v>5824.66</v>
+        <v>7542.1</v>
       </c>
       <c r="J28" s="3">
         <v>0</v>
@@ -2145,24 +2145,24 @@
         <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>0</v>
+        <v>4985.49</v>
       </c>
       <c r="M28" s="4">
-        <v>0</v>
+        <v>4985.49</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>90177</v>
+        <v>94156</v>
       </c>
       <c r="B29" s="2">
         <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D29" s="11">
-        <v>43949</v>
+        <v>44159</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>51</v>
@@ -2174,10 +2174,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>5199.32</v>
+        <v>6945.5</v>
       </c>
       <c r="I29" s="4">
-        <v>5199.32</v>
+        <v>6945.5</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2194,16 +2194,16 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>80925</v>
+        <v>109007</v>
       </c>
       <c r="B30" s="2">
         <v>2043</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D30" s="11">
-        <v>43439</v>
+        <v>45525</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>51</v>
@@ -2215,10 +2215,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>5149.7700000000004</v>
+        <v>6197.51</v>
       </c>
       <c r="I30" s="4">
-        <v>5149.7700000000004</v>
+        <v>6197.51</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2235,16 +2235,16 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>115047</v>
+        <v>109998</v>
       </c>
       <c r="B31" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="D31" s="11">
-        <v>45944</v>
+        <v>45596</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>51</v>
@@ -2256,10 +2256,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>5025.2</v>
+        <v>5824.66</v>
       </c>
       <c r="I31" s="4">
-        <v>5025.2</v>
+        <v>5824.66</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -2268,24 +2268,24 @@
         <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>35787.599999999999</v>
+        <v>0</v>
       </c>
       <c r="M31" s="4">
-        <v>35787.599999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>113076</v>
+        <v>90177</v>
       </c>
       <c r="B32" s="2">
         <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="D32" s="11">
-        <v>45806</v>
+        <v>43949</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>51</v>
@@ -2297,10 +2297,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>4558.5200000000004</v>
+        <v>5199.32</v>
       </c>
       <c r="I32" s="4">
-        <v>4558.5200000000004</v>
+        <v>5199.32</v>
       </c>
       <c r="J32" s="3">
         <v>0</v>
@@ -2309,24 +2309,24 @@
         <v>0</v>
       </c>
       <c r="L32" s="4">
-        <v>9117.0400000000009</v>
+        <v>0</v>
       </c>
       <c r="M32" s="4">
-        <v>9117.0400000000009</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>88234</v>
+        <v>80925</v>
       </c>
       <c r="B33" s="2">
         <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="D33" s="11">
-        <v>43794</v>
+        <v>43439</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>51</v>
@@ -2338,36 +2338,36 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>4242.34</v>
+        <v>5149.7700000000004</v>
       </c>
       <c r="I33" s="4">
-        <v>4242.34</v>
+        <v>5149.7700000000004</v>
       </c>
       <c r="J33" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33" s="4">
-        <v>3454.14</v>
+        <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>15745.12</v>
+        <v>0</v>
       </c>
       <c r="M33" s="4">
-        <v>19199.259999999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>95148</v>
+        <v>115047</v>
       </c>
       <c r="B34" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="D34" s="11">
-        <v>44916</v>
+        <v>45944</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>51</v>
@@ -2379,10 +2379,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>3887.59</v>
+        <v>5025.2</v>
       </c>
       <c r="I34" s="4">
-        <v>3887.59</v>
+        <v>5025.2</v>
       </c>
       <c r="J34" s="3">
         <v>0</v>
@@ -2391,24 +2391,24 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>0</v>
+        <v>35787.599999999999</v>
       </c>
       <c r="M34" s="4">
-        <v>0</v>
+        <v>35787.599999999999</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>114157</v>
+        <v>88234</v>
       </c>
       <c r="B35" s="2">
         <v>2043</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D35" s="11">
-        <v>45904</v>
+        <v>43794</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>51</v>
@@ -2420,36 +2420,36 @@
         <v>0</v>
       </c>
       <c r="H35" s="4">
-        <v>3335.25</v>
+        <v>4242.34</v>
       </c>
       <c r="I35" s="4">
-        <v>3335.25</v>
+        <v>4242.34</v>
       </c>
       <c r="J35" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K35" s="4">
-        <v>0</v>
+        <v>3454.14</v>
       </c>
       <c r="L35" s="4">
-        <v>36259.129999999997</v>
+        <v>15745.12</v>
       </c>
       <c r="M35" s="4">
-        <v>36259.129999999997</v>
+        <v>19199.259999999998</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>94156</v>
+        <v>95148</v>
       </c>
       <c r="B36" s="2">
         <v>2043</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D36" s="11">
-        <v>44159</v>
+        <v>44916</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>51</v>
@@ -2461,10 +2461,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="4">
-        <v>2302.81</v>
+        <v>3887.59</v>
       </c>
       <c r="I36" s="4">
-        <v>2302.81</v>
+        <v>3887.59</v>
       </c>
       <c r="J36" s="3">
         <v>0</v>
@@ -2473,24 +2473,24 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>5163.3500000000004</v>
+        <v>0</v>
       </c>
       <c r="M36" s="4">
-        <v>5163.3500000000004</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>116876</v>
+        <v>114157</v>
       </c>
       <c r="B37" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D37" s="11">
-        <v>46111</v>
+        <v>45904</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>51</v>
@@ -2502,10 +2502,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="4">
-        <v>2020.62</v>
+        <v>3335.25</v>
       </c>
       <c r="I37" s="4">
-        <v>2020.62</v>
+        <v>3335.25</v>
       </c>
       <c r="J37" s="3">
         <v>0</v>
@@ -2514,39 +2514,39 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>16164.97</v>
+        <v>36259.129999999997</v>
       </c>
       <c r="M37" s="4">
-        <v>16164.97</v>
+        <v>36259.129999999997</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>112083</v>
+        <v>116876</v>
       </c>
       <c r="B38" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="D38" s="11">
-        <v>45736</v>
+        <v>46111</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F38" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G38" s="4">
-        <v>1795.63</v>
+        <v>0</v>
       </c>
       <c r="H38" s="4">
-        <v>0</v>
+        <v>2020.62</v>
       </c>
       <c r="I38" s="4">
-        <v>1795.63</v>
+        <v>2020.62</v>
       </c>
       <c r="J38" s="3">
         <v>0</v>
@@ -2555,39 +2555,39 @@
         <v>0</v>
       </c>
       <c r="L38" s="4">
-        <v>19751.93</v>
+        <v>16164.97</v>
       </c>
       <c r="M38" s="4">
-        <v>19751.93</v>
+        <v>16164.97</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>118069</v>
+        <v>112083</v>
       </c>
       <c r="B39" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D39" s="11">
-        <v>46105</v>
+        <v>45736</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G39" s="4">
-        <v>0</v>
+        <v>1795.63</v>
       </c>
       <c r="H39" s="4">
-        <v>1778.41</v>
+        <v>0</v>
       </c>
       <c r="I39" s="4">
-        <v>1778.41</v>
+        <v>1795.63</v>
       </c>
       <c r="J39" s="3">
         <v>0</v>
@@ -2596,24 +2596,24 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>17784.11</v>
+        <v>19751.93</v>
       </c>
       <c r="M39" s="4">
-        <v>17784.11</v>
+        <v>19751.93</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>112522</v>
+        <v>118069</v>
       </c>
       <c r="B40" s="2">
         <v>2856</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="D40" s="11">
-        <v>45776</v>
+        <v>46105</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>51</v>
@@ -2625,10 +2625,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="4">
-        <v>1750.74</v>
+        <v>1778.41</v>
       </c>
       <c r="I40" s="4">
-        <v>1750.74</v>
+        <v>1778.41</v>
       </c>
       <c r="J40" s="3">
         <v>0</v>
@@ -2637,24 +2637,24 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>4934.1099999999997</v>
+        <v>17784.11</v>
       </c>
       <c r="M40" s="4">
-        <v>4934.1099999999997</v>
+        <v>17784.11</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>115404</v>
+        <v>112522</v>
       </c>
       <c r="B41" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D41" s="11">
-        <v>45986</v>
+        <v>45776</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>51</v>
@@ -2666,10 +2666,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="4">
-        <v>1738.61</v>
+        <v>1750.74</v>
       </c>
       <c r="I41" s="4">
-        <v>1738.61</v>
+        <v>1750.74</v>
       </c>
       <c r="J41" s="3">
         <v>0</v>
@@ -2678,27 +2678,27 @@
         <v>0</v>
       </c>
       <c r="L41" s="4">
-        <v>10431.68</v>
+        <v>4934.1099999999997</v>
       </c>
       <c r="M41" s="4">
-        <v>10431.68</v>
+        <v>4934.1099999999997</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>116795</v>
+        <v>115404</v>
       </c>
       <c r="B42" s="2">
         <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="D42" s="11">
-        <v>46000</v>
+        <v>45986</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="F42" s="3">
         <v>0</v>
@@ -2707,10 +2707,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="4">
-        <v>1594.18</v>
+        <v>1738.61</v>
       </c>
       <c r="I42" s="4">
-        <v>1594.18</v>
+        <v>1738.61</v>
       </c>
       <c r="J42" s="3">
         <v>0</v>
@@ -2719,27 +2719,27 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>0</v>
+        <v>10431.68</v>
       </c>
       <c r="M42" s="4">
-        <v>0</v>
+        <v>10431.68</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>114431</v>
+        <v>116795</v>
       </c>
       <c r="B43" s="2">
         <v>2043</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="D43" s="11">
-        <v>45930</v>
+        <v>46000</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F43" s="3">
         <v>0</v>
@@ -2748,10 +2748,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="4">
-        <v>0</v>
+        <v>1594.18</v>
       </c>
       <c r="I43" s="4">
-        <v>0</v>
+        <v>1594.18</v>
       </c>
       <c r="J43" s="3">
         <v>0</v>
@@ -2760,24 +2760,24 @@
         <v>0</v>
       </c>
       <c r="L43" s="4">
-        <v>21758.76</v>
+        <v>0</v>
       </c>
       <c r="M43" s="4">
-        <v>21758.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>102825</v>
+        <v>65046</v>
       </c>
       <c r="B44" s="2">
         <v>2043</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D44" s="11">
-        <v>45117</v>
+        <v>44763</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>51</v>
@@ -2789,39 +2789,39 @@
         <v>0</v>
       </c>
       <c r="H44" s="4">
-        <v>0</v>
+        <v>1037.77</v>
       </c>
       <c r="I44" s="4">
-        <v>0</v>
+        <v>1037.77</v>
       </c>
       <c r="J44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K44" s="4">
-        <v>30557.77</v>
+        <v>0</v>
       </c>
       <c r="L44" s="4">
-        <v>21637.32</v>
+        <v>16347.18</v>
       </c>
       <c r="M44" s="4">
-        <v>52195.09</v>
+        <v>16347.18</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
-        <v>81618</v>
+        <v>114431</v>
       </c>
       <c r="B45" s="2">
         <v>2043</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="D45" s="11">
-        <v>43447</v>
+        <v>45930</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F45" s="3">
         <v>0</v>
@@ -2842,27 +2842,27 @@
         <v>0</v>
       </c>
       <c r="L45" s="4">
-        <v>15063.56</v>
+        <v>21758.76</v>
       </c>
       <c r="M45" s="4">
-        <v>15063.56</v>
+        <v>21758.76</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
-        <v>65046</v>
+        <v>81618</v>
       </c>
       <c r="B46" s="2">
         <v>2043</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="D46" s="11">
-        <v>44763</v>
+        <v>43447</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F46" s="3">
         <v>0</v>
@@ -2883,10 +2883,10 @@
         <v>0</v>
       </c>
       <c r="L46" s="4">
-        <v>17384.95</v>
+        <v>15063.56</v>
       </c>
       <c r="M46" s="4">
-        <v>17384.95</v>
+        <v>15063.56</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.2">
@@ -2991,7 +2991,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48:M50">
-    <cfRule type="expression" dxfId="18" priority="89" stopIfTrue="1">
+    <cfRule type="expression" dxfId="18" priority="101" stopIfTrue="1">
       <formula>$S47=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-05-06 11:24)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26620C4B-3B17-DA47-9A27-E950498A5E5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1BBA08C-9890-9446-90BF-74719EA17217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -1047,7 +1047,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1146,25 +1146,25 @@
         <v>6</v>
       </c>
       <c r="G4" s="4">
-        <v>234521.60000000001</v>
+        <v>235834.33</v>
       </c>
       <c r="H4" s="4">
-        <v>71225.600000000006</v>
+        <v>71624.28</v>
       </c>
       <c r="I4" s="4">
-        <v>305747.20000000001</v>
+        <v>307458.61</v>
       </c>
       <c r="J4" s="5">
         <v>1</v>
       </c>
       <c r="K4" s="4">
-        <v>23801.34</v>
+        <v>23934.57</v>
       </c>
       <c r="L4" s="4">
-        <v>157070.54999999999</v>
+        <v>157949.76000000001</v>
       </c>
       <c r="M4" s="4">
-        <v>180871.89</v>
+        <v>181884.33</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1184,28 +1184,28 @@
         <v>51</v>
       </c>
       <c r="F5" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G5" s="4">
-        <v>127823.03</v>
+        <v>203888.37</v>
       </c>
       <c r="H5" s="4">
-        <v>86433.33</v>
+        <v>85383.07</v>
       </c>
       <c r="I5" s="4">
-        <v>214256.36</v>
+        <v>289271.44</v>
       </c>
       <c r="J5" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" s="4">
-        <v>75822.33</v>
+        <v>0</v>
       </c>
       <c r="L5" s="4">
-        <v>299717.86</v>
+        <v>296938.46999999997</v>
       </c>
       <c r="M5" s="4">
-        <v>375540.19</v>
+        <v>296938.46999999997</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -1228,13 +1228,13 @@
         <v>5</v>
       </c>
       <c r="G6" s="4">
-        <v>71150.12</v>
+        <v>71548.39</v>
       </c>
       <c r="H6" s="4">
-        <v>98607.02</v>
+        <v>102457.96</v>
       </c>
       <c r="I6" s="4">
-        <v>169757.14</v>
+        <v>174006.35</v>
       </c>
       <c r="J6" s="3">
         <v>0</v>
@@ -1243,10 +1243,10 @@
         <v>0</v>
       </c>
       <c r="L6" s="4">
-        <v>41958.02</v>
+        <v>38893.919999999998</v>
       </c>
       <c r="M6" s="4">
-        <v>41958.02</v>
+        <v>38893.919999999998</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -1269,25 +1269,25 @@
         <v>3</v>
       </c>
       <c r="G7" s="4">
-        <v>23526.36</v>
+        <v>23658.05</v>
       </c>
       <c r="H7" s="4">
-        <v>45171.7</v>
+        <v>47393.48</v>
       </c>
       <c r="I7" s="4">
-        <v>68698.06</v>
+        <v>71051.53</v>
       </c>
       <c r="J7" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7" s="4">
-        <v>0</v>
+        <v>34074.879999999997</v>
       </c>
       <c r="L7" s="4">
-        <v>138388.95000000001</v>
+        <v>137194.64000000001</v>
       </c>
       <c r="M7" s="4">
-        <v>138388.95000000001</v>
+        <v>171269.52</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
@@ -1310,13 +1310,13 @@
         <v>1</v>
       </c>
       <c r="G8" s="4">
-        <v>3045.6</v>
+        <v>3062.65</v>
       </c>
       <c r="H8" s="4">
-        <v>58706.61</v>
+        <v>64510.75</v>
       </c>
       <c r="I8" s="4">
-        <v>61752.21</v>
+        <v>67573.399999999994</v>
       </c>
       <c r="J8" s="3">
         <v>0</v>
@@ -1325,10 +1325,10 @@
         <v>0</v>
       </c>
       <c r="L8" s="4">
-        <v>56209.91</v>
+        <v>51049.02</v>
       </c>
       <c r="M8" s="4">
-        <v>56209.91</v>
+        <v>51049.02</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -1348,16 +1348,16 @@
         <v>51</v>
       </c>
       <c r="F9" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G9" s="4">
-        <v>45839.11</v>
+        <v>47762.78</v>
       </c>
       <c r="H9" s="4">
-        <v>11209.44</v>
+        <v>11272.17</v>
       </c>
       <c r="I9" s="4">
-        <v>57048.55</v>
+        <v>59034.95</v>
       </c>
       <c r="J9" s="3">
         <v>0</v>
@@ -1366,10 +1366,10 @@
         <v>0</v>
       </c>
       <c r="L9" s="4">
-        <v>63065.88</v>
+        <v>81756.639999999999</v>
       </c>
       <c r="M9" s="4">
-        <v>63065.88</v>
+        <v>81756.639999999999</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
@@ -1392,13 +1392,13 @@
         <v>2</v>
       </c>
       <c r="G10" s="4">
-        <v>17487.169999999998</v>
+        <v>17585.05</v>
       </c>
       <c r="H10" s="4">
-        <v>19976.490000000002</v>
+        <v>26125.63</v>
       </c>
       <c r="I10" s="4">
-        <v>37463.660000000003</v>
+        <v>43710.68</v>
       </c>
       <c r="J10" s="3">
         <v>0</v>
@@ -1407,10 +1407,10 @@
         <v>0</v>
       </c>
       <c r="L10" s="4">
-        <v>74830.31</v>
+        <v>75084.59</v>
       </c>
       <c r="M10" s="4">
-        <v>74830.31</v>
+        <v>75084.59</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
@@ -1433,13 +1433,13 @@
         <v>2</v>
       </c>
       <c r="G11" s="4">
-        <v>27295.61</v>
+        <v>27448.400000000001</v>
       </c>
       <c r="H11" s="4">
-        <v>7611.32</v>
+        <v>7653.93</v>
       </c>
       <c r="I11" s="4">
-        <v>34906.93</v>
+        <v>35102.33</v>
       </c>
       <c r="J11" s="3">
         <v>0</v>
@@ -1448,10 +1448,10 @@
         <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>81241.899999999994</v>
+        <v>81696.649999999994</v>
       </c>
       <c r="M11" s="4">
-        <v>81241.899999999994</v>
+        <v>81696.649999999994</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
@@ -1474,13 +1474,13 @@
         <v>2</v>
       </c>
       <c r="G12" s="4">
-        <v>1799.5</v>
+        <v>1809.57</v>
       </c>
       <c r="H12" s="4">
-        <v>31457.13</v>
+        <v>31633.200000000001</v>
       </c>
       <c r="I12" s="4">
-        <v>33256.629999999997</v>
+        <v>33442.769999999997</v>
       </c>
       <c r="J12" s="3">
         <v>0</v>
@@ -1489,10 +1489,10 @@
         <v>0</v>
       </c>
       <c r="L12" s="4">
-        <v>31450.71</v>
+        <v>31626.75</v>
       </c>
       <c r="M12" s="4">
-        <v>31450.71</v>
+        <v>31626.75</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
@@ -1518,22 +1518,22 @@
         <v>0</v>
       </c>
       <c r="H13" s="4">
-        <v>32519.97</v>
+        <v>32702</v>
       </c>
       <c r="I13" s="4">
-        <v>32519.97</v>
+        <v>32702</v>
       </c>
       <c r="J13" s="3">
         <v>1</v>
       </c>
       <c r="K13" s="4">
-        <v>20413.86</v>
+        <v>20528.12</v>
       </c>
       <c r="L13" s="4">
-        <v>27571.52</v>
+        <v>27725.85</v>
       </c>
       <c r="M13" s="4">
-        <v>47985.38</v>
+        <v>48253.97</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="4">
-        <v>28771.72</v>
+        <v>28932.77</v>
       </c>
       <c r="I14" s="4">
-        <v>28771.72</v>
+        <v>28932.77</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1571,10 +1571,10 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>71929.289999999994</v>
+        <v>72331.92</v>
       </c>
       <c r="M14" s="4">
-        <v>71929.289999999994</v>
+        <v>72331.92</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
@@ -1600,10 +1600,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>27387.119999999999</v>
+        <v>27170.38</v>
       </c>
       <c r="I15" s="4">
-        <v>27387.119999999999</v>
+        <v>27170.38</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>90033.83</v>
+        <v>88687.54</v>
       </c>
       <c r="M15" s="4">
-        <v>90033.83</v>
+        <v>88687.54</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
@@ -1641,10 +1641,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>20308.48</v>
+        <v>22129.06</v>
       </c>
       <c r="I16" s="4">
-        <v>20308.48</v>
+        <v>22129.06</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1653,10 +1653,10 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>41972.38</v>
+        <v>40871.43</v>
       </c>
       <c r="M16" s="4">
-        <v>41972.38</v>
+        <v>40871.43</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
@@ -1679,13 +1679,13 @@
         <v>1</v>
       </c>
       <c r="G17" s="4">
-        <v>5401.65</v>
+        <v>5431.88</v>
       </c>
       <c r="H17" s="4">
-        <v>12985.22</v>
+        <v>13057.9</v>
       </c>
       <c r="I17" s="4">
-        <v>18386.87</v>
+        <v>18489.78</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1694,10 +1694,10 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>59418.13</v>
+        <v>59750.73</v>
       </c>
       <c r="M17" s="4">
-        <v>59418.13</v>
+        <v>59750.73</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
@@ -1723,10 +1723,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>17545.669999999998</v>
+        <v>17643.88</v>
       </c>
       <c r="I18" s="4">
-        <v>17545.669999999998</v>
+        <v>17643.88</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1735,24 +1735,24 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>13967.81</v>
+        <v>14045.98</v>
       </c>
       <c r="M18" s="4">
-        <v>13967.81</v>
+        <v>14045.98</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>104718</v>
+        <v>100677</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D19" s="11">
-        <v>45264</v>
+        <v>44999</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>51</v>
@@ -1764,10 +1764,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>12348.02</v>
+        <v>14628.23</v>
       </c>
       <c r="I19" s="4">
-        <v>12348.02</v>
+        <v>14628.23</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1776,24 +1776,24 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>94292.13</v>
+        <v>28892.68</v>
       </c>
       <c r="M19" s="4">
-        <v>94292.13</v>
+        <v>28892.68</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>100677</v>
+        <v>104718</v>
       </c>
       <c r="B20" s="2">
         <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="D20" s="11">
-        <v>44999</v>
+        <v>45264</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>51</v>
@@ -1805,10 +1805,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>12060.56</v>
+        <v>12417.13</v>
       </c>
       <c r="I20" s="4">
-        <v>12060.56</v>
+        <v>12417.13</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1817,10 +1817,10 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>33070.61</v>
+        <v>94819.93</v>
       </c>
       <c r="M20" s="4">
-        <v>33070.61</v>
+        <v>94819.93</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
@@ -1846,10 +1846,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>10253.4</v>
+        <v>10269.32</v>
       </c>
       <c r="I21" s="4">
-        <v>10253.4</v>
+        <v>10269.32</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1858,10 +1858,10 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>4006.82</v>
+        <v>3904.8</v>
       </c>
       <c r="M21" s="4">
-        <v>4006.82</v>
+        <v>3904.8</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
@@ -1887,10 +1887,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>9835.77</v>
+        <v>9890.82</v>
       </c>
       <c r="I22" s="4">
-        <v>9835.77</v>
+        <v>9890.82</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1899,24 +1899,24 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>20240.93</v>
+        <v>15958.97</v>
       </c>
       <c r="M22" s="4">
-        <v>20240.93</v>
+        <v>15958.97</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>113076</v>
+        <v>80925</v>
       </c>
       <c r="B23" s="2">
         <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="D23" s="11">
-        <v>45806</v>
+        <v>43439</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>51</v>
@@ -1928,10 +1928,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>9117.0400000000009</v>
+        <v>9535.86</v>
       </c>
       <c r="I23" s="4">
-        <v>9117.0400000000009</v>
+        <v>9535.86</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1940,24 +1940,24 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>4558.5200000000004</v>
+        <v>0</v>
       </c>
       <c r="M23" s="4">
-        <v>4558.5200000000004</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>110105</v>
+        <v>113076</v>
       </c>
       <c r="B24" s="2">
         <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D24" s="11">
-        <v>45560</v>
+        <v>45806</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>51</v>
@@ -1969,10 +1969,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>8925.7000000000007</v>
+        <v>9168.08</v>
       </c>
       <c r="I24" s="4">
-        <v>8925.7000000000007</v>
+        <v>9168.08</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1981,24 +1981,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>4151.0600000000004</v>
+        <v>4584.04</v>
       </c>
       <c r="M24" s="4">
-        <v>4151.0600000000004</v>
+        <v>4584.04</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>101640</v>
+        <v>110105</v>
       </c>
       <c r="B25" s="2">
         <v>2043</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="D25" s="11">
-        <v>45104</v>
+        <v>45560</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>51</v>
@@ -2010,10 +2010,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>8802.09</v>
+        <v>8975.67</v>
       </c>
       <c r="I25" s="4">
-        <v>8802.09</v>
+        <v>8975.67</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -2022,39 +2022,39 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>0</v>
+        <v>4174.3</v>
       </c>
       <c r="M25" s="4">
-        <v>0</v>
+        <v>4174.3</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>104343</v>
+        <v>101640</v>
       </c>
       <c r="B26" s="2">
         <v>2043</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="D26" s="11">
-        <v>45201</v>
+        <v>45104</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F26" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G26" s="4">
-        <v>1732.64</v>
+        <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>6954.33</v>
+        <v>8851.3700000000008</v>
       </c>
       <c r="I26" s="4">
-        <v>8686.9699999999993</v>
+        <v>8851.3700000000008</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2063,65 +2063,65 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>53096.78</v>
+        <v>0</v>
       </c>
       <c r="M26" s="4">
-        <v>53096.78</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>102825</v>
+        <v>104343</v>
       </c>
       <c r="B27" s="2">
         <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="D27" s="11">
-        <v>45117</v>
+        <v>45201</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F27" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G27" s="4">
-        <v>0</v>
+        <v>1742.34</v>
       </c>
       <c r="H27" s="4">
-        <v>8047.52</v>
+        <v>6993.26</v>
       </c>
       <c r="I27" s="4">
-        <v>8047.52</v>
+        <v>8735.6</v>
       </c>
       <c r="J27" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" s="4">
-        <v>30557.77</v>
+        <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>13589.8</v>
+        <v>53393.98</v>
       </c>
       <c r="M27" s="4">
-        <v>44147.57</v>
+        <v>53393.98</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>108405</v>
+        <v>102825</v>
       </c>
       <c r="B28" s="2">
         <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="D28" s="11">
-        <v>45471</v>
+        <v>45117</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>51</v>
@@ -2133,51 +2133,51 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>7542.1</v>
+        <v>8092.57</v>
       </c>
       <c r="I28" s="4">
-        <v>7542.1</v>
+        <v>8092.57</v>
       </c>
       <c r="J28" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28" s="4">
-        <v>0</v>
+        <v>30728.82</v>
       </c>
       <c r="L28" s="4">
-        <v>4985.49</v>
+        <v>13665.87</v>
       </c>
       <c r="M28" s="4">
-        <v>4985.49</v>
+        <v>44394.69</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>94156</v>
+        <v>88234</v>
       </c>
       <c r="B29" s="2">
         <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D29" s="11">
-        <v>44159</v>
+        <v>43794</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F29" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" s="4">
-        <v>0</v>
+        <v>2170.37</v>
       </c>
       <c r="H29" s="4">
-        <v>6945.5</v>
+        <v>5569.34</v>
       </c>
       <c r="I29" s="4">
-        <v>6945.5</v>
+        <v>7739.71</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2186,24 +2186,24 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>0</v>
+        <v>15833.25</v>
       </c>
       <c r="M29" s="4">
-        <v>0</v>
+        <v>15833.25</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>109007</v>
+        <v>108405</v>
       </c>
       <c r="B30" s="2">
         <v>2043</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="D30" s="11">
-        <v>45525</v>
+        <v>45471</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>51</v>
@@ -2215,10 +2215,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>6197.51</v>
+        <v>7584.32</v>
       </c>
       <c r="I30" s="4">
-        <v>6197.51</v>
+        <v>7584.32</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2227,24 +2227,24 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>0</v>
+        <v>5013.3900000000003</v>
       </c>
       <c r="M30" s="4">
-        <v>0</v>
+        <v>5013.3900000000003</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>109998</v>
+        <v>109007</v>
       </c>
       <c r="B31" s="2">
         <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D31" s="11">
-        <v>45596</v>
+        <v>45525</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>51</v>
@@ -2256,10 +2256,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>5824.66</v>
+        <v>7097.28</v>
       </c>
       <c r="I31" s="4">
-        <v>5824.66</v>
+        <v>7097.28</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -2276,16 +2276,16 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>90177</v>
+        <v>94156</v>
       </c>
       <c r="B32" s="2">
         <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D32" s="11">
-        <v>43949</v>
+        <v>44159</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>51</v>
@@ -2297,10 +2297,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>5199.32</v>
+        <v>6984.37</v>
       </c>
       <c r="I32" s="4">
-        <v>5199.32</v>
+        <v>6984.37</v>
       </c>
       <c r="J32" s="3">
         <v>0</v>
@@ -2317,16 +2317,16 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>80925</v>
+        <v>115047</v>
       </c>
       <c r="B33" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="D33" s="11">
-        <v>43439</v>
+        <v>45944</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>51</v>
@@ -2338,10 +2338,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>5149.7700000000004</v>
+        <v>6880.21</v>
       </c>
       <c r="I33" s="4">
-        <v>5149.7700000000004</v>
+        <v>6880.21</v>
       </c>
       <c r="J33" s="3">
         <v>0</v>
@@ -2350,24 +2350,24 @@
         <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>0</v>
+        <v>34161.040000000001</v>
       </c>
       <c r="M33" s="4">
-        <v>0</v>
+        <v>34161.040000000001</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>115047</v>
+        <v>109998</v>
       </c>
       <c r="B34" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="D34" s="11">
-        <v>45944</v>
+        <v>45596</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>51</v>
@@ -2379,10 +2379,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>5025.2</v>
+        <v>5857.26</v>
       </c>
       <c r="I34" s="4">
-        <v>5025.2</v>
+        <v>5857.26</v>
       </c>
       <c r="J34" s="3">
         <v>0</v>
@@ -2391,24 +2391,24 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>35787.599999999999</v>
+        <v>0</v>
       </c>
       <c r="M34" s="4">
-        <v>35787.599999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>88234</v>
+        <v>90177</v>
       </c>
       <c r="B35" s="2">
         <v>2043</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="D35" s="11">
-        <v>43794</v>
+        <v>43949</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>51</v>
@@ -2420,22 +2420,22 @@
         <v>0</v>
       </c>
       <c r="H35" s="4">
-        <v>4242.34</v>
+        <v>5228.43</v>
       </c>
       <c r="I35" s="4">
-        <v>4242.34</v>
+        <v>5228.43</v>
       </c>
       <c r="J35" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K35" s="4">
-        <v>3454.14</v>
+        <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>15745.12</v>
+        <v>0</v>
       </c>
       <c r="M35" s="4">
-        <v>19199.259999999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
@@ -2461,10 +2461,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="4">
-        <v>3887.59</v>
+        <v>3909.35</v>
       </c>
       <c r="I36" s="4">
-        <v>3887.59</v>
+        <v>3909.35</v>
       </c>
       <c r="J36" s="3">
         <v>0</v>
@@ -2502,10 +2502,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="4">
-        <v>3335.25</v>
+        <v>3353.92</v>
       </c>
       <c r="I37" s="4">
-        <v>3335.25</v>
+        <v>3353.92</v>
       </c>
       <c r="J37" s="3">
         <v>0</v>
@@ -2514,10 +2514,10 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>36259.129999999997</v>
+        <v>36462.1</v>
       </c>
       <c r="M37" s="4">
-        <v>36259.129999999997</v>
+        <v>36462.1</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
@@ -2543,10 +2543,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="4">
-        <v>2020.62</v>
+        <v>2031.93</v>
       </c>
       <c r="I38" s="4">
-        <v>2020.62</v>
+        <v>2031.93</v>
       </c>
       <c r="J38" s="3">
         <v>0</v>
@@ -2555,10 +2555,10 @@
         <v>0</v>
       </c>
       <c r="L38" s="4">
-        <v>16164.97</v>
+        <v>16255.46</v>
       </c>
       <c r="M38" s="4">
-        <v>16164.97</v>
+        <v>16255.46</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
@@ -2581,13 +2581,13 @@
         <v>1</v>
       </c>
       <c r="G39" s="4">
-        <v>1795.63</v>
+        <v>1805.68</v>
       </c>
       <c r="H39" s="4">
         <v>0</v>
       </c>
       <c r="I39" s="4">
-        <v>1795.63</v>
+        <v>1805.68</v>
       </c>
       <c r="J39" s="3">
         <v>0</v>
@@ -2596,10 +2596,10 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>19751.93</v>
+        <v>19862.490000000002</v>
       </c>
       <c r="M39" s="4">
-        <v>19751.93</v>
+        <v>19862.490000000002</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
@@ -2625,10 +2625,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="4">
-        <v>1778.41</v>
+        <v>1788.37</v>
       </c>
       <c r="I40" s="4">
-        <v>1778.41</v>
+        <v>1788.37</v>
       </c>
       <c r="J40" s="3">
         <v>0</v>
@@ -2637,10 +2637,10 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>17784.11</v>
+        <v>17883.650000000001</v>
       </c>
       <c r="M40" s="4">
-        <v>17784.11</v>
+        <v>17883.650000000001</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
@@ -2666,10 +2666,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="4">
-        <v>1750.74</v>
+        <v>1760.54</v>
       </c>
       <c r="I41" s="4">
-        <v>1750.74</v>
+        <v>1760.54</v>
       </c>
       <c r="J41" s="3">
         <v>0</v>
@@ -2678,10 +2678,10 @@
         <v>0</v>
       </c>
       <c r="L41" s="4">
-        <v>4934.1099999999997</v>
+        <v>4961.7299999999996</v>
       </c>
       <c r="M41" s="4">
-        <v>4934.1099999999997</v>
+        <v>4961.7299999999996</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
@@ -2707,10 +2707,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="4">
-        <v>1738.61</v>
+        <v>1748.34</v>
       </c>
       <c r="I42" s="4">
-        <v>1738.61</v>
+        <v>1748.34</v>
       </c>
       <c r="J42" s="3">
         <v>0</v>
@@ -2719,27 +2719,27 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>10431.68</v>
+        <v>10490.07</v>
       </c>
       <c r="M42" s="4">
-        <v>10431.68</v>
+        <v>10490.07</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>116795</v>
+        <v>114431</v>
       </c>
       <c r="B43" s="2">
         <v>2043</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="D43" s="11">
-        <v>46000</v>
+        <v>45930</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="F43" s="3">
         <v>0</v>
@@ -2748,10 +2748,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="4">
-        <v>1594.18</v>
+        <v>1698.61</v>
       </c>
       <c r="I43" s="4">
-        <v>1594.18</v>
+        <v>1698.61</v>
       </c>
       <c r="J43" s="3">
         <v>0</v>
@@ -2760,27 +2760,27 @@
         <v>0</v>
       </c>
       <c r="L43" s="4">
-        <v>0</v>
+        <v>20181.939999999999</v>
       </c>
       <c r="M43" s="4">
-        <v>0</v>
+        <v>20181.939999999999</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>65046</v>
+        <v>116795</v>
       </c>
       <c r="B44" s="2">
         <v>2043</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>16</v>
+        <v>56</v>
       </c>
       <c r="D44" s="11">
-        <v>44763</v>
+        <v>46000</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F44" s="3">
         <v>0</v>
@@ -2789,10 +2789,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="4">
-        <v>1037.77</v>
+        <v>1603.11</v>
       </c>
       <c r="I44" s="4">
-        <v>1037.77</v>
+        <v>1603.11</v>
       </c>
       <c r="J44" s="3">
         <v>0</v>
@@ -2801,24 +2801,24 @@
         <v>0</v>
       </c>
       <c r="L44" s="4">
-        <v>16347.18</v>
+        <v>0</v>
       </c>
       <c r="M44" s="4">
-        <v>16347.18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
-        <v>114431</v>
+        <v>65046</v>
       </c>
       <c r="B45" s="2">
         <v>2043</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="D45" s="11">
-        <v>45930</v>
+        <v>44763</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>51</v>
@@ -2830,10 +2830,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="4">
-        <v>0</v>
+        <v>1043.58</v>
       </c>
       <c r="I45" s="4">
-        <v>0</v>
+        <v>1043.58</v>
       </c>
       <c r="J45" s="3">
         <v>0</v>
@@ -2842,10 +2842,10 @@
         <v>0</v>
       </c>
       <c r="L45" s="4">
-        <v>21758.76</v>
+        <v>16438.689999999999</v>
       </c>
       <c r="M45" s="4">
-        <v>21758.76</v>
+        <v>16438.689999999999</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
@@ -2883,10 +2883,10 @@
         <v>0</v>
       </c>
       <c r="L46" s="4">
-        <v>15063.56</v>
+        <v>15147.88</v>
       </c>
       <c r="M46" s="4">
-        <v>15063.56</v>
+        <v>15147.88</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.2">
@@ -2924,10 +2924,10 @@
         <v>0</v>
       </c>
       <c r="L47" s="4">
-        <v>9207.01</v>
+        <v>9258.5400000000009</v>
       </c>
       <c r="M47" s="4">
-        <v>9207.01</v>
+        <v>9258.5400000000009</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.2">
@@ -2991,7 +2991,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48:M50">
-    <cfRule type="expression" dxfId="18" priority="101" stopIfTrue="1">
+    <cfRule type="expression" dxfId="18" priority="113" stopIfTrue="1">
       <formula>$S47=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-05-18 10:23)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{672C5976-8717-6D4B-AF91-4A157272E43C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FBE000-FA2E-7048-AAAE-FBBCF1BCFC8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -1041,7 +1041,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46150</v>
+        <v>46155</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1149,45 +1149,45 @@
         <v>64988.26</v>
       </c>
       <c r="J4" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" s="4">
-        <v>0</v>
+        <v>70933.600000000006</v>
       </c>
       <c r="L4" s="4">
         <v>79316.52</v>
       </c>
       <c r="M4" s="4">
-        <v>79316.52</v>
+        <v>150250.12</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
-        <v>110453</v>
+        <v>87538</v>
       </c>
       <c r="B5" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D5" s="11">
-        <v>45600</v>
+        <v>43731</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F5" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" s="4">
-        <v>1602.22</v>
+        <v>0</v>
       </c>
       <c r="H5" s="4">
-        <v>37882.449999999997</v>
+        <v>45940.15</v>
       </c>
       <c r="I5" s="4">
-        <v>39484.67</v>
+        <v>45940.15</v>
       </c>
       <c r="J5" s="3">
         <v>0</v>
@@ -1196,24 +1196,24 @@
         <v>0</v>
       </c>
       <c r="L5" s="4">
-        <v>135856.64000000001</v>
+        <v>265206.39</v>
       </c>
       <c r="M5" s="4">
-        <v>135856.64000000001</v>
+        <v>265206.39</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>100677</v>
+        <v>110453</v>
       </c>
       <c r="B6" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="D6" s="11">
-        <v>44999</v>
+        <v>45600</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>50</v>
@@ -1222,13 +1222,13 @@
         <v>1</v>
       </c>
       <c r="G6" s="4">
-        <v>2646.37</v>
+        <v>1602.22</v>
       </c>
       <c r="H6" s="4">
-        <v>23292.74</v>
+        <v>37882.449999999997</v>
       </c>
       <c r="I6" s="4">
-        <v>25939.11</v>
+        <v>39484.67</v>
       </c>
       <c r="J6" s="3">
         <v>0</v>
@@ -1237,24 +1237,24 @@
         <v>0</v>
       </c>
       <c r="L6" s="4">
-        <v>14264.78</v>
+        <v>135856.64000000001</v>
       </c>
       <c r="M6" s="4">
-        <v>14264.78</v>
+        <v>135856.64000000001</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>114100</v>
+        <v>118069</v>
       </c>
       <c r="B7" s="2">
         <v>2856</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>14</v>
+        <v>53</v>
       </c>
       <c r="D7" s="11">
-        <v>45863</v>
+        <v>46105</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>50</v>
@@ -1263,39 +1263,39 @@
         <v>1</v>
       </c>
       <c r="G7" s="4">
-        <v>2455.46</v>
+        <v>1582.52</v>
       </c>
       <c r="H7" s="4">
-        <v>20499.45</v>
+        <v>31354.39</v>
       </c>
       <c r="I7" s="4">
-        <v>22954.91</v>
+        <v>32936.910000000003</v>
       </c>
       <c r="J7" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7" s="4">
-        <v>0</v>
+        <v>1484.19</v>
       </c>
       <c r="L7" s="4">
-        <v>25302.33</v>
+        <v>17883.650000000001</v>
       </c>
       <c r="M7" s="4">
-        <v>25302.33</v>
+        <v>19367.84</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>102825</v>
+        <v>100677</v>
       </c>
       <c r="B8" s="2">
         <v>2043</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D8" s="11">
-        <v>45117</v>
+        <v>44999</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>50</v>
@@ -1304,13 +1304,13 @@
         <v>1</v>
       </c>
       <c r="G8" s="4">
-        <v>1494.27</v>
+        <v>2646.37</v>
       </c>
       <c r="H8" s="4">
-        <v>21235.73</v>
+        <v>25549.86</v>
       </c>
       <c r="I8" s="4">
-        <v>22730</v>
+        <v>28196.23</v>
       </c>
       <c r="J8" s="3">
         <v>0</v>
@@ -1319,39 +1319,39 @@
         <v>0</v>
       </c>
       <c r="L8" s="4">
-        <v>8829.19</v>
+        <v>12007.66</v>
       </c>
       <c r="M8" s="4">
-        <v>8829.19</v>
+        <v>12007.66</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>88234</v>
+        <v>114100</v>
       </c>
       <c r="B9" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D9" s="11">
-        <v>43794</v>
+        <v>45863</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F9" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="4">
-        <v>0</v>
+        <v>2455.46</v>
       </c>
       <c r="H9" s="4">
-        <v>7739.54</v>
+        <v>21456.49</v>
       </c>
       <c r="I9" s="4">
-        <v>7739.54</v>
+        <v>23911.95</v>
       </c>
       <c r="J9" s="3">
         <v>0</v>
@@ -1360,39 +1360,39 @@
         <v>0</v>
       </c>
       <c r="L9" s="4">
-        <v>11567.17</v>
+        <v>25302.33</v>
       </c>
       <c r="M9" s="4">
-        <v>11567.17</v>
+        <v>25302.33</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>117440</v>
+        <v>102825</v>
       </c>
       <c r="B10" s="2">
         <v>2043</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="D10" s="11">
-        <v>46149</v>
+        <v>45117</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F10" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="4">
-        <v>0</v>
+        <v>1494.27</v>
       </c>
       <c r="H10" s="4">
-        <v>7572.39</v>
+        <v>21235.73</v>
       </c>
       <c r="I10" s="4">
-        <v>7572.39</v>
+        <v>22730</v>
       </c>
       <c r="J10" s="3">
         <v>0</v>
@@ -1401,80 +1401,80 @@
         <v>0</v>
       </c>
       <c r="L10" s="4">
-        <v>65236.3</v>
+        <v>8829.19</v>
       </c>
       <c r="M10" s="4">
-        <v>65236.3</v>
+        <v>8829.19</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>80122</v>
+        <v>80925</v>
       </c>
       <c r="B11" s="2">
         <v>2043</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D11" s="11">
-        <v>43371</v>
+        <v>43439</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F11" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" s="4">
-        <v>0</v>
+        <v>22698.89</v>
       </c>
       <c r="H11" s="4">
-        <v>6101.01</v>
+        <v>0</v>
       </c>
       <c r="I11" s="4">
-        <v>6101.01</v>
+        <v>22698.89</v>
       </c>
       <c r="J11" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" s="4">
-        <v>23934.57</v>
+        <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>156248.23000000001</v>
+        <v>15382.81</v>
       </c>
       <c r="M11" s="4">
-        <v>180182.8</v>
+        <v>15382.81</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>104718</v>
+        <v>104750</v>
       </c>
       <c r="B12" s="2">
         <v>2043</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D12" s="11">
-        <v>45264</v>
+        <v>45236</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" s="4">
-        <v>0</v>
+        <v>1562.11</v>
       </c>
       <c r="H12" s="4">
-        <v>5436.12</v>
+        <v>16583.3</v>
       </c>
       <c r="I12" s="4">
-        <v>5436.12</v>
+        <v>18145.41</v>
       </c>
       <c r="J12" s="3">
         <v>0</v>
@@ -1483,24 +1483,24 @@
         <v>0</v>
       </c>
       <c r="L12" s="4">
-        <v>94744.69</v>
+        <v>26942.720000000001</v>
       </c>
       <c r="M12" s="4">
-        <v>94744.69</v>
+        <v>26942.720000000001</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>47116</v>
+        <v>115047</v>
       </c>
       <c r="B13" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="D13" s="11">
-        <v>44616</v>
+        <v>45944</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>50</v>
@@ -1512,10 +1512,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="4">
-        <v>4896.25</v>
+        <v>9504.58</v>
       </c>
       <c r="I13" s="4">
-        <v>4896.25</v>
+        <v>9504.58</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1524,24 +1524,24 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>61089.919999999998</v>
+        <v>29704.73</v>
       </c>
       <c r="M13" s="4">
-        <v>61089.919999999998</v>
+        <v>29704.73</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>104750</v>
+        <v>88234</v>
       </c>
       <c r="B14" s="2">
         <v>2043</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D14" s="11">
-        <v>45236</v>
+        <v>43794</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>50</v>
@@ -1553,10 +1553,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="4">
-        <v>4478.46</v>
+        <v>7739.54</v>
       </c>
       <c r="I14" s="4">
-        <v>4478.46</v>
+        <v>7739.54</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1565,24 +1565,24 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>28603.15</v>
+        <v>11567.17</v>
       </c>
       <c r="M14" s="4">
-        <v>28603.15</v>
+        <v>11567.17</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>115047</v>
+        <v>117440</v>
       </c>
       <c r="B15" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>5</v>
+        <v>51</v>
       </c>
       <c r="D15" s="11">
-        <v>45944</v>
+        <v>46149</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>50</v>
@@ -1594,10 +1594,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>4456.29</v>
+        <v>7572.39</v>
       </c>
       <c r="I15" s="4">
-        <v>4456.29</v>
+        <v>7572.39</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1606,24 +1606,24 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>34753.07</v>
+        <v>65236.3</v>
       </c>
       <c r="M15" s="4">
-        <v>34753.07</v>
+        <v>65236.3</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>108404</v>
+        <v>80122</v>
       </c>
       <c r="B16" s="2">
         <v>2043</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D16" s="11">
-        <v>45467</v>
+        <v>43371</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>50</v>
@@ -1635,10 +1635,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>3982.49</v>
+        <v>6362.33</v>
       </c>
       <c r="I16" s="4">
-        <v>3982.49</v>
+        <v>6362.33</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1647,24 +1647,24 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>14324.23</v>
+        <v>151848.75</v>
       </c>
       <c r="M16" s="4">
-        <v>14324.23</v>
+        <v>151848.75</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>107488</v>
+        <v>104718</v>
       </c>
       <c r="B17" s="2">
         <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="D17" s="11">
-        <v>45440</v>
+        <v>45264</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>50</v>
@@ -1676,10 +1676,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>3303.04</v>
+        <v>5436.12</v>
       </c>
       <c r="I17" s="4">
-        <v>3303.04</v>
+        <v>5436.12</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1688,24 +1688,24 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>90799.97</v>
+        <v>94744.69</v>
       </c>
       <c r="M17" s="4">
-        <v>90799.97</v>
+        <v>94744.69</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>106018</v>
+        <v>47116</v>
       </c>
       <c r="B18" s="2">
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="D18" s="11">
-        <v>45344</v>
+        <v>44616</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>50</v>
@@ -1717,36 +1717,36 @@
         <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>3116.45</v>
+        <v>4896.25</v>
       </c>
       <c r="I18" s="4">
-        <v>3116.45</v>
+        <v>4896.25</v>
       </c>
       <c r="J18" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" s="4">
-        <v>0</v>
+        <v>30484.55</v>
       </c>
       <c r="L18" s="4">
-        <v>16834.04</v>
+        <v>61089.919999999998</v>
       </c>
       <c r="M18" s="4">
-        <v>16834.04</v>
+        <v>91574.47</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>109998</v>
+        <v>101640</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="D19" s="11">
-        <v>45596</v>
+        <v>45104</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>50</v>
@@ -1758,10 +1758,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>2974.66</v>
+        <v>4745.09</v>
       </c>
       <c r="I19" s="4">
-        <v>2974.66</v>
+        <v>4745.09</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1770,24 +1770,24 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>0</v>
+        <v>3222.89</v>
       </c>
       <c r="M19" s="4">
-        <v>0</v>
+        <v>3222.89</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>108405</v>
+        <v>108404</v>
       </c>
       <c r="B20" s="2">
         <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="D20" s="11">
-        <v>45471</v>
+        <v>45467</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>50</v>
@@ -1799,10 +1799,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>2506.6999999999998</v>
+        <v>3982.49</v>
       </c>
       <c r="I20" s="4">
-        <v>2506.6999999999998</v>
+        <v>3982.49</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1811,24 +1811,24 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>5556.45</v>
+        <v>14324.23</v>
       </c>
       <c r="M20" s="4">
-        <v>5556.45</v>
+        <v>14324.23</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>101640</v>
+        <v>107488</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="D21" s="11">
-        <v>45104</v>
+        <v>45440</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>50</v>
@@ -1840,10 +1840,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>2347.6799999999998</v>
+        <v>3303.04</v>
       </c>
       <c r="I21" s="4">
-        <v>2347.6799999999998</v>
+        <v>3303.04</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1852,27 +1852,27 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>5620.28</v>
+        <v>90799.97</v>
       </c>
       <c r="M21" s="4">
-        <v>5620.28</v>
+        <v>90799.97</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>63441</v>
+        <v>106018</v>
       </c>
       <c r="B22" s="2">
-        <v>2511</v>
+        <v>2043</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="D22" s="11">
-        <v>44733</v>
+        <v>45344</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F22" s="3">
         <v>0</v>
@@ -1881,10 +1881,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>1851.71</v>
+        <v>3116.45</v>
       </c>
       <c r="I22" s="4">
-        <v>1851.71</v>
+        <v>3116.45</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1893,24 +1893,24 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>7406.83</v>
+        <v>16834.04</v>
       </c>
       <c r="M22" s="4">
-        <v>7406.83</v>
+        <v>16834.04</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>112083</v>
+        <v>109998</v>
       </c>
       <c r="B23" s="2">
         <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="D23" s="11">
-        <v>45736</v>
+        <v>45596</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>50</v>
@@ -1922,10 +1922,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>1805.68</v>
+        <v>2974.66</v>
       </c>
       <c r="I23" s="4">
-        <v>1805.68</v>
+        <v>2974.66</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1934,24 +1934,24 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>18056.810000000001</v>
+        <v>0</v>
       </c>
       <c r="M23" s="4">
-        <v>18056.810000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>87538</v>
+        <v>108405</v>
       </c>
       <c r="B24" s="2">
         <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="D24" s="11">
-        <v>43731</v>
+        <v>45471</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>50</v>
@@ -1963,10 +1963,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>1781.12</v>
+        <v>2506.6999999999998</v>
       </c>
       <c r="I24" s="4">
-        <v>1781.12</v>
+        <v>2506.6999999999998</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1975,24 +1975,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>309365.42</v>
+        <v>5556.45</v>
       </c>
       <c r="M24" s="4">
-        <v>309365.42</v>
+        <v>5556.45</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>65046</v>
+        <v>63441</v>
       </c>
       <c r="B25" s="2">
-        <v>2043</v>
+        <v>2511</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D25" s="11">
-        <v>44763</v>
+        <v>44733</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>50</v>
@@ -2004,10 +2004,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>1752.06</v>
+        <v>1851.71</v>
       </c>
       <c r="I25" s="4">
-        <v>1752.06</v>
+        <v>1851.71</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -2016,24 +2016,24 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>14686.63</v>
+        <v>7406.83</v>
       </c>
       <c r="M25" s="4">
-        <v>14686.63</v>
+        <v>7406.83</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>105696</v>
+        <v>112083</v>
       </c>
       <c r="B26" s="2">
         <v>2043</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="D26" s="11">
-        <v>45279</v>
+        <v>45736</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>50</v>
@@ -2045,10 +2045,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>1742.16</v>
+        <v>1805.68</v>
       </c>
       <c r="I26" s="4">
-        <v>1742.16</v>
+        <v>1805.68</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2057,24 +2057,24 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>85511.7</v>
+        <v>18056.810000000001</v>
       </c>
       <c r="M26" s="4">
-        <v>85511.7</v>
+        <v>18056.810000000001</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>115404</v>
+        <v>65046</v>
       </c>
       <c r="B27" s="2">
         <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D27" s="11">
-        <v>45986</v>
+        <v>44763</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>50</v>
@@ -2086,10 +2086,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>662.59</v>
+        <v>1752.06</v>
       </c>
       <c r="I27" s="4">
-        <v>662.59</v>
+        <v>1752.06</v>
       </c>
       <c r="J27" s="3">
         <v>0</v>
@@ -2098,24 +2098,24 @@
         <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>10490.07</v>
+        <v>14686.63</v>
       </c>
       <c r="M27" s="4">
-        <v>10490.07</v>
+        <v>14686.63</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>118069</v>
+        <v>105696</v>
       </c>
       <c r="B28" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="D28" s="11">
-        <v>46105</v>
+        <v>45279</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>50</v>
@@ -2127,36 +2127,36 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>0</v>
+        <v>1742.16</v>
       </c>
       <c r="I28" s="4">
-        <v>0</v>
+        <v>1742.16</v>
       </c>
       <c r="J28" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" s="4">
-        <v>1484.19</v>
+        <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>17883.650000000001</v>
+        <v>85511.7</v>
       </c>
       <c r="M28" s="4">
-        <v>19367.84</v>
+        <v>85511.7</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>116883</v>
+        <v>114157</v>
       </c>
       <c r="B29" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="D29" s="11">
-        <v>46126</v>
+        <v>45904</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>50</v>
@@ -2168,10 +2168,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>0</v>
+        <v>1646.66</v>
       </c>
       <c r="I29" s="4">
-        <v>0</v>
+        <v>1646.66</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2180,24 +2180,24 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>85605.95</v>
+        <v>62230.01</v>
       </c>
       <c r="M29" s="4">
-        <v>85605.95</v>
+        <v>62230.01</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>116876</v>
+        <v>115404</v>
       </c>
       <c r="B30" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D30" s="11">
-        <v>46111</v>
+        <v>45986</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>50</v>
@@ -2209,10 +2209,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>0</v>
+        <v>662.59</v>
       </c>
       <c r="I30" s="4">
-        <v>0</v>
+        <v>662.59</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2221,24 +2221,24 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>16255.46</v>
+        <v>10490.07</v>
       </c>
       <c r="M30" s="4">
-        <v>16255.46</v>
+        <v>10490.07</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>116060</v>
+        <v>116883</v>
       </c>
       <c r="B31" s="2">
         <v>2856</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D31" s="11">
-        <v>46010</v>
+        <v>46126</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>50</v>
@@ -2262,27 +2262,27 @@
         <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>45412.23</v>
+        <v>85605.95</v>
       </c>
       <c r="M31" s="4">
-        <v>45412.23</v>
+        <v>85605.95</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>114431</v>
+        <v>116876</v>
       </c>
       <c r="B32" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D32" s="11">
-        <v>45930</v>
+        <v>46111</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F32" s="3">
         <v>0</v>
@@ -2303,24 +2303,24 @@
         <v>0</v>
       </c>
       <c r="L32" s="4">
-        <v>20181.939999999999</v>
+        <v>16255.46</v>
       </c>
       <c r="M32" s="4">
-        <v>20181.939999999999</v>
+        <v>16255.46</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>114157</v>
+        <v>116060</v>
       </c>
       <c r="B33" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="D33" s="11">
-        <v>45904</v>
+        <v>46010</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>50</v>
@@ -2344,27 +2344,27 @@
         <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>63876.67</v>
+        <v>45412.23</v>
       </c>
       <c r="M33" s="4">
-        <v>63876.67</v>
+        <v>45412.23</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>113450</v>
+        <v>114431</v>
       </c>
       <c r="B34" s="2">
         <v>2043</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D34" s="11">
-        <v>45852</v>
+        <v>45930</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F34" s="3">
         <v>0</v>
@@ -2385,27 +2385,27 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>3904.8</v>
+        <v>20181.939999999999</v>
       </c>
       <c r="M34" s="4">
-        <v>3904.8</v>
+        <v>20181.939999999999</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>113076</v>
+        <v>113450</v>
       </c>
       <c r="B35" s="2">
         <v>2043</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D35" s="11">
-        <v>45806</v>
+        <v>45852</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F35" s="3">
         <v>0</v>
@@ -2426,27 +2426,27 @@
         <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>4584.04</v>
+        <v>3904.8</v>
       </c>
       <c r="M35" s="4">
-        <v>4584.04</v>
+        <v>3904.8</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>112522</v>
+        <v>113076</v>
       </c>
       <c r="B36" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D36" s="11">
-        <v>45776</v>
+        <v>45806</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F36" s="3">
         <v>0</v>
@@ -2467,24 +2467,24 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>4961.7299999999996</v>
+        <v>4584.04</v>
       </c>
       <c r="M36" s="4">
-        <v>4961.7299999999996</v>
+        <v>4584.04</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>111056</v>
+        <v>112522</v>
       </c>
       <c r="B37" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="D37" s="11">
-        <v>45639</v>
+        <v>45776</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>50</v>
@@ -2508,24 +2508,24 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>10951.05</v>
+        <v>4961.7299999999996</v>
       </c>
       <c r="M37" s="4">
-        <v>10951.05</v>
+        <v>4961.7299999999996</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>110575</v>
+        <v>111056</v>
       </c>
       <c r="B38" s="2">
         <v>2043</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="D38" s="11">
-        <v>45583</v>
+        <v>45639</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>50</v>
@@ -2549,24 +2549,24 @@
         <v>0</v>
       </c>
       <c r="L38" s="4">
-        <v>72331.92</v>
+        <v>10951.05</v>
       </c>
       <c r="M38" s="4">
-        <v>72331.92</v>
+        <v>10951.05</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>110105</v>
+        <v>110575</v>
       </c>
       <c r="B39" s="2">
         <v>2043</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D39" s="11">
-        <v>45560</v>
+        <v>45583</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>50</v>
@@ -2590,24 +2590,24 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>9502.52</v>
+        <v>72331.92</v>
       </c>
       <c r="M39" s="4">
-        <v>9502.52</v>
+        <v>72331.92</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>109007</v>
+        <v>110105</v>
       </c>
       <c r="B40" s="2">
         <v>2043</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D40" s="11">
-        <v>45525</v>
+        <v>45560</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>50</v>
@@ -2631,24 +2631,24 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>6211.67</v>
+        <v>9502.52</v>
       </c>
       <c r="M40" s="4">
-        <v>6211.67</v>
+        <v>9502.52</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>104343</v>
+        <v>109007</v>
       </c>
       <c r="B41" s="2">
         <v>2043</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="D41" s="11">
-        <v>45201</v>
+        <v>45525</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>50</v>
@@ -2672,27 +2672,27 @@
         <v>0</v>
       </c>
       <c r="L41" s="4">
-        <v>49471.7</v>
+        <v>6211.67</v>
       </c>
       <c r="M41" s="4">
-        <v>49471.7</v>
+        <v>6211.67</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>95148</v>
+        <v>104343</v>
       </c>
       <c r="B42" s="2">
         <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="D42" s="11">
-        <v>44916</v>
+        <v>45201</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F42" s="3">
         <v>0</v>
@@ -2713,27 +2713,27 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>3909.3</v>
+        <v>49471.7</v>
       </c>
       <c r="M42" s="4">
-        <v>3909.3</v>
+        <v>49471.7</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>94156</v>
+        <v>95148</v>
       </c>
       <c r="B43" s="2">
         <v>2043</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D43" s="11">
-        <v>44159</v>
+        <v>44916</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F43" s="3">
         <v>0</v>
@@ -2754,27 +2754,27 @@
         <v>0</v>
       </c>
       <c r="L43" s="4">
-        <v>7507.91</v>
+        <v>3909.3</v>
       </c>
       <c r="M43" s="4">
-        <v>7507.91</v>
+        <v>3909.3</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>81618</v>
+        <v>94156</v>
       </c>
       <c r="B44" s="2">
         <v>2043</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D44" s="11">
-        <v>43447</v>
+        <v>44159</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F44" s="3">
         <v>0</v>
@@ -2795,27 +2795,27 @@
         <v>0</v>
       </c>
       <c r="L44" s="4">
-        <v>15147.88</v>
+        <v>7507.91</v>
       </c>
       <c r="M44" s="4">
-        <v>15147.88</v>
+        <v>7507.91</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
-        <v>80925</v>
+        <v>81618</v>
       </c>
       <c r="B45" s="2">
         <v>2043</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D45" s="11">
-        <v>43439</v>
+        <v>43447</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F45" s="3">
         <v>0</v>
@@ -2830,16 +2830,16 @@
         <v>0</v>
       </c>
       <c r="J45" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K45" s="4">
-        <v>22698.89</v>
+        <v>0</v>
       </c>
       <c r="L45" s="4">
-        <v>15382.81</v>
+        <v>15147.88</v>
       </c>
       <c r="M45" s="4">
-        <v>38081.699999999997</v>
+        <v>15147.88</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
@@ -2927,34 +2927,19 @@
       <formula>$S45=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C46:H47 K46:L47">
-    <cfRule type="expression" dxfId="20" priority="19" stopIfTrue="1">
-      <formula>$S45=1</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="C46:H50 K46:L50">
     <cfRule type="expression" dxfId="19" priority="18" stopIfTrue="1">
       <formula>$S46=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C48:M50">
-    <cfRule type="expression" dxfId="18" priority="125" stopIfTrue="1">
-      <formula>$S47=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I46:I47 M46:M47">
-    <cfRule type="expression" dxfId="16" priority="21" stopIfTrue="1">
+  <conditionalFormatting sqref="C46:M50">
+    <cfRule type="expression" dxfId="18" priority="29" stopIfTrue="1">
       <formula>$S45=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I46:I50 M46:M50">
     <cfRule type="expression" dxfId="15" priority="20" stopIfTrue="1">
       <formula>$S46=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J46:J47">
-    <cfRule type="expression" dxfId="13" priority="17" stopIfTrue="1">
-      <formula>$S45=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J46:J50">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-05-20 10:21)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FBE000-FA2E-7048-AAAE-FBBCF1BCFC8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6F0FEFD-CC0B-C148-9F9C-E2DC14C43D53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -1041,7 +1041,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46155</v>
+        <v>46160</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1143,51 +1143,51 @@
         <v>35163.03</v>
       </c>
       <c r="H4" s="4">
-        <v>29825.23</v>
+        <v>53587.79</v>
       </c>
       <c r="I4" s="4">
-        <v>64988.26</v>
+        <v>88750.82</v>
       </c>
       <c r="J4" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" s="4">
-        <v>70933.600000000006</v>
+        <v>102294.53</v>
       </c>
       <c r="L4" s="4">
-        <v>79316.52</v>
+        <v>72521.25</v>
       </c>
       <c r="M4" s="4">
-        <v>150250.12</v>
+        <v>174815.78</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
-        <v>87538</v>
+        <v>47116</v>
       </c>
       <c r="B5" s="2">
         <v>2043</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="D5" s="11">
-        <v>43731</v>
+        <v>44616</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F5" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G5" s="4">
-        <v>0</v>
+        <v>32258.07</v>
       </c>
       <c r="H5" s="4">
-        <v>45940.15</v>
+        <v>21224.59</v>
       </c>
       <c r="I5" s="4">
-        <v>45940.15</v>
+        <v>53482.66</v>
       </c>
       <c r="J5" s="3">
         <v>0</v>
@@ -1196,39 +1196,39 @@
         <v>0</v>
       </c>
       <c r="L5" s="4">
-        <v>265206.39</v>
+        <v>61089.919999999998</v>
       </c>
       <c r="M5" s="4">
-        <v>265206.39</v>
+        <v>61089.919999999998</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>110453</v>
+        <v>87538</v>
       </c>
       <c r="B6" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D6" s="11">
-        <v>45600</v>
+        <v>43731</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F6" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="4">
-        <v>1602.22</v>
+        <v>0</v>
       </c>
       <c r="H6" s="4">
-        <v>37882.449999999997</v>
+        <v>48957.39</v>
       </c>
       <c r="I6" s="4">
-        <v>39484.67</v>
+        <v>48957.39</v>
       </c>
       <c r="J6" s="3">
         <v>0</v>
@@ -1237,24 +1237,24 @@
         <v>0</v>
       </c>
       <c r="L6" s="4">
-        <v>135856.64000000001</v>
+        <v>262189.14</v>
       </c>
       <c r="M6" s="4">
-        <v>135856.64000000001</v>
+        <v>262189.14</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>118069</v>
+        <v>110453</v>
       </c>
       <c r="B7" s="2">
         <v>2856</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="D7" s="11">
-        <v>46105</v>
+        <v>45600</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>50</v>
@@ -1263,80 +1263,80 @@
         <v>1</v>
       </c>
       <c r="G7" s="4">
-        <v>1582.52</v>
+        <v>1602.22</v>
       </c>
       <c r="H7" s="4">
-        <v>31354.39</v>
+        <v>45528.69</v>
       </c>
       <c r="I7" s="4">
-        <v>32936.910000000003</v>
+        <v>47130.91</v>
       </c>
       <c r="J7" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" s="4">
-        <v>1484.19</v>
+        <v>0</v>
       </c>
       <c r="L7" s="4">
-        <v>17883.650000000001</v>
+        <v>128210.4</v>
       </c>
       <c r="M7" s="4">
-        <v>19367.84</v>
+        <v>128210.4</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>100677</v>
+        <v>118069</v>
       </c>
       <c r="B8" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="D8" s="11">
-        <v>44999</v>
+        <v>46105</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F8" s="3">
+        <v>2</v>
+      </c>
+      <c r="G8" s="4">
+        <v>3249.59</v>
+      </c>
+      <c r="H8" s="4">
+        <v>31354.39</v>
+      </c>
+      <c r="I8" s="4">
+        <v>34603.980000000003</v>
+      </c>
+      <c r="J8" s="3">
         <v>1</v>
       </c>
-      <c r="G8" s="4">
-        <v>2646.37</v>
-      </c>
-      <c r="H8" s="4">
-        <v>25549.86</v>
-      </c>
-      <c r="I8" s="4">
-        <v>28196.23</v>
-      </c>
-      <c r="J8" s="3">
-        <v>0</v>
-      </c>
       <c r="K8" s="4">
-        <v>0</v>
+        <v>1484.19</v>
       </c>
       <c r="L8" s="4">
-        <v>12007.66</v>
+        <v>36221.39</v>
       </c>
       <c r="M8" s="4">
-        <v>12007.66</v>
+        <v>37705.58</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>114100</v>
+        <v>100677</v>
       </c>
       <c r="B9" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D9" s="11">
-        <v>45863</v>
+        <v>44999</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>50</v>
@@ -1345,13 +1345,13 @@
         <v>1</v>
       </c>
       <c r="G9" s="4">
-        <v>2455.46</v>
+        <v>-9557.41</v>
       </c>
       <c r="H9" s="4">
-        <v>21456.49</v>
+        <v>40200.800000000003</v>
       </c>
       <c r="I9" s="4">
-        <v>23911.95</v>
+        <v>30643.39</v>
       </c>
       <c r="J9" s="3">
         <v>0</v>
@@ -1360,24 +1360,24 @@
         <v>0</v>
       </c>
       <c r="L9" s="4">
-        <v>25302.33</v>
+        <v>12007.66</v>
       </c>
       <c r="M9" s="4">
-        <v>25302.33</v>
+        <v>12007.66</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>102825</v>
+        <v>114100</v>
       </c>
       <c r="B10" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D10" s="11">
-        <v>45117</v>
+        <v>45863</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>50</v>
@@ -1386,13 +1386,13 @@
         <v>1</v>
       </c>
       <c r="G10" s="4">
-        <v>1494.27</v>
+        <v>2455.46</v>
       </c>
       <c r="H10" s="4">
-        <v>21235.73</v>
+        <v>24472.14</v>
       </c>
       <c r="I10" s="4">
-        <v>22730</v>
+        <v>26927.599999999999</v>
       </c>
       <c r="J10" s="3">
         <v>0</v>
@@ -1401,39 +1401,39 @@
         <v>0</v>
       </c>
       <c r="L10" s="4">
-        <v>8829.19</v>
+        <v>25302.33</v>
       </c>
       <c r="M10" s="4">
-        <v>8829.19</v>
+        <v>25302.33</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>80925</v>
+        <v>80122</v>
       </c>
       <c r="B11" s="2">
         <v>2043</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D11" s="11">
-        <v>43439</v>
+        <v>43371</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F11" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" s="4">
-        <v>22698.89</v>
+        <v>0</v>
       </c>
       <c r="H11" s="4">
-        <v>0</v>
+        <v>24845.05</v>
       </c>
       <c r="I11" s="4">
-        <v>22698.89</v>
+        <v>24845.05</v>
       </c>
       <c r="J11" s="3">
         <v>0</v>
@@ -1442,24 +1442,24 @@
         <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>15382.81</v>
+        <v>141422.20000000001</v>
       </c>
       <c r="M11" s="4">
-        <v>15382.81</v>
+        <v>141422.20000000001</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>104750</v>
+        <v>102825</v>
       </c>
       <c r="B12" s="2">
         <v>2043</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D12" s="11">
-        <v>45236</v>
+        <v>45117</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>50</v>
@@ -1468,13 +1468,13 @@
         <v>1</v>
       </c>
       <c r="G12" s="4">
-        <v>1562.11</v>
+        <v>1494.27</v>
       </c>
       <c r="H12" s="4">
-        <v>16583.3</v>
+        <v>21235.73</v>
       </c>
       <c r="I12" s="4">
-        <v>18145.41</v>
+        <v>22730</v>
       </c>
       <c r="J12" s="3">
         <v>0</v>
@@ -1483,39 +1483,39 @@
         <v>0</v>
       </c>
       <c r="L12" s="4">
-        <v>26942.720000000001</v>
+        <v>8829.19</v>
       </c>
       <c r="M12" s="4">
-        <v>26942.720000000001</v>
+        <v>8829.19</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>115047</v>
+        <v>80925</v>
       </c>
       <c r="B13" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="D13" s="11">
-        <v>45944</v>
+        <v>43439</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F13" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" s="4">
-        <v>0</v>
+        <v>22698.89</v>
       </c>
       <c r="H13" s="4">
-        <v>9504.58</v>
+        <v>0</v>
       </c>
       <c r="I13" s="4">
-        <v>9504.58</v>
+        <v>22698.89</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1524,39 +1524,39 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>29704.73</v>
+        <v>15382.81</v>
       </c>
       <c r="M13" s="4">
-        <v>29704.73</v>
+        <v>15382.81</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>88234</v>
+        <v>104750</v>
       </c>
       <c r="B14" s="2">
         <v>2043</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D14" s="11">
-        <v>43794</v>
+        <v>45236</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F14" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" s="4">
-        <v>0</v>
+        <v>1562.11</v>
       </c>
       <c r="H14" s="4">
-        <v>7739.54</v>
+        <v>16583.3</v>
       </c>
       <c r="I14" s="4">
-        <v>7739.54</v>
+        <v>18145.41</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1565,27 +1565,27 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>11567.17</v>
+        <v>26942.720000000001</v>
       </c>
       <c r="M14" s="4">
-        <v>11567.17</v>
+        <v>26942.720000000001</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>117440</v>
+        <v>81618</v>
       </c>
       <c r="B15" s="2">
         <v>2043</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D15" s="11">
-        <v>46149</v>
+        <v>43447</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F15" s="3">
         <v>0</v>
@@ -1594,10 +1594,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="4">
-        <v>7572.39</v>
+        <v>15147.88</v>
       </c>
       <c r="I15" s="4">
-        <v>7572.39</v>
+        <v>15147.88</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1606,24 +1606,24 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>65236.3</v>
+        <v>0</v>
       </c>
       <c r="M15" s="4">
-        <v>65236.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>80122</v>
+        <v>107488</v>
       </c>
       <c r="B16" s="2">
         <v>2043</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="D16" s="11">
-        <v>43371</v>
+        <v>45440</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>50</v>
@@ -1635,10 +1635,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>6362.33</v>
+        <v>13902.02</v>
       </c>
       <c r="I16" s="4">
-        <v>6362.33</v>
+        <v>13902.02</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1647,24 +1647,24 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>151848.75</v>
+        <v>80200.98</v>
       </c>
       <c r="M16" s="4">
-        <v>151848.75</v>
+        <v>80200.98</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>104718</v>
+        <v>115047</v>
       </c>
       <c r="B17" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D17" s="11">
-        <v>45264</v>
+        <v>45944</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>50</v>
@@ -1676,10 +1676,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>5436.12</v>
+        <v>9504.58</v>
       </c>
       <c r="I17" s="4">
-        <v>5436.12</v>
+        <v>9504.58</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1688,24 +1688,24 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>94744.69</v>
+        <v>15766.03</v>
       </c>
       <c r="M17" s="4">
-        <v>94744.69</v>
+        <v>15766.03</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>47116</v>
+        <v>88234</v>
       </c>
       <c r="B18" s="2">
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="D18" s="11">
-        <v>44616</v>
+        <v>43794</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>50</v>
@@ -1717,36 +1717,36 @@
         <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>4896.25</v>
+        <v>7739.54</v>
       </c>
       <c r="I18" s="4">
-        <v>4896.25</v>
+        <v>7739.54</v>
       </c>
       <c r="J18" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" s="4">
-        <v>30484.55</v>
+        <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>61089.919999999998</v>
+        <v>11567.17</v>
       </c>
       <c r="M18" s="4">
-        <v>91574.47</v>
+        <v>11567.17</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>101640</v>
+        <v>117440</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>9</v>
+        <v>51</v>
       </c>
       <c r="D19" s="11">
-        <v>45104</v>
+        <v>46149</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>50</v>
@@ -1758,10 +1758,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>4745.09</v>
+        <v>7572.39</v>
       </c>
       <c r="I19" s="4">
-        <v>4745.09</v>
+        <v>7572.39</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1770,24 +1770,24 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>3222.89</v>
+        <v>65236.3</v>
       </c>
       <c r="M19" s="4">
-        <v>3222.89</v>
+        <v>65236.3</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>108404</v>
+        <v>110105</v>
       </c>
       <c r="B20" s="2">
         <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D20" s="11">
-        <v>45467</v>
+        <v>45560</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>50</v>
@@ -1799,10 +1799,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>3982.49</v>
+        <v>7482.55</v>
       </c>
       <c r="I20" s="4">
-        <v>3982.49</v>
+        <v>7482.55</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1811,24 +1811,24 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>14324.23</v>
+        <v>2087.15</v>
       </c>
       <c r="M20" s="4">
-        <v>14324.23</v>
+        <v>2087.15</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>107488</v>
+        <v>104343</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D21" s="11">
-        <v>45440</v>
+        <v>45201</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>50</v>
@@ -1840,10 +1840,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>3303.04</v>
+        <v>7287.22</v>
       </c>
       <c r="I21" s="4">
-        <v>3303.04</v>
+        <v>7287.22</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1852,27 +1852,27 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>90799.97</v>
+        <v>47705.86</v>
       </c>
       <c r="M21" s="4">
-        <v>90799.97</v>
+        <v>47705.86</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>106018</v>
+        <v>104718</v>
       </c>
       <c r="B22" s="2">
         <v>2043</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D22" s="11">
-        <v>45344</v>
+        <v>45264</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F22" s="3">
         <v>0</v>
@@ -1881,10 +1881,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>3116.45</v>
+        <v>7178.46</v>
       </c>
       <c r="I22" s="4">
-        <v>3116.45</v>
+        <v>7178.46</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1893,24 +1893,24 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>16834.04</v>
+        <v>93002.35</v>
       </c>
       <c r="M22" s="4">
-        <v>16834.04</v>
+        <v>93002.35</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>109998</v>
+        <v>108405</v>
       </c>
       <c r="B23" s="2">
         <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="D23" s="11">
-        <v>45596</v>
+        <v>45471</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>50</v>
@@ -1922,10 +1922,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>2974.66</v>
+        <v>5556.45</v>
       </c>
       <c r="I23" s="4">
-        <v>2974.66</v>
+        <v>5556.45</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1934,24 +1934,24 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>0</v>
+        <v>2506.6999999999998</v>
       </c>
       <c r="M23" s="4">
-        <v>0</v>
+        <v>2506.6999999999998</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>108405</v>
+        <v>101640</v>
       </c>
       <c r="B24" s="2">
         <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="D24" s="11">
-        <v>45471</v>
+        <v>45104</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>50</v>
@@ -1963,10 +1963,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>2506.6999999999998</v>
+        <v>4745.09</v>
       </c>
       <c r="I24" s="4">
-        <v>2506.6999999999998</v>
+        <v>4745.09</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1975,24 +1975,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>5556.45</v>
+        <v>3222.89</v>
       </c>
       <c r="M24" s="4">
-        <v>5556.45</v>
+        <v>3222.89</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>63441</v>
+        <v>108404</v>
       </c>
       <c r="B25" s="2">
-        <v>2511</v>
+        <v>2043</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="D25" s="11">
-        <v>44733</v>
+        <v>45467</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>50</v>
@@ -2004,10 +2004,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>1851.71</v>
+        <v>3982.49</v>
       </c>
       <c r="I25" s="4">
-        <v>1851.71</v>
+        <v>3982.49</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -2016,27 +2016,27 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>7406.83</v>
+        <v>14324.23</v>
       </c>
       <c r="M25" s="4">
-        <v>7406.83</v>
+        <v>14324.23</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>112083</v>
+        <v>95148</v>
       </c>
       <c r="B26" s="2">
         <v>2043</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="D26" s="11">
-        <v>45736</v>
+        <v>44916</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F26" s="3">
         <v>0</v>
@@ -2045,10 +2045,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>1805.68</v>
+        <v>3909.35</v>
       </c>
       <c r="I26" s="4">
-        <v>1805.68</v>
+        <v>3909.35</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2057,27 +2057,27 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>18056.810000000001</v>
+        <v>0</v>
       </c>
       <c r="M26" s="4">
-        <v>18056.810000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>65046</v>
+        <v>106018</v>
       </c>
       <c r="B27" s="2">
         <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D27" s="11">
-        <v>44763</v>
+        <v>45344</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F27" s="3">
         <v>0</v>
@@ -2086,10 +2086,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>1752.06</v>
+        <v>3337.31</v>
       </c>
       <c r="I27" s="4">
-        <v>1752.06</v>
+        <v>3337.31</v>
       </c>
       <c r="J27" s="3">
         <v>0</v>
@@ -2098,24 +2098,24 @@
         <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>14686.63</v>
+        <v>14325.13</v>
       </c>
       <c r="M27" s="4">
-        <v>14686.63</v>
+        <v>14325.13</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>105696</v>
+        <v>116060</v>
       </c>
       <c r="B28" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D28" s="11">
-        <v>45279</v>
+        <v>46010</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>50</v>
@@ -2127,10 +2127,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>1742.16</v>
+        <v>3206.92</v>
       </c>
       <c r="I28" s="4">
-        <v>1742.16</v>
+        <v>3206.92</v>
       </c>
       <c r="J28" s="3">
         <v>0</v>
@@ -2139,24 +2139,24 @@
         <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>85511.7</v>
+        <v>42207.32</v>
       </c>
       <c r="M28" s="4">
-        <v>85511.7</v>
+        <v>42207.32</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>114157</v>
+        <v>109998</v>
       </c>
       <c r="B29" s="2">
         <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="D29" s="11">
-        <v>45904</v>
+        <v>45596</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>50</v>
@@ -2168,10 +2168,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>1646.66</v>
+        <v>2974.66</v>
       </c>
       <c r="I29" s="4">
-        <v>1646.66</v>
+        <v>2974.66</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2180,24 +2180,24 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>62230.01</v>
+        <v>0</v>
       </c>
       <c r="M29" s="4">
-        <v>62230.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>115404</v>
+        <v>63441</v>
       </c>
       <c r="B30" s="2">
-        <v>2043</v>
+        <v>2511</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="D30" s="11">
-        <v>45986</v>
+        <v>44733</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>50</v>
@@ -2209,10 +2209,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>662.59</v>
+        <v>1851.71</v>
       </c>
       <c r="I30" s="4">
-        <v>662.59</v>
+        <v>1851.71</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2221,24 +2221,24 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>10490.07</v>
+        <v>7406.83</v>
       </c>
       <c r="M30" s="4">
-        <v>10490.07</v>
+        <v>7406.83</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>116883</v>
+        <v>112083</v>
       </c>
       <c r="B31" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="D31" s="11">
-        <v>46126</v>
+        <v>45736</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>50</v>
@@ -2250,10 +2250,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>0</v>
+        <v>1805.68</v>
       </c>
       <c r="I31" s="4">
-        <v>0</v>
+        <v>1805.68</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -2262,27 +2262,27 @@
         <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>85605.95</v>
+        <v>18056.810000000001</v>
       </c>
       <c r="M31" s="4">
-        <v>85605.95</v>
+        <v>18056.810000000001</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>116876</v>
+        <v>114431</v>
       </c>
       <c r="B32" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D32" s="11">
-        <v>46111</v>
+        <v>45930</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F32" s="3">
         <v>0</v>
@@ -2291,10 +2291,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>0</v>
+        <v>1752.06</v>
       </c>
       <c r="I32" s="4">
-        <v>0</v>
+        <v>1752.06</v>
       </c>
       <c r="J32" s="3">
         <v>0</v>
@@ -2303,24 +2303,24 @@
         <v>0</v>
       </c>
       <c r="L32" s="4">
-        <v>16255.46</v>
+        <v>18429.88</v>
       </c>
       <c r="M32" s="4">
-        <v>16255.46</v>
+        <v>18429.88</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>116060</v>
+        <v>65046</v>
       </c>
       <c r="B33" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="D33" s="11">
-        <v>46010</v>
+        <v>44763</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>50</v>
@@ -2332,10 +2332,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>0</v>
+        <v>1752.06</v>
       </c>
       <c r="I33" s="4">
-        <v>0</v>
+        <v>1752.06</v>
       </c>
       <c r="J33" s="3">
         <v>0</v>
@@ -2344,27 +2344,27 @@
         <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>45412.23</v>
+        <v>14686.63</v>
       </c>
       <c r="M33" s="4">
-        <v>45412.23</v>
+        <v>14686.63</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>114431</v>
+        <v>105696</v>
       </c>
       <c r="B34" s="2">
         <v>2043</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="D34" s="11">
-        <v>45930</v>
+        <v>45279</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F34" s="3">
         <v>0</v>
@@ -2373,10 +2373,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>0</v>
+        <v>1742.16</v>
       </c>
       <c r="I34" s="4">
-        <v>0</v>
+        <v>1742.16</v>
       </c>
       <c r="J34" s="3">
         <v>0</v>
@@ -2385,24 +2385,24 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>20181.939999999999</v>
+        <v>85511.7</v>
       </c>
       <c r="M34" s="4">
-        <v>20181.939999999999</v>
+        <v>85511.7</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>113450</v>
+        <v>114157</v>
       </c>
       <c r="B35" s="2">
         <v>2043</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="D35" s="11">
-        <v>45852</v>
+        <v>45904</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>50</v>
@@ -2414,10 +2414,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="4">
-        <v>0</v>
+        <v>1646.66</v>
       </c>
       <c r="I35" s="4">
-        <v>0</v>
+        <v>1646.66</v>
       </c>
       <c r="J35" s="3">
         <v>0</v>
@@ -2426,27 +2426,27 @@
         <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>3904.8</v>
+        <v>62230.01</v>
       </c>
       <c r="M35" s="4">
-        <v>3904.8</v>
+        <v>62230.01</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>113076</v>
+        <v>115404</v>
       </c>
       <c r="B36" s="2">
         <v>2043</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D36" s="11">
-        <v>45806</v>
+        <v>45986</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F36" s="3">
         <v>0</v>
@@ -2455,10 +2455,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="4">
-        <v>0</v>
+        <v>662.59</v>
       </c>
       <c r="I36" s="4">
-        <v>0</v>
+        <v>662.59</v>
       </c>
       <c r="J36" s="3">
         <v>0</v>
@@ -2467,24 +2467,24 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>4584.04</v>
+        <v>10490.07</v>
       </c>
       <c r="M36" s="4">
-        <v>4584.04</v>
+        <v>10490.07</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>112522</v>
+        <v>116883</v>
       </c>
       <c r="B37" s="2">
         <v>2856</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D37" s="11">
-        <v>45776</v>
+        <v>46126</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>50</v>
@@ -2508,24 +2508,24 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>4961.7299999999996</v>
+        <v>85605.95</v>
       </c>
       <c r="M37" s="4">
-        <v>4961.7299999999996</v>
+        <v>85605.95</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>111056</v>
+        <v>116876</v>
       </c>
       <c r="B38" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="D38" s="11">
-        <v>45639</v>
+        <v>46111</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>50</v>
@@ -2549,24 +2549,24 @@
         <v>0</v>
       </c>
       <c r="L38" s="4">
-        <v>10951.05</v>
+        <v>16255.46</v>
       </c>
       <c r="M38" s="4">
-        <v>10951.05</v>
+        <v>16255.46</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>110575</v>
+        <v>113450</v>
       </c>
       <c r="B39" s="2">
         <v>2043</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="D39" s="11">
-        <v>45583</v>
+        <v>45852</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>50</v>
@@ -2590,27 +2590,27 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>72331.92</v>
+        <v>3904.8</v>
       </c>
       <c r="M39" s="4">
-        <v>72331.92</v>
+        <v>3904.8</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>110105</v>
+        <v>113076</v>
       </c>
       <c r="B40" s="2">
         <v>2043</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D40" s="11">
-        <v>45560</v>
+        <v>45806</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F40" s="3">
         <v>0</v>
@@ -2631,24 +2631,24 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>9502.52</v>
+        <v>4584.04</v>
       </c>
       <c r="M40" s="4">
-        <v>9502.52</v>
+        <v>4584.04</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>109007</v>
+        <v>112522</v>
       </c>
       <c r="B41" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D41" s="11">
-        <v>45525</v>
+        <v>45776</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>50</v>
@@ -2672,24 +2672,24 @@
         <v>0</v>
       </c>
       <c r="L41" s="4">
-        <v>6211.67</v>
+        <v>4961.7299999999996</v>
       </c>
       <c r="M41" s="4">
-        <v>6211.67</v>
+        <v>4961.7299999999996</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>104343</v>
+        <v>111056</v>
       </c>
       <c r="B42" s="2">
         <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="D42" s="11">
-        <v>45201</v>
+        <v>45639</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>50</v>
@@ -2713,27 +2713,27 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>49471.7</v>
+        <v>10951.05</v>
       </c>
       <c r="M42" s="4">
-        <v>49471.7</v>
+        <v>10951.05</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>95148</v>
+        <v>110575</v>
       </c>
       <c r="B43" s="2">
         <v>2043</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D43" s="11">
-        <v>44916</v>
+        <v>45583</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F43" s="3">
         <v>0</v>
@@ -2754,24 +2754,24 @@
         <v>0</v>
       </c>
       <c r="L43" s="4">
-        <v>3909.3</v>
+        <v>72331.92</v>
       </c>
       <c r="M43" s="4">
-        <v>3909.3</v>
+        <v>72331.92</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>94156</v>
+        <v>109007</v>
       </c>
       <c r="B44" s="2">
         <v>2043</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D44" s="11">
-        <v>44159</v>
+        <v>45525</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>50</v>
@@ -2795,27 +2795,27 @@
         <v>0</v>
       </c>
       <c r="L44" s="4">
-        <v>7507.91</v>
+        <v>6211.67</v>
       </c>
       <c r="M44" s="4">
-        <v>7507.91</v>
+        <v>6211.67</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
-        <v>81618</v>
+        <v>94156</v>
       </c>
       <c r="B45" s="2">
         <v>2043</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D45" s="11">
-        <v>43447</v>
+        <v>44159</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F45" s="3">
         <v>0</v>
@@ -2836,10 +2836,10 @@
         <v>0</v>
       </c>
       <c r="L45" s="4">
-        <v>15147.88</v>
+        <v>7507.91</v>
       </c>
       <c r="M45" s="4">
-        <v>15147.88</v>
+        <v>7507.91</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
@@ -2933,7 +2933,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C46:M50">
-    <cfRule type="expression" dxfId="18" priority="29" stopIfTrue="1">
+    <cfRule type="expression" dxfId="18" priority="41" stopIfTrue="1">
       <formula>$S45=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-05-25 09:47)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6F0FEFD-CC0B-C148-9F9C-E2DC14C43D53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59A685E2-054D-954F-9A03-B73430EF0EB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="58">
   <si>
     <t>Asesor</t>
   </si>
@@ -204,6 +204,12 @@
   </si>
   <si>
     <t>5</t>
+  </si>
+  <si>
+    <t>GERARDO DANIEL BARAJAS TORRES</t>
+  </si>
+  <si>
+    <t>MARIA FERNANDA RIOS BERNAL</t>
   </si>
 </sst>
 </file>
@@ -1041,7 +1047,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46160</v>
+        <v>46163</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1163,31 +1169,31 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
-        <v>47116</v>
+        <v>80122</v>
       </c>
       <c r="B5" s="2">
         <v>2043</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D5" s="11">
-        <v>44616</v>
+        <v>43371</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F5" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5" s="4">
-        <v>32258.07</v>
+        <v>1985.9</v>
       </c>
       <c r="H5" s="4">
-        <v>21224.59</v>
+        <v>71320.72</v>
       </c>
       <c r="I5" s="4">
-        <v>53482.66</v>
+        <v>73306.62</v>
       </c>
       <c r="J5" s="3">
         <v>0</v>
@@ -1196,39 +1202,39 @@
         <v>0</v>
       </c>
       <c r="L5" s="4">
-        <v>61089.919999999998</v>
+        <v>141422.20000000001</v>
       </c>
       <c r="M5" s="4">
-        <v>61089.919999999998</v>
+        <v>141422.20000000001</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>87538</v>
+        <v>47116</v>
       </c>
       <c r="B6" s="2">
         <v>2043</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="D6" s="11">
-        <v>43731</v>
+        <v>44616</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F6" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G6" s="4">
-        <v>0</v>
+        <v>32258.07</v>
       </c>
       <c r="H6" s="4">
-        <v>48957.39</v>
+        <v>21224.59</v>
       </c>
       <c r="I6" s="4">
-        <v>48957.39</v>
+        <v>53482.66</v>
       </c>
       <c r="J6" s="3">
         <v>0</v>
@@ -1237,10 +1243,10 @@
         <v>0</v>
       </c>
       <c r="L6" s="4">
-        <v>262189.14</v>
+        <v>61089.919999999998</v>
       </c>
       <c r="M6" s="4">
-        <v>262189.14</v>
+        <v>61089.919999999998</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -1266,10 +1272,10 @@
         <v>1602.22</v>
       </c>
       <c r="H7" s="4">
-        <v>45528.69</v>
+        <v>49283.35</v>
       </c>
       <c r="I7" s="4">
-        <v>47130.91</v>
+        <v>50885.57</v>
       </c>
       <c r="J7" s="3">
         <v>0</v>
@@ -1286,98 +1292,98 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>118069</v>
+        <v>87538</v>
       </c>
       <c r="B8" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>53</v>
+        <v>3</v>
       </c>
       <c r="D8" s="11">
-        <v>46105</v>
+        <v>43731</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F8" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G8" s="4">
-        <v>3249.59</v>
+        <v>0</v>
       </c>
       <c r="H8" s="4">
-        <v>31354.39</v>
+        <v>48957.39</v>
       </c>
       <c r="I8" s="4">
-        <v>34603.980000000003</v>
+        <v>48957.39</v>
       </c>
       <c r="J8" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" s="4">
-        <v>1484.19</v>
+        <v>0</v>
       </c>
       <c r="L8" s="4">
-        <v>36221.39</v>
+        <v>262189.14</v>
       </c>
       <c r="M8" s="4">
-        <v>37705.58</v>
+        <v>262189.14</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>100677</v>
+        <v>118069</v>
       </c>
       <c r="B9" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="D9" s="11">
-        <v>44999</v>
+        <v>46105</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F9" s="3">
+        <v>2</v>
+      </c>
+      <c r="G9" s="4">
+        <v>3249.59</v>
+      </c>
+      <c r="H9" s="4">
+        <v>31354.39</v>
+      </c>
+      <c r="I9" s="4">
+        <v>34603.980000000003</v>
+      </c>
+      <c r="J9" s="3">
         <v>1</v>
       </c>
-      <c r="G9" s="4">
-        <v>-9557.41</v>
-      </c>
-      <c r="H9" s="4">
-        <v>40200.800000000003</v>
-      </c>
-      <c r="I9" s="4">
-        <v>30643.39</v>
-      </c>
-      <c r="J9" s="3">
-        <v>0</v>
-      </c>
       <c r="K9" s="4">
-        <v>0</v>
+        <v>1484.19</v>
       </c>
       <c r="L9" s="4">
-        <v>12007.66</v>
+        <v>36221.39</v>
       </c>
       <c r="M9" s="4">
-        <v>12007.66</v>
+        <v>37705.58</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>114100</v>
+        <v>100677</v>
       </c>
       <c r="B10" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D10" s="11">
-        <v>45863</v>
+        <v>44999</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>50</v>
@@ -1386,13 +1392,13 @@
         <v>1</v>
       </c>
       <c r="G10" s="4">
-        <v>2455.46</v>
+        <v>-9557.41</v>
       </c>
       <c r="H10" s="4">
-        <v>24472.14</v>
+        <v>41946.23</v>
       </c>
       <c r="I10" s="4">
-        <v>26927.599999999999</v>
+        <v>32388.82</v>
       </c>
       <c r="J10" s="3">
         <v>0</v>
@@ -1401,39 +1407,39 @@
         <v>0</v>
       </c>
       <c r="L10" s="4">
-        <v>25302.33</v>
+        <v>10262.23</v>
       </c>
       <c r="M10" s="4">
-        <v>25302.33</v>
+        <v>10262.23</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>80122</v>
+        <v>114100</v>
       </c>
       <c r="B11" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="D11" s="11">
-        <v>43371</v>
+        <v>45863</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F11" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" s="4">
-        <v>0</v>
+        <v>2455.46</v>
       </c>
       <c r="H11" s="4">
-        <v>24845.05</v>
+        <v>26614.68</v>
       </c>
       <c r="I11" s="4">
-        <v>24845.05</v>
+        <v>29070.14</v>
       </c>
       <c r="J11" s="3">
         <v>0</v>
@@ -1442,39 +1448,39 @@
         <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>141422.20000000001</v>
+        <v>23159.79</v>
       </c>
       <c r="M11" s="4">
-        <v>141422.20000000001</v>
+        <v>23159.79</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>102825</v>
+        <v>107488</v>
       </c>
       <c r="B12" s="2">
         <v>2043</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D12" s="11">
-        <v>45117</v>
+        <v>45440</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F12" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" s="4">
-        <v>1494.27</v>
+        <v>0</v>
       </c>
       <c r="H12" s="4">
-        <v>21235.73</v>
+        <v>22804.639999999999</v>
       </c>
       <c r="I12" s="4">
-        <v>22730</v>
+        <v>22804.639999999999</v>
       </c>
       <c r="J12" s="3">
         <v>0</v>
@@ -1483,24 +1489,24 @@
         <v>0</v>
       </c>
       <c r="L12" s="4">
-        <v>8829.19</v>
+        <v>71298.36</v>
       </c>
       <c r="M12" s="4">
-        <v>8829.19</v>
+        <v>71298.36</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>80925</v>
+        <v>102825</v>
       </c>
       <c r="B13" s="2">
         <v>2043</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>37</v>
+        <v>6</v>
       </c>
       <c r="D13" s="11">
-        <v>43439</v>
+        <v>45117</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>50</v>
@@ -1509,13 +1515,13 @@
         <v>1</v>
       </c>
       <c r="G13" s="4">
-        <v>22698.89</v>
+        <v>1494.27</v>
       </c>
       <c r="H13" s="4">
-        <v>0</v>
+        <v>21235.73</v>
       </c>
       <c r="I13" s="4">
-        <v>22698.89</v>
+        <v>22730</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1524,24 +1530,24 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>15382.81</v>
+        <v>8829.19</v>
       </c>
       <c r="M13" s="4">
-        <v>15382.81</v>
+        <v>8829.19</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>104750</v>
+        <v>80925</v>
       </c>
       <c r="B14" s="2">
         <v>2043</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="D14" s="11">
-        <v>45236</v>
+        <v>43439</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>50</v>
@@ -1550,13 +1556,13 @@
         <v>1</v>
       </c>
       <c r="G14" s="4">
-        <v>1562.11</v>
+        <v>22698.89</v>
       </c>
       <c r="H14" s="4">
-        <v>16583.3</v>
+        <v>0</v>
       </c>
       <c r="I14" s="4">
-        <v>18145.41</v>
+        <v>22698.89</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1565,39 +1571,39 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>26942.720000000001</v>
+        <v>15382.81</v>
       </c>
       <c r="M14" s="4">
-        <v>26942.720000000001</v>
+        <v>15382.81</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>81618</v>
+        <v>104750</v>
       </c>
       <c r="B15" s="2">
         <v>2043</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="D15" s="11">
-        <v>43447</v>
+        <v>45236</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F15" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" s="4">
-        <v>0</v>
+        <v>1562.11</v>
       </c>
       <c r="H15" s="4">
-        <v>15147.88</v>
+        <v>16583.3</v>
       </c>
       <c r="I15" s="4">
-        <v>15147.88</v>
+        <v>18145.41</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1606,24 +1612,24 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>0</v>
+        <v>26942.720000000001</v>
       </c>
       <c r="M15" s="4">
-        <v>0</v>
+        <v>26942.720000000001</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>107488</v>
+        <v>115047</v>
       </c>
       <c r="B16" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="D16" s="11">
-        <v>45440</v>
+        <v>45944</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>50</v>
@@ -1635,10 +1641,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>13902.02</v>
+        <v>16136.19</v>
       </c>
       <c r="I16" s="4">
-        <v>13902.02</v>
+        <v>16136.19</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1647,27 +1653,27 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>80200.98</v>
+        <v>9134.42</v>
       </c>
       <c r="M16" s="4">
-        <v>80200.98</v>
+        <v>9134.42</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>115047</v>
+        <v>81618</v>
       </c>
       <c r="B17" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="D17" s="11">
-        <v>45944</v>
+        <v>43447</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F17" s="3">
         <v>0</v>
@@ -1676,10 +1682,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>9504.58</v>
+        <v>15147.88</v>
       </c>
       <c r="I17" s="4">
-        <v>9504.58</v>
+        <v>15147.88</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1688,24 +1694,24 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>15766.03</v>
+        <v>0</v>
       </c>
       <c r="M17" s="4">
-        <v>15766.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>88234</v>
+        <v>117440</v>
       </c>
       <c r="B18" s="2">
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>11</v>
+        <v>51</v>
       </c>
       <c r="D18" s="11">
-        <v>43794</v>
+        <v>46149</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>50</v>
@@ -1717,10 +1723,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>7739.54</v>
+        <v>10579.65</v>
       </c>
       <c r="I18" s="4">
-        <v>7739.54</v>
+        <v>10579.65</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1729,24 +1735,24 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>11567.17</v>
+        <v>62229</v>
       </c>
       <c r="M18" s="4">
-        <v>11567.17</v>
+        <v>62229</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>117440</v>
+        <v>106018</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="D19" s="11">
-        <v>46149</v>
+        <v>45344</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>50</v>
@@ -1758,10 +1764,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>7572.39</v>
+        <v>9315.52</v>
       </c>
       <c r="I19" s="4">
-        <v>7572.39</v>
+        <v>9315.52</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1770,24 +1776,24 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>65236.3</v>
+        <v>11444.81</v>
       </c>
       <c r="M19" s="4">
-        <v>65236.3</v>
+        <v>11444.81</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>110105</v>
+        <v>114157</v>
       </c>
       <c r="B20" s="2">
         <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="D20" s="11">
-        <v>45560</v>
+        <v>45904</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>50</v>
@@ -1799,10 +1805,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>7482.55</v>
+        <v>8173.66</v>
       </c>
       <c r="I20" s="4">
-        <v>7482.55</v>
+        <v>8173.66</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1811,24 +1817,24 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>2087.15</v>
+        <v>55703</v>
       </c>
       <c r="M20" s="4">
-        <v>2087.15</v>
+        <v>55703</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>104343</v>
+        <v>88234</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="D21" s="11">
-        <v>45201</v>
+        <v>43794</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>50</v>
@@ -1840,10 +1846,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>7287.22</v>
+        <v>7739.54</v>
       </c>
       <c r="I21" s="4">
-        <v>7287.22</v>
+        <v>7739.54</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1852,24 +1858,24 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>47705.86</v>
+        <v>11567.17</v>
       </c>
       <c r="M21" s="4">
-        <v>47705.86</v>
+        <v>11567.17</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>104718</v>
+        <v>105696</v>
       </c>
       <c r="B22" s="2">
         <v>2043</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="D22" s="11">
-        <v>45264</v>
+        <v>45279</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>50</v>
@@ -1881,10 +1887,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>7178.46</v>
+        <v>7700.31</v>
       </c>
       <c r="I22" s="4">
-        <v>7178.46</v>
+        <v>7700.31</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1893,24 +1899,24 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>93002.35</v>
+        <v>80014.48</v>
       </c>
       <c r="M22" s="4">
-        <v>93002.35</v>
+        <v>80014.48</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>108405</v>
+        <v>110105</v>
       </c>
       <c r="B23" s="2">
         <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="D23" s="11">
-        <v>45471</v>
+        <v>45560</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>50</v>
@@ -1922,10 +1928,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>5556.45</v>
+        <v>7482.55</v>
       </c>
       <c r="I23" s="4">
-        <v>5556.45</v>
+        <v>7482.55</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1934,24 +1940,24 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>2506.6999999999998</v>
+        <v>2087.15</v>
       </c>
       <c r="M23" s="4">
-        <v>2506.6999999999998</v>
+        <v>2087.15</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>101640</v>
+        <v>104343</v>
       </c>
       <c r="B24" s="2">
         <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="D24" s="11">
-        <v>45104</v>
+        <v>45201</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>50</v>
@@ -1963,10 +1969,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>4745.09</v>
+        <v>7287.22</v>
       </c>
       <c r="I24" s="4">
-        <v>4745.09</v>
+        <v>7287.22</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1975,24 +1981,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>3222.89</v>
+        <v>47705.86</v>
       </c>
       <c r="M24" s="4">
-        <v>3222.89</v>
+        <v>47705.86</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>108404</v>
+        <v>104718</v>
       </c>
       <c r="B25" s="2">
         <v>2043</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D25" s="11">
-        <v>45467</v>
+        <v>45264</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>50</v>
@@ -2004,10 +2010,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>3982.49</v>
+        <v>7178.46</v>
       </c>
       <c r="I25" s="4">
-        <v>3982.49</v>
+        <v>7178.46</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -2016,27 +2022,27 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>14324.23</v>
+        <v>93002.35</v>
       </c>
       <c r="M25" s="4">
-        <v>14324.23</v>
+        <v>93002.35</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>95148</v>
+        <v>116060</v>
       </c>
       <c r="B26" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D26" s="11">
-        <v>44916</v>
+        <v>46010</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F26" s="3">
         <v>0</v>
@@ -2045,10 +2051,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>3909.35</v>
+        <v>6833.65</v>
       </c>
       <c r="I26" s="4">
-        <v>3909.35</v>
+        <v>6833.65</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2057,27 +2063,27 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>0</v>
+        <v>38580.589999999997</v>
       </c>
       <c r="M26" s="4">
-        <v>0</v>
+        <v>38580.589999999997</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>106018</v>
+        <v>108405</v>
       </c>
       <c r="B27" s="2">
         <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="D27" s="11">
-        <v>45344</v>
+        <v>45471</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F27" s="3">
         <v>0</v>
@@ -2086,10 +2092,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>3337.31</v>
+        <v>5556.45</v>
       </c>
       <c r="I27" s="4">
-        <v>3337.31</v>
+        <v>5556.45</v>
       </c>
       <c r="J27" s="3">
         <v>0</v>
@@ -2098,24 +2104,24 @@
         <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>14325.13</v>
+        <v>2506.6999999999998</v>
       </c>
       <c r="M27" s="4">
-        <v>14325.13</v>
+        <v>2506.6999999999998</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>116060</v>
+        <v>101640</v>
       </c>
       <c r="B28" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="D28" s="11">
-        <v>46010</v>
+        <v>45104</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>50</v>
@@ -2127,10 +2133,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>3206.92</v>
+        <v>4745.09</v>
       </c>
       <c r="I28" s="4">
-        <v>3206.92</v>
+        <v>4745.09</v>
       </c>
       <c r="J28" s="3">
         <v>0</v>
@@ -2139,24 +2145,24 @@
         <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>42207.32</v>
+        <v>3222.89</v>
       </c>
       <c r="M28" s="4">
-        <v>42207.32</v>
+        <v>3222.89</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>109998</v>
+        <v>108404</v>
       </c>
       <c r="B29" s="2">
         <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="D29" s="11">
-        <v>45596</v>
+        <v>45467</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>50</v>
@@ -2168,10 +2174,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>2974.66</v>
+        <v>3982.49</v>
       </c>
       <c r="I29" s="4">
-        <v>2974.66</v>
+        <v>3982.49</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2180,27 +2186,27 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>0</v>
+        <v>14324.23</v>
       </c>
       <c r="M29" s="4">
-        <v>0</v>
+        <v>14324.23</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>63441</v>
+        <v>95148</v>
       </c>
       <c r="B30" s="2">
-        <v>2511</v>
+        <v>2043</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D30" s="11">
-        <v>44733</v>
+        <v>44916</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F30" s="3">
         <v>0</v>
@@ -2209,10 +2215,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>1851.71</v>
+        <v>3909.35</v>
       </c>
       <c r="I30" s="4">
-        <v>1851.71</v>
+        <v>3909.35</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2221,27 +2227,27 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>7406.83</v>
+        <v>0</v>
       </c>
       <c r="M30" s="4">
-        <v>7406.83</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>112083</v>
+        <v>114431</v>
       </c>
       <c r="B31" s="2">
         <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="D31" s="11">
-        <v>45736</v>
+        <v>45930</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F31" s="3">
         <v>0</v>
@@ -2250,10 +2256,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>1805.68</v>
+        <v>3504.11</v>
       </c>
       <c r="I31" s="4">
-        <v>1805.68</v>
+        <v>3504.11</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -2262,27 +2268,27 @@
         <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>18056.810000000001</v>
+        <v>16677.830000000002</v>
       </c>
       <c r="M31" s="4">
-        <v>18056.810000000001</v>
+        <v>16677.830000000002</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>114431</v>
+        <v>109998</v>
       </c>
       <c r="B32" s="2">
         <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D32" s="11">
-        <v>45930</v>
+        <v>45596</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F32" s="3">
         <v>0</v>
@@ -2291,10 +2297,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>1752.06</v>
+        <v>2974.66</v>
       </c>
       <c r="I32" s="4">
-        <v>1752.06</v>
+        <v>2974.66</v>
       </c>
       <c r="J32" s="3">
         <v>0</v>
@@ -2303,24 +2309,24 @@
         <v>0</v>
       </c>
       <c r="L32" s="4">
-        <v>18429.88</v>
+        <v>0</v>
       </c>
       <c r="M32" s="4">
-        <v>18429.88</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>65046</v>
+        <v>94156</v>
       </c>
       <c r="B33" s="2">
         <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="D33" s="11">
-        <v>44763</v>
+        <v>44159</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>50</v>
@@ -2332,10 +2338,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>1752.06</v>
+        <v>2315.6999999999998</v>
       </c>
       <c r="I33" s="4">
-        <v>1752.06</v>
+        <v>2315.6999999999998</v>
       </c>
       <c r="J33" s="3">
         <v>0</v>
@@ -2344,24 +2350,24 @@
         <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>14686.63</v>
+        <v>5192.26</v>
       </c>
       <c r="M33" s="4">
-        <v>14686.63</v>
+        <v>5192.26</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>105696</v>
+        <v>63441</v>
       </c>
       <c r="B34" s="2">
-        <v>2043</v>
+        <v>2511</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="D34" s="11">
-        <v>45279</v>
+        <v>44733</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>50</v>
@@ -2373,10 +2379,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>1742.16</v>
+        <v>1851.71</v>
       </c>
       <c r="I34" s="4">
-        <v>1742.16</v>
+        <v>1851.71</v>
       </c>
       <c r="J34" s="3">
         <v>0</v>
@@ -2385,24 +2391,24 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>85511.7</v>
+        <v>7406.83</v>
       </c>
       <c r="M34" s="4">
-        <v>85511.7</v>
+        <v>7406.83</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>114157</v>
+        <v>116883</v>
       </c>
       <c r="B35" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D35" s="11">
-        <v>45904</v>
+        <v>46126</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>50</v>
@@ -2414,10 +2420,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="4">
-        <v>1646.66</v>
+        <v>1844.64</v>
       </c>
       <c r="I35" s="4">
-        <v>1646.66</v>
+        <v>1844.64</v>
       </c>
       <c r="J35" s="3">
         <v>0</v>
@@ -2426,24 +2432,24 @@
         <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>62230.01</v>
+        <v>83761.31</v>
       </c>
       <c r="M35" s="4">
-        <v>62230.01</v>
+        <v>83761.31</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>115404</v>
+        <v>112083</v>
       </c>
       <c r="B36" s="2">
         <v>2043</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>22</v>
+        <v>54</v>
       </c>
       <c r="D36" s="11">
-        <v>45986</v>
+        <v>45736</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>50</v>
@@ -2455,10 +2461,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="4">
-        <v>662.59</v>
+        <v>1805.68</v>
       </c>
       <c r="I36" s="4">
-        <v>662.59</v>
+        <v>1805.68</v>
       </c>
       <c r="J36" s="3">
         <v>0</v>
@@ -2467,24 +2473,24 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>10490.07</v>
+        <v>18056.810000000001</v>
       </c>
       <c r="M36" s="4">
-        <v>10490.07</v>
+        <v>18056.810000000001</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>116883</v>
+        <v>112522</v>
       </c>
       <c r="B37" s="2">
         <v>2856</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D37" s="11">
-        <v>46126</v>
+        <v>45776</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>50</v>
@@ -2496,10 +2502,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="4">
-        <v>0</v>
+        <v>1760.54</v>
       </c>
       <c r="I37" s="4">
-        <v>0</v>
+        <v>1760.54</v>
       </c>
       <c r="J37" s="3">
         <v>0</v>
@@ -2508,24 +2514,24 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>85605.95</v>
+        <v>3201.19</v>
       </c>
       <c r="M37" s="4">
-        <v>85605.95</v>
+        <v>3201.19</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>116876</v>
+        <v>65046</v>
       </c>
       <c r="B38" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D38" s="11">
-        <v>46111</v>
+        <v>44763</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>50</v>
@@ -2537,10 +2543,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="4">
-        <v>0</v>
+        <v>1752.06</v>
       </c>
       <c r="I38" s="4">
-        <v>0</v>
+        <v>1752.06</v>
       </c>
       <c r="J38" s="3">
         <v>0</v>
@@ -2549,27 +2555,27 @@
         <v>0</v>
       </c>
       <c r="L38" s="4">
-        <v>16255.46</v>
+        <v>14686.63</v>
       </c>
       <c r="M38" s="4">
-        <v>16255.46</v>
+        <v>14686.63</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>113450</v>
+        <v>116795</v>
       </c>
       <c r="B39" s="2">
         <v>2043</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
       <c r="D39" s="11">
-        <v>45852</v>
+        <v>46000</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F39" s="3">
         <v>0</v>
@@ -2578,10 +2584,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="4">
-        <v>0</v>
+        <v>1603.11</v>
       </c>
       <c r="I39" s="4">
-        <v>0</v>
+        <v>1603.11</v>
       </c>
       <c r="J39" s="3">
         <v>0</v>
@@ -2590,27 +2596,27 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>3904.8</v>
+        <v>0</v>
       </c>
       <c r="M39" s="4">
-        <v>3904.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>113076</v>
+        <v>115404</v>
       </c>
       <c r="B40" s="2">
         <v>2043</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D40" s="11">
-        <v>45806</v>
+        <v>45986</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F40" s="3">
         <v>0</v>
@@ -2619,10 +2625,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="4">
-        <v>0</v>
+        <v>662.59</v>
       </c>
       <c r="I40" s="4">
-        <v>0</v>
+        <v>662.59</v>
       </c>
       <c r="J40" s="3">
         <v>0</v>
@@ -2631,24 +2637,24 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>4584.04</v>
+        <v>10490.07</v>
       </c>
       <c r="M40" s="4">
-        <v>4584.04</v>
+        <v>10490.07</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>112522</v>
+        <v>116876</v>
       </c>
       <c r="B41" s="2">
         <v>2856</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D41" s="11">
-        <v>45776</v>
+        <v>46111</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>50</v>
@@ -2672,24 +2678,24 @@
         <v>0</v>
       </c>
       <c r="L41" s="4">
-        <v>4961.7299999999996</v>
+        <v>16255.46</v>
       </c>
       <c r="M41" s="4">
-        <v>4961.7299999999996</v>
+        <v>16255.46</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>111056</v>
+        <v>113450</v>
       </c>
       <c r="B42" s="2">
         <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D42" s="11">
-        <v>45639</v>
+        <v>45852</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>50</v>
@@ -2713,27 +2719,27 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>10951.05</v>
+        <v>3904.8</v>
       </c>
       <c r="M42" s="4">
-        <v>10951.05</v>
+        <v>3904.8</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>110575</v>
+        <v>113076</v>
       </c>
       <c r="B43" s="2">
         <v>2043</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D43" s="11">
-        <v>45583</v>
+        <v>45806</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F43" s="3">
         <v>0</v>
@@ -2754,24 +2760,24 @@
         <v>0</v>
       </c>
       <c r="L43" s="4">
-        <v>72331.92</v>
+        <v>4584.04</v>
       </c>
       <c r="M43" s="4">
-        <v>72331.92</v>
+        <v>4584.04</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>109007</v>
+        <v>111056</v>
       </c>
       <c r="B44" s="2">
         <v>2043</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="D44" s="11">
-        <v>45525</v>
+        <v>45639</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>50</v>
@@ -2795,24 +2801,24 @@
         <v>0</v>
       </c>
       <c r="L44" s="4">
-        <v>6211.67</v>
+        <v>10951.05</v>
       </c>
       <c r="M44" s="4">
-        <v>6211.67</v>
+        <v>10951.05</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
-        <v>94156</v>
+        <v>110575</v>
       </c>
       <c r="B45" s="2">
         <v>2043</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="D45" s="11">
-        <v>44159</v>
+        <v>45583</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>50</v>
@@ -2836,41 +2842,93 @@
         <v>0</v>
       </c>
       <c r="L45" s="4">
-        <v>7507.91</v>
+        <v>72331.92</v>
       </c>
       <c r="M45" s="4">
-        <v>7507.91</v>
+        <v>72331.92</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="11"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="3"/>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4"/>
-      <c r="I46" s="4"/>
-      <c r="J46" s="3"/>
-      <c r="K46" s="4"/>
-      <c r="L46" s="4"/>
-      <c r="M46" s="4"/>
+      <c r="A46" s="2">
+        <v>109007</v>
+      </c>
+      <c r="B46" s="2">
+        <v>2043</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D46" s="11">
+        <v>45525</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F46" s="3">
+        <v>0</v>
+      </c>
+      <c r="G46" s="4">
+        <v>0</v>
+      </c>
+      <c r="H46" s="4">
+        <v>0</v>
+      </c>
+      <c r="I46" s="4">
+        <v>0</v>
+      </c>
+      <c r="J46" s="3">
+        <v>0</v>
+      </c>
+      <c r="K46" s="4">
+        <v>0</v>
+      </c>
+      <c r="L46" s="4">
+        <v>6211.67</v>
+      </c>
+      <c r="M46" s="4">
+        <v>6211.67</v>
+      </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4"/>
-      <c r="I47" s="4"/>
-      <c r="J47" s="3"/>
-      <c r="K47" s="4"/>
-      <c r="L47" s="4"/>
-      <c r="M47" s="4"/>
+      <c r="A47" s="2">
+        <v>103982</v>
+      </c>
+      <c r="B47" s="2">
+        <v>2043</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D47" s="11">
+        <v>45216</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F47" s="3">
+        <v>0</v>
+      </c>
+      <c r="G47" s="4">
+        <v>0</v>
+      </c>
+      <c r="H47" s="4">
+        <v>0</v>
+      </c>
+      <c r="I47" s="4">
+        <v>0</v>
+      </c>
+      <c r="J47" s="3">
+        <v>1</v>
+      </c>
+      <c r="K47" s="4">
+        <v>32936.910000000003</v>
+      </c>
+      <c r="L47" s="4">
+        <v>0</v>
+      </c>
+      <c r="M47" s="4">
+        <v>32936.910000000003</v>
+      </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
@@ -2919,35 +2977,35 @@
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="A46:B50">
+  <conditionalFormatting sqref="A48:B50">
     <cfRule type="expression" dxfId="23" priority="13" stopIfTrue="1">
-      <formula>$S46=1</formula>
+      <formula>$S48=1</formula>
     </cfRule>
     <cfRule type="expression" dxfId="22" priority="14" stopIfTrue="1">
-      <formula>$S45=1</formula>
+      <formula>$S47=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C46:H50 K46:L50">
+  <conditionalFormatting sqref="C48:H50 K48:L50">
     <cfRule type="expression" dxfId="19" priority="18" stopIfTrue="1">
-      <formula>$S46=1</formula>
+      <formula>$S48=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C46:M50">
-    <cfRule type="expression" dxfId="18" priority="41" stopIfTrue="1">
-      <formula>$S45=1</formula>
+  <conditionalFormatting sqref="C48:M50">
+    <cfRule type="expression" dxfId="18" priority="53" stopIfTrue="1">
+      <formula>$S47=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I46:I50 M46:M50">
+  <conditionalFormatting sqref="I48:I50 M48:M50">
     <cfRule type="expression" dxfId="15" priority="20" stopIfTrue="1">
-      <formula>$S46=1</formula>
+      <formula>$S48=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J46:J50">
+  <conditionalFormatting sqref="J48:J50">
     <cfRule type="expression" dxfId="12" priority="16" stopIfTrue="1">
-      <formula>$S46=1</formula>
+      <formula>$S48=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A45 J5:J45">
+  <conditionalFormatting sqref="A5:A47 J5:J47">
     <cfRule type="expression" dxfId="11" priority="4" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
@@ -2955,7 +3013,7 @@
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:L45 C5:H45">
+  <conditionalFormatting sqref="K5:L47 C5:H47">
     <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
@@ -2963,7 +3021,7 @@
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I45 M5:M45">
+  <conditionalFormatting sqref="I5:I47 M5:M47">
     <cfRule type="expression" dxfId="7" priority="8" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
@@ -2991,7 +3049,7 @@
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B45">
+  <conditionalFormatting sqref="B5:B47">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-05-26 13:50)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59A685E2-054D-954F-9A03-B73430EF0EB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B9FA064-25C4-C84B-9507-90054B4E6E8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="59">
   <si>
     <t>Asesor</t>
   </si>
@@ -210,6 +210,9 @@
   </si>
   <si>
     <t>MARIA FERNANDA RIOS BERNAL</t>
+  </si>
+  <si>
+    <t>JOSE ANTEMIO OLIVA SANTOS</t>
   </si>
 </sst>
 </file>
@@ -1047,7 +1050,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46163</v>
+        <v>46167</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1143,28 +1146,28 @@
         <v>50</v>
       </c>
       <c r="F4" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G4" s="4">
-        <v>35163.03</v>
+        <v>41350.53</v>
       </c>
       <c r="H4" s="4">
-        <v>53587.79</v>
+        <v>123990.17</v>
       </c>
       <c r="I4" s="4">
-        <v>88750.82</v>
+        <v>165340.70000000001</v>
       </c>
       <c r="J4" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K4" s="4">
-        <v>102294.53</v>
+        <v>31360.93</v>
       </c>
       <c r="L4" s="4">
         <v>72521.25</v>
       </c>
       <c r="M4" s="4">
-        <v>174815.78</v>
+        <v>103882.18</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -1190,22 +1193,22 @@
         <v>1985.9</v>
       </c>
       <c r="H5" s="4">
-        <v>71320.72</v>
+        <v>67664.039999999994</v>
       </c>
       <c r="I5" s="4">
-        <v>73306.62</v>
+        <v>69649.94</v>
       </c>
       <c r="J5" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" s="4">
-        <v>0</v>
+        <v>22574.41</v>
       </c>
       <c r="L5" s="4">
         <v>141422.20000000001</v>
       </c>
       <c r="M5" s="4">
-        <v>141422.20000000001</v>
+        <v>163996.60999999999</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -1231,10 +1234,10 @@
         <v>32258.07</v>
       </c>
       <c r="H6" s="4">
-        <v>21224.59</v>
+        <v>28647.06</v>
       </c>
       <c r="I6" s="4">
-        <v>53482.66</v>
+        <v>60905.13</v>
       </c>
       <c r="J6" s="3">
         <v>0</v>
@@ -1243,39 +1246,39 @@
         <v>0</v>
       </c>
       <c r="L6" s="4">
-        <v>61089.919999999998</v>
+        <v>59360.72</v>
       </c>
       <c r="M6" s="4">
-        <v>61089.919999999998</v>
+        <v>59360.72</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>110453</v>
+        <v>87538</v>
       </c>
       <c r="B7" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D7" s="11">
-        <v>45600</v>
+        <v>43731</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F7" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" s="4">
-        <v>1602.22</v>
+        <v>0</v>
       </c>
       <c r="H7" s="4">
-        <v>49283.35</v>
+        <v>59212.9</v>
       </c>
       <c r="I7" s="4">
-        <v>50885.57</v>
+        <v>59212.9</v>
       </c>
       <c r="J7" s="3">
         <v>0</v>
@@ -1284,39 +1287,39 @@
         <v>0</v>
       </c>
       <c r="L7" s="4">
-        <v>128210.4</v>
+        <v>251933.62</v>
       </c>
       <c r="M7" s="4">
-        <v>128210.4</v>
+        <v>251933.62</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>87538</v>
+        <v>110453</v>
       </c>
       <c r="B8" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D8" s="11">
-        <v>43731</v>
+        <v>45600</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="4">
-        <v>0</v>
+        <v>1602.22</v>
       </c>
       <c r="H8" s="4">
-        <v>48957.39</v>
+        <v>54162.73</v>
       </c>
       <c r="I8" s="4">
-        <v>48957.39</v>
+        <v>55764.95</v>
       </c>
       <c r="J8" s="3">
         <v>0</v>
@@ -1325,10 +1328,10 @@
         <v>0</v>
       </c>
       <c r="L8" s="4">
-        <v>262189.14</v>
+        <v>123887.07</v>
       </c>
       <c r="M8" s="4">
-        <v>262189.14</v>
+        <v>123887.07</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -1374,16 +1377,16 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>100677</v>
+        <v>103982</v>
       </c>
       <c r="B10" s="2">
         <v>2043</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="D10" s="11">
-        <v>44999</v>
+        <v>45216</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>50</v>
@@ -1392,13 +1395,13 @@
         <v>1</v>
       </c>
       <c r="G10" s="4">
-        <v>-9557.41</v>
+        <v>1572.63</v>
       </c>
       <c r="H10" s="4">
-        <v>41946.23</v>
+        <v>31364.28</v>
       </c>
       <c r="I10" s="4">
-        <v>32388.82</v>
+        <v>32936.910000000003</v>
       </c>
       <c r="J10" s="3">
         <v>0</v>
@@ -1407,24 +1410,24 @@
         <v>0</v>
       </c>
       <c r="L10" s="4">
-        <v>10262.23</v>
+        <v>0</v>
       </c>
       <c r="M10" s="4">
-        <v>10262.23</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>114100</v>
+        <v>100677</v>
       </c>
       <c r="B11" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D11" s="11">
-        <v>45863</v>
+        <v>44999</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>50</v>
@@ -1433,13 +1436,13 @@
         <v>1</v>
       </c>
       <c r="G11" s="4">
-        <v>2455.46</v>
+        <v>-9557.41</v>
       </c>
       <c r="H11" s="4">
-        <v>26614.68</v>
+        <v>41946.23</v>
       </c>
       <c r="I11" s="4">
-        <v>29070.14</v>
+        <v>32388.82</v>
       </c>
       <c r="J11" s="3">
         <v>0</v>
@@ -1448,39 +1451,39 @@
         <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>23159.79</v>
+        <v>10262.23</v>
       </c>
       <c r="M11" s="4">
-        <v>23159.79</v>
+        <v>10262.23</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>107488</v>
+        <v>105696</v>
       </c>
       <c r="B12" s="2">
         <v>2043</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D12" s="11">
-        <v>45440</v>
+        <v>45279</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" s="4">
-        <v>0</v>
+        <v>24295.37</v>
       </c>
       <c r="H12" s="4">
-        <v>22804.639999999999</v>
+        <v>7700.31</v>
       </c>
       <c r="I12" s="4">
-        <v>22804.639999999999</v>
+        <v>31995.68</v>
       </c>
       <c r="J12" s="3">
         <v>0</v>
@@ -1489,24 +1492,24 @@
         <v>0</v>
       </c>
       <c r="L12" s="4">
-        <v>71298.36</v>
+        <v>80014.48</v>
       </c>
       <c r="M12" s="4">
-        <v>71298.36</v>
+        <v>80014.48</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>102825</v>
+        <v>114100</v>
       </c>
       <c r="B13" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D13" s="11">
-        <v>45117</v>
+        <v>45863</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>50</v>
@@ -1515,13 +1518,13 @@
         <v>1</v>
       </c>
       <c r="G13" s="4">
-        <v>1494.27</v>
+        <v>2455.46</v>
       </c>
       <c r="H13" s="4">
-        <v>21235.73</v>
+        <v>26614.68</v>
       </c>
       <c r="I13" s="4">
-        <v>22730</v>
+        <v>29070.14</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1530,10 +1533,10 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>8829.19</v>
+        <v>23159.79</v>
       </c>
       <c r="M13" s="4">
-        <v>8829.19</v>
+        <v>23159.79</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
@@ -1559,10 +1562,10 @@
         <v>22698.89</v>
       </c>
       <c r="H14" s="4">
-        <v>0</v>
+        <v>5178.6000000000004</v>
       </c>
       <c r="I14" s="4">
-        <v>22698.89</v>
+        <v>27877.49</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1571,10 +1574,10 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>15382.81</v>
+        <v>10866.76</v>
       </c>
       <c r="M14" s="4">
-        <v>15382.81</v>
+        <v>10866.76</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
@@ -1600,10 +1603,10 @@
         <v>1562.11</v>
       </c>
       <c r="H15" s="4">
-        <v>16583.3</v>
+        <v>22160.6</v>
       </c>
       <c r="I15" s="4">
-        <v>18145.41</v>
+        <v>23722.71</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1620,16 +1623,16 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>115047</v>
+        <v>107488</v>
       </c>
       <c r="B16" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="D16" s="11">
-        <v>45944</v>
+        <v>45440</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>50</v>
@@ -1641,10 +1644,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="4">
-        <v>16136.19</v>
+        <v>22804.639999999999</v>
       </c>
       <c r="I16" s="4">
-        <v>16136.19</v>
+        <v>22804.639999999999</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1653,39 +1656,39 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>9134.42</v>
+        <v>71298.36</v>
       </c>
       <c r="M16" s="4">
-        <v>9134.42</v>
+        <v>71298.36</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>81618</v>
+        <v>102825</v>
       </c>
       <c r="B17" s="2">
         <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="D17" s="11">
-        <v>43447</v>
+        <v>45117</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F17" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" s="4">
-        <v>0</v>
+        <v>1494.27</v>
       </c>
       <c r="H17" s="4">
-        <v>15147.88</v>
+        <v>21235.73</v>
       </c>
       <c r="I17" s="4">
-        <v>15147.88</v>
+        <v>22730</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1694,24 +1697,24 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>0</v>
+        <v>8829.19</v>
       </c>
       <c r="M17" s="4">
-        <v>0</v>
+        <v>8829.19</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>117440</v>
+        <v>115047</v>
       </c>
       <c r="B18" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="D18" s="11">
-        <v>46149</v>
+        <v>45944</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>50</v>
@@ -1723,10 +1726,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="4">
-        <v>10579.65</v>
+        <v>16136.19</v>
       </c>
       <c r="I18" s="4">
-        <v>10579.65</v>
+        <v>16136.19</v>
       </c>
       <c r="J18" s="3">
         <v>0</v>
@@ -1735,27 +1738,27 @@
         <v>0</v>
       </c>
       <c r="L18" s="4">
-        <v>62229</v>
+        <v>9134.42</v>
       </c>
       <c r="M18" s="4">
-        <v>62229</v>
+        <v>9134.42</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>106018</v>
+        <v>81618</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="D19" s="11">
-        <v>45344</v>
+        <v>43447</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F19" s="3">
         <v>0</v>
@@ -1764,10 +1767,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>9315.52</v>
+        <v>15147.88</v>
       </c>
       <c r="I19" s="4">
-        <v>9315.52</v>
+        <v>15147.88</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1776,24 +1779,24 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>11444.81</v>
+        <v>0</v>
       </c>
       <c r="M19" s="4">
-        <v>11444.81</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>114157</v>
+        <v>104343</v>
       </c>
       <c r="B20" s="2">
         <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D20" s="11">
-        <v>45904</v>
+        <v>45201</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>50</v>
@@ -1805,10 +1808,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>8173.66</v>
+        <v>13213.75</v>
       </c>
       <c r="I20" s="4">
-        <v>8173.66</v>
+        <v>13213.75</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1817,24 +1820,24 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>55703</v>
+        <v>41779.370000000003</v>
       </c>
       <c r="M20" s="4">
-        <v>55703</v>
+        <v>41779.370000000003</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>88234</v>
+        <v>117440</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>11</v>
+        <v>51</v>
       </c>
       <c r="D21" s="11">
-        <v>43794</v>
+        <v>46149</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>50</v>
@@ -1846,10 +1849,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>7739.54</v>
+        <v>10579.65</v>
       </c>
       <c r="I21" s="4">
-        <v>7739.54</v>
+        <v>10579.65</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1858,24 +1861,24 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>11567.17</v>
+        <v>62229</v>
       </c>
       <c r="M21" s="4">
-        <v>11567.17</v>
+        <v>62229</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>105696</v>
+        <v>104718</v>
       </c>
       <c r="B22" s="2">
         <v>2043</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="D22" s="11">
-        <v>45279</v>
+        <v>45264</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>50</v>
@@ -1887,10 +1890,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>7700.31</v>
+        <v>9656.7099999999991</v>
       </c>
       <c r="I22" s="4">
-        <v>7700.31</v>
+        <v>9656.7099999999991</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1899,24 +1902,24 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>80014.48</v>
+        <v>90524.08</v>
       </c>
       <c r="M22" s="4">
-        <v>80014.48</v>
+        <v>90524.08</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>110105</v>
+        <v>106018</v>
       </c>
       <c r="B23" s="2">
         <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="D23" s="11">
-        <v>45560</v>
+        <v>45344</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>50</v>
@@ -1928,10 +1931,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>7482.55</v>
+        <v>9315.52</v>
       </c>
       <c r="I23" s="4">
-        <v>7482.55</v>
+        <v>9315.52</v>
       </c>
       <c r="J23" s="3">
         <v>0</v>
@@ -1940,24 +1943,24 @@
         <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>2087.15</v>
+        <v>11444.81</v>
       </c>
       <c r="M23" s="4">
-        <v>2087.15</v>
+        <v>11444.81</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>104343</v>
+        <v>114157</v>
       </c>
       <c r="B24" s="2">
         <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D24" s="11">
-        <v>45201</v>
+        <v>45904</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>50</v>
@@ -1969,10 +1972,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>7287.22</v>
+        <v>8173.66</v>
       </c>
       <c r="I24" s="4">
-        <v>7287.22</v>
+        <v>8173.66</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1981,24 +1984,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>47705.86</v>
+        <v>55703</v>
       </c>
       <c r="M24" s="4">
-        <v>47705.86</v>
+        <v>55703</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>104718</v>
+        <v>88234</v>
       </c>
       <c r="B25" s="2">
         <v>2043</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D25" s="11">
-        <v>45264</v>
+        <v>43794</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>50</v>
@@ -2010,10 +2013,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>7178.46</v>
+        <v>7739.54</v>
       </c>
       <c r="I25" s="4">
-        <v>7178.46</v>
+        <v>7739.54</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -2022,24 +2025,24 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>93002.35</v>
+        <v>11567.17</v>
       </c>
       <c r="M25" s="4">
-        <v>93002.35</v>
+        <v>11567.17</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>116060</v>
+        <v>110105</v>
       </c>
       <c r="B26" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D26" s="11">
-        <v>46010</v>
+        <v>45560</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>50</v>
@@ -2051,10 +2054,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>6833.65</v>
+        <v>7482.55</v>
       </c>
       <c r="I26" s="4">
-        <v>6833.65</v>
+        <v>7482.55</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2063,24 +2066,24 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>38580.589999999997</v>
+        <v>2087.15</v>
       </c>
       <c r="M26" s="4">
-        <v>38580.589999999997</v>
+        <v>2087.15</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>108405</v>
+        <v>109007</v>
       </c>
       <c r="B27" s="2">
         <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="D27" s="11">
-        <v>45471</v>
+        <v>45525</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>50</v>
@@ -2092,10 +2095,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>5556.45</v>
+        <v>6933.13</v>
       </c>
       <c r="I27" s="4">
-        <v>5556.45</v>
+        <v>6933.13</v>
       </c>
       <c r="J27" s="3">
         <v>0</v>
@@ -2104,24 +2107,24 @@
         <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>2506.6999999999998</v>
+        <v>0</v>
       </c>
       <c r="M27" s="4">
-        <v>2506.6999999999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>101640</v>
+        <v>116060</v>
       </c>
       <c r="B28" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="D28" s="11">
-        <v>45104</v>
+        <v>46010</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>50</v>
@@ -2133,10 +2136,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>4745.09</v>
+        <v>6833.65</v>
       </c>
       <c r="I28" s="4">
-        <v>4745.09</v>
+        <v>6833.65</v>
       </c>
       <c r="J28" s="3">
         <v>0</v>
@@ -2145,24 +2148,24 @@
         <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>3222.89</v>
+        <v>38580.589999999997</v>
       </c>
       <c r="M28" s="4">
-        <v>3222.89</v>
+        <v>38580.589999999997</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>108404</v>
+        <v>108405</v>
       </c>
       <c r="B29" s="2">
         <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="D29" s="11">
-        <v>45467</v>
+        <v>45471</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>50</v>
@@ -2174,10 +2177,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>3982.49</v>
+        <v>5556.45</v>
       </c>
       <c r="I29" s="4">
-        <v>3982.49</v>
+        <v>5556.45</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2186,27 +2189,27 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>14324.23</v>
+        <v>2506.6999999999998</v>
       </c>
       <c r="M29" s="4">
-        <v>14324.23</v>
+        <v>2506.6999999999998</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>95148</v>
+        <v>113450</v>
       </c>
       <c r="B30" s="2">
         <v>2043</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="D30" s="11">
-        <v>44916</v>
+        <v>45852</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F30" s="3">
         <v>0</v>
@@ -2215,10 +2218,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>3909.35</v>
+        <v>4884.07</v>
       </c>
       <c r="I30" s="4">
-        <v>3909.35</v>
+        <v>4884.07</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2227,27 +2230,27 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>0</v>
+        <v>2603.1999999999998</v>
       </c>
       <c r="M30" s="4">
-        <v>0</v>
+        <v>2603.1999999999998</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>114431</v>
+        <v>101640</v>
       </c>
       <c r="B31" s="2">
         <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="D31" s="11">
-        <v>45930</v>
+        <v>45104</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F31" s="3">
         <v>0</v>
@@ -2256,10 +2259,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>3504.11</v>
+        <v>4745.09</v>
       </c>
       <c r="I31" s="4">
-        <v>3504.11</v>
+        <v>4745.09</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -2268,24 +2271,24 @@
         <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>16677.830000000002</v>
+        <v>3222.89</v>
       </c>
       <c r="M31" s="4">
-        <v>16677.830000000002</v>
+        <v>3222.89</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>109998</v>
+        <v>108404</v>
       </c>
       <c r="B32" s="2">
         <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="D32" s="11">
-        <v>45596</v>
+        <v>45467</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>50</v>
@@ -2297,10 +2300,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>2974.66</v>
+        <v>3982.49</v>
       </c>
       <c r="I32" s="4">
-        <v>2974.66</v>
+        <v>3982.49</v>
       </c>
       <c r="J32" s="3">
         <v>0</v>
@@ -2309,24 +2312,24 @@
         <v>0</v>
       </c>
       <c r="L32" s="4">
-        <v>0</v>
+        <v>14324.23</v>
       </c>
       <c r="M32" s="4">
-        <v>0</v>
+        <v>14324.23</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>94156</v>
+        <v>95148</v>
       </c>
       <c r="B33" s="2">
         <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D33" s="11">
-        <v>44159</v>
+        <v>44916</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>50</v>
@@ -2338,10 +2341,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>2315.6999999999998</v>
+        <v>3909.35</v>
       </c>
       <c r="I33" s="4">
-        <v>2315.6999999999998</v>
+        <v>3909.35</v>
       </c>
       <c r="J33" s="3">
         <v>0</v>
@@ -2350,27 +2353,27 @@
         <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>5192.26</v>
+        <v>0</v>
       </c>
       <c r="M33" s="4">
-        <v>5192.26</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>63441</v>
+        <v>114431</v>
       </c>
       <c r="B34" s="2">
-        <v>2511</v>
+        <v>2043</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="D34" s="11">
-        <v>44733</v>
+        <v>45930</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F34" s="3">
         <v>0</v>
@@ -2379,10 +2382,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>1851.71</v>
+        <v>3504.11</v>
       </c>
       <c r="I34" s="4">
-        <v>1851.71</v>
+        <v>3504.11</v>
       </c>
       <c r="J34" s="3">
         <v>0</v>
@@ -2391,24 +2394,24 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>7406.83</v>
+        <v>16677.830000000002</v>
       </c>
       <c r="M34" s="4">
-        <v>7406.83</v>
+        <v>16677.830000000002</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>116883</v>
+        <v>109998</v>
       </c>
       <c r="B35" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="D35" s="11">
-        <v>46126</v>
+        <v>45596</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>50</v>
@@ -2420,10 +2423,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="4">
-        <v>1844.64</v>
+        <v>2974.66</v>
       </c>
       <c r="I35" s="4">
-        <v>1844.64</v>
+        <v>2974.66</v>
       </c>
       <c r="J35" s="3">
         <v>0</v>
@@ -2432,24 +2435,24 @@
         <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>83761.31</v>
+        <v>0</v>
       </c>
       <c r="M35" s="4">
-        <v>83761.31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>112083</v>
+        <v>94156</v>
       </c>
       <c r="B36" s="2">
         <v>2043</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="D36" s="11">
-        <v>45736</v>
+        <v>44159</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>50</v>
@@ -2461,10 +2464,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="4">
-        <v>1805.68</v>
+        <v>2315.6999999999998</v>
       </c>
       <c r="I36" s="4">
-        <v>1805.68</v>
+        <v>2315.6999999999998</v>
       </c>
       <c r="J36" s="3">
         <v>0</v>
@@ -2473,24 +2476,24 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>18056.810000000001</v>
+        <v>5192.26</v>
       </c>
       <c r="M36" s="4">
-        <v>18056.810000000001</v>
+        <v>5192.26</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>112522</v>
+        <v>63441</v>
       </c>
       <c r="B37" s="2">
-        <v>2856</v>
+        <v>2511</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D37" s="11">
-        <v>45776</v>
+        <v>44733</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>50</v>
@@ -2502,10 +2505,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="4">
-        <v>1760.54</v>
+        <v>1851.71</v>
       </c>
       <c r="I37" s="4">
-        <v>1760.54</v>
+        <v>1851.71</v>
       </c>
       <c r="J37" s="3">
         <v>0</v>
@@ -2514,24 +2517,24 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>3201.19</v>
+        <v>7406.83</v>
       </c>
       <c r="M37" s="4">
-        <v>3201.19</v>
+        <v>7406.83</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>65046</v>
+        <v>116883</v>
       </c>
       <c r="B38" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D38" s="11">
-        <v>44763</v>
+        <v>46126</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>50</v>
@@ -2543,39 +2546,39 @@
         <v>0</v>
       </c>
       <c r="H38" s="4">
-        <v>1752.06</v>
+        <v>1844.64</v>
       </c>
       <c r="I38" s="4">
-        <v>1752.06</v>
+        <v>1844.64</v>
       </c>
       <c r="J38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K38" s="4">
-        <v>0</v>
+        <v>2001.98</v>
       </c>
       <c r="L38" s="4">
-        <v>14686.63</v>
+        <v>105783.12</v>
       </c>
       <c r="M38" s="4">
-        <v>14686.63</v>
+        <v>107785.1</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>116795</v>
+        <v>112083</v>
       </c>
       <c r="B39" s="2">
         <v>2043</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D39" s="11">
-        <v>46000</v>
+        <v>45736</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F39" s="3">
         <v>0</v>
@@ -2584,10 +2587,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="4">
-        <v>1603.11</v>
+        <v>1805.68</v>
       </c>
       <c r="I39" s="4">
-        <v>1603.11</v>
+        <v>1805.68</v>
       </c>
       <c r="J39" s="3">
         <v>0</v>
@@ -2596,24 +2599,24 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>0</v>
+        <v>18056.810000000001</v>
       </c>
       <c r="M39" s="4">
-        <v>0</v>
+        <v>18056.810000000001</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>115404</v>
+        <v>112522</v>
       </c>
       <c r="B40" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D40" s="11">
-        <v>45986</v>
+        <v>45776</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>50</v>
@@ -2625,10 +2628,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="4">
-        <v>662.59</v>
+        <v>1760.54</v>
       </c>
       <c r="I40" s="4">
-        <v>662.59</v>
+        <v>1760.54</v>
       </c>
       <c r="J40" s="3">
         <v>0</v>
@@ -2637,24 +2640,24 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>10490.07</v>
+        <v>3201.19</v>
       </c>
       <c r="M40" s="4">
-        <v>10490.07</v>
+        <v>3201.19</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>116876</v>
+        <v>65046</v>
       </c>
       <c r="B41" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D41" s="11">
-        <v>46111</v>
+        <v>44763</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>50</v>
@@ -2666,10 +2669,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="4">
-        <v>0</v>
+        <v>1752.06</v>
       </c>
       <c r="I41" s="4">
-        <v>0</v>
+        <v>1752.06</v>
       </c>
       <c r="J41" s="3">
         <v>0</v>
@@ -2678,27 +2681,27 @@
         <v>0</v>
       </c>
       <c r="L41" s="4">
-        <v>16255.46</v>
+        <v>14686.63</v>
       </c>
       <c r="M41" s="4">
-        <v>16255.46</v>
+        <v>14686.63</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>113450</v>
+        <v>116795</v>
       </c>
       <c r="B42" s="2">
         <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
       <c r="D42" s="11">
-        <v>45852</v>
+        <v>46000</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F42" s="3">
         <v>0</v>
@@ -2707,10 +2710,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="4">
-        <v>0</v>
+        <v>1603.11</v>
       </c>
       <c r="I42" s="4">
-        <v>0</v>
+        <v>1603.11</v>
       </c>
       <c r="J42" s="3">
         <v>0</v>
@@ -2719,27 +2722,27 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>3904.8</v>
+        <v>0</v>
       </c>
       <c r="M42" s="4">
-        <v>3904.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>113076</v>
+        <v>115404</v>
       </c>
       <c r="B43" s="2">
         <v>2043</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D43" s="11">
-        <v>45806</v>
+        <v>45986</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F43" s="3">
         <v>0</v>
@@ -2748,10 +2751,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="4">
-        <v>0</v>
+        <v>662.59</v>
       </c>
       <c r="I43" s="4">
-        <v>0</v>
+        <v>662.59</v>
       </c>
       <c r="J43" s="3">
         <v>0</v>
@@ -2760,24 +2763,24 @@
         <v>0</v>
       </c>
       <c r="L43" s="4">
-        <v>4584.04</v>
+        <v>10490.07</v>
       </c>
       <c r="M43" s="4">
-        <v>4584.04</v>
+        <v>10490.07</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>111056</v>
+        <v>118246</v>
       </c>
       <c r="B44" s="2">
         <v>2043</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>7</v>
+        <v>58</v>
       </c>
       <c r="D44" s="11">
-        <v>45639</v>
+        <v>46121</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>50</v>
@@ -2795,30 +2798,30 @@
         <v>0</v>
       </c>
       <c r="J44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K44" s="4">
-        <v>0</v>
+        <v>19016.41</v>
       </c>
       <c r="L44" s="4">
-        <v>10951.05</v>
+        <v>0</v>
       </c>
       <c r="M44" s="4">
-        <v>10951.05</v>
+        <v>19016.41</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
-        <v>110575</v>
+        <v>116876</v>
       </c>
       <c r="B45" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D45" s="11">
-        <v>45583</v>
+        <v>46111</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>50</v>
@@ -2842,27 +2845,27 @@
         <v>0</v>
       </c>
       <c r="L45" s="4">
-        <v>72331.92</v>
+        <v>16255.46</v>
       </c>
       <c r="M45" s="4">
-        <v>72331.92</v>
+        <v>16255.46</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
-        <v>109007</v>
+        <v>113076</v>
       </c>
       <c r="B46" s="2">
         <v>2043</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D46" s="11">
-        <v>45525</v>
+        <v>45806</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F46" s="3">
         <v>0</v>
@@ -2883,24 +2886,24 @@
         <v>0</v>
       </c>
       <c r="L46" s="4">
-        <v>6211.67</v>
+        <v>4584.04</v>
       </c>
       <c r="M46" s="4">
-        <v>6211.67</v>
+        <v>4584.04</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
-        <v>103982</v>
+        <v>111056</v>
       </c>
       <c r="B47" s="2">
         <v>2043</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="D47" s="11">
-        <v>45216</v>
+        <v>45639</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>50</v>
@@ -2918,32 +2921,58 @@
         <v>0</v>
       </c>
       <c r="J47" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K47" s="4">
-        <v>32936.910000000003</v>
+        <v>0</v>
       </c>
       <c r="L47" s="4">
-        <v>0</v>
+        <v>10951.05</v>
       </c>
       <c r="M47" s="4">
-        <v>32936.910000000003</v>
+        <v>10951.05</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="2"/>
-      <c r="F48" s="3"/>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-      <c r="I48" s="4"/>
-      <c r="J48" s="3"/>
-      <c r="K48" s="4"/>
-      <c r="L48" s="4"/>
-      <c r="M48" s="4"/>
+      <c r="A48" s="2">
+        <v>110575</v>
+      </c>
+      <c r="B48" s="2">
+        <v>2043</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D48" s="11">
+        <v>45583</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F48" s="3">
+        <v>0</v>
+      </c>
+      <c r="G48" s="4">
+        <v>0</v>
+      </c>
+      <c r="H48" s="4">
+        <v>0</v>
+      </c>
+      <c r="I48" s="4">
+        <v>0</v>
+      </c>
+      <c r="J48" s="3">
+        <v>0</v>
+      </c>
+      <c r="K48" s="4">
+        <v>0</v>
+      </c>
+      <c r="L48" s="4">
+        <v>72331.92</v>
+      </c>
+      <c r="M48" s="4">
+        <v>72331.92</v>
+      </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
@@ -2977,35 +3006,35 @@
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="A48:B50">
+  <conditionalFormatting sqref="A49:B50">
     <cfRule type="expression" dxfId="23" priority="13" stopIfTrue="1">
-      <formula>$S48=1</formula>
+      <formula>$S49=1</formula>
     </cfRule>
     <cfRule type="expression" dxfId="22" priority="14" stopIfTrue="1">
-      <formula>$S47=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C48:H50 K48:L50">
-    <cfRule type="expression" dxfId="19" priority="18" stopIfTrue="1">
       <formula>$S48=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C48:M50">
-    <cfRule type="expression" dxfId="18" priority="53" stopIfTrue="1">
-      <formula>$S47=1</formula>
+  <conditionalFormatting sqref="C49:H50 K49:L50">
+    <cfRule type="expression" dxfId="19" priority="18" stopIfTrue="1">
+      <formula>$S49=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I48:I50 M48:M50">
-    <cfRule type="expression" dxfId="15" priority="20" stopIfTrue="1">
+  <conditionalFormatting sqref="C49:M50">
+    <cfRule type="expression" dxfId="18" priority="65" stopIfTrue="1">
       <formula>$S48=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J48:J50">
-    <cfRule type="expression" dxfId="12" priority="16" stopIfTrue="1">
-      <formula>$S48=1</formula>
+  <conditionalFormatting sqref="I49:I50 M49:M50">
+    <cfRule type="expression" dxfId="15" priority="20" stopIfTrue="1">
+      <formula>$S49=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A47 J5:J47">
+  <conditionalFormatting sqref="J49:J50">
+    <cfRule type="expression" dxfId="12" priority="16" stopIfTrue="1">
+      <formula>$S49=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:A48 J5:J48">
     <cfRule type="expression" dxfId="11" priority="4" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
@@ -3013,7 +3042,7 @@
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:L47 C5:H47">
+  <conditionalFormatting sqref="K5:L48 C5:H48">
     <cfRule type="expression" dxfId="9" priority="6" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
@@ -3021,7 +3050,7 @@
       <formula>$S4=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I47 M5:M47">
+  <conditionalFormatting sqref="I5:I48 M5:M48">
     <cfRule type="expression" dxfId="7" priority="8" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>
@@ -3049,7 +3078,7 @@
       <formula>$S$34=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B47">
+  <conditionalFormatting sqref="B5:B48">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>$S5=1</formula>
     </cfRule>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-05-29 10:52)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B9FA064-25C4-C84B-9507-90054B4E6E8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{595C0D70-DCBA-A348-8BC9-0F7B09A757B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -1050,7 +1050,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46167</v>
+        <v>46169</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1152,10 +1152,10 @@
         <v>41350.53</v>
       </c>
       <c r="H4" s="4">
-        <v>123990.17</v>
+        <v>156748.19</v>
       </c>
       <c r="I4" s="4">
-        <v>165340.70000000001</v>
+        <v>198098.72</v>
       </c>
       <c r="J4" s="5">
         <v>1</v>
@@ -1187,57 +1187,57 @@
         <v>50</v>
       </c>
       <c r="F5" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" s="4">
-        <v>1985.9</v>
+        <v>24560.31</v>
       </c>
       <c r="H5" s="4">
         <v>67664.039999999994</v>
       </c>
       <c r="I5" s="4">
-        <v>69649.94</v>
+        <v>92224.35</v>
       </c>
       <c r="J5" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" s="4">
-        <v>22574.41</v>
+        <v>0</v>
       </c>
       <c r="L5" s="4">
         <v>141422.20000000001</v>
       </c>
       <c r="M5" s="4">
-        <v>163996.60999999999</v>
+        <v>141422.20000000001</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>47116</v>
+        <v>87538</v>
       </c>
       <c r="B6" s="2">
         <v>2043</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="D6" s="11">
-        <v>44616</v>
+        <v>43731</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F6" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G6" s="4">
-        <v>32258.07</v>
+        <v>0</v>
       </c>
       <c r="H6" s="4">
-        <v>28647.06</v>
+        <v>71500.17</v>
       </c>
       <c r="I6" s="4">
-        <v>60905.13</v>
+        <v>71500.17</v>
       </c>
       <c r="J6" s="3">
         <v>0</v>
@@ -1246,39 +1246,39 @@
         <v>0</v>
       </c>
       <c r="L6" s="4">
-        <v>59360.72</v>
+        <v>239646.38</v>
       </c>
       <c r="M6" s="4">
-        <v>59360.72</v>
+        <v>239646.38</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>87538</v>
+        <v>47116</v>
       </c>
       <c r="B7" s="2">
         <v>2043</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="D7" s="11">
-        <v>43731</v>
+        <v>44616</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F7" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G7" s="4">
-        <v>0</v>
+        <v>32258.07</v>
       </c>
       <c r="H7" s="4">
-        <v>59212.9</v>
+        <v>28647.06</v>
       </c>
       <c r="I7" s="4">
-        <v>59212.9</v>
+        <v>60905.13</v>
       </c>
       <c r="J7" s="3">
         <v>0</v>
@@ -1287,10 +1287,10 @@
         <v>0</v>
       </c>
       <c r="L7" s="4">
-        <v>251933.62</v>
+        <v>59360.72</v>
       </c>
       <c r="M7" s="4">
-        <v>251933.62</v>
+        <v>59360.72</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
@@ -1316,10 +1316,10 @@
         <v>1602.22</v>
       </c>
       <c r="H8" s="4">
-        <v>54162.73</v>
+        <v>58671.85</v>
       </c>
       <c r="I8" s="4">
-        <v>55764.95</v>
+        <v>60274.07</v>
       </c>
       <c r="J8" s="3">
         <v>0</v>
@@ -1328,10 +1328,10 @@
         <v>0</v>
       </c>
       <c r="L8" s="4">
-        <v>123887.07</v>
+        <v>121639.84</v>
       </c>
       <c r="M8" s="4">
-        <v>123887.07</v>
+        <v>121639.84</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -1351,16 +1351,16 @@
         <v>50</v>
       </c>
       <c r="F9" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G9" s="4">
-        <v>3249.59</v>
+        <v>4870.54</v>
       </c>
       <c r="H9" s="4">
-        <v>31354.39</v>
+        <v>45669.88</v>
       </c>
       <c r="I9" s="4">
-        <v>34603.980000000003</v>
+        <v>50540.42</v>
       </c>
       <c r="J9" s="3">
         <v>1</v>
@@ -1377,16 +1377,16 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>103982</v>
+        <v>115047</v>
       </c>
       <c r="B10" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>57</v>
+        <v>5</v>
       </c>
       <c r="D10" s="11">
-        <v>45216</v>
+        <v>45944</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>50</v>
@@ -1395,13 +1395,13 @@
         <v>1</v>
       </c>
       <c r="G10" s="4">
-        <v>1572.63</v>
+        <v>30532.25</v>
       </c>
       <c r="H10" s="4">
-        <v>31364.28</v>
+        <v>16136.19</v>
       </c>
       <c r="I10" s="4">
-        <v>32936.910000000003</v>
+        <v>46668.44</v>
       </c>
       <c r="J10" s="3">
         <v>0</v>
@@ -1410,24 +1410,24 @@
         <v>0</v>
       </c>
       <c r="L10" s="4">
-        <v>0</v>
+        <v>9134.42</v>
       </c>
       <c r="M10" s="4">
-        <v>0</v>
+        <v>9134.42</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>100677</v>
+        <v>105696</v>
       </c>
       <c r="B11" s="2">
         <v>2043</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D11" s="11">
-        <v>44999</v>
+        <v>45279</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>50</v>
@@ -1436,13 +1436,13 @@
         <v>1</v>
       </c>
       <c r="G11" s="4">
-        <v>-9557.41</v>
+        <v>24295.37</v>
       </c>
       <c r="H11" s="4">
-        <v>41946.23</v>
+        <v>11506.56</v>
       </c>
       <c r="I11" s="4">
-        <v>32388.82</v>
+        <v>35801.93</v>
       </c>
       <c r="J11" s="3">
         <v>0</v>
@@ -1451,24 +1451,24 @@
         <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>10262.23</v>
+        <v>76208.23</v>
       </c>
       <c r="M11" s="4">
-        <v>10262.23</v>
+        <v>76208.23</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>105696</v>
+        <v>103982</v>
       </c>
       <c r="B12" s="2">
         <v>2043</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="D12" s="11">
-        <v>45279</v>
+        <v>45216</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>50</v>
@@ -1477,39 +1477,39 @@
         <v>1</v>
       </c>
       <c r="G12" s="4">
-        <v>24295.37</v>
+        <v>1572.63</v>
       </c>
       <c r="H12" s="4">
-        <v>7700.31</v>
+        <v>31364.28</v>
       </c>
       <c r="I12" s="4">
-        <v>31995.68</v>
+        <v>32936.910000000003</v>
       </c>
       <c r="J12" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K12" s="4">
-        <v>0</v>
+        <v>9674.17</v>
       </c>
       <c r="L12" s="4">
-        <v>80014.48</v>
+        <v>0</v>
       </c>
       <c r="M12" s="4">
-        <v>80014.48</v>
+        <v>9674.17</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>114100</v>
+        <v>100677</v>
       </c>
       <c r="B13" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D13" s="11">
-        <v>45863</v>
+        <v>44999</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>50</v>
@@ -1518,13 +1518,13 @@
         <v>1</v>
       </c>
       <c r="G13" s="4">
-        <v>2455.46</v>
+        <v>-9557.41</v>
       </c>
       <c r="H13" s="4">
-        <v>26614.68</v>
+        <v>41946.23</v>
       </c>
       <c r="I13" s="4">
-        <v>29070.14</v>
+        <v>32388.82</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1533,24 +1533,24 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>23159.79</v>
+        <v>10262.23</v>
       </c>
       <c r="M13" s="4">
-        <v>23159.79</v>
+        <v>10262.23</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>80925</v>
+        <v>114100</v>
       </c>
       <c r="B14" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="D14" s="11">
-        <v>43439</v>
+        <v>45863</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>50</v>
@@ -1559,13 +1559,13 @@
         <v>1</v>
       </c>
       <c r="G14" s="4">
-        <v>22698.89</v>
+        <v>2455.46</v>
       </c>
       <c r="H14" s="4">
-        <v>5178.6000000000004</v>
+        <v>26614.68</v>
       </c>
       <c r="I14" s="4">
-        <v>27877.49</v>
+        <v>29070.14</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1574,24 +1574,24 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>10866.76</v>
+        <v>23159.79</v>
       </c>
       <c r="M14" s="4">
-        <v>10866.76</v>
+        <v>23159.79</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>104750</v>
+        <v>80925</v>
       </c>
       <c r="B15" s="2">
         <v>2043</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="D15" s="11">
-        <v>45236</v>
+        <v>43439</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>50</v>
@@ -1600,13 +1600,13 @@
         <v>1</v>
       </c>
       <c r="G15" s="4">
-        <v>1562.11</v>
+        <v>22698.89</v>
       </c>
       <c r="H15" s="4">
-        <v>22160.6</v>
+        <v>5178.6000000000004</v>
       </c>
       <c r="I15" s="4">
-        <v>23722.71</v>
+        <v>27877.49</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1615,39 +1615,39 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>26942.720000000001</v>
+        <v>10866.76</v>
       </c>
       <c r="M15" s="4">
-        <v>26942.720000000001</v>
+        <v>10866.76</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>107488</v>
+        <v>104750</v>
       </c>
       <c r="B16" s="2">
         <v>2043</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="D16" s="11">
-        <v>45440</v>
+        <v>45236</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F16" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="4">
-        <v>0</v>
+        <v>1562.11</v>
       </c>
       <c r="H16" s="4">
-        <v>22804.639999999999</v>
+        <v>22160.6</v>
       </c>
       <c r="I16" s="4">
-        <v>22804.639999999999</v>
+        <v>23722.71</v>
       </c>
       <c r="J16" s="3">
         <v>0</v>
@@ -1656,39 +1656,39 @@
         <v>0</v>
       </c>
       <c r="L16" s="4">
-        <v>71298.36</v>
+        <v>26942.720000000001</v>
       </c>
       <c r="M16" s="4">
-        <v>71298.36</v>
+        <v>26942.720000000001</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>102825</v>
+        <v>107488</v>
       </c>
       <c r="B17" s="2">
         <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D17" s="11">
-        <v>45117</v>
+        <v>45440</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F17" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" s="4">
-        <v>1494.27</v>
+        <v>0</v>
       </c>
       <c r="H17" s="4">
-        <v>21235.73</v>
+        <v>22804.639999999999</v>
       </c>
       <c r="I17" s="4">
-        <v>22730</v>
+        <v>22804.639999999999</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1697,80 +1697,80 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>8829.19</v>
+        <v>71298.36</v>
       </c>
       <c r="M17" s="4">
-        <v>8829.19</v>
+        <v>71298.36</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>115047</v>
+        <v>102825</v>
       </c>
       <c r="B18" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D18" s="11">
-        <v>45944</v>
+        <v>45117</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F18" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" s="4">
-        <v>0</v>
+        <v>1494.27</v>
       </c>
       <c r="H18" s="4">
-        <v>16136.19</v>
+        <v>21235.73</v>
       </c>
       <c r="I18" s="4">
-        <v>16136.19</v>
+        <v>22730</v>
       </c>
       <c r="J18" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" s="4">
-        <v>0</v>
+        <v>2520.35</v>
       </c>
       <c r="L18" s="4">
-        <v>9134.42</v>
+        <v>8829.19</v>
       </c>
       <c r="M18" s="4">
-        <v>9134.42</v>
+        <v>11349.54</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>81618</v>
+        <v>118246</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="D19" s="11">
-        <v>43447</v>
+        <v>46121</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" s="4">
-        <v>0</v>
+        <v>19016.41</v>
       </c>
       <c r="H19" s="4">
-        <v>15147.88</v>
+        <v>0</v>
       </c>
       <c r="I19" s="4">
-        <v>15147.88</v>
+        <v>19016.41</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1787,16 +1787,16 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>104343</v>
+        <v>104718</v>
       </c>
       <c r="B20" s="2">
         <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="D20" s="11">
-        <v>45201</v>
+        <v>45264</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>50</v>
@@ -1808,10 +1808,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="4">
-        <v>13213.75</v>
+        <v>15439.15</v>
       </c>
       <c r="I20" s="4">
-        <v>13213.75</v>
+        <v>15439.15</v>
       </c>
       <c r="J20" s="3">
         <v>0</v>
@@ -1820,27 +1820,27 @@
         <v>0</v>
       </c>
       <c r="L20" s="4">
-        <v>41779.370000000003</v>
+        <v>84741.64</v>
       </c>
       <c r="M20" s="4">
-        <v>41779.370000000003</v>
+        <v>84741.64</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>117440</v>
+        <v>81618</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D21" s="11">
-        <v>46149</v>
+        <v>43447</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F21" s="3">
         <v>0</v>
@@ -1849,10 +1849,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="4">
-        <v>10579.65</v>
+        <v>15147.88</v>
       </c>
       <c r="I21" s="4">
-        <v>10579.65</v>
+        <v>15147.88</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1861,24 +1861,24 @@
         <v>0</v>
       </c>
       <c r="L21" s="4">
-        <v>62229</v>
+        <v>0</v>
       </c>
       <c r="M21" s="4">
-        <v>62229</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>104718</v>
+        <v>104343</v>
       </c>
       <c r="B22" s="2">
         <v>2043</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D22" s="11">
-        <v>45264</v>
+        <v>45201</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>50</v>
@@ -1890,10 +1890,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>9656.7099999999991</v>
+        <v>13213.75</v>
       </c>
       <c r="I22" s="4">
-        <v>9656.7099999999991</v>
+        <v>13213.75</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1902,24 +1902,24 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>90524.08</v>
+        <v>38791.620000000003</v>
       </c>
       <c r="M22" s="4">
-        <v>90524.08</v>
+        <v>38791.620000000003</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>106018</v>
+        <v>117440</v>
       </c>
       <c r="B23" s="2">
         <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="D23" s="11">
-        <v>45344</v>
+        <v>46149</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>50</v>
@@ -1931,36 +1931,36 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>9315.52</v>
+        <v>10579.65</v>
       </c>
       <c r="I23" s="4">
-        <v>9315.52</v>
+        <v>10579.65</v>
       </c>
       <c r="J23" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" s="4">
-        <v>0</v>
+        <v>35696.19</v>
       </c>
       <c r="L23" s="4">
-        <v>11444.81</v>
+        <v>62229</v>
       </c>
       <c r="M23" s="4">
-        <v>11444.81</v>
+        <v>97925.19</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>114157</v>
+        <v>106018</v>
       </c>
       <c r="B24" s="2">
         <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D24" s="11">
-        <v>45904</v>
+        <v>45344</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>50</v>
@@ -1972,10 +1972,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>8173.66</v>
+        <v>9315.52</v>
       </c>
       <c r="I24" s="4">
-        <v>8173.66</v>
+        <v>9315.52</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1984,24 +1984,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>55703</v>
+        <v>11444.81</v>
       </c>
       <c r="M24" s="4">
-        <v>55703</v>
+        <v>11444.81</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>88234</v>
+        <v>114157</v>
       </c>
       <c r="B25" s="2">
         <v>2043</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D25" s="11">
-        <v>43794</v>
+        <v>45904</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>50</v>
@@ -2013,10 +2013,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>7739.54</v>
+        <v>8173.66</v>
       </c>
       <c r="I25" s="4">
-        <v>7739.54</v>
+        <v>8173.66</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -2025,24 +2025,24 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>11567.17</v>
+        <v>55703</v>
       </c>
       <c r="M25" s="4">
-        <v>11567.17</v>
+        <v>55703</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>110105</v>
+        <v>88234</v>
       </c>
       <c r="B26" s="2">
         <v>2043</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="D26" s="11">
-        <v>45560</v>
+        <v>43794</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>50</v>
@@ -2054,10 +2054,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>7482.55</v>
+        <v>7739.54</v>
       </c>
       <c r="I26" s="4">
-        <v>7482.55</v>
+        <v>7739.54</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2066,24 +2066,24 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>2087.15</v>
+        <v>11567.17</v>
       </c>
       <c r="M26" s="4">
-        <v>2087.15</v>
+        <v>11567.17</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>109007</v>
+        <v>110105</v>
       </c>
       <c r="B27" s="2">
         <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D27" s="11">
-        <v>45525</v>
+        <v>45560</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>50</v>
@@ -2095,10 +2095,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>6933.13</v>
+        <v>7482.55</v>
       </c>
       <c r="I27" s="4">
-        <v>6933.13</v>
+        <v>7482.55</v>
       </c>
       <c r="J27" s="3">
         <v>0</v>
@@ -2107,24 +2107,24 @@
         <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>0</v>
+        <v>2087.15</v>
       </c>
       <c r="M27" s="4">
-        <v>0</v>
+        <v>2087.15</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>116060</v>
+        <v>109007</v>
       </c>
       <c r="B28" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="D28" s="11">
-        <v>46010</v>
+        <v>45525</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>50</v>
@@ -2136,10 +2136,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>6833.65</v>
+        <v>6933.13</v>
       </c>
       <c r="I28" s="4">
-        <v>6833.65</v>
+        <v>6933.13</v>
       </c>
       <c r="J28" s="3">
         <v>0</v>
@@ -2148,24 +2148,24 @@
         <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>38580.589999999997</v>
+        <v>0</v>
       </c>
       <c r="M28" s="4">
-        <v>38580.589999999997</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>108405</v>
+        <v>116060</v>
       </c>
       <c r="B29" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="D29" s="11">
-        <v>45471</v>
+        <v>46010</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>50</v>
@@ -2177,10 +2177,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>5556.45</v>
+        <v>6833.65</v>
       </c>
       <c r="I29" s="4">
-        <v>5556.45</v>
+        <v>6833.65</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2189,39 +2189,39 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>2506.6999999999998</v>
+        <v>38580.589999999997</v>
       </c>
       <c r="M29" s="4">
-        <v>2506.6999999999998</v>
+        <v>38580.589999999997</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>113450</v>
+        <v>116883</v>
       </c>
       <c r="B30" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D30" s="11">
-        <v>45852</v>
+        <v>46126</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F30" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30" s="4">
-        <v>0</v>
+        <v>2001.98</v>
       </c>
       <c r="H30" s="4">
-        <v>4884.07</v>
+        <v>3590.07</v>
       </c>
       <c r="I30" s="4">
-        <v>4884.07</v>
+        <v>5592.05</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2230,24 +2230,24 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>2603.1999999999998</v>
+        <v>104037.69</v>
       </c>
       <c r="M30" s="4">
-        <v>2603.1999999999998</v>
+        <v>104037.69</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>101640</v>
+        <v>108405</v>
       </c>
       <c r="B31" s="2">
         <v>2043</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="D31" s="11">
-        <v>45104</v>
+        <v>45471</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>50</v>
@@ -2259,10 +2259,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>4745.09</v>
+        <v>5556.45</v>
       </c>
       <c r="I31" s="4">
-        <v>4745.09</v>
+        <v>5556.45</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -2271,24 +2271,24 @@
         <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>3222.89</v>
+        <v>2506.6999999999998</v>
       </c>
       <c r="M31" s="4">
-        <v>3222.89</v>
+        <v>2506.6999999999998</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>108404</v>
+        <v>113450</v>
       </c>
       <c r="B32" s="2">
         <v>2043</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D32" s="11">
-        <v>45467</v>
+        <v>45852</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>50</v>
@@ -2300,36 +2300,36 @@
         <v>0</v>
       </c>
       <c r="H32" s="4">
-        <v>3982.49</v>
+        <v>4884.07</v>
       </c>
       <c r="I32" s="4">
-        <v>3982.49</v>
+        <v>4884.07</v>
       </c>
       <c r="J32" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K32" s="4">
-        <v>0</v>
+        <v>45287.66</v>
       </c>
       <c r="L32" s="4">
-        <v>14324.23</v>
+        <v>2603.1999999999998</v>
       </c>
       <c r="M32" s="4">
-        <v>14324.23</v>
+        <v>47890.86</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>95148</v>
+        <v>101640</v>
       </c>
       <c r="B33" s="2">
         <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="D33" s="11">
-        <v>44916</v>
+        <v>45104</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>50</v>
@@ -2341,10 +2341,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>3909.35</v>
+        <v>4745.09</v>
       </c>
       <c r="I33" s="4">
-        <v>3909.35</v>
+        <v>4745.09</v>
       </c>
       <c r="J33" s="3">
         <v>0</v>
@@ -2353,27 +2353,27 @@
         <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>0</v>
+        <v>3222.89</v>
       </c>
       <c r="M33" s="4">
-        <v>0</v>
+        <v>3222.89</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>114431</v>
+        <v>108404</v>
       </c>
       <c r="B34" s="2">
         <v>2043</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="D34" s="11">
-        <v>45930</v>
+        <v>45467</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F34" s="3">
         <v>0</v>
@@ -2382,10 +2382,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>3504.11</v>
+        <v>3982.49</v>
       </c>
       <c r="I34" s="4">
-        <v>3504.11</v>
+        <v>3982.49</v>
       </c>
       <c r="J34" s="3">
         <v>0</v>
@@ -2394,24 +2394,24 @@
         <v>0</v>
       </c>
       <c r="L34" s="4">
-        <v>16677.830000000002</v>
+        <v>14324.23</v>
       </c>
       <c r="M34" s="4">
-        <v>16677.830000000002</v>
+        <v>14324.23</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>109998</v>
+        <v>95148</v>
       </c>
       <c r="B35" s="2">
         <v>2043</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D35" s="11">
-        <v>45596</v>
+        <v>44916</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>50</v>
@@ -2423,10 +2423,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="4">
-        <v>2974.66</v>
+        <v>3909.35</v>
       </c>
       <c r="I35" s="4">
-        <v>2974.66</v>
+        <v>3909.35</v>
       </c>
       <c r="J35" s="3">
         <v>0</v>
@@ -2443,16 +2443,16 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>94156</v>
+        <v>63441</v>
       </c>
       <c r="B36" s="2">
-        <v>2043</v>
+        <v>2511</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="D36" s="11">
-        <v>44159</v>
+        <v>44733</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>50</v>
@@ -2464,10 +2464,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="4">
-        <v>2315.6999999999998</v>
+        <v>3703.42</v>
       </c>
       <c r="I36" s="4">
-        <v>2315.6999999999998</v>
+        <v>3703.42</v>
       </c>
       <c r="J36" s="3">
         <v>0</v>
@@ -2476,27 +2476,27 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>5192.26</v>
+        <v>5555.13</v>
       </c>
       <c r="M36" s="4">
-        <v>5192.26</v>
+        <v>5555.13</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>63441</v>
+        <v>114431</v>
       </c>
       <c r="B37" s="2">
-        <v>2511</v>
+        <v>2043</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="D37" s="11">
-        <v>44733</v>
+        <v>45930</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F37" s="3">
         <v>0</v>
@@ -2505,10 +2505,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="4">
-        <v>1851.71</v>
+        <v>3504.11</v>
       </c>
       <c r="I37" s="4">
-        <v>1851.71</v>
+        <v>3504.11</v>
       </c>
       <c r="J37" s="3">
         <v>0</v>
@@ -2517,24 +2517,24 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>7406.83</v>
+        <v>16677.830000000002</v>
       </c>
       <c r="M37" s="4">
-        <v>7406.83</v>
+        <v>16677.830000000002</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>116883</v>
+        <v>109998</v>
       </c>
       <c r="B38" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="D38" s="11">
-        <v>46126</v>
+        <v>45596</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>50</v>
@@ -2546,36 +2546,36 @@
         <v>0</v>
       </c>
       <c r="H38" s="4">
-        <v>1844.64</v>
+        <v>2974.66</v>
       </c>
       <c r="I38" s="4">
-        <v>1844.64</v>
+        <v>2974.66</v>
       </c>
       <c r="J38" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K38" s="4">
-        <v>2001.98</v>
+        <v>0</v>
       </c>
       <c r="L38" s="4">
-        <v>105783.12</v>
+        <v>0</v>
       </c>
       <c r="M38" s="4">
-        <v>107785.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>112083</v>
+        <v>115404</v>
       </c>
       <c r="B39" s="2">
         <v>2043</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="D39" s="11">
-        <v>45736</v>
+        <v>45986</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>50</v>
@@ -2587,10 +2587,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="4">
-        <v>1805.68</v>
+        <v>2410.9299999999998</v>
       </c>
       <c r="I39" s="4">
-        <v>1805.68</v>
+        <v>2410.9299999999998</v>
       </c>
       <c r="J39" s="3">
         <v>0</v>
@@ -2599,24 +2599,24 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>18056.810000000001</v>
+        <v>8741.7199999999993</v>
       </c>
       <c r="M39" s="4">
-        <v>18056.810000000001</v>
+        <v>8741.7199999999993</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>112522</v>
+        <v>94156</v>
       </c>
       <c r="B40" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D40" s="11">
-        <v>45776</v>
+        <v>44159</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>50</v>
@@ -2628,10 +2628,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="4">
-        <v>1760.54</v>
+        <v>2315.6999999999998</v>
       </c>
       <c r="I40" s="4">
-        <v>1760.54</v>
+        <v>2315.6999999999998</v>
       </c>
       <c r="J40" s="3">
         <v>0</v>
@@ -2640,68 +2640,68 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>3201.19</v>
+        <v>5192.26</v>
       </c>
       <c r="M40" s="4">
-        <v>3201.19</v>
+        <v>5192.26</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>65046</v>
+        <v>116876</v>
       </c>
       <c r="B41" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D41" s="11">
-        <v>44763</v>
+        <v>46111</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G41" s="4">
-        <v>0</v>
+        <v>2065.86</v>
       </c>
       <c r="H41" s="4">
-        <v>1752.06</v>
+        <v>0</v>
       </c>
       <c r="I41" s="4">
-        <v>1752.06</v>
+        <v>2065.86</v>
       </c>
       <c r="J41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K41" s="4">
-        <v>0</v>
+        <v>18844.310000000001</v>
       </c>
       <c r="L41" s="4">
-        <v>14686.63</v>
+        <v>57824.19</v>
       </c>
       <c r="M41" s="4">
-        <v>14686.63</v>
+        <v>76668.5</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>116795</v>
+        <v>112083</v>
       </c>
       <c r="B42" s="2">
         <v>2043</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D42" s="11">
-        <v>46000</v>
+        <v>45736</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F42" s="3">
         <v>0</v>
@@ -2710,10 +2710,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="4">
-        <v>1603.11</v>
+        <v>1805.68</v>
       </c>
       <c r="I42" s="4">
-        <v>1603.11</v>
+        <v>1805.68</v>
       </c>
       <c r="J42" s="3">
         <v>0</v>
@@ -2722,24 +2722,24 @@
         <v>0</v>
       </c>
       <c r="L42" s="4">
-        <v>0</v>
+        <v>18056.810000000001</v>
       </c>
       <c r="M42" s="4">
-        <v>0</v>
+        <v>18056.810000000001</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>115404</v>
+        <v>112522</v>
       </c>
       <c r="B43" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D43" s="11">
-        <v>45986</v>
+        <v>45776</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>50</v>
@@ -2751,10 +2751,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="4">
-        <v>662.59</v>
+        <v>1760.54</v>
       </c>
       <c r="I43" s="4">
-        <v>662.59</v>
+        <v>1760.54</v>
       </c>
       <c r="J43" s="3">
         <v>0</v>
@@ -2763,24 +2763,24 @@
         <v>0</v>
       </c>
       <c r="L43" s="4">
-        <v>10490.07</v>
+        <v>3201.19</v>
       </c>
       <c r="M43" s="4">
-        <v>10490.07</v>
+        <v>3201.19</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>118246</v>
+        <v>65046</v>
       </c>
       <c r="B44" s="2">
         <v>2043</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="D44" s="11">
-        <v>46121</v>
+        <v>44763</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>50</v>
@@ -2792,39 +2792,39 @@
         <v>0</v>
       </c>
       <c r="H44" s="4">
-        <v>0</v>
+        <v>1752.06</v>
       </c>
       <c r="I44" s="4">
-        <v>0</v>
+        <v>1752.06</v>
       </c>
       <c r="J44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K44" s="4">
-        <v>19016.41</v>
+        <v>0</v>
       </c>
       <c r="L44" s="4">
-        <v>0</v>
+        <v>14686.63</v>
       </c>
       <c r="M44" s="4">
-        <v>19016.41</v>
+        <v>14686.63</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
-        <v>116876</v>
+        <v>116795</v>
       </c>
       <c r="B45" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="D45" s="11">
-        <v>46111</v>
+        <v>46000</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F45" s="3">
         <v>0</v>
@@ -2833,10 +2833,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="4">
-        <v>0</v>
+        <v>1603.11</v>
       </c>
       <c r="I45" s="4">
-        <v>0</v>
+        <v>1603.11</v>
       </c>
       <c r="J45" s="3">
         <v>0</v>
@@ -2845,10 +2845,10 @@
         <v>0</v>
       </c>
       <c r="L45" s="4">
-        <v>16255.46</v>
+        <v>0</v>
       </c>
       <c r="M45" s="4">
-        <v>16255.46</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
@@ -3020,7 +3020,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C49:M50">
-    <cfRule type="expression" dxfId="18" priority="65" stopIfTrue="1">
+    <cfRule type="expression" dxfId="18" priority="77" stopIfTrue="1">
       <formula>$S48=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-06-01 17:16)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/pagado_emitidido/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{595C0D70-DCBA-A348-8BC9-0F7B09A757B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF2E9844-CC63-474D-B32E-91CB327D8055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{0B03E385-4D70-1443-97FA-03D8B48AE23F}"/>
   </bookViews>
@@ -1050,7 +1050,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="7">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
@@ -1336,98 +1336,98 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>118069</v>
+        <v>117440</v>
       </c>
       <c r="B9" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D9" s="11">
-        <v>46105</v>
+        <v>46149</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F9" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G9" s="4">
-        <v>4870.54</v>
+        <v>1644.72</v>
       </c>
       <c r="H9" s="4">
-        <v>45669.88</v>
+        <v>52541.25</v>
       </c>
       <c r="I9" s="4">
-        <v>50540.42</v>
+        <v>54185.97</v>
       </c>
       <c r="J9" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" s="4">
-        <v>1484.19</v>
+        <v>0</v>
       </c>
       <c r="L9" s="4">
-        <v>36221.39</v>
+        <v>54318.84</v>
       </c>
       <c r="M9" s="4">
-        <v>37705.58</v>
+        <v>54318.84</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>115047</v>
+        <v>118069</v>
       </c>
       <c r="B10" s="2">
         <v>2856</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="D10" s="11">
-        <v>45944</v>
+        <v>46105</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F10" s="3">
+        <v>3</v>
+      </c>
+      <c r="G10" s="4">
+        <v>4870.54</v>
+      </c>
+      <c r="H10" s="4">
+        <v>47458.25</v>
+      </c>
+      <c r="I10" s="4">
+        <v>52328.79</v>
+      </c>
+      <c r="J10" s="3">
         <v>1</v>
       </c>
-      <c r="G10" s="4">
-        <v>30532.25</v>
-      </c>
-      <c r="H10" s="4">
-        <v>16136.19</v>
-      </c>
-      <c r="I10" s="4">
-        <v>46668.44</v>
-      </c>
-      <c r="J10" s="3">
-        <v>0</v>
-      </c>
       <c r="K10" s="4">
-        <v>0</v>
+        <v>1484.19</v>
       </c>
       <c r="L10" s="4">
-        <v>9134.42</v>
+        <v>34433.03</v>
       </c>
       <c r="M10" s="4">
-        <v>9134.42</v>
+        <v>35917.22</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>105696</v>
+        <v>115047</v>
       </c>
       <c r="B11" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="D11" s="11">
-        <v>45279</v>
+        <v>45944</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>50</v>
@@ -1436,13 +1436,13 @@
         <v>1</v>
       </c>
       <c r="G11" s="4">
-        <v>24295.37</v>
+        <v>30532.25</v>
       </c>
       <c r="H11" s="4">
-        <v>11506.56</v>
+        <v>16136.19</v>
       </c>
       <c r="I11" s="4">
-        <v>35801.93</v>
+        <v>46668.44</v>
       </c>
       <c r="J11" s="3">
         <v>0</v>
@@ -1451,10 +1451,10 @@
         <v>0</v>
       </c>
       <c r="L11" s="4">
-        <v>76208.23</v>
+        <v>9134.42</v>
       </c>
       <c r="M11" s="4">
-        <v>76208.23</v>
+        <v>9134.42</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
@@ -1474,42 +1474,42 @@
         <v>50</v>
       </c>
       <c r="F12" s="3">
+        <v>2</v>
+      </c>
+      <c r="G12" s="4">
+        <v>5032.57</v>
+      </c>
+      <c r="H12" s="4">
+        <v>33981.760000000002</v>
+      </c>
+      <c r="I12" s="4">
+        <v>39014.33</v>
+      </c>
+      <c r="J12" s="3">
         <v>1</v>
       </c>
-      <c r="G12" s="4">
-        <v>1572.63</v>
-      </c>
-      <c r="H12" s="4">
-        <v>31364.28</v>
-      </c>
-      <c r="I12" s="4">
-        <v>32936.910000000003</v>
-      </c>
-      <c r="J12" s="3">
-        <v>2</v>
-      </c>
       <c r="K12" s="4">
-        <v>9674.17</v>
+        <v>3596.79</v>
       </c>
       <c r="L12" s="4">
         <v>0</v>
       </c>
       <c r="M12" s="4">
-        <v>9674.17</v>
+        <v>3596.79</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>100677</v>
+        <v>105696</v>
       </c>
       <c r="B13" s="2">
         <v>2043</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D13" s="11">
-        <v>44999</v>
+        <v>45279</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>50</v>
@@ -1518,13 +1518,13 @@
         <v>1</v>
       </c>
       <c r="G13" s="4">
-        <v>-9557.41</v>
+        <v>24295.37</v>
       </c>
       <c r="H13" s="4">
-        <v>41946.23</v>
+        <v>11506.56</v>
       </c>
       <c r="I13" s="4">
-        <v>32388.82</v>
+        <v>35801.93</v>
       </c>
       <c r="J13" s="3">
         <v>0</v>
@@ -1533,24 +1533,24 @@
         <v>0</v>
       </c>
       <c r="L13" s="4">
-        <v>10262.23</v>
+        <v>76208.23</v>
       </c>
       <c r="M13" s="4">
-        <v>10262.23</v>
+        <v>76208.23</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>114100</v>
+        <v>100677</v>
       </c>
       <c r="B14" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D14" s="11">
-        <v>45863</v>
+        <v>44999</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>50</v>
@@ -1559,13 +1559,13 @@
         <v>1</v>
       </c>
       <c r="G14" s="4">
-        <v>2455.46</v>
+        <v>-9557.41</v>
       </c>
       <c r="H14" s="4">
-        <v>26614.68</v>
+        <v>41946.23</v>
       </c>
       <c r="I14" s="4">
-        <v>29070.14</v>
+        <v>32388.82</v>
       </c>
       <c r="J14" s="3">
         <v>0</v>
@@ -1574,24 +1574,24 @@
         <v>0</v>
       </c>
       <c r="L14" s="4">
-        <v>23159.79</v>
+        <v>10262.23</v>
       </c>
       <c r="M14" s="4">
-        <v>23159.79</v>
+        <v>10262.23</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>80925</v>
+        <v>114100</v>
       </c>
       <c r="B15" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="D15" s="11">
-        <v>43439</v>
+        <v>45863</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>50</v>
@@ -1600,13 +1600,13 @@
         <v>1</v>
       </c>
       <c r="G15" s="4">
-        <v>22698.89</v>
+        <v>2455.46</v>
       </c>
       <c r="H15" s="4">
-        <v>5178.6000000000004</v>
+        <v>26614.68</v>
       </c>
       <c r="I15" s="4">
-        <v>27877.49</v>
+        <v>29070.14</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
@@ -1615,24 +1615,24 @@
         <v>0</v>
       </c>
       <c r="L15" s="4">
-        <v>10866.76</v>
+        <v>23159.79</v>
       </c>
       <c r="M15" s="4">
-        <v>10866.76</v>
+        <v>23159.79</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>104750</v>
+        <v>80925</v>
       </c>
       <c r="B16" s="2">
         <v>2043</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="D16" s="11">
-        <v>45236</v>
+        <v>43439</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>50</v>
@@ -1641,54 +1641,54 @@
         <v>1</v>
       </c>
       <c r="G16" s="4">
-        <v>1562.11</v>
+        <v>22698.89</v>
       </c>
       <c r="H16" s="4">
-        <v>22160.6</v>
+        <v>5178.6000000000004</v>
       </c>
       <c r="I16" s="4">
-        <v>23722.71</v>
+        <v>27877.49</v>
       </c>
       <c r="J16" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" s="4">
-        <v>0</v>
+        <v>2997.01</v>
       </c>
       <c r="L16" s="4">
-        <v>26942.720000000001</v>
+        <v>5187.6099999999997</v>
       </c>
       <c r="M16" s="4">
-        <v>26942.720000000001</v>
+        <v>8184.62</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>107488</v>
+        <v>104750</v>
       </c>
       <c r="B17" s="2">
         <v>2043</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="D17" s="11">
-        <v>45440</v>
+        <v>45236</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F17" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" s="4">
-        <v>0</v>
+        <v>1562.11</v>
       </c>
       <c r="H17" s="4">
-        <v>22804.639999999999</v>
+        <v>22160.6</v>
       </c>
       <c r="I17" s="4">
-        <v>22804.639999999999</v>
+        <v>23722.71</v>
       </c>
       <c r="J17" s="3">
         <v>0</v>
@@ -1697,80 +1697,80 @@
         <v>0</v>
       </c>
       <c r="L17" s="4">
-        <v>71298.36</v>
+        <v>26942.720000000001</v>
       </c>
       <c r="M17" s="4">
-        <v>71298.36</v>
+        <v>26942.720000000001</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>102825</v>
+        <v>116876</v>
       </c>
       <c r="B18" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="D18" s="11">
-        <v>45117</v>
+        <v>46111</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F18" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G18" s="4">
-        <v>1494.27</v>
+        <v>20910.169999999998</v>
       </c>
       <c r="H18" s="4">
-        <v>21235.73</v>
+        <v>2031.93</v>
       </c>
       <c r="I18" s="4">
-        <v>22730</v>
+        <v>22942.1</v>
       </c>
       <c r="J18" s="3">
         <v>1</v>
       </c>
       <c r="K18" s="4">
-        <v>2520.35</v>
+        <v>15577.41</v>
       </c>
       <c r="L18" s="4">
-        <v>8829.19</v>
+        <v>71369.66</v>
       </c>
       <c r="M18" s="4">
-        <v>11349.54</v>
+        <v>86947.07</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>118246</v>
+        <v>107488</v>
       </c>
       <c r="B19" s="2">
         <v>2043</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>58</v>
+        <v>19</v>
       </c>
       <c r="D19" s="11">
-        <v>46121</v>
+        <v>45440</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F19" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" s="4">
-        <v>19016.41</v>
+        <v>0</v>
       </c>
       <c r="H19" s="4">
-        <v>0</v>
+        <v>22804.639999999999</v>
       </c>
       <c r="I19" s="4">
-        <v>19016.41</v>
+        <v>22804.639999999999</v>
       </c>
       <c r="J19" s="3">
         <v>0</v>
@@ -1779,80 +1779,80 @@
         <v>0</v>
       </c>
       <c r="L19" s="4">
-        <v>0</v>
+        <v>71298.36</v>
       </c>
       <c r="M19" s="4">
-        <v>0</v>
+        <v>71298.36</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>104718</v>
+        <v>102825</v>
       </c>
       <c r="B20" s="2">
         <v>2043</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D20" s="11">
-        <v>45264</v>
+        <v>45117</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F20" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" s="4">
-        <v>0</v>
+        <v>1494.27</v>
       </c>
       <c r="H20" s="4">
-        <v>15439.15</v>
+        <v>21235.73</v>
       </c>
       <c r="I20" s="4">
-        <v>15439.15</v>
+        <v>22730</v>
       </c>
       <c r="J20" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" s="4">
-        <v>0</v>
+        <v>2520.35</v>
       </c>
       <c r="L20" s="4">
-        <v>84741.64</v>
+        <v>8829.19</v>
       </c>
       <c r="M20" s="4">
-        <v>84741.64</v>
+        <v>11349.54</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>81618</v>
+        <v>118246</v>
       </c>
       <c r="B21" s="2">
         <v>2043</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="D21" s="11">
-        <v>43447</v>
+        <v>46121</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F21" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21" s="4">
-        <v>0</v>
+        <v>19016.41</v>
       </c>
       <c r="H21" s="4">
-        <v>15147.88</v>
+        <v>0</v>
       </c>
       <c r="I21" s="4">
-        <v>15147.88</v>
+        <v>19016.41</v>
       </c>
       <c r="J21" s="3">
         <v>0</v>
@@ -1869,16 +1869,16 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>104343</v>
+        <v>104718</v>
       </c>
       <c r="B22" s="2">
         <v>2043</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="D22" s="11">
-        <v>45201</v>
+        <v>45264</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>50</v>
@@ -1890,10 +1890,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="4">
-        <v>13213.75</v>
+        <v>15439.15</v>
       </c>
       <c r="I22" s="4">
-        <v>13213.75</v>
+        <v>15439.15</v>
       </c>
       <c r="J22" s="3">
         <v>0</v>
@@ -1902,27 +1902,27 @@
         <v>0</v>
       </c>
       <c r="L22" s="4">
-        <v>38791.620000000003</v>
+        <v>84741.64</v>
       </c>
       <c r="M22" s="4">
-        <v>38791.620000000003</v>
+        <v>84741.64</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>117440</v>
+        <v>81618</v>
       </c>
       <c r="B23" s="2">
         <v>2043</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="D23" s="11">
-        <v>46149</v>
+        <v>43447</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F23" s="3">
         <v>0</v>
@@ -1931,36 +1931,36 @@
         <v>0</v>
       </c>
       <c r="H23" s="4">
-        <v>10579.65</v>
+        <v>15147.88</v>
       </c>
       <c r="I23" s="4">
-        <v>10579.65</v>
+        <v>15147.88</v>
       </c>
       <c r="J23" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23" s="4">
-        <v>35696.19</v>
+        <v>0</v>
       </c>
       <c r="L23" s="4">
-        <v>62229</v>
+        <v>0</v>
       </c>
       <c r="M23" s="4">
-        <v>97925.19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>106018</v>
+        <v>104343</v>
       </c>
       <c r="B24" s="2">
         <v>2043</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="D24" s="11">
-        <v>45344</v>
+        <v>45201</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>50</v>
@@ -1972,10 +1972,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="4">
-        <v>9315.52</v>
+        <v>13213.75</v>
       </c>
       <c r="I24" s="4">
-        <v>9315.52</v>
+        <v>13213.75</v>
       </c>
       <c r="J24" s="3">
         <v>0</v>
@@ -1984,24 +1984,24 @@
         <v>0</v>
       </c>
       <c r="L24" s="4">
-        <v>11444.81</v>
+        <v>38791.620000000003</v>
       </c>
       <c r="M24" s="4">
-        <v>11444.81</v>
+        <v>38791.620000000003</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>114157</v>
+        <v>106018</v>
       </c>
       <c r="B25" s="2">
         <v>2043</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D25" s="11">
-        <v>45904</v>
+        <v>45344</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>50</v>
@@ -2013,10 +2013,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <v>8173.66</v>
+        <v>9315.52</v>
       </c>
       <c r="I25" s="4">
-        <v>8173.66</v>
+        <v>9315.52</v>
       </c>
       <c r="J25" s="3">
         <v>0</v>
@@ -2025,24 +2025,24 @@
         <v>0</v>
       </c>
       <c r="L25" s="4">
-        <v>55703</v>
+        <v>11444.81</v>
       </c>
       <c r="M25" s="4">
-        <v>55703</v>
+        <v>11444.81</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>88234</v>
+        <v>101640</v>
       </c>
       <c r="B26" s="2">
         <v>2043</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D26" s="11">
-        <v>43794</v>
+        <v>45104</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>50</v>
@@ -2054,10 +2054,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="4">
-        <v>7739.54</v>
+        <v>8851.4500000000007</v>
       </c>
       <c r="I26" s="4">
-        <v>7739.54</v>
+        <v>8851.4500000000007</v>
       </c>
       <c r="J26" s="3">
         <v>0</v>
@@ -2066,24 +2066,24 @@
         <v>0</v>
       </c>
       <c r="L26" s="4">
-        <v>11567.17</v>
+        <v>0</v>
       </c>
       <c r="M26" s="4">
-        <v>11567.17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>110105</v>
+        <v>114157</v>
       </c>
       <c r="B27" s="2">
         <v>2043</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="D27" s="11">
-        <v>45560</v>
+        <v>45904</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>50</v>
@@ -2095,10 +2095,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="4">
-        <v>7482.55</v>
+        <v>8173.66</v>
       </c>
       <c r="I27" s="4">
-        <v>7482.55</v>
+        <v>8173.66</v>
       </c>
       <c r="J27" s="3">
         <v>0</v>
@@ -2107,24 +2107,24 @@
         <v>0</v>
       </c>
       <c r="L27" s="4">
-        <v>2087.15</v>
+        <v>55703</v>
       </c>
       <c r="M27" s="4">
-        <v>2087.15</v>
+        <v>55703</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>109007</v>
+        <v>88234</v>
       </c>
       <c r="B28" s="2">
         <v>2043</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="D28" s="11">
-        <v>45525</v>
+        <v>43794</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>50</v>
@@ -2136,10 +2136,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>6933.13</v>
+        <v>7739.54</v>
       </c>
       <c r="I28" s="4">
-        <v>6933.13</v>
+        <v>7739.54</v>
       </c>
       <c r="J28" s="3">
         <v>0</v>
@@ -2148,24 +2148,24 @@
         <v>0</v>
       </c>
       <c r="L28" s="4">
-        <v>0</v>
+        <v>11567.17</v>
       </c>
       <c r="M28" s="4">
-        <v>0</v>
+        <v>11567.17</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>116060</v>
+        <v>110105</v>
       </c>
       <c r="B29" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D29" s="11">
-        <v>46010</v>
+        <v>45560</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>50</v>
@@ -2177,10 +2177,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="4">
-        <v>6833.65</v>
+        <v>7482.55</v>
       </c>
       <c r="I29" s="4">
-        <v>6833.65</v>
+        <v>7482.55</v>
       </c>
       <c r="J29" s="3">
         <v>0</v>
@@ -2189,39 +2189,39 @@
         <v>0</v>
       </c>
       <c r="L29" s="4">
-        <v>38580.589999999997</v>
+        <v>2087.15</v>
       </c>
       <c r="M29" s="4">
-        <v>38580.589999999997</v>
+        <v>2087.15</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>116883</v>
+        <v>109007</v>
       </c>
       <c r="B30" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="D30" s="11">
-        <v>46126</v>
+        <v>45525</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F30" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G30" s="4">
-        <v>2001.98</v>
+        <v>0</v>
       </c>
       <c r="H30" s="4">
-        <v>3590.07</v>
+        <v>6933.13</v>
       </c>
       <c r="I30" s="4">
-        <v>5592.05</v>
+        <v>6933.13</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -2230,27 +2230,27 @@
         <v>0</v>
       </c>
       <c r="L30" s="4">
-        <v>104037.69</v>
+        <v>0</v>
       </c>
       <c r="M30" s="4">
-        <v>104037.69</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>108405</v>
+        <v>116060</v>
       </c>
       <c r="B31" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="D31" s="11">
-        <v>45471</v>
+        <v>46010</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F31" s="3">
         <v>0</v>
@@ -2259,10 +2259,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="4">
-        <v>5556.45</v>
+        <v>6833.65</v>
       </c>
       <c r="I31" s="4">
-        <v>5556.45</v>
+        <v>6833.65</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -2271,65 +2271,65 @@
         <v>0</v>
       </c>
       <c r="L31" s="4">
-        <v>2506.6999999999998</v>
+        <v>38580.589999999997</v>
       </c>
       <c r="M31" s="4">
-        <v>2506.6999999999998</v>
+        <v>38580.589999999997</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>113450</v>
+        <v>116883</v>
       </c>
       <c r="B32" s="2">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D32" s="11">
-        <v>45852</v>
+        <v>46126</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F32" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="4">
-        <v>0</v>
+        <v>2001.98</v>
       </c>
       <c r="H32" s="4">
-        <v>4884.07</v>
+        <v>3590.07</v>
       </c>
       <c r="I32" s="4">
-        <v>4884.07</v>
+        <v>5592.05</v>
       </c>
       <c r="J32" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32" s="4">
-        <v>45287.66</v>
+        <v>0</v>
       </c>
       <c r="L32" s="4">
-        <v>2603.1999999999998</v>
+        <v>104037.69</v>
       </c>
       <c r="M32" s="4">
-        <v>47890.86</v>
+        <v>104037.69</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>101640</v>
+        <v>108405</v>
       </c>
       <c r="B33" s="2">
         <v>2043</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="D33" s="11">
-        <v>45104</v>
+        <v>45471</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>50</v>
@@ -2341,10 +2341,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="4">
-        <v>4745.09</v>
+        <v>5556.45</v>
       </c>
       <c r="I33" s="4">
-        <v>4745.09</v>
+        <v>5556.45</v>
       </c>
       <c r="J33" s="3">
         <v>0</v>
@@ -2353,24 +2353,24 @@
         <v>0</v>
       </c>
       <c r="L33" s="4">
-        <v>3222.89</v>
+        <v>2506.6999999999998</v>
       </c>
       <c r="M33" s="4">
-        <v>3222.89</v>
+        <v>2506.6999999999998</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>108404</v>
+        <v>113450</v>
       </c>
       <c r="B34" s="2">
         <v>2043</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D34" s="11">
-        <v>45467</v>
+        <v>45852</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>50</v>
@@ -2382,36 +2382,36 @@
         <v>0</v>
       </c>
       <c r="H34" s="4">
-        <v>3982.49</v>
+        <v>4884.07</v>
       </c>
       <c r="I34" s="4">
-        <v>3982.49</v>
+        <v>4884.07</v>
       </c>
       <c r="J34" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K34" s="4">
-        <v>0</v>
+        <v>45287.66</v>
       </c>
       <c r="L34" s="4">
-        <v>14324.23</v>
+        <v>2603.1999999999998</v>
       </c>
       <c r="M34" s="4">
-        <v>14324.23</v>
+        <v>47890.86</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>95148</v>
+        <v>108404</v>
       </c>
       <c r="B35" s="2">
         <v>2043</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="D35" s="11">
-        <v>44916</v>
+        <v>45467</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>50</v>
@@ -2423,10 +2423,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="4">
-        <v>3909.35</v>
+        <v>3982.49</v>
       </c>
       <c r="I35" s="4">
-        <v>3909.35</v>
+        <v>3982.49</v>
       </c>
       <c r="J35" s="3">
         <v>0</v>
@@ -2435,24 +2435,24 @@
         <v>0</v>
       </c>
       <c r="L35" s="4">
-        <v>0</v>
+        <v>14324.23</v>
       </c>
       <c r="M35" s="4">
-        <v>0</v>
+        <v>14324.23</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>63441</v>
+        <v>95148</v>
       </c>
       <c r="B36" s="2">
-        <v>2511</v>
+        <v>2043</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D36" s="11">
-        <v>44733</v>
+        <v>44916</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>50</v>
@@ -2464,10 +2464,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="4">
-        <v>3703.42</v>
+        <v>3909.35</v>
       </c>
       <c r="I36" s="4">
-        <v>3703.42</v>
+        <v>3909.35</v>
       </c>
       <c r="J36" s="3">
         <v>0</v>
@@ -2476,27 +2476,27 @@
         <v>0</v>
       </c>
       <c r="L36" s="4">
-        <v>5555.13</v>
+        <v>0</v>
       </c>
       <c r="M36" s="4">
-        <v>5555.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>114431</v>
+        <v>63441</v>
       </c>
       <c r="B37" s="2">
-        <v>2043</v>
+        <v>2511</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="D37" s="11">
-        <v>45930</v>
+        <v>44733</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F37" s="3">
         <v>0</v>
@@ -2505,10 +2505,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="4">
-        <v>3504.11</v>
+        <v>3703.42</v>
       </c>
       <c r="I37" s="4">
-        <v>3504.11</v>
+        <v>3703.42</v>
       </c>
       <c r="J37" s="3">
         <v>0</v>
@@ -2517,27 +2517,27 @@
         <v>0</v>
       </c>
       <c r="L37" s="4">
-        <v>16677.830000000002</v>
+        <v>5555.13</v>
       </c>
       <c r="M37" s="4">
-        <v>16677.830000000002</v>
+        <v>5555.13</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>109998</v>
+        <v>114431</v>
       </c>
       <c r="B38" s="2">
         <v>2043</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="D38" s="11">
-        <v>45596</v>
+        <v>45930</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F38" s="3">
         <v>0</v>
@@ -2546,10 +2546,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="4">
-        <v>2974.66</v>
+        <v>3504.11</v>
       </c>
       <c r="I38" s="4">
-        <v>2974.66</v>
+        <v>3504.11</v>
       </c>
       <c r="J38" s="3">
         <v>0</v>
@@ -2558,24 +2558,24 @@
         <v>0</v>
       </c>
       <c r="L38" s="4">
-        <v>0</v>
+        <v>16677.830000000002</v>
       </c>
       <c r="M38" s="4">
-        <v>0</v>
+        <v>16677.830000000002</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>115404</v>
+        <v>109998</v>
       </c>
       <c r="B39" s="2">
         <v>2043</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="D39" s="11">
-        <v>45986</v>
+        <v>45596</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>50</v>
@@ -2587,10 +2587,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="4">
-        <v>2410.9299999999998</v>
+        <v>2974.66</v>
       </c>
       <c r="I39" s="4">
-        <v>2410.9299999999998</v>
+        <v>2974.66</v>
       </c>
       <c r="J39" s="3">
         <v>0</v>
@@ -2599,24 +2599,24 @@
         <v>0</v>
       </c>
       <c r="L39" s="4">
-        <v>8741.7199999999993</v>
+        <v>0</v>
       </c>
       <c r="M39" s="4">
-        <v>8741.7199999999993</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>94156</v>
+        <v>115404</v>
       </c>
       <c r="B40" s="2">
         <v>2043</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="D40" s="11">
-        <v>44159</v>
+        <v>45986</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>50</v>
@@ -2628,10 +2628,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="4">
-        <v>2315.6999999999998</v>
+        <v>2410.9299999999998</v>
       </c>
       <c r="I40" s="4">
-        <v>2315.6999999999998</v>
+        <v>2410.9299999999998</v>
       </c>
       <c r="J40" s="3">
         <v>0</v>
@@ -2640,51 +2640,51 @@
         <v>0</v>
       </c>
       <c r="L40" s="4">
-        <v>5192.26</v>
+        <v>8741.7199999999993</v>
       </c>
       <c r="M40" s="4">
-        <v>5192.26</v>
+        <v>8741.7199999999993</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>116876</v>
+        <v>94156</v>
       </c>
       <c r="B41" s="2">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="D41" s="11">
-        <v>46111</v>
+        <v>44159</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>50</v>
       </c>
       <c r="F41" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G41" s="4">
-        <v>2065.86</v>
+        <v>0</v>
       </c>
       <c r="H41" s="4">
-        <v>0</v>
+        <v>2315.6999999999998</v>
       </c>
       <c r="I41" s="4">
-        <v>2065.86</v>
+        <v>2315.6999999999998</v>
       </c>
       <c r="J41" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K41" s="4">
-        <v>18844.310000000001</v>
+        <v>0</v>
       </c>
       <c r="L41" s="4">
-        <v>57824.19</v>
+        <v>5192.26</v>
       </c>
       <c r="M41" s="4">
-        <v>76668.5</v>
+        <v>5192.26</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
@@ -3020,7 +3020,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C49:M50">
-    <cfRule type="expression" dxfId="18" priority="77" stopIfTrue="1">
+    <cfRule type="expression" dxfId="18" priority="89" stopIfTrue="1">
       <formula>$S48=1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-06-08 11:29)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -417,7 +417,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr"/>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>4 de junio de 2026</t>
+        </is>
+      </c>
       <c r="B1" t="inlineStr"/>
       <c r="C1" t="inlineStr"/>
       <c r="D1" t="inlineStr"/>

</xml_diff>

<commit_message>
data: actualizar PagPend.xls y pagado_emitido.xlsx
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M44"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>4 de junio de 2026</t>
+          <t>25 de mayo de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -468,7 +468,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -478,40 +478,40 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>41350.53</v>
+      </c>
+      <c r="H4" t="n">
+        <v>123990.17</v>
+      </c>
+      <c r="I4" t="n">
+        <v>165340.7</v>
+      </c>
+      <c r="J4" t="n">
         <v>1</v>
       </c>
-      <c r="G4" t="n">
-        <v>6333.21</v>
-      </c>
-      <c r="H4" t="n">
-        <v>145097.32</v>
-      </c>
-      <c r="I4" t="n">
-        <v>151430.53</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>31360.93</v>
       </c>
       <c r="L4" t="n">
-        <v>5478.23</v>
+        <v>72521.25</v>
       </c>
       <c r="M4" t="n">
-        <v>5478.23</v>
+        <v>103882.18</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -521,40 +521,40 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>1985.9</v>
       </c>
       <c r="H5" t="n">
-        <v>14473.52</v>
+        <v>67664.03999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>14473.52</v>
+        <v>69649.94</v>
       </c>
       <c r="J5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5" t="n">
-        <v>2126038.83</v>
+        <v>22574.41</v>
       </c>
       <c r="L5" t="n">
-        <v>2183932.9</v>
+        <v>141422.2</v>
       </c>
       <c r="M5" t="n">
-        <v>4309971.73</v>
+        <v>163996.61</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -573,13 +573,13 @@
         <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>5165.6</v>
+        <v>32258.07</v>
       </c>
       <c r="H6" t="n">
-        <v>8472.299999999999</v>
+        <v>28647.06</v>
       </c>
       <c r="I6" t="n">
-        <v>13637.9</v>
+        <v>60905.13</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,16 +588,16 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>10200.24</v>
+        <v>59360.72</v>
       </c>
       <c r="M6" t="n">
-        <v>10200.24</v>
+        <v>59360.72</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -619,10 +619,10 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>7576.13</v>
+        <v>59212.9</v>
       </c>
       <c r="I7" t="n">
-        <v>7576.13</v>
+        <v>59212.9</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,41 +631,41 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>59833.9</v>
+        <v>251933.62</v>
       </c>
       <c r="M7" t="n">
-        <v>59833.9</v>
+        <v>251933.62</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1602.22</v>
       </c>
       <c r="H8" t="n">
-        <v>6311.07</v>
+        <v>54162.73</v>
       </c>
       <c r="I8" t="n">
-        <v>6311.07</v>
+        <v>55764.95</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,16 +674,16 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>81428.77</v>
+        <v>123887.07</v>
       </c>
       <c r="M8" t="n">
-        <v>81428.77</v>
+        <v>123887.07</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,40 +693,40 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>3249.59</v>
       </c>
       <c r="H9" t="n">
-        <v>6286.27</v>
+        <v>31354.39</v>
       </c>
       <c r="I9" t="n">
-        <v>6286.27</v>
+        <v>34603.98</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>1484.19</v>
       </c>
       <c r="L9" t="n">
-        <v>12361.96</v>
+        <v>36221.39</v>
       </c>
       <c r="M9" t="n">
-        <v>12361.96</v>
+        <v>37705.58</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -736,83 +736,83 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>1572.63</v>
       </c>
       <c r="H10" t="n">
-        <v>5622.65</v>
+        <v>31364.28</v>
       </c>
       <c r="I10" t="n">
-        <v>5622.65</v>
+        <v>32936.91</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>23108.1</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>122442.35</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>145550.45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>-9557.41</v>
       </c>
       <c r="H11" t="n">
-        <v>5571.56</v>
+        <v>41946.23</v>
       </c>
       <c r="I11" t="n">
-        <v>5571.56</v>
+        <v>32388.82</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>1368208.15</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>118391.29</v>
+        <v>10262.23</v>
       </c>
       <c r="M11" t="n">
-        <v>1486599.44</v>
+        <v>10262.23</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,22 +822,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>24295.37</v>
       </c>
       <c r="H12" t="n">
-        <v>5564.58</v>
+        <v>7700.31</v>
       </c>
       <c r="I12" t="n">
-        <v>5564.58</v>
+        <v>31995.68</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,41 +846,41 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>50165.88</v>
+        <v>80014.48</v>
       </c>
       <c r="M12" t="n">
-        <v>50165.88</v>
+        <v>80014.48</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>2455.46</v>
       </c>
       <c r="H13" t="n">
-        <v>5403.98</v>
+        <v>26614.68</v>
       </c>
       <c r="I13" t="n">
-        <v>5403.98</v>
+        <v>29070.14</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -889,16 +889,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>9644.059999999999</v>
+        <v>23159.79</v>
       </c>
       <c r="M13" t="n">
-        <v>9644.059999999999</v>
+        <v>23159.79</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,22 +908,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>22698.89</v>
       </c>
       <c r="H14" t="n">
-        <v>4747.43</v>
+        <v>5178.6</v>
       </c>
       <c r="I14" t="n">
-        <v>4747.43</v>
+        <v>27877.49</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>3224.48</v>
+        <v>10866.76</v>
       </c>
       <c r="M14" t="n">
-        <v>3224.48</v>
+        <v>10866.76</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,22 +951,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>1562.11</v>
       </c>
       <c r="H15" t="n">
-        <v>4670.98</v>
+        <v>22160.6</v>
       </c>
       <c r="I15" t="n">
-        <v>4670.98</v>
+        <v>23722.71</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>2316.79</v>
+        <v>26942.72</v>
       </c>
       <c r="M15" t="n">
-        <v>2316.79</v>
+        <v>26942.72</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>4480.67</v>
+        <v>22804.64</v>
       </c>
       <c r="I16" t="n">
-        <v>4480.67</v>
+        <v>22804.64</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>30607.01</v>
+        <v>71298.36</v>
       </c>
       <c r="M16" t="n">
-        <v>30607.01</v>
+        <v>71298.36</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,22 +1037,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>1494.27</v>
       </c>
       <c r="H17" t="n">
-        <v>2976.13</v>
+        <v>21235.73</v>
       </c>
       <c r="I17" t="n">
-        <v>2976.13</v>
+        <v>22730</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,26 +1061,26 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>8829.190000000001</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>8829.190000000001</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>2695.94</v>
+        <v>16136.19</v>
       </c>
       <c r="I18" t="n">
-        <v>2695.94</v>
+        <v>16136.19</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,26 +1104,26 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>244220.82</v>
+        <v>9134.42</v>
       </c>
       <c r="M18" t="n">
-        <v>244220.82</v>
+        <v>9134.42</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>81618</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>ALEJANDRA IVETTE PEDROZA MACIAS</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>2424.76</v>
+        <v>15147.88</v>
       </c>
       <c r="I19" t="n">
-        <v>2424.76</v>
+        <v>15147.88</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,26 +1147,26 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>41273.83</v>
+        <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>41273.83</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>2187.26</v>
+        <v>13213.75</v>
       </c>
       <c r="I20" t="n">
-        <v>2187.26</v>
+        <v>13213.75</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,16 +1190,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>101901.74</v>
+        <v>41779.37</v>
       </c>
       <c r="M20" t="n">
-        <v>101901.74</v>
+        <v>41779.37</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>1806.57</v>
+        <v>10579.65</v>
       </c>
       <c r="I21" t="n">
-        <v>1806.57</v>
+        <v>10579.65</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,16 +1233,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>16259.14</v>
+        <v>62229</v>
       </c>
       <c r="M21" t="n">
-        <v>16259.14</v>
+        <v>62229</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>1766.71</v>
+        <v>9656.709999999999</v>
       </c>
       <c r="I22" t="n">
-        <v>1766.71</v>
+        <v>9656.709999999999</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,16 +1276,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>12660.79</v>
+        <v>90524.08</v>
       </c>
       <c r="M22" t="n">
-        <v>12660.79</v>
+        <v>90524.08</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,10 +1307,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>1752.92</v>
+        <v>9315.52</v>
       </c>
       <c r="I23" t="n">
-        <v>1752.92</v>
+        <v>9315.52</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,16 +1319,16 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>11896.87</v>
+        <v>11444.81</v>
       </c>
       <c r="M23" t="n">
-        <v>11896.87</v>
+        <v>11444.81</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>1743.02</v>
+        <v>8173.66</v>
       </c>
       <c r="I24" t="n">
-        <v>1743.02</v>
+        <v>8173.66</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,16 +1362,16 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>92342.45</v>
+        <v>55703</v>
       </c>
       <c r="M24" t="n">
-        <v>92342.45</v>
+        <v>55703</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1393,10 +1393,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>1742.67</v>
+        <v>7739.54</v>
       </c>
       <c r="I25" t="n">
-        <v>1742.67</v>
+        <v>7739.54</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,16 +1405,16 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>100823.26</v>
+        <v>11567.17</v>
       </c>
       <c r="M25" t="n">
-        <v>100823.26</v>
+        <v>11567.17</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>110105</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>ROCIO YANETH OCHOA IBARRA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>1699.44</v>
+        <v>7482.55</v>
       </c>
       <c r="I26" t="n">
-        <v>1699.44</v>
+        <v>7482.55</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>14986.62</v>
+        <v>2087.15</v>
       </c>
       <c r="M26" t="n">
-        <v>14986.62</v>
+        <v>2087.15</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,10 +1479,10 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>1635.54</v>
+        <v>6933.13</v>
       </c>
       <c r="I27" t="n">
-        <v>1635.54</v>
+        <v>6933.13</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1491,26 +1491,26 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>10748.48</v>
+        <v>0</v>
       </c>
       <c r="M27" t="n">
-        <v>10748.48</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>662.91</v>
+        <v>6833.65</v>
       </c>
       <c r="I28" t="n">
-        <v>662.91</v>
+        <v>6833.65</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>8746.040000000001</v>
+        <v>38580.59</v>
       </c>
       <c r="M28" t="n">
-        <v>8746.040000000001</v>
+        <v>38580.59</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>48.79</v>
+        <v>5556.45</v>
       </c>
       <c r="I29" t="n">
-        <v>48.79</v>
+        <v>5556.45</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,26 +1577,26 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>16842.35</v>
+        <v>2506.7</v>
       </c>
       <c r="M29" t="n">
-        <v>16842.35</v>
+        <v>2506.7</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,38 +1608,38 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>4884.07</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>4884.07</v>
       </c>
       <c r="J30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>17081.33</v>
+        <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>35934.94</v>
+        <v>2603.2</v>
       </c>
       <c r="M30" t="n">
-        <v>53016.27</v>
+        <v>2603.2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,28 +1651,28 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>4745.09</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>4745.09</v>
       </c>
       <c r="J31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>15585.09</v>
+        <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>71404.87</v>
+        <v>3222.89</v>
       </c>
       <c r="M31" t="n">
-        <v>86989.96000000001</v>
+        <v>3222.89</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1694,10 +1694,10 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>3982.49</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>3982.49</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,26 +1706,26 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>4811.58</v>
+        <v>14324.23</v>
       </c>
       <c r="M32" t="n">
-        <v>4811.58</v>
+        <v>14324.23</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>3909.35</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>3909.35</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,16 +1749,16 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>41806.1</v>
+        <v>0</v>
       </c>
       <c r="M33" t="n">
-        <v>41806.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>3504.11</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>3504.11</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,16 +1792,16 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>2584.02</v>
+        <v>16677.83</v>
       </c>
       <c r="M34" t="n">
-        <v>2584.02</v>
+        <v>16677.83</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>110105</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ROCIO YANETH OCHOA IBARRA</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>2974.66</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>2974.66</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>7419.03</v>
+        <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>7419.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>2315.7</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>2315.7</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,26 +1878,26 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>4865.25</v>
+        <v>5192.26</v>
       </c>
       <c r="M36" t="n">
-        <v>4865.25</v>
+        <v>5192.26</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>63441</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2511</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>1851.71</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>1851.71</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,26 +1921,26 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>5559.19</v>
+        <v>7406.83</v>
       </c>
       <c r="M37" t="n">
-        <v>5559.19</v>
+        <v>7406.83</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1952,28 +1952,28 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>1844.64</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>1844.64</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>2001.98</v>
       </c>
       <c r="L38" t="n">
-        <v>43244.52</v>
+        <v>105783.12</v>
       </c>
       <c r="M38" t="n">
-        <v>43244.52</v>
+        <v>107785.1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1995,10 +1995,10 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>1805.68</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>1805.68</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2007,26 +2007,26 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>9678.940000000001</v>
+        <v>18056.81</v>
       </c>
       <c r="M39" t="n">
-        <v>9678.940000000001</v>
+        <v>18056.81</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>112522</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>LAURA DOLORES MONTAÐO MONTAÐO</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2038,10 +2038,10 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>1760.54</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>1760.54</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>15738.58</v>
+        <v>3201.19</v>
       </c>
       <c r="M40" t="n">
-        <v>15738.58</v>
+        <v>3201.19</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2081,10 +2081,10 @@
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>1752.06</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>1752.06</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>3911.23</v>
+        <v>14686.63</v>
       </c>
       <c r="M41" t="n">
-        <v>3911.23</v>
+        <v>14686.63</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2124,10 +2124,10 @@
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>1603.11</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>1603.11</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -2136,16 +2136,16 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>62978.13</v>
+        <v>0</v>
       </c>
       <c r="M42" t="n">
-        <v>62978.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2167,10 +2167,10 @@
         <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>662.59</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>662.59</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
@@ -2179,26 +2179,26 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>167844.24</v>
+        <v>10490.07</v>
       </c>
       <c r="M43" t="n">
-        <v>167844.24</v>
+        <v>10490.07</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>63441</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2216,16 +2216,188 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K44" t="n">
-        <v>0</v>
+        <v>19016.41</v>
       </c>
       <c r="L44" t="n">
-        <v>5557.87</v>
+        <v>0</v>
       </c>
       <c r="M44" t="n">
-        <v>5557.87</v>
+        <v>19016.41</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>116876</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2856</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="n">
+        <v>16255.46</v>
+      </c>
+      <c r="M45" t="n">
+        <v>16255.46</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>113076</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2043</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>BRUNO BRAULIO MACIAS ALVAREZ</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="n">
+        <v>4584.04</v>
+      </c>
+      <c r="M46" t="n">
+        <v>4584.04</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>111056</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2043</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>JORGE ANTONIO LUNA LARA</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" t="n">
+        <v>10951.05</v>
+      </c>
+      <c r="M47" t="n">
+        <v>10951.05</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>110575</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2043</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>JOSE RENE DE ALBA MORALES</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" t="n">
+        <v>72331.92</v>
+      </c>
+      <c r="M48" t="n">
+        <v>72331.92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: actualizar PagPend.xls correcto (5 de junio)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>25 de mayo de 2026</t>
+          <t>5 de junio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -468,50 +468,50 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>41350.53</v>
+        <v>1368208.15</v>
       </c>
       <c r="H4" t="n">
-        <v>123990.17</v>
+        <v>5571.56</v>
       </c>
       <c r="I4" t="n">
-        <v>165340.7</v>
+        <v>1373779.71</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>31360.93</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>72521.25</v>
+        <v>118391.29</v>
       </c>
       <c r="M4" t="n">
-        <v>103882.18</v>
+        <v>118391.29</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -521,7 +521,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -530,25 +530,25 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>1985.9</v>
+        <v>6333.21</v>
       </c>
       <c r="H5" t="n">
-        <v>67664.03999999999</v>
+        <v>145097.32</v>
       </c>
       <c r="I5" t="n">
-        <v>69649.94</v>
+        <v>151430.53</v>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>22574.41</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>141422.2</v>
+        <v>5478.23</v>
       </c>
       <c r="M5" t="n">
-        <v>163996.61</v>
+        <v>5478.23</v>
       </c>
     </row>
     <row r="6">
@@ -570,16 +570,16 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>32258.07</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>28647.06</v>
+        <v>16201.74</v>
       </c>
       <c r="I6" t="n">
-        <v>60905.13</v>
+        <v>16201.74</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,16 +588,16 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>59360.72</v>
+        <v>81428.77</v>
       </c>
       <c r="M6" t="n">
-        <v>59360.72</v>
+        <v>81428.77</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -619,53 +619,53 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>59212.9</v>
+        <v>14473.52</v>
       </c>
       <c r="I7" t="n">
-        <v>59212.9</v>
+        <v>14473.52</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>2126038.83</v>
       </c>
       <c r="L7" t="n">
-        <v>251933.62</v>
+        <v>2183932.9</v>
       </c>
       <c r="M7" t="n">
-        <v>251933.62</v>
+        <v>4309971.73</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>1602.22</v>
+        <v>5165.6</v>
       </c>
       <c r="H8" t="n">
-        <v>54162.73</v>
+        <v>8472.299999999999</v>
       </c>
       <c r="I8" t="n">
-        <v>55764.95</v>
+        <v>13637.9</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,59 +674,59 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>123887.07</v>
+        <v>10200.24</v>
       </c>
       <c r="M8" t="n">
-        <v>123887.07</v>
+        <v>10200.24</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>3249.59</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>31354.39</v>
+        <v>9360.959999999999</v>
       </c>
       <c r="I9" t="n">
-        <v>34603.98</v>
+        <v>9360.959999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>1484.19</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>36221.39</v>
+        <v>237555.82</v>
       </c>
       <c r="M9" t="n">
-        <v>37705.58</v>
+        <v>237555.82</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -736,22 +736,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>1572.63</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>31364.28</v>
+        <v>7576.13</v>
       </c>
       <c r="I10" t="n">
-        <v>32936.91</v>
+        <v>7576.13</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,41 +760,41 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>59833.9</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>59833.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>-9557.41</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>41946.23</v>
+        <v>6286.27</v>
       </c>
       <c r="I11" t="n">
-        <v>32388.82</v>
+        <v>6286.27</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,16 +803,16 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>10262.23</v>
+        <v>12361.96</v>
       </c>
       <c r="M11" t="n">
-        <v>10262.23</v>
+        <v>12361.96</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,65 +822,65 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>5622.65</v>
+      </c>
+      <c r="I12" t="n">
+        <v>5622.65</v>
+      </c>
+      <c r="J12" t="n">
         <v>1</v>
       </c>
-      <c r="G12" t="n">
-        <v>24295.37</v>
-      </c>
-      <c r="H12" t="n">
-        <v>7700.31</v>
-      </c>
-      <c r="I12" t="n">
-        <v>31995.68</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>23108.1</v>
       </c>
       <c r="L12" t="n">
-        <v>80014.48</v>
+        <v>122442.35</v>
       </c>
       <c r="M12" t="n">
-        <v>80014.48</v>
+        <v>145550.45</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>2455.46</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>26614.68</v>
+        <v>5564.58</v>
       </c>
       <c r="I13" t="n">
-        <v>29070.14</v>
+        <v>5564.58</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -889,16 +889,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>23159.79</v>
+        <v>50165.88</v>
       </c>
       <c r="M13" t="n">
-        <v>23159.79</v>
+        <v>50165.88</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,22 +908,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>22698.89</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>5178.6</v>
+        <v>5403.98</v>
       </c>
       <c r="I14" t="n">
-        <v>27877.49</v>
+        <v>5403.98</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>10866.76</v>
+        <v>9644.059999999999</v>
       </c>
       <c r="M14" t="n">
-        <v>10866.76</v>
+        <v>9644.059999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,22 +951,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>1562.11</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>22160.6</v>
+        <v>4747.43</v>
       </c>
       <c r="I15" t="n">
-        <v>23722.71</v>
+        <v>4747.43</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>26942.72</v>
+        <v>3224.48</v>
       </c>
       <c r="M15" t="n">
-        <v>26942.72</v>
+        <v>3224.48</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>22804.64</v>
+        <v>4670.98</v>
       </c>
       <c r="I16" t="n">
-        <v>22804.64</v>
+        <v>4670.98</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>71298.36</v>
+        <v>2316.79</v>
       </c>
       <c r="M16" t="n">
-        <v>71298.36</v>
+        <v>2316.79</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,22 +1037,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>1494.27</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>21235.73</v>
+        <v>4480.67</v>
       </c>
       <c r="I17" t="n">
-        <v>22730</v>
+        <v>4480.67</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,26 +1061,26 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>8829.190000000001</v>
+        <v>30607.01</v>
       </c>
       <c r="M17" t="n">
-        <v>8829.190000000001</v>
+        <v>30607.01</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>16136.19</v>
+        <v>4287.9</v>
       </c>
       <c r="I18" t="n">
-        <v>16136.19</v>
+        <v>4287.9</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,16 +1104,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>9134.42</v>
+        <v>10139.19</v>
       </c>
       <c r="M18" t="n">
-        <v>9134.42</v>
+        <v>10139.19</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>81618</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ALEJANDRA IVETTE PEDROZA MACIAS</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>15147.88</v>
+        <v>3484.54</v>
       </c>
       <c r="I19" t="n">
-        <v>15147.88</v>
+        <v>3484.54</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,16 +1147,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>99081.39</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>99081.39</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>13213.75</v>
+        <v>2976.13</v>
       </c>
       <c r="I20" t="n">
-        <v>13213.75</v>
+        <v>2976.13</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,16 +1190,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>41779.37</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>41779.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>10579.65</v>
+        <v>2507.93</v>
       </c>
       <c r="I21" t="n">
-        <v>10579.65</v>
+        <v>2507.93</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,16 +1233,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>62229</v>
+        <v>3051.26</v>
       </c>
       <c r="M21" t="n">
-        <v>62229</v>
+        <v>3051.26</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>9656.709999999999</v>
+        <v>2451.9</v>
       </c>
       <c r="I22" t="n">
-        <v>9656.709999999999</v>
+        <v>2451.9</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,26 +1276,26 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>90524.08</v>
+        <v>15738.58</v>
       </c>
       <c r="M22" t="n">
-        <v>90524.08</v>
+        <v>15738.58</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,10 +1307,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>9315.52</v>
+        <v>2424.76</v>
       </c>
       <c r="I23" t="n">
-        <v>9315.52</v>
+        <v>2424.76</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,26 +1319,26 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>11444.81</v>
+        <v>41273.83</v>
       </c>
       <c r="M23" t="n">
-        <v>11444.81</v>
+        <v>41273.83</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>8173.66</v>
+        <v>2187.26</v>
       </c>
       <c r="I24" t="n">
-        <v>8173.66</v>
+        <v>2187.26</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,16 +1362,16 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>55703</v>
+        <v>101901.74</v>
       </c>
       <c r="M24" t="n">
-        <v>55703</v>
+        <v>101901.74</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1393,10 +1393,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>7739.54</v>
+        <v>1806.57</v>
       </c>
       <c r="I25" t="n">
-        <v>7739.54</v>
+        <v>1806.57</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,16 +1405,16 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>11567.17</v>
+        <v>16259.14</v>
       </c>
       <c r="M25" t="n">
-        <v>11567.17</v>
+        <v>16259.14</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>110105</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ROCIO YANETH OCHOA IBARRA</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>7482.55</v>
+        <v>1752.92</v>
       </c>
       <c r="I26" t="n">
-        <v>7482.55</v>
+        <v>1752.92</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>2087.15</v>
+        <v>11896.87</v>
       </c>
       <c r="M26" t="n">
-        <v>2087.15</v>
+        <v>11896.87</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,10 +1479,10 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>6933.13</v>
+        <v>1743.02</v>
       </c>
       <c r="I27" t="n">
-        <v>6933.13</v>
+        <v>1743.02</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1491,26 +1491,26 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>92342.45</v>
       </c>
       <c r="M27" t="n">
-        <v>0</v>
+        <v>92342.45</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>6833.65</v>
+        <v>1699.44</v>
       </c>
       <c r="I28" t="n">
-        <v>6833.65</v>
+        <v>1699.44</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>38580.59</v>
+        <v>14986.62</v>
       </c>
       <c r="M28" t="n">
-        <v>38580.59</v>
+        <v>14986.62</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>5556.45</v>
+        <v>1635.54</v>
       </c>
       <c r="I29" t="n">
-        <v>5556.45</v>
+        <v>1635.54</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,16 +1577,16 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>2506.7</v>
+        <v>10748.48</v>
       </c>
       <c r="M29" t="n">
-        <v>2506.7</v>
+        <v>10748.48</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>4884.07</v>
+        <v>662.91</v>
       </c>
       <c r="I30" t="n">
-        <v>4884.07</v>
+        <v>662.91</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>2603.2</v>
+        <v>8746.040000000001</v>
       </c>
       <c r="M30" t="n">
-        <v>2603.2</v>
+        <v>8746.040000000001</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>4745.09</v>
+        <v>48.79</v>
       </c>
       <c r="I31" t="n">
-        <v>4745.09</v>
+        <v>48.79</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,26 +1663,26 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>3222.89</v>
+        <v>16842.35</v>
       </c>
       <c r="M31" t="n">
-        <v>3222.89</v>
+        <v>16842.35</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1694,38 +1694,38 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>3982.49</v>
+        <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>3982.49</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K32" t="n">
-        <v>0</v>
+        <v>17081.33</v>
       </c>
       <c r="L32" t="n">
-        <v>14324.23</v>
+        <v>35934.94</v>
       </c>
       <c r="M32" t="n">
-        <v>14324.23</v>
+        <v>53016.27</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,28 +1737,28 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>3909.35</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>3909.35</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K33" t="n">
-        <v>0</v>
+        <v>15585.09</v>
       </c>
       <c r="L33" t="n">
-        <v>0</v>
+        <v>71404.87</v>
       </c>
       <c r="M33" t="n">
-        <v>0</v>
+        <v>86989.96000000001</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>3504.11</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>3504.11</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,26 +1792,26 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>16677.83</v>
+        <v>4811.58</v>
       </c>
       <c r="M34" t="n">
-        <v>16677.83</v>
+        <v>4811.58</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>2974.66</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>2974.66</v>
+        <v>0</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>0</v>
+        <v>41806.1</v>
       </c>
       <c r="M35" t="n">
-        <v>0</v>
+        <v>41806.1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>2315.7</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>2315.7</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,26 +1878,26 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>5192.26</v>
+        <v>2584.02</v>
       </c>
       <c r="M36" t="n">
-        <v>5192.26</v>
+        <v>2584.02</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>63441</t>
+          <t>110105</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+          <t>ROCIO YANETH OCHOA IBARRA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>1851.71</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>1851.71</v>
+        <v>0</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,26 +1921,26 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>7406.83</v>
+        <v>7419.03</v>
       </c>
       <c r="M37" t="n">
-        <v>7406.83</v>
+        <v>7419.03</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1952,28 +1952,28 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>1844.64</v>
+        <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>1844.64</v>
+        <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>2001.98</v>
+        <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>105783.12</v>
+        <v>4865.25</v>
       </c>
       <c r="M38" t="n">
-        <v>107785.1</v>
+        <v>4865.25</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1995,10 +1995,10 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>1805.68</v>
+        <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>1805.68</v>
+        <v>0</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2007,26 +2007,26 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>18056.81</v>
+        <v>43244.52</v>
       </c>
       <c r="M39" t="n">
-        <v>18056.81</v>
+        <v>43244.52</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>112522</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>LAURA DOLORES MONTAÐO MONTAÐO</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2038,10 +2038,10 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>1760.54</v>
+        <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>1760.54</v>
+        <v>0</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>3201.19</v>
+        <v>9678.940000000001</v>
       </c>
       <c r="M40" t="n">
-        <v>3201.19</v>
+        <v>9678.940000000001</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2081,10 +2081,10 @@
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>1752.06</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>1752.06</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>14686.63</v>
+        <v>3911.23</v>
       </c>
       <c r="M41" t="n">
-        <v>14686.63</v>
+        <v>3911.23</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2124,10 +2124,10 @@
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>1603.11</v>
+        <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>1603.11</v>
+        <v>0</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -2136,16 +2136,16 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>0</v>
+        <v>62978.13</v>
       </c>
       <c r="M42" t="n">
-        <v>0</v>
+        <v>62978.13</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2167,10 +2167,10 @@
         <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>662.59</v>
+        <v>0</v>
       </c>
       <c r="I43" t="n">
-        <v>662.59</v>
+        <v>0</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
@@ -2179,26 +2179,26 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>10490.07</v>
+        <v>167844.24</v>
       </c>
       <c r="M43" t="n">
-        <v>10490.07</v>
+        <v>167844.24</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>63441</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2511</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2216,188 +2216,16 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>19016.41</v>
+        <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>0</v>
+        <v>5557.87</v>
       </c>
       <c r="M44" t="n">
-        <v>19016.41</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>116876</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>2856</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="n">
-        <v>0</v>
-      </c>
-      <c r="G45" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" t="n">
-        <v>0</v>
-      </c>
-      <c r="I45" t="n">
-        <v>0</v>
-      </c>
-      <c r="J45" t="n">
-        <v>0</v>
-      </c>
-      <c r="K45" t="n">
-        <v>0</v>
-      </c>
-      <c r="L45" t="n">
-        <v>16255.46</v>
-      </c>
-      <c r="M45" t="n">
-        <v>16255.46</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>113076</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>2043</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>BRUNO BRAULIO MACIAS ALVAREZ</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" t="n">
-        <v>0</v>
-      </c>
-      <c r="I46" t="n">
-        <v>0</v>
-      </c>
-      <c r="J46" t="n">
-        <v>0</v>
-      </c>
-      <c r="K46" t="n">
-        <v>0</v>
-      </c>
-      <c r="L46" t="n">
-        <v>4584.04</v>
-      </c>
-      <c r="M46" t="n">
-        <v>4584.04</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>111056</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>2043</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" t="n">
-        <v>0</v>
-      </c>
-      <c r="I47" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" t="n">
-        <v>0</v>
-      </c>
-      <c r="K47" t="n">
-        <v>0</v>
-      </c>
-      <c r="L47" t="n">
-        <v>10951.05</v>
-      </c>
-      <c r="M47" t="n">
-        <v>10951.05</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>110575</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>2043</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" t="n">
-        <v>0</v>
-      </c>
-      <c r="I48" t="n">
-        <v>0</v>
-      </c>
-      <c r="J48" t="n">
-        <v>0</v>
-      </c>
-      <c r="K48" t="n">
-        <v>0</v>
-      </c>
-      <c r="L48" t="n">
-        <v>72331.92</v>
-      </c>
-      <c r="M48" t="n">
-        <v>72331.92</v>
+        <v>5557.87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-06-10 11:08)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>5 de junio de 2026</t>
+          <t>8 de junio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -576,10 +576,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>16201.74</v>
+        <v>22688.39</v>
       </c>
       <c r="I6" t="n">
-        <v>16201.74</v>
+        <v>22688.39</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -705,10 +705,10 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>9360.959999999999</v>
+        <v>11128.96</v>
       </c>
       <c r="I9" t="n">
-        <v>9360.959999999999</v>
+        <v>11128.96</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,10 +717,10 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>237555.82</v>
+        <v>235787.82</v>
       </c>
       <c r="M9" t="n">
-        <v>237555.82</v>
+        <v>235787.82</v>
       </c>
     </row>
     <row r="10">
@@ -769,17 +769,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -791,38 +791,38 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>6286.27</v>
+        <v>7389.36</v>
       </c>
       <c r="I11" t="n">
-        <v>6286.27</v>
+        <v>7389.36</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>23108.1</v>
       </c>
       <c r="L11" t="n">
-        <v>12361.96</v>
+        <v>120675.64</v>
       </c>
       <c r="M11" t="n">
-        <v>12361.96</v>
+        <v>143783.74</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,22 +834,22 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>5622.65</v>
+        <v>6286.27</v>
       </c>
       <c r="I12" t="n">
-        <v>5622.65</v>
+        <v>6286.27</v>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>23108.1</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>122442.35</v>
+        <v>12361.96</v>
       </c>
       <c r="M12" t="n">
-        <v>145550.45</v>
+        <v>12361.96</v>
       </c>
     </row>
     <row r="13">
@@ -898,7 +898,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>5403.98</v>
+        <v>5438.63</v>
       </c>
       <c r="I14" t="n">
-        <v>5403.98</v>
+        <v>5438.63</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>9644.059999999999</v>
+        <v>97127.28999999999</v>
       </c>
       <c r="M14" t="n">
-        <v>9644.059999999999</v>
+        <v>97127.28999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>4747.43</v>
+        <v>5403.98</v>
       </c>
       <c r="I15" t="n">
-        <v>4747.43</v>
+        <v>5403.98</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>3224.48</v>
+        <v>9644.059999999999</v>
       </c>
       <c r="M15" t="n">
-        <v>3224.48</v>
+        <v>9644.059999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>4670.98</v>
+        <v>5238.69</v>
       </c>
       <c r="I16" t="n">
-        <v>4670.98</v>
+        <v>5238.69</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>2316.79</v>
+        <v>88846.77</v>
       </c>
       <c r="M16" t="n">
-        <v>2316.79</v>
+        <v>88846.77</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,28 +1049,28 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>4480.67</v>
+        <v>4747.43</v>
       </c>
       <c r="I17" t="n">
-        <v>4480.67</v>
+        <v>4747.43</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>4983.76</v>
       </c>
       <c r="L17" t="n">
-        <v>30607.01</v>
+        <v>3224.48</v>
       </c>
       <c r="M17" t="n">
-        <v>30607.01</v>
+        <v>8208.24</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>4287.9</v>
+        <v>4670.98</v>
       </c>
       <c r="I18" t="n">
-        <v>4287.9</v>
+        <v>4670.98</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,16 +1104,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>10139.19</v>
+        <v>2316.79</v>
       </c>
       <c r="M18" t="n">
-        <v>10139.19</v>
+        <v>2316.79</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>3484.54</v>
+        <v>4480.67</v>
       </c>
       <c r="I19" t="n">
-        <v>3484.54</v>
+        <v>4480.67</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,16 +1147,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>99081.39</v>
+        <v>30607.01</v>
       </c>
       <c r="M19" t="n">
-        <v>99081.39</v>
+        <v>30607.01</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>2976.13</v>
+        <v>4287.9</v>
       </c>
       <c r="I20" t="n">
-        <v>2976.13</v>
+        <v>4287.9</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,16 +1190,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>0</v>
+        <v>10139.19</v>
       </c>
       <c r="M20" t="n">
-        <v>0</v>
+        <v>10139.19</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>2507.93</v>
+        <v>2976.13</v>
       </c>
       <c r="I21" t="n">
-        <v>2507.93</v>
+        <v>2976.13</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,16 +1233,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>3051.26</v>
+        <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>3051.26</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>2451.9</v>
+        <v>2507.93</v>
       </c>
       <c r="I22" t="n">
-        <v>2451.9</v>
+        <v>2507.93</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,26 +1276,26 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>15738.58</v>
+        <v>3051.26</v>
       </c>
       <c r="M22" t="n">
-        <v>15738.58</v>
+        <v>3051.26</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,10 +1307,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>2424.76</v>
+        <v>2451.9</v>
       </c>
       <c r="I23" t="n">
-        <v>2424.76</v>
+        <v>2451.9</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,16 +1319,16 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>41273.83</v>
+        <v>15738.58</v>
       </c>
       <c r="M23" t="n">
-        <v>41273.83</v>
+        <v>15738.58</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>2187.26</v>
+        <v>2424.76</v>
       </c>
       <c r="I24" t="n">
-        <v>2187.26</v>
+        <v>2424.76</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,26 +1362,26 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>101901.74</v>
+        <v>41273.83</v>
       </c>
       <c r="M24" t="n">
-        <v>101901.74</v>
+        <v>41273.83</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1393,10 +1393,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>1806.57</v>
+        <v>2187.26</v>
       </c>
       <c r="I25" t="n">
-        <v>1806.57</v>
+        <v>2187.26</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,16 +1405,16 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>16259.14</v>
+        <v>101901.74</v>
       </c>
       <c r="M25" t="n">
-        <v>16259.14</v>
+        <v>101901.74</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>1752.92</v>
+        <v>1806.57</v>
       </c>
       <c r="I26" t="n">
-        <v>1752.92</v>
+        <v>1806.57</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>11896.87</v>
+        <v>16259.14</v>
       </c>
       <c r="M26" t="n">
-        <v>11896.87</v>
+        <v>16259.14</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,10 +1479,10 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>1743.02</v>
+        <v>1752.92</v>
       </c>
       <c r="I27" t="n">
-        <v>1743.02</v>
+        <v>1752.92</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1491,10 +1491,10 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>92342.45</v>
+        <v>11896.87</v>
       </c>
       <c r="M27" t="n">
-        <v>92342.45</v>
+        <v>11896.87</v>
       </c>
     </row>
     <row r="28">
@@ -1534,10 +1534,10 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>14986.62</v>
+        <v>8550.700000000001</v>
       </c>
       <c r="M28" t="n">
-        <v>14986.62</v>
+        <v>8550.700000000001</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-06-16 11:01)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>8 de junio de 2026</t>
+          <t>11 de junio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -490,22 +490,22 @@
         <v>1368208.15</v>
       </c>
       <c r="H4" t="n">
-        <v>5571.56</v>
+        <v>11417.31</v>
       </c>
       <c r="I4" t="n">
-        <v>1373779.71</v>
+        <v>1379625.46</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>35973.34</v>
       </c>
       <c r="L4" t="n">
-        <v>118391.29</v>
+        <v>140630.52</v>
       </c>
       <c r="M4" t="n">
-        <v>118391.29</v>
+        <v>176603.86</v>
       </c>
     </row>
     <row r="5">
@@ -554,7 +554,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -576,10 +576,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>22688.39</v>
+        <v>32186.47</v>
       </c>
       <c r="I6" t="n">
-        <v>22688.39</v>
+        <v>32186.47</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,16 +588,16 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>81428.77</v>
+        <v>131517.57</v>
       </c>
       <c r="M6" t="n">
-        <v>81428.77</v>
+        <v>131517.57</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -619,28 +619,28 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>14473.52</v>
+        <v>22688.39</v>
       </c>
       <c r="I7" t="n">
-        <v>14473.52</v>
+        <v>22688.39</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>2126038.83</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>2183932.9</v>
+        <v>81428.77</v>
       </c>
       <c r="M7" t="n">
-        <v>4309971.73</v>
+        <v>81428.77</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,22 +650,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>5165.6</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>8472.299999999999</v>
+        <v>21748.19</v>
       </c>
       <c r="I8" t="n">
-        <v>13637.9</v>
+        <v>21748.19</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,16 +674,16 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>10200.24</v>
+        <v>1292.01</v>
       </c>
       <c r="M8" t="n">
-        <v>10200.24</v>
+        <v>1292.01</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,22 +693,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>1019.74</v>
       </c>
       <c r="H9" t="n">
-        <v>11128.96</v>
+        <v>13575.59</v>
       </c>
       <c r="I9" t="n">
-        <v>11128.96</v>
+        <v>14595.33</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,16 +717,16 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>235787.82</v>
+        <v>8009.05</v>
       </c>
       <c r="M9" t="n">
-        <v>235787.82</v>
+        <v>8009.05</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,28 +748,28 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>7576.13</v>
+        <v>14473.52</v>
       </c>
       <c r="I10" t="n">
-        <v>7576.13</v>
+        <v>14473.52</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>2126038.83</v>
       </c>
       <c r="L10" t="n">
-        <v>59833.9</v>
+        <v>2183932.9</v>
       </c>
       <c r="M10" t="n">
-        <v>59833.9</v>
+        <v>4309971.73</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,50 +779,50 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>5165.6</v>
       </c>
       <c r="H11" t="n">
-        <v>7389.36</v>
+        <v>8472.299999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>7389.36</v>
+        <v>13637.9</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>23108.1</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>120675.64</v>
+        <v>10200.24</v>
       </c>
       <c r="M11" t="n">
-        <v>143783.74</v>
+        <v>10200.24</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>6286.27</v>
+        <v>12351.32</v>
       </c>
       <c r="I12" t="n">
-        <v>6286.27</v>
+        <v>12351.32</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,26 +846,26 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>12361.96</v>
+        <v>77390.42</v>
       </c>
       <c r="M12" t="n">
-        <v>12361.96</v>
+        <v>77390.42</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,10 +877,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>5564.58</v>
+        <v>11337.05</v>
       </c>
       <c r="I13" t="n">
-        <v>5564.58</v>
+        <v>11337.05</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -889,16 +889,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>50165.88</v>
+        <v>7311.14</v>
       </c>
       <c r="M13" t="n">
-        <v>50165.88</v>
+        <v>7311.14</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>5438.63</v>
+        <v>11128.96</v>
       </c>
       <c r="I14" t="n">
-        <v>5438.63</v>
+        <v>11128.96</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>97127.28999999999</v>
+        <v>235787.82</v>
       </c>
       <c r="M14" t="n">
-        <v>97127.28999999999</v>
+        <v>235787.82</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,38 +963,38 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>5403.98</v>
+        <v>9661.030000000001</v>
       </c>
       <c r="I15" t="n">
-        <v>5403.98</v>
+        <v>9661.030000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>25264.95</v>
       </c>
       <c r="L15" t="n">
-        <v>9644.059999999999</v>
+        <v>142129.36</v>
       </c>
       <c r="M15" t="n">
-        <v>9644.059999999999</v>
+        <v>167394.31</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>5238.69</v>
+        <v>8018.51</v>
       </c>
       <c r="I16" t="n">
-        <v>5238.69</v>
+        <v>8018.51</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>88846.77</v>
+        <v>106912.7</v>
       </c>
       <c r="M16" t="n">
-        <v>88846.77</v>
+        <v>106912.7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,28 +1049,28 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>4747.43</v>
+        <v>7576.13</v>
       </c>
       <c r="I17" t="n">
-        <v>4747.43</v>
+        <v>7576.13</v>
       </c>
       <c r="J17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>4983.76</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>3224.48</v>
+        <v>59833.9</v>
       </c>
       <c r="M17" t="n">
-        <v>8208.24</v>
+        <v>59833.9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>4670.98</v>
+        <v>5564.58</v>
       </c>
       <c r="I18" t="n">
-        <v>4670.98</v>
+        <v>5564.58</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,16 +1104,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>2316.79</v>
+        <v>50165.88</v>
       </c>
       <c r="M18" t="n">
-        <v>2316.79</v>
+        <v>50165.88</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>4480.67</v>
+        <v>5403.98</v>
       </c>
       <c r="I19" t="n">
-        <v>4480.67</v>
+        <v>5403.98</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,16 +1147,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>30607.01</v>
+        <v>9644.059999999999</v>
       </c>
       <c r="M19" t="n">
-        <v>30607.01</v>
+        <v>9644.059999999999</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,28 +1178,28 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>4287.9</v>
+        <v>5238.69</v>
       </c>
       <c r="I20" t="n">
-        <v>4287.9</v>
+        <v>5238.69</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>2948.64</v>
       </c>
       <c r="L20" t="n">
-        <v>10139.19</v>
+        <v>121281.79</v>
       </c>
       <c r="M20" t="n">
-        <v>10139.19</v>
+        <v>124230.43</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,28 +1221,28 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>2976.13</v>
+        <v>4747.43</v>
       </c>
       <c r="I21" t="n">
-        <v>2976.13</v>
+        <v>4747.43</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>4983.76</v>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>3224.48</v>
       </c>
       <c r="M21" t="n">
-        <v>0</v>
+        <v>8208.24</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>2507.93</v>
+        <v>4670.98</v>
       </c>
       <c r="I22" t="n">
-        <v>2507.93</v>
+        <v>4670.98</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,16 +1276,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>3051.26</v>
+        <v>2316.79</v>
       </c>
       <c r="M22" t="n">
-        <v>3051.26</v>
+        <v>2316.79</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,10 +1307,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>2451.9</v>
+        <v>4480.67</v>
       </c>
       <c r="I23" t="n">
-        <v>2451.9</v>
+        <v>4480.67</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,26 +1319,26 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>15738.58</v>
+        <v>30607.01</v>
       </c>
       <c r="M23" t="n">
-        <v>15738.58</v>
+        <v>30607.01</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,38 +1350,38 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>2424.76</v>
+        <v>4287.9</v>
       </c>
       <c r="I24" t="n">
-        <v>2424.76</v>
+        <v>4287.9</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>2347.66</v>
       </c>
       <c r="L24" t="n">
-        <v>41273.83</v>
+        <v>10139.19</v>
       </c>
       <c r="M24" t="n">
-        <v>41273.83</v>
+        <v>12486.85</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1393,10 +1393,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>2187.26</v>
+        <v>2976.13</v>
       </c>
       <c r="I25" t="n">
-        <v>2187.26</v>
+        <v>2976.13</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,16 +1405,16 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>101901.74</v>
+        <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>101901.74</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>1806.57</v>
+        <v>2507.93</v>
       </c>
       <c r="I26" t="n">
-        <v>1806.57</v>
+        <v>2507.93</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,26 +1448,26 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>16259.14</v>
+        <v>3051.26</v>
       </c>
       <c r="M26" t="n">
-        <v>16259.14</v>
+        <v>3051.26</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,10 +1479,10 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>1752.92</v>
+        <v>2424.76</v>
       </c>
       <c r="I27" t="n">
-        <v>1752.92</v>
+        <v>2424.76</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1491,16 +1491,16 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>11896.87</v>
+        <v>41273.83</v>
       </c>
       <c r="M27" t="n">
-        <v>11896.87</v>
+        <v>41273.83</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>1699.44</v>
+        <v>1806.57</v>
       </c>
       <c r="I28" t="n">
-        <v>1699.44</v>
+        <v>1806.57</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>8550.700000000001</v>
+        <v>16259.14</v>
       </c>
       <c r="M28" t="n">
-        <v>8550.700000000001</v>
+        <v>16259.14</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>1635.54</v>
+        <v>1752.92</v>
       </c>
       <c r="I29" t="n">
-        <v>1635.54</v>
+        <v>1752.92</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,16 +1577,16 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>10748.48</v>
+        <v>11896.87</v>
       </c>
       <c r="M29" t="n">
-        <v>10748.48</v>
+        <v>11896.87</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>662.91</v>
+        <v>1699.44</v>
       </c>
       <c r="I30" t="n">
-        <v>662.91</v>
+        <v>1699.44</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>8746.040000000001</v>
+        <v>8550.700000000001</v>
       </c>
       <c r="M30" t="n">
-        <v>8746.040000000001</v>
+        <v>8550.700000000001</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>48.79</v>
+        <v>1635.54</v>
       </c>
       <c r="I31" t="n">
-        <v>48.79</v>
+        <v>1635.54</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,26 +1663,26 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>16842.35</v>
+        <v>10748.48</v>
       </c>
       <c r="M31" t="n">
-        <v>16842.35</v>
+        <v>10748.48</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1694,38 +1694,38 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>662.91</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>662.91</v>
       </c>
       <c r="J32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>17081.33</v>
+        <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>35934.94</v>
+        <v>8746.040000000001</v>
       </c>
       <c r="M32" t="n">
-        <v>53016.27</v>
+        <v>8746.040000000001</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,38 +1737,38 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>48.79</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>48.79</v>
       </c>
       <c r="J33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>15585.09</v>
+        <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>71404.87</v>
+        <v>16842.35</v>
       </c>
       <c r="M33" t="n">
-        <v>86989.96000000001</v>
+        <v>16842.35</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1786,22 +1786,22 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>17081.33</v>
       </c>
       <c r="L34" t="n">
-        <v>4811.58</v>
+        <v>35934.94</v>
       </c>
       <c r="M34" t="n">
-        <v>4811.58</v>
+        <v>53016.27</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1829,22 +1829,22 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>15585.09</v>
       </c>
       <c r="L35" t="n">
-        <v>41806.1</v>
+        <v>71404.87</v>
       </c>
       <c r="M35" t="n">
-        <v>41806.1</v>
+        <v>86989.96000000001</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1878,26 +1878,26 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>2584.02</v>
+        <v>4811.58</v>
       </c>
       <c r="M36" t="n">
-        <v>2584.02</v>
+        <v>4811.58</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>110105</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ROCIO YANETH OCHOA IBARRA</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>7419.03</v>
+        <v>41806.1</v>
       </c>
       <c r="M37" t="n">
-        <v>7419.03</v>
+        <v>41806.1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>110105</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>ROCIO YANETH OCHOA IBARRA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>4865.25</v>
+        <v>7419.03</v>
       </c>
       <c r="M38" t="n">
-        <v>4865.25</v>
+        <v>7419.03</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>43244.52</v>
+        <v>4865.25</v>
       </c>
       <c r="M39" t="n">
-        <v>43244.52</v>
+        <v>4865.25</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>9678.940000000001</v>
+        <v>43244.52</v>
       </c>
       <c r="M40" t="n">
-        <v>9678.940000000001</v>
+        <v>43244.52</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>3911.23</v>
+        <v>9678.940000000001</v>
       </c>
       <c r="M41" t="n">
-        <v>3911.23</v>
+        <v>9678.940000000001</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2130,22 +2130,22 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K42" t="n">
-        <v>0</v>
+        <v>4094.59</v>
       </c>
       <c r="L42" t="n">
-        <v>62978.13</v>
+        <v>48951.77</v>
       </c>
       <c r="M42" t="n">
-        <v>62978.13</v>
+        <v>53046.36</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2179,10 +2179,10 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>167844.24</v>
+        <v>62978.13</v>
       </c>
       <c r="M43" t="n">
-        <v>167844.24</v>
+        <v>62978.13</v>
       </c>
     </row>
     <row r="44">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-06-17 13:09)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M44"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>11 de junio de 2026</t>
+          <t>16 de junio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -484,28 +484,28 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1377569.81</v>
+      </c>
+      <c r="H4" t="n">
+        <v>13221.58</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1390791.39</v>
+      </c>
+      <c r="J4" t="n">
         <v>1</v>
       </c>
-      <c r="G4" t="n">
-        <v>1368208.15</v>
-      </c>
-      <c r="H4" t="n">
-        <v>11417.31</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1379625.46</v>
-      </c>
-      <c r="J4" t="n">
-        <v>2</v>
-      </c>
       <c r="K4" t="n">
-        <v>35973.34</v>
+        <v>26611.68</v>
       </c>
       <c r="L4" t="n">
-        <v>140630.52</v>
+        <v>138826.25</v>
       </c>
       <c r="M4" t="n">
-        <v>176603.86</v>
+        <v>165437.93</v>
       </c>
     </row>
     <row r="5">
@@ -576,10 +576,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>32186.47</v>
+        <v>45386.23</v>
       </c>
       <c r="I6" t="n">
-        <v>32186.47</v>
+        <v>45386.23</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,10 +588,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>131517.57</v>
+        <v>101720.41</v>
       </c>
       <c r="M6" t="n">
-        <v>131517.57</v>
+        <v>101720.41</v>
       </c>
     </row>
     <row r="7">
@@ -613,34 +613,34 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>20152.56</v>
       </c>
       <c r="H7" t="n">
-        <v>22688.39</v>
+        <v>24430.88</v>
       </c>
       <c r="I7" t="n">
-        <v>22688.39</v>
+        <v>44583.44</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>199095.91</v>
       </c>
       <c r="L7" t="n">
-        <v>81428.77</v>
+        <v>79686.28</v>
       </c>
       <c r="M7" t="n">
-        <v>81428.77</v>
+        <v>278782.19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -662,28 +662,28 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>21748.19</v>
+        <v>22723.02</v>
       </c>
       <c r="I8" t="n">
-        <v>21748.19</v>
+        <v>22723.02</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>25264.95</v>
       </c>
       <c r="L8" t="n">
-        <v>1292.01</v>
+        <v>129067.31</v>
       </c>
       <c r="M8" t="n">
-        <v>1292.01</v>
+        <v>154332.26</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,22 +693,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>1019.74</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>13575.59</v>
+        <v>21748.19</v>
       </c>
       <c r="I9" t="n">
-        <v>14595.33</v>
+        <v>21748.19</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,10 +717,10 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>8009.05</v>
+        <v>1292.01</v>
       </c>
       <c r="M9" t="n">
-        <v>8009.05</v>
+        <v>1292.01</v>
       </c>
     </row>
     <row r="10">
@@ -769,7 +769,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,40 +779,40 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>5165.6</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>8472.299999999999</v>
+        <v>13724.04</v>
       </c>
       <c r="I11" t="n">
-        <v>13637.9</v>
+        <v>13724.04</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>3977.57</v>
       </c>
       <c r="L11" t="n">
-        <v>10200.24</v>
+        <v>276945.99</v>
       </c>
       <c r="M11" t="n">
-        <v>10200.24</v>
+        <v>280923.56</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,50 +822,50 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>5165.6</v>
       </c>
       <c r="H12" t="n">
-        <v>12351.32</v>
+        <v>8472.299999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>12351.32</v>
+        <v>13637.9</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>10913.33</v>
       </c>
       <c r="L12" t="n">
-        <v>77390.42</v>
+        <v>10200.24</v>
       </c>
       <c r="M12" t="n">
-        <v>77390.42</v>
+        <v>21113.57</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,28 +877,28 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>11337.05</v>
+        <v>13575.59</v>
       </c>
       <c r="I13" t="n">
-        <v>11337.05</v>
+        <v>13575.59</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>17895.39</v>
       </c>
       <c r="L13" t="n">
-        <v>7311.14</v>
+        <v>8009.05</v>
       </c>
       <c r="M13" t="n">
-        <v>7311.14</v>
+        <v>25904.44</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>11128.96</v>
+        <v>12351.32</v>
       </c>
       <c r="I14" t="n">
-        <v>11128.96</v>
+        <v>12351.32</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>235787.82</v>
+        <v>77390.42</v>
       </c>
       <c r="M14" t="n">
-        <v>235787.82</v>
+        <v>77390.42</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,28 +963,28 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>9661.030000000001</v>
+        <v>11827.87</v>
       </c>
       <c r="I15" t="n">
-        <v>9661.030000000001</v>
+        <v>11827.87</v>
       </c>
       <c r="J15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>25264.95</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>142129.36</v>
+        <v>43902.59</v>
       </c>
       <c r="M15" t="n">
-        <v>167394.31</v>
+        <v>43902.59</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>8018.51</v>
+        <v>11337.05</v>
       </c>
       <c r="I16" t="n">
-        <v>8018.51</v>
+        <v>11337.05</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,26 +1018,26 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>106912.7</v>
+        <v>7311.14</v>
       </c>
       <c r="M16" t="n">
-        <v>106912.7</v>
+        <v>7311.14</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>7576.13</v>
+        <v>9791.139999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>7576.13</v>
+        <v>9791.139999999999</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>59833.9</v>
+        <v>105140.07</v>
       </c>
       <c r="M17" t="n">
-        <v>59833.9</v>
+        <v>105140.07</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,40 +1080,40 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>4094.59</v>
       </c>
       <c r="H18" t="n">
-        <v>5564.58</v>
+        <v>3911.28</v>
       </c>
       <c r="I18" t="n">
-        <v>5564.58</v>
+        <v>8005.87</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>1793.93</v>
       </c>
       <c r="L18" t="n">
-        <v>50165.88</v>
+        <v>64773.79</v>
       </c>
       <c r="M18" t="n">
-        <v>50165.88</v>
+        <v>66567.72</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>5403.98</v>
+        <v>7576.13</v>
       </c>
       <c r="I19" t="n">
-        <v>5403.98</v>
+        <v>7576.13</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,16 +1147,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>9644.059999999999</v>
+        <v>59833.9</v>
       </c>
       <c r="M19" t="n">
-        <v>9644.059999999999</v>
+        <v>59833.9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>110105</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>ROCIO YANETH OCHOA IBARRA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,38 +1178,38 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>5238.69</v>
+        <v>7418.53</v>
       </c>
       <c r="I20" t="n">
-        <v>5238.69</v>
+        <v>7418.53</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>2948.64</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>121281.79</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>124230.43</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,28 +1221,28 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>4747.43</v>
+        <v>6399.41</v>
       </c>
       <c r="I21" t="n">
-        <v>4747.43</v>
+        <v>6399.41</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>4983.76</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>3224.48</v>
+        <v>23171.21</v>
       </c>
       <c r="M21" t="n">
-        <v>8208.24</v>
+        <v>23171.21</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>4670.98</v>
+        <v>5559.19</v>
       </c>
       <c r="I22" t="n">
-        <v>4670.98</v>
+        <v>5559.19</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,16 +1276,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>2316.79</v>
+        <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>2316.79</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,28 +1307,28 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>4480.67</v>
+        <v>5403.98</v>
       </c>
       <c r="I23" t="n">
-        <v>4480.67</v>
+        <v>5403.98</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>3115.46</v>
       </c>
       <c r="L23" t="n">
-        <v>30607.01</v>
+        <v>9644.059999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>30607.01</v>
+        <v>12759.52</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,28 +1350,28 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>4287.9</v>
+        <v>5238.69</v>
       </c>
       <c r="I24" t="n">
-        <v>4287.9</v>
+        <v>5238.69</v>
       </c>
       <c r="J24" t="n">
         <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>2347.66</v>
+        <v>2948.64</v>
       </c>
       <c r="L24" t="n">
-        <v>10139.19</v>
+        <v>121281.79</v>
       </c>
       <c r="M24" t="n">
-        <v>12486.85</v>
+        <v>124230.43</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1393,28 +1393,28 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>2976.13</v>
+        <v>4747.43</v>
       </c>
       <c r="I25" t="n">
-        <v>2976.13</v>
+        <v>4747.43</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>4983.76</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>3224.48</v>
       </c>
       <c r="M25" t="n">
-        <v>0</v>
+        <v>8208.24</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,38 +1436,38 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>2507.93</v>
+        <v>4670.98</v>
       </c>
       <c r="I26" t="n">
-        <v>2507.93</v>
+        <v>4670.98</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>79362.39</v>
       </c>
       <c r="L26" t="n">
-        <v>3051.26</v>
+        <v>2316.79</v>
       </c>
       <c r="M26" t="n">
-        <v>3051.26</v>
+        <v>81679.17999999999</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,10 +1479,10 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>2424.76</v>
+        <v>4480.67</v>
       </c>
       <c r="I27" t="n">
-        <v>2424.76</v>
+        <v>4480.67</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1491,16 +1491,16 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>41273.83</v>
+        <v>30607.01</v>
       </c>
       <c r="M27" t="n">
-        <v>41273.83</v>
+        <v>30607.01</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,28 +1522,28 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>1806.57</v>
+        <v>4287.9</v>
       </c>
       <c r="I28" t="n">
-        <v>1806.57</v>
+        <v>4287.9</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>2347.66</v>
       </c>
       <c r="L28" t="n">
-        <v>16259.14</v>
+        <v>10139.19</v>
       </c>
       <c r="M28" t="n">
-        <v>16259.14</v>
+        <v>12486.85</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>1752.92</v>
+        <v>2976.13</v>
       </c>
       <c r="I29" t="n">
-        <v>1752.92</v>
+        <v>2976.13</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,16 +1577,16 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>11896.87</v>
+        <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>11896.87</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>1699.44</v>
+        <v>1806.57</v>
       </c>
       <c r="I30" t="n">
-        <v>1699.44</v>
+        <v>1806.57</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>8550.700000000001</v>
+        <v>16259.14</v>
       </c>
       <c r="M30" t="n">
-        <v>8550.700000000001</v>
+        <v>16259.14</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>1635.54</v>
+        <v>1752.92</v>
       </c>
       <c r="I31" t="n">
-        <v>1635.54</v>
+        <v>1752.92</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>10748.48</v>
+        <v>11896.87</v>
       </c>
       <c r="M31" t="n">
-        <v>10748.48</v>
+        <v>11896.87</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1694,10 +1694,10 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>662.91</v>
+        <v>1699.44</v>
       </c>
       <c r="I32" t="n">
-        <v>662.91</v>
+        <v>1699.44</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,26 +1706,26 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>8746.040000000001</v>
+        <v>8550.700000000001</v>
       </c>
       <c r="M32" t="n">
-        <v>8746.040000000001</v>
+        <v>8550.700000000001</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,38 +1737,38 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>48.79</v>
+        <v>1667.89</v>
       </c>
       <c r="I33" t="n">
-        <v>48.79</v>
+        <v>1667.89</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K33" t="n">
-        <v>0</v>
+        <v>17081.33</v>
       </c>
       <c r="L33" t="n">
-        <v>16842.35</v>
+        <v>32782.12</v>
       </c>
       <c r="M33" t="n">
-        <v>16842.35</v>
+        <v>49863.45</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,38 +1780,38 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>1635.54</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>1635.54</v>
       </c>
       <c r="J34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>17081.33</v>
+        <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>35934.94</v>
+        <v>10748.48</v>
       </c>
       <c r="M34" t="n">
-        <v>53016.27</v>
+        <v>10748.48</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,28 +1823,28 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>662.91</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>662.91</v>
       </c>
       <c r="J35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>15585.09</v>
+        <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>71404.87</v>
+        <v>8746.040000000001</v>
       </c>
       <c r="M35" t="n">
-        <v>86989.96000000001</v>
+        <v>8746.040000000001</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>48.79</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>48.79</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,26 +1878,26 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>4811.58</v>
+        <v>16842.35</v>
       </c>
       <c r="M36" t="n">
-        <v>4811.58</v>
+        <v>16842.35</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1915,32 +1915,32 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>8278.549999999999</v>
       </c>
       <c r="L37" t="n">
-        <v>41806.1</v>
+        <v>24835.65</v>
       </c>
       <c r="M37" t="n">
-        <v>41806.1</v>
+        <v>33114.2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>110105</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ROCIO YANETH OCHOA IBARRA</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1958,22 +1958,22 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>15585.09</v>
       </c>
       <c r="L38" t="n">
-        <v>7419.03</v>
+        <v>71404.87</v>
       </c>
       <c r="M38" t="n">
-        <v>7419.03</v>
+        <v>86989.96000000001</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2007,26 +2007,26 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>4865.25</v>
+        <v>4811.58</v>
       </c>
       <c r="M39" t="n">
-        <v>4865.25</v>
+        <v>4811.58</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>43244.52</v>
+        <v>41806.1</v>
       </c>
       <c r="M40" t="n">
-        <v>43244.52</v>
+        <v>41806.1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>9678.940000000001</v>
+        <v>4865.25</v>
       </c>
       <c r="M41" t="n">
-        <v>9678.940000000001</v>
+        <v>4865.25</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2130,22 +2130,22 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K42" t="n">
-        <v>4094.59</v>
+        <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>48951.77</v>
+        <v>43244.52</v>
       </c>
       <c r="M42" t="n">
-        <v>53046.36</v>
+        <v>43244.52</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2179,26 +2179,26 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>62978.13</v>
+        <v>9678.940000000001</v>
       </c>
       <c r="M43" t="n">
-        <v>62978.13</v>
+        <v>9678.940000000001</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>63441</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2222,9 +2222,52 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
+        <v>62978.13</v>
+      </c>
+      <c r="M44" t="n">
+        <v>62978.13</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>63441</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2511</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="n">
         <v>5557.87</v>
       </c>
-      <c r="M44" t="n">
+      <c r="M45" t="n">
         <v>5557.87</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-06-19 11:15)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>16 de junio de 2026</t>
+          <t>17 de junio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -576,10 +576,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>45386.23</v>
+        <v>51819.85</v>
       </c>
       <c r="I6" t="n">
-        <v>45386.23</v>
+        <v>51819.85</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,10 +588,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>101720.41</v>
+        <v>95286.8</v>
       </c>
       <c r="M6" t="n">
-        <v>101720.41</v>
+        <v>95286.8</v>
       </c>
     </row>
     <row r="7">
@@ -625,16 +625,16 @@
         <v>44583.44</v>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" t="n">
-        <v>199095.91</v>
+        <v>262979.08</v>
       </c>
       <c r="L7" t="n">
         <v>79686.28</v>
       </c>
       <c r="M7" t="n">
-        <v>278782.19</v>
+        <v>342665.36</v>
       </c>
     </row>
     <row r="8">
@@ -656,28 +656,28 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>2156.85</v>
       </c>
       <c r="H8" t="n">
-        <v>22723.02</v>
+        <v>31377.49</v>
       </c>
       <c r="I8" t="n">
-        <v>22723.02</v>
+        <v>33534.34</v>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>25264.95</v>
+        <v>23108.1</v>
       </c>
       <c r="L8" t="n">
-        <v>129067.31</v>
+        <v>120415.19</v>
       </c>
       <c r="M8" t="n">
-        <v>154332.26</v>
+        <v>143523.29</v>
       </c>
     </row>
     <row r="9">
@@ -711,65 +711,65 @@
         <v>21748.19</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>2078.9</v>
       </c>
       <c r="L9" t="n">
-        <v>1292.01</v>
+        <v>24159.87</v>
       </c>
       <c r="M9" t="n">
-        <v>1292.01</v>
+        <v>26238.77</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>1192.09</v>
       </c>
       <c r="H10" t="n">
-        <v>14473.52</v>
+        <v>17557.13</v>
       </c>
       <c r="I10" t="n">
-        <v>14473.52</v>
+        <v>18749.22</v>
       </c>
       <c r="J10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>2126038.83</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>2183932.9</v>
+        <v>32782.12</v>
       </c>
       <c r="M10" t="n">
-        <v>4309971.73</v>
+        <v>32782.12</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -791,28 +791,28 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>13724.04</v>
+        <v>14473.52</v>
       </c>
       <c r="I11" t="n">
-        <v>13724.04</v>
+        <v>14473.52</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
-        <v>3977.57</v>
+        <v>2317913.6</v>
       </c>
       <c r="L11" t="n">
-        <v>276945.99</v>
+        <v>2183932.9</v>
       </c>
       <c r="M11" t="n">
-        <v>280923.56</v>
+        <v>4501846.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,40 +822,40 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>5165.6</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>8472.299999999999</v>
+        <v>13724.04</v>
       </c>
       <c r="I12" t="n">
-        <v>13637.9</v>
+        <v>13724.04</v>
       </c>
       <c r="J12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>10913.33</v>
+        <v>3977.57</v>
       </c>
       <c r="L12" t="n">
-        <v>10200.24</v>
+        <v>276945.99</v>
       </c>
       <c r="M12" t="n">
-        <v>21113.57</v>
+        <v>280923.56</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,40 +865,40 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>5165.6</v>
       </c>
       <c r="H13" t="n">
-        <v>13575.59</v>
+        <v>8472.299999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>13575.59</v>
+        <v>13637.9</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" t="n">
-        <v>17895.39</v>
+        <v>10913.33</v>
       </c>
       <c r="L13" t="n">
-        <v>8009.05</v>
+        <v>10200.24</v>
       </c>
       <c r="M13" t="n">
-        <v>25904.44</v>
+        <v>21113.57</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,28 +920,28 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>12351.32</v>
+        <v>13575.59</v>
       </c>
       <c r="I14" t="n">
-        <v>12351.32</v>
+        <v>13575.59</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>17895.39</v>
       </c>
       <c r="L14" t="n">
-        <v>77390.42</v>
+        <v>8009.05</v>
       </c>
       <c r="M14" t="n">
-        <v>77390.42</v>
+        <v>25904.44</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>11827.87</v>
+        <v>12351.32</v>
       </c>
       <c r="I15" t="n">
-        <v>11827.87</v>
+        <v>12351.32</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,26 +975,26 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>43902.59</v>
+        <v>77390.42</v>
       </c>
       <c r="M15" t="n">
-        <v>43902.59</v>
+        <v>77390.42</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>11337.05</v>
+        <v>11827.87</v>
       </c>
       <c r="I16" t="n">
-        <v>11337.05</v>
+        <v>11827.87</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>7311.14</v>
+        <v>43902.59</v>
       </c>
       <c r="M16" t="n">
-        <v>7311.14</v>
+        <v>43902.59</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>9791.139999999999</v>
+        <v>11337.05</v>
       </c>
       <c r="I17" t="n">
-        <v>9791.139999999999</v>
+        <v>11337.05</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>105140.07</v>
+        <v>7311.14</v>
       </c>
       <c r="M17" t="n">
-        <v>105140.07</v>
+        <v>7311.14</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,40 +1080,40 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>4094.59</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>3911.28</v>
+        <v>10584.87</v>
       </c>
       <c r="I18" t="n">
-        <v>8005.87</v>
+        <v>10584.87</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>1793.93</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>64773.79</v>
+        <v>56825.12</v>
       </c>
       <c r="M18" t="n">
-        <v>66567.72</v>
+        <v>56825.12</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,22 +1123,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>5888.52</v>
       </c>
       <c r="H19" t="n">
-        <v>7576.13</v>
+        <v>3911.28</v>
       </c>
       <c r="I19" t="n">
-        <v>7576.13</v>
+        <v>9799.799999999999</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,26 +1147,26 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>59833.9</v>
+        <v>64773.79</v>
       </c>
       <c r="M19" t="n">
-        <v>59833.9</v>
+        <v>64773.79</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>110105</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ROCIO YANETH OCHOA IBARRA</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>7418.53</v>
+        <v>9791.139999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>7418.53</v>
+        <v>9791.139999999999</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,10 +1190,10 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>0</v>
+        <v>105140.07</v>
       </c>
       <c r="M20" t="n">
-        <v>0</v>
+        <v>105140.07</v>
       </c>
     </row>
     <row r="21">
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>6399.41</v>
+        <v>8543.01</v>
       </c>
       <c r="I21" t="n">
-        <v>6399.41</v>
+        <v>8543.01</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,16 +1233,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>23171.21</v>
+        <v>21027.61</v>
       </c>
       <c r="M21" t="n">
-        <v>23171.21</v>
+        <v>21027.61</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,22 +1252,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>1675.67</v>
       </c>
       <c r="H22" t="n">
-        <v>5559.19</v>
+        <v>6844.09</v>
       </c>
       <c r="I22" t="n">
-        <v>5559.19</v>
+        <v>8519.76</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,16 +1276,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>9644.059999999999</v>
       </c>
       <c r="M22" t="n">
-        <v>0</v>
+        <v>9644.059999999999</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,28 +1307,28 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>5403.98</v>
+        <v>8122.72</v>
       </c>
       <c r="I23" t="n">
-        <v>5403.98</v>
+        <v>8122.72</v>
       </c>
       <c r="J23" t="n">
         <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>3115.46</v>
+        <v>2948.64</v>
       </c>
       <c r="L23" t="n">
-        <v>9644.059999999999</v>
+        <v>118397.75</v>
       </c>
       <c r="M23" t="n">
-        <v>12759.52</v>
+        <v>121346.39</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>110105</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>ROCIO YANETH OCHOA IBARRA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,28 +1350,28 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>5238.69</v>
+        <v>7418.53</v>
       </c>
       <c r="I24" t="n">
-        <v>5238.69</v>
+        <v>7418.53</v>
       </c>
       <c r="J24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>2948.64</v>
+        <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>121281.79</v>
+        <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>124230.43</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1393,28 +1393,28 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>4747.43</v>
+        <v>5559.19</v>
       </c>
       <c r="I25" t="n">
-        <v>4747.43</v>
+        <v>5559.19</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>4983.76</v>
+        <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>3224.48</v>
+        <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>8208.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,28 +1436,28 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>4670.98</v>
+        <v>4747.43</v>
       </c>
       <c r="I26" t="n">
-        <v>4670.98</v>
+        <v>4747.43</v>
       </c>
       <c r="J26" t="n">
         <v>1</v>
       </c>
       <c r="K26" t="n">
-        <v>79362.39</v>
+        <v>4983.76</v>
       </c>
       <c r="L26" t="n">
-        <v>2316.79</v>
+        <v>3224.48</v>
       </c>
       <c r="M26" t="n">
-        <v>81679.17999999999</v>
+        <v>8208.24</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,28 +1479,28 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>4480.67</v>
+        <v>4670.98</v>
       </c>
       <c r="I27" t="n">
-        <v>4480.67</v>
+        <v>4670.98</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>79362.39</v>
       </c>
       <c r="L27" t="n">
-        <v>30607.01</v>
+        <v>2316.79</v>
       </c>
       <c r="M27" t="n">
-        <v>30607.01</v>
+        <v>81679.17999999999</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,28 +1522,28 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>4287.9</v>
+        <v>4480.67</v>
       </c>
       <c r="I28" t="n">
-        <v>4287.9</v>
+        <v>4480.67</v>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>2347.66</v>
+        <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>10139.19</v>
+        <v>30607.01</v>
       </c>
       <c r="M28" t="n">
-        <v>12486.85</v>
+        <v>30607.01</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,28 +1565,28 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>2976.13</v>
+        <v>4287.9</v>
       </c>
       <c r="I29" t="n">
-        <v>2976.13</v>
+        <v>4287.9</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>2347.66</v>
       </c>
       <c r="L29" t="n">
-        <v>0</v>
+        <v>10139.19</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>12486.85</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>1806.57</v>
+        <v>2976.13</v>
       </c>
       <c r="I30" t="n">
-        <v>1806.57</v>
+        <v>2976.13</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>16259.14</v>
+        <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>16259.14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>1752.92</v>
+        <v>1806.57</v>
       </c>
       <c r="I31" t="n">
-        <v>1752.92</v>
+        <v>1806.57</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,26 +1663,26 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>11896.87</v>
+        <v>16259.14</v>
       </c>
       <c r="M31" t="n">
-        <v>11896.87</v>
+        <v>16259.14</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1694,10 +1694,10 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>1699.44</v>
+        <v>1786.77</v>
       </c>
       <c r="I32" t="n">
-        <v>1699.44</v>
+        <v>1786.77</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,26 +1706,26 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>8550.700000000001</v>
+        <v>40019.33</v>
       </c>
       <c r="M32" t="n">
-        <v>8550.700000000001</v>
+        <v>40019.33</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,28 +1737,28 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>1667.89</v>
+        <v>1752.92</v>
       </c>
       <c r="I33" t="n">
-        <v>1667.89</v>
+        <v>1752.92</v>
       </c>
       <c r="J33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>17081.33</v>
+        <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>32782.12</v>
+        <v>11896.87</v>
       </c>
       <c r="M33" t="n">
-        <v>49863.45</v>
+        <v>11896.87</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>1635.54</v>
+        <v>1699.44</v>
       </c>
       <c r="I34" t="n">
-        <v>1635.54</v>
+        <v>1699.44</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,16 +1792,16 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>10748.48</v>
+        <v>8550.700000000001</v>
       </c>
       <c r="M34" t="n">
-        <v>10748.48</v>
+        <v>8550.700000000001</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>662.91</v>
+        <v>1635.54</v>
       </c>
       <c r="I35" t="n">
-        <v>662.91</v>
+        <v>1635.54</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>8746.040000000001</v>
+        <v>10748.48</v>
       </c>
       <c r="M35" t="n">
-        <v>8746.040000000001</v>
+        <v>10748.48</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>48.79</v>
+        <v>662.91</v>
       </c>
       <c r="I36" t="n">
-        <v>48.79</v>
+        <v>662.91</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>16842.35</v>
+        <v>8746.040000000001</v>
       </c>
       <c r="M36" t="n">
-        <v>16842.35</v>
+        <v>8746.040000000001</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,38 +1909,38 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>48.79</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>48.79</v>
       </c>
       <c r="J37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>8278.549999999999</v>
+        <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>24835.65</v>
+        <v>16842.35</v>
       </c>
       <c r="M37" t="n">
-        <v>33114.2</v>
+        <v>16842.35</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1961,29 +1961,29 @@
         <v>1</v>
       </c>
       <c r="K38" t="n">
-        <v>15585.09</v>
+        <v>8278.549999999999</v>
       </c>
       <c r="L38" t="n">
-        <v>71404.87</v>
+        <v>24835.65</v>
       </c>
       <c r="M38" t="n">
-        <v>86989.96000000001</v>
+        <v>33114.2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2001,32 +2001,32 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>15585.09</v>
       </c>
       <c r="L39" t="n">
-        <v>4811.58</v>
+        <v>71404.87</v>
       </c>
       <c r="M39" t="n">
-        <v>4811.58</v>
+        <v>86989.96000000001</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2050,10 +2050,10 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>41806.1</v>
+        <v>4811.58</v>
       </c>
       <c r="M40" t="n">
-        <v>41806.1</v>
+        <v>4811.58</v>
       </c>
     </row>
     <row r="41">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-06-22 09:12)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>17 de junio de 2026</t>
+          <t>18 de junio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -511,7 +511,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -521,22 +521,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G5" t="n">
-        <v>6333.21</v>
+        <v>283131.64</v>
       </c>
       <c r="H5" t="n">
-        <v>145097.32</v>
+        <v>24430.88</v>
       </c>
       <c r="I5" t="n">
-        <v>151430.53</v>
+        <v>307562.52</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -545,16 +545,16 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>5478.23</v>
+        <v>79686.28</v>
       </c>
       <c r="M5" t="n">
-        <v>5478.23</v>
+        <v>79686.28</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,22 +564,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>6333.21</v>
       </c>
       <c r="H6" t="n">
-        <v>51819.85</v>
+        <v>145097.32</v>
       </c>
       <c r="I6" t="n">
-        <v>51819.85</v>
+        <v>151430.53</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,16 +588,16 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>95286.8</v>
+        <v>5478.23</v>
       </c>
       <c r="M6" t="n">
-        <v>95286.8</v>
+        <v>5478.23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -616,31 +616,31 @@
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>20152.56</v>
+        <v>2156.85</v>
       </c>
       <c r="H7" t="n">
-        <v>24430.88</v>
+        <v>31377.49</v>
       </c>
       <c r="I7" t="n">
-        <v>44583.44</v>
+        <v>33534.34</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>262979.08</v>
+        <v>23108.1</v>
       </c>
       <c r="L7" t="n">
-        <v>79686.28</v>
+        <v>120415.19</v>
       </c>
       <c r="M7" t="n">
-        <v>342665.36</v>
+        <v>143523.29</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -659,31 +659,31 @@
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>2156.85</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>31377.49</v>
+        <v>31470.98</v>
       </c>
       <c r="I8" t="n">
-        <v>33534.34</v>
+        <v>31470.98</v>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>23108.1</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>120415.19</v>
+        <v>8009.05</v>
       </c>
       <c r="M8" t="n">
-        <v>143523.29</v>
+        <v>8009.05</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>94205</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>JOSE ALBERTO CORONADO ROSAS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -705,114 +705,114 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>21748.19</v>
+        <v>27662.22</v>
       </c>
       <c r="I9" t="n">
-        <v>21748.19</v>
+        <v>27662.22</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>2078.9</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>24159.87</v>
+        <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>26238.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>21748.19</v>
+      </c>
+      <c r="I10" t="n">
+        <v>21748.19</v>
+      </c>
+      <c r="J10" t="n">
         <v>1</v>
       </c>
-      <c r="G10" t="n">
-        <v>1192.09</v>
-      </c>
-      <c r="H10" t="n">
-        <v>17557.13</v>
-      </c>
-      <c r="I10" t="n">
-        <v>18749.22</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>2078.9</v>
       </c>
       <c r="L10" t="n">
-        <v>32782.12</v>
+        <v>24159.87</v>
       </c>
       <c r="M10" t="n">
-        <v>32782.12</v>
+        <v>26238.77</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>1192.09</v>
       </c>
       <c r="H11" t="n">
-        <v>14473.52</v>
+        <v>17557.13</v>
       </c>
       <c r="I11" t="n">
-        <v>14473.52</v>
+        <v>18749.22</v>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>2317913.6</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>2183932.9</v>
+        <v>32782.12</v>
       </c>
       <c r="M11" t="n">
-        <v>4501846.5</v>
+        <v>32782.12</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,28 +834,28 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>13724.04</v>
+        <v>14473.52</v>
       </c>
       <c r="I12" t="n">
-        <v>13724.04</v>
+        <v>14473.52</v>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K12" t="n">
-        <v>3977.57</v>
+        <v>2317913.6</v>
       </c>
       <c r="L12" t="n">
-        <v>276945.99</v>
+        <v>2183932.9</v>
       </c>
       <c r="M12" t="n">
-        <v>280923.56</v>
+        <v>4501846.5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,40 +865,40 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>5165.6</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>8472.299999999999</v>
+        <v>13724.04</v>
       </c>
       <c r="I13" t="n">
-        <v>13637.9</v>
+        <v>13724.04</v>
       </c>
       <c r="J13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>10913.33</v>
+        <v>3977.57</v>
       </c>
       <c r="L13" t="n">
-        <v>10200.24</v>
+        <v>276945.99</v>
       </c>
       <c r="M13" t="n">
-        <v>21113.57</v>
+        <v>280923.56</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,40 +908,40 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>5165.6</v>
       </c>
       <c r="H14" t="n">
-        <v>13575.59</v>
+        <v>8472.299999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>13575.59</v>
+        <v>13637.9</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14" t="n">
-        <v>17895.39</v>
+        <v>10913.33</v>
       </c>
       <c r="L14" t="n">
-        <v>8009.05</v>
+        <v>10200.24</v>
       </c>
       <c r="M14" t="n">
-        <v>25904.44</v>
+        <v>21113.57</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>12351.32</v>
+        <v>13535.98</v>
       </c>
       <c r="I15" t="n">
-        <v>12351.32</v>
+        <v>13535.98</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>77390.42</v>
+        <v>42194.48</v>
       </c>
       <c r="M15" t="n">
-        <v>77390.42</v>
+        <v>42194.48</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>11827.87</v>
+        <v>12351.32</v>
       </c>
       <c r="I16" t="n">
-        <v>11827.87</v>
+        <v>12351.32</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,10 +1018,10 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>43902.59</v>
+        <v>77390.42</v>
       </c>
       <c r="M16" t="n">
-        <v>43902.59</v>
+        <v>77390.42</v>
       </c>
     </row>
     <row r="17">
@@ -1586,7 +1586,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>2976.13</v>
+        <v>3519.8</v>
       </c>
       <c r="I30" t="n">
-        <v>2976.13</v>
+        <v>3519.8</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>0</v>
+        <v>13960.61</v>
       </c>
       <c r="M30" t="n">
-        <v>0</v>
+        <v>13960.61</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1648,13 +1648,13 @@
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>-1986.88</v>
       </c>
       <c r="H31" t="n">
-        <v>1806.57</v>
+        <v>5321.25</v>
       </c>
       <c r="I31" t="n">
-        <v>1806.57</v>
+        <v>3334.37</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,26 +1663,26 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>16259.14</v>
+        <v>95286.8</v>
       </c>
       <c r="M31" t="n">
-        <v>16259.14</v>
+        <v>95286.8</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1694,10 +1694,10 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>1786.77</v>
+        <v>2976.13</v>
       </c>
       <c r="I32" t="n">
-        <v>1786.77</v>
+        <v>2976.13</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,16 +1706,16 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>40019.33</v>
+        <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>40019.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>1752.92</v>
+        <v>1806.57</v>
       </c>
       <c r="I33" t="n">
-        <v>1752.92</v>
+        <v>1806.57</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,26 +1749,26 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>11896.87</v>
+        <v>16259.14</v>
       </c>
       <c r="M33" t="n">
-        <v>11896.87</v>
+        <v>16259.14</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>1699.44</v>
+        <v>1786.77</v>
       </c>
       <c r="I34" t="n">
-        <v>1699.44</v>
+        <v>1786.77</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,16 +1792,16 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>8550.700000000001</v>
+        <v>40019.33</v>
       </c>
       <c r="M34" t="n">
-        <v>8550.700000000001</v>
+        <v>40019.33</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>1635.54</v>
+        <v>1752.92</v>
       </c>
       <c r="I35" t="n">
-        <v>1635.54</v>
+        <v>1752.92</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>10748.48</v>
+        <v>11896.87</v>
       </c>
       <c r="M35" t="n">
-        <v>10748.48</v>
+        <v>11896.87</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>662.91</v>
+        <v>1699.44</v>
       </c>
       <c r="I36" t="n">
-        <v>662.91</v>
+        <v>1699.44</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>8746.040000000001</v>
+        <v>8550.700000000001</v>
       </c>
       <c r="M36" t="n">
-        <v>8746.040000000001</v>
+        <v>8550.700000000001</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>48.79</v>
+        <v>1635.54</v>
       </c>
       <c r="I37" t="n">
-        <v>48.79</v>
+        <v>1635.54</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>16842.35</v>
+        <v>10748.48</v>
       </c>
       <c r="M37" t="n">
-        <v>16842.35</v>
+        <v>10748.48</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1952,38 +1952,38 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>662.91</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>662.91</v>
       </c>
       <c r="J38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>8278.549999999999</v>
+        <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>24835.65</v>
+        <v>8746.040000000001</v>
       </c>
       <c r="M38" t="n">
-        <v>33114.2</v>
+        <v>8746.040000000001</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2004,29 +2004,29 @@
         <v>1</v>
       </c>
       <c r="K39" t="n">
-        <v>15585.09</v>
+        <v>8278.549999999999</v>
       </c>
       <c r="L39" t="n">
-        <v>71404.87</v>
+        <v>24835.65</v>
       </c>
       <c r="M39" t="n">
-        <v>86989.96000000001</v>
+        <v>33114.2</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2044,22 +2044,22 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K40" t="n">
-        <v>0</v>
+        <v>15585.09</v>
       </c>
       <c r="L40" t="n">
-        <v>4811.58</v>
+        <v>71404.87</v>
       </c>
       <c r="M40" t="n">
-        <v>4811.58</v>
+        <v>86989.96000000001</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>4865.25</v>
+        <v>4811.58</v>
       </c>
       <c r="M41" t="n">
-        <v>4865.25</v>
+        <v>4811.58</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2136,16 +2136,16 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>43244.52</v>
+        <v>4865.25</v>
       </c>
       <c r="M42" t="n">
-        <v>43244.52</v>
+        <v>4865.25</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2179,16 +2179,16 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>9678.940000000001</v>
+        <v>43244.52</v>
       </c>
       <c r="M43" t="n">
-        <v>9678.940000000001</v>
+        <v>43244.52</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2222,26 +2222,26 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>62978.13</v>
+        <v>9678.940000000001</v>
       </c>
       <c r="M44" t="n">
-        <v>62978.13</v>
+        <v>9678.940000000001</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>63441</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -2265,9 +2265,52 @@
         <v>0</v>
       </c>
       <c r="L45" t="n">
+        <v>62978.13</v>
+      </c>
+      <c r="M45" t="n">
+        <v>62978.13</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>63441</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2511</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="n">
         <v>5557.87</v>
       </c>
-      <c r="M45" t="n">
+      <c r="M46" t="n">
         <v>5557.87</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-06-22 15:34)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>18 de junio de 2026</t>
+          <t>19 de junio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -484,28 +484,28 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>1377569.81</v>
+        <v>1404181.49</v>
       </c>
       <c r="H4" t="n">
         <v>13221.58</v>
       </c>
       <c r="I4" t="n">
-        <v>1390791.39</v>
+        <v>1417403.07</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>26611.68</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
         <v>138826.25</v>
       </c>
       <c r="M4" t="n">
-        <v>165437.93</v>
+        <v>138826.25</v>
       </c>
     </row>
     <row r="5">
@@ -742,120 +742,120 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>2078.9</v>
       </c>
       <c r="H10" t="n">
         <v>21748.19</v>
       </c>
       <c r="I10" t="n">
-        <v>21748.19</v>
+        <v>23827.09</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>2078.9</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
         <v>24159.87</v>
       </c>
       <c r="M10" t="n">
-        <v>26238.77</v>
+        <v>24159.87</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>8406.719999999999</v>
+      </c>
+      <c r="H11" t="n">
+        <v>10655.41</v>
+      </c>
+      <c r="I11" t="n">
+        <v>19062.13</v>
+      </c>
+      <c r="J11" t="n">
         <v>1</v>
       </c>
-      <c r="G11" t="n">
-        <v>1192.09</v>
-      </c>
-      <c r="H11" t="n">
-        <v>17557.13</v>
-      </c>
-      <c r="I11" t="n">
-        <v>18749.22</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>5488.87</v>
       </c>
       <c r="L11" t="n">
-        <v>32782.12</v>
+        <v>10200.24</v>
       </c>
       <c r="M11" t="n">
-        <v>32782.12</v>
+        <v>15689.11</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>1192.09</v>
       </c>
       <c r="H12" t="n">
-        <v>14473.52</v>
+        <v>17557.13</v>
       </c>
       <c r="I12" t="n">
-        <v>14473.52</v>
+        <v>18749.22</v>
       </c>
       <c r="J12" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>2317913.6</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>2183932.9</v>
+        <v>32782.12</v>
       </c>
       <c r="M12" t="n">
-        <v>4501846.5</v>
+        <v>32782.12</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,28 +877,28 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>13724.04</v>
+        <v>14473.52</v>
       </c>
       <c r="I13" t="n">
-        <v>13724.04</v>
+        <v>14473.52</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>3977.57</v>
+        <v>2317913.6</v>
       </c>
       <c r="L13" t="n">
-        <v>276945.99</v>
+        <v>2183932.9</v>
       </c>
       <c r="M13" t="n">
-        <v>280923.56</v>
+        <v>4501846.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,40 +908,40 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>5165.6</v>
+        <v>3021.65</v>
       </c>
       <c r="H14" t="n">
-        <v>8472.299999999999</v>
+        <v>11199.79</v>
       </c>
       <c r="I14" t="n">
-        <v>13637.9</v>
+        <v>14221.44</v>
       </c>
       <c r="J14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>10913.33</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>10200.24</v>
+        <v>116584.96</v>
       </c>
       <c r="M14" t="n">
-        <v>21113.57</v>
+        <v>116584.96</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,28 +963,28 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>13535.98</v>
+        <v>13724.04</v>
       </c>
       <c r="I15" t="n">
-        <v>13535.98</v>
+        <v>13724.04</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>3977.57</v>
       </c>
       <c r="L15" t="n">
-        <v>42194.48</v>
+        <v>276945.99</v>
       </c>
       <c r="M15" t="n">
-        <v>42194.48</v>
+        <v>280923.56</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>12351.32</v>
+        <v>13535.98</v>
       </c>
       <c r="I16" t="n">
-        <v>12351.32</v>
+        <v>13535.98</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,26 +1018,26 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>77390.42</v>
+        <v>39672.88</v>
       </c>
       <c r="M16" t="n">
-        <v>77390.42</v>
+        <v>39672.88</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>11337.05</v>
+        <v>12351.32</v>
       </c>
       <c r="I17" t="n">
-        <v>11337.05</v>
+        <v>12351.32</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,26 +1061,26 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>7311.14</v>
+        <v>77390.42</v>
       </c>
       <c r="M17" t="n">
-        <v>7311.14</v>
+        <v>77390.42</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>10584.87</v>
+        <v>11337.05</v>
       </c>
       <c r="I18" t="n">
-        <v>10584.87</v>
+        <v>11337.05</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,16 +1104,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>56825.12</v>
+        <v>7311.14</v>
       </c>
       <c r="M18" t="n">
-        <v>56825.12</v>
+        <v>7311.14</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,22 +1123,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>5888.52</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>3911.28</v>
+        <v>10584.87</v>
       </c>
       <c r="I19" t="n">
-        <v>9799.799999999999</v>
+        <v>10584.87</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,41 +1147,41 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>64773.79</v>
+        <v>56825.12</v>
       </c>
       <c r="M19" t="n">
-        <v>64773.79</v>
+        <v>56825.12</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>5888.52</v>
       </c>
       <c r="H20" t="n">
-        <v>9791.139999999999</v>
+        <v>3911.28</v>
       </c>
       <c r="I20" t="n">
-        <v>9791.139999999999</v>
+        <v>9799.799999999999</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,16 +1190,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>105140.07</v>
+        <v>64773.79</v>
       </c>
       <c r="M20" t="n">
-        <v>105140.07</v>
+        <v>64773.79</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>8543.01</v>
+        <v>9791.139999999999</v>
       </c>
       <c r="I21" t="n">
-        <v>8543.01</v>
+        <v>9791.139999999999</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,41 +1233,41 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>21027.61</v>
+        <v>105140.07</v>
       </c>
       <c r="M21" t="n">
-        <v>21027.61</v>
+        <v>105140.07</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>1675.67</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>6844.09</v>
+        <v>8543.01</v>
       </c>
       <c r="I22" t="n">
-        <v>8519.76</v>
+        <v>8543.01</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,16 +1276,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>9644.059999999999</v>
+        <v>21027.61</v>
       </c>
       <c r="M22" t="n">
-        <v>9644.059999999999</v>
+        <v>21027.61</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,34 +1295,34 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>1675.67</v>
       </c>
       <c r="H23" t="n">
-        <v>8122.72</v>
+        <v>6844.09</v>
       </c>
       <c r="I23" t="n">
-        <v>8122.72</v>
+        <v>8519.76</v>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>2948.64</v>
+        <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>118397.75</v>
+        <v>9644.059999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>121346.39</v>
+        <v>9644.059999999999</v>
       </c>
     </row>
     <row r="24">
@@ -1371,7 +1371,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1390,13 +1390,13 @@
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>-1986.88</v>
       </c>
       <c r="H25" t="n">
-        <v>5559.19</v>
+        <v>7906.44</v>
       </c>
       <c r="I25" t="n">
-        <v>5559.19</v>
+        <v>5919.56</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,16 +1405,16 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>92701.61</v>
       </c>
       <c r="M25" t="n">
-        <v>0</v>
+        <v>92701.61</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,28 +1436,28 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>4747.43</v>
+        <v>5559.19</v>
       </c>
       <c r="I26" t="n">
-        <v>4747.43</v>
+        <v>5559.19</v>
       </c>
       <c r="J26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>4983.76</v>
+        <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>3224.48</v>
+        <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>8208.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,28 +1479,28 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>4670.98</v>
+        <v>4747.43</v>
       </c>
       <c r="I27" t="n">
-        <v>4670.98</v>
+        <v>4747.43</v>
       </c>
       <c r="J27" t="n">
         <v>1</v>
       </c>
       <c r="K27" t="n">
-        <v>79362.39</v>
+        <v>4983.76</v>
       </c>
       <c r="L27" t="n">
-        <v>2316.79</v>
+        <v>3224.48</v>
       </c>
       <c r="M27" t="n">
-        <v>81679.17999999999</v>
+        <v>8208.24</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,28 +1522,28 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>4480.67</v>
+        <v>4670.98</v>
       </c>
       <c r="I28" t="n">
-        <v>4480.67</v>
+        <v>4670.98</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>79362.39</v>
       </c>
       <c r="L28" t="n">
-        <v>30607.01</v>
+        <v>2316.79</v>
       </c>
       <c r="M28" t="n">
-        <v>30607.01</v>
+        <v>81679.17999999999</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,28 +1565,28 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>4287.9</v>
+        <v>4480.67</v>
       </c>
       <c r="I29" t="n">
-        <v>4287.9</v>
+        <v>4480.67</v>
       </c>
       <c r="J29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>2347.66</v>
+        <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>10139.19</v>
+        <v>30607.01</v>
       </c>
       <c r="M29" t="n">
-        <v>12486.85</v>
+        <v>30607.01</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,28 +1608,28 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>3519.8</v>
+        <v>4287.9</v>
       </c>
       <c r="I30" t="n">
-        <v>3519.8</v>
+        <v>4287.9</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K30" t="n">
-        <v>0</v>
+        <v>2347.66</v>
       </c>
       <c r="L30" t="n">
-        <v>13960.61</v>
+        <v>10139.19</v>
       </c>
       <c r="M30" t="n">
-        <v>13960.61</v>
+        <v>12486.85</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1648,13 +1648,13 @@
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>-1986.88</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>5321.25</v>
+        <v>3519.8</v>
       </c>
       <c r="I31" t="n">
-        <v>3334.37</v>
+        <v>3519.8</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,10 +1663,10 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>95286.8</v>
+        <v>13960.61</v>
       </c>
       <c r="M31" t="n">
-        <v>95286.8</v>
+        <v>13960.61</v>
       </c>
     </row>
     <row r="32">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-06-23 15:08)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>19 de junio de 2026</t>
+          <t>22 de junio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -490,10 +490,10 @@
         <v>1404181.49</v>
       </c>
       <c r="H4" t="n">
-        <v>13221.58</v>
+        <v>15284.04</v>
       </c>
       <c r="I4" t="n">
-        <v>1417403.07</v>
+        <v>1419465.53</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -502,10 +502,10 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>138826.25</v>
+        <v>136763.79</v>
       </c>
       <c r="M4" t="n">
-        <v>138826.25</v>
+        <v>136763.79</v>
       </c>
     </row>
     <row r="5">
@@ -533,10 +533,10 @@
         <v>283131.64</v>
       </c>
       <c r="H5" t="n">
-        <v>24430.88</v>
+        <v>25296.38</v>
       </c>
       <c r="I5" t="n">
-        <v>307562.52</v>
+        <v>308428.02</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -1227,16 +1227,16 @@
         <v>9791.139999999999</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>1742.84</v>
       </c>
       <c r="L21" t="n">
-        <v>105140.07</v>
+        <v>124311.35</v>
       </c>
       <c r="M21" t="n">
-        <v>105140.07</v>
+        <v>126054.19</v>
       </c>
     </row>
     <row r="22">
@@ -1371,7 +1371,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1390,31 +1390,31 @@
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>-1986.88</v>
+        <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>7906.44</v>
+        <v>6987.82</v>
       </c>
       <c r="I25" t="n">
-        <v>5919.56</v>
+        <v>6987.82</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>79362.39</v>
       </c>
       <c r="L25" t="n">
-        <v>92701.61</v>
+        <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>92701.61</v>
+        <v>79362.39</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>5559.19</v>
+        <v>6257.28</v>
       </c>
       <c r="I26" t="n">
-        <v>5559.19</v>
+        <v>6257.28</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>28945.76</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>28945.76</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1476,31 +1476,31 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>-1986.88</v>
       </c>
       <c r="H27" t="n">
-        <v>4747.43</v>
+        <v>7906.44</v>
       </c>
       <c r="I27" t="n">
-        <v>4747.43</v>
+        <v>5919.56</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>4983.76</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>3224.48</v>
+        <v>92701.61</v>
       </c>
       <c r="M27" t="n">
-        <v>8208.24</v>
+        <v>92701.61</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,28 +1522,28 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>4670.98</v>
+        <v>5559.19</v>
       </c>
       <c r="I28" t="n">
-        <v>4670.98</v>
+        <v>5559.19</v>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>79362.39</v>
+        <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>2316.79</v>
+        <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>81679.17999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,22 +1565,22 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>4480.67</v>
+        <v>4747.43</v>
       </c>
       <c r="I29" t="n">
-        <v>4480.67</v>
+        <v>4747.43</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>4983.76</v>
       </c>
       <c r="L29" t="n">
-        <v>30607.01</v>
+        <v>3224.48</v>
       </c>
       <c r="M29" t="n">
-        <v>30607.01</v>
+        <v>8208.24</v>
       </c>
     </row>
     <row r="30">
@@ -1930,7 +1930,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1952,10 +1952,10 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>662.91</v>
+        <v>1603.9</v>
       </c>
       <c r="I38" t="n">
-        <v>662.91</v>
+        <v>1603.9</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>8746.040000000001</v>
+        <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>8746.040000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1995,38 +1995,38 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>1075.86</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>1075.86</v>
       </c>
       <c r="J39" t="n">
         <v>1</v>
       </c>
       <c r="K39" t="n">
-        <v>8278.549999999999</v>
+        <v>1433.08</v>
       </c>
       <c r="L39" t="n">
-        <v>24835.65</v>
+        <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v>33114.2</v>
+        <v>1433.08</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2038,28 +2038,28 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>662.91</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>662.91</v>
       </c>
       <c r="J40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K40" t="n">
-        <v>15585.09</v>
+        <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>71404.87</v>
+        <v>8746.040000000001</v>
       </c>
       <c r="M40" t="n">
-        <v>86989.96000000001</v>
+        <v>8746.040000000001</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2087,32 +2087,32 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>8278.549999999999</v>
       </c>
       <c r="L41" t="n">
-        <v>4811.58</v>
+        <v>24835.65</v>
       </c>
       <c r="M41" t="n">
-        <v>4811.58</v>
+        <v>33114.2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2130,16 +2130,16 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K42" t="n">
-        <v>0</v>
+        <v>15585.09</v>
       </c>
       <c r="L42" t="n">
-        <v>4865.25</v>
+        <v>71404.87</v>
       </c>
       <c r="M42" t="n">
-        <v>4865.25</v>
+        <v>86989.96000000001</v>
       </c>
     </row>
     <row r="43">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-06-24 13:43)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>22 de junio de 2026</t>
+          <t>23 de junio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -533,10 +533,10 @@
         <v>283131.64</v>
       </c>
       <c r="H5" t="n">
-        <v>25296.38</v>
+        <v>30126.99</v>
       </c>
       <c r="I5" t="n">
-        <v>308428.02</v>
+        <v>313258.63</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -545,10 +545,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>79686.28</v>
+        <v>77956.22</v>
       </c>
       <c r="M5" t="n">
-        <v>79686.28</v>
+        <v>77956.22</v>
       </c>
     </row>
     <row r="6">
@@ -662,10 +662,10 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>31470.98</v>
+        <v>33217.27</v>
       </c>
       <c r="I8" t="n">
-        <v>31470.98</v>
+        <v>33217.27</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,10 +674,10 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>8009.05</v>
+        <v>6262.76</v>
       </c>
       <c r="M8" t="n">
-        <v>8009.05</v>
+        <v>6262.76</v>
       </c>
     </row>
     <row r="9">
@@ -748,10 +748,10 @@
         <v>2078.9</v>
       </c>
       <c r="H10" t="n">
-        <v>21748.19</v>
+        <v>25332.43</v>
       </c>
       <c r="I10" t="n">
-        <v>23827.09</v>
+        <v>27411.33</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -791,10 +791,10 @@
         <v>8406.719999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>10655.41</v>
+        <v>15836.56</v>
       </c>
       <c r="I11" t="n">
-        <v>19062.13</v>
+        <v>24243.28</v>
       </c>
       <c r="J11" t="n">
         <v>1</v>
@@ -803,102 +803,102 @@
         <v>5488.87</v>
       </c>
       <c r="L11" t="n">
-        <v>10200.24</v>
+        <v>5681.96</v>
       </c>
       <c r="M11" t="n">
-        <v>15689.11</v>
+        <v>11170.83</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>21929.23</v>
+      </c>
+      <c r="I12" t="n">
+        <v>21929.23</v>
+      </c>
+      <c r="J12" t="n">
         <v>1</v>
       </c>
-      <c r="G12" t="n">
-        <v>1192.09</v>
-      </c>
-      <c r="H12" t="n">
-        <v>17557.13</v>
-      </c>
-      <c r="I12" t="n">
-        <v>18749.22</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>3977.57</v>
       </c>
       <c r="L12" t="n">
-        <v>32782.12</v>
+        <v>268740.8</v>
       </c>
       <c r="M12" t="n">
-        <v>32782.12</v>
+        <v>272718.37</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>1192.09</v>
       </c>
       <c r="H13" t="n">
-        <v>14473.52</v>
+        <v>17557.13</v>
       </c>
       <c r="I13" t="n">
-        <v>14473.52</v>
+        <v>18749.22</v>
       </c>
       <c r="J13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>2317913.6</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>2183932.9</v>
+        <v>32782.12</v>
       </c>
       <c r="M13" t="n">
-        <v>4501846.5</v>
+        <v>32782.12</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,40 +908,40 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>3021.65</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>11199.79</v>
+        <v>14473.52</v>
       </c>
       <c r="I14" t="n">
-        <v>14221.44</v>
+        <v>14473.52</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>2317913.6</v>
       </c>
       <c r="L14" t="n">
-        <v>116584.96</v>
+        <v>2183932.9</v>
       </c>
       <c r="M14" t="n">
-        <v>116584.96</v>
+        <v>4501846.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,50 +951,50 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>3021.65</v>
       </c>
       <c r="H15" t="n">
-        <v>13724.04</v>
+        <v>11199.79</v>
       </c>
       <c r="I15" t="n">
-        <v>13724.04</v>
+        <v>14221.44</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>3977.57</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>276945.99</v>
+        <v>116584.96</v>
       </c>
       <c r="M15" t="n">
-        <v>280923.56</v>
+        <v>116584.96</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,28 +1006,28 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>13535.98</v>
+        <v>13639.66</v>
       </c>
       <c r="I16" t="n">
-        <v>13535.98</v>
+        <v>13639.66</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>1742.84</v>
       </c>
       <c r="L16" t="n">
-        <v>39672.88</v>
+        <v>120462.83</v>
       </c>
       <c r="M16" t="n">
-        <v>39672.88</v>
+        <v>122205.67</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>12351.32</v>
+        <v>13535.98</v>
       </c>
       <c r="I17" t="n">
-        <v>12351.32</v>
+        <v>13535.98</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,26 +1061,26 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>77390.42</v>
+        <v>39672.88</v>
       </c>
       <c r="M17" t="n">
-        <v>77390.42</v>
+        <v>39672.88</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>11337.05</v>
+        <v>12351.32</v>
       </c>
       <c r="I18" t="n">
-        <v>11337.05</v>
+        <v>12351.32</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,26 +1104,26 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>7311.14</v>
+        <v>77390.42</v>
       </c>
       <c r="M18" t="n">
-        <v>7311.14</v>
+        <v>77390.42</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>10584.87</v>
+        <v>11337.05</v>
       </c>
       <c r="I19" t="n">
-        <v>10584.87</v>
+        <v>11337.05</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,16 +1147,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>56825.12</v>
+        <v>7311.14</v>
       </c>
       <c r="M19" t="n">
-        <v>56825.12</v>
+        <v>7311.14</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,22 +1166,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>5888.52</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>3911.28</v>
+        <v>10584.87</v>
       </c>
       <c r="I20" t="n">
-        <v>9799.799999999999</v>
+        <v>10584.87</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,53 +1190,53 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>64773.79</v>
+        <v>56825.12</v>
       </c>
       <c r="M20" t="n">
-        <v>64773.79</v>
+        <v>56825.12</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>5888.52</v>
       </c>
       <c r="H21" t="n">
-        <v>9791.139999999999</v>
+        <v>3911.28</v>
       </c>
       <c r="I21" t="n">
-        <v>9791.139999999999</v>
+        <v>9799.799999999999</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>1742.84</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>124311.35</v>
+        <v>64773.79</v>
       </c>
       <c r="M21" t="n">
-        <v>126054.19</v>
+        <v>64773.79</v>
       </c>
     </row>
     <row r="22">
@@ -1457,7 +1457,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1476,13 +1476,13 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>-1986.88</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>7906.44</v>
+        <v>6080.42</v>
       </c>
       <c r="I27" t="n">
-        <v>5919.56</v>
+        <v>6080.42</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1491,16 +1491,16 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>92701.61</v>
+        <v>3598.57</v>
       </c>
       <c r="M27" t="n">
-        <v>92701.61</v>
+        <v>3598.57</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1519,31 +1519,31 @@
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>-1986.88</v>
       </c>
       <c r="H28" t="n">
-        <v>5559.19</v>
+        <v>7906.44</v>
       </c>
       <c r="I28" t="n">
-        <v>5559.19</v>
+        <v>5919.56</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>66840.31</v>
       </c>
       <c r="L28" t="n">
-        <v>0</v>
+        <v>92701.61</v>
       </c>
       <c r="M28" t="n">
-        <v>0</v>
+        <v>159541.92</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,28 +1565,28 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>4747.43</v>
+        <v>5559.19</v>
       </c>
       <c r="I29" t="n">
-        <v>4747.43</v>
+        <v>5559.19</v>
       </c>
       <c r="J29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>4983.76</v>
+        <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>3224.48</v>
+        <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>8208.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,28 +1608,28 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>4287.9</v>
+        <v>4747.43</v>
       </c>
       <c r="I30" t="n">
-        <v>4287.9</v>
+        <v>4747.43</v>
       </c>
       <c r="J30" t="n">
         <v>1</v>
       </c>
       <c r="K30" t="n">
-        <v>2347.66</v>
+        <v>4983.76</v>
       </c>
       <c r="L30" t="n">
-        <v>10139.19</v>
+        <v>3224.48</v>
       </c>
       <c r="M30" t="n">
-        <v>12486.85</v>
+        <v>8208.24</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,38 +1651,38 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>3519.8</v>
+        <v>4287.9</v>
       </c>
       <c r="I31" t="n">
-        <v>3519.8</v>
+        <v>4287.9</v>
       </c>
       <c r="J31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>2347.66</v>
       </c>
       <c r="L31" t="n">
-        <v>13960.61</v>
+        <v>10139.19</v>
       </c>
       <c r="M31" t="n">
-        <v>13960.61</v>
+        <v>12486.85</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1694,10 +1694,10 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>2976.13</v>
+        <v>3628.52</v>
       </c>
       <c r="I32" t="n">
-        <v>2976.13</v>
+        <v>3628.52</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,16 +1706,16 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>0</v>
+        <v>38177.58</v>
       </c>
       <c r="M32" t="n">
-        <v>0</v>
+        <v>38177.58</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>1806.57</v>
+        <v>3519.8</v>
       </c>
       <c r="I33" t="n">
-        <v>1806.57</v>
+        <v>3519.8</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,26 +1749,26 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>16259.14</v>
+        <v>13960.61</v>
       </c>
       <c r="M33" t="n">
-        <v>16259.14</v>
+        <v>13960.61</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>1786.77</v>
+        <v>2976.13</v>
       </c>
       <c r="I34" t="n">
-        <v>1786.77</v>
+        <v>2976.13</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,16 +1792,16 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>40019.33</v>
+        <v>0</v>
       </c>
       <c r="M34" t="n">
-        <v>40019.33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>1752.92</v>
+        <v>1806.57</v>
       </c>
       <c r="I35" t="n">
-        <v>1752.92</v>
+        <v>1806.57</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>11896.87</v>
+        <v>16259.14</v>
       </c>
       <c r="M35" t="n">
-        <v>11896.87</v>
+        <v>16259.14</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>1699.44</v>
+        <v>1752.92</v>
       </c>
       <c r="I36" t="n">
-        <v>1699.44</v>
+        <v>1752.92</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>8550.700000000001</v>
+        <v>11896.87</v>
       </c>
       <c r="M36" t="n">
-        <v>8550.700000000001</v>
+        <v>11896.87</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>1635.54</v>
+        <v>1699.44</v>
       </c>
       <c r="I37" t="n">
-        <v>1635.54</v>
+        <v>1699.44</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>10748.48</v>
+        <v>8550.700000000001</v>
       </c>
       <c r="M37" t="n">
-        <v>10748.48</v>
+        <v>8550.700000000001</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1952,10 +1952,10 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>1603.9</v>
+        <v>1635.54</v>
       </c>
       <c r="I38" t="n">
-        <v>1603.9</v>
+        <v>1635.54</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>0</v>
+        <v>10748.48</v>
       </c>
       <c r="M38" t="n">
-        <v>0</v>
+        <v>10748.48</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1995,28 +1995,28 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>1075.86</v>
+        <v>1603.9</v>
       </c>
       <c r="I39" t="n">
-        <v>1075.86</v>
+        <v>1603.9</v>
       </c>
       <c r="J39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>1433.08</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
         <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v>1433.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2038,28 +2038,28 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>662.91</v>
+        <v>1075.86</v>
       </c>
       <c r="I40" t="n">
-        <v>662.91</v>
+        <v>1075.86</v>
       </c>
       <c r="J40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K40" t="n">
-        <v>0</v>
+        <v>1433.08</v>
       </c>
       <c r="L40" t="n">
-        <v>8746.040000000001</v>
+        <v>0</v>
       </c>
       <c r="M40" t="n">
-        <v>8746.040000000001</v>
+        <v>1433.08</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2081,38 +2081,38 @@
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>662.91</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>662.91</v>
       </c>
       <c r="J41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K41" t="n">
-        <v>8278.549999999999</v>
+        <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>24835.65</v>
+        <v>8746.040000000001</v>
       </c>
       <c r="M41" t="n">
-        <v>33114.2</v>
+        <v>8746.040000000001</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2133,29 +2133,29 @@
         <v>1</v>
       </c>
       <c r="K42" t="n">
-        <v>15585.09</v>
+        <v>8278.549999999999</v>
       </c>
       <c r="L42" t="n">
-        <v>71404.87</v>
+        <v>24835.65</v>
       </c>
       <c r="M42" t="n">
-        <v>86989.96000000001</v>
+        <v>33114.2</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2173,22 +2173,22 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>0</v>
+        <v>15585.09</v>
       </c>
       <c r="L43" t="n">
-        <v>43244.52</v>
+        <v>71404.87</v>
       </c>
       <c r="M43" t="n">
-        <v>43244.52</v>
+        <v>86989.96000000001</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2222,10 +2222,10 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>9678.940000000001</v>
+        <v>43244.52</v>
       </c>
       <c r="M44" t="n">
-        <v>9678.940000000001</v>
+        <v>43244.52</v>
       </c>
     </row>
     <row r="45">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-06-25 12:52)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>23 de junio de 2026</t>
+          <t>24 de junio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -490,10 +490,10 @@
         <v>1404181.49</v>
       </c>
       <c r="H4" t="n">
-        <v>15284.04</v>
+        <v>16824.83</v>
       </c>
       <c r="I4" t="n">
-        <v>1419465.53</v>
+        <v>1421006.32</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -554,7 +554,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -573,31 +573,31 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>6333.21</v>
+        <v>191874.77</v>
       </c>
       <c r="H6" t="n">
-        <v>145097.32</v>
+        <v>14473.52</v>
       </c>
       <c r="I6" t="n">
-        <v>151430.53</v>
+        <v>206348.29</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>2126038.83</v>
       </c>
       <c r="L6" t="n">
-        <v>5478.23</v>
+        <v>2183932.9</v>
       </c>
       <c r="M6" t="n">
-        <v>5478.23</v>
+        <v>4309971.73</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -616,31 +616,31 @@
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>2156.85</v>
+        <v>6333.21</v>
       </c>
       <c r="H7" t="n">
-        <v>31377.49</v>
+        <v>145097.32</v>
       </c>
       <c r="I7" t="n">
-        <v>33534.34</v>
+        <v>151430.53</v>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>23108.1</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>120415.19</v>
+        <v>5478.23</v>
       </c>
       <c r="M7" t="n">
-        <v>143523.29</v>
+        <v>5478.23</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -659,31 +659,31 @@
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>2156.85</v>
       </c>
       <c r="H8" t="n">
-        <v>33217.27</v>
+        <v>31377.49</v>
       </c>
       <c r="I8" t="n">
-        <v>33217.27</v>
+        <v>33534.34</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>23108.1</v>
       </c>
       <c r="L8" t="n">
-        <v>6262.76</v>
+        <v>120415.19</v>
       </c>
       <c r="M8" t="n">
-        <v>6262.76</v>
+        <v>143523.29</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>94205</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,22 +693,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>JOSE ALBERTO CORONADO ROSAS</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>27662.22</v>
+        <v>33217.27</v>
       </c>
       <c r="I9" t="n">
-        <v>27662.22</v>
+        <v>33217.27</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,10 +717,10 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>6262.76</v>
       </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>6262.76</v>
       </c>
     </row>
     <row r="10">
@@ -748,10 +748,10 @@
         <v>2078.9</v>
       </c>
       <c r="H10" t="n">
-        <v>25332.43</v>
+        <v>26624.44</v>
       </c>
       <c r="I10" t="n">
-        <v>27411.33</v>
+        <v>28703.34</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,16 +760,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>24159.87</v>
+        <v>22867.86</v>
       </c>
       <c r="M10" t="n">
-        <v>24159.87</v>
+        <v>22867.86</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>94205</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,40 +779,40 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>JOSE ALBERTO CORONADO ROSAS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>8406.719999999999</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>15836.56</v>
+        <v>27662.22</v>
       </c>
       <c r="I11" t="n">
-        <v>24243.28</v>
+        <v>27662.22</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>5488.87</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>5681.96</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>11170.83</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,71 +834,71 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>21929.23</v>
+        <v>27488.71</v>
       </c>
       <c r="I12" t="n">
-        <v>21929.23</v>
+        <v>27488.71</v>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>3977.57</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>268740.8</v>
+        <v>25720.15</v>
       </c>
       <c r="M12" t="n">
-        <v>272718.37</v>
+        <v>25720.15</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>26683.02</v>
+      </c>
+      <c r="I13" t="n">
+        <v>26683.02</v>
+      </c>
+      <c r="J13" t="n">
         <v>1</v>
       </c>
-      <c r="G13" t="n">
-        <v>1192.09</v>
-      </c>
-      <c r="H13" t="n">
-        <v>17557.13</v>
-      </c>
-      <c r="I13" t="n">
-        <v>18749.22</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>3977.57</v>
       </c>
       <c r="L13" t="n">
-        <v>32782.12</v>
+        <v>263987.05</v>
       </c>
       <c r="M13" t="n">
-        <v>32782.12</v>
+        <v>267964.62</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,50 +908,50 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>8406.719999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>14473.52</v>
+        <v>15836.56</v>
       </c>
       <c r="I14" t="n">
-        <v>14473.52</v>
+        <v>24243.28</v>
       </c>
       <c r="J14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>2317913.6</v>
+        <v>5488.87</v>
       </c>
       <c r="L14" t="n">
-        <v>2183932.9</v>
+        <v>5681.96</v>
       </c>
       <c r="M14" t="n">
-        <v>4501846.5</v>
+        <v>11170.83</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -960,13 +960,13 @@
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>3021.65</v>
+        <v>1192.09</v>
       </c>
       <c r="H15" t="n">
-        <v>11199.79</v>
+        <v>17557.13</v>
       </c>
       <c r="I15" t="n">
-        <v>14221.44</v>
+        <v>18749.22</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,69 +975,69 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>116584.96</v>
+        <v>32782.12</v>
       </c>
       <c r="M15" t="n">
-        <v>116584.96</v>
+        <v>32782.12</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>3021.65</v>
       </c>
       <c r="H16" t="n">
-        <v>13639.66</v>
+        <v>11199.79</v>
       </c>
       <c r="I16" t="n">
-        <v>13639.66</v>
+        <v>14221.44</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>1742.84</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>120462.83</v>
+        <v>116584.96</v>
       </c>
       <c r="M16" t="n">
-        <v>122205.67</v>
+        <v>116584.96</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,22 +1049,22 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>13535.98</v>
+        <v>13639.66</v>
       </c>
       <c r="I17" t="n">
-        <v>13535.98</v>
+        <v>13639.66</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>1742.84</v>
       </c>
       <c r="L17" t="n">
-        <v>39672.88</v>
+        <v>120462.83</v>
       </c>
       <c r="M17" t="n">
-        <v>39672.88</v>
+        <v>122205.67</v>
       </c>
     </row>
     <row r="18">
@@ -1531,13 +1531,13 @@
         <v>1</v>
       </c>
       <c r="K28" t="n">
-        <v>66840.31</v>
+        <v>65790.7</v>
       </c>
       <c r="L28" t="n">
         <v>92701.61</v>
       </c>
       <c r="M28" t="n">
-        <v>159541.92</v>
+        <v>158492.31</v>
       </c>
     </row>
     <row r="29">
@@ -1801,7 +1801,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,22 +1811,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G35" t="n">
-        <v>0</v>
+        <v>88.39</v>
       </c>
       <c r="H35" t="n">
-        <v>1806.57</v>
+        <v>2509.34</v>
       </c>
       <c r="I35" t="n">
-        <v>1806.57</v>
+        <v>2597.73</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>16259.14</v>
+        <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>16259.14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>1752.92</v>
+        <v>2488.66</v>
       </c>
       <c r="I36" t="n">
-        <v>1752.92</v>
+        <v>2488.66</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>11896.87</v>
+        <v>40755.88</v>
       </c>
       <c r="M36" t="n">
-        <v>11896.87</v>
+        <v>40755.88</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>1699.44</v>
+        <v>1806.57</v>
       </c>
       <c r="I37" t="n">
-        <v>1699.44</v>
+        <v>1806.57</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>8550.700000000001</v>
+        <v>16259.14</v>
       </c>
       <c r="M37" t="n">
-        <v>8550.700000000001</v>
+        <v>16259.14</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1952,10 +1952,10 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>1635.54</v>
+        <v>1752.92</v>
       </c>
       <c r="I38" t="n">
-        <v>1635.54</v>
+        <v>1752.92</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>10748.48</v>
+        <v>11896.87</v>
       </c>
       <c r="M38" t="n">
-        <v>10748.48</v>
+        <v>11896.87</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1995,10 +1995,10 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>1603.9</v>
+        <v>1699.44</v>
       </c>
       <c r="I39" t="n">
-        <v>1603.9</v>
+        <v>1699.44</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>0</v>
+        <v>8550.700000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>0</v>
+        <v>8550.700000000001</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2038,28 +2038,28 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>1075.86</v>
+        <v>1635.54</v>
       </c>
       <c r="I40" t="n">
-        <v>1075.86</v>
+        <v>1635.54</v>
       </c>
       <c r="J40" t="n">
         <v>1</v>
       </c>
       <c r="K40" t="n">
-        <v>1433.08</v>
+        <v>9900.389999999999</v>
       </c>
       <c r="L40" t="n">
-        <v>0</v>
+        <v>20648.87</v>
       </c>
       <c r="M40" t="n">
-        <v>1433.08</v>
+        <v>30549.26</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2081,10 +2081,10 @@
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>662.91</v>
+        <v>1603.9</v>
       </c>
       <c r="I41" t="n">
-        <v>662.91</v>
+        <v>1603.9</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>8746.040000000001</v>
+        <v>0</v>
       </c>
       <c r="M41" t="n">
-        <v>8746.040000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2124,38 +2124,38 @@
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>662.91</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>662.91</v>
       </c>
       <c r="J42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K42" t="n">
-        <v>8278.549999999999</v>
+        <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>24835.65</v>
+        <v>8746.040000000001</v>
       </c>
       <c r="M42" t="n">
-        <v>33114.2</v>
+        <v>8746.040000000001</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2176,29 +2176,29 @@
         <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>15585.09</v>
+        <v>8278.549999999999</v>
       </c>
       <c r="L43" t="n">
-        <v>71404.87</v>
+        <v>24835.65</v>
       </c>
       <c r="M43" t="n">
-        <v>86989.96000000001</v>
+        <v>33114.2</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2216,16 +2216,16 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K44" t="n">
-        <v>0</v>
+        <v>15585.09</v>
       </c>
       <c r="L44" t="n">
-        <v>43244.52</v>
+        <v>71404.87</v>
       </c>
       <c r="M44" t="n">
-        <v>43244.52</v>
+        <v>86989.96000000001</v>
       </c>
     </row>
     <row r="45">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-07-08 15:03)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M46"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>30 de junio de 2026</t>
+          <t>7 de julio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -468,44 +468,44 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>1421726.6</v>
+        <v>4665.02</v>
       </c>
       <c r="H4" t="n">
-        <v>21279.16</v>
+        <v>79155.34</v>
       </c>
       <c r="I4" t="n">
-        <v>1443005.76</v>
+        <v>83820.36</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>8629</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>131899.05</v>
+        <v>2310.6</v>
       </c>
       <c r="M4" t="n">
-        <v>140528.05</v>
+        <v>2310.6</v>
       </c>
     </row>
     <row r="5">
@@ -527,34 +527,34 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>308451.52</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>34008.43</v>
+        <v>19707.14</v>
       </c>
       <c r="I5" t="n">
-        <v>342459.95</v>
+        <v>19707.14</v>
       </c>
       <c r="J5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K5" t="n">
-        <v>5462.26</v>
+        <v>3925.94</v>
       </c>
       <c r="L5" t="n">
-        <v>138991.73</v>
+        <v>113630.58</v>
       </c>
       <c r="M5" t="n">
-        <v>144453.99</v>
+        <v>117556.52</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,40 +564,40 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>191362.05</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>28869.69</v>
+        <v>12104.18</v>
       </c>
       <c r="I6" t="n">
-        <v>220231.74</v>
+        <v>12104.18</v>
       </c>
       <c r="J6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>2140380.13</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>2183684.66</v>
+        <v>6978.13</v>
       </c>
       <c r="M6" t="n">
-        <v>4324064.79</v>
+        <v>6978.13</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -607,22 +607,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>6316.29</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>150173.18</v>
+        <v>8496.639999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>156489.47</v>
+        <v>8496.639999999999</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,16 +631,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>7694.63</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>7694.63</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,22 +650,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>63633.32</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>57507.18</v>
+        <v>7555.89</v>
       </c>
       <c r="I8" t="n">
-        <v>121140.5</v>
+        <v>7555.89</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,41 +674,41 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>92453.89999999999</v>
+        <v>54253.97</v>
       </c>
       <c r="M8" t="n">
-        <v>92453.89999999999</v>
+        <v>54253.97</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>96052.28</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>13444.1</v>
+        <v>5018.34</v>
       </c>
       <c r="I9" t="n">
-        <v>109496.38</v>
+        <v>5018.34</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,16 +717,16 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>52737.61</v>
+        <v>5468.7</v>
       </c>
       <c r="M9" t="n">
-        <v>52737.61</v>
+        <v>5468.7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -736,22 +736,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>52787.07</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>18449.48</v>
+        <v>4468.7</v>
       </c>
       <c r="I10" t="n">
-        <v>71236.55</v>
+        <v>4468.7</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,16 +760,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>48780.37</v>
+        <v>22506.75</v>
       </c>
       <c r="M10" t="n">
-        <v>48780.37</v>
+        <v>22506.75</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,65 +779,65 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>3925.24</v>
+        <v>-3232.45</v>
       </c>
       <c r="H11" t="n">
-        <v>51296.31</v>
+        <v>7580.21</v>
       </c>
       <c r="I11" t="n">
-        <v>55221.55</v>
+        <v>4347.76</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>23046.35</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>120151.02</v>
+        <v>29481.97</v>
       </c>
       <c r="M11" t="n">
-        <v>143197.37</v>
+        <v>29481.97</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>11380.54</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>39223.64</v>
+        <v>3199.93</v>
       </c>
       <c r="I12" t="n">
-        <v>50604.18</v>
+        <v>3199.93</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,16 +846,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>333287.1</v>
+        <v>34877.64</v>
       </c>
       <c r="M12" t="n">
-        <v>333287.1</v>
+        <v>34877.64</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,22 +865,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>11737.38</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>26357.78</v>
+        <v>2968.17</v>
       </c>
       <c r="I13" t="n">
-        <v>38095.16</v>
+        <v>2968.17</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -914,59 +914,59 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2445.34</v>
+      </c>
+      <c r="I14" t="n">
+        <v>2445.34</v>
+      </c>
+      <c r="J14" t="n">
         <v>1</v>
       </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
-        <v>33128.49</v>
-      </c>
-      <c r="I14" t="n">
-        <v>33128.49</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>73595.67</v>
       </c>
       <c r="L14" t="n">
-        <v>6246.02</v>
+        <v>15980.3</v>
       </c>
       <c r="M14" t="n">
-        <v>6246.02</v>
+        <v>89575.97</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>2073.34</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>26583.82</v>
+        <v>2418.28</v>
       </c>
       <c r="I15" t="n">
-        <v>28657.16</v>
+        <v>2418.28</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>22806.75</v>
+        <v>20971.42</v>
       </c>
       <c r="M15" t="n">
-        <v>22806.75</v>
+        <v>20971.42</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>94205</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>JOSE ALBERTO CORONADO ROSAS</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>27588.3</v>
+        <v>2391.83</v>
       </c>
       <c r="I16" t="n">
-        <v>27588.3</v>
+        <v>2391.83</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>18651.6</v>
       </c>
       <c r="M16" t="n">
-        <v>0</v>
+        <v>18651.6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>27415.26</v>
+        <v>2340.27</v>
       </c>
       <c r="I17" t="n">
-        <v>27415.26</v>
+        <v>2340.27</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>25651.43</v>
+        <v>3215.87</v>
       </c>
       <c r="M17" t="n">
-        <v>25651.43</v>
+        <v>3215.87</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,22 +1080,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>1188.91</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>17510.21</v>
+        <v>2181.42</v>
       </c>
       <c r="I18" t="n">
-        <v>18699.12</v>
+        <v>2181.42</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,16 +1104,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>32694.52</v>
+        <v>136368.48</v>
       </c>
       <c r="M18" t="n">
-        <v>32694.52</v>
+        <v>136368.48</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,40 +1123,40 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>3215.45</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>15344.85</v>
+        <v>2061.35</v>
       </c>
       <c r="I19" t="n">
-        <v>18560.3</v>
+        <v>2061.35</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>15543.45</v>
       </c>
       <c r="L19" t="n">
-        <v>134649.12</v>
+        <v>77925.53999999999</v>
       </c>
       <c r="M19" t="n">
-        <v>134649.12</v>
+        <v>93468.99000000001</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>18267.36</v>
+        <v>1784.16</v>
       </c>
       <c r="I20" t="n">
-        <v>18267.36</v>
+        <v>1784.16</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,16 +1190,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>71234.57000000001</v>
+        <v>348268.17</v>
       </c>
       <c r="M20" t="n">
-        <v>71234.57000000001</v>
+        <v>348268.17</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,22 +1209,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>16380.01</v>
+        <v>1774.15</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>16380.01</v>
+        <v>1774.15</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,16 +1233,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>49140.03</v>
+        <v>36313.01</v>
       </c>
       <c r="M21" t="n">
-        <v>49140.03</v>
+        <v>36313.01</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,40 +1252,40 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1761.99</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1761.99</v>
+      </c>
+      <c r="J22" t="n">
         <v>1</v>
       </c>
-      <c r="G22" t="n">
-        <v>3013.57</v>
-      </c>
-      <c r="H22" t="n">
-        <v>13228.03</v>
-      </c>
-      <c r="I22" t="n">
-        <v>16241.6</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0</v>
-      </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>23046.35</v>
       </c>
       <c r="L22" t="n">
-        <v>114215.26</v>
+        <v>123791.17</v>
       </c>
       <c r="M22" t="n">
-        <v>114215.26</v>
+        <v>146837.52</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,22 +1295,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>11392.35</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>4454.77</v>
+        <v>1761.99</v>
       </c>
       <c r="I23" t="n">
-        <v>15847.12</v>
+        <v>1761.99</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,26 +1319,26 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>18651.6</v>
+        <v>13206.35</v>
       </c>
       <c r="M23" t="n">
-        <v>18651.6</v>
+        <v>13206.35</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>13129.66</v>
+        <v>1748.24</v>
       </c>
       <c r="I24" t="n">
-        <v>13129.66</v>
+        <v>1748.24</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,16 +1362,16 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>5468.7</v>
+        <v>9075.540000000001</v>
       </c>
       <c r="M24" t="n">
-        <v>5468.7</v>
+        <v>9075.540000000001</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1393,10 +1393,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>10386.49</v>
+        <v>1738.36</v>
       </c>
       <c r="I25" t="n">
-        <v>10386.49</v>
+        <v>1738.36</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,16 +1405,16 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>29761.26</v>
+        <v>117962.13</v>
       </c>
       <c r="M25" t="n">
-        <v>29761.26</v>
+        <v>117962.13</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,22 +1424,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>5872.79</v>
+        <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>3900.83</v>
+        <v>1737.22</v>
       </c>
       <c r="I26" t="n">
-        <v>9773.620000000001</v>
+        <v>1737.22</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>64600.71</v>
+        <v>54969.92</v>
       </c>
       <c r="M26" t="n">
-        <v>64600.71</v>
+        <v>54969.92</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,28 +1479,28 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>8832.15</v>
+        <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>8832.15</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>4970.44</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>49140.03</v>
       </c>
       <c r="M27" t="n">
-        <v>4970.44</v>
+        <v>49140.03</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>8520.18</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>8520.18</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>20971.42</v>
+        <v>32694.52</v>
       </c>
       <c r="M28" t="n">
-        <v>20971.42</v>
+        <v>32694.52</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,22 +1553,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>1671.19</v>
+        <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>6825.8</v>
+        <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>8496.99</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,16 +1577,16 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>9618.290000000001</v>
+        <v>6832.95</v>
       </c>
       <c r="M29" t="n">
-        <v>9618.290000000001</v>
+        <v>6832.95</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>110105</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ROCIO YANETH OCHOA IBARRA</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>7398.71</v>
+        <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>7398.71</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>0</v>
+        <v>25651.43</v>
       </c>
       <c r="M30" t="n">
-        <v>0</v>
+        <v>25651.43</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,28 +1651,28 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>6969.14</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>6969.14</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>79150.32000000001</v>
+        <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>0</v>
+        <v>22806.75</v>
       </c>
       <c r="M31" t="n">
-        <v>79150.32000000001</v>
+        <v>22806.75</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1694,10 +1694,10 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>6240.56</v>
+        <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>6240.56</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,16 +1706,16 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>28868.4</v>
+        <v>16215.69</v>
       </c>
       <c r="M32" t="n">
-        <v>28868.4</v>
+        <v>16215.69</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,38 +1737,38 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>6064.17</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>6064.17</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>0</v>
+        <v>2140380.13</v>
       </c>
       <c r="L33" t="n">
-        <v>3588.95</v>
+        <v>2183684.66</v>
       </c>
       <c r="M33" t="n">
-        <v>3588.95</v>
+        <v>4324064.79</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>5544.33</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>5544.33</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,26 +1792,26 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>0</v>
+        <v>134156.01</v>
       </c>
       <c r="M34" t="n">
-        <v>0</v>
+        <v>134156.01</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>5322.02</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>5322.02</v>
+        <v>0</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>36742.58</v>
+        <v>6281.5</v>
       </c>
       <c r="M35" t="n">
-        <v>36742.58</v>
+        <v>6281.5</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,28 +1866,28 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>4276.44</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>4276.44</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>2341.38</v>
+        <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>10112.1</v>
+        <v>3043.1</v>
       </c>
       <c r="M36" t="n">
-        <v>12453.48</v>
+        <v>3043.1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>3510.4</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>3510.4</v>
+        <v>0</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>13923.3</v>
+        <v>35224.49</v>
       </c>
       <c r="M37" t="n">
-        <v>13923.3</v>
+        <v>35224.49</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1952,10 +1952,10 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>3389.81</v>
+        <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>3389.81</v>
+        <v>0</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>6832.95</v>
+        <v>9653.08</v>
       </c>
       <c r="M38" t="n">
-        <v>6832.95</v>
+        <v>9653.08</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1995,10 +1995,10 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>2968.17</v>
+        <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>2968.17</v>
+        <v>0</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>0</v>
+        <v>68501.49000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>0</v>
+        <v>68501.49000000001</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2038,10 +2038,10 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>2789.54</v>
+        <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>2789.54</v>
+        <v>0</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>10823.78</v>
+        <v>59518.06</v>
       </c>
       <c r="M40" t="n">
-        <v>10823.78</v>
+        <v>59518.06</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,22 +2069,22 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>88.15000000000001</v>
+        <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>2502.64</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>2590.79</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2093,26 +2093,26 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>0</v>
+        <v>92453.89999999999</v>
       </c>
       <c r="M41" t="n">
-        <v>0</v>
+        <v>92453.89999999999</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>63441</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2511</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2124,194 +2124,22 @@
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>2027.5</v>
+        <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>2027.5</v>
+        <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K42" t="n">
-        <v>15543.45</v>
+        <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>69186.56</v>
+        <v>3695.34</v>
       </c>
       <c r="M42" t="n">
-        <v>84730.00999999999</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>63441</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>2511</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" t="n">
-        <v>1847.67</v>
-      </c>
-      <c r="I43" t="n">
-        <v>1847.67</v>
-      </c>
-      <c r="J43" t="n">
-        <v>0</v>
-      </c>
-      <c r="K43" t="n">
-        <v>0</v>
-      </c>
-      <c r="L43" t="n">
         <v>3695.34</v>
-      </c>
-      <c r="M43" t="n">
-        <v>3695.34</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>112083</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>2043</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="n">
-        <v>0</v>
-      </c>
-      <c r="G44" t="n">
-        <v>0</v>
-      </c>
-      <c r="H44" t="n">
-        <v>1801.74</v>
-      </c>
-      <c r="I44" t="n">
-        <v>1801.74</v>
-      </c>
-      <c r="J44" t="n">
-        <v>0</v>
-      </c>
-      <c r="K44" t="n">
-        <v>0</v>
-      </c>
-      <c r="L44" t="n">
-        <v>16215.69</v>
-      </c>
-      <c r="M44" t="n">
-        <v>16215.69</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>116795</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>2043</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="n">
-        <v>0</v>
-      </c>
-      <c r="G45" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" t="n">
-        <v>1599.61</v>
-      </c>
-      <c r="I45" t="n">
-        <v>1599.61</v>
-      </c>
-      <c r="J45" t="n">
-        <v>0</v>
-      </c>
-      <c r="K45" t="n">
-        <v>0</v>
-      </c>
-      <c r="L45" t="n">
-        <v>0</v>
-      </c>
-      <c r="M45" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>115404</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>2043</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" t="n">
-        <v>661.14</v>
-      </c>
-      <c r="I46" t="n">
-        <v>661.14</v>
-      </c>
-      <c r="J46" t="n">
-        <v>0</v>
-      </c>
-      <c r="K46" t="n">
-        <v>0</v>
-      </c>
-      <c r="L46" t="n">
-        <v>8722.67</v>
-      </c>
-      <c r="M46" t="n">
-        <v>8722.67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-07-15 12:07)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>9 de julio de 2026</t>
+          <t>14 de julio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -468,7 +468,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -478,7 +478,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -487,13 +487,13 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>4665.02</v>
+        <v>4377.64</v>
       </c>
       <c r="H4" t="n">
-        <v>79155.34</v>
+        <v>87640.96000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>83820.36</v>
+        <v>92018.60000000001</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -502,16 +502,16 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>2310.6</v>
+        <v>8271.43</v>
       </c>
       <c r="M4" t="n">
-        <v>2310.6</v>
+        <v>8271.43</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -521,7 +521,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -530,13 +530,13 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>4377.64</v>
+        <v>4665.02</v>
       </c>
       <c r="H5" t="n">
-        <v>71663.37</v>
+        <v>79155.34</v>
       </c>
       <c r="I5" t="n">
-        <v>76041.00999999999</v>
+        <v>83820.36</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -545,10 +545,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>15980.3</v>
+        <v>2310.6</v>
       </c>
       <c r="M5" t="n">
-        <v>15980.3</v>
+        <v>2310.6</v>
       </c>
     </row>
     <row r="6">
@@ -576,10 +576,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>20232.35</v>
+        <v>22480.76</v>
       </c>
       <c r="I6" t="n">
-        <v>20232.35</v>
+        <v>22480.76</v>
       </c>
       <c r="J6" t="n">
         <v>2</v>
@@ -588,10 +588,10 @@
         <v>3925.94</v>
       </c>
       <c r="L6" t="n">
-        <v>111014</v>
+        <v>106740.25</v>
       </c>
       <c r="M6" t="n">
-        <v>114939.94</v>
+        <v>110666.19</v>
       </c>
     </row>
     <row r="7">
@@ -668,32 +668,32 @@
         <v>9483.780000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>1793.28</v>
       </c>
       <c r="L8" t="n">
-        <v>5468.7</v>
+        <v>25194.79</v>
       </c>
       <c r="M8" t="n">
-        <v>5468.7</v>
+        <v>26988.07</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -705,10 +705,10 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>8496.639999999999</v>
+        <v>9422.16</v>
       </c>
       <c r="I9" t="n">
-        <v>8496.639999999999</v>
+        <v>9422.16</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,16 +717,16 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>7694.63</v>
+        <v>124733.86</v>
       </c>
       <c r="M9" t="n">
-        <v>7694.63</v>
+        <v>124733.86</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,10 +748,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>7555.89</v>
+        <v>8496.639999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>7555.89</v>
+        <v>8496.639999999999</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,26 +760,26 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>54253.97</v>
+        <v>7694.63</v>
       </c>
       <c r="M10" t="n">
-        <v>54253.97</v>
+        <v>7694.63</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -791,10 +791,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>6236.42</v>
+        <v>8422.459999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>6236.42</v>
+        <v>8422.459999999999</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,26 +803,26 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>132467.7</v>
+        <v>341940.48</v>
       </c>
       <c r="M11" t="n">
-        <v>132467.7</v>
+        <v>341940.48</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>5224.69</v>
+        <v>8004.31</v>
       </c>
       <c r="I12" t="n">
-        <v>5224.69</v>
+        <v>8004.31</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,16 +846,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>114475.8</v>
+        <v>130699.81</v>
       </c>
       <c r="M12" t="n">
-        <v>114475.8</v>
+        <v>130699.81</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,10 +877,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>4785.92</v>
+        <v>7555.89</v>
       </c>
       <c r="I13" t="n">
-        <v>4785.92</v>
+        <v>7555.89</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -889,16 +889,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>345577.01</v>
+        <v>54253.97</v>
       </c>
       <c r="M13" t="n">
-        <v>345577.01</v>
+        <v>54253.97</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>4468.7</v>
+        <v>7489.86</v>
       </c>
       <c r="I14" t="n">
-        <v>4468.7</v>
+        <v>7489.86</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>22506.75</v>
+        <v>52093.59</v>
       </c>
       <c r="M14" t="n">
-        <v>22506.75</v>
+        <v>52093.59</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -960,13 +960,13 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>-3232.45</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>7580.21</v>
+        <v>5224.69</v>
       </c>
       <c r="I15" t="n">
-        <v>4347.76</v>
+        <v>5224.69</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>23815.2</v>
+        <v>114475.8</v>
       </c>
       <c r="M15" t="n">
-        <v>23815.2</v>
+        <v>114475.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>4023</v>
+        <v>4468.7</v>
       </c>
       <c r="I16" t="n">
-        <v>4023</v>
+        <v>4468.7</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,26 +1018,26 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>17020.43</v>
+        <v>22506.75</v>
       </c>
       <c r="M16" t="n">
-        <v>17020.43</v>
+        <v>22506.75</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1046,13 +1046,13 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>-3232.45</v>
       </c>
       <c r="H17" t="n">
-        <v>3199.93</v>
+        <v>7580.21</v>
       </c>
       <c r="I17" t="n">
-        <v>3199.93</v>
+        <v>4347.76</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>34877.64</v>
+        <v>23815.2</v>
       </c>
       <c r="M17" t="n">
-        <v>34877.64</v>
+        <v>23815.2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>2968.17</v>
+        <v>4023</v>
       </c>
       <c r="I18" t="n">
-        <v>2968.17</v>
+        <v>4023</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,10 +1104,10 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>17020.43</v>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>17020.43</v>
       </c>
     </row>
     <row r="19">
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>2418.28</v>
+        <v>3373.23</v>
       </c>
       <c r="I19" t="n">
-        <v>2418.28</v>
+        <v>3373.23</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1156,7 +1156,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,28 +1178,28 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>2340.27</v>
+        <v>3294.34</v>
       </c>
       <c r="I20" t="n">
-        <v>2340.27</v>
+        <v>3294.34</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>23046.35</v>
       </c>
       <c r="L20" t="n">
-        <v>3215.87</v>
+        <v>122258.85</v>
       </c>
       <c r="M20" t="n">
-        <v>3215.87</v>
+        <v>145305.2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,38 +1221,38 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>2061.35</v>
+        <v>3199.93</v>
       </c>
       <c r="I21" t="n">
-        <v>2061.35</v>
+        <v>3199.93</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>15543.45</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>77925.53999999999</v>
+        <v>34877.64</v>
       </c>
       <c r="M21" t="n">
-        <v>93468.99000000001</v>
+        <v>34877.64</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>1853.84</v>
+        <v>2968.17</v>
       </c>
       <c r="I22" t="n">
-        <v>1853.84</v>
+        <v>2968.17</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,16 +1276,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>132302.17</v>
+        <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>132302.17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,22 +1295,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>1774.15</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>2340.27</v>
       </c>
       <c r="I23" t="n">
-        <v>1774.15</v>
+        <v>2340.27</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,16 +1319,16 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>36313.01</v>
+        <v>3215.87</v>
       </c>
       <c r="M23" t="n">
-        <v>36313.01</v>
+        <v>3215.87</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,50 +1338,50 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>2142.19</v>
       </c>
       <c r="H24" t="n">
-        <v>1761.99</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>1761.99</v>
+        <v>2142.19</v>
       </c>
       <c r="J24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K24" t="n">
-        <v>23046.35</v>
+        <v>4880.95</v>
       </c>
       <c r="L24" t="n">
-        <v>123791.17</v>
+        <v>47128.14</v>
       </c>
       <c r="M24" t="n">
-        <v>146837.52</v>
+        <v>52009.09</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1393,10 +1393,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>1761.99</v>
+        <v>2061.35</v>
       </c>
       <c r="I25" t="n">
-        <v>1761.99</v>
+        <v>2061.35</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,16 +1405,16 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>13206.35</v>
+        <v>62382.09</v>
       </c>
       <c r="M25" t="n">
-        <v>13206.35</v>
+        <v>62382.09</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>1748.24</v>
+        <v>1801.74</v>
       </c>
       <c r="I26" t="n">
-        <v>1748.24</v>
+        <v>1801.74</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>9075.540000000001</v>
+        <v>14413.95</v>
       </c>
       <c r="M26" t="n">
-        <v>9075.540000000001</v>
+        <v>14413.95</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,40 +1467,40 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>1774.15</v>
       </c>
       <c r="H27" t="n">
-        <v>1737.22</v>
+        <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>1737.22</v>
+        <v>1774.15</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>20794.19</v>
       </c>
       <c r="L27" t="n">
-        <v>54969.92</v>
+        <v>36313.01</v>
       </c>
       <c r="M27" t="n">
-        <v>54969.92</v>
+        <v>57107.2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>1761.99</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>1761.99</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>49140.03</v>
+        <v>13206.35</v>
       </c>
       <c r="M28" t="n">
-        <v>49140.03</v>
+        <v>13206.35</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,38 +1565,38 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>1748.24</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>1748.24</v>
       </c>
       <c r="J29" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>7023.14</v>
+        <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>47128.14</v>
+        <v>9075.540000000001</v>
       </c>
       <c r="M29" t="n">
-        <v>54151.28</v>
+        <v>9075.540000000001</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1620,26 +1620,26 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>32694.52</v>
+        <v>49140.03</v>
       </c>
       <c r="M30" t="n">
-        <v>32694.52</v>
+        <v>49140.03</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>6832.95</v>
+        <v>32694.52</v>
       </c>
       <c r="M31" t="n">
-        <v>6832.95</v>
+        <v>32694.52</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1706,16 +1706,16 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>25651.43</v>
+        <v>6832.95</v>
       </c>
       <c r="M32" t="n">
-        <v>25651.43</v>
+        <v>6832.95</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1749,16 +1749,16 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>22806.75</v>
+        <v>25651.43</v>
       </c>
       <c r="M33" t="n">
-        <v>22806.75</v>
+        <v>25651.43</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1792,10 +1792,10 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>16215.69</v>
+        <v>22806.75</v>
       </c>
       <c r="M34" t="n">
-        <v>16215.69</v>
+        <v>22806.75</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-07-16 13:14)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>14 de julio de 2026</t>
+          <t>15 de julio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -640,17 +640,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -662,28 +662,28 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>9483.780000000001</v>
+        <v>10742.45</v>
       </c>
       <c r="I8" t="n">
-        <v>9483.780000000001</v>
+        <v>10742.45</v>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>1793.28</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>25194.79</v>
+        <v>339352.33</v>
       </c>
       <c r="M8" t="n">
-        <v>26988.07</v>
+        <v>339352.33</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -705,38 +705,38 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>9422.16</v>
+        <v>9483.780000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>9422.16</v>
+        <v>9483.780000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>1793.28</v>
       </c>
       <c r="L9" t="n">
-        <v>124733.86</v>
+        <v>25194.79</v>
       </c>
       <c r="M9" t="n">
-        <v>124733.86</v>
+        <v>26988.07</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,10 +748,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>8496.639999999999</v>
+        <v>9422.16</v>
       </c>
       <c r="I10" t="n">
-        <v>8496.639999999999</v>
+        <v>9422.16</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,16 +760,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>7694.63</v>
+        <v>124733.86</v>
       </c>
       <c r="M10" t="n">
-        <v>7694.63</v>
+        <v>124733.86</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -791,10 +791,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>8422.459999999999</v>
+        <v>8496.639999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>8422.459999999999</v>
+        <v>8496.639999999999</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,10 +803,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>341940.48</v>
+        <v>7694.63</v>
       </c>
       <c r="M11" t="n">
-        <v>341940.48</v>
+        <v>7694.63</v>
       </c>
     </row>
     <row r="12">
@@ -855,7 +855,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,28 +877,28 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>7555.89</v>
+        <v>7752.11</v>
       </c>
       <c r="I13" t="n">
-        <v>7555.89</v>
+        <v>7752.11</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>23046.35</v>
       </c>
       <c r="L13" t="n">
-        <v>54253.97</v>
+        <v>117801.08</v>
       </c>
       <c r="M13" t="n">
-        <v>54253.97</v>
+        <v>140847.43</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>7489.86</v>
+        <v>7555.89</v>
       </c>
       <c r="I14" t="n">
-        <v>7489.86</v>
+        <v>7555.89</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>52093.59</v>
+        <v>54253.97</v>
       </c>
       <c r="M14" t="n">
-        <v>52093.59</v>
+        <v>54253.97</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,38 +963,38 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>5224.69</v>
+        <v>7489.86</v>
       </c>
       <c r="I15" t="n">
-        <v>5224.69</v>
+        <v>7489.86</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>43237.93</v>
       </c>
       <c r="L15" t="n">
-        <v>114475.8</v>
+        <v>52093.59</v>
       </c>
       <c r="M15" t="n">
-        <v>114475.8</v>
+        <v>95331.52</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>4468.7</v>
+        <v>6382.31</v>
       </c>
       <c r="I16" t="n">
-        <v>4468.7</v>
+        <v>6382.31</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>22506.75</v>
+        <v>20971.42</v>
       </c>
       <c r="M16" t="n">
-        <v>22506.75</v>
+        <v>20971.42</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1046,13 +1046,13 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>-3232.45</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>7580.21</v>
+        <v>5224.69</v>
       </c>
       <c r="I17" t="n">
-        <v>4347.76</v>
+        <v>5224.69</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>23815.2</v>
+        <v>114475.8</v>
       </c>
       <c r="M17" t="n">
-        <v>23815.2</v>
+        <v>114475.8</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>4023</v>
+        <v>4745.85</v>
       </c>
       <c r="I18" t="n">
-        <v>4023</v>
+        <v>4745.85</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,26 +1104,26 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>17020.43</v>
+        <v>88137.78999999999</v>
       </c>
       <c r="M18" t="n">
-        <v>17020.43</v>
+        <v>88137.78999999999</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>3373.23</v>
+        <v>4468.7</v>
       </c>
       <c r="I19" t="n">
-        <v>3373.23</v>
+        <v>4468.7</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,16 +1147,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>20971.42</v>
+        <v>22506.75</v>
       </c>
       <c r="M19" t="n">
-        <v>20971.42</v>
+        <v>22506.75</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1175,41 +1175,41 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>-3232.45</v>
       </c>
       <c r="H20" t="n">
-        <v>3294.34</v>
+        <v>7580.21</v>
       </c>
       <c r="I20" t="n">
-        <v>3294.34</v>
+        <v>4347.76</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>23046.35</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>122258.85</v>
+        <v>23815.2</v>
       </c>
       <c r="M20" t="n">
-        <v>145305.2</v>
+        <v>23815.2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,38 +1221,38 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>3199.93</v>
+        <v>4023</v>
       </c>
       <c r="I21" t="n">
-        <v>3199.93</v>
+        <v>4023</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>33210.52</v>
       </c>
       <c r="L21" t="n">
-        <v>34877.64</v>
+        <v>17020.43</v>
       </c>
       <c r="M21" t="n">
-        <v>34877.64</v>
+        <v>50230.95</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>2968.17</v>
+        <v>3199.93</v>
       </c>
       <c r="I22" t="n">
-        <v>2968.17</v>
+        <v>3199.93</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,16 +1276,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>34877.64</v>
       </c>
       <c r="M22" t="n">
-        <v>0</v>
+        <v>34877.64</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,10 +1307,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>2340.27</v>
+        <v>2968.17</v>
       </c>
       <c r="I23" t="n">
-        <v>2340.27</v>
+        <v>2968.17</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,16 +1319,16 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>3215.87</v>
+        <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>3215.87</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,93 +1338,93 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>2142.19</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>2340.27</v>
       </c>
       <c r="I24" t="n">
-        <v>2142.19</v>
+        <v>2340.27</v>
       </c>
       <c r="J24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>4880.95</v>
+        <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>47128.14</v>
+        <v>3215.87</v>
       </c>
       <c r="M24" t="n">
-        <v>52009.09</v>
+        <v>3215.87</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>2142.19</v>
       </c>
       <c r="H25" t="n">
-        <v>2061.35</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>2061.35</v>
+        <v>2142.19</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>4880.95</v>
       </c>
       <c r="L25" t="n">
-        <v>62382.09</v>
+        <v>47128.14</v>
       </c>
       <c r="M25" t="n">
-        <v>62382.09</v>
+        <v>52009.09</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>1801.74</v>
+        <v>2061.35</v>
       </c>
       <c r="I26" t="n">
-        <v>1801.74</v>
+        <v>2061.35</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>14413.95</v>
+        <v>62382.09</v>
       </c>
       <c r="M26" t="n">
-        <v>14413.95</v>
+        <v>62382.09</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,40 +1467,40 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>1774.15</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>1801.74</v>
       </c>
       <c r="I27" t="n">
-        <v>1774.15</v>
+        <v>1801.74</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>20794.19</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>36313.01</v>
+        <v>14413.95</v>
       </c>
       <c r="M27" t="n">
-        <v>57107.2</v>
+        <v>14413.95</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,40 +1510,40 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>1774.15</v>
       </c>
       <c r="H28" t="n">
-        <v>1761.99</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>1761.99</v>
+        <v>1774.15</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>20794.19</v>
       </c>
       <c r="L28" t="n">
-        <v>13206.35</v>
+        <v>36313.01</v>
       </c>
       <c r="M28" t="n">
-        <v>13206.35</v>
+        <v>57107.2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>1748.24</v>
+        <v>1761.99</v>
       </c>
       <c r="I29" t="n">
-        <v>1748.24</v>
+        <v>1761.99</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,16 +1577,16 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>9075.540000000001</v>
+        <v>13206.35</v>
       </c>
       <c r="M29" t="n">
-        <v>9075.540000000001</v>
+        <v>13206.35</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>1748.24</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>1748.24</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,10 +1620,10 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>49140.03</v>
+        <v>9075.540000000001</v>
       </c>
       <c r="M30" t="n">
-        <v>49140.03</v>
+        <v>9075.540000000001</v>
       </c>
     </row>
     <row r="31">
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>1663.43</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>1663.43</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>32694.52</v>
+        <v>31031.09</v>
       </c>
       <c r="M31" t="n">
-        <v>32694.52</v>
+        <v>31031.09</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1706,16 +1706,16 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>6832.95</v>
+        <v>49140.03</v>
       </c>
       <c r="M32" t="n">
-        <v>6832.95</v>
+        <v>49140.03</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1749,16 +1749,16 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>25651.43</v>
+        <v>6832.95</v>
       </c>
       <c r="M33" t="n">
-        <v>25651.43</v>
+        <v>6832.95</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1792,16 +1792,16 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>22806.75</v>
+        <v>25651.43</v>
       </c>
       <c r="M34" t="n">
-        <v>22806.75</v>
+        <v>25651.43</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1829,22 +1829,22 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>2140380.13</v>
+        <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>2183684.66</v>
+        <v>22806.75</v>
       </c>
       <c r="M35" t="n">
-        <v>4324064.79</v>
+        <v>22806.75</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1872,22 +1872,22 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>2140380.13</v>
       </c>
       <c r="L36" t="n">
-        <v>6281.5</v>
+        <v>2183684.66</v>
       </c>
       <c r="M36" t="n">
-        <v>6281.5</v>
+        <v>4324064.79</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>3043.1</v>
+        <v>6281.5</v>
       </c>
       <c r="M37" t="n">
-        <v>3043.1</v>
+        <v>6281.5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>28176.54</v>
+        <v>3043.1</v>
       </c>
       <c r="M38" t="n">
-        <v>28176.54</v>
+        <v>3043.1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>9653.08</v>
+        <v>28176.54</v>
       </c>
       <c r="M39" t="n">
-        <v>9653.08</v>
+        <v>28176.54</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>68501.49000000001</v>
+        <v>9653.08</v>
       </c>
       <c r="M40" t="n">
-        <v>68501.49000000001</v>
+        <v>9653.08</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>59518.06</v>
+        <v>68501.49000000001</v>
       </c>
       <c r="M41" t="n">
-        <v>59518.06</v>
+        <v>68501.49000000001</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2136,10 +2136,10 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>92453.89999999999</v>
+        <v>59518.06</v>
       </c>
       <c r="M42" t="n">
-        <v>92453.89999999999</v>
+        <v>59518.06</v>
       </c>
     </row>
     <row r="43">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-07-20 12:11)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>15 de julio de 2026</t>
+          <t>17 de julio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -468,7 +468,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -478,7 +478,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -487,13 +487,13 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>4377.64</v>
+        <v>4665.02</v>
       </c>
       <c r="H4" t="n">
-        <v>87640.96000000001</v>
+        <v>79155.34</v>
       </c>
       <c r="I4" t="n">
-        <v>92018.60000000001</v>
+        <v>83820.36</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -502,26 +502,26 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>8271.43</v>
+        <v>2310.6</v>
       </c>
       <c r="M4" t="n">
-        <v>8271.43</v>
+        <v>2310.6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -530,13 +530,13 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>4665.02</v>
+        <v>56273.13</v>
       </c>
       <c r="H5" t="n">
-        <v>79155.34</v>
+        <v>1663.43</v>
       </c>
       <c r="I5" t="n">
-        <v>83820.36</v>
+        <v>57936.56</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -545,16 +545,16 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>2310.6</v>
+        <v>31031.09</v>
       </c>
       <c r="M5" t="n">
-        <v>2310.6</v>
+        <v>31031.09</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,40 +564,40 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>4019.13</v>
       </c>
       <c r="H6" t="n">
-        <v>22480.76</v>
+        <v>48439.14</v>
       </c>
       <c r="I6" t="n">
-        <v>22480.76</v>
+        <v>52458.27</v>
       </c>
       <c r="J6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>3925.94</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>106740.25</v>
+        <v>50355.05</v>
       </c>
       <c r="M6" t="n">
-        <v>110666.19</v>
+        <v>50355.05</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -619,28 +619,28 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>12104.18</v>
+        <v>22480.76</v>
       </c>
       <c r="I7" t="n">
-        <v>12104.18</v>
+        <v>22480.76</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>3925.94</v>
       </c>
       <c r="L7" t="n">
-        <v>6978.13</v>
+        <v>106740.25</v>
       </c>
       <c r="M7" t="n">
-        <v>6978.13</v>
+        <v>110666.19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -662,10 +662,10 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>10742.45</v>
+        <v>19439.59</v>
       </c>
       <c r="I8" t="n">
-        <v>10742.45</v>
+        <v>19439.59</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,26 +674,26 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>339352.33</v>
+        <v>8271.43</v>
       </c>
       <c r="M8" t="n">
-        <v>339352.33</v>
+        <v>8271.43</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -705,38 +705,38 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>9483.780000000001</v>
+        <v>15796.53</v>
       </c>
       <c r="I9" t="n">
-        <v>9483.780000000001</v>
+        <v>15796.53</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>1793.28</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>25194.79</v>
+        <v>103903.95</v>
       </c>
       <c r="M9" t="n">
-        <v>26988.07</v>
+        <v>103903.95</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,28 +748,28 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>9422.16</v>
+        <v>14925.31</v>
       </c>
       <c r="I10" t="n">
-        <v>9422.16</v>
+        <v>14925.31</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>23046.35</v>
       </c>
       <c r="L10" t="n">
-        <v>124733.86</v>
+        <v>110627.88</v>
       </c>
       <c r="M10" t="n">
-        <v>124733.86</v>
+        <v>133674.23</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -791,10 +791,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>8496.639999999999</v>
+        <v>12104.18</v>
       </c>
       <c r="I11" t="n">
-        <v>8496.639999999999</v>
+        <v>12104.18</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,16 +803,16 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>7694.63</v>
+        <v>6978.13</v>
       </c>
       <c r="M11" t="n">
-        <v>7694.63</v>
+        <v>6978.13</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>8004.31</v>
+        <v>11221.61</v>
       </c>
       <c r="I12" t="n">
-        <v>8004.31</v>
+        <v>11221.61</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,16 +846,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>130699.81</v>
+        <v>122934.4</v>
       </c>
       <c r="M12" t="n">
-        <v>130699.81</v>
+        <v>122934.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,22 +877,22 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>7752.11</v>
+        <v>10742.45</v>
       </c>
       <c r="I13" t="n">
-        <v>7752.11</v>
+        <v>10742.45</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>23046.35</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>117801.08</v>
+        <v>339352.33</v>
       </c>
       <c r="M13" t="n">
-        <v>140847.43</v>
+        <v>339352.33</v>
       </c>
     </row>
     <row r="14">
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>7555.89</v>
+        <v>10556.59</v>
       </c>
       <c r="I14" t="n">
-        <v>7555.89</v>
+        <v>10556.59</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>54253.97</v>
+        <v>51253.23</v>
       </c>
       <c r="M14" t="n">
-        <v>54253.97</v>
+        <v>51253.23</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,28 +963,28 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>7489.86</v>
+        <v>9773.620000000001</v>
       </c>
       <c r="I15" t="n">
-        <v>7489.86</v>
+        <v>9773.620000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>43237.93</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>52093.59</v>
+        <v>58727.91</v>
       </c>
       <c r="M15" t="n">
-        <v>95331.52</v>
+        <v>58727.91</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,28 +1006,28 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>6382.31</v>
+        <v>9483.780000000001</v>
       </c>
       <c r="I16" t="n">
-        <v>6382.31</v>
+        <v>9483.780000000001</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>1793.28</v>
       </c>
       <c r="L16" t="n">
-        <v>20971.42</v>
+        <v>25194.79</v>
       </c>
       <c r="M16" t="n">
-        <v>20971.42</v>
+        <v>26988.07</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1046,13 +1046,13 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>-3232.45</v>
       </c>
       <c r="H17" t="n">
-        <v>5224.69</v>
+        <v>12516.83</v>
       </c>
       <c r="I17" t="n">
-        <v>5224.69</v>
+        <v>9284.379999999999</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>114475.8</v>
+        <v>18405.23</v>
       </c>
       <c r="M17" t="n">
-        <v>114475.8</v>
+        <v>18405.23</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>4745.85</v>
+        <v>8496.639999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>4745.85</v>
+        <v>8496.639999999999</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,16 +1104,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>88137.78999999999</v>
+        <v>7694.63</v>
       </c>
       <c r="M18" t="n">
-        <v>88137.78999999999</v>
+        <v>7694.63</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>4468.7</v>
+        <v>8394.559999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>4468.7</v>
+        <v>8394.559999999999</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,26 +1147,26 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>22506.75</v>
+        <v>88137.78999999999</v>
       </c>
       <c r="M19" t="n">
-        <v>22506.75</v>
+        <v>88137.78999999999</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1175,31 +1175,31 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>-3232.45</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>7580.21</v>
+        <v>8004.31</v>
       </c>
       <c r="I20" t="n">
-        <v>4347.76</v>
+        <v>8004.31</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>2535.92</v>
       </c>
       <c r="L20" t="n">
-        <v>23815.2</v>
+        <v>130699.81</v>
       </c>
       <c r="M20" t="n">
-        <v>23815.2</v>
+        <v>133235.73</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,40 +1209,40 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>5863.45</v>
       </c>
       <c r="H21" t="n">
-        <v>4023</v>
+        <v>1160.7</v>
       </c>
       <c r="I21" t="n">
-        <v>4023</v>
+        <v>7024.15</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>33210.52</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>17020.43</v>
+        <v>47128.14</v>
       </c>
       <c r="M21" t="n">
-        <v>50230.95</v>
+        <v>47128.14</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>3199.93</v>
+        <v>6382.31</v>
       </c>
       <c r="I22" t="n">
-        <v>3199.93</v>
+        <v>6382.31</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,16 +1276,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>34877.64</v>
+        <v>20971.42</v>
       </c>
       <c r="M22" t="n">
-        <v>34877.64</v>
+        <v>20971.42</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,10 +1307,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>2968.17</v>
+        <v>6064.17</v>
       </c>
       <c r="I23" t="n">
-        <v>2968.17</v>
+        <v>6064.17</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,16 +1319,16 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>3588.95</v>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>3588.95</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>110105</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>ROCIO YANETH OCHOA IBARRA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>2340.27</v>
+        <v>5255.37</v>
       </c>
       <c r="I24" t="n">
-        <v>2340.27</v>
+        <v>5255.37</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,69 +1362,69 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>3215.87</v>
+        <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>3215.87</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>2142.19</v>
+        <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>4981.93</v>
       </c>
       <c r="I25" t="n">
-        <v>2142.19</v>
+        <v>4981.93</v>
       </c>
       <c r="J25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>4880.95</v>
+        <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>47128.14</v>
+        <v>33095.64</v>
       </c>
       <c r="M25" t="n">
-        <v>52009.09</v>
+        <v>33095.64</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>2061.35</v>
+        <v>4468.7</v>
       </c>
       <c r="I26" t="n">
-        <v>2061.35</v>
+        <v>4468.7</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>62382.09</v>
+        <v>22506.75</v>
       </c>
       <c r="M26" t="n">
-        <v>62382.09</v>
+        <v>22506.75</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,28 +1479,28 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>1801.74</v>
+        <v>4023</v>
       </c>
       <c r="I27" t="n">
-        <v>1801.74</v>
+        <v>4023</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>33210.52</v>
       </c>
       <c r="L27" t="n">
-        <v>14413.95</v>
+        <v>17020.43</v>
       </c>
       <c r="M27" t="n">
-        <v>14413.95</v>
+        <v>50230.95</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,40 +1510,40 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>1774.15</v>
+        <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>2968.17</v>
       </c>
       <c r="I28" t="n">
-        <v>1774.15</v>
+        <v>2968.17</v>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>20794.19</v>
+        <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>36313.01</v>
+        <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>57107.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>1761.99</v>
+        <v>2340.27</v>
       </c>
       <c r="I29" t="n">
-        <v>1761.99</v>
+        <v>2340.27</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,26 +1577,26 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>13206.35</v>
+        <v>3215.87</v>
       </c>
       <c r="M29" t="n">
-        <v>13206.35</v>
+        <v>3215.87</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>1748.24</v>
+        <v>2061.35</v>
       </c>
       <c r="I30" t="n">
-        <v>1748.24</v>
+        <v>2061.35</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,26 +1620,26 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>9075.540000000001</v>
+        <v>62382.09</v>
       </c>
       <c r="M30" t="n">
-        <v>9075.540000000001</v>
+        <v>62382.09</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>1663.43</v>
+        <v>1801.74</v>
       </c>
       <c r="I31" t="n">
-        <v>1663.43</v>
+        <v>1801.74</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>31031.09</v>
+        <v>14413.95</v>
       </c>
       <c r="M31" t="n">
-        <v>31031.09</v>
+        <v>14413.95</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,40 +1682,40 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>1774.15</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>1774.15</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K32" t="n">
-        <v>0</v>
+        <v>20794.19</v>
       </c>
       <c r="L32" t="n">
-        <v>49140.03</v>
+        <v>36313.01</v>
       </c>
       <c r="M32" t="n">
-        <v>49140.03</v>
+        <v>57107.2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>1761.99</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>1761.99</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,16 +1749,16 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>6832.95</v>
+        <v>10864.97</v>
       </c>
       <c r="M33" t="n">
-        <v>6832.95</v>
+        <v>10864.97</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>1748.24</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>1748.24</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,16 +1792,16 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>25651.43</v>
+        <v>9075.540000000001</v>
       </c>
       <c r="M34" t="n">
-        <v>25651.43</v>
+        <v>9075.540000000001</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>22806.75</v>
+        <v>49140.03</v>
       </c>
       <c r="M35" t="n">
-        <v>22806.75</v>
+        <v>49140.03</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1872,22 +1872,22 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>2140380.13</v>
+        <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>2183684.66</v>
+        <v>6832.95</v>
       </c>
       <c r="M36" t="n">
-        <v>4324064.79</v>
+        <v>6832.95</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>6281.5</v>
+        <v>25651.43</v>
       </c>
       <c r="M37" t="n">
-        <v>6281.5</v>
+        <v>25651.43</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>3043.1</v>
+        <v>22806.75</v>
       </c>
       <c r="M38" t="n">
-        <v>3043.1</v>
+        <v>22806.75</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>2140380.13</v>
       </c>
       <c r="L39" t="n">
-        <v>28176.54</v>
+        <v>2183684.66</v>
       </c>
       <c r="M39" t="n">
-        <v>28176.54</v>
+        <v>4324064.79</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>9653.08</v>
+        <v>6281.5</v>
       </c>
       <c r="M40" t="n">
-        <v>9653.08</v>
+        <v>6281.5</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>68501.49000000001</v>
+        <v>3043.1</v>
       </c>
       <c r="M41" t="n">
-        <v>68501.49000000001</v>
+        <v>3043.1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2136,26 +2136,26 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>59518.06</v>
+        <v>28176.54</v>
       </c>
       <c r="M42" t="n">
-        <v>59518.06</v>
+        <v>28176.54</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>63441</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2173,15 +2173,58 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>0</v>
+        <v>57661.97</v>
       </c>
       <c r="L43" t="n">
+        <v>59518.06</v>
+      </c>
+      <c r="M43" t="n">
+        <v>117180.03</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>63441</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2511</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" t="n">
         <v>3695.34</v>
       </c>
-      <c r="M43" t="n">
+      <c r="M44" t="n">
         <v>3695.34</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: Actualización de Camino a la Cumbre, Proactiva Tech, MDRT y Pagos Pendientes (2026-07-20)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>17 de julio de 2026</t>
+          <t>20 de julio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -576,10 +576,10 @@
         <v>4019.13</v>
       </c>
       <c r="H6" t="n">
-        <v>48439.14</v>
+        <v>51315.46</v>
       </c>
       <c r="I6" t="n">
-        <v>52458.27</v>
+        <v>55334.59</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -705,10 +705,10 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>15796.53</v>
+        <v>18810.1</v>
       </c>
       <c r="I9" t="n">
-        <v>15796.53</v>
+        <v>18810.1</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,10 +717,10 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>103903.95</v>
+        <v>100890.38</v>
       </c>
       <c r="M9" t="n">
-        <v>103903.95</v>
+        <v>100890.38</v>
       </c>
     </row>
     <row r="10">
@@ -748,28 +748,28 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>14925.31</v>
+        <v>16663.14</v>
       </c>
       <c r="I10" t="n">
-        <v>14925.31</v>
+        <v>16663.14</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>23046.35</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>110627.88</v>
+        <v>85843.7</v>
       </c>
       <c r="M10" t="n">
-        <v>133674.23</v>
+        <v>85843.7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -788,13 +788,13 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>-3232.45</v>
       </c>
       <c r="H11" t="n">
-        <v>12104.18</v>
+        <v>17991</v>
       </c>
       <c r="I11" t="n">
-        <v>12104.18</v>
+        <v>14758.55</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,26 +803,26 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>6978.13</v>
+        <v>12931.03</v>
       </c>
       <c r="M11" t="n">
-        <v>6978.13</v>
+        <v>12931.03</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>11221.61</v>
+        <v>12104.18</v>
       </c>
       <c r="I12" t="n">
-        <v>11221.61</v>
+        <v>12104.18</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,26 +846,26 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>122934.4</v>
+        <v>6978.13</v>
       </c>
       <c r="M12" t="n">
-        <v>122934.4</v>
+        <v>6978.13</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,10 +877,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>10742.45</v>
+        <v>11221.61</v>
       </c>
       <c r="I13" t="n">
-        <v>10742.45</v>
+        <v>11221.61</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -889,16 +889,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>339352.33</v>
+        <v>122934.4</v>
       </c>
       <c r="M13" t="n">
-        <v>339352.33</v>
+        <v>122934.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>10556.59</v>
+        <v>10742.45</v>
       </c>
       <c r="I14" t="n">
-        <v>10556.59</v>
+        <v>10742.45</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>51253.23</v>
+        <v>339352.33</v>
       </c>
       <c r="M14" t="n">
-        <v>51253.23</v>
+        <v>339352.33</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>9773.620000000001</v>
+        <v>10556.59</v>
       </c>
       <c r="I15" t="n">
-        <v>9773.620000000001</v>
+        <v>10556.59</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,26 +975,26 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>58727.91</v>
+        <v>51253.23</v>
       </c>
       <c r="M15" t="n">
-        <v>58727.91</v>
+        <v>51253.23</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,28 +1006,28 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>9483.780000000001</v>
+        <v>10152.32</v>
       </c>
       <c r="I16" t="n">
-        <v>9483.780000000001</v>
+        <v>10152.32</v>
       </c>
       <c r="J16" t="n">
         <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>1793.28</v>
+        <v>57661.97</v>
       </c>
       <c r="L16" t="n">
-        <v>25194.79</v>
+        <v>52737.61</v>
       </c>
       <c r="M16" t="n">
-        <v>26988.07</v>
+        <v>110399.58</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1046,13 +1046,13 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>-3232.45</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>12516.83</v>
+        <v>9773.620000000001</v>
       </c>
       <c r="I17" t="n">
-        <v>9284.379999999999</v>
+        <v>9773.620000000001</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,26 +1061,26 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>18405.23</v>
+        <v>58727.91</v>
       </c>
       <c r="M17" t="n">
-        <v>18405.23</v>
+        <v>58727.91</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,28 +1092,28 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>8496.639999999999</v>
+        <v>9483.780000000001</v>
       </c>
       <c r="I18" t="n">
-        <v>8496.639999999999</v>
+        <v>9483.780000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>1793.28</v>
       </c>
       <c r="L18" t="n">
-        <v>7694.63</v>
+        <v>25194.79</v>
       </c>
       <c r="M18" t="n">
-        <v>7694.63</v>
+        <v>26988.07</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>8394.559999999999</v>
+        <v>8496.639999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>8394.559999999999</v>
+        <v>8496.639999999999</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,26 +1147,26 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>88137.78999999999</v>
+        <v>7694.63</v>
       </c>
       <c r="M19" t="n">
-        <v>88137.78999999999</v>
+        <v>7694.63</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,96 +1178,96 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>8004.31</v>
+        <v>8394.559999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>8004.31</v>
+        <v>8394.559999999999</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>2535.92</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>130699.81</v>
+        <v>88137.78999999999</v>
       </c>
       <c r="M20" t="n">
-        <v>133235.73</v>
+        <v>88137.78999999999</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>5863.45</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>1160.7</v>
+        <v>8004.31</v>
       </c>
       <c r="I21" t="n">
-        <v>7024.15</v>
+        <v>8004.31</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>2535.92</v>
       </c>
       <c r="L21" t="n">
-        <v>47128.14</v>
+        <v>130699.81</v>
       </c>
       <c r="M21" t="n">
-        <v>47128.14</v>
+        <v>133235.73</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>5863.45</v>
       </c>
       <c r="H22" t="n">
-        <v>6382.31</v>
+        <v>1160.7</v>
       </c>
       <c r="I22" t="n">
-        <v>6382.31</v>
+        <v>7024.15</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,26 +1276,26 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>20971.42</v>
+        <v>47128.14</v>
       </c>
       <c r="M22" t="n">
-        <v>20971.42</v>
+        <v>47128.14</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,10 +1307,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>6064.17</v>
+        <v>6382.31</v>
       </c>
       <c r="I23" t="n">
-        <v>6064.17</v>
+        <v>6382.31</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,16 +1319,16 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>3588.95</v>
+        <v>20971.42</v>
       </c>
       <c r="M23" t="n">
-        <v>3588.95</v>
+        <v>20971.42</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>110105</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ROCIO YANETH OCHOA IBARRA</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>5255.37</v>
+        <v>6064.17</v>
       </c>
       <c r="I24" t="n">
-        <v>5255.37</v>
+        <v>6064.17</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,59 +1362,59 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>3588.95</v>
       </c>
       <c r="M24" t="n">
-        <v>0</v>
+        <v>3588.95</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>1774.15</v>
       </c>
       <c r="H25" t="n">
-        <v>4981.93</v>
+        <v>3682.12</v>
       </c>
       <c r="I25" t="n">
-        <v>4981.93</v>
+        <v>5456.27</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>20794.19</v>
       </c>
       <c r="L25" t="n">
-        <v>33095.64</v>
+        <v>30935.53</v>
       </c>
       <c r="M25" t="n">
-        <v>33095.64</v>
+        <v>51729.72</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>110105</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>ROCIO YANETH OCHOA IBARRA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>4468.7</v>
+        <v>5255.37</v>
       </c>
       <c r="I26" t="n">
-        <v>4468.7</v>
+        <v>5255.37</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,26 +1448,26 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>22506.75</v>
+        <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>22506.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,28 +1479,28 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>4023</v>
+        <v>4981.93</v>
       </c>
       <c r="I27" t="n">
-        <v>4023</v>
+        <v>4981.93</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>33210.52</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>17020.43</v>
+        <v>33095.64</v>
       </c>
       <c r="M27" t="n">
-        <v>50230.95</v>
+        <v>33095.64</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>2968.17</v>
+        <v>4468.7</v>
       </c>
       <c r="I28" t="n">
-        <v>2968.17</v>
+        <v>4468.7</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>0</v>
+        <v>22506.75</v>
       </c>
       <c r="M28" t="n">
-        <v>0</v>
+        <v>22506.75</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,38 +1565,38 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>2340.27</v>
+        <v>4023</v>
       </c>
       <c r="I29" t="n">
-        <v>2340.27</v>
+        <v>4023</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>33210.52</v>
       </c>
       <c r="L29" t="n">
-        <v>3215.87</v>
+        <v>17020.43</v>
       </c>
       <c r="M29" t="n">
-        <v>3215.87</v>
+        <v>50230.95</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>2061.35</v>
+        <v>2968.17</v>
       </c>
       <c r="I30" t="n">
-        <v>2061.35</v>
+        <v>2968.17</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>62382.09</v>
+        <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>62382.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>1801.74</v>
+        <v>2340.27</v>
       </c>
       <c r="I31" t="n">
-        <v>1801.74</v>
+        <v>2340.27</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>14413.95</v>
+        <v>3215.87</v>
       </c>
       <c r="M31" t="n">
-        <v>14413.95</v>
+        <v>3215.87</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,50 +1682,50 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>1774.15</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>2073.34</v>
       </c>
       <c r="I32" t="n">
-        <v>1774.15</v>
+        <v>2073.34</v>
       </c>
       <c r="J32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>20794.19</v>
+        <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>36313.01</v>
+        <v>20733.41</v>
       </c>
       <c r="M32" t="n">
-        <v>57107.2</v>
+        <v>20733.41</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>1761.99</v>
+        <v>2061.35</v>
       </c>
       <c r="I33" t="n">
-        <v>1761.99</v>
+        <v>2061.35</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,16 +1749,16 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>10864.97</v>
+        <v>62382.09</v>
       </c>
       <c r="M33" t="n">
-        <v>10864.97</v>
+        <v>62382.09</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>1748.24</v>
+        <v>1801.74</v>
       </c>
       <c r="I34" t="n">
-        <v>1748.24</v>
+        <v>1801.74</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,16 +1792,16 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>9075.540000000001</v>
+        <v>14413.95</v>
       </c>
       <c r="M34" t="n">
-        <v>9075.540000000001</v>
+        <v>14413.95</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>1761.99</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>1761.99</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>49140.03</v>
+        <v>10864.97</v>
       </c>
       <c r="M35" t="n">
-        <v>49140.03</v>
+        <v>10864.97</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>1748.24</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>1748.24</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>6832.95</v>
+        <v>9075.540000000001</v>
       </c>
       <c r="M36" t="n">
-        <v>6832.95</v>
+        <v>9075.540000000001</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>25651.43</v>
+        <v>49140.03</v>
       </c>
       <c r="M37" t="n">
-        <v>25651.43</v>
+        <v>49140.03</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>22806.75</v>
+        <v>6832.95</v>
       </c>
       <c r="M38" t="n">
-        <v>22806.75</v>
+        <v>6832.95</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>2140380.13</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>2183684.66</v>
+        <v>25651.43</v>
       </c>
       <c r="M39" t="n">
-        <v>4324064.79</v>
+        <v>25651.43</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2044,22 +2044,22 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K40" t="n">
-        <v>0</v>
+        <v>2140380.13</v>
       </c>
       <c r="L40" t="n">
-        <v>6281.5</v>
+        <v>2183684.66</v>
       </c>
       <c r="M40" t="n">
-        <v>6281.5</v>
+        <v>4324064.79</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>3043.1</v>
+        <v>6281.5</v>
       </c>
       <c r="M41" t="n">
-        <v>3043.1</v>
+        <v>6281.5</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2136,16 +2136,16 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>28176.54</v>
+        <v>3043.1</v>
       </c>
       <c r="M42" t="n">
-        <v>28176.54</v>
+        <v>3043.1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2173,16 +2173,16 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K43" t="n">
-        <v>57661.97</v>
+        <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>59518.06</v>
+        <v>28176.54</v>
       </c>
       <c r="M43" t="n">
-        <v>117180.03</v>
+        <v>28176.54</v>
       </c>
     </row>
     <row r="44">

</xml_diff>

<commit_message>
data: Actualización reporte de pagos pendientes PagPend (corte 21 de julio de 2026)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M44"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>20 de julio de 2026</t>
+          <t>21 de julio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -490,10 +490,10 @@
         <v>4665.02</v>
       </c>
       <c r="H4" t="n">
-        <v>79155.34</v>
+        <v>81465.99000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>83820.36</v>
+        <v>86131.00999999999</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -502,10 +502,10 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>2310.6</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>2310.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -640,7 +640,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -662,10 +662,10 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>19439.59</v>
+        <v>21878.94</v>
       </c>
       <c r="I8" t="n">
-        <v>19439.59</v>
+        <v>21878.94</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,16 +674,16 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>8271.43</v>
+        <v>98281.48</v>
       </c>
       <c r="M8" t="n">
-        <v>8271.43</v>
+        <v>98281.48</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -705,10 +705,10 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>18810.1</v>
+        <v>21181.21</v>
       </c>
       <c r="I9" t="n">
-        <v>18810.1</v>
+        <v>21181.21</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,26 +717,26 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>100890.38</v>
+        <v>6529.81</v>
       </c>
       <c r="M9" t="n">
-        <v>100890.38</v>
+        <v>6529.81</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,10 +748,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>16663.14</v>
+        <v>18802.26</v>
       </c>
       <c r="I10" t="n">
-        <v>16663.14</v>
+        <v>18802.26</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,16 +760,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>85843.7</v>
+        <v>8551.469999999999</v>
       </c>
       <c r="M10" t="n">
-        <v>85843.7</v>
+        <v>8551.469999999999</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -788,13 +788,13 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>-3232.45</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>17991</v>
+        <v>16663.14</v>
       </c>
       <c r="I11" t="n">
-        <v>14758.55</v>
+        <v>16663.14</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,10 +803,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>12931.03</v>
+        <v>85843.7</v>
       </c>
       <c r="M11" t="n">
-        <v>12931.03</v>
+        <v>85843.7</v>
       </c>
     </row>
     <row r="12">
@@ -932,10 +932,10 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>339352.33</v>
+        <v>334194.1</v>
       </c>
       <c r="M14" t="n">
-        <v>339352.33</v>
+        <v>334194.1</v>
       </c>
     </row>
     <row r="15">
@@ -1242,7 +1242,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,65 +1252,65 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>5863.45</v>
+        <v>1774.15</v>
       </c>
       <c r="H22" t="n">
-        <v>1160.7</v>
+        <v>6185.56</v>
       </c>
       <c r="I22" t="n">
-        <v>7024.15</v>
+        <v>7959.71</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>20794.19</v>
       </c>
       <c r="L22" t="n">
-        <v>47128.14</v>
+        <v>30935.53</v>
       </c>
       <c r="M22" t="n">
-        <v>47128.14</v>
+        <v>51729.72</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>5863.45</v>
       </c>
       <c r="H23" t="n">
-        <v>6382.31</v>
+        <v>1160.7</v>
       </c>
       <c r="I23" t="n">
-        <v>6382.31</v>
+        <v>7024.15</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,26 +1319,26 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>20971.42</v>
+        <v>47128.14</v>
       </c>
       <c r="M23" t="n">
-        <v>20971.42</v>
+        <v>47128.14</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>6064.17</v>
+        <v>6818.76</v>
       </c>
       <c r="I24" t="n">
-        <v>6064.17</v>
+        <v>6818.76</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,16 +1362,16 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>3588.95</v>
+        <v>31258.81</v>
       </c>
       <c r="M24" t="n">
-        <v>3588.95</v>
+        <v>31258.81</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1381,34 +1381,34 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>1774.15</v>
+        <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>3682.12</v>
+        <v>6064.17</v>
       </c>
       <c r="I25" t="n">
-        <v>5456.27</v>
+        <v>6064.17</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>20794.19</v>
+        <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>30935.53</v>
+        <v>3588.95</v>
       </c>
       <c r="M25" t="n">
-        <v>51729.72</v>
+        <v>3588.95</v>
       </c>
     </row>
     <row r="26">
@@ -1457,17 +1457,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,10 +1479,10 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>4981.93</v>
+        <v>4468.7</v>
       </c>
       <c r="I27" t="n">
-        <v>4981.93</v>
+        <v>4468.7</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1491,16 +1491,16 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>33095.64</v>
+        <v>22506.75</v>
       </c>
       <c r="M27" t="n">
-        <v>33095.64</v>
+        <v>22506.75</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>4468.7</v>
+        <v>4276.89</v>
       </c>
       <c r="I28" t="n">
-        <v>4468.7</v>
+        <v>4276.89</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,10 +1534,10 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>22506.75</v>
+        <v>8350.110000000001</v>
       </c>
       <c r="M28" t="n">
-        <v>22506.75</v>
+        <v>8350.110000000001</v>
       </c>
     </row>
     <row r="29">
@@ -1586,7 +1586,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1605,13 +1605,13 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>-6586.29</v>
       </c>
       <c r="H30" t="n">
-        <v>2968.17</v>
+        <v>10378.79</v>
       </c>
       <c r="I30" t="n">
-        <v>2968.17</v>
+        <v>3792.5</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>0</v>
+        <v>12931.03</v>
       </c>
       <c r="M30" t="n">
-        <v>0</v>
+        <v>12931.03</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>2340.27</v>
+        <v>3603.49</v>
       </c>
       <c r="I31" t="n">
-        <v>2340.27</v>
+        <v>3603.49</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>3215.87</v>
+        <v>12612.21</v>
       </c>
       <c r="M31" t="n">
-        <v>3215.87</v>
+        <v>12612.21</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1694,10 +1694,10 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>2073.34</v>
+        <v>2968.17</v>
       </c>
       <c r="I32" t="n">
-        <v>2073.34</v>
+        <v>2968.17</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,26 +1706,26 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>20733.41</v>
+        <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>20733.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>2061.35</v>
+        <v>2340.27</v>
       </c>
       <c r="I33" t="n">
-        <v>2061.35</v>
+        <v>2340.27</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,16 +1749,16 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>62382.09</v>
+        <v>3215.87</v>
       </c>
       <c r="M33" t="n">
-        <v>62382.09</v>
+        <v>3215.87</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>1801.74</v>
+        <v>2073.34</v>
       </c>
       <c r="I34" t="n">
-        <v>1801.74</v>
+        <v>2073.34</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,26 +1792,26 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>14413.95</v>
+        <v>20733.41</v>
       </c>
       <c r="M34" t="n">
-        <v>14413.95</v>
+        <v>20733.41</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>1761.99</v>
+        <v>2061.35</v>
       </c>
       <c r="I35" t="n">
-        <v>1761.99</v>
+        <v>2061.35</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,10 +1835,10 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>10864.97</v>
+        <v>62382.09</v>
       </c>
       <c r="M35" t="n">
-        <v>10864.97</v>
+        <v>62382.09</v>
       </c>
     </row>
     <row r="36">
@@ -1887,7 +1887,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>1599.61</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>1599.61</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>49140.03</v>
+        <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>49140.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>6832.95</v>
+        <v>49140.03</v>
       </c>
       <c r="M38" t="n">
-        <v>6832.95</v>
+        <v>49140.03</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>25651.43</v>
+        <v>6832.95</v>
       </c>
       <c r="M39" t="n">
-        <v>25651.43</v>
+        <v>6832.95</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2044,22 +2044,22 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K40" t="n">
-        <v>2140380.13</v>
+        <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>2183684.66</v>
+        <v>25651.43</v>
       </c>
       <c r="M40" t="n">
-        <v>4324064.79</v>
+        <v>25651.43</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2087,22 +2087,22 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>2140380.13</v>
       </c>
       <c r="L41" t="n">
-        <v>6281.5</v>
+        <v>2183684.66</v>
       </c>
       <c r="M41" t="n">
-        <v>6281.5</v>
+        <v>4324064.79</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2136,16 +2136,16 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>3043.1</v>
+        <v>6281.5</v>
       </c>
       <c r="M42" t="n">
-        <v>3043.1</v>
+        <v>6281.5</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2179,26 +2179,26 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>28176.54</v>
+        <v>3043.1</v>
       </c>
       <c r="M43" t="n">
-        <v>28176.54</v>
+        <v>3043.1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>63441</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2222,9 +2222,52 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
+        <v>28176.54</v>
+      </c>
+      <c r="M44" t="n">
+        <v>28176.54</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>63441</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2511</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="n">
         <v>3695.34</v>
       </c>
-      <c r="M44" t="n">
+      <c r="M45" t="n">
         <v>3695.34</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update: PagPend (24 de julio de 2026)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>21 de julio de 2026</t>
+          <t>24 de julio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -496,16 +496,16 @@
         <v>86131.00999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>28672.05</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>28672.05</v>
       </c>
     </row>
     <row r="5">
@@ -533,10 +533,10 @@
         <v>56273.13</v>
       </c>
       <c r="H5" t="n">
-        <v>1663.43</v>
+        <v>3447.9</v>
       </c>
       <c r="I5" t="n">
-        <v>57936.56</v>
+        <v>59721.03</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -545,10 +545,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>31031.09</v>
+        <v>29246.63</v>
       </c>
       <c r="M5" t="n">
-        <v>31031.09</v>
+        <v>29246.63</v>
       </c>
     </row>
     <row r="6">
@@ -597,7 +597,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -619,28 +619,28 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>22480.76</v>
+        <v>37796.22</v>
       </c>
       <c r="I7" t="n">
-        <v>22480.76</v>
+        <v>37796.22</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>3925.94</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>106740.25</v>
+        <v>312298.6</v>
       </c>
       <c r="M7" t="n">
-        <v>110666.19</v>
+        <v>312298.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -662,28 +662,28 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>21878.94</v>
+        <v>24772.19</v>
       </c>
       <c r="I8" t="n">
-        <v>21878.94</v>
+        <v>24772.19</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>3925.94</v>
       </c>
       <c r="L8" t="n">
-        <v>98281.48</v>
+        <v>105014.82</v>
       </c>
       <c r="M8" t="n">
-        <v>98281.48</v>
+        <v>108940.76</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -705,10 +705,10 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>21181.21</v>
+        <v>21878.94</v>
       </c>
       <c r="I9" t="n">
-        <v>21181.21</v>
+        <v>21878.94</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,26 +717,26 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>6529.81</v>
+        <v>98281.48</v>
       </c>
       <c r="M9" t="n">
-        <v>6529.81</v>
+        <v>98281.48</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,10 +748,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>18802.26</v>
+        <v>21181.21</v>
       </c>
       <c r="I10" t="n">
-        <v>18802.26</v>
+        <v>21181.21</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,16 +760,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>8551.469999999999</v>
+        <v>6529.81</v>
       </c>
       <c r="M10" t="n">
-        <v>8551.469999999999</v>
+        <v>6529.81</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,50 +779,50 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>1774.15</v>
       </c>
       <c r="H11" t="n">
-        <v>16663.14</v>
+        <v>17605.42</v>
       </c>
       <c r="I11" t="n">
-        <v>16663.14</v>
+        <v>19379.57</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>20794.19</v>
       </c>
       <c r="L11" t="n">
-        <v>85843.7</v>
+        <v>19515.67</v>
       </c>
       <c r="M11" t="n">
-        <v>85843.7</v>
+        <v>40309.86</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>12104.18</v>
+        <v>18802.26</v>
       </c>
       <c r="I12" t="n">
-        <v>12104.18</v>
+        <v>18802.26</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,26 +846,26 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>6978.13</v>
+        <v>8551.469999999999</v>
       </c>
       <c r="M12" t="n">
-        <v>6978.13</v>
+        <v>8551.469999999999</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,10 +877,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>11221.61</v>
+        <v>16663.14</v>
       </c>
       <c r="I13" t="n">
-        <v>11221.61</v>
+        <v>16663.14</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -889,26 +889,26 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>122934.4</v>
+        <v>85843.7</v>
       </c>
       <c r="M13" t="n">
-        <v>122934.4</v>
+        <v>85843.7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>10742.45</v>
+        <v>15243.2</v>
       </c>
       <c r="I14" t="n">
-        <v>10742.45</v>
+        <v>15243.2</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>334194.1</v>
+        <v>118912.8</v>
       </c>
       <c r="M14" t="n">
-        <v>334194.1</v>
+        <v>118912.8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -960,13 +960,13 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>-6586.29</v>
       </c>
       <c r="H15" t="n">
-        <v>10556.59</v>
+        <v>21344.84</v>
       </c>
       <c r="I15" t="n">
-        <v>10556.59</v>
+        <v>14758.55</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>51253.23</v>
+        <v>12931.03</v>
       </c>
       <c r="M15" t="n">
-        <v>51253.23</v>
+        <v>12931.03</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,28 +1006,28 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>10152.32</v>
+        <v>14434.84</v>
       </c>
       <c r="I16" t="n">
-        <v>10152.32</v>
+        <v>14434.84</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K16" t="n">
-        <v>57661.97</v>
+        <v>2140380.13</v>
       </c>
       <c r="L16" t="n">
-        <v>52737.61</v>
+        <v>2169249.82</v>
       </c>
       <c r="M16" t="n">
-        <v>110399.58</v>
+        <v>4309629.95</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>9773.620000000001</v>
+        <v>12104.18</v>
       </c>
       <c r="I17" t="n">
-        <v>9773.620000000001</v>
+        <v>12104.18</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,26 +1061,26 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>58727.91</v>
+        <v>6978.13</v>
       </c>
       <c r="M17" t="n">
-        <v>58727.91</v>
+        <v>6978.13</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,28 +1092,28 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>9483.780000000001</v>
+        <v>10556.59</v>
       </c>
       <c r="I18" t="n">
-        <v>9483.780000000001</v>
+        <v>10556.59</v>
       </c>
       <c r="J18" t="n">
         <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>1793.28</v>
+        <v>20327.64</v>
       </c>
       <c r="L18" t="n">
-        <v>25194.79</v>
+        <v>51253.23</v>
       </c>
       <c r="M18" t="n">
-        <v>26988.07</v>
+        <v>71580.87</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,28 +1135,28 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>8496.639999999999</v>
+        <v>10152.32</v>
       </c>
       <c r="I19" t="n">
-        <v>8496.639999999999</v>
+        <v>10152.32</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>57661.97</v>
       </c>
       <c r="L19" t="n">
-        <v>7694.63</v>
+        <v>52737.61</v>
       </c>
       <c r="M19" t="n">
-        <v>7694.63</v>
+        <v>110399.58</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>8394.559999999999</v>
+        <v>9773.620000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>8394.559999999999</v>
+        <v>9773.620000000001</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,16 +1190,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>88137.78999999999</v>
+        <v>58727.91</v>
       </c>
       <c r="M20" t="n">
-        <v>88137.78999999999</v>
+        <v>58727.91</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,28 +1221,28 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>8004.31</v>
+        <v>9483.780000000001</v>
       </c>
       <c r="I21" t="n">
-        <v>8004.31</v>
+        <v>9483.780000000001</v>
       </c>
       <c r="J21" t="n">
         <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>2535.92</v>
+        <v>1793.28</v>
       </c>
       <c r="L21" t="n">
-        <v>130699.81</v>
+        <v>25194.79</v>
       </c>
       <c r="M21" t="n">
-        <v>133235.73</v>
+        <v>26988.07</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,40 +1252,40 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>1774.15</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>6185.56</v>
+        <v>8496.639999999999</v>
       </c>
       <c r="I22" t="n">
-        <v>7959.71</v>
+        <v>8496.639999999999</v>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>20794.19</v>
+        <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>30935.53</v>
+        <v>7694.63</v>
       </c>
       <c r="M22" t="n">
-        <v>51729.72</v>
+        <v>7694.63</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,22 +1295,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>5863.45</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>1160.7</v>
+        <v>8394.559999999999</v>
       </c>
       <c r="I23" t="n">
-        <v>7024.15</v>
+        <v>8394.559999999999</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,16 +1319,16 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>47128.14</v>
+        <v>88137.78999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>47128.14</v>
+        <v>88137.78999999999</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,28 +1350,28 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>6818.76</v>
+        <v>8004.31</v>
       </c>
       <c r="I24" t="n">
-        <v>6818.76</v>
+        <v>8004.31</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>2535.92</v>
       </c>
       <c r="L24" t="n">
-        <v>31258.81</v>
+        <v>130699.81</v>
       </c>
       <c r="M24" t="n">
-        <v>31258.81</v>
+        <v>133235.73</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1381,22 +1381,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>5863.45</v>
       </c>
       <c r="H25" t="n">
-        <v>6064.17</v>
+        <v>1160.7</v>
       </c>
       <c r="I25" t="n">
-        <v>6064.17</v>
+        <v>7024.15</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,26 +1405,26 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>3588.95</v>
+        <v>47128.14</v>
       </c>
       <c r="M25" t="n">
-        <v>3588.95</v>
+        <v>47128.14</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>110105</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ROCIO YANETH OCHOA IBARRA</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>5255.37</v>
+        <v>6818.76</v>
       </c>
       <c r="I26" t="n">
-        <v>5255.37</v>
+        <v>6818.76</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>31258.81</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>31258.81</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,10 +1479,10 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>4468.7</v>
+        <v>6064.17</v>
       </c>
       <c r="I27" t="n">
-        <v>4468.7</v>
+        <v>6064.17</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1491,16 +1491,16 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>22506.75</v>
+        <v>3588.95</v>
       </c>
       <c r="M27" t="n">
-        <v>22506.75</v>
+        <v>3588.95</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>4276.89</v>
+        <v>5648</v>
       </c>
       <c r="I28" t="n">
-        <v>4276.89</v>
+        <v>5648</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>8350.110000000001</v>
+        <v>20733.41</v>
       </c>
       <c r="M28" t="n">
-        <v>8350.110000000001</v>
+        <v>20733.41</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>110105</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>ROCIO YANETH OCHOA IBARRA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,28 +1565,28 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>4023</v>
+        <v>5255.37</v>
       </c>
       <c r="I29" t="n">
-        <v>4023</v>
+        <v>5255.37</v>
       </c>
       <c r="J29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>33210.52</v>
+        <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>17020.43</v>
+        <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>50230.95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1605,13 +1605,13 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>-6586.29</v>
+        <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>10378.79</v>
+        <v>4468.7</v>
       </c>
       <c r="I30" t="n">
-        <v>3792.5</v>
+        <v>4468.7</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>12931.03</v>
+        <v>22506.75</v>
       </c>
       <c r="M30" t="n">
-        <v>12931.03</v>
+        <v>22506.75</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>3603.49</v>
+        <v>4276.89</v>
       </c>
       <c r="I31" t="n">
-        <v>3603.49</v>
+        <v>4276.89</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>12612.21</v>
+        <v>8350.110000000001</v>
       </c>
       <c r="M31" t="n">
-        <v>12612.21</v>
+        <v>8350.110000000001</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1694,28 +1694,28 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>2968.17</v>
+        <v>4023</v>
       </c>
       <c r="I32" t="n">
-        <v>2968.17</v>
+        <v>4023</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K32" t="n">
-        <v>0</v>
+        <v>33210.52</v>
       </c>
       <c r="L32" t="n">
-        <v>0</v>
+        <v>17020.43</v>
       </c>
       <c r="M32" t="n">
-        <v>0</v>
+        <v>50230.95</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>2340.27</v>
+        <v>3603.49</v>
       </c>
       <c r="I33" t="n">
-        <v>2340.27</v>
+        <v>3603.49</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,16 +1749,16 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>3215.87</v>
+        <v>12612.21</v>
       </c>
       <c r="M33" t="n">
-        <v>3215.87</v>
+        <v>12612.21</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>2073.34</v>
+        <v>2968.17</v>
       </c>
       <c r="I34" t="n">
-        <v>2073.34</v>
+        <v>2968.17</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,26 +1792,26 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>20733.41</v>
+        <v>0</v>
       </c>
       <c r="M34" t="n">
-        <v>20733.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>2061.35</v>
+        <v>2340.27</v>
       </c>
       <c r="I35" t="n">
-        <v>2061.35</v>
+        <v>2340.27</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,26 +1835,26 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>62382.09</v>
+        <v>3215.87</v>
       </c>
       <c r="M35" t="n">
-        <v>62382.09</v>
+        <v>3215.87</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>1748.24</v>
+        <v>2061.35</v>
       </c>
       <c r="I36" t="n">
-        <v>1748.24</v>
+        <v>2061.35</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>9075.540000000001</v>
+        <v>62382.09</v>
       </c>
       <c r="M36" t="n">
-        <v>9075.540000000001</v>
+        <v>62382.09</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>1599.61</v>
+        <v>1748.24</v>
       </c>
       <c r="I37" t="n">
-        <v>1599.61</v>
+        <v>1748.24</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>0</v>
+        <v>9075.540000000001</v>
       </c>
       <c r="M37" t="n">
-        <v>0</v>
+        <v>9075.540000000001</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1952,10 +1952,10 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>1599.61</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>1599.61</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>49140.03</v>
+        <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>49140.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>6832.95</v>
+        <v>49140.03</v>
       </c>
       <c r="M39" t="n">
-        <v>6832.95</v>
+        <v>49140.03</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>25651.43</v>
+        <v>6832.95</v>
       </c>
       <c r="M40" t="n">
-        <v>25651.43</v>
+        <v>6832.95</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2087,16 +2087,16 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K41" t="n">
-        <v>2140380.13</v>
+        <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>2183684.66</v>
+        <v>25651.43</v>
       </c>
       <c r="M41" t="n">
-        <v>4324064.79</v>
+        <v>25651.43</v>
       </c>
     </row>
     <row r="42">
@@ -2136,10 +2136,10 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>6281.5</v>
+        <v>1429.25</v>
       </c>
       <c r="M42" t="n">
-        <v>6281.5</v>
+        <v>1429.25</v>
       </c>
     </row>
     <row r="43">
@@ -2222,10 +2222,10 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>28176.54</v>
+        <v>25195.3</v>
       </c>
       <c r="M44" t="n">
-        <v>28176.54</v>
+        <v>25195.3</v>
       </c>
     </row>
     <row r="45">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-07-29 15:27)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>28 de julio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -496,16 +496,16 @@
         <v>86131.00999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" t="n">
-        <v>28672.05</v>
+        <v>30565.3</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>28672.05</v>
+        <v>30565.3</v>
       </c>
     </row>
     <row r="5">
@@ -533,10 +533,10 @@
         <v>56273.13</v>
       </c>
       <c r="H5" t="n">
-        <v>3447.9</v>
+        <v>5232.36</v>
       </c>
       <c r="I5" t="n">
-        <v>59721.03</v>
+        <v>61505.49</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -545,10 +545,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>29246.63</v>
+        <v>27462.16</v>
       </c>
       <c r="M5" t="n">
-        <v>29246.63</v>
+        <v>27462.16</v>
       </c>
     </row>
     <row r="6">
@@ -576,10 +576,10 @@
         <v>4019.13</v>
       </c>
       <c r="H6" t="n">
-        <v>51315.46</v>
+        <v>53788.31</v>
       </c>
       <c r="I6" t="n">
-        <v>55334.59</v>
+        <v>57807.44</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,10 +588,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>50355.05</v>
+        <v>47882.19</v>
       </c>
       <c r="M6" t="n">
-        <v>50355.05</v>
+        <v>47882.19</v>
       </c>
     </row>
     <row r="7">
@@ -619,10 +619,10 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>37796.22</v>
+        <v>51343.54</v>
       </c>
       <c r="I7" t="n">
-        <v>37796.22</v>
+        <v>51343.54</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,16 +631,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>312298.6</v>
+        <v>298751.28</v>
       </c>
       <c r="M7" t="n">
-        <v>312298.6</v>
+        <v>298751.28</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,40 +650,40 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>2670.57</v>
       </c>
       <c r="H8" t="n">
-        <v>24772.19</v>
+        <v>34562.91</v>
       </c>
       <c r="I8" t="n">
-        <v>24772.19</v>
+        <v>37233.48</v>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>3925.94</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>105014.82</v>
+        <v>17020.43</v>
       </c>
       <c r="M8" t="n">
-        <v>108940.76</v>
+        <v>17020.43</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -705,28 +705,28 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>21878.94</v>
+        <v>24772.19</v>
       </c>
       <c r="I9" t="n">
-        <v>21878.94</v>
+        <v>24772.19</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>3925.94</v>
       </c>
       <c r="L9" t="n">
-        <v>98281.48</v>
+        <v>105014.82</v>
       </c>
       <c r="M9" t="n">
-        <v>98281.48</v>
+        <v>108940.76</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,10 +748,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>21181.21</v>
+        <v>23937.12</v>
       </c>
       <c r="I10" t="n">
-        <v>21181.21</v>
+        <v>23937.12</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,69 +760,69 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>6529.81</v>
+        <v>96223.3</v>
       </c>
       <c r="M10" t="n">
-        <v>6529.81</v>
+        <v>96223.3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>1774.15</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>17605.42</v>
+        <v>23577.55</v>
       </c>
       <c r="I11" t="n">
-        <v>19379.57</v>
+        <v>23577.55</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>20794.19</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>19515.67</v>
+        <v>17699.94</v>
       </c>
       <c r="M11" t="n">
-        <v>40309.86</v>
+        <v>17699.94</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>18802.26</v>
+        <v>21181.21</v>
       </c>
       <c r="I12" t="n">
-        <v>18802.26</v>
+        <v>21181.21</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,16 +846,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>8551.469999999999</v>
+        <v>6529.81</v>
       </c>
       <c r="M12" t="n">
-        <v>8551.469999999999</v>
+        <v>6529.81</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,40 +865,40 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>1774.15</v>
       </c>
       <c r="H13" t="n">
-        <v>16663.14</v>
+        <v>17605.42</v>
       </c>
       <c r="I13" t="n">
-        <v>16663.14</v>
+        <v>19379.57</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>20794.19</v>
       </c>
       <c r="L13" t="n">
-        <v>85843.7</v>
+        <v>19515.67</v>
       </c>
       <c r="M13" t="n">
-        <v>85843.7</v>
+        <v>40309.86</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>15243.2</v>
+        <v>18802.26</v>
       </c>
       <c r="I14" t="n">
-        <v>15243.2</v>
+        <v>18802.26</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>118912.8</v>
+        <v>8551.469999999999</v>
       </c>
       <c r="M14" t="n">
-        <v>118912.8</v>
+        <v>8551.469999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -960,41 +960,41 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>-6586.29</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>21344.84</v>
+        <v>18449.48</v>
       </c>
       <c r="I15" t="n">
-        <v>14758.55</v>
+        <v>18449.48</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>40607.95</v>
       </c>
       <c r="L15" t="n">
-        <v>12931.03</v>
+        <v>43360.33</v>
       </c>
       <c r="M15" t="n">
-        <v>12931.03</v>
+        <v>83968.28</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,28 +1006,28 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>14434.84</v>
+        <v>17573.59</v>
       </c>
       <c r="I16" t="n">
-        <v>14434.84</v>
+        <v>17573.59</v>
       </c>
       <c r="J16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>2140380.13</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>2169249.82</v>
+        <v>116655.84</v>
       </c>
       <c r="M16" t="n">
-        <v>4309629.95</v>
+        <v>116655.84</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>12104.18</v>
+        <v>16663.14</v>
       </c>
       <c r="I17" t="n">
-        <v>12104.18</v>
+        <v>16663.14</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,26 +1061,26 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>6978.13</v>
+        <v>85843.7</v>
       </c>
       <c r="M17" t="n">
-        <v>6978.13</v>
+        <v>85843.7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,28 +1092,28 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>10556.59</v>
+        <v>15061.43</v>
       </c>
       <c r="I18" t="n">
-        <v>10556.59</v>
+        <v>15061.43</v>
       </c>
       <c r="J18" t="n">
         <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>20327.64</v>
+        <v>2535.92</v>
       </c>
       <c r="L18" t="n">
-        <v>51253.23</v>
+        <v>123642.69</v>
       </c>
       <c r="M18" t="n">
-        <v>71580.87</v>
+        <v>126178.61</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1132,31 +1132,31 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>-6586.29</v>
       </c>
       <c r="H19" t="n">
-        <v>10152.32</v>
+        <v>21344.84</v>
       </c>
       <c r="I19" t="n">
-        <v>10152.32</v>
+        <v>14758.55</v>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>57661.97</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>52737.61</v>
+        <v>12931.03</v>
       </c>
       <c r="M19" t="n">
-        <v>110399.58</v>
+        <v>12931.03</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,38 +1178,38 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>9773.620000000001</v>
+        <v>14434.84</v>
       </c>
       <c r="I20" t="n">
-        <v>9773.620000000001</v>
+        <v>14434.84</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>2230648.56</v>
       </c>
       <c r="L20" t="n">
-        <v>58727.91</v>
+        <v>2169249.82</v>
       </c>
       <c r="M20" t="n">
-        <v>58727.91</v>
+        <v>4399898.38</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,53 +1221,53 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>9483.780000000001</v>
+        <v>13848.72</v>
       </c>
       <c r="I21" t="n">
-        <v>9483.780000000001</v>
+        <v>13848.72</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>1793.28</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>25194.79</v>
+        <v>5233.6</v>
       </c>
       <c r="M21" t="n">
-        <v>26988.07</v>
+        <v>5233.6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>1793.28</v>
       </c>
       <c r="H22" t="n">
-        <v>8496.639999999999</v>
+        <v>9483.780000000001</v>
       </c>
       <c r="I22" t="n">
-        <v>8496.639999999999</v>
+        <v>11277.06</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,16 +1276,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>7694.63</v>
+        <v>25194.79</v>
       </c>
       <c r="M22" t="n">
-        <v>7694.63</v>
+        <v>25194.79</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,38 +1307,38 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>8394.559999999999</v>
+        <v>10152.32</v>
       </c>
       <c r="I23" t="n">
-        <v>8394.559999999999</v>
+        <v>10152.32</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>57661.97</v>
       </c>
       <c r="L23" t="n">
-        <v>88137.78999999999</v>
+        <v>52737.61</v>
       </c>
       <c r="M23" t="n">
-        <v>88137.78999999999</v>
+        <v>110399.58</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,28 +1350,28 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>8004.31</v>
+        <v>9773.620000000001</v>
       </c>
       <c r="I24" t="n">
-        <v>8004.31</v>
+        <v>9773.620000000001</v>
       </c>
       <c r="J24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>2535.92</v>
+        <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>130699.81</v>
+        <v>58727.91</v>
       </c>
       <c r="M24" t="n">
-        <v>133235.73</v>
+        <v>58727.91</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1381,22 +1381,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>5863.45</v>
+        <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>1160.7</v>
+        <v>8496.639999999999</v>
       </c>
       <c r="I25" t="n">
-        <v>7024.15</v>
+        <v>8496.639999999999</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,26 +1405,26 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>47128.14</v>
+        <v>7694.63</v>
       </c>
       <c r="M25" t="n">
-        <v>47128.14</v>
+        <v>7694.63</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>6818.76</v>
+        <v>8394.559999999999</v>
       </c>
       <c r="I26" t="n">
-        <v>6818.76</v>
+        <v>8394.559999999999</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>31258.81</v>
+        <v>88137.78999999999</v>
       </c>
       <c r="M26" t="n">
-        <v>31258.81</v>
+        <v>88137.78999999999</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,22 +1467,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>5863.45</v>
       </c>
       <c r="H27" t="n">
-        <v>6064.17</v>
+        <v>1160.7</v>
       </c>
       <c r="I27" t="n">
-        <v>6064.17</v>
+        <v>7024.15</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1491,16 +1491,16 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>3588.95</v>
+        <v>47128.14</v>
       </c>
       <c r="M27" t="n">
-        <v>3588.95</v>
+        <v>47128.14</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>5648</v>
+        <v>6064.17</v>
       </c>
       <c r="I28" t="n">
-        <v>5648</v>
+        <v>6064.17</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>20733.41</v>
+        <v>3588.95</v>
       </c>
       <c r="M28" t="n">
-        <v>20733.41</v>
+        <v>3588.95</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>110105</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ROCIO YANETH OCHOA IBARRA</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>5255.37</v>
+        <v>5648</v>
       </c>
       <c r="I29" t="n">
-        <v>5255.37</v>
+        <v>5648</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,16 +1577,16 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>0</v>
+        <v>20733.41</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>20733.41</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>110105</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>ROCIO YANETH OCHOA IBARRA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>4468.7</v>
+        <v>5255.37</v>
       </c>
       <c r="I30" t="n">
-        <v>4468.7</v>
+        <v>5255.37</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>22506.75</v>
+        <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>22506.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>4276.89</v>
+        <v>4468.7</v>
       </c>
       <c r="I31" t="n">
-        <v>4276.89</v>
+        <v>4468.7</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>8350.110000000001</v>
+        <v>22506.75</v>
       </c>
       <c r="M31" t="n">
-        <v>8350.110000000001</v>
+        <v>22506.75</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1694,28 +1694,28 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>4023</v>
+        <v>4276.89</v>
       </c>
       <c r="I32" t="n">
-        <v>4023</v>
+        <v>4276.89</v>
       </c>
       <c r="J32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>33210.52</v>
+        <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>17020.43</v>
+        <v>8350.110000000001</v>
       </c>
       <c r="M32" t="n">
-        <v>50230.95</v>
+        <v>8350.110000000001</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>3603.49</v>
+        <v>4108.16</v>
       </c>
       <c r="I33" t="n">
-        <v>3603.49</v>
+        <v>4108.16</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,26 +1749,26 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>12612.21</v>
+        <v>21543.27</v>
       </c>
       <c r="M33" t="n">
-        <v>12612.21</v>
+        <v>21543.27</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>2968.17</v>
+        <v>4088.85</v>
       </c>
       <c r="I34" t="n">
-        <v>2968.17</v>
+        <v>4088.85</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,10 +1792,10 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>0</v>
+        <v>60354.59</v>
       </c>
       <c r="M34" t="n">
-        <v>0</v>
+        <v>60354.59</v>
       </c>
     </row>
     <row r="35">
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>2340.27</v>
+        <v>4054.21</v>
       </c>
       <c r="I35" t="n">
-        <v>2340.27</v>
+        <v>4054.21</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,26 +1835,26 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>3215.87</v>
+        <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>3215.87</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>2061.35</v>
+        <v>3603.49</v>
       </c>
       <c r="I36" t="n">
-        <v>2061.35</v>
+        <v>3603.49</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>62382.09</v>
+        <v>12612.21</v>
       </c>
       <c r="M36" t="n">
-        <v>62382.09</v>
+        <v>12612.21</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>1748.24</v>
+        <v>2968.17</v>
       </c>
       <c r="I37" t="n">
-        <v>1748.24</v>
+        <v>2968.17</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>9075.540000000001</v>
+        <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>9075.540000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1952,10 +1952,10 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>1599.61</v>
+        <v>2482.01</v>
       </c>
       <c r="I38" t="n">
-        <v>1599.61</v>
+        <v>2482.01</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>0</v>
+        <v>22713.31</v>
       </c>
       <c r="M38" t="n">
-        <v>0</v>
+        <v>22713.31</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1995,10 +1995,10 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>1748.24</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>1748.24</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>49140.03</v>
+        <v>9075.540000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>49140.03</v>
+        <v>9075.540000000001</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2038,10 +2038,10 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>1599.61</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>1599.61</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>6832.95</v>
+        <v>0</v>
       </c>
       <c r="M40" t="n">
-        <v>6832.95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>25651.43</v>
+        <v>49140.03</v>
       </c>
       <c r="M41" t="n">
-        <v>25651.43</v>
+        <v>49140.03</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2136,16 +2136,16 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>1429.25</v>
+        <v>6832.95</v>
       </c>
       <c r="M42" t="n">
-        <v>1429.25</v>
+        <v>6832.95</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2179,16 +2179,16 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>3043.1</v>
+        <v>1429.25</v>
       </c>
       <c r="M43" t="n">
-        <v>3043.1</v>
+        <v>1429.25</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2222,10 +2222,10 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>25195.3</v>
+        <v>3043.1</v>
       </c>
       <c r="M44" t="n">
-        <v>25195.3</v>
+        <v>3043.1</v>
       </c>
     </row>
     <row r="45">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-07-30 13:30)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>28 de julio de 2026</t>
+          <t>29 de julio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -812,7 +812,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>21181.21</v>
+        <v>21194.34</v>
       </c>
       <c r="I12" t="n">
-        <v>21181.21</v>
+        <v>21194.34</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,16 +846,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>6529.81</v>
+        <v>81312.5</v>
       </c>
       <c r="M12" t="n">
-        <v>6529.81</v>
+        <v>81312.5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,93 +865,93 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>1774.15</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>17605.42</v>
+        <v>21181.21</v>
       </c>
       <c r="I13" t="n">
-        <v>19379.57</v>
+        <v>21181.21</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>20794.19</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>19515.67</v>
+        <v>6529.81</v>
       </c>
       <c r="M13" t="n">
-        <v>40309.86</v>
+        <v>6529.81</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>1774.15</v>
       </c>
       <c r="H14" t="n">
-        <v>18802.26</v>
+        <v>17605.42</v>
       </c>
       <c r="I14" t="n">
-        <v>18802.26</v>
+        <v>19379.57</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>20794.19</v>
       </c>
       <c r="L14" t="n">
-        <v>8551.469999999999</v>
+        <v>19515.67</v>
       </c>
       <c r="M14" t="n">
-        <v>8551.469999999999</v>
+        <v>40309.86</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,38 +963,38 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>18449.48</v>
+        <v>18802.26</v>
       </c>
       <c r="I15" t="n">
-        <v>18449.48</v>
+        <v>18802.26</v>
       </c>
       <c r="J15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>40607.95</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>43360.33</v>
+        <v>8551.469999999999</v>
       </c>
       <c r="M15" t="n">
-        <v>83968.28</v>
+        <v>8551.469999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,38 +1006,38 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>17573.59</v>
+        <v>18449.48</v>
       </c>
       <c r="I16" t="n">
-        <v>17573.59</v>
+        <v>18449.48</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>40607.95</v>
       </c>
       <c r="L16" t="n">
-        <v>116655.84</v>
+        <v>43360.33</v>
       </c>
       <c r="M16" t="n">
-        <v>116655.84</v>
+        <v>83968.28</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>16663.14</v>
+        <v>17573.59</v>
       </c>
       <c r="I17" t="n">
-        <v>16663.14</v>
+        <v>17573.59</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,10 +1061,10 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>85843.7</v>
+        <v>116655.84</v>
       </c>
       <c r="M17" t="n">
-        <v>85843.7</v>
+        <v>116655.84</v>
       </c>
     </row>
     <row r="18">
@@ -1098,16 +1098,16 @@
         <v>15061.43</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K18" t="n">
-        <v>2535.92</v>
+        <v>9712.389999999999</v>
       </c>
       <c r="L18" t="n">
         <v>123642.69</v>
       </c>
       <c r="M18" t="n">
-        <v>126178.61</v>
+        <v>133355.08</v>
       </c>
     </row>
     <row r="19">
@@ -1313,16 +1313,16 @@
         <v>10152.32</v>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K23" t="n">
-        <v>57661.97</v>
+        <v>76168.03999999999</v>
       </c>
       <c r="L23" t="n">
-        <v>52737.61</v>
+        <v>71243.67999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>110399.58</v>
+        <v>147411.72</v>
       </c>
     </row>
     <row r="24">
@@ -1887,7 +1887,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>2968.17</v>
+        <v>3523.31</v>
       </c>
       <c r="I37" t="n">
-        <v>2968.17</v>
+        <v>3523.31</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>0</v>
+        <v>21672.01</v>
       </c>
       <c r="M37" t="n">
-        <v>0</v>
+        <v>21672.01</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1952,10 +1952,10 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>2482.01</v>
+        <v>2968.17</v>
       </c>
       <c r="I38" t="n">
-        <v>2482.01</v>
+        <v>2968.17</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,10 +1964,10 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>22713.31</v>
+        <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>22713.31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -1995,10 +1995,10 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>1748.24</v>
+        <v>2789.54</v>
       </c>
       <c r="I39" t="n">
-        <v>1748.24</v>
+        <v>2789.54</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2007,10 +2007,10 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>9075.540000000001</v>
+        <v>8034.24</v>
       </c>
       <c r="M39" t="n">
-        <v>9075.540000000001</v>
+        <v>8034.24</v>
       </c>
     </row>
     <row r="40">

</xml_diff>

<commit_message>
data: update PagPend report with cutoff date July 30, 2026
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>29 de julio de 2026</t>
+          <t>30 de julio de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -484,28 +484,28 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>4665.02</v>
+        <v>33337.07</v>
       </c>
       <c r="H4" t="n">
         <v>81465.99000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>86131.00999999999</v>
+        <v>114803.06</v>
       </c>
       <c r="J4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K4" t="n">
-        <v>30565.3</v>
+        <v>1893.25</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>30565.3</v>
+        <v>1893.25</v>
       </c>
     </row>
     <row r="5">
@@ -576,10 +576,10 @@
         <v>4019.13</v>
       </c>
       <c r="H6" t="n">
-        <v>53788.31</v>
+        <v>55526.32</v>
       </c>
       <c r="I6" t="n">
-        <v>57807.44</v>
+        <v>59545.45</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,16 +588,16 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>47882.19</v>
+        <v>46144.18</v>
       </c>
       <c r="M6" t="n">
-        <v>47882.19</v>
+        <v>46144.18</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -607,22 +607,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>40607.95</v>
       </c>
       <c r="H7" t="n">
-        <v>51343.54</v>
+        <v>18449.48</v>
       </c>
       <c r="I7" t="n">
-        <v>51343.54</v>
+        <v>59057.43</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,16 +631,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>298751.28</v>
+        <v>43360.33</v>
       </c>
       <c r="M7" t="n">
-        <v>298751.28</v>
+        <v>43360.33</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,22 +650,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>2670.57</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>34562.91</v>
+        <v>58757.14</v>
       </c>
       <c r="I8" t="n">
-        <v>37233.48</v>
+        <v>58757.14</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,16 +674,16 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>17020.43</v>
+        <v>291337.67</v>
       </c>
       <c r="M8" t="n">
-        <v>17020.43</v>
+        <v>291337.67</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,40 +693,40 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>2670.57</v>
       </c>
       <c r="H9" t="n">
-        <v>24772.19</v>
+        <v>36504.99</v>
       </c>
       <c r="I9" t="n">
-        <v>24772.19</v>
+        <v>39175.56</v>
       </c>
       <c r="J9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>3925.94</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>105014.82</v>
+        <v>15078.35</v>
       </c>
       <c r="M9" t="n">
-        <v>108940.76</v>
+        <v>15078.35</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -736,50 +736,50 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>18506.07</v>
       </c>
       <c r="H10" t="n">
-        <v>23937.12</v>
+        <v>13444.1</v>
       </c>
       <c r="I10" t="n">
-        <v>23937.12</v>
+        <v>31950.17</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>5054.91</v>
       </c>
       <c r="L10" t="n">
-        <v>96223.3</v>
+        <v>123555.96</v>
       </c>
       <c r="M10" t="n">
-        <v>96223.3</v>
+        <v>128610.87</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -791,10 +791,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>23577.55</v>
+        <v>25458.8</v>
       </c>
       <c r="I11" t="n">
-        <v>23577.55</v>
+        <v>25458.8</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,26 +803,26 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>17699.94</v>
+        <v>2252.2</v>
       </c>
       <c r="M11" t="n">
-        <v>17699.94</v>
+        <v>2252.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>21194.34</v>
+        <v>25280.74</v>
       </c>
       <c r="I12" t="n">
-        <v>21194.34</v>
+        <v>25280.74</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,16 +846,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>81312.5</v>
+        <v>16366.96</v>
       </c>
       <c r="M12" t="n">
-        <v>81312.5</v>
+        <v>16366.96</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,28 +877,28 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>21181.21</v>
+        <v>24772.19</v>
       </c>
       <c r="I13" t="n">
-        <v>21181.21</v>
+        <v>24772.19</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>3925.94</v>
       </c>
       <c r="L13" t="n">
-        <v>6529.81</v>
+        <v>105014.82</v>
       </c>
       <c r="M13" t="n">
-        <v>6529.81</v>
+        <v>108940.76</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,50 +908,50 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>1774.15</v>
+        <v>-6586.29</v>
       </c>
       <c r="H14" t="n">
-        <v>17605.42</v>
+        <v>31126.91</v>
       </c>
       <c r="I14" t="n">
-        <v>19379.57</v>
+        <v>24540.62</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>20794.19</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>19515.67</v>
+        <v>7496.68</v>
       </c>
       <c r="M14" t="n">
-        <v>40309.86</v>
+        <v>7496.68</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>18802.26</v>
+        <v>23937.12</v>
       </c>
       <c r="I15" t="n">
-        <v>18802.26</v>
+        <v>23937.12</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>8551.469999999999</v>
+        <v>96223.3</v>
       </c>
       <c r="M15" t="n">
-        <v>8551.469999999999</v>
+        <v>96223.3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,22 +1006,22 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>18449.48</v>
+        <v>21194.34</v>
       </c>
       <c r="I16" t="n">
-        <v>18449.48</v>
+        <v>21194.34</v>
       </c>
       <c r="J16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>40607.95</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>43360.33</v>
+        <v>81312.5</v>
       </c>
       <c r="M16" t="n">
-        <v>83968.28</v>
+        <v>81312.5</v>
       </c>
     </row>
     <row r="17">
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>17573.59</v>
+        <v>19815.92</v>
       </c>
       <c r="I17" t="n">
-        <v>17573.59</v>
+        <v>19815.92</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,69 +1061,69 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>116655.84</v>
+        <v>114413.51</v>
       </c>
       <c r="M17" t="n">
-        <v>116655.84</v>
+        <v>114413.51</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>1774.15</v>
       </c>
       <c r="H18" t="n">
-        <v>15061.43</v>
+        <v>17605.42</v>
       </c>
       <c r="I18" t="n">
-        <v>15061.43</v>
+        <v>19379.57</v>
       </c>
       <c r="J18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>9712.389999999999</v>
+        <v>20794.19</v>
       </c>
       <c r="L18" t="n">
-        <v>123642.69</v>
+        <v>19515.67</v>
       </c>
       <c r="M18" t="n">
-        <v>133355.08</v>
+        <v>40309.86</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1132,41 +1132,41 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>-6586.29</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>21344.84</v>
+        <v>18981.03</v>
       </c>
       <c r="I19" t="n">
-        <v>14758.55</v>
+        <v>18981.03</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>9712.389999999999</v>
       </c>
       <c r="L19" t="n">
-        <v>12931.03</v>
+        <v>119723.08</v>
       </c>
       <c r="M19" t="n">
-        <v>12931.03</v>
+        <v>129435.47</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,28 +1178,28 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>14434.84</v>
+        <v>18802.26</v>
       </c>
       <c r="I20" t="n">
-        <v>14434.84</v>
+        <v>18802.26</v>
       </c>
       <c r="J20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>2230648.56</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>2169249.82</v>
+        <v>8551.469999999999</v>
       </c>
       <c r="M20" t="n">
-        <v>4399898.38</v>
+        <v>8551.469999999999</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,53 +1221,53 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>13848.72</v>
+        <v>14434.84</v>
       </c>
       <c r="I21" t="n">
-        <v>13848.72</v>
+        <v>14434.84</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>2230648.56</v>
       </c>
       <c r="L21" t="n">
-        <v>5233.6</v>
+        <v>2169249.82</v>
       </c>
       <c r="M21" t="n">
-        <v>5233.6</v>
+        <v>4399898.38</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>1793.28</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>9483.780000000001</v>
+        <v>13848.72</v>
       </c>
       <c r="I22" t="n">
-        <v>11277.06</v>
+        <v>13848.72</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,53 +1276,53 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>25194.79</v>
+        <v>5233.6</v>
       </c>
       <c r="M22" t="n">
-        <v>25194.79</v>
+        <v>5233.6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>1793.28</v>
       </c>
       <c r="H23" t="n">
-        <v>10152.32</v>
+        <v>11306.68</v>
       </c>
       <c r="I23" t="n">
-        <v>10152.32</v>
+        <v>13099.96</v>
       </c>
       <c r="J23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>76168.03999999999</v>
+        <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>71243.67999999999</v>
+        <v>23371.89</v>
       </c>
       <c r="M23" t="n">
-        <v>147411.72</v>
+        <v>23371.89</v>
       </c>
     </row>
     <row r="24">
@@ -1500,7 +1500,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>6064.17</v>
+        <v>6512.77</v>
       </c>
       <c r="I28" t="n">
-        <v>6064.17</v>
+        <v>6512.77</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>3588.95</v>
+        <v>19138.65</v>
       </c>
       <c r="M28" t="n">
-        <v>3588.95</v>
+        <v>19138.65</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>5648</v>
+        <v>6064.17</v>
       </c>
       <c r="I29" t="n">
-        <v>5648</v>
+        <v>6064.17</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,16 +1577,16 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>20733.41</v>
+        <v>3588.95</v>
       </c>
       <c r="M29" t="n">
-        <v>20733.41</v>
+        <v>3588.95</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>110105</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ROCIO YANETH OCHOA IBARRA</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>5255.37</v>
+        <v>5648</v>
       </c>
       <c r="I30" t="n">
-        <v>5255.37</v>
+        <v>5648</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>0</v>
+        <v>20733.41</v>
       </c>
       <c r="M30" t="n">
-        <v>0</v>
+        <v>20733.41</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>110105</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>ROCIO YANETH OCHOA IBARRA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>4468.7</v>
+        <v>5255.37</v>
       </c>
       <c r="I31" t="n">
-        <v>4468.7</v>
+        <v>5255.37</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>22506.75</v>
+        <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>22506.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1694,10 +1694,10 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>4276.89</v>
+        <v>4468.7</v>
       </c>
       <c r="I32" t="n">
-        <v>4276.89</v>
+        <v>4468.7</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,16 +1706,16 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>8350.110000000001</v>
+        <v>22506.75</v>
       </c>
       <c r="M32" t="n">
-        <v>8350.110000000001</v>
+        <v>22506.75</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>4108.16</v>
+        <v>4276.89</v>
       </c>
       <c r="I33" t="n">
-        <v>4108.16</v>
+        <v>4276.89</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,10 +1749,10 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>21543.27</v>
+        <v>8350.110000000001</v>
       </c>
       <c r="M33" t="n">
-        <v>21543.27</v>
+        <v>8350.110000000001</v>
       </c>
     </row>
     <row r="34">
@@ -2016,7 +2016,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2038,10 +2038,10 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>1599.61</v>
+        <v>1694.9</v>
       </c>
       <c r="I40" t="n">
-        <v>1599.61</v>
+        <v>1694.9</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>0</v>
+        <v>5138.05</v>
       </c>
       <c r="M40" t="n">
-        <v>0</v>
+        <v>5138.05</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2081,10 +2081,10 @@
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>1599.61</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>1599.61</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>49140.03</v>
+        <v>0</v>
       </c>
       <c r="M41" t="n">
-        <v>49140.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2136,10 +2136,10 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>6832.95</v>
+        <v>49140.03</v>
       </c>
       <c r="M42" t="n">
-        <v>6832.95</v>
+        <v>49140.03</v>
       </c>
     </row>
     <row r="43">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-08-10 16:04)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>30 de julio de 2026</t>
+          <t>7 de agosto de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -468,7 +468,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -478,7 +478,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -487,31 +487,31 @@
         <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>33337.07</v>
+        <v>162964</v>
       </c>
       <c r="H4" t="n">
-        <v>81465.99000000001</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>114803.06</v>
+        <v>162964</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>1893.25</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>84466.67</v>
       </c>
       <c r="M4" t="n">
-        <v>1893.25</v>
+        <v>84466.67</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -521,22 +521,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>56273.13</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>5232.36</v>
+        <v>21079.98</v>
       </c>
       <c r="I5" t="n">
-        <v>61505.49</v>
+        <v>21079.98</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -545,16 +545,16 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>27462.16</v>
+        <v>49434.03</v>
       </c>
       <c r="M5" t="n">
-        <v>27462.16</v>
+        <v>49434.03</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,22 +564,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>4019.13</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>55526.32</v>
+        <v>8476.02</v>
       </c>
       <c r="I6" t="n">
-        <v>59545.45</v>
+        <v>8476.02</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,16 +588,16 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>46144.18</v>
+        <v>5756.97</v>
       </c>
       <c r="M6" t="n">
-        <v>46144.18</v>
+        <v>5756.97</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -607,22 +607,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>40607.95</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>18449.48</v>
+        <v>8393.23</v>
       </c>
       <c r="I7" t="n">
-        <v>59057.43</v>
+        <v>8393.23</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,16 +631,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>43360.33</v>
+        <v>293606.54</v>
       </c>
       <c r="M7" t="n">
-        <v>43360.33</v>
+        <v>293606.54</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -662,10 +662,10 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>58757.14</v>
+        <v>7537.55</v>
       </c>
       <c r="I8" t="n">
-        <v>58757.14</v>
+        <v>7537.55</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,16 +674,16 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>291337.67</v>
+        <v>72817.25999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>291337.67</v>
+        <v>72817.25999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,22 +693,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>2670.57</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>36504.99</v>
+        <v>5019.7</v>
       </c>
       <c r="I9" t="n">
-        <v>39175.56</v>
+        <v>5019.7</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,16 +717,16 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>15078.35</v>
+        <v>77443.85000000001</v>
       </c>
       <c r="M9" t="n">
-        <v>15078.35</v>
+        <v>77443.85000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -736,50 +736,50 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>18506.07</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>13444.1</v>
+        <v>4699.16</v>
       </c>
       <c r="I10" t="n">
-        <v>31950.17</v>
+        <v>4699.16</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>5054.91</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>123555.96</v>
+        <v>4193.66</v>
       </c>
       <c r="M10" t="n">
-        <v>128610.87</v>
+        <v>4193.66</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -791,10 +791,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>25458.8</v>
+        <v>3933.48</v>
       </c>
       <c r="I11" t="n">
-        <v>25458.8</v>
+        <v>3933.48</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,26 +803,26 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>2252.2</v>
+        <v>114538.09</v>
       </c>
       <c r="M11" t="n">
-        <v>2252.2</v>
+        <v>114538.09</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>25280.74</v>
+        <v>3468.29</v>
       </c>
       <c r="I12" t="n">
-        <v>25280.74</v>
+        <v>3468.29</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,10 +846,10 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>16366.96</v>
+        <v>47900.16</v>
       </c>
       <c r="M12" t="n">
-        <v>16366.96</v>
+        <v>47900.16</v>
       </c>
     </row>
     <row r="13">
@@ -877,28 +877,28 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>24772.19</v>
+        <v>3443.75</v>
       </c>
       <c r="I13" t="n">
-        <v>24772.19</v>
+        <v>3443.75</v>
       </c>
       <c r="J13" t="n">
         <v>2</v>
       </c>
       <c r="K13" t="n">
-        <v>3925.94</v>
+        <v>3916.42</v>
       </c>
       <c r="L13" t="n">
-        <v>105014.82</v>
+        <v>105415.99</v>
       </c>
       <c r="M13" t="n">
-        <v>108940.76</v>
+        <v>109332.41</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -917,13 +917,13 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>-6586.29</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>31126.91</v>
+        <v>3215.73</v>
       </c>
       <c r="I14" t="n">
-        <v>24540.62</v>
+        <v>3215.73</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>7496.68</v>
+        <v>28233.37</v>
       </c>
       <c r="M14" t="n">
-        <v>7496.68</v>
+        <v>28233.37</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>23937.12</v>
+        <v>2960.97</v>
       </c>
       <c r="I15" t="n">
-        <v>23937.12</v>
+        <v>2960.97</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>96223.3</v>
+        <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>96223.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>21194.34</v>
+        <v>2439.24</v>
       </c>
       <c r="I16" t="n">
-        <v>21194.34</v>
+        <v>2439.24</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,41 +1018,41 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>81312.5</v>
+        <v>7690.17</v>
       </c>
       <c r="M16" t="n">
-        <v>81312.5</v>
+        <v>7690.17</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>2396.76</v>
       </c>
       <c r="H17" t="n">
-        <v>19815.92</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>19815.92</v>
+        <v>2396.76</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,69 +1061,69 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>114413.51</v>
+        <v>26364.37</v>
       </c>
       <c r="M17" t="n">
-        <v>114413.51</v>
+        <v>26364.37</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>63441</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2511</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>1774.15</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>17605.42</v>
+        <v>1843.19</v>
       </c>
       <c r="I18" t="n">
-        <v>19379.57</v>
+        <v>1843.19</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>20794.19</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>19515.67</v>
+        <v>1843.19</v>
       </c>
       <c r="M18" t="n">
-        <v>40309.86</v>
+        <v>1843.19</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,38 +1135,38 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>18981.03</v>
+        <v>1757.71</v>
       </c>
       <c r="I19" t="n">
-        <v>18981.03</v>
+        <v>1757.71</v>
       </c>
       <c r="J19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>9712.389999999999</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>119723.08</v>
+        <v>9080.91</v>
       </c>
       <c r="M19" t="n">
-        <v>129435.47</v>
+        <v>9080.91</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>18802.26</v>
+        <v>1627.21</v>
       </c>
       <c r="I20" t="n">
-        <v>18802.26</v>
+        <v>1627.21</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,16 +1190,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>8551.469999999999</v>
+        <v>15800.91</v>
       </c>
       <c r="M20" t="n">
-        <v>8551.469999999999</v>
+        <v>15800.91</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,28 +1221,28 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>14434.84</v>
+        <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>14434.84</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>2230648.56</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>2169249.82</v>
+        <v>49020.81</v>
       </c>
       <c r="M21" t="n">
-        <v>4399898.38</v>
+        <v>49020.81</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,28 +1264,28 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>13848.72</v>
+        <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>13848.72</v>
+        <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>24377.75</v>
       </c>
       <c r="L22" t="n">
-        <v>5233.6</v>
+        <v>26239.01</v>
       </c>
       <c r="M22" t="n">
-        <v>5233.6</v>
+        <v>50616.76</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,22 +1295,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>1793.28</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>11306.68</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>13099.96</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,26 +1319,26 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>23371.89</v>
+        <v>27395.54</v>
       </c>
       <c r="M23" t="n">
-        <v>23371.89</v>
+        <v>27395.54</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>9773.620000000001</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>9773.620000000001</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,26 +1362,26 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>58727.91</v>
+        <v>109437.94</v>
       </c>
       <c r="M24" t="n">
-        <v>58727.91</v>
+        <v>109437.94</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1393,10 +1393,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>8496.639999999999</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>8496.639999999999</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,16 +1405,16 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>7694.63</v>
+        <v>20847.16</v>
       </c>
       <c r="M25" t="n">
-        <v>7694.63</v>
+        <v>20847.16</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>8394.559999999999</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>8394.559999999999</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,41 +1448,41 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>88137.78999999999</v>
+        <v>20285.63</v>
       </c>
       <c r="M26" t="n">
-        <v>88137.78999999999</v>
+        <v>20285.63</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>5863.45</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>1160.7</v>
+        <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>7024.15</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1491,16 +1491,16 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>47128.14</v>
+        <v>28340.31</v>
       </c>
       <c r="M27" t="n">
-        <v>47128.14</v>
+        <v>28340.31</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>6512.77</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>6512.77</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>19138.65</v>
+        <v>3381.58</v>
       </c>
       <c r="M28" t="n">
-        <v>19138.65</v>
+        <v>3381.58</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>6064.17</v>
+        <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>6064.17</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,26 +1577,26 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>3588.95</v>
+        <v>19092.22</v>
       </c>
       <c r="M29" t="n">
-        <v>3588.95</v>
+        <v>19092.22</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>5648</v>
+        <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>5648</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>20733.41</v>
+        <v>8530.73</v>
       </c>
       <c r="M30" t="n">
-        <v>20733.41</v>
+        <v>8530.73</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>110105</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ROCIO YANETH OCHOA IBARRA</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>5255.37</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>5255.37</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>0</v>
+        <v>20683.11</v>
       </c>
       <c r="M31" t="n">
-        <v>0</v>
+        <v>20683.11</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1694,10 +1694,10 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>4468.7</v>
+        <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>4468.7</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,16 +1706,16 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>22506.75</v>
+        <v>12581.61</v>
       </c>
       <c r="M32" t="n">
-        <v>22506.75</v>
+        <v>12581.61</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,38 +1737,38 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>4276.89</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>4276.89</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K33" t="n">
-        <v>0</v>
+        <v>2211997.08</v>
       </c>
       <c r="L33" t="n">
-        <v>8350.110000000001</v>
+        <v>2150747.29</v>
       </c>
       <c r="M33" t="n">
-        <v>8350.110000000001</v>
+        <v>4362744.37</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>4088.85</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>4088.85</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,16 +1792,16 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>60354.59</v>
+        <v>1425.78</v>
       </c>
       <c r="M34" t="n">
-        <v>60354.59</v>
+        <v>1425.78</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>4054.21</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>4054.21</v>
+        <v>0</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>0</v>
+        <v>3035.72</v>
       </c>
       <c r="M35" t="n">
-        <v>0</v>
+        <v>3035.72</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>3603.49</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>3603.49</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>12612.21</v>
+        <v>24832.77</v>
       </c>
       <c r="M36" t="n">
-        <v>12612.21</v>
+        <v>24832.77</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>3523.31</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>3523.31</v>
+        <v>0</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>21672.01</v>
+        <v>99727.64</v>
       </c>
       <c r="M37" t="n">
-        <v>21672.01</v>
+        <v>99727.64</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1952,10 +1952,10 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>2968.17</v>
+        <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>2968.17</v>
+        <v>0</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>0</v>
+        <v>24095.39</v>
       </c>
       <c r="M38" t="n">
-        <v>0</v>
+        <v>24095.39</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1995,10 +1995,10 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>2789.54</v>
+        <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>2789.54</v>
+        <v>0</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>8034.24</v>
+        <v>6049.41</v>
       </c>
       <c r="M39" t="n">
-        <v>8034.24</v>
+        <v>6049.41</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2038,10 +2038,10 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>1694.9</v>
+        <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>1694.9</v>
+        <v>0</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>5138.05</v>
+        <v>3208.07</v>
       </c>
       <c r="M40" t="n">
-        <v>5138.05</v>
+        <v>3208.07</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2081,10 +2081,10 @@
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>1599.61</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>1599.61</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>0</v>
+        <v>62476.76</v>
       </c>
       <c r="M41" t="n">
-        <v>0</v>
+        <v>62476.76</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2130,22 +2130,22 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K42" t="n">
-        <v>0</v>
+        <v>5042.65</v>
       </c>
       <c r="L42" t="n">
-        <v>49140.03</v>
+        <v>130020.2</v>
       </c>
       <c r="M42" t="n">
-        <v>49140.03</v>
+        <v>135062.85</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2179,16 +2179,16 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>1429.25</v>
+        <v>23460.24</v>
       </c>
       <c r="M43" t="n">
-        <v>1429.25</v>
+        <v>23460.24</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2222,53 +2222,10 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>3043.1</v>
+        <v>6270.75</v>
       </c>
       <c r="M44" t="n">
-        <v>3043.1</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>63441</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>2511</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="n">
-        <v>0</v>
-      </c>
-      <c r="G45" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" t="n">
-        <v>0</v>
-      </c>
-      <c r="I45" t="n">
-        <v>0</v>
-      </c>
-      <c r="J45" t="n">
-        <v>0</v>
-      </c>
-      <c r="K45" t="n">
-        <v>0</v>
-      </c>
-      <c r="L45" t="n">
-        <v>3695.34</v>
-      </c>
-      <c r="M45" t="n">
-        <v>3695.34</v>
+        <v>6270.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: update Pagado / Pendiente report to August 10 2026 date cutoff
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>7 de agosto de 2026</t>
+          <t>10 de agosto de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -683,7 +683,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,22 +693,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>2019.94</v>
       </c>
       <c r="H9" t="n">
-        <v>5019.7</v>
+        <v>4273.63</v>
       </c>
       <c r="I9" t="n">
-        <v>5019.7</v>
+        <v>6293.57</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,26 +717,26 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>77443.85000000001</v>
+        <v>28233.37</v>
       </c>
       <c r="M9" t="n">
-        <v>77443.85000000001</v>
+        <v>28233.37</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,10 +748,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>4699.16</v>
+        <v>5667.45</v>
       </c>
       <c r="I10" t="n">
-        <v>4699.16</v>
+        <v>5667.45</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,26 +760,26 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>4193.66</v>
+        <v>112804.12</v>
       </c>
       <c r="M10" t="n">
-        <v>4193.66</v>
+        <v>112804.12</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -791,28 +791,28 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>3933.48</v>
+        <v>5177.37</v>
       </c>
       <c r="I11" t="n">
-        <v>3933.48</v>
+        <v>5177.37</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>3916.42</v>
       </c>
       <c r="L11" t="n">
-        <v>114538.09</v>
+        <v>103682.37</v>
       </c>
       <c r="M11" t="n">
-        <v>114538.09</v>
+        <v>107598.79</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>3468.29</v>
+        <v>5019.7</v>
       </c>
       <c r="I12" t="n">
-        <v>3468.29</v>
+        <v>5019.7</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,16 +846,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>47900.16</v>
+        <v>77443.85000000001</v>
       </c>
       <c r="M12" t="n">
-        <v>47900.16</v>
+        <v>77443.85000000001</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,28 +877,28 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>3443.75</v>
+        <v>4699.16</v>
       </c>
       <c r="I13" t="n">
-        <v>3443.75</v>
+        <v>4699.16</v>
       </c>
       <c r="J13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>3916.42</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>105415.99</v>
+        <v>4193.66</v>
       </c>
       <c r="M13" t="n">
-        <v>109332.41</v>
+        <v>4193.66</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>3215.73</v>
+        <v>3468.29</v>
       </c>
       <c r="I14" t="n">
-        <v>3215.73</v>
+        <v>3468.29</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,10 +932,10 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>28233.37</v>
+        <v>47900.16</v>
       </c>
       <c r="M14" t="n">
-        <v>28233.37</v>
+        <v>47900.16</v>
       </c>
     </row>
     <row r="15">
@@ -1743,16 +1743,16 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K33" t="n">
-        <v>2211997.08</v>
+        <v>90049.44</v>
       </c>
       <c r="L33" t="n">
-        <v>2150747.29</v>
+        <v>28799.65</v>
       </c>
       <c r="M33" t="n">
-        <v>4362744.37</v>
+        <v>118849.09</v>
       </c>
     </row>
     <row r="34">

</xml_diff>

<commit_message>
data: update Pagado / Pendiente report to August 11 2026 cutoff date
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>10 de agosto de 2026</t>
+          <t>11 de agosto de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -478,7 +478,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>DESIREE DE LA PE╤A OROZCO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -554,7 +554,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -576,28 +576,28 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>8476.02</v>
+        <v>13525.02</v>
       </c>
       <c r="I6" t="n">
-        <v>8476.02</v>
+        <v>13525.02</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>3916.42</v>
       </c>
       <c r="L6" t="n">
-        <v>5756.97</v>
+        <v>98542.37</v>
       </c>
       <c r="M6" t="n">
-        <v>5756.97</v>
+        <v>102458.79</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -619,10 +619,10 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>8393.23</v>
+        <v>13506.29</v>
       </c>
       <c r="I7" t="n">
-        <v>8393.23</v>
+        <v>13506.29</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,16 +631,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>293606.54</v>
+        <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>293606.54</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>ANDREA CELESTE IBA╤EZ RINCON</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -662,10 +662,10 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>7537.55</v>
+        <v>8476.02</v>
       </c>
       <c r="I8" t="n">
-        <v>7537.55</v>
+        <v>8476.02</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,16 +674,16 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>72817.25999999999</v>
+        <v>5756.97</v>
       </c>
       <c r="M8" t="n">
-        <v>72817.25999999999</v>
+        <v>5756.97</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,22 +693,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>2019.94</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>4273.63</v>
+        <v>8393.23</v>
       </c>
       <c r="I9" t="n">
-        <v>6293.57</v>
+        <v>8393.23</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,26 +717,26 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>28233.37</v>
+        <v>293606.54</v>
       </c>
       <c r="M9" t="n">
-        <v>28233.37</v>
+        <v>293606.54</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,10 +748,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>5667.45</v>
+        <v>7537.55</v>
       </c>
       <c r="I10" t="n">
-        <v>5667.45</v>
+        <v>7537.55</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,16 +760,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>112804.12</v>
+        <v>72817.25999999999</v>
       </c>
       <c r="M10" t="n">
-        <v>112804.12</v>
+        <v>72817.25999999999</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,50 +779,50 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>PAULINA LIZBETH SOTO MU╤IZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>2019.94</v>
       </c>
       <c r="H11" t="n">
-        <v>5177.37</v>
+        <v>4273.63</v>
       </c>
       <c r="I11" t="n">
-        <v>5177.37</v>
+        <v>6293.57</v>
       </c>
       <c r="J11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>3916.42</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>103682.37</v>
+        <v>28233.37</v>
       </c>
       <c r="M11" t="n">
-        <v>107598.79</v>
+        <v>28233.37</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>5019.7</v>
+        <v>5667.45</v>
       </c>
       <c r="I12" t="n">
-        <v>5019.7</v>
+        <v>5667.45</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,26 +846,26 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>77443.85000000001</v>
+        <v>112804.12</v>
       </c>
       <c r="M12" t="n">
-        <v>77443.85000000001</v>
+        <v>112804.12</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,10 +877,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>4699.16</v>
+        <v>5025.06</v>
       </c>
       <c r="I13" t="n">
-        <v>4699.16</v>
+        <v>5025.06</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -889,16 +889,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>4193.66</v>
+        <v>23315.2</v>
       </c>
       <c r="M13" t="n">
-        <v>4193.66</v>
+        <v>23315.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>ORLANDA JIMENA CERVANTES NU╤EZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>3468.29</v>
+        <v>5019.7</v>
       </c>
       <c r="I14" t="n">
-        <v>3468.29</v>
+        <v>5019.7</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>47900.16</v>
+        <v>77443.85000000001</v>
       </c>
       <c r="M14" t="n">
-        <v>47900.16</v>
+        <v>77443.85000000001</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>2960.97</v>
+        <v>4699.16</v>
       </c>
       <c r="I15" t="n">
-        <v>2960.97</v>
+        <v>4699.16</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>4193.66</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>4193.66</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>2439.24</v>
+        <v>3468.29</v>
       </c>
       <c r="I16" t="n">
-        <v>2439.24</v>
+        <v>3468.29</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>7690.17</v>
+        <v>42067.73</v>
       </c>
       <c r="M16" t="n">
-        <v>7690.17</v>
+        <v>42067.73</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,22 +1037,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>EVELYN CAROLINA VENEGAS I╤IGUEZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>2396.76</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>2960.97</v>
       </c>
       <c r="I17" t="n">
-        <v>2396.76</v>
+        <v>2960.97</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,41 +1061,41 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>26364.37</v>
+        <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>26364.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>63441</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>2396.76</v>
       </c>
       <c r="H18" t="n">
-        <v>1843.19</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>1843.19</v>
+        <v>2396.76</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,26 +1104,26 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>1843.19</v>
+        <v>26364.37</v>
       </c>
       <c r="M18" t="n">
-        <v>1843.19</v>
+        <v>26364.37</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>63441</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2511</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>1757.71</v>
+        <v>1843.19</v>
       </c>
       <c r="I19" t="n">
-        <v>1757.71</v>
+        <v>1843.19</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,16 +1147,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>9080.91</v>
+        <v>1843.19</v>
       </c>
       <c r="M19" t="n">
-        <v>9080.91</v>
+        <v>1843.19</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>1627.21</v>
+        <v>1757.71</v>
       </c>
       <c r="I20" t="n">
-        <v>1627.21</v>
+        <v>1757.71</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,16 +1190,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>15800.91</v>
+        <v>9080.91</v>
       </c>
       <c r="M20" t="n">
-        <v>15800.91</v>
+        <v>9080.91</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>GABRIELA CASTA╤EDA SALAZAR</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>1659.4</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>1659.4</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,16 +1233,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>49020.81</v>
+        <v>98068.24000000001</v>
       </c>
       <c r="M21" t="n">
-        <v>49020.81</v>
+        <v>98068.24000000001</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,38 +1264,38 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>1627.21</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>1627.21</v>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>24377.75</v>
+        <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>26239.01</v>
+        <v>15800.91</v>
       </c>
       <c r="M22" t="n">
-        <v>50616.76</v>
+        <v>15800.91</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1313,32 +1313,32 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>33305.7</v>
       </c>
       <c r="L23" t="n">
-        <v>27395.54</v>
+        <v>49020.81</v>
       </c>
       <c r="M23" t="n">
-        <v>27395.54</v>
+        <v>82326.50999999999</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1356,22 +1356,22 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>26341.77</v>
       </c>
       <c r="L24" t="n">
-        <v>109437.94</v>
+        <v>26239.01</v>
       </c>
       <c r="M24" t="n">
-        <v>109437.94</v>
+        <v>52580.78</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1399,32 +1399,32 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>18368.13</v>
       </c>
       <c r="L25" t="n">
-        <v>20847.16</v>
+        <v>45763.67</v>
       </c>
       <c r="M25" t="n">
-        <v>20847.16</v>
+        <v>64131.8</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>20285.63</v>
+        <v>109437.94</v>
       </c>
       <c r="M26" t="n">
-        <v>20285.63</v>
+        <v>109437.94</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1491,16 +1491,16 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>28340.31</v>
+        <v>20847.16</v>
       </c>
       <c r="M27" t="n">
-        <v>28340.31</v>
+        <v>20847.16</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>3381.58</v>
+        <v>20285.63</v>
       </c>
       <c r="M28" t="n">
-        <v>3381.58</v>
+        <v>20285.63</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1577,26 +1577,26 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>19092.22</v>
+        <v>3381.58</v>
       </c>
       <c r="M29" t="n">
-        <v>19092.22</v>
+        <v>3381.58</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>HANA SOFIA LOPEZ QUI╤ONEZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1620,26 +1620,26 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>8530.73</v>
+        <v>19092.22</v>
       </c>
       <c r="M30" t="n">
-        <v>8530.73</v>
+        <v>19092.22</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>20683.11</v>
+        <v>8530.73</v>
       </c>
       <c r="M31" t="n">
-        <v>20683.11</v>
+        <v>8530.73</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>ANA LAURA CONTRERAS I╤IGUEZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1706,16 +1706,16 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>12581.61</v>
+        <v>20683.11</v>
       </c>
       <c r="M32" t="n">
-        <v>12581.61</v>
+        <v>20683.11</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1743,22 +1743,22 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>90049.44</v>
+        <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>28799.65</v>
+        <v>12581.61</v>
       </c>
       <c r="M33" t="n">
-        <v>118849.09</v>
+        <v>12581.61</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1786,22 +1786,22 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>90049.44</v>
       </c>
       <c r="L34" t="n">
-        <v>1425.78</v>
+        <v>28799.65</v>
       </c>
       <c r="M34" t="n">
-        <v>1425.78</v>
+        <v>118849.09</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>3035.72</v>
+        <v>1425.78</v>
       </c>
       <c r="M35" t="n">
-        <v>3035.72</v>
+        <v>1425.78</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>24832.77</v>
+        <v>3035.72</v>
       </c>
       <c r="M36" t="n">
-        <v>24832.77</v>
+        <v>3035.72</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1921,10 +1921,10 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>99727.64</v>
+        <v>24832.77</v>
       </c>
       <c r="M37" t="n">
-        <v>99727.64</v>
+        <v>24832.77</v>
       </c>
     </row>
     <row r="38">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>SAMUEL NU╤O RIVERA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>DARINKA URE╤A CASILLAS</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-08-17 10:15)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>11 de agosto de 2026</t>
+          <t>13 de agosto de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -478,7 +478,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PE╤A OROZCO</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -511,32 +511,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>2019.94</v>
       </c>
       <c r="H5" t="n">
-        <v>21079.98</v>
+        <v>35508.38</v>
       </c>
       <c r="I5" t="n">
-        <v>21079.98</v>
+        <v>37528.32</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -545,16 +545,16 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>49434.03</v>
+        <v>28233.37</v>
       </c>
       <c r="M5" t="n">
-        <v>49434.03</v>
+        <v>28233.37</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,40 +564,40 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>33305.7</v>
       </c>
       <c r="H6" t="n">
-        <v>13525.02</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>13525.02</v>
+        <v>33305.7</v>
       </c>
       <c r="J6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>3916.42</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>98542.37</v>
+        <v>49020.81</v>
       </c>
       <c r="M6" t="n">
-        <v>102458.79</v>
+        <v>49020.81</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -619,28 +619,28 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>13506.29</v>
+        <v>15302.69</v>
       </c>
       <c r="I7" t="n">
-        <v>13506.29</v>
+        <v>15302.69</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>1958.21</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>75224.37</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>77182.58</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBA╤EZ RINCON</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -662,10 +662,10 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>8476.02</v>
+        <v>13506.29</v>
       </c>
       <c r="I8" t="n">
-        <v>8476.02</v>
+        <v>13506.29</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,26 +674,26 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>5756.97</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>5756.97</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -705,10 +705,10 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>8393.23</v>
+        <v>11483.43</v>
       </c>
       <c r="I9" t="n">
-        <v>8393.23</v>
+        <v>11483.43</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,16 +717,16 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>293606.54</v>
+        <v>106988.14</v>
       </c>
       <c r="M9" t="n">
-        <v>293606.54</v>
+        <v>106988.14</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,10 +748,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>7537.55</v>
+        <v>8476.02</v>
       </c>
       <c r="I10" t="n">
-        <v>7537.55</v>
+        <v>8476.02</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,16 +760,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>72817.25999999999</v>
+        <v>5756.97</v>
       </c>
       <c r="M10" t="n">
-        <v>72817.25999999999</v>
+        <v>5756.97</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,22 +779,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MU╤IZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>2019.94</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>4273.63</v>
+        <v>8393.23</v>
       </c>
       <c r="I11" t="n">
-        <v>6293.57</v>
+        <v>8393.23</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,26 +803,26 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>28233.37</v>
+        <v>291024.67</v>
       </c>
       <c r="M11" t="n">
-        <v>28233.37</v>
+        <v>291024.67</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,22 +834,22 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>5667.45</v>
+        <v>7537.55</v>
       </c>
       <c r="I12" t="n">
-        <v>5667.45</v>
+        <v>7537.55</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>58297.52</v>
       </c>
       <c r="L12" t="n">
-        <v>112804.12</v>
+        <v>72817.25999999999</v>
       </c>
       <c r="M12" t="n">
-        <v>112804.12</v>
+        <v>131114.78</v>
       </c>
     </row>
     <row r="13">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NU╤EZ</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -984,17 +984,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>3468.29</v>
+        <v>3954.41</v>
       </c>
       <c r="I16" t="n">
-        <v>3468.29</v>
+        <v>3954.41</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>42067.73</v>
+        <v>8530.73</v>
       </c>
       <c r="M16" t="n">
-        <v>42067.73</v>
+        <v>8530.73</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS I╤IGUEZ</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>2960.97</v>
+        <v>3468.29</v>
       </c>
       <c r="I17" t="n">
-        <v>2960.97</v>
+        <v>3468.29</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>42067.73</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>42067.73</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,22 +1080,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>2396.76</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>2960.97</v>
       </c>
       <c r="I18" t="n">
-        <v>2396.76</v>
+        <v>2960.97</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,41 +1104,41 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>26364.37</v>
+        <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>26364.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>63441</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>2396.76</v>
       </c>
       <c r="H19" t="n">
-        <v>1843.19</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>1843.19</v>
+        <v>2396.76</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,16 +1147,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>1843.19</v>
+        <v>26364.37</v>
       </c>
       <c r="M19" t="n">
-        <v>1843.19</v>
+        <v>26364.37</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,50 +1166,50 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>1454.68</v>
       </c>
       <c r="H20" t="n">
-        <v>1757.71</v>
+        <v>509.43</v>
       </c>
       <c r="I20" t="n">
-        <v>1757.71</v>
+        <v>1964.11</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>24377.75</v>
       </c>
       <c r="L20" t="n">
-        <v>9080.91</v>
+        <v>26239.01</v>
       </c>
       <c r="M20" t="n">
-        <v>9080.91</v>
+        <v>50616.76</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>63441</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2511</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GABRIELA CASTA╤EDA SALAZAR</t>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>1659.4</v>
+        <v>1843.19</v>
       </c>
       <c r="I21" t="n">
-        <v>1659.4</v>
+        <v>1843.19</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,26 +1233,26 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>98068.24000000001</v>
+        <v>1843.19</v>
       </c>
       <c r="M21" t="n">
-        <v>98068.24000000001</v>
+        <v>1843.19</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>1627.21</v>
+        <v>1763.6</v>
       </c>
       <c r="I22" t="n">
-        <v>1627.21</v>
+        <v>1763.6</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,16 +1276,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>15800.91</v>
+        <v>107674.33</v>
       </c>
       <c r="M22" t="n">
-        <v>15800.91</v>
+        <v>107674.33</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,28 +1307,28 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>1757.71</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>1757.71</v>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>33305.7</v>
+        <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>49020.81</v>
+        <v>9080.91</v>
       </c>
       <c r="M23" t="n">
-        <v>82326.50999999999</v>
+        <v>9080.91</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,38 +1350,38 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>1659.4</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>1659.4</v>
       </c>
       <c r="J24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>26341.77</v>
+        <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>26239.01</v>
+        <v>98068.24000000001</v>
       </c>
       <c r="M24" t="n">
-        <v>52580.78</v>
+        <v>98068.24000000001</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1393,28 +1393,28 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>1627.21</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>1627.21</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>18368.13</v>
+        <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>45763.67</v>
+        <v>15800.91</v>
       </c>
       <c r="M25" t="n">
-        <v>64131.8</v>
+        <v>15800.91</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1442,22 +1442,22 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>18368.13</v>
       </c>
       <c r="L26" t="n">
-        <v>109437.94</v>
+        <v>45763.67</v>
       </c>
       <c r="M26" t="n">
-        <v>109437.94</v>
+        <v>64131.8</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1476,10 +1476,10 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>-21079.98</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>21079.98</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -1491,26 +1491,26 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>20847.16</v>
+        <v>70514.00999999999</v>
       </c>
       <c r="M27" t="n">
-        <v>20847.16</v>
+        <v>70514.00999999999</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>20285.63</v>
+        <v>20847.16</v>
       </c>
       <c r="M28" t="n">
-        <v>20285.63</v>
+        <v>20847.16</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1577,16 +1577,16 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>3381.58</v>
+        <v>20285.63</v>
       </c>
       <c r="M29" t="n">
-        <v>3381.58</v>
+        <v>20285.63</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUI╤ONEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1620,26 +1620,26 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>19092.22</v>
+        <v>3381.58</v>
       </c>
       <c r="M30" t="n">
-        <v>19092.22</v>
+        <v>3381.58</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1663,10 +1663,10 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>8530.73</v>
+        <v>19092.22</v>
       </c>
       <c r="M31" t="n">
-        <v>8530.73</v>
+        <v>19092.22</v>
       </c>
     </row>
     <row r="32">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS I╤IGUEZ</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SAMUEL NU╤O RIVERA</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>DARINKA URE╤A CASILLAS</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-08-18 11:14)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>13 de agosto de 2026</t>
+          <t>14 de agosto de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -597,7 +597,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -619,38 +619,38 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>15302.69</v>
+        <v>16532.42</v>
       </c>
       <c r="I7" t="n">
-        <v>15302.69</v>
+        <v>16532.42</v>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>1958.21</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>75224.37</v>
+        <v>65931.12</v>
       </c>
       <c r="M7" t="n">
-        <v>77182.58</v>
+        <v>65931.12</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -662,10 +662,10 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>13506.29</v>
+        <v>15495.26</v>
       </c>
       <c r="I8" t="n">
-        <v>13506.29</v>
+        <v>15495.26</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,26 +674,26 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>102976.31</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>102976.31</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -705,10 +705,10 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>11483.43</v>
+        <v>15302.69</v>
       </c>
       <c r="I9" t="n">
-        <v>11483.43</v>
+        <v>15302.69</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,16 +717,16 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>106988.14</v>
+        <v>53684.04</v>
       </c>
       <c r="M9" t="n">
-        <v>106988.14</v>
+        <v>53684.04</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,10 +748,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>8476.02</v>
+        <v>13506.29</v>
       </c>
       <c r="I10" t="n">
-        <v>8476.02</v>
+        <v>13506.29</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,16 +760,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>5756.97</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>5756.97</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -791,10 +791,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>8393.23</v>
+        <v>8476.02</v>
       </c>
       <c r="I11" t="n">
-        <v>8393.23</v>
+        <v>8476.02</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,16 +803,16 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>291024.67</v>
+        <v>5756.97</v>
       </c>
       <c r="M11" t="n">
-        <v>291024.67</v>
+        <v>5756.97</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,38 +834,38 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>7537.55</v>
+        <v>8393.23</v>
       </c>
       <c r="I12" t="n">
-        <v>7537.55</v>
+        <v>8393.23</v>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>58297.52</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>72817.25999999999</v>
+        <v>291024.67</v>
       </c>
       <c r="M12" t="n">
-        <v>131114.78</v>
+        <v>291024.67</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,38 +877,38 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>5025.06</v>
+        <v>7537.55</v>
       </c>
       <c r="I13" t="n">
-        <v>5025.06</v>
+        <v>7537.55</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>58297.52</v>
       </c>
       <c r="L13" t="n">
-        <v>23315.2</v>
+        <v>72817.25999999999</v>
       </c>
       <c r="M13" t="n">
-        <v>23315.2</v>
+        <v>131114.78</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>5019.7</v>
+        <v>5025.06</v>
       </c>
       <c r="I14" t="n">
-        <v>5019.7</v>
+        <v>5025.06</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,10 +932,10 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>77443.85000000001</v>
+        <v>23315.2</v>
       </c>
       <c r="M14" t="n">
-        <v>77443.85000000001</v>
+        <v>23315.2</v>
       </c>
     </row>
     <row r="15">
@@ -1485,16 +1485,16 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>16392.68</v>
       </c>
       <c r="L27" t="n">
         <v>70514.00999999999</v>
       </c>
       <c r="M27" t="n">
-        <v>70514.00999999999</v>
+        <v>86906.69</v>
       </c>
     </row>
     <row r="28">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-08-19 13:46)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>14 de agosto de 2026</t>
+          <t>18 de agosto de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -490,10 +490,10 @@
         <v>162964</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>8374.200000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>162964</v>
+        <v>171338.2</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -502,10 +502,10 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>84466.67</v>
+        <v>80161.03</v>
       </c>
       <c r="M4" t="n">
-        <v>84466.67</v>
+        <v>80161.03</v>
       </c>
     </row>
     <row r="5">
@@ -597,32 +597,32 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>18368.13</v>
       </c>
       <c r="H7" t="n">
-        <v>16532.42</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>16532.42</v>
+        <v>18368.13</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,10 +631,10 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>65931.12</v>
+        <v>45763.67</v>
       </c>
       <c r="M7" t="n">
-        <v>65931.12</v>
+        <v>45763.67</v>
       </c>
     </row>
     <row r="8">
@@ -662,10 +662,10 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>15495.26</v>
+        <v>17290.35</v>
       </c>
       <c r="I8" t="n">
-        <v>15495.26</v>
+        <v>17290.35</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,16 +674,16 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>102976.31</v>
+        <v>101181.23</v>
       </c>
       <c r="M8" t="n">
-        <v>102976.31</v>
+        <v>101181.23</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -705,10 +705,10 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>15302.69</v>
+        <v>16532.42</v>
       </c>
       <c r="I9" t="n">
-        <v>15302.69</v>
+        <v>16532.42</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,41 +717,41 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>53684.04</v>
+        <v>65931.12</v>
       </c>
       <c r="M9" t="n">
-        <v>53684.04</v>
+        <v>65931.12</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>-19514.59</v>
       </c>
       <c r="H10" t="n">
-        <v>13506.29</v>
+        <v>35907.27</v>
       </c>
       <c r="I10" t="n">
-        <v>13506.29</v>
+        <v>16392.68</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,16 +760,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>70514.00999999999</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>70514.00999999999</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -791,10 +791,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>8476.02</v>
+        <v>15302.69</v>
       </c>
       <c r="I11" t="n">
-        <v>8476.02</v>
+        <v>15302.69</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,16 +803,16 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>5756.97</v>
+        <v>53684.04</v>
       </c>
       <c r="M11" t="n">
-        <v>5756.97</v>
+        <v>53684.04</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>8393.23</v>
+        <v>13506.29</v>
       </c>
       <c r="I12" t="n">
-        <v>8393.23</v>
+        <v>13506.29</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,16 +846,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>291024.67</v>
+        <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>291024.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,38 +877,38 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>7537.55</v>
+        <v>12093.46</v>
       </c>
       <c r="I13" t="n">
-        <v>7537.55</v>
+        <v>12093.46</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>58297.52</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>72817.25999999999</v>
+        <v>33442.54</v>
       </c>
       <c r="M13" t="n">
-        <v>131114.78</v>
+        <v>33442.54</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,28 +920,28 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>5025.06</v>
+        <v>10530.97</v>
       </c>
       <c r="I14" t="n">
-        <v>5025.06</v>
+        <v>10530.97</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>58297.52</v>
       </c>
       <c r="L14" t="n">
-        <v>23315.2</v>
+        <v>69823.8</v>
       </c>
       <c r="M14" t="n">
-        <v>23315.2</v>
+        <v>128121.32</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>4699.16</v>
+        <v>9886.120000000001</v>
       </c>
       <c r="I15" t="n">
-        <v>4699.16</v>
+        <v>9886.120000000001</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,26 +975,26 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>4193.66</v>
+        <v>18063.4</v>
       </c>
       <c r="M15" t="n">
-        <v>4193.66</v>
+        <v>18063.4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>3954.41</v>
+        <v>8476.02</v>
       </c>
       <c r="I16" t="n">
-        <v>3954.41</v>
+        <v>8476.02</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>8530.73</v>
+        <v>5756.97</v>
       </c>
       <c r="M16" t="n">
-        <v>8530.73</v>
+        <v>5756.97</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>3468.29</v>
+        <v>8393.23</v>
       </c>
       <c r="I17" t="n">
-        <v>3468.29</v>
+        <v>8393.23</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>42067.73</v>
+        <v>291024.67</v>
       </c>
       <c r="M17" t="n">
-        <v>42067.73</v>
+        <v>291024.67</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>2960.97</v>
+        <v>7590.14</v>
       </c>
       <c r="I18" t="n">
-        <v>2960.97</v>
+        <v>7590.14</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,41 +1104,41 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>92596.31</v>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>92596.31</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>2396.76</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>6087.09</v>
       </c>
       <c r="I19" t="n">
-        <v>2396.76</v>
+        <v>6087.09</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,16 +1147,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>26364.37</v>
+        <v>6398.05</v>
       </c>
       <c r="M19" t="n">
-        <v>26364.37</v>
+        <v>6398.05</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,50 +1166,50 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>1454.68</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>509.43</v>
+        <v>6049.46</v>
       </c>
       <c r="I20" t="n">
-        <v>1964.11</v>
+        <v>6049.46</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>24377.75</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>26239.01</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>50616.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>63441</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>1843.19</v>
+        <v>5808.77</v>
       </c>
       <c r="I21" t="n">
-        <v>1843.19</v>
+        <v>5808.77</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,26 +1233,26 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>1843.19</v>
+        <v>103783.01</v>
       </c>
       <c r="M21" t="n">
-        <v>1843.19</v>
+        <v>103783.01</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>1763.6</v>
+        <v>5465.98</v>
       </c>
       <c r="I22" t="n">
-        <v>1763.6</v>
+        <v>5465.98</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,16 +1276,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>107674.33</v>
+        <v>57010.81</v>
       </c>
       <c r="M22" t="n">
-        <v>107674.33</v>
+        <v>57010.81</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,10 +1307,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>1757.71</v>
+        <v>5443.04</v>
       </c>
       <c r="I23" t="n">
-        <v>1757.71</v>
+        <v>5443.04</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,26 +1319,26 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>9080.91</v>
+        <v>17698.48</v>
       </c>
       <c r="M23" t="n">
-        <v>9080.91</v>
+        <v>17698.48</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>1659.4</v>
+        <v>5025.06</v>
       </c>
       <c r="I24" t="n">
-        <v>1659.4</v>
+        <v>5025.06</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,16 +1362,16 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>98068.24000000001</v>
+        <v>23315.2</v>
       </c>
       <c r="M24" t="n">
-        <v>98068.24000000001</v>
+        <v>23315.2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1393,10 +1393,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>1627.21</v>
+        <v>4699.16</v>
       </c>
       <c r="I25" t="n">
-        <v>1627.21</v>
+        <v>4699.16</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,26 +1405,26 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>15800.91</v>
+        <v>4193.66</v>
       </c>
       <c r="M25" t="n">
-        <v>15800.91</v>
+        <v>4193.66</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,81 +1436,81 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>2960.97</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>2960.97</v>
       </c>
       <c r="J26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>18368.13</v>
+        <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>45763.67</v>
+        <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>64131.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>-21079.98</v>
+        <v>2396.76</v>
       </c>
       <c r="H27" t="n">
-        <v>21079.98</v>
+        <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>2396.76</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>16392.68</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>70514.00999999999</v>
+        <v>26364.37</v>
       </c>
       <c r="M27" t="n">
-        <v>86906.69</v>
+        <v>26364.37</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>2068.31</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>2068.31</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>20847.16</v>
+        <v>18614.8</v>
       </c>
       <c r="M28" t="n">
-        <v>20847.16</v>
+        <v>18614.8</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,50 +1553,50 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>1454.68</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>509.43</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>1964.11</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>24377.75</v>
       </c>
       <c r="L29" t="n">
-        <v>20285.63</v>
+        <v>26239.01</v>
       </c>
       <c r="M29" t="n">
-        <v>20285.63</v>
+        <v>50616.76</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>63441</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2511</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>1843.19</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>1843.19</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,26 +1620,26 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>3381.58</v>
+        <v>1843.19</v>
       </c>
       <c r="M30" t="n">
-        <v>3381.58</v>
+        <v>1843.19</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>1777.67</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>1777.67</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>19092.22</v>
+        <v>19069.49</v>
       </c>
       <c r="M31" t="n">
-        <v>19092.22</v>
+        <v>19069.49</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1694,10 +1694,10 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>1757.71</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>1757.71</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,16 +1706,16 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>20683.11</v>
+        <v>9080.91</v>
       </c>
       <c r="M32" t="n">
-        <v>20683.11</v>
+        <v>9080.91</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>1627.21</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>1627.21</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,16 +1749,16 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>12581.61</v>
+        <v>15800.91</v>
       </c>
       <c r="M33" t="n">
-        <v>12581.61</v>
+        <v>15800.91</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1786,22 +1786,22 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>90049.44</v>
+        <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>28799.65</v>
+        <v>20285.63</v>
       </c>
       <c r="M34" t="n">
-        <v>118849.09</v>
+        <v>20285.63</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>1425.78</v>
+        <v>3381.58</v>
       </c>
       <c r="M35" t="n">
-        <v>1425.78</v>
+        <v>3381.58</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>3035.72</v>
+        <v>19092.22</v>
       </c>
       <c r="M36" t="n">
-        <v>3035.72</v>
+        <v>19092.22</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>24832.77</v>
+        <v>12581.61</v>
       </c>
       <c r="M37" t="n">
-        <v>24832.77</v>
+        <v>12581.61</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1958,22 +1958,22 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>90049.44</v>
       </c>
       <c r="L38" t="n">
-        <v>24095.39</v>
+        <v>28799.65</v>
       </c>
       <c r="M38" t="n">
-        <v>24095.39</v>
+        <v>118849.09</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>6049.41</v>
+        <v>1425.78</v>
       </c>
       <c r="M39" t="n">
-        <v>6049.41</v>
+        <v>1425.78</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>3208.07</v>
+        <v>3035.72</v>
       </c>
       <c r="M40" t="n">
-        <v>3208.07</v>
+        <v>3035.72</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>62476.76</v>
+        <v>24095.39</v>
       </c>
       <c r="M41" t="n">
-        <v>62476.76</v>
+        <v>24095.39</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2130,22 +2130,22 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K42" t="n">
-        <v>5042.65</v>
+        <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>130020.2</v>
+        <v>3208.07</v>
       </c>
       <c r="M42" t="n">
-        <v>135062.85</v>
+        <v>3208.07</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2173,16 +2173,16 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>0</v>
+        <v>5042.65</v>
       </c>
       <c r="L43" t="n">
-        <v>23460.24</v>
+        <v>130020.2</v>
       </c>
       <c r="M43" t="n">
-        <v>23460.24</v>
+        <v>135062.85</v>
       </c>
     </row>
     <row r="44">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-08-24 12:26)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>19 de agosto de 2026</t>
+          <t>20 de agosto de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -496,16 +496,16 @@
         <v>171338.2</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>93618.86</v>
       </c>
       <c r="L4" t="n">
         <v>80161.03</v>
       </c>
       <c r="M4" t="n">
-        <v>80161.03</v>
+        <v>173779.89</v>
       </c>
     </row>
     <row r="5">
@@ -554,7 +554,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,22 +564,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>33305.7</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>52177.88</v>
       </c>
       <c r="I6" t="n">
-        <v>33305.7</v>
+        <v>52177.88</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,26 +588,26 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>49020.81</v>
+        <v>247240.02</v>
       </c>
       <c r="M6" t="n">
-        <v>49020.81</v>
+        <v>247240.02</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -616,13 +616,13 @@
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>-19514.59</v>
+        <v>33305.7</v>
       </c>
       <c r="H7" t="n">
-        <v>37963.62</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>18449.03</v>
+        <v>33305.7</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,10 +631,10 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>68457.66</v>
+        <v>49020.81</v>
       </c>
       <c r="M7" t="n">
-        <v>68457.66</v>
+        <v>49020.81</v>
       </c>
     </row>
     <row r="8">
@@ -662,10 +662,10 @@
         <v>18368.13</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>1659.4</v>
       </c>
       <c r="I8" t="n">
-        <v>18368.13</v>
+        <v>20027.53</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,16 +674,16 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>45763.67</v>
+        <v>44104.27</v>
       </c>
       <c r="M8" t="n">
-        <v>45763.67</v>
+        <v>44104.27</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,22 +693,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>-19514.59</v>
       </c>
       <c r="H9" t="n">
-        <v>17290.35</v>
+        <v>37963.62</v>
       </c>
       <c r="I9" t="n">
-        <v>17290.35</v>
+        <v>18449.03</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,26 +717,26 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>101181.23</v>
+        <v>68457.66</v>
       </c>
       <c r="M9" t="n">
-        <v>101181.23</v>
+        <v>68457.66</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,10 +748,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>16532.42</v>
+        <v>17290.35</v>
       </c>
       <c r="I10" t="n">
-        <v>16532.42</v>
+        <v>17290.35</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,16 +760,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>65931.12</v>
+        <v>101181.23</v>
       </c>
       <c r="M10" t="n">
-        <v>65931.12</v>
+        <v>101181.23</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -791,10 +791,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>15302.69</v>
+        <v>16532.42</v>
       </c>
       <c r="I11" t="n">
-        <v>15302.69</v>
+        <v>16532.42</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,16 +803,16 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>53684.04</v>
+        <v>65931.12</v>
       </c>
       <c r="M11" t="n">
-        <v>53684.04</v>
+        <v>65931.12</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>15064.73</v>
+        <v>15302.69</v>
       </c>
       <c r="I12" t="n">
-        <v>15064.73</v>
+        <v>15302.69</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,16 +846,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>5220.9</v>
+        <v>53684.04</v>
       </c>
       <c r="M12" t="n">
-        <v>5220.9</v>
+        <v>53684.04</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,10 +877,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>13506.29</v>
+        <v>15064.73</v>
       </c>
       <c r="I13" t="n">
-        <v>13506.29</v>
+        <v>15064.73</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -889,16 +889,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>5220.9</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>5220.9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>12093.46</v>
+        <v>13506.29</v>
       </c>
       <c r="I14" t="n">
-        <v>12093.46</v>
+        <v>13506.29</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>33442.54</v>
+        <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>33442.54</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,28 +963,28 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>10530.97</v>
+        <v>12093.46</v>
       </c>
       <c r="I15" t="n">
-        <v>10530.97</v>
+        <v>12093.46</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>58297.52</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>69823.8</v>
+        <v>33442.54</v>
       </c>
       <c r="M15" t="n">
-        <v>128121.32</v>
+        <v>33442.54</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,28 +1006,28 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>9886.120000000001</v>
+        <v>10530.97</v>
       </c>
       <c r="I16" t="n">
-        <v>9886.120000000001</v>
+        <v>10530.97</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>58297.52</v>
       </c>
       <c r="L16" t="n">
-        <v>18063.4</v>
+        <v>69823.8</v>
       </c>
       <c r="M16" t="n">
-        <v>18063.4</v>
+        <v>128121.32</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>9749.9</v>
+        <v>9886.120000000001</v>
       </c>
       <c r="I17" t="n">
-        <v>9749.9</v>
+        <v>9886.120000000001</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>52726.89</v>
+        <v>18063.4</v>
       </c>
       <c r="M17" t="n">
-        <v>52726.89</v>
+        <v>18063.4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>8476.02</v>
+        <v>9749.9</v>
       </c>
       <c r="I18" t="n">
-        <v>8476.02</v>
+        <v>9749.9</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,16 +1104,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>5756.97</v>
+        <v>52726.89</v>
       </c>
       <c r="M18" t="n">
-        <v>5756.97</v>
+        <v>52726.89</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>8393.23</v>
+        <v>8476.02</v>
       </c>
       <c r="I19" t="n">
-        <v>8393.23</v>
+        <v>8476.02</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,10 +1147,10 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>291024.67</v>
+        <v>5756.97</v>
       </c>
       <c r="M19" t="n">
-        <v>291024.67</v>
+        <v>5756.97</v>
       </c>
     </row>
     <row r="20">
@@ -1242,17 +1242,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>6087.09</v>
+        <v>7004.2</v>
       </c>
       <c r="I22" t="n">
-        <v>6087.09</v>
+        <v>7004.2</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,26 +1276,26 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>6398.05</v>
+        <v>1888.66</v>
       </c>
       <c r="M22" t="n">
-        <v>6398.05</v>
+        <v>1888.66</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,10 +1307,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>6049.46</v>
+        <v>6087.09</v>
       </c>
       <c r="I23" t="n">
-        <v>6049.46</v>
+        <v>6087.09</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,69 +1319,69 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>6398.05</v>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>6398.05</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>6086.13</v>
       </c>
       <c r="H24" t="n">
-        <v>5808.77</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>5808.77</v>
+        <v>6086.13</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>114882.54</v>
       </c>
       <c r="L24" t="n">
-        <v>103783.01</v>
+        <v>66947.41</v>
       </c>
       <c r="M24" t="n">
-        <v>103783.01</v>
+        <v>181829.95</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1393,10 +1393,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>5025.06</v>
+        <v>6049.46</v>
       </c>
       <c r="I25" t="n">
-        <v>5025.06</v>
+        <v>6049.46</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,26 +1405,26 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>23315.2</v>
+        <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>23315.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>4699.16</v>
+        <v>5808.77</v>
       </c>
       <c r="I26" t="n">
-        <v>4699.16</v>
+        <v>5808.77</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,26 +1448,26 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>4193.66</v>
+        <v>103783.01</v>
       </c>
       <c r="M26" t="n">
-        <v>4193.66</v>
+        <v>103783.01</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,10 +1479,10 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>4266.5</v>
+        <v>5025.06</v>
       </c>
       <c r="I27" t="n">
-        <v>4266.5</v>
+        <v>5025.06</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1491,16 +1491,16 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>6572.15</v>
+        <v>23315.2</v>
       </c>
       <c r="M27" t="n">
-        <v>6572.15</v>
+        <v>23315.2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>2960.97</v>
+        <v>4266.5</v>
       </c>
       <c r="I28" t="n">
-        <v>2960.97</v>
+        <v>4266.5</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>0</v>
+        <v>6572.15</v>
       </c>
       <c r="M28" t="n">
-        <v>0</v>
+        <v>6572.15</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,22 +1553,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>2396.76</v>
+        <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>2960.97</v>
       </c>
       <c r="I29" t="n">
-        <v>2396.76</v>
+        <v>2960.97</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,16 +1577,16 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>26364.37</v>
+        <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>26364.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,22 +1596,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>2396.76</v>
       </c>
       <c r="H30" t="n">
-        <v>2068.31</v>
+        <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>2068.31</v>
+        <v>2396.76</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>18614.8</v>
+        <v>26364.37</v>
       </c>
       <c r="M30" t="n">
-        <v>18614.8</v>
+        <v>26364.37</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,93 +1639,93 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>1454.68</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>509.43</v>
+        <v>2068.31</v>
       </c>
       <c r="I31" t="n">
-        <v>1964.11</v>
+        <v>2068.31</v>
       </c>
       <c r="J31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>24377.75</v>
+        <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>26239.01</v>
+        <v>18614.8</v>
       </c>
       <c r="M31" t="n">
-        <v>50616.76</v>
+        <v>18614.8</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>63441</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>1454.68</v>
       </c>
       <c r="H32" t="n">
-        <v>1843.19</v>
+        <v>509.43</v>
       </c>
       <c r="I32" t="n">
-        <v>1843.19</v>
+        <v>1964.11</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K32" t="n">
-        <v>0</v>
+        <v>24377.75</v>
       </c>
       <c r="L32" t="n">
-        <v>1843.19</v>
+        <v>26239.01</v>
       </c>
       <c r="M32" t="n">
-        <v>1843.19</v>
+        <v>50616.76</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>63441</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2511</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>1777.67</v>
+        <v>1843.19</v>
       </c>
       <c r="I33" t="n">
-        <v>1777.67</v>
+        <v>1843.19</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,26 +1749,26 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>19069.49</v>
+        <v>1843.19</v>
       </c>
       <c r="M33" t="n">
-        <v>19069.49</v>
+        <v>1843.19</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>1627.21</v>
+        <v>1777.67</v>
       </c>
       <c r="I34" t="n">
-        <v>1627.21</v>
+        <v>1777.67</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,16 +1792,16 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>15800.91</v>
+        <v>19069.49</v>
       </c>
       <c r="M34" t="n">
-        <v>15800.91</v>
+        <v>19069.49</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>1699.41</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>1699.41</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>3381.58</v>
+        <v>17392.81</v>
       </c>
       <c r="M35" t="n">
-        <v>3381.58</v>
+        <v>17392.81</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>1627.21</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>1627.21</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>19092.22</v>
+        <v>15800.91</v>
       </c>
       <c r="M36" t="n">
-        <v>19092.22</v>
+        <v>15800.91</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>1595.73</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>1595.73</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>12581.61</v>
+        <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>12581.61</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1958,22 +1958,22 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>6086.13</v>
+        <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>66947.41</v>
+        <v>3381.58</v>
       </c>
       <c r="M38" t="n">
-        <v>73033.53999999999</v>
+        <v>3381.58</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>90049.44</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>28799.65</v>
+        <v>12581.61</v>
       </c>
       <c r="M39" t="n">
-        <v>118849.09</v>
+        <v>12581.61</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2044,22 +2044,22 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K40" t="n">
-        <v>0</v>
+        <v>90049.44</v>
       </c>
       <c r="L40" t="n">
-        <v>1425.78</v>
+        <v>28799.65</v>
       </c>
       <c r="M40" t="n">
-        <v>1425.78</v>
+        <v>118849.09</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>3035.72</v>
+        <v>1425.78</v>
       </c>
       <c r="M41" t="n">
-        <v>3035.72</v>
+        <v>1425.78</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2136,16 +2136,16 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>24095.39</v>
+        <v>3035.72</v>
       </c>
       <c r="M42" t="n">
-        <v>24095.39</v>
+        <v>3035.72</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2179,16 +2179,16 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>3208.07</v>
+        <v>24095.39</v>
       </c>
       <c r="M43" t="n">
-        <v>3208.07</v>
+        <v>24095.39</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2216,22 +2216,22 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>5042.65</v>
+        <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>130020.2</v>
+        <v>3208.07</v>
       </c>
       <c r="M44" t="n">
-        <v>135062.85</v>
+        <v>3208.07</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -2259,15 +2259,58 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K45" t="n">
-        <v>0</v>
+        <v>5042.65</v>
       </c>
       <c r="L45" t="n">
+        <v>130020.2</v>
+      </c>
+      <c r="M45" t="n">
+        <v>135062.85</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>65046</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2043</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="n">
         <v>6270.75</v>
       </c>
-      <c r="M45" t="n">
+      <c r="M46" t="n">
         <v>6270.75</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Actualizar reporte Pagado y Pendiente (Corte al 21 de agosto de 2026)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M46"/>
+  <dimension ref="A1:M47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>20 de agosto de 2026</t>
+          <t>21 de agosto de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -576,22 +576,22 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>52177.88</v>
+        <v>56135.2</v>
       </c>
       <c r="I6" t="n">
-        <v>52177.88</v>
+        <v>56135.2</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>84784.83</v>
       </c>
       <c r="L6" t="n">
-        <v>247240.02</v>
+        <v>243282.71</v>
       </c>
       <c r="M6" t="n">
-        <v>247240.02</v>
+        <v>328067.54</v>
       </c>
     </row>
     <row r="7">
@@ -803,10 +803,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>65931.12</v>
+        <v>62070.69</v>
       </c>
       <c r="M11" t="n">
-        <v>65931.12</v>
+        <v>62070.69</v>
       </c>
     </row>
     <row r="12">
@@ -1543,17 +1543,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>2960.97</v>
+        <v>3610.04</v>
       </c>
       <c r="I29" t="n">
-        <v>2960.97</v>
+        <v>3610.04</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,26 +1577,26 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>0</v>
+        <v>17237.12</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>17237.12</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1605,13 +1605,13 @@
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>2396.76</v>
+        <v>3052.25</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>2396.76</v>
+        <v>3052.25</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>26364.37</v>
+        <v>33574.79</v>
       </c>
       <c r="M30" t="n">
-        <v>26364.37</v>
+        <v>33574.79</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>2068.31</v>
+        <v>2960.97</v>
       </c>
       <c r="I31" t="n">
-        <v>2068.31</v>
+        <v>2960.97</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>18614.8</v>
+        <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>18614.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1691,41 +1691,41 @@
         <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>1454.68</v>
+        <v>2396.76</v>
       </c>
       <c r="H32" t="n">
-        <v>509.43</v>
+        <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>1964.11</v>
+        <v>2396.76</v>
       </c>
       <c r="J32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>24377.75</v>
+        <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>26239.01</v>
+        <v>26364.37</v>
       </c>
       <c r="M32" t="n">
-        <v>50616.76</v>
+        <v>26364.37</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>63441</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>1843.19</v>
+        <v>2068.31</v>
       </c>
       <c r="I33" t="n">
-        <v>1843.19</v>
+        <v>2068.31</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,69 +1749,69 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>1843.19</v>
+        <v>18614.8</v>
       </c>
       <c r="M33" t="n">
-        <v>1843.19</v>
+        <v>18614.8</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>1454.68</v>
       </c>
       <c r="H34" t="n">
-        <v>1777.67</v>
+        <v>509.43</v>
       </c>
       <c r="I34" t="n">
-        <v>1777.67</v>
+        <v>1964.11</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>24377.75</v>
       </c>
       <c r="L34" t="n">
-        <v>19069.49</v>
+        <v>26239.01</v>
       </c>
       <c r="M34" t="n">
-        <v>19069.49</v>
+        <v>50616.76</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>63441</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2511</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>1699.41</v>
+        <v>1843.19</v>
       </c>
       <c r="I35" t="n">
-        <v>1699.41</v>
+        <v>1843.19</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>17392.81</v>
+        <v>1843.19</v>
       </c>
       <c r="M35" t="n">
-        <v>17392.81</v>
+        <v>1843.19</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>1627.21</v>
+        <v>1699.41</v>
       </c>
       <c r="I36" t="n">
-        <v>1627.21</v>
+        <v>1699.41</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>15800.91</v>
+        <v>17392.81</v>
       </c>
       <c r="M36" t="n">
-        <v>15800.91</v>
+        <v>17392.81</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,28 +1909,28 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>1595.73</v>
+        <v>1627.21</v>
       </c>
       <c r="I37" t="n">
-        <v>1595.73</v>
+        <v>1627.21</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>1958.21</v>
       </c>
       <c r="L37" t="n">
-        <v>0</v>
+        <v>37341.24</v>
       </c>
       <c r="M37" t="n">
-        <v>0</v>
+        <v>39299.45</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1952,10 +1952,10 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>1595.73</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>1595.73</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>3381.58</v>
+        <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>3381.58</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>12581.61</v>
+        <v>3381.58</v>
       </c>
       <c r="M39" t="n">
-        <v>12581.61</v>
+        <v>3381.58</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2044,22 +2044,22 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K40" t="n">
-        <v>90049.44</v>
+        <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>28799.65</v>
+        <v>12581.61</v>
       </c>
       <c r="M40" t="n">
-        <v>118849.09</v>
+        <v>12581.61</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2087,22 +2087,22 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>90049.44</v>
       </c>
       <c r="L41" t="n">
-        <v>1425.78</v>
+        <v>28799.65</v>
       </c>
       <c r="M41" t="n">
-        <v>1425.78</v>
+        <v>118849.09</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2136,16 +2136,16 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>3035.72</v>
+        <v>1425.78</v>
       </c>
       <c r="M42" t="n">
-        <v>3035.72</v>
+        <v>1425.78</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2179,16 +2179,16 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>24095.39</v>
+        <v>3035.72</v>
       </c>
       <c r="M43" t="n">
-        <v>24095.39</v>
+        <v>3035.72</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2222,16 +2222,16 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>3208.07</v>
+        <v>24095.39</v>
       </c>
       <c r="M44" t="n">
-        <v>3208.07</v>
+        <v>24095.39</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -2259,22 +2259,22 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K45" t="n">
-        <v>5042.65</v>
+        <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>130020.2</v>
+        <v>3208.07</v>
       </c>
       <c r="M45" t="n">
-        <v>135062.85</v>
+        <v>3208.07</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -2302,15 +2302,58 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K46" t="n">
-        <v>0</v>
+        <v>5042.65</v>
       </c>
       <c r="L46" t="n">
+        <v>130020.2</v>
+      </c>
+      <c r="M46" t="n">
+        <v>135062.85</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>65046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2043</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" t="n">
         <v>6270.75</v>
       </c>
-      <c r="M46" t="n">
+      <c r="M47" t="n">
         <v>6270.75</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-08-28 15:21)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>25 de agosto de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -490,10 +490,10 @@
         <v>162964</v>
       </c>
       <c r="H4" t="n">
-        <v>8374.200000000001</v>
+        <v>9770.84</v>
       </c>
       <c r="I4" t="n">
-        <v>171338.2</v>
+        <v>172734.84</v>
       </c>
       <c r="J4" t="n">
         <v>1</v>
@@ -533,10 +533,10 @@
         <v>85004.67999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>63882.48</v>
+        <v>77510.67</v>
       </c>
       <c r="I5" t="n">
-        <v>148887.16</v>
+        <v>162515.35</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -545,10 +545,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>235535.47</v>
+        <v>228558.77</v>
       </c>
       <c r="M5" t="n">
-        <v>235535.47</v>
+        <v>228558.77</v>
       </c>
     </row>
     <row r="6">
@@ -726,17 +726,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -745,31 +745,31 @@
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>18368.13</v>
+        <v>12340.66</v>
       </c>
       <c r="H10" t="n">
-        <v>1659.4</v>
+        <v>10127.69</v>
       </c>
       <c r="I10" t="n">
-        <v>20027.53</v>
+        <v>22468.35</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>7957.05</v>
       </c>
       <c r="L10" t="n">
-        <v>44104.27</v>
+        <v>135596.86</v>
       </c>
       <c r="M10" t="n">
-        <v>44104.27</v>
+        <v>143553.91</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,22 +779,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>-19514.59</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>37963.62</v>
+        <v>21851.98</v>
       </c>
       <c r="I11" t="n">
-        <v>18449.03</v>
+        <v>21851.98</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,16 +803,16 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>68457.66</v>
+        <v>96692.85000000001</v>
       </c>
       <c r="M11" t="n">
-        <v>68457.66</v>
+        <v>96692.85000000001</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,22 +822,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>18368.13</v>
       </c>
       <c r="H12" t="n">
-        <v>17363.6</v>
+        <v>1659.4</v>
       </c>
       <c r="I12" t="n">
-        <v>17363.6</v>
+        <v>20027.53</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,59 +846,59 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>98929.74000000001</v>
+        <v>44104.27</v>
       </c>
       <c r="M12" t="n">
-        <v>98929.74000000001</v>
+        <v>44104.27</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>-19514.59</v>
       </c>
       <c r="H13" t="n">
-        <v>16956.37</v>
+        <v>37963.62</v>
       </c>
       <c r="I13" t="n">
-        <v>16956.37</v>
+        <v>18449.03</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>2308.82</v>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>93854.71000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>96163.53</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>16532.42</v>
+        <v>16956.37</v>
       </c>
       <c r="I14" t="n">
-        <v>16532.42</v>
+        <v>16956.37</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>38466.09</v>
+        <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>38466.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>15302.69</v>
+        <v>16532.42</v>
       </c>
       <c r="I15" t="n">
-        <v>15302.69</v>
+        <v>16532.42</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>51962.79</v>
+        <v>38466.09</v>
       </c>
       <c r="M15" t="n">
-        <v>51962.79</v>
+        <v>38466.09</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>15064.73</v>
+        <v>15302.69</v>
       </c>
       <c r="I16" t="n">
-        <v>15064.73</v>
+        <v>15302.69</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>5220.9</v>
+        <v>51962.79</v>
       </c>
       <c r="M16" t="n">
-        <v>5220.9</v>
+        <v>51962.79</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>15040.89</v>
+        <v>15064.73</v>
       </c>
       <c r="I17" t="n">
-        <v>15040.89</v>
+        <v>15064.73</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>13568.13</v>
+        <v>5220.9</v>
       </c>
       <c r="M17" t="n">
-        <v>13568.13</v>
+        <v>5220.9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>14560.31</v>
+        <v>15040.89</v>
       </c>
       <c r="I18" t="n">
-        <v>14560.31</v>
+        <v>15040.89</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,16 +1104,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>30975.68</v>
+        <v>13568.13</v>
       </c>
       <c r="M18" t="n">
-        <v>30975.68</v>
+        <v>13568.13</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,34 +1123,34 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>12340.66</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>14560.31</v>
       </c>
       <c r="I19" t="n">
-        <v>12340.66</v>
+        <v>14560.31</v>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>5042.65</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>142360.86</v>
+        <v>30975.68</v>
       </c>
       <c r="M19" t="n">
-        <v>147403.51</v>
+        <v>30975.68</v>
       </c>
     </row>
     <row r="20">
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>10596.4</v>
+        <v>12649.59</v>
       </c>
       <c r="I20" t="n">
-        <v>10596.4</v>
+        <v>12649.59</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,10 +1190,10 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>89590.05</v>
+        <v>87536.87</v>
       </c>
       <c r="M20" t="n">
-        <v>89590.05</v>
+        <v>87536.87</v>
       </c>
     </row>
     <row r="21">
@@ -1399,16 +1399,16 @@
         <v>6813.99</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>38963.3</v>
       </c>
       <c r="L25" t="n">
         <v>21526.27</v>
       </c>
       <c r="M25" t="n">
-        <v>21526.27</v>
+        <v>60489.57</v>
       </c>
     </row>
     <row r="26">
@@ -1629,17 +1629,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>63441</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2511</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>3610.04</v>
+        <v>3686.38</v>
       </c>
       <c r="I31" t="n">
-        <v>3610.04</v>
+        <v>3686.38</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,41 +1663,41 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>17237.12</v>
+        <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>17237.12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>1958.21</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>1627.21</v>
+        <v>3610.04</v>
       </c>
       <c r="I32" t="n">
-        <v>3585.42</v>
+        <v>3610.04</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,26 +1706,26 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>37341.24</v>
+        <v>17237.12</v>
       </c>
       <c r="M32" t="n">
-        <v>37341.24</v>
+        <v>17237.12</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>119447</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1734,13 +1734,13 @@
         <v>1</v>
       </c>
       <c r="G33" t="n">
-        <v>3052.25</v>
+        <v>1958.21</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>1627.21</v>
       </c>
       <c r="I33" t="n">
-        <v>3052.25</v>
+        <v>3585.42</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,41 +1749,41 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>33574.79</v>
+        <v>37341.24</v>
       </c>
       <c r="M33" t="n">
-        <v>33574.79</v>
+        <v>37341.24</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>3052.25</v>
       </c>
       <c r="H34" t="n">
-        <v>2960.97</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>2960.97</v>
+        <v>3052.25</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,16 +1792,16 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>0</v>
+        <v>33574.79</v>
       </c>
       <c r="M34" t="n">
-        <v>0</v>
+        <v>33574.79</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,22 +1811,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>2396.76</v>
+        <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>2960.97</v>
       </c>
       <c r="I35" t="n">
-        <v>2396.76</v>
+        <v>2960.97</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>26364.37</v>
+        <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>26364.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,22 +1854,22 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>2396.76</v>
       </c>
       <c r="H36" t="n">
-        <v>2068.31</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>2068.31</v>
+        <v>2396.76</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>18614.8</v>
+        <v>26364.37</v>
       </c>
       <c r="M36" t="n">
-        <v>18614.8</v>
+        <v>26364.37</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,22 +1897,22 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>1454.68</v>
+        <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>509.43</v>
+        <v>2068.31</v>
       </c>
       <c r="I37" t="n">
-        <v>1964.11</v>
+        <v>2068.31</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,41 +1921,41 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>26239.01</v>
+        <v>18614.8</v>
       </c>
       <c r="M37" t="n">
-        <v>26239.01</v>
+        <v>18614.8</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>63441</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>1454.68</v>
       </c>
       <c r="H38" t="n">
-        <v>1843.19</v>
+        <v>509.43</v>
       </c>
       <c r="I38" t="n">
-        <v>1843.19</v>
+        <v>1964.11</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,10 +1964,10 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>1843.19</v>
+        <v>26239.01</v>
       </c>
       <c r="M38" t="n">
-        <v>1843.19</v>
+        <v>26239.01</v>
       </c>
     </row>
     <row r="39">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-08-31 16:09)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>27 de agosto de 2026</t>
+          <t>28 de agosto de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -619,10 +619,10 @@
         <v>31798.96</v>
       </c>
       <c r="H7" t="n">
-        <v>37240.77</v>
+        <v>49011.06</v>
       </c>
       <c r="I7" t="n">
-        <v>69039.73</v>
+        <v>80810.02</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,10 +631,10 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>28233.37</v>
+        <v>16463.08</v>
       </c>
       <c r="M7" t="n">
-        <v>28233.37</v>
+        <v>16463.08</v>
       </c>
     </row>
     <row r="8">
@@ -662,10 +662,10 @@
         <v>2211.03</v>
       </c>
       <c r="H8" t="n">
-        <v>66617.46000000001</v>
+        <v>72024.35000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>68828.49000000001</v>
+        <v>74235.38</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,10 +674,10 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>69823.8</v>
+        <v>64416.9</v>
       </c>
       <c r="M8" t="n">
-        <v>69823.8</v>
+        <v>64416.9</v>
       </c>
     </row>
     <row r="9">
@@ -941,7 +941,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>16532.42</v>
+        <v>16805.03</v>
       </c>
       <c r="I15" t="n">
-        <v>16532.42</v>
+        <v>16805.03</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>38466.09</v>
+        <v>3480.6</v>
       </c>
       <c r="M15" t="n">
-        <v>38466.09</v>
+        <v>3480.6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>15302.69</v>
+        <v>16532.42</v>
       </c>
       <c r="I16" t="n">
-        <v>15302.69</v>
+        <v>16532.42</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>51962.79</v>
+        <v>38466.09</v>
       </c>
       <c r="M16" t="n">
-        <v>51962.79</v>
+        <v>38466.09</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>15064.73</v>
+        <v>16294.28</v>
       </c>
       <c r="I17" t="n">
-        <v>15064.73</v>
+        <v>16294.28</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>5220.9</v>
+        <v>29241.71</v>
       </c>
       <c r="M17" t="n">
-        <v>5220.9</v>
+        <v>29241.71</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>15040.89</v>
+        <v>15302.69</v>
       </c>
       <c r="I18" t="n">
-        <v>15040.89</v>
+        <v>15302.69</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,16 +1104,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>13568.13</v>
+        <v>51962.79</v>
       </c>
       <c r="M18" t="n">
-        <v>13568.13</v>
+        <v>51962.79</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>14560.31</v>
+        <v>15040.89</v>
       </c>
       <c r="I19" t="n">
-        <v>14560.31</v>
+        <v>15040.89</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,10 +1147,10 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>30975.68</v>
+        <v>13568.13</v>
       </c>
       <c r="M19" t="n">
-        <v>30975.68</v>
+        <v>13568.13</v>
       </c>
     </row>
     <row r="20">
@@ -1586,7 +1586,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,22 +1596,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>1958.21</v>
       </c>
       <c r="H30" t="n">
-        <v>4266.5</v>
+        <v>3564.58</v>
       </c>
       <c r="I30" t="n">
-        <v>4266.5</v>
+        <v>5522.79</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,26 +1620,26 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>6572.15</v>
+        <v>35403.87</v>
       </c>
       <c r="M30" t="n">
-        <v>6572.15</v>
+        <v>35403.87</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>63441</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>3686.38</v>
+        <v>4266.5</v>
       </c>
       <c r="I31" t="n">
-        <v>3686.38</v>
+        <v>4266.5</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,26 +1663,26 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>0</v>
+        <v>6572.15</v>
       </c>
       <c r="M31" t="n">
-        <v>0</v>
+        <v>6572.15</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>63441</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2511</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1694,10 +1694,10 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>3610.04</v>
+        <v>3686.38</v>
       </c>
       <c r="I32" t="n">
-        <v>3610.04</v>
+        <v>3686.38</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,41 +1706,41 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>17237.12</v>
+        <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>17237.12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>1958.21</v>
+        <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>1627.21</v>
+        <v>3610.04</v>
       </c>
       <c r="I33" t="n">
-        <v>3585.42</v>
+        <v>3610.04</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,10 +1749,10 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>37341.24</v>
+        <v>17237.12</v>
       </c>
       <c r="M33" t="n">
-        <v>37341.24</v>
+        <v>17237.12</v>
       </c>
     </row>
     <row r="34">
@@ -1786,16 +1786,16 @@
         <v>3052.25</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>1739.6</v>
       </c>
       <c r="L34" t="n">
-        <v>33574.79</v>
+        <v>52710.36</v>
       </c>
       <c r="M34" t="n">
-        <v>33574.79</v>
+        <v>54449.96</v>
       </c>
     </row>
     <row r="35">
@@ -1844,7 +1844,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,22 +1854,22 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>2396.76</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>2475.99</v>
       </c>
       <c r="I36" t="n">
-        <v>2396.76</v>
+        <v>2475.99</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>26364.37</v>
+        <v>21619.43</v>
       </c>
       <c r="M36" t="n">
-        <v>26364.37</v>
+        <v>21619.43</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,22 +1897,22 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G37" t="n">
-        <v>0</v>
+        <v>2396.76</v>
       </c>
       <c r="H37" t="n">
-        <v>2068.31</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>2068.31</v>
+        <v>2396.76</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>18614.8</v>
+        <v>26364.37</v>
       </c>
       <c r="M37" t="n">
-        <v>18614.8</v>
+        <v>26364.37</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,22 +1940,22 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>1454.68</v>
+        <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>509.43</v>
+        <v>2068.31</v>
       </c>
       <c r="I38" t="n">
-        <v>1964.11</v>
+        <v>2068.31</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>26239.01</v>
+        <v>18614.8</v>
       </c>
       <c r="M38" t="n">
-        <v>26239.01</v>
+        <v>18614.8</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,22 +1983,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>0</v>
+        <v>1454.68</v>
       </c>
       <c r="H39" t="n">
-        <v>1699.41</v>
+        <v>509.43</v>
       </c>
       <c r="I39" t="n">
-        <v>1699.41</v>
+        <v>1964.11</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>17392.81</v>
+        <v>26239.01</v>
       </c>
       <c r="M39" t="n">
-        <v>17392.81</v>
+        <v>26239.01</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2038,10 +2038,10 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>1595.73</v>
+        <v>1699.41</v>
       </c>
       <c r="I40" t="n">
-        <v>1595.73</v>
+        <v>1699.41</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>0</v>
+        <v>17392.81</v>
       </c>
       <c r="M40" t="n">
-        <v>0</v>
+        <v>17392.81</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2081,10 +2081,10 @@
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>1595.73</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>1595.73</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>3381.58</v>
+        <v>0</v>
       </c>
       <c r="M41" t="n">
-        <v>3381.58</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2136,16 +2136,16 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>12581.61</v>
+        <v>3381.58</v>
       </c>
       <c r="M42" t="n">
-        <v>12581.61</v>
+        <v>3381.58</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2179,16 +2179,16 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>1425.78</v>
+        <v>12581.61</v>
       </c>
       <c r="M43" t="n">
-        <v>1425.78</v>
+        <v>12581.61</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2222,16 +2222,16 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>3035.72</v>
+        <v>1425.78</v>
       </c>
       <c r="M44" t="n">
-        <v>3035.72</v>
+        <v>1425.78</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -2265,16 +2265,16 @@
         <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>24095.39</v>
+        <v>3035.72</v>
       </c>
       <c r="M45" t="n">
-        <v>24095.39</v>
+        <v>3035.72</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -2308,52 +2308,9 @@
         <v>0</v>
       </c>
       <c r="L46" t="n">
-        <v>3208.07</v>
+        <v>6270.75</v>
       </c>
       <c r="M46" t="n">
-        <v>3208.07</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>65046</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>2043</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" t="n">
-        <v>0</v>
-      </c>
-      <c r="I47" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" t="n">
-        <v>0</v>
-      </c>
-      <c r="K47" t="n">
-        <v>0</v>
-      </c>
-      <c r="L47" t="n">
-        <v>6270.75</v>
-      </c>
-      <c r="M47" t="n">
         <v>6270.75</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-09-03 11:12)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M46"/>
+  <dimension ref="A1:M47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>28 de agosto de 2026</t>
+          <t>31 de agosto de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -487,25 +487,25 @@
         <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>162964</v>
+        <v>163272.44</v>
       </c>
       <c r="H4" t="n">
-        <v>9770.84</v>
+        <v>9789.33</v>
       </c>
       <c r="I4" t="n">
-        <v>172734.84</v>
+        <v>173061.77</v>
       </c>
       <c r="J4" t="n">
         <v>1</v>
       </c>
       <c r="K4" t="n">
-        <v>72756.09</v>
+        <v>72893.8</v>
       </c>
       <c r="L4" t="n">
-        <v>80161.03</v>
+        <v>80312.75</v>
       </c>
       <c r="M4" t="n">
-        <v>152917.12</v>
+        <v>153206.55</v>
       </c>
     </row>
     <row r="5">
@@ -530,13 +530,13 @@
         <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>85004.67999999999</v>
+        <v>83421.06</v>
       </c>
       <c r="H5" t="n">
-        <v>77510.67</v>
+        <v>76661.97</v>
       </c>
       <c r="I5" t="n">
-        <v>162515.35</v>
+        <v>160083.03</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -545,10 +545,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>228558.77</v>
+        <v>228605.9</v>
       </c>
       <c r="M5" t="n">
-        <v>228558.77</v>
+        <v>228605.9</v>
       </c>
     </row>
     <row r="6">
@@ -573,13 +573,13 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>90049.44</v>
+        <v>90219.87</v>
       </c>
       <c r="H6" t="n">
-        <v>14399.82</v>
+        <v>14427.08</v>
       </c>
       <c r="I6" t="n">
-        <v>104449.26</v>
+        <v>104646.95</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,10 +588,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>14399.82</v>
+        <v>14427.08</v>
       </c>
       <c r="M6" t="n">
-        <v>14399.82</v>
+        <v>14427.08</v>
       </c>
     </row>
     <row r="7">
@@ -616,13 +616,13 @@
         <v>2</v>
       </c>
       <c r="G7" t="n">
-        <v>31798.96</v>
+        <v>31859.15</v>
       </c>
       <c r="H7" t="n">
-        <v>49011.06</v>
+        <v>49103.83</v>
       </c>
       <c r="I7" t="n">
-        <v>80810.02</v>
+        <v>80962.98</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,10 +631,10 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>16463.08</v>
+        <v>16494.24</v>
       </c>
       <c r="M7" t="n">
-        <v>16463.08</v>
+        <v>16494.24</v>
       </c>
     </row>
     <row r="8">
@@ -659,13 +659,13 @@
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>2211.03</v>
+        <v>2215.22</v>
       </c>
       <c r="H8" t="n">
-        <v>72024.35000000001</v>
+        <v>72160.67</v>
       </c>
       <c r="I8" t="n">
-        <v>74235.38</v>
+        <v>74375.89</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,10 +674,10 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>64416.9</v>
+        <v>64538.83</v>
       </c>
       <c r="M8" t="n">
-        <v>64416.9</v>
+        <v>64538.83</v>
       </c>
     </row>
     <row r="9">
@@ -702,13 +702,13 @@
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>33305.7</v>
+        <v>33368.74</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>33305.7</v>
+        <v>33368.74</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,10 +717,10 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>49020.81</v>
+        <v>49113.6</v>
       </c>
       <c r="M9" t="n">
-        <v>49020.81</v>
+        <v>49113.6</v>
       </c>
     </row>
     <row r="10">
@@ -742,34 +742,34 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>14025.77</v>
+      </c>
+      <c r="H10" t="n">
+        <v>14138.01</v>
+      </c>
+      <c r="I10" t="n">
+        <v>28163.78</v>
+      </c>
+      <c r="J10" t="n">
         <v>1</v>
       </c>
-      <c r="G10" t="n">
-        <v>12340.66</v>
-      </c>
-      <c r="H10" t="n">
-        <v>10127.69</v>
-      </c>
-      <c r="I10" t="n">
-        <v>22468.35</v>
-      </c>
-      <c r="J10" t="n">
-        <v>2</v>
-      </c>
       <c r="K10" t="n">
-        <v>7957.05</v>
+        <v>5052.2</v>
       </c>
       <c r="L10" t="n">
-        <v>135596.86</v>
+        <v>132563.5</v>
       </c>
       <c r="M10" t="n">
-        <v>143553.91</v>
+        <v>137615.7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,22 +779,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>-17238.33</v>
       </c>
       <c r="H11" t="n">
-        <v>21851.98</v>
+        <v>42122.13</v>
       </c>
       <c r="I11" t="n">
-        <v>21851.98</v>
+        <v>24883.8</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,41 +803,41 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>96692.85000000001</v>
+        <v>89945.69</v>
       </c>
       <c r="M11" t="n">
-        <v>96692.85000000001</v>
+        <v>89945.69</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>18368.13</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>1659.4</v>
+        <v>22403.65</v>
       </c>
       <c r="I12" t="n">
-        <v>20027.53</v>
+        <v>22403.65</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,16 +846,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>44104.27</v>
+        <v>10604.95</v>
       </c>
       <c r="M12" t="n">
-        <v>44104.27</v>
+        <v>10604.95</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,65 +865,65 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>-19514.59</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>37963.62</v>
+        <v>21893.33</v>
       </c>
       <c r="I13" t="n">
-        <v>18449.03</v>
+        <v>21893.33</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>2308.82</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>93854.71000000001</v>
+        <v>97042.89</v>
       </c>
       <c r="M13" t="n">
-        <v>96163.53</v>
+        <v>97042.89</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>18402.9</v>
       </c>
       <c r="H14" t="n">
-        <v>16956.37</v>
+        <v>3446.05</v>
       </c>
       <c r="I14" t="n">
-        <v>16956.37</v>
+        <v>21848.95</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>42404.25</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>42404.25</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>16805.03</v>
+        <v>16988.45</v>
       </c>
       <c r="I15" t="n">
-        <v>16805.03</v>
+        <v>16988.45</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>3480.6</v>
+        <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>3480.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>16532.42</v>
+        <v>16904.67</v>
       </c>
       <c r="I16" t="n">
-        <v>16532.42</v>
+        <v>16904.67</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>38466.09</v>
+        <v>50488.12</v>
       </c>
       <c r="M16" t="n">
-        <v>38466.09</v>
+        <v>50488.12</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>16294.28</v>
+        <v>16836.83</v>
       </c>
       <c r="I17" t="n">
-        <v>16294.28</v>
+        <v>16836.83</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>29241.71</v>
+        <v>3487.19</v>
       </c>
       <c r="M17" t="n">
-        <v>29241.71</v>
+        <v>3487.19</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>15302.69</v>
+        <v>16326.83</v>
       </c>
       <c r="I18" t="n">
-        <v>15302.69</v>
+        <v>16326.83</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,16 +1104,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>51962.79</v>
+        <v>38302.03</v>
       </c>
       <c r="M18" t="n">
-        <v>51962.79</v>
+        <v>38302.03</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>15040.89</v>
+        <v>16325.12</v>
       </c>
       <c r="I19" t="n">
-        <v>15040.89</v>
+        <v>16325.12</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,10 +1147,10 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>13568.13</v>
+        <v>29297.06</v>
       </c>
       <c r="M19" t="n">
-        <v>13568.13</v>
+        <v>29297.06</v>
       </c>
     </row>
     <row r="20">
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>12649.59</v>
+        <v>12673.52</v>
       </c>
       <c r="I20" t="n">
-        <v>12649.59</v>
+        <v>12673.52</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,10 +1190,10 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>87536.87</v>
+        <v>87702.55</v>
       </c>
       <c r="M20" t="n">
-        <v>87536.87</v>
+        <v>87702.55</v>
       </c>
     </row>
     <row r="21">
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>9749.9</v>
+        <v>9768.370000000001</v>
       </c>
       <c r="I21" t="n">
-        <v>9749.9</v>
+        <v>9768.370000000001</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,10 +1233,10 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>52726.89</v>
+        <v>52826.69</v>
       </c>
       <c r="M21" t="n">
-        <v>52726.89</v>
+        <v>52826.69</v>
       </c>
     </row>
     <row r="22">
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>8476.02</v>
+        <v>8492.07</v>
       </c>
       <c r="I22" t="n">
-        <v>8476.02</v>
+        <v>8492.07</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,10 +1276,10 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>5756.97</v>
+        <v>5767.87</v>
       </c>
       <c r="M22" t="n">
-        <v>5756.97</v>
+        <v>5767.87</v>
       </c>
     </row>
     <row r="23">
@@ -1307,10 +1307,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>7940.4</v>
+        <v>7955.43</v>
       </c>
       <c r="I23" t="n">
-        <v>7940.4</v>
+        <v>7955.43</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,10 +1319,10 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>17698.48</v>
+        <v>17731.98</v>
       </c>
       <c r="M23" t="n">
-        <v>17698.48</v>
+        <v>17731.98</v>
       </c>
     </row>
     <row r="24">
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>7004.2</v>
+        <v>7017.46</v>
       </c>
       <c r="I24" t="n">
-        <v>7004.2</v>
+        <v>7017.46</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,10 +1362,10 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>1888.66</v>
+        <v>1892.23</v>
       </c>
       <c r="M24" t="n">
-        <v>1888.66</v>
+        <v>1892.23</v>
       </c>
     </row>
     <row r="25">
@@ -1393,22 +1393,22 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>6813.99</v>
+        <v>6826.89</v>
       </c>
       <c r="I25" t="n">
-        <v>6813.99</v>
+        <v>6826.89</v>
       </c>
       <c r="J25" t="n">
         <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>38963.3</v>
+        <v>39037.05</v>
       </c>
       <c r="L25" t="n">
-        <v>21526.27</v>
+        <v>21567.01</v>
       </c>
       <c r="M25" t="n">
-        <v>60489.57</v>
+        <v>60604.06</v>
       </c>
     </row>
     <row r="26">
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>6087.09</v>
+        <v>6098.62</v>
       </c>
       <c r="I26" t="n">
-        <v>6087.09</v>
+        <v>6098.62</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,10 +1448,10 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>6398.05</v>
+        <v>6410.16</v>
       </c>
       <c r="M26" t="n">
-        <v>6398.05</v>
+        <v>6410.16</v>
       </c>
     </row>
     <row r="27">
@@ -1476,25 +1476,25 @@
         <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>6086.13</v>
+        <v>6097.65</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>6086.13</v>
+        <v>6097.65</v>
       </c>
       <c r="J27" t="n">
         <v>1</v>
       </c>
       <c r="K27" t="n">
-        <v>114882.54</v>
+        <v>115099.97</v>
       </c>
       <c r="L27" t="n">
-        <v>66947.41</v>
+        <v>67074.12</v>
       </c>
       <c r="M27" t="n">
-        <v>181829.95</v>
+        <v>182174.09</v>
       </c>
     </row>
     <row r="28">
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>6049.46</v>
+        <v>6060.91</v>
       </c>
       <c r="I28" t="n">
-        <v>6049.46</v>
+        <v>6060.91</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>5808.77</v>
+        <v>5819.76</v>
       </c>
       <c r="I29" t="n">
-        <v>5808.77</v>
+        <v>5819.76</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,10 +1577,10 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>103783.01</v>
+        <v>103979.43</v>
       </c>
       <c r="M29" t="n">
-        <v>103783.01</v>
+        <v>103979.43</v>
       </c>
     </row>
     <row r="30">
@@ -1605,13 +1605,13 @@
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>1958.21</v>
+        <v>1961.92</v>
       </c>
       <c r="H30" t="n">
-        <v>3564.58</v>
+        <v>3571.33</v>
       </c>
       <c r="I30" t="n">
-        <v>5522.79</v>
+        <v>5533.25</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,26 +1620,26 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>35403.87</v>
+        <v>35470.88</v>
       </c>
       <c r="M30" t="n">
-        <v>35403.87</v>
+        <v>35470.88</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>4266.5</v>
+        <v>5319.15</v>
       </c>
       <c r="I31" t="n">
-        <v>4266.5</v>
+        <v>5319.15</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,41 +1663,41 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>6572.15</v>
+        <v>15937.48</v>
       </c>
       <c r="M31" t="n">
-        <v>6572.15</v>
+        <v>15937.48</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>63441</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>4800.92</v>
       </c>
       <c r="H32" t="n">
-        <v>3686.38</v>
+        <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>3686.38</v>
+        <v>4800.92</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,26 +1706,26 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>0</v>
+        <v>52810.13</v>
       </c>
       <c r="M32" t="n">
-        <v>0</v>
+        <v>52810.13</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>3610.04</v>
+        <v>4274.58</v>
       </c>
       <c r="I33" t="n">
-        <v>3610.04</v>
+        <v>4274.58</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,59 +1749,59 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>17237.12</v>
+        <v>6584.58</v>
       </c>
       <c r="M33" t="n">
-        <v>17237.12</v>
+        <v>6584.58</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>119447</t>
+          <t>63441</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2511</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>3052.25</v>
+        <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>3693.35</v>
       </c>
       <c r="I34" t="n">
-        <v>3052.25</v>
+        <v>3693.35</v>
       </c>
       <c r="J34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>1739.6</v>
+        <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>52710.36</v>
+        <v>0</v>
       </c>
       <c r="M34" t="n">
-        <v>54449.96</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>2960.97</v>
+        <v>3521.42</v>
       </c>
       <c r="I35" t="n">
-        <v>2960.97</v>
+        <v>3521.42</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>0</v>
+        <v>20619.61</v>
       </c>
       <c r="M35" t="n">
-        <v>0</v>
+        <v>20619.61</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>2475.99</v>
+        <v>2966.58</v>
       </c>
       <c r="I36" t="n">
-        <v>2475.99</v>
+        <v>2966.58</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,10 +1878,10 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>21619.43</v>
+        <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>21619.43</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -1906,13 +1906,13 @@
         <v>1</v>
       </c>
       <c r="G37" t="n">
-        <v>2396.76</v>
+        <v>2401.3</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>2396.76</v>
+        <v>2401.3</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,10 +1921,10 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>26364.37</v>
+        <v>26414.27</v>
       </c>
       <c r="M37" t="n">
-        <v>26364.37</v>
+        <v>26414.27</v>
       </c>
     </row>
     <row r="38">
@@ -1952,10 +1952,10 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>2068.31</v>
+        <v>2072.23</v>
       </c>
       <c r="I38" t="n">
-        <v>2068.31</v>
+        <v>2072.23</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,10 +1964,10 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>18614.8</v>
+        <v>18650.03</v>
       </c>
       <c r="M38" t="n">
-        <v>18614.8</v>
+        <v>18650.03</v>
       </c>
     </row>
     <row r="39">
@@ -1992,13 +1992,13 @@
         <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>1454.68</v>
+        <v>1457.43</v>
       </c>
       <c r="H39" t="n">
-        <v>509.43</v>
+        <v>510.39</v>
       </c>
       <c r="I39" t="n">
-        <v>1964.11</v>
+        <v>1967.82</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2007,10 +2007,10 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>26239.01</v>
+        <v>26288.67</v>
       </c>
       <c r="M39" t="n">
-        <v>26239.01</v>
+        <v>26288.67</v>
       </c>
     </row>
     <row r="40">
@@ -2038,10 +2038,10 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>1699.41</v>
+        <v>1702.63</v>
       </c>
       <c r="I40" t="n">
-        <v>1699.41</v>
+        <v>1702.63</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>17392.81</v>
+        <v>17425.73</v>
       </c>
       <c r="M40" t="n">
-        <v>17392.81</v>
+        <v>17425.73</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2081,10 +2081,10 @@
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>1595.73</v>
+        <v>1693.99</v>
       </c>
       <c r="I41" t="n">
-        <v>1595.73</v>
+        <v>1693.99</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>0</v>
+        <v>1693.99</v>
       </c>
       <c r="M41" t="n">
-        <v>0</v>
+        <v>1693.99</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2124,10 +2124,10 @@
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>1598.75</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>1598.75</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -2136,16 +2136,16 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>3381.58</v>
+        <v>0</v>
       </c>
       <c r="M42" t="n">
-        <v>3381.58</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2167,10 +2167,10 @@
         <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>1040.74</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>1040.74</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
@@ -2179,26 +2179,26 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>12581.61</v>
+        <v>5241.88</v>
       </c>
       <c r="M43" t="n">
-        <v>12581.61</v>
+        <v>5241.88</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>120051</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2216,22 +2216,22 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K44" t="n">
-        <v>0</v>
+        <v>2488.17</v>
       </c>
       <c r="L44" t="n">
-        <v>1425.78</v>
+        <v>27369.85</v>
       </c>
       <c r="M44" t="n">
-        <v>1425.78</v>
+        <v>29858.02</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -2265,16 +2265,16 @@
         <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>3035.72</v>
+        <v>12605.42</v>
       </c>
       <c r="M45" t="n">
-        <v>3035.72</v>
+        <v>12605.42</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -2308,10 +2308,53 @@
         <v>0</v>
       </c>
       <c r="L46" t="n">
-        <v>6270.75</v>
+        <v>1428.48</v>
       </c>
       <c r="M46" t="n">
-        <v>6270.75</v>
+        <v>1428.48</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>108405</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2043</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" t="n">
+        <v>3041.47</v>
+      </c>
+      <c r="M47" t="n">
+        <v>3041.47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-09-08 14:09)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>31 de agosto de 2026</t>
+          <t>4 de septiembre de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -468,75 +468,75 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>163272.44</v>
+        <v>39037.05</v>
       </c>
       <c r="H4" t="n">
-        <v>9789.33</v>
+        <v>1821.92</v>
       </c>
       <c r="I4" t="n">
-        <v>173061.77</v>
+        <v>40858.97</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>72893.8</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>80312.75</v>
+        <v>24779.71</v>
       </c>
       <c r="M4" t="n">
-        <v>153206.55</v>
+        <v>24779.71</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>83421.06</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>76661.97</v>
+        <v>13505.41</v>
       </c>
       <c r="I5" t="n">
-        <v>160083.03</v>
+        <v>13505.41</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -545,16 +545,16 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>228605.9</v>
+        <v>94372.73</v>
       </c>
       <c r="M5" t="n">
-        <v>228605.9</v>
+        <v>94372.73</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,22 +564,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>90219.87</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>14427.08</v>
+        <v>10023.33</v>
       </c>
       <c r="I6" t="n">
-        <v>104646.95</v>
+        <v>10023.33</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,41 +588,41 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>14427.08</v>
+        <v>65066.43</v>
       </c>
       <c r="M6" t="n">
-        <v>14427.08</v>
+        <v>65066.43</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>31859.15</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>49103.83</v>
+        <v>9440.07</v>
       </c>
       <c r="I7" t="n">
-        <v>80962.98</v>
+        <v>9440.07</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,16 +631,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>16494.24</v>
+        <v>89858.53999999999</v>
       </c>
       <c r="M7" t="n">
-        <v>16494.24</v>
+        <v>89858.53999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,22 +650,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>2215.22</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>72160.67</v>
+        <v>8492.07</v>
       </c>
       <c r="I8" t="n">
-        <v>74375.89</v>
+        <v>8492.07</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,16 +674,16 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>64538.83</v>
+        <v>3845.25</v>
       </c>
       <c r="M8" t="n">
-        <v>64538.83</v>
+        <v>3845.25</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,22 +693,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>33368.74</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>7409.62</v>
       </c>
       <c r="I9" t="n">
-        <v>33368.74</v>
+        <v>7409.62</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,16 +717,16 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>49113.6</v>
+        <v>235826.63</v>
       </c>
       <c r="M9" t="n">
-        <v>49113.6</v>
+        <v>235826.63</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -736,65 +736,65 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>14025.77</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>14138.01</v>
+        <v>5431.4</v>
       </c>
       <c r="I10" t="n">
-        <v>28163.78</v>
+        <v>5431.4</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>5052.2</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>132563.5</v>
+        <v>12899.71</v>
       </c>
       <c r="M10" t="n">
-        <v>137615.7</v>
+        <v>12899.71</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>-17238.33</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>42122.13</v>
+        <v>5152.9</v>
       </c>
       <c r="I11" t="n">
-        <v>24883.8</v>
+        <v>5152.9</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,16 +803,16 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>89945.69</v>
+        <v>29490.48</v>
       </c>
       <c r="M11" t="n">
-        <v>89945.69</v>
+        <v>29490.48</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>22403.65</v>
+        <v>5090.96</v>
       </c>
       <c r="I12" t="n">
-        <v>22403.65</v>
+        <v>5090.96</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,26 +846,26 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>10604.95</v>
+        <v>48657.15</v>
       </c>
       <c r="M12" t="n">
-        <v>10604.95</v>
+        <v>48657.15</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,10 +877,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>21893.33</v>
+        <v>4709.73</v>
       </c>
       <c r="I13" t="n">
-        <v>21893.33</v>
+        <v>4709.73</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -889,41 +889,41 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>97042.89</v>
+        <v>2309.36</v>
       </c>
       <c r="M13" t="n">
-        <v>97042.89</v>
+        <v>2309.36</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>18402.9</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>3446.05</v>
+        <v>4021.19</v>
       </c>
       <c r="I14" t="n">
-        <v>21848.95</v>
+        <v>4021.19</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>42404.25</v>
+        <v>31449.72</v>
       </c>
       <c r="M14" t="n">
-        <v>42404.25</v>
+        <v>31449.72</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>16988.45</v>
+        <v>2966.58</v>
       </c>
       <c r="I15" t="n">
-        <v>16988.45</v>
+        <v>2966.58</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -984,7 +984,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>16904.67</v>
+        <v>2426.76</v>
       </c>
       <c r="I16" t="n">
-        <v>16904.67</v>
+        <v>2426.76</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>50488.12</v>
+        <v>38711.19</v>
       </c>
       <c r="M16" t="n">
-        <v>50488.12</v>
+        <v>38711.19</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>16836.83</v>
+        <v>2408.61</v>
       </c>
       <c r="I17" t="n">
-        <v>16836.83</v>
+        <v>2408.61</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>3487.19</v>
+        <v>5453.73</v>
       </c>
       <c r="M17" t="n">
-        <v>3487.19</v>
+        <v>5453.73</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>16326.83</v>
+        <v>1800.77</v>
       </c>
       <c r="I18" t="n">
-        <v>16326.83</v>
+        <v>1800.77</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,16 +1104,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>38302.03</v>
+        <v>10804.65</v>
       </c>
       <c r="M18" t="n">
-        <v>38302.03</v>
+        <v>10804.65</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>16325.12</v>
+        <v>1761.04</v>
       </c>
       <c r="I19" t="n">
-        <v>16325.12</v>
+        <v>1761.04</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,16 +1147,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>29297.06</v>
+        <v>7337.05</v>
       </c>
       <c r="M19" t="n">
-        <v>29297.06</v>
+        <v>7337.05</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>12673.52</v>
+        <v>1747.29</v>
       </c>
       <c r="I20" t="n">
-        <v>12673.52</v>
+        <v>1747.29</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,16 +1190,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>87702.55</v>
+        <v>3494.59</v>
       </c>
       <c r="M20" t="n">
-        <v>87702.55</v>
+        <v>3494.59</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>9768.370000000001</v>
+        <v>1737.43</v>
       </c>
       <c r="I21" t="n">
-        <v>9768.370000000001</v>
+        <v>1737.43</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,16 +1233,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>52826.69</v>
+        <v>91447.39999999999</v>
       </c>
       <c r="M21" t="n">
-        <v>52826.69</v>
+        <v>91447.39999999999</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>8492.07</v>
+        <v>1516.55</v>
       </c>
       <c r="I22" t="n">
-        <v>8492.07</v>
+        <v>1516.55</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,26 +1276,26 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>5767.87</v>
+        <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>5767.87</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>120051</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,38 +1307,38 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>7955.43</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>7955.43</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>2488.17</v>
       </c>
       <c r="L23" t="n">
-        <v>17731.98</v>
+        <v>27369.85</v>
       </c>
       <c r="M23" t="n">
-        <v>17731.98</v>
+        <v>29858.02</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>7017.46</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>7017.46</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,26 +1362,26 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>1892.23</v>
+        <v>52810.13</v>
       </c>
       <c r="M24" t="n">
-        <v>1892.23</v>
+        <v>52810.13</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1393,38 +1393,38 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>6826.89</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>6826.89</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>39037.05</v>
+        <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>21567.01</v>
+        <v>26414.27</v>
       </c>
       <c r="M25" t="n">
-        <v>60604.06</v>
+        <v>26414.27</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>6098.62</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>6098.62</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>6410.16</v>
+        <v>49113.6</v>
       </c>
       <c r="M26" t="n">
-        <v>6410.16</v>
+        <v>49113.6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,50 +1467,50 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>6097.65</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>6097.65</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>115099.97</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>67074.12</v>
+        <v>28256.41</v>
       </c>
       <c r="M27" t="n">
-        <v>182174.09</v>
+        <v>28256.41</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>6060.91</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>6060.91</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>0</v>
+        <v>42404.25</v>
       </c>
       <c r="M28" t="n">
-        <v>0</v>
+        <v>42404.25</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>5819.76</v>
+        <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>5819.76</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,16 +1577,16 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>103979.43</v>
+        <v>68825.82000000001</v>
       </c>
       <c r="M29" t="n">
-        <v>103979.43</v>
+        <v>68825.82000000001</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,22 +1596,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>1961.92</v>
+        <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>3571.33</v>
+        <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>5533.25</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,10 +1620,10 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>35470.88</v>
+        <v>4796.14</v>
       </c>
       <c r="M30" t="n">
-        <v>35470.88</v>
+        <v>4796.14</v>
       </c>
     </row>
     <row r="31">
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>5319.15</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>5319.15</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,41 +1663,41 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>15937.48</v>
+        <v>17269.74</v>
       </c>
       <c r="M31" t="n">
-        <v>15937.48</v>
+        <v>17269.74</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>119447</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>4800.92</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>4800.92</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,16 +1706,16 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>52810.13</v>
+        <v>3487.19</v>
       </c>
       <c r="M32" t="n">
-        <v>52810.13</v>
+        <v>3487.19</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>4274.58</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>4274.58</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,26 +1749,26 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>6584.58</v>
+        <v>1693.99</v>
       </c>
       <c r="M33" t="n">
-        <v>6584.58</v>
+        <v>1693.99</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>63441</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA CARLOS VAZQUEZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>3693.35</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>3693.35</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,26 +1792,26 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>0</v>
+        <v>17425.73</v>
       </c>
       <c r="M34" t="n">
-        <v>0</v>
+        <v>17425.73</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>3521.42</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>3521.42</v>
+        <v>0</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>20619.61</v>
+        <v>6410.16</v>
       </c>
       <c r="M35" t="n">
-        <v>20619.61</v>
+        <v>6410.16</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>2966.58</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>2966.58</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>0</v>
+        <v>18650.03</v>
       </c>
       <c r="M36" t="n">
-        <v>0</v>
+        <v>18650.03</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,22 +1897,22 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>2401.3</v>
+        <v>0</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>2401.3</v>
+        <v>0</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>26414.27</v>
+        <v>67074.12</v>
       </c>
       <c r="M37" t="n">
-        <v>26414.27</v>
+        <v>67074.12</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1952,10 +1952,10 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>2072.23</v>
+        <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>2072.23</v>
+        <v>0</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>18650.03</v>
+        <v>14427.08</v>
       </c>
       <c r="M38" t="n">
-        <v>18650.03</v>
+        <v>14427.08</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,22 +1983,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>1457.43</v>
+        <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>510.39</v>
+        <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>1967.82</v>
+        <v>0</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>26288.67</v>
+        <v>3041.47</v>
       </c>
       <c r="M39" t="n">
-        <v>26288.67</v>
+        <v>3041.47</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2038,10 +2038,10 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>1702.63</v>
+        <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>1702.63</v>
+        <v>0</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>17425.73</v>
+        <v>39833.53</v>
       </c>
       <c r="M40" t="n">
-        <v>17425.73</v>
+        <v>39833.53</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2081,10 +2081,10 @@
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>1693.99</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>1693.99</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>1693.99</v>
+        <v>23106.58</v>
       </c>
       <c r="M41" t="n">
-        <v>1693.99</v>
+        <v>23106.58</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2124,10 +2124,10 @@
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>1598.75</v>
+        <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>1598.75</v>
+        <v>0</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -2136,16 +2136,16 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>0</v>
+        <v>12811.03</v>
       </c>
       <c r="M42" t="n">
-        <v>0</v>
+        <v>12811.03</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2167,10 +2167,10 @@
         <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>1040.74</v>
+        <v>0</v>
       </c>
       <c r="I43" t="n">
-        <v>1040.74</v>
+        <v>0</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
@@ -2179,26 +2179,26 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>5241.88</v>
+        <v>6060.86</v>
       </c>
       <c r="M43" t="n">
-        <v>5241.88</v>
+        <v>6060.86</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>120051</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2216,22 +2216,22 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>2488.17</v>
+        <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>27369.85</v>
+        <v>3214.14</v>
       </c>
       <c r="M44" t="n">
-        <v>29858.02</v>
+        <v>3214.14</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -2265,16 +2265,16 @@
         <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>12605.42</v>
+        <v>56725.37</v>
       </c>
       <c r="M45" t="n">
-        <v>12605.42</v>
+        <v>56725.37</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -2308,16 +2308,16 @@
         <v>0</v>
       </c>
       <c r="L46" t="n">
-        <v>1428.48</v>
+        <v>86129.07000000001</v>
       </c>
       <c r="M46" t="n">
-        <v>1428.48</v>
+        <v>86129.07000000001</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -2345,16 +2345,16 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>72893.8</v>
       </c>
       <c r="L47" t="n">
-        <v>3041.47</v>
+        <v>80312.75</v>
       </c>
       <c r="M47" t="n">
-        <v>3041.47</v>
+        <v>153206.55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-09-09 19:32)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>4 de septiembre de 2026</t>
+          <t>8 de septiembre de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -490,10 +490,10 @@
         <v>39037.05</v>
       </c>
       <c r="H4" t="n">
-        <v>1821.92</v>
+        <v>6821.96</v>
       </c>
       <c r="I4" t="n">
-        <v>40858.97</v>
+        <v>45859.01</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -502,16 +502,16 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>24779.71</v>
+        <v>19745.09</v>
       </c>
       <c r="M4" t="n">
-        <v>24779.71</v>
+        <v>19745.09</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -521,22 +521,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>29655.2</v>
       </c>
       <c r="H5" t="n">
-        <v>13505.41</v>
+        <v>11503.4</v>
       </c>
       <c r="I5" t="n">
-        <v>13505.41</v>
+        <v>41158.6</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -545,26 +545,26 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>94372.73</v>
+        <v>89858.53999999999</v>
       </c>
       <c r="M5" t="n">
-        <v>94372.73</v>
+        <v>89858.53999999999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -576,10 +576,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>10023.33</v>
+        <v>14976.76</v>
       </c>
       <c r="I6" t="n">
-        <v>10023.33</v>
+        <v>14976.76</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,26 +588,26 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>65066.43</v>
+        <v>94372.73</v>
       </c>
       <c r="M6" t="n">
-        <v>65066.43</v>
+        <v>94372.73</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -619,10 +619,10 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>9440.07</v>
+        <v>10023.33</v>
       </c>
       <c r="I7" t="n">
-        <v>9440.07</v>
+        <v>10023.33</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,16 +631,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>89858.53999999999</v>
+        <v>65066.43</v>
       </c>
       <c r="M7" t="n">
-        <v>89858.53999999999</v>
+        <v>65066.43</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -662,28 +662,28 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>8492.07</v>
+        <v>9142.639999999999</v>
       </c>
       <c r="I8" t="n">
-        <v>8492.07</v>
+        <v>9142.639999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>9832.18</v>
       </c>
       <c r="L8" t="n">
-        <v>3845.25</v>
+        <v>234093.61</v>
       </c>
       <c r="M8" t="n">
-        <v>3845.25</v>
+        <v>243925.79</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -705,10 +705,10 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>7409.62</v>
+        <v>8492.07</v>
       </c>
       <c r="I9" t="n">
-        <v>7409.62</v>
+        <v>8492.07</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,10 +717,10 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>235826.63</v>
+        <v>3845.25</v>
       </c>
       <c r="M9" t="n">
-        <v>235826.63</v>
+        <v>3845.25</v>
       </c>
     </row>
     <row r="10">
@@ -941,17 +941,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>2966.58</v>
+        <v>3524.19</v>
       </c>
       <c r="I15" t="n">
-        <v>2966.58</v>
+        <v>3524.19</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>68825.82000000001</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>68825.82000000001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>2426.76</v>
+        <v>2966.58</v>
       </c>
       <c r="I16" t="n">
-        <v>2426.76</v>
+        <v>2966.58</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>38711.19</v>
+        <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>38711.19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>2408.61</v>
+        <v>2426.76</v>
       </c>
       <c r="I17" t="n">
-        <v>2408.61</v>
+        <v>2426.76</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>5453.73</v>
+        <v>38711.19</v>
       </c>
       <c r="M17" t="n">
-        <v>5453.73</v>
+        <v>38711.19</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>1800.77</v>
+        <v>2408.61</v>
       </c>
       <c r="I18" t="n">
-        <v>1800.77</v>
+        <v>2408.61</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,16 +1104,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>10804.65</v>
+        <v>5453.73</v>
       </c>
       <c r="M18" t="n">
-        <v>10804.65</v>
+        <v>5453.73</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>1761.04</v>
+        <v>1967.73</v>
       </c>
       <c r="I19" t="n">
-        <v>1761.04</v>
+        <v>1967.73</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,16 +1147,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>7337.05</v>
+        <v>26288.67</v>
       </c>
       <c r="M19" t="n">
-        <v>7337.05</v>
+        <v>26288.67</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>1747.29</v>
+        <v>1800.77</v>
       </c>
       <c r="I20" t="n">
-        <v>1747.29</v>
+        <v>1800.77</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,16 +1190,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>3494.59</v>
+        <v>10804.65</v>
       </c>
       <c r="M20" t="n">
-        <v>3494.59</v>
+        <v>10804.65</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>1737.43</v>
+        <v>1761.04</v>
       </c>
       <c r="I21" t="n">
-        <v>1737.43</v>
+        <v>1761.04</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,16 +1233,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>91447.39999999999</v>
+        <v>7337.05</v>
       </c>
       <c r="M21" t="n">
-        <v>91447.39999999999</v>
+        <v>7337.05</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>1516.55</v>
+        <v>1747.29</v>
       </c>
       <c r="I22" t="n">
-        <v>1516.55</v>
+        <v>1747.29</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,26 +1276,26 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>3494.59</v>
       </c>
       <c r="M22" t="n">
-        <v>0</v>
+        <v>3494.59</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>120051</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,38 +1307,38 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>1737.43</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>1737.43</v>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>2488.17</v>
+        <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>27369.85</v>
+        <v>91447.39999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>29858.02</v>
+        <v>91447.39999999999</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>119447</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>1516.55</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>1516.55</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,26 +1362,26 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>52810.13</v>
+        <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>52810.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>120051</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1399,32 +1399,32 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>2488.17</v>
       </c>
       <c r="L25" t="n">
-        <v>26414.27</v>
+        <v>27369.85</v>
       </c>
       <c r="M25" t="n">
-        <v>26414.27</v>
+        <v>29858.02</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>49113.6</v>
+        <v>52810.13</v>
       </c>
       <c r="M26" t="n">
-        <v>49113.6</v>
+        <v>52810.13</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1491,26 +1491,26 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>28256.41</v>
+        <v>26414.27</v>
       </c>
       <c r="M27" t="n">
-        <v>28256.41</v>
+        <v>26414.27</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>42404.25</v>
+        <v>49113.6</v>
       </c>
       <c r="M28" t="n">
-        <v>42404.25</v>
+        <v>49113.6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1577,10 +1577,10 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>68825.82000000001</v>
+        <v>42404.25</v>
       </c>
       <c r="M29" t="n">
-        <v>68825.82000000001</v>
+        <v>42404.25</v>
       </c>
     </row>
     <row r="30">

</xml_diff>